<commit_message>
model: spread five-year historical financials
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,25 +2,87 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R0c69ace4a5ec40d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R98be73b4bf584de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rf626eadddd694e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Rec32ee12721a4dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rd85d99bb70ab4a62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R638323f9d5f543fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R72ab56be9f40490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Rfa16436eb5ac4d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="Rebed8124df1f4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rfebcad45192241aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Rd2adf58f65944f75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rcbea4bbd3f5d4a17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Ra2ed21c48fa549eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="Rffa6f8247f384404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Rc07289511ccd408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R61285c0446a24602"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Rc37c36aa09bb4a03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R596b0530d4b54598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R439030d13ec3485a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R44764e2e52264363"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R6a420828d5b649a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R459609d15f5a4d53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R2036425053ac4873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R755958d44d8c462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Rf7efe5c360d347ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R9a05b379003944bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R8f6851970db242a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R1031f119379743f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R12afe89f196a4f32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R41f9b19dcca2475c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R3b3330b6778749a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R9e901b0e9c2c4c0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rebe754c17b9b42ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Rb5437824698b412c"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={F6DB3FAA-A1EC-7D77-2866-86E73D1A637E}</x:author>
+    <x:author>tc={CC4A0B00-5474-EF44-8ACC-00181B81D655}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="G7" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Sources: Rockwell FY2022 and FY2025 Forms 10-K; SEC Company Facts. Total segment operating earnings is a company-defined non-GAAP measure.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="G35" authorId="1">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Balance sheet and financing-capacity inputs are sourced from audited Rockwell Forms 10-K.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={85CE8A89-E83C-1D89-0606-CC1110311CD7}</x:author>
+    <x:author>tc={F880D00B-EDF4-F6C0-6143-47B16B480219}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="G7" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Sources: Cognex FY2023 and FY2025 Forms 10-K; SEC Company Facts. See the Sources worksheet for URLs and filing dates.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="G47" authorId="1">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Balance sheet inputs are taken from Cognex's audited Forms 10-K and reconciled to total assets, liabilities, and equity.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -29,14 +91,22 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="13">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
     <x:numFmt numFmtId="203" formatCode="0.0%;[Red](0.0%);-"/>
     <x:numFmt numFmtId="204" formatCode="$#,##0;[Red]($#,##0);-"/>
+    <x:numFmt numFmtId="205" formatCode="yyyy&quot;A&quot;"/>
+    <x:numFmt numFmtId="206" formatCode="$#,##0.0;[Red]($#,##0.0);-"/>
+    <x:numFmt numFmtId="207" formatCode="0.0;[Red](0.0);-"/>
+    <x:numFmt numFmtId="208" formatCode="$0.000;[Red]($0.000);-"/>
+    <x:numFmt numFmtId="209" formatCode="0.0"/>
+    <x:numFmt numFmtId="210" formatCode="0.0x;[Red](0.0x);-"/>
+    <x:numFmt numFmtId="211" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="212" formatCode="0.000;[Red](0.000);-"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="28">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -115,8 +185,85 @@
       <x:color rgb="FF0563C1"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -158,8 +305,28 @@
         <x:fgColor rgb="FFC6E0B4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="6">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -191,11 +358,21 @@
         <x:color rgb="FFA6A6A6"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="137">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -268,15 +445,257 @@
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="212" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="212" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="212" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="212" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="2">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF008000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC00000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:person displayName="Rohan Dravid" id="{51843E4D-6D01-459A-8247-31E61F25B311}"/>
   <xltc:person displayName="Rohan Dravid" id="{80509790-5AC7-4B70-9CDF-14DA69F61825}"/>
 </xltc:personList>
 </file>
@@ -472,6 +891,28 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="G7" dT="2026-08-21T04:02:47.572" personId="{51843E4D-6D01-459A-8247-31E61F25B311}" id="{F6DB3FAA-A1EC-7D77-2866-86E73D1A637E}">
+    <xltc:text>Sources: Rockwell FY2022 and FY2025 Forms 10-K; SEC Company Facts. Total segment operating earnings is a company-defined non-GAAP measure.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="G35" dT="2026-08-21T04:02:47.572" personId="{51843E4D-6D01-459A-8247-31E61F25B311}" id="{CC4A0B00-5474-EF44-8ACC-00181B81D655}">
+    <xltc:text>Balance sheet and financing-capacity inputs are sourced from audited Rockwell Forms 10-K.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
+<file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="G7" dT="2026-08-21T04:02:47.532" personId="{51843E4D-6D01-459A-8247-31E61F25B311}" id="{85CE8A89-E83C-1D89-0606-CC1110311CD7}">
+    <xltc:text>Sources: Cognex FY2023 and FY2025 Forms 10-K; SEC Company Facts. See the Sources worksheet for URLs and filing dates.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="G47" dT="2026-08-21T04:02:47.534" personId="{51843E4D-6D01-459A-8247-31E61F25B311}" id="{F880D00B-EDF4-F6C0-6143-47B16B480219}">
+    <xltc:text>Balance sheet inputs are taken from Cognex's audited Forms 10-K and reconciled to total assets, liabilities, and equity.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -525,7 +966,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.1 — architecture shell</x:v>
+        <x:v>0.2 — historicals complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -580,9 +1021,9 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="21" t="str">
+      <x:c r="B9" s="136" t="str">
         <x:f>'Checks'!B3</x:f>
-        <x:v>SETUP</x:v>
+        <x:v>HISTORICALS COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -1621,212 +2062,281 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="119" t="str">
         <x:v>Model Checks</x:v>
       </x:c>
-      <x:c r="B1" s="2"/>
-      <x:c r="C1" s="2"/>
-      <x:c r="D1" s="2"/>
-      <x:c r="E1" s="2"/>
-      <x:c r="F1" s="2"/>
-      <x:c r="G1" s="2"/>
+      <x:c r="B1" s="119"/>
+      <x:c r="C1" s="119"/>
+      <x:c r="D1" s="119"/>
+      <x:c r="E1" s="119"/>
+      <x:c r="F1" s="119"/>
+      <x:c r="G1" s="119"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="122"/>
+      <x:c r="B2" s="122"/>
+      <x:c r="C2" s="122"/>
+      <x:c r="D2" s="122"/>
+      <x:c r="E2" s="122"/>
+      <x:c r="F2" s="122"/>
+      <x:c r="G2" s="122"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="13" t="str">
+      <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="48" t="str">
-        <x:f>IF(COUNTIF(F6:F15,"FAIL")&gt;0,"FAIL",IF(COUNTIF(F6:F15,"NOT STARTED")&gt;0,"SETUP","OK"))</x:f>
-        <x:v>SETUP</x:v>
-      </x:c>
+      <x:c r="B3" s="133" t="str">
+        <x:f>IF(COUNTIF(F6:F11,"FAIL")&gt;0,"CHECK REQUIRED","HISTORICALS COMPLETE")</x:f>
+        <x:v>HISTORICALS COMPLETE</x:v>
+      </x:c>
+      <x:c r="C3" s="122"/>
+      <x:c r="D3" s="122"/>
+      <x:c r="E3" s="122"/>
+      <x:c r="F3" s="122"/>
+      <x:c r="G3" s="122"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="122"/>
+      <x:c r="B4" s="122"/>
+      <x:c r="C4" s="122"/>
+      <x:c r="D4" s="122"/>
+      <x:c r="E4" s="122"/>
+      <x:c r="F4" s="122"/>
+      <x:c r="G4" s="122"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="49" t="str">
+      <x:c r="A5" s="121" t="str">
         <x:v>Check</x:v>
       </x:c>
-      <x:c r="B5" s="49" t="str">
+      <x:c r="B5" s="121" t="str">
         <x:v>Actual</x:v>
       </x:c>
-      <x:c r="C5" s="49" t="str">
+      <x:c r="C5" s="121" t="str">
         <x:v>Expected</x:v>
       </x:c>
-      <x:c r="D5" s="49" t="str">
+      <x:c r="D5" s="121" t="str">
         <x:v>Difference</x:v>
       </x:c>
-      <x:c r="E5" s="49" t="str">
+      <x:c r="E5" s="121" t="str">
         <x:v>Tolerance</x:v>
       </x:c>
-      <x:c r="F5" s="49" t="str">
+      <x:c r="F5" s="121" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="G5" s="49" t="str">
+      <x:c r="G5" s="121" t="str">
         <x:v>Fix / location</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="122" t="str">
         <x:v>Source completeness</x:v>
       </x:c>
-      <x:c r="B6"/>
-      <x:c r="C6"/>
-      <x:c r="D6"/>
-      <x:c r="E6"/>
-      <x:c r="F6" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G6" t="str">
-        <x:v>Sources / historical tabs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Historical statement tie-out</x:v>
-      </x:c>
-      <x:c r="B7"/>
-      <x:c r="C7"/>
-      <x:c r="D7"/>
-      <x:c r="E7"/>
-      <x:c r="F7" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G7" t="str">
-        <x:v>ROK and CGNX Historical</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Cash roll-forward</x:v>
-      </x:c>
-      <x:c r="B8"/>
-      <x:c r="C8"/>
-      <x:c r="D8"/>
-      <x:c r="E8"/>
-      <x:c r="F8" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:v>Operating model</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>Debt roll-forward</x:v>
-      </x:c>
-      <x:c r="B9"/>
-      <x:c r="C9"/>
-      <x:c r="D9"/>
-      <x:c r="E9"/>
-      <x:c r="F9" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G9" t="str">
-        <x:v>ROK Forecast / Sources &amp; Uses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Diluted shares</x:v>
-      </x:c>
-      <x:c r="B10"/>
-      <x:c r="C10"/>
-      <x:c r="D10"/>
-      <x:c r="E10"/>
-      <x:c r="F10" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G10" t="str">
-        <x:v>Historical and A/D tabs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>DCF component tie-out</x:v>
-      </x:c>
-      <x:c r="B11"/>
-      <x:c r="C11"/>
-      <x:c r="D11"/>
-      <x:c r="E11"/>
-      <x:c r="F11" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G11" t="str">
-        <x:v>DCF</x:v>
+      <x:c r="B6" s="134" t="n">
+        <x:f>COUNTA('Sources'!A4:A9)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C6" s="135" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D6" s="135" t="n">
+        <x:f>B6-C6</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="122" t="str">
+        <x:f>IF(ABS(D6)&lt;=E6,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G6" s="124" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="122" t="str">
+        <x:v>CGNX gross profit tie-out</x:v>
+      </x:c>
+      <x:c r="B7" s="134" t="n">
+        <x:f>MAX(ABS('CGNX Historical'!B12),ABS('CGNX Historical'!C12),ABS('CGNX Historical'!D12),ABS('CGNX Historical'!E12),ABS('CGNX Historical'!F12))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="135" t="n">
+        <x:f>B7-C7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="135" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F7" s="122" t="str">
+        <x:f>IF(ABS(D7)&lt;=E7,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G7" s="124" t="str">
+        <x:v>CGNX Historical row 12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="122" t="str">
+        <x:v>CGNX diluted EPS tie-out</x:v>
+      </x:c>
+      <x:c r="B8" s="134" t="n">
+        <x:f>MAX(ABS('CGNX Historical'!B30),ABS('CGNX Historical'!C30),ABS('CGNX Historical'!D30),ABS('CGNX Historical'!E30),ABS('CGNX Historical'!F30))</x:f>
+        <x:v>0.004911737954128026</x:v>
+      </x:c>
+      <x:c r="C8" s="135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8" s="135" t="n">
+        <x:f>B8-C8</x:f>
+        <x:v>0.004911737954128026</x:v>
+      </x:c>
+      <x:c r="E8" s="135" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F8" s="122" t="str">
+        <x:f>IF(ABS(D8)&lt;=E8,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G8" s="124" t="str">
+        <x:v>CGNX Historical row 30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="122" t="str">
+        <x:v>CGNX balance sheet tie-out</x:v>
+      </x:c>
+      <x:c r="B9" s="134" t="n">
+        <x:f>MAX(ABS('CGNX Historical'!B59),ABS('CGNX Historical'!C59),ABS('CGNX Historical'!D59),ABS('CGNX Historical'!E59),ABS('CGNX Historical'!F59))</x:f>
+        <x:v>2.2737367544323206e-13</x:v>
+      </x:c>
+      <x:c r="C9" s="135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="135" t="n">
+        <x:f>B9-C9</x:f>
+        <x:v>2.2737367544323206e-13</x:v>
+      </x:c>
+      <x:c r="E9" s="135" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F9" s="122" t="str">
+        <x:f>IF(ABS(D9)&lt;=E9,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G9" s="124" t="str">
+        <x:v>CGNX Historical row 59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" hidden="0" customHeight="1">
+      <x:c r="A10" s="122" t="str">
+        <x:v>ROK diluted EPS tie-out</x:v>
+      </x:c>
+      <x:c r="B10" s="134" t="n">
+        <x:f>MAX(ABS('ROK Historical'!B20),ABS('ROK Historical'!C20),ABS('ROK Historical'!D20),ABS('ROK Historical'!E20),ABS('ROK Historical'!F20))</x:f>
+        <x:v>0.048269896193772865</x:v>
+      </x:c>
+      <x:c r="C10" s="135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="135" t="n">
+        <x:f>B10-C10</x:f>
+        <x:v>0.048269896193772865</x:v>
+      </x:c>
+      <x:c r="E10" s="135" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="F10" s="122" t="str">
+        <x:f>IF(ABS(D10)&lt;=E10,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G10" s="124" t="str">
+        <x:v>ROK Historical row 20; tolerance reflects rounded $mm and share disclosures</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="122" t="str">
+        <x:v>ROK balance sheet tie-out</x:v>
+      </x:c>
+      <x:c r="B11" s="134" t="n">
+        <x:f>MAX(ABS('ROK Historical'!B47),ABS('ROK Historical'!C47),ABS('ROK Historical'!D47),ABS('ROK Historical'!E47),ABS('ROK Historical'!F47))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C11" s="135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="135" t="n">
+        <x:f>B11-C11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="135" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F11" s="122" t="str">
+        <x:f>IF(ABS(D11)&lt;=E11,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G11" s="124" t="str">
+        <x:v>ROK Historical row 47</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>Enterprise-to-equity bridge</x:v>
-      </x:c>
+      <x:c r="A12"/>
       <x:c r="B12"/>
       <x:c r="C12"/>
       <x:c r="D12"/>
       <x:c r="E12"/>
-      <x:c r="F12" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G12" t="str">
-        <x:v>DCF / Valuation Summary</x:v>
-      </x:c>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>Sources equal uses</x:v>
-      </x:c>
+      <x:c r="A13"/>
       <x:c r="B13"/>
       <x:c r="C13"/>
       <x:c r="D13"/>
       <x:c r="E13"/>
-      <x:c r="F13" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
-        <x:v>Sources &amp; Uses</x:v>
-      </x:c>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>Purchase accounting</x:v>
-      </x:c>
+      <x:c r="A14"/>
       <x:c r="B14"/>
       <x:c r="C14"/>
       <x:c r="D14"/>
       <x:c r="E14"/>
-      <x:c r="F14" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>Purchase Accounting</x:v>
-      </x:c>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>Pro forma EPS</x:v>
-      </x:c>
+      <x:c r="A15"/>
       <x:c r="B15"/>
       <x:c r="C15"/>
       <x:c r="D15"/>
       <x:c r="E15"/>
-      <x:c r="F15" s="10" t="str">
-        <x:v>NOT STARTED</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>Accretion Dilution</x:v>
-      </x:c>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="F6:F11">
+    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="OK"/>
+    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="FAIL"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -2058,107 +2568,224 @@
   <x:cols>
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="62" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="119" t="str">
         <x:v>Sources &amp; Audit Trail</x:v>
       </x:c>
-      <x:c r="B1" s="2"/>
-      <x:c r="C1" s="2"/>
-      <x:c r="D1" s="2"/>
-      <x:c r="E1" s="2"/>
-      <x:c r="F1" s="2"/>
-      <x:c r="G1" s="2"/>
-      <x:c r="H1" s="2"/>
+      <x:c r="B1" s="119"/>
+      <x:c r="C1" s="119"/>
+      <x:c r="D1" s="119"/>
+      <x:c r="E1" s="119"/>
+      <x:c r="F1" s="119"/>
+      <x:c r="G1" s="119"/>
+      <x:c r="H1" s="119"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="120" t="str">
+        <x:v>Primary-source documents supporting historical financial statements and model inputs</x:v>
+      </x:c>
+      <x:c r="B2" s="120"/>
+      <x:c r="C2" s="120"/>
+      <x:c r="D2" s="120"/>
+      <x:c r="E2" s="120"/>
+      <x:c r="F2" s="120"/>
+      <x:c r="G2" s="120"/>
+      <x:c r="H2" s="120"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="42" t="str">
+      <x:c r="A3" s="121" t="str">
         <x:v>Source ID</x:v>
       </x:c>
-      <x:c r="B3" s="43" t="str">
+      <x:c r="B3" s="121" t="str">
         <x:v>Company</x:v>
       </x:c>
-      <x:c r="C3" s="43" t="str">
+      <x:c r="C3" s="121" t="str">
         <x:v>Document</x:v>
       </x:c>
-      <x:c r="D3" s="43" t="str">
+      <x:c r="D3" s="121" t="str">
         <x:v>Publication date</x:v>
       </x:c>
-      <x:c r="E3" s="43" t="str">
+      <x:c r="E3" s="121" t="str">
         <x:v>Access date</x:v>
       </x:c>
-      <x:c r="F3" s="43" t="str">
+      <x:c r="F3" s="121" t="str">
         <x:v>Model use</x:v>
       </x:c>
-      <x:c r="G3" s="43" t="str">
+      <x:c r="G3" s="121" t="str">
         <x:v>URL</x:v>
       </x:c>
-      <x:c r="H3" s="44" t="str">
+      <x:c r="H3" s="121" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="46" t="str">
-        <x:v>S-001</x:v>
-      </x:c>
-      <x:c r="B4" s="14" t="str">
+    <x:row r="4" ht="24" hidden="0" customHeight="1">
+      <x:c r="A4" s="128" t="str">
+        <x:v>S-017</x:v>
+      </x:c>
+      <x:c r="B4" s="126" t="str">
         <x:v>Rockwell Automation</x:v>
       </x:c>
-      <x:c r="C4" s="14" t="str">
-        <x:v>2025 Form 10-K archive</x:v>
-      </x:c>
-      <x:c r="D4" s="14" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="E4" s="14" t="str">
-        <x:v>2026-08-20</x:v>
-      </x:c>
-      <x:c r="F4" s="14" t="str">
-        <x:v>Historical financials and company research</x:v>
-      </x:c>
-      <x:c r="G4" s="47" t="str">
-        <x:v>https://www.rockwellautomation.com/en-us/company/investor-relations/annual-reports.html</x:v>
-      </x:c>
-      <x:c r="H4" s="14" t="str">
-        <x:v>Primary company source</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="46" t="str">
-        <x:v>S-002</x:v>
-      </x:c>
-      <x:c r="B5" s="14" t="str">
+      <x:c r="C4" s="126" t="str">
+        <x:v>FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="D4" s="127" t="n">
+        <x:v>45973.5</x:v>
+      </x:c>
+      <x:c r="E4" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="F4" s="126" t="str">
+        <x:v>FY2023-FY2025 historicals; business and segment research</x:v>
+      </x:c>
+      <x:c r="G4" s="126" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1024478/000102447825000116/rok-20250930.htm</x:v>
+      </x:c>
+      <x:c r="H4" s="126" t="str">
+        <x:v>Primary audited filing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="128" t="str">
+        <x:v>S-019</x:v>
+      </x:c>
+      <x:c r="B5" s="126" t="str">
         <x:v>Cognex</x:v>
       </x:c>
-      <x:c r="C5" s="14" t="str">
-        <x:v>SEC filings archive</x:v>
-      </x:c>
-      <x:c r="D5" s="14" t="str">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="E5" s="14" t="str">
-        <x:v>2026-08-20</x:v>
-      </x:c>
-      <x:c r="F5" s="14" t="str">
-        <x:v>Historical financials and company research</x:v>
-      </x:c>
-      <x:c r="G5" s="47" t="str">
-        <x:v>https://investor.cognex.com/financial-reports/sec-filings/default.aspx</x:v>
-      </x:c>
-      <x:c r="H5" s="14" t="str">
-        <x:v>Primary company source</x:v>
+      <x:c r="C5" s="126" t="str">
+        <x:v>FY2025 Form 10-K</x:v>
+      </x:c>
+      <x:c r="D5" s="127" t="n">
+        <x:v>46065.5</x:v>
+      </x:c>
+      <x:c r="E5" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="F5" s="126" t="str">
+        <x:v>FY2023-FY2025 historical statements and operating data</x:v>
+      </x:c>
+      <x:c r="G5" s="126" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/851205/000085120526000012/cgnx-20251231.htm</x:v>
+      </x:c>
+      <x:c r="H5" s="126" t="str">
+        <x:v>Primary audited filing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="128" t="str">
+        <x:v>S-025</x:v>
+      </x:c>
+      <x:c r="B6" s="126" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C6" s="126" t="str">
+        <x:v>FY2023 Form 10-K</x:v>
+      </x:c>
+      <x:c r="D6" s="127" t="n">
+        <x:v>45337.5</x:v>
+      </x:c>
+      <x:c r="E6" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="F6" s="126" t="str">
+        <x:v>FY2021-FY2023 comparative historical statements</x:v>
+      </x:c>
+      <x:c r="G6" s="126" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/851205/000085120524000027/cgnx-20231231.htm</x:v>
+      </x:c>
+      <x:c r="H6" s="126" t="str">
+        <x:v>Primary audited filing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
+      <x:c r="A7" s="128" t="str">
+        <x:v>S-026</x:v>
+      </x:c>
+      <x:c r="B7" s="126" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C7" s="126" t="str">
+        <x:v>FY2022 Form 10-K</x:v>
+      </x:c>
+      <x:c r="D7" s="127" t="n">
+        <x:v>44873.5</x:v>
+      </x:c>
+      <x:c r="E7" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="F7" s="126" t="str">
+        <x:v>FY2021-FY2022 history and total segment operating earnings</x:v>
+      </x:c>
+      <x:c r="G7" s="126" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1024478/000102447822000093/rok-20220930.htm</x:v>
+      </x:c>
+      <x:c r="H7" s="126" t="str">
+        <x:v>Primary audited filing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="128" t="str">
+        <x:v>S-027</x:v>
+      </x:c>
+      <x:c r="B8" s="126" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C8" s="126" t="str">
+        <x:v>SEC Company Facts API</x:v>
+      </x:c>
+      <x:c r="D8" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="E8" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="F8" s="126" t="str">
+        <x:v>XBRL extraction and statement tie-out</x:v>
+      </x:c>
+      <x:c r="G8" s="126" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0001024478.json</x:v>
+      </x:c>
+      <x:c r="H8" s="126" t="str">
+        <x:v>Primary SEC structured data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="128" t="str">
+        <x:v>S-028</x:v>
+      </x:c>
+      <x:c r="B9" s="126" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C9" s="126" t="str">
+        <x:v>SEC Company Facts API</x:v>
+      </x:c>
+      <x:c r="D9" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="E9" s="127" t="n">
+        <x:v>46254.5</x:v>
+      </x:c>
+      <x:c r="F9" s="126" t="str">
+        <x:v>XBRL extraction and statement tie-out</x:v>
+      </x:c>
+      <x:c r="G9" s="126" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0000851205.json</x:v>
+      </x:c>
+      <x:c r="H9" s="126" t="str">
+        <x:v>Primary SEC structured data</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2168,112 +2795,1402 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="61" t="str">
         <x:v>ROK Historical</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Rockwell historical financial statements and operating KPIs</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
+      <x:c r="B1" s="62"/>
+      <x:c r="C1" s="62"/>
+      <x:c r="D1" s="62"/>
+      <x:c r="E1" s="62"/>
+      <x:c r="F1" s="62"/>
+      <x:c r="G1" s="63"/>
+      <x:c r="H1" s="64"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="69" t="str">
+        <x:v>Rockwell Automation historical financial and transaction-capacity summary | USD millions, except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="70"/>
+      <x:c r="C2" s="70"/>
+      <x:c r="D2" s="70"/>
+      <x:c r="E2" s="70"/>
+      <x:c r="F2" s="70"/>
+      <x:c r="G2" s="71"/>
+      <x:c r="H2" s="72"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="A3" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
+      <x:c r="B3" s="75" t="str">
+        <x:v>Complete — FY2021 to FY2025 audited history loaded</x:v>
+      </x:c>
+      <x:c r="C3" s="75"/>
+      <x:c r="D3" s="75"/>
+      <x:c r="E3" s="75"/>
+      <x:c r="F3" s="75"/>
+      <x:c r="G3" s="54"/>
+      <x:c r="H3" s="56"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="52"/>
+      <x:c r="B4" s="53"/>
+      <x:c r="C4" s="53"/>
+      <x:c r="D4" s="53"/>
+      <x:c r="E4" s="53"/>
+      <x:c r="F4" s="53"/>
+      <x:c r="G4" s="54"/>
+      <x:c r="H4" s="56"/>
+    </x:row>
+    <x:row r="5" ht="19" customHeight="1">
+      <x:c r="A5" s="76" t="str">
+        <x:v>EARNINGS AND PROFITABILITY</x:v>
+      </x:c>
+      <x:c r="B5" s="77"/>
+      <x:c r="C5" s="77"/>
+      <x:c r="D5" s="77"/>
+      <x:c r="E5" s="77"/>
+      <x:c r="F5" s="77"/>
+      <x:c r="G5" s="78"/>
+      <x:c r="H5" s="79"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
+      <x:c r="A6" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B6" s="92" t="n">
+        <x:v>44469.5</x:v>
+      </x:c>
+      <x:c r="C6" s="92" t="n">
+        <x:v>44834.5</x:v>
+      </x:c>
+      <x:c r="D6" s="92" t="n">
+        <x:v>45199.5</x:v>
+      </x:c>
+      <x:c r="E6" s="92" t="n">
+        <x:v>45565.5</x:v>
+      </x:c>
+      <x:c r="F6" s="92" t="n">
+        <x:v>45930.5</x:v>
+      </x:c>
+      <x:c r="G6" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H6" s="91" t="str">
+        <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
+      <x:c r="A7" s="52" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="n">
+        <x:v>6997.4</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="n">
+        <x:v>7760.4</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="n">
+        <x:v>9058</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="n">
+        <x:v>8264</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="n">
+        <x:v>8342</x:v>
+      </x:c>
+      <x:c r="G7" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H7" s="56" t="str"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
+      <x:c r="A8" s="52" t="str">
+        <x:v>% growth</x:v>
+      </x:c>
+      <x:c r="B8" s="94"/>
+      <x:c r="C8" s="94" t="n">
+        <x:f>C7/B7-1</x:f>
+        <x:v>0.10904050075742422</x:v>
+      </x:c>
+      <x:c r="D8" s="94" t="n">
+        <x:f>D7/C7-1</x:f>
+        <x:v>0.16720787588268649</x:v>
+      </x:c>
+      <x:c r="E8" s="94" t="n">
+        <x:f>E7/D7-1</x:f>
+        <x:v>-0.08765731949657762</x:v>
+      </x:c>
+      <x:c r="F8" s="94" t="n">
+        <x:f>F7/E7-1</x:f>
+        <x:v>0.009438528557599302</x:v>
+      </x:c>
+      <x:c r="G8" s="54"/>
+      <x:c r="H8" s="56"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
+      <x:c r="A9" s="99" t="str">
+        <x:v>Total segment operating earnings</x:v>
+      </x:c>
+      <x:c r="B9" s="100" t="n">
+        <x:v>1391.3</x:v>
+      </x:c>
+      <x:c r="C9" s="100" t="n">
+        <x:v>1542.6</x:v>
+      </x:c>
+      <x:c r="D9" s="100" t="n">
+        <x:v>1929</x:v>
+      </x:c>
+      <x:c r="E9" s="100" t="n">
+        <x:v>1595</x:v>
+      </x:c>
+      <x:c r="F9" s="100" t="n">
+        <x:v>1703</x:v>
+      </x:c>
+      <x:c r="G9" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H9" s="56" t="str">
+        <x:v>Company-defined non-GAAP measure; best consistent operating-profit series</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="52" t="str">
+        <x:v>Total segment operating margin</x:v>
+      </x:c>
+      <x:c r="B10" s="94" t="n">
+        <x:f>B9/B7</x:f>
+        <x:v>0.19883099436933718</x:v>
+      </x:c>
+      <x:c r="C10" s="94" t="n">
+        <x:f>C9/C7</x:f>
+        <x:v>0.19877841348384104</x:v>
+      </x:c>
+      <x:c r="D10" s="94" t="n">
+        <x:f>D9/D7</x:f>
+        <x:v>0.21296091852506072</x:v>
+      </x:c>
+      <x:c r="E10" s="94" t="n">
+        <x:f>E9/E7</x:f>
+        <x:v>0.1930058083252662</x:v>
+      </x:c>
+      <x:c r="F10" s="94" t="n">
+        <x:f>F9/F7</x:f>
+        <x:v>0.20414768640613762</x:v>
+      </x:c>
+      <x:c r="G10" s="54"/>
+      <x:c r="H10" s="56"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="A11" s="52" t="str">
+        <x:v>Net non-segment items</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="n">
+        <x:f>B12-B9</x:f>
+        <x:v>134.9000000000001</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="n">
+        <x:f>C12-C9</x:f>
+        <x:v>-469</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="n">
+        <x:f>D12-D9</x:f>
+        <x:v>-321</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="n">
+        <x:f>E12-E9</x:f>
+        <x:v>-495</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="n">
+        <x:f>F12-F9</x:f>
+        <x:v>-786</x:v>
+      </x:c>
+      <x:c r="G11" s="54"/>
+      <x:c r="H11" s="56"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="99" t="str">
+        <x:v>Income before income taxes</x:v>
+      </x:c>
+      <x:c r="B12" s="100" t="n">
+        <x:v>1526.2</x:v>
+      </x:c>
+      <x:c r="C12" s="100" t="n">
+        <x:v>1073.6</x:v>
+      </x:c>
+      <x:c r="D12" s="100" t="n">
+        <x:v>1608</x:v>
+      </x:c>
+      <x:c r="E12" s="100" t="n">
+        <x:v>1100</x:v>
+      </x:c>
+      <x:c r="F12" s="100" t="n">
+        <x:v>917</x:v>
+      </x:c>
+      <x:c r="G12" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H12" s="56" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="52" t="str">
+        <x:v>Income tax expense</x:v>
+      </x:c>
+      <x:c r="B13" s="93" t="n">
+        <x:v>181.9</x:v>
+      </x:c>
+      <x:c r="C13" s="93" t="n">
+        <x:v>154.5</x:v>
+      </x:c>
+      <x:c r="D13" s="93" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E13" s="93" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="F13" s="93" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="G13" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H13" s="56" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="52" t="str">
+        <x:v>Effective tax rate</x:v>
+      </x:c>
+      <x:c r="B14" s="94" t="n">
+        <x:f>B13/B12</x:f>
+        <x:v>0.11918490368234831</x:v>
+      </x:c>
+      <x:c r="C14" s="94" t="n">
+        <x:f>C13/C12</x:f>
+        <x:v>0.14390834575260805</x:v>
+      </x:c>
+      <x:c r="D14" s="94" t="n">
+        <x:f>D13/D12</x:f>
+        <x:v>0.20522388059701493</x:v>
+      </x:c>
+      <x:c r="E14" s="94" t="n">
+        <x:f>E13/E12</x:f>
+        <x:v>0.13818181818181818</x:v>
+      </x:c>
+      <x:c r="F14" s="94" t="n">
+        <x:f>F13/F12</x:f>
+        <x:v>0.183206106870229</x:v>
+      </x:c>
+      <x:c r="G14" s="54"/>
+      <x:c r="H14" s="56"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="99" t="str">
+        <x:v>Net income attributable to Rockwell</x:v>
+      </x:c>
+      <x:c r="B15" s="100" t="n">
+        <x:v>1358.1</x:v>
+      </x:c>
+      <x:c r="C15" s="100" t="n">
+        <x:v>932.2</x:v>
+      </x:c>
+      <x:c r="D15" s="100" t="n">
+        <x:v>1387</x:v>
+      </x:c>
+      <x:c r="E15" s="100" t="n">
+        <x:v>953</x:v>
+      </x:c>
+      <x:c r="F15" s="100" t="n">
+        <x:v>869</x:v>
+      </x:c>
+      <x:c r="G15" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H15" s="56" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="52" t="str">
+        <x:v>Net income margin</x:v>
+      </x:c>
+      <x:c r="B16" s="94" t="n">
+        <x:f>B15/B7</x:f>
+        <x:v>0.19408637493926315</x:v>
+      </x:c>
+      <x:c r="C16" s="94" t="n">
+        <x:f>C15/C7</x:f>
+        <x:v>0.1201226740889645</x:v>
+      </x:c>
+      <x:c r="D16" s="94" t="n">
+        <x:f>D15/D7</x:f>
+        <x:v>0.153124310002208</x:v>
+      </x:c>
+      <x:c r="E16" s="94" t="n">
+        <x:f>E15/E7</x:f>
+        <x:v>0.11531945788964182</x:v>
+      </x:c>
+      <x:c r="F16" s="94" t="n">
+        <x:f>F15/F7</x:f>
+        <x:v>0.10417166147206905</x:v>
+      </x:c>
+      <x:c r="G16" s="54"/>
+      <x:c r="H16" s="56"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="52" t="str">
+        <x:v>Diluted weighted average shares</x:v>
+      </x:c>
+      <x:c r="B17" s="95" t="n">
+        <x:v>117.1</x:v>
+      </x:c>
+      <x:c r="C17" s="95" t="n">
+        <x:v>116.7</x:v>
+      </x:c>
+      <x:c r="D17" s="95" t="n">
+        <x:v>115.6</x:v>
+      </x:c>
+      <x:c r="E17" s="95" t="n">
+        <x:v>114.5</x:v>
+      </x:c>
+      <x:c r="F17" s="95" t="n">
+        <x:v>113.1</x:v>
+      </x:c>
+      <x:c r="G17" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H17" s="56" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="99" t="str">
+        <x:v>Diluted EPS — calculated</x:v>
+      </x:c>
+      <x:c r="B18" s="102" t="n">
+        <x:f>B15/B17</x:f>
+        <x:v>11.597779675491033</x:v>
+      </x:c>
+      <x:c r="C18" s="102" t="n">
+        <x:f>C15/C17</x:f>
+        <x:v>7.988003427592116</x:v>
+      </x:c>
+      <x:c r="D18" s="102" t="n">
+        <x:f>D15/D17</x:f>
+        <x:v>11.998269896193772</x:v>
+      </x:c>
+      <x:c r="E18" s="102" t="n">
+        <x:f>E15/E17</x:f>
+        <x:v>8.323144104803493</x:v>
+      </x:c>
+      <x:c r="F18" s="102" t="n">
+        <x:f>F15/F17</x:f>
+        <x:v>7.683465959328029</x:v>
+      </x:c>
+      <x:c r="G18" s="54"/>
+      <x:c r="H18" s="56"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="52" t="str">
+        <x:v>Diluted EPS — reported</x:v>
+      </x:c>
+      <x:c r="B19" s="96" t="n">
+        <x:v>11.58</x:v>
+      </x:c>
+      <x:c r="C19" s="96" t="n">
+        <x:v>7.97</x:v>
+      </x:c>
+      <x:c r="D19" s="96" t="n">
+        <x:v>11.95</x:v>
+      </x:c>
+      <x:c r="E19" s="96" t="n">
+        <x:v>8.28</x:v>
+      </x:c>
+      <x:c r="F19" s="96" t="n">
+        <x:v>7.67</x:v>
+      </x:c>
+      <x:c r="G19" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H19" s="56" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="52" t="str">
+        <x:v>EPS tie-out</x:v>
+      </x:c>
+      <x:c r="B20" s="97" t="n">
+        <x:f>B18-B19</x:f>
+        <x:v>0.017779675491032876</x:v>
+      </x:c>
+      <x:c r="C20" s="97" t="n">
+        <x:f>C18-C19</x:f>
+        <x:v>0.018003427592116594</x:v>
+      </x:c>
+      <x:c r="D20" s="97" t="n">
+        <x:f>D18-D19</x:f>
+        <x:v>0.048269896193772865</x:v>
+      </x:c>
+      <x:c r="E20" s="97" t="n">
+        <x:f>E18-E19</x:f>
+        <x:v>0.04314410480349373</x:v>
+      </x:c>
+      <x:c r="F20" s="97" t="n">
+        <x:f>F18-F19</x:f>
+        <x:v>0.013465959328028632</x:v>
+      </x:c>
+      <x:c r="G20" s="54"/>
+      <x:c r="H20" s="56"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="52"/>
+      <x:c r="B21" s="53"/>
+      <x:c r="C21" s="53"/>
+      <x:c r="D21" s="53"/>
+      <x:c r="E21" s="53"/>
+      <x:c r="F21" s="53"/>
+      <x:c r="G21" s="54"/>
+      <x:c r="H21" s="56"/>
+    </x:row>
+    <x:row r="22" ht="19" customHeight="1">
+      <x:c r="A22" s="76" t="str">
+        <x:v>CASH FLOW AND FINANCING CAPACITY</x:v>
+      </x:c>
+      <x:c r="B22" s="77"/>
+      <x:c r="C22" s="77"/>
+      <x:c r="D22" s="77"/>
+      <x:c r="E22" s="77"/>
+      <x:c r="F22" s="77"/>
+      <x:c r="G22" s="78"/>
+      <x:c r="H22" s="79"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B23" s="92" t="n">
+        <x:v>44469.5</x:v>
+      </x:c>
+      <x:c r="C23" s="92" t="n">
+        <x:v>44834.5</x:v>
+      </x:c>
+      <x:c r="D23" s="92" t="n">
+        <x:v>45199.5</x:v>
+      </x:c>
+      <x:c r="E23" s="92" t="n">
+        <x:v>45565.5</x:v>
+      </x:c>
+      <x:c r="F23" s="92" t="n">
+        <x:v>45930.5</x:v>
+      </x:c>
+      <x:c r="G23" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H23" s="91" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="52" t="str">
+        <x:v>Net income</x:v>
+      </x:c>
+      <x:c r="B24" s="93" t="n">
+        <x:f>B15</x:f>
+        <x:v>1358.1</x:v>
+      </x:c>
+      <x:c r="C24" s="93" t="n">
+        <x:f>C15</x:f>
+        <x:v>932.2</x:v>
+      </x:c>
+      <x:c r="D24" s="93" t="n">
+        <x:f>D15</x:f>
+        <x:v>1387</x:v>
+      </x:c>
+      <x:c r="E24" s="93" t="n">
+        <x:f>E15</x:f>
+        <x:v>953</x:v>
+      </x:c>
+      <x:c r="F24" s="93" t="n">
+        <x:f>F15</x:f>
+        <x:v>869</x:v>
+      </x:c>
+      <x:c r="G24" s="54"/>
+      <x:c r="H24" s="56"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="52" t="str">
+        <x:v>Depreciation &amp; amortization</x:v>
+      </x:c>
+      <x:c r="B25" s="93" t="n">
+        <x:v>189.8</x:v>
+      </x:c>
+      <x:c r="C25" s="93" t="n">
+        <x:v>238.9</x:v>
+      </x:c>
+      <x:c r="D25" s="93" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="E25" s="93" t="n">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="F25" s="93" t="n">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="G25" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H25" s="56" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="52" t="str">
+        <x:v>Stock-based compensation</x:v>
+      </x:c>
+      <x:c r="B26" s="93" t="n">
+        <x:v>51.7</x:v>
+      </x:c>
+      <x:c r="C26" s="93" t="n">
+        <x:v>68.1</x:v>
+      </x:c>
+      <x:c r="D26" s="93" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="E26" s="93" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F26" s="93" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="G26" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H26" s="56" t="str"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="99" t="str">
+        <x:v>Cash provided by operating activities</x:v>
+      </x:c>
+      <x:c r="B27" s="100" t="n">
+        <x:v>1261</x:v>
+      </x:c>
+      <x:c r="C27" s="100" t="n">
+        <x:v>823.1</x:v>
+      </x:c>
+      <x:c r="D27" s="100" t="n">
+        <x:v>1374</x:v>
+      </x:c>
+      <x:c r="E27" s="100" t="n">
+        <x:v>864</x:v>
+      </x:c>
+      <x:c r="F27" s="100" t="n">
+        <x:v>1544</x:v>
+      </x:c>
+      <x:c r="G27" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H27" s="56" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="52" t="str">
+        <x:v>Capital expenditures</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="n">
+        <x:v>-120.3</x:v>
+      </x:c>
+      <x:c r="C28" s="93" t="n">
+        <x:v>-141.1</x:v>
+      </x:c>
+      <x:c r="D28" s="93" t="n">
+        <x:v>-160.5</x:v>
+      </x:c>
+      <x:c r="E28" s="93" t="n">
+        <x:v>-225</x:v>
+      </x:c>
+      <x:c r="F28" s="93" t="n">
+        <x:v>-186</x:v>
+      </x:c>
+      <x:c r="G28" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H28" s="56" t="str">
+        <x:v>Presented as a cash outflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="99" t="str">
+        <x:v>Free cash flow</x:v>
+      </x:c>
+      <x:c r="B29" s="100" t="n">
+        <x:f>SUM(B27:B28)</x:f>
+        <x:v>1140.7</x:v>
+      </x:c>
+      <x:c r="C29" s="100" t="n">
+        <x:f>SUM(C27:C28)</x:f>
+        <x:v>682</x:v>
+      </x:c>
+      <x:c r="D29" s="100" t="n">
+        <x:f>SUM(D27:D28)</x:f>
+        <x:v>1213.5</x:v>
+      </x:c>
+      <x:c r="E29" s="100" t="n">
+        <x:f>SUM(E27:E28)</x:f>
+        <x:v>639</x:v>
+      </x:c>
+      <x:c r="F29" s="100" t="n">
+        <x:f>SUM(F27:F28)</x:f>
+        <x:v>1358</x:v>
+      </x:c>
+      <x:c r="G29" s="54"/>
+      <x:c r="H29" s="56"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="52" t="str">
+        <x:v>Free cash flow margin</x:v>
+      </x:c>
+      <x:c r="B30" s="94" t="n">
+        <x:f>B29/B7</x:f>
+        <x:v>0.16301769228570615</x:v>
+      </x:c>
+      <x:c r="C30" s="94" t="n">
+        <x:f>C29/C7</x:f>
+        <x:v>0.08788206793464255</x:v>
+      </x:c>
+      <x:c r="D30" s="94" t="n">
+        <x:f>D29/D7</x:f>
+        <x:v>0.13396997129609184</x:v>
+      </x:c>
+      <x:c r="E30" s="94" t="n">
+        <x:f>E29/E7</x:f>
+        <x:v>0.07732333010648597</x:v>
+      </x:c>
+      <x:c r="F30" s="94" t="n">
+        <x:f>F29/F7</x:f>
+        <x:v>0.16279069767441862</x:v>
+      </x:c>
+      <x:c r="G30" s="54"/>
+      <x:c r="H30" s="56"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="52" t="str">
+        <x:v>Free cash flow / net income</x:v>
+      </x:c>
+      <x:c r="B31" s="94" t="n">
+        <x:f>B29/B24</x:f>
+        <x:v>0.8399234224283927</x:v>
+      </x:c>
+      <x:c r="C31" s="94" t="n">
+        <x:f>C29/C24</x:f>
+        <x:v>0.7316026603733105</x:v>
+      </x:c>
+      <x:c r="D31" s="94" t="n">
+        <x:f>D29/D24</x:f>
+        <x:v>0.8749098774333093</x:v>
+      </x:c>
+      <x:c r="E31" s="94" t="n">
+        <x:f>E29/E24</x:f>
+        <x:v>0.670514165792235</x:v>
+      </x:c>
+      <x:c r="F31" s="94" t="n">
+        <x:f>F29/F24</x:f>
+        <x:v>1.5627157652474108</x:v>
+      </x:c>
+      <x:c r="G31" s="54"/>
+      <x:c r="H31" s="56"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="52"/>
+      <x:c r="B32" s="53"/>
+      <x:c r="C32" s="53"/>
+      <x:c r="D32" s="53"/>
+      <x:c r="E32" s="53"/>
+      <x:c r="F32" s="53"/>
+      <x:c r="G32" s="54"/>
+      <x:c r="H32" s="56"/>
+    </x:row>
+    <x:row r="33" ht="19" customHeight="1">
+      <x:c r="A33" s="76" t="str">
+        <x:v>BALANCE SHEET, LIQUIDITY AND LEVERAGE</x:v>
+      </x:c>
+      <x:c r="B33" s="77"/>
+      <x:c r="C33" s="77"/>
+      <x:c r="D33" s="77"/>
+      <x:c r="E33" s="77"/>
+      <x:c r="F33" s="77"/>
+      <x:c r="G33" s="78"/>
+      <x:c r="H33" s="79"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B34" s="92" t="n">
+        <x:v>44469.5</x:v>
+      </x:c>
+      <x:c r="C34" s="92" t="n">
+        <x:v>44834.5</x:v>
+      </x:c>
+      <x:c r="D34" s="92" t="n">
+        <x:v>45199.5</x:v>
+      </x:c>
+      <x:c r="E34" s="92" t="n">
+        <x:v>45565.5</x:v>
+      </x:c>
+      <x:c r="F34" s="92" t="n">
+        <x:v>45930.5</x:v>
+      </x:c>
+      <x:c r="G34" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H34" s="91" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="52" t="str">
+        <x:v>Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="B35" s="93" t="n">
+        <x:v>662.2</x:v>
+      </x:c>
+      <x:c r="C35" s="93" t="n">
+        <x:v>490.7</x:v>
+      </x:c>
+      <x:c r="D35" s="93" t="n">
+        <x:v>1072</x:v>
+      </x:c>
+      <x:c r="E35" s="93" t="n">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="F35" s="93" t="n">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="G35" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H35" s="56" t="str"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="52" t="str">
+        <x:v>Short-term investments</x:v>
+      </x:c>
+      <x:c r="B36" s="93" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="C36" s="93" t="n">
+        <x:v>12.6</x:v>
+      </x:c>
+      <x:c r="D36" s="93" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="E36" s="93" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="F36" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G36" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H36" s="56" t="str"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="52" t="str">
+        <x:v>Receivables</x:v>
+      </x:c>
+      <x:c r="B37" s="93" t="n">
+        <x:v>1424.5</x:v>
+      </x:c>
+      <x:c r="C37" s="93" t="n">
+        <x:v>1736.7</x:v>
+      </x:c>
+      <x:c r="D37" s="93" t="n">
+        <x:v>2167.4</x:v>
+      </x:c>
+      <x:c r="E37" s="93" t="n">
+        <x:v>1802</x:v>
+      </x:c>
+      <x:c r="F37" s="93" t="n">
+        <x:v>1931</x:v>
+      </x:c>
+      <x:c r="G37" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H37" s="56" t="str"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="52" t="str">
+        <x:v>Inventory</x:v>
+      </x:c>
+      <x:c r="B38" s="93" t="n">
+        <x:v>798.1</x:v>
+      </x:c>
+      <x:c r="C38" s="93" t="n">
+        <x:v>1054.2</x:v>
+      </x:c>
+      <x:c r="D38" s="93" t="n">
+        <x:v>1404.9</x:v>
+      </x:c>
+      <x:c r="E38" s="93" t="n">
+        <x:v>1293</x:v>
+      </x:c>
+      <x:c r="F38" s="93" t="n">
+        <x:v>1247</x:v>
+      </x:c>
+      <x:c r="G38" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H38" s="56" t="str"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="99" t="str">
+        <x:v>Current assets</x:v>
+      </x:c>
+      <x:c r="B39" s="100" t="n">
+        <x:v>3063.4</x:v>
+      </x:c>
+      <x:c r="C39" s="100" t="n">
+        <x:v>3610.7</x:v>
+      </x:c>
+      <x:c r="D39" s="100" t="n">
+        <x:v>4910.8</x:v>
+      </x:c>
+      <x:c r="E39" s="100" t="n">
+        <x:v>3881</x:v>
+      </x:c>
+      <x:c r="F39" s="100" t="n">
+        <x:v>3911</x:v>
+      </x:c>
+      <x:c r="G39" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H39" s="56" t="str"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="52" t="str">
+        <x:v>Accounts payable</x:v>
+      </x:c>
+      <x:c r="B40" s="93" t="n">
+        <x:v>889.8</x:v>
+      </x:c>
+      <x:c r="C40" s="93" t="n">
+        <x:v>1028</x:v>
+      </x:c>
+      <x:c r="D40" s="93" t="n">
+        <x:v>1150.2</x:v>
+      </x:c>
+      <x:c r="E40" s="93" t="n">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="F40" s="93" t="n">
+        <x:v>930</x:v>
+      </x:c>
+      <x:c r="G40" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H40" s="56" t="str"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="52" t="str">
+        <x:v>Current liabilities</x:v>
+      </x:c>
+      <x:c r="B41" s="93" t="n">
+        <x:v>2992.2</x:v>
+      </x:c>
+      <x:c r="C41" s="93" t="n">
+        <x:v>3572.2</x:v>
+      </x:c>
+      <x:c r="D41" s="93" t="n">
+        <x:v>3365.3</x:v>
+      </x:c>
+      <x:c r="E41" s="93" t="n">
+        <x:v>3604</x:v>
+      </x:c>
+      <x:c r="F41" s="93" t="n">
+        <x:v>3445</x:v>
+      </x:c>
+      <x:c r="G41" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H41" s="56" t="str"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="99" t="str">
+        <x:v>Total assets</x:v>
+      </x:c>
+      <x:c r="B42" s="100" t="n">
+        <x:v>10701.6</x:v>
+      </x:c>
+      <x:c r="C42" s="100" t="n">
+        <x:v>10758.7</x:v>
+      </x:c>
+      <x:c r="D42" s="100" t="n">
+        <x:v>11304</x:v>
+      </x:c>
+      <x:c r="E42" s="100" t="n">
+        <x:v>11232</x:v>
+      </x:c>
+      <x:c r="F42" s="100" t="n">
+        <x:v>11219</x:v>
+      </x:c>
+      <x:c r="G42" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H42" s="56" t="str"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="52" t="str">
+        <x:v>Total equity including noncontrolling interests</x:v>
+      </x:c>
+      <x:c r="B43" s="93" t="n">
+        <x:v>2694.1</x:v>
+      </x:c>
+      <x:c r="C43" s="93" t="n">
+        <x:v>3016</x:v>
+      </x:c>
+      <x:c r="D43" s="93" t="n">
+        <x:v>3743</x:v>
+      </x:c>
+      <x:c r="E43" s="93" t="n">
+        <x:v>3675</x:v>
+      </x:c>
+      <x:c r="F43" s="93" t="n">
+        <x:v>3711</x:v>
+      </x:c>
+      <x:c r="G43" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H43" s="56" t="str"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="99" t="str">
+        <x:v>Total liabilities</x:v>
+      </x:c>
+      <x:c r="B44" s="100" t="n">
+        <x:f>B42-B43</x:f>
+        <x:v>8007.5</x:v>
+      </x:c>
+      <x:c r="C44" s="100" t="n">
+        <x:f>C42-C43</x:f>
+        <x:v>7742.700000000001</x:v>
+      </x:c>
+      <x:c r="D44" s="100" t="n">
+        <x:f>D42-D43</x:f>
+        <x:v>7561</x:v>
+      </x:c>
+      <x:c r="E44" s="100" t="n">
+        <x:f>E42-E43</x:f>
+        <x:v>7557</x:v>
+      </x:c>
+      <x:c r="F44" s="100" t="n">
+        <x:f>F42-F43</x:f>
+        <x:v>7508</x:v>
+      </x:c>
+      <x:c r="G44" s="54"/>
+      <x:c r="H44" s="56"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="52" t="str">
+        <x:v>Total debt and finance leases</x:v>
+      </x:c>
+      <x:c r="B45" s="93" t="n">
+        <x:v>3471.4</x:v>
+      </x:c>
+      <x:c r="C45" s="93" t="n">
+        <x:v>3476.9</x:v>
+      </x:c>
+      <x:c r="D45" s="93" t="n">
+        <x:v>2871.5</x:v>
+      </x:c>
+      <x:c r="E45" s="93" t="n">
+        <x:v>2868</x:v>
+      </x:c>
+      <x:c r="F45" s="93" t="n">
+        <x:v>2616</x:v>
+      </x:c>
+      <x:c r="G45" s="54" t="str">
+        <x:v>S-026 / S-017</x:v>
+      </x:c>
+      <x:c r="H45" s="56" t="str"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="99" t="str">
+        <x:v>Net debt</x:v>
+      </x:c>
+      <x:c r="B46" s="100" t="n">
+        <x:f>B45-B35-B36</x:f>
+        <x:v>2808.6</x:v>
+      </x:c>
+      <x:c r="C46" s="100" t="n">
+        <x:f>C45-C35-C36</x:f>
+        <x:v>2973.6000000000004</x:v>
+      </x:c>
+      <x:c r="D46" s="100" t="n">
+        <x:f>D45-D35-D36</x:f>
+        <x:v>1798.9</x:v>
+      </x:c>
+      <x:c r="E46" s="100" t="n">
+        <x:f>E45-E35-E36</x:f>
+        <x:v>2396.7</x:v>
+      </x:c>
+      <x:c r="F46" s="100" t="n">
+        <x:f>F45-F35-F36</x:f>
+        <x:v>2148</x:v>
+      </x:c>
+      <x:c r="G46" s="54"/>
+      <x:c r="H46" s="56"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="99" t="str">
+        <x:v>Balance sheet check</x:v>
+      </x:c>
+      <x:c r="B47" s="100" t="n">
+        <x:f>B42-B43-B44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C47" s="100" t="n">
+        <x:f>C42-C43-C44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D47" s="100" t="n">
+        <x:f>D42-D43-D44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E47" s="100" t="n">
+        <x:f>E42-E43-E44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F47" s="100" t="n">
+        <x:f>F42-F43-F44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G47" s="54"/>
+      <x:c r="H47" s="56"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="52" t="str">
+        <x:v>Net working capital</x:v>
+      </x:c>
+      <x:c r="B48" s="93" t="n">
+        <x:f>B39-B41</x:f>
+        <x:v>71.20000000000027</x:v>
+      </x:c>
+      <x:c r="C48" s="93" t="n">
+        <x:f>C39-C41</x:f>
+        <x:v>38.5</x:v>
+      </x:c>
+      <x:c r="D48" s="93" t="n">
+        <x:f>D39-D41</x:f>
+        <x:v>1545.5</x:v>
+      </x:c>
+      <x:c r="E48" s="93" t="n">
+        <x:f>E39-E41</x:f>
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="F48" s="93" t="n">
+        <x:f>F39-F41</x:f>
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="G48" s="54"/>
+      <x:c r="H48" s="56"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="52" t="str">
+        <x:v>Indicative net leverage</x:v>
+      </x:c>
+      <x:c r="B49" s="110" t="n">
+        <x:f>B46/(B9+B25)</x:f>
+        <x:v>1.776358231610904</x:v>
+      </x:c>
+      <x:c r="C49" s="110" t="n">
+        <x:f>C46/(C9+C25)</x:f>
+        <x:v>1.6691552062868371</x:v>
+      </x:c>
+      <x:c r="D49" s="110" t="n">
+        <x:f>D46/(D9+D25)</x:f>
+        <x:v>0.8255621844882974</x:v>
+      </x:c>
+      <x:c r="E49" s="110" t="n">
+        <x:f>E46/(E9+E25)</x:f>
+        <x:v>1.2535041841004184</x:v>
+      </x:c>
+      <x:c r="F49" s="110" t="n">
+        <x:f>F46/(F9+F25)</x:f>
+        <x:v>1.0591715976331362</x:v>
+      </x:c>
+      <x:c r="G49" s="54"/>
+      <x:c r="H49" s="56"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="52"/>
+      <x:c r="B50" s="53"/>
+      <x:c r="C50" s="53"/>
+      <x:c r="D50" s="53"/>
+      <x:c r="E50" s="53"/>
+      <x:c r="F50" s="53"/>
+      <x:c r="G50" s="54"/>
+      <x:c r="H50" s="56"/>
+    </x:row>
+    <x:row r="51" ht="19" customHeight="1">
+      <x:c r="A51" s="76" t="str">
+        <x:v>KEY PERFORMANCE INDICATORS</x:v>
+      </x:c>
+      <x:c r="B51" s="77"/>
+      <x:c r="C51" s="77"/>
+      <x:c r="D51" s="77"/>
+      <x:c r="E51" s="77"/>
+      <x:c r="F51" s="77"/>
+      <x:c r="G51" s="78"/>
+      <x:c r="H51" s="79"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B52" s="92" t="n">
+        <x:v>44469.5</x:v>
+      </x:c>
+      <x:c r="C52" s="92" t="n">
+        <x:v>44834.5</x:v>
+      </x:c>
+      <x:c r="D52" s="92" t="n">
+        <x:v>45199.5</x:v>
+      </x:c>
+      <x:c r="E52" s="92" t="n">
+        <x:v>45565.5</x:v>
+      </x:c>
+      <x:c r="F52" s="92" t="n">
+        <x:v>45930.5</x:v>
+      </x:c>
+      <x:c r="G52" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H52" s="91" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="52" t="str">
+        <x:v>Days sales outstanding</x:v>
+      </x:c>
+      <x:c r="B53" s="103" t="n">
+        <x:f>B37/B7*365</x:f>
+        <x:v>74.3050990367851</x:v>
+      </x:c>
+      <x:c r="C53" s="103" t="n">
+        <x:f>C37/C7*365</x:f>
+        <x:v>81.68335395082728</x:v>
+      </x:c>
+      <x:c r="D53" s="103" t="n">
+        <x:f>D37/D7*365</x:f>
+        <x:v>87.33727092073306</x:v>
+      </x:c>
+      <x:c r="E53" s="103" t="n">
+        <x:f>E37/E7*365</x:f>
+        <x:v>79.58978702807357</x:v>
+      </x:c>
+      <x:c r="F53" s="103" t="n">
+        <x:f>F37/F7*365</x:f>
+        <x:v>84.4899304723088</x:v>
+      </x:c>
+      <x:c r="G53" s="54"/>
+      <x:c r="H53" s="56"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="52" t="str">
+        <x:v>Revenue CAGR since FY2021</x:v>
+      </x:c>
+      <x:c r="B54" s="94"/>
+      <x:c r="C54" s="94" t="n">
+        <x:f>(C7/$B$7)^(1/1)-1</x:f>
+        <x:v>0.10904050075742422</x:v>
+      </x:c>
+      <x:c r="D54" s="94" t="n">
+        <x:f>(D7/$B$7)^(1/2)-1</x:f>
+        <x:v>0.1377525245662803</x:v>
+      </x:c>
+      <x:c r="E54" s="94" t="n">
+        <x:f>(E7/$B$7)^(1/3)-1</x:f>
+        <x:v>0.05702324004441017</x:v>
+      </x:c>
+      <x:c r="F54" s="94" t="n">
+        <x:f>(F7/$B$7)^(1/4)-1</x:f>
+        <x:v>0.04492079268656135</x:v>
+      </x:c>
+      <x:c r="G54" s="54"/>
+      <x:c r="H54" s="56"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="52" t="str">
+        <x:v>Total segment operating margin</x:v>
+      </x:c>
+      <x:c r="B55" s="94" t="n">
+        <x:f>B10</x:f>
+        <x:v>0.19883099436933718</x:v>
+      </x:c>
+      <x:c r="C55" s="94" t="n">
+        <x:f>C10</x:f>
+        <x:v>0.19877841348384104</x:v>
+      </x:c>
+      <x:c r="D55" s="94" t="n">
+        <x:f>D10</x:f>
+        <x:v>0.21296091852506072</x:v>
+      </x:c>
+      <x:c r="E55" s="94" t="n">
+        <x:f>E10</x:f>
+        <x:v>0.1930058083252662</x:v>
+      </x:c>
+      <x:c r="F55" s="94" t="n">
+        <x:f>F10</x:f>
+        <x:v>0.20414768640613762</x:v>
+      </x:c>
+      <x:c r="G55" s="54"/>
+      <x:c r="H55" s="56"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="52" t="str">
+        <x:v>Free cash flow margin</x:v>
+      </x:c>
+      <x:c r="B56" s="94" t="n">
+        <x:f>B30</x:f>
+        <x:v>0.16301769228570615</x:v>
+      </x:c>
+      <x:c r="C56" s="94" t="n">
+        <x:f>C30</x:f>
+        <x:v>0.08788206793464255</x:v>
+      </x:c>
+      <x:c r="D56" s="94" t="n">
+        <x:f>D30</x:f>
+        <x:v>0.13396997129609184</x:v>
+      </x:c>
+      <x:c r="E56" s="94" t="n">
+        <x:f>E30</x:f>
+        <x:v>0.07732333010648597</x:v>
+      </x:c>
+      <x:c r="F56" s="94" t="n">
+        <x:f>F30</x:f>
+        <x:v>0.16279069767441862</x:v>
+      </x:c>
+      <x:c r="G56" s="54"/>
+      <x:c r="H56" s="56"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="52" t="str">
+        <x:v>Net debt</x:v>
+      </x:c>
+      <x:c r="B57" s="93" t="n">
+        <x:f>B46</x:f>
+        <x:v>2808.6</x:v>
+      </x:c>
+      <x:c r="C57" s="93" t="n">
+        <x:f>C46</x:f>
+        <x:v>2973.6000000000004</x:v>
+      </x:c>
+      <x:c r="D57" s="93" t="n">
+        <x:f>D46</x:f>
+        <x:v>1798.9</x:v>
+      </x:c>
+      <x:c r="E57" s="93" t="n">
+        <x:f>E46</x:f>
+        <x:v>2396.7</x:v>
+      </x:c>
+      <x:c r="F57" s="93" t="n">
+        <x:f>F46</x:f>
+        <x:v>2148</x:v>
+      </x:c>
+      <x:c r="G57" s="54"/>
+      <x:c r="H57" s="56"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="52"/>
+      <x:c r="B58" s="53"/>
+      <x:c r="C58" s="53"/>
+      <x:c r="D58" s="53"/>
+      <x:c r="E58" s="53"/>
+      <x:c r="F58" s="53"/>
+      <x:c r="G58" s="54"/>
+      <x:c r="H58" s="56"/>
+    </x:row>
+    <x:row r="59" ht="19" customHeight="1">
+      <x:c r="A59" s="76" t="str">
+        <x:v>ANALYST TAKEAWAYS</x:v>
+      </x:c>
+      <x:c r="B59" s="77"/>
+      <x:c r="C59" s="77"/>
+      <x:c r="D59" s="77"/>
+      <x:c r="E59" s="77"/>
+      <x:c r="F59" s="77"/>
+      <x:c r="G59" s="78"/>
+      <x:c r="H59" s="79"/>
+    </x:row>
+    <x:row r="60" ht="28" customHeight="1">
+      <x:c r="A60" s="107" t="str">
+        <x:v>• Rockwell's revenue grew over the five-year period but remained cyclical, peaking in FY2023, declining in FY2024, and returning to modest growth in FY2025.</x:v>
+      </x:c>
+      <x:c r="B60" s="108"/>
+      <x:c r="C60" s="108"/>
+      <x:c r="D60" s="108"/>
+      <x:c r="E60" s="108"/>
+      <x:c r="F60" s="108"/>
+      <x:c r="G60" s="109"/>
+      <x:c r="H60" s="107"/>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="107" t="str">
+        <x:v>• Total segment operating margin remained near 20% across the cycle, supporting the buyer's earnings base and financing capacity.</x:v>
+      </x:c>
+      <x:c r="B61" s="108"/>
+      <x:c r="C61" s="108"/>
+      <x:c r="D61" s="108"/>
+      <x:c r="E61" s="108"/>
+      <x:c r="F61" s="108"/>
+      <x:c r="G61" s="109"/>
+      <x:c r="H61" s="107"/>
+    </x:row>
+    <x:row r="62" ht="28" customHeight="1">
+      <x:c r="A62" s="107" t="str">
+        <x:v>• Free cash flow was volatile but recovered strongly in FY2025, which is important for debt capacity and post-close deleveraging.</x:v>
+      </x:c>
+      <x:c r="B62" s="108"/>
+      <x:c r="C62" s="108"/>
+      <x:c r="D62" s="108"/>
+      <x:c r="E62" s="108"/>
+      <x:c r="F62" s="108"/>
+      <x:c r="G62" s="109"/>
+      <x:c r="H62" s="107"/>
+    </x:row>
+    <x:row r="63" ht="28" customHeight="1">
+      <x:c r="A63" s="107" t="str">
+        <x:v>• Reported EPS is affected by non-operating items, including fair-value changes in Rockwell's PTC investment; later accretion/dilution work will distinguish reported and normalized earnings.</x:v>
+      </x:c>
+      <x:c r="B63" s="108"/>
+      <x:c r="C63" s="108"/>
+      <x:c r="D63" s="108"/>
+      <x:c r="E63" s="108"/>
+      <x:c r="F63" s="108"/>
+      <x:c r="G63" s="109"/>
+      <x:c r="H63" s="107"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="B3:F3"/>
     <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A22:H22"/>
+    <x:mergeCell ref="A33:H33"/>
+    <x:mergeCell ref="A51:H51"/>
+    <x:mergeCell ref="A59:H59"/>
+    <x:mergeCell ref="A60:H60"/>
+    <x:mergeCell ref="A61:H61"/>
+    <x:mergeCell ref="A62:H62"/>
+    <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaeefc80b35a43fe"/>
 </x:worksheet>
 </file>
 
@@ -2281,112 +4198,1722 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" s="61" t="str">
         <x:v>CGNX Historical</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Cognex historical financial statements and operating KPIs</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
+      <x:c r="B1" s="62"/>
+      <x:c r="C1" s="62"/>
+      <x:c r="D1" s="62"/>
+      <x:c r="E1" s="62"/>
+      <x:c r="F1" s="62"/>
+      <x:c r="G1" s="63"/>
+      <x:c r="H1" s="64"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="69" t="str">
+        <x:v>Cognex historical financial statements and operating KPIs | USD millions, except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="70"/>
+      <x:c r="C2" s="70"/>
+      <x:c r="D2" s="70"/>
+      <x:c r="E2" s="70"/>
+      <x:c r="F2" s="70"/>
+      <x:c r="G2" s="71"/>
+      <x:c r="H2" s="72"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="A3" s="73" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
+      <x:c r="B3" s="75" t="str">
+        <x:v>Complete — FY2021 to FY2025 audited history loaded</x:v>
+      </x:c>
+      <x:c r="C3" s="75"/>
+      <x:c r="D3" s="75"/>
+      <x:c r="E3" s="75"/>
+      <x:c r="F3" s="75"/>
+      <x:c r="G3" s="54"/>
+      <x:c r="H3" s="56"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="52"/>
+      <x:c r="B4" s="53"/>
+      <x:c r="C4" s="53"/>
+      <x:c r="D4" s="53"/>
+      <x:c r="E4" s="53"/>
+      <x:c r="F4" s="53"/>
+      <x:c r="G4" s="54"/>
+      <x:c r="H4" s="56"/>
+    </x:row>
+    <x:row r="5" ht="19" customHeight="1">
+      <x:c r="A5" s="76" t="str">
+        <x:v>INCOME STATEMENT AND PROFITABILITY</x:v>
+      </x:c>
+      <x:c r="B5" s="77"/>
+      <x:c r="C5" s="77"/>
+      <x:c r="D5" s="77"/>
+      <x:c r="E5" s="77"/>
+      <x:c r="F5" s="77"/>
+      <x:c r="G5" s="78"/>
+      <x:c r="H5" s="79"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
+      <x:c r="A6" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B6" s="92" t="n">
+        <x:v>44561.5</x:v>
+      </x:c>
+      <x:c r="C6" s="92" t="n">
+        <x:v>44926.5</x:v>
+      </x:c>
+      <x:c r="D6" s="92" t="n">
+        <x:v>45291.5</x:v>
+      </x:c>
+      <x:c r="E6" s="92" t="n">
+        <x:v>45657.5</x:v>
+      </x:c>
+      <x:c r="F6" s="92" t="n">
+        <x:v>46022.5</x:v>
+      </x:c>
+      <x:c r="G6" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H6" s="91" t="str">
+        <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
+      <x:c r="A7" s="52" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B7" s="93" t="n">
+        <x:v>1037.098</x:v>
+      </x:c>
+      <x:c r="C7" s="93" t="n">
+        <x:v>1006.09</x:v>
+      </x:c>
+      <x:c r="D7" s="93" t="n">
+        <x:v>837.547</x:v>
+      </x:c>
+      <x:c r="E7" s="93" t="n">
+        <x:v>914.515</x:v>
+      </x:c>
+      <x:c r="F7" s="93" t="n">
+        <x:v>994.359</x:v>
+      </x:c>
+      <x:c r="G7" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H7" s="56" t="str">
+        <x:v>Revenue from contracts with customers</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
+      <x:c r="A8" s="52" t="str">
+        <x:v>% growth</x:v>
+      </x:c>
+      <x:c r="B8" s="94"/>
+      <x:c r="C8" s="94" t="n">
+        <x:f>C7/B7-1</x:f>
+        <x:v>-0.029898813805445457</x:v>
+      </x:c>
+      <x:c r="D8" s="94" t="n">
+        <x:f>D7/C7-1</x:f>
+        <x:v>-0.16752278623184802</x:v>
+      </x:c>
+      <x:c r="E8" s="94" t="n">
+        <x:f>E7/D7-1</x:f>
+        <x:v>0.09189693235125906</x:v>
+      </x:c>
+      <x:c r="F8" s="94" t="n">
+        <x:f>F7/E7-1</x:f>
+        <x:v>0.08730747992105115</x:v>
+      </x:c>
+      <x:c r="G8" s="54"/>
+      <x:c r="H8" s="56"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
+      <x:c r="A9" s="52" t="str">
+        <x:v>Cost of goods sold</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="n">
+        <x:v>277.271</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="n">
+        <x:v>284.185</x:v>
+      </x:c>
+      <x:c r="D9" s="93" t="n">
+        <x:v>236.306</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="n">
+        <x:v>288.721</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="n">
+        <x:v>328.966</x:v>
+      </x:c>
+      <x:c r="G9" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H9" s="56" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="99" t="str">
+        <x:v>Gross profit — calculated</x:v>
+      </x:c>
+      <x:c r="B10" s="100" t="n">
+        <x:f>B7-B9</x:f>
+        <x:v>759.827</x:v>
+      </x:c>
+      <x:c r="C10" s="100" t="n">
+        <x:f>C7-C9</x:f>
+        <x:v>721.905</x:v>
+      </x:c>
+      <x:c r="D10" s="100" t="n">
+        <x:f>D7-D9</x:f>
+        <x:v>601.241</x:v>
+      </x:c>
+      <x:c r="E10" s="100" t="n">
+        <x:f>E7-E9</x:f>
+        <x:v>625.794</x:v>
+      </x:c>
+      <x:c r="F10" s="100" t="n">
+        <x:f>F7-F9</x:f>
+        <x:v>665.393</x:v>
+      </x:c>
+      <x:c r="G10" s="54"/>
+      <x:c r="H10" s="56"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="A11" s="52" t="str">
+        <x:v>Gross profit — reported</x:v>
+      </x:c>
+      <x:c r="B11" s="93" t="n">
+        <x:v>759.827</x:v>
+      </x:c>
+      <x:c r="C11" s="93" t="n">
+        <x:v>721.905</x:v>
+      </x:c>
+      <x:c r="D11" s="93" t="n">
+        <x:v>601.241</x:v>
+      </x:c>
+      <x:c r="E11" s="93" t="n">
+        <x:v>625.794</x:v>
+      </x:c>
+      <x:c r="F11" s="93" t="n">
+        <x:v>665.393</x:v>
+      </x:c>
+      <x:c r="G11" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H11" s="56" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="52" t="str">
+        <x:v>Gross profit tie-out</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="n">
+        <x:f>B10-B11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="n">
+        <x:f>C10-C11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="n">
+        <x:f>D10-D11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="n">
+        <x:f>E10-E11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="93" t="n">
+        <x:f>F10-F11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="54"/>
+      <x:c r="H12" s="56"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="52" t="str">
+        <x:v>Gross margin</x:v>
+      </x:c>
+      <x:c r="B13" s="94" t="n">
+        <x:f>B10/B7</x:f>
+        <x:v>0.7326472522365293</x:v>
+      </x:c>
+      <x:c r="C13" s="94" t="n">
+        <x:f>C10/C7</x:f>
+        <x:v>0.717535210567643</x:v>
+      </x:c>
+      <x:c r="D13" s="94" t="n">
+        <x:f>D10/D7</x:f>
+        <x:v>0.7178594156507038</x:v>
+      </x:c>
+      <x:c r="E13" s="94" t="n">
+        <x:f>E10/E7</x:f>
+        <x:v>0.6842905802529209</x:v>
+      </x:c>
+      <x:c r="F13" s="94" t="n">
+        <x:f>F10/F7</x:f>
+        <x:v>0.6691677754211507</x:v>
+      </x:c>
+      <x:c r="G13" s="54"/>
+      <x:c r="H13" s="56"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="52"/>
+      <x:c r="B14" s="53"/>
+      <x:c r="C14" s="53"/>
+      <x:c r="D14" s="53"/>
+      <x:c r="E14" s="53"/>
+      <x:c r="F14" s="53"/>
+      <x:c r="G14" s="54"/>
+      <x:c r="H14" s="56"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="52" t="str">
+        <x:v>Research, development &amp; engineering</x:v>
+      </x:c>
+      <x:c r="B15" s="93" t="n">
+        <x:v>135.372</x:v>
+      </x:c>
+      <x:c r="C15" s="93" t="n">
+        <x:v>141.133</x:v>
+      </x:c>
+      <x:c r="D15" s="93" t="n">
+        <x:v>139.4</x:v>
+      </x:c>
+      <x:c r="E15" s="93" t="n">
+        <x:v>139.815</x:v>
+      </x:c>
+      <x:c r="F15" s="93" t="n">
+        <x:v>138.97</x:v>
+      </x:c>
+      <x:c r="G15" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H15" s="56" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="52" t="str">
+        <x:v>% of revenue</x:v>
+      </x:c>
+      <x:c r="B16" s="94" t="n">
+        <x:f>B15/B7</x:f>
+        <x:v>0.13052961243778313</x:v>
+      </x:c>
+      <x:c r="C16" s="94" t="n">
+        <x:f>C15/C7</x:f>
+        <x:v>0.14027870270055362</x:v>
+      </x:c>
+      <x:c r="D16" s="94" t="n">
+        <x:f>D15/D7</x:f>
+        <x:v>0.1664384207692225</x:v>
+      </x:c>
+      <x:c r="E16" s="94" t="n">
+        <x:f>E15/E7</x:f>
+        <x:v>0.15288431573019579</x:v>
+      </x:c>
+      <x:c r="F16" s="94" t="n">
+        <x:f>F15/F7</x:f>
+        <x:v>0.1397583770046834</x:v>
+      </x:c>
+      <x:c r="G16" s="54"/>
+      <x:c r="H16" s="56"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="52" t="str">
+        <x:v>Selling, general &amp; administrative</x:v>
+      </x:c>
+      <x:c r="B17" s="93" t="n">
+        <x:v>309.354</x:v>
+      </x:c>
+      <x:c r="C17" s="93" t="n">
+        <x:v>312.107</x:v>
+      </x:c>
+      <x:c r="D17" s="93" t="n">
+        <x:v>339.139</x:v>
+      </x:c>
+      <x:c r="E17" s="93" t="n">
+        <x:v>370.914</x:v>
+      </x:c>
+      <x:c r="F17" s="93" t="n">
+        <x:v>363.857</x:v>
+      </x:c>
+      <x:c r="G17" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H17" s="56" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="52" t="str">
+        <x:v>% of revenue</x:v>
+      </x:c>
+      <x:c r="B18" s="94" t="n">
+        <x:f>B17/B7</x:f>
+        <x:v>0.29828810777766424</x:v>
+      </x:c>
+      <x:c r="C18" s="94" t="n">
+        <x:f>C17/C7</x:f>
+        <x:v>0.31021777375781495</x:v>
+      </x:c>
+      <x:c r="D18" s="94" t="n">
+        <x:f>D17/D7</x:f>
+        <x:v>0.4049193657191775</x:v>
+      </x:c>
+      <x:c r="E18" s="94" t="n">
+        <x:f>E17/E7</x:f>
+        <x:v>0.4055854742677813</x:v>
+      </x:c>
+      <x:c r="F18" s="94" t="n">
+        <x:f>F17/F7</x:f>
+        <x:v>0.3659211612707282</x:v>
+      </x:c>
+      <x:c r="G18" s="54"/>
+      <x:c r="H18" s="56"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="99" t="str">
+        <x:v>Operating income</x:v>
+      </x:c>
+      <x:c r="B19" s="100" t="n">
+        <x:v>315.101</x:v>
+      </x:c>
+      <x:c r="C19" s="100" t="n">
+        <x:v>246.229</x:v>
+      </x:c>
+      <x:c r="D19" s="100" t="n">
+        <x:v>130.702</x:v>
+      </x:c>
+      <x:c r="E19" s="100" t="n">
+        <x:v>115.065</x:v>
+      </x:c>
+      <x:c r="F19" s="100" t="n">
+        <x:v>162.566</x:v>
+      </x:c>
+      <x:c r="G19" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H19" s="56" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="52" t="str">
+        <x:v>Operating margin</x:v>
+      </x:c>
+      <x:c r="B20" s="94" t="n">
+        <x:f>B19/B7</x:f>
+        <x:v>0.3038295320210819</x:v>
+      </x:c>
+      <x:c r="C20" s="94" t="n">
+        <x:f>C19/C7</x:f>
+        <x:v>0.24473854227752984</x:v>
+      </x:c>
+      <x:c r="D20" s="94" t="n">
+        <x:f>D19/D7</x:f>
+        <x:v>0.1560533319324169</x:v>
+      </x:c>
+      <x:c r="E20" s="94" t="n">
+        <x:f>E19/E7</x:f>
+        <x:v>0.1258207902549439</x:v>
+      </x:c>
+      <x:c r="F20" s="94" t="n">
+        <x:f>F19/F7</x:f>
+        <x:v>0.16348823714573912</x:v>
+      </x:c>
+      <x:c r="G20" s="54"/>
+      <x:c r="H20" s="56"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="52" t="str">
+        <x:v>Net interest and other income</x:v>
+      </x:c>
+      <x:c r="B21" s="93" t="n">
+        <x:f>B22-B19</x:f>
+        <x:v>3.798999999999978</x:v>
+      </x:c>
+      <x:c r="C21" s="93" t="n">
+        <x:f>C22-C19</x:f>
+        <x:v>4.46599999999998</x:v>
+      </x:c>
+      <x:c r="D21" s="93" t="n">
+        <x:f>D22-D19</x:f>
+        <x:v>4.646000000000015</x:v>
+      </x:c>
+      <x:c r="E21" s="93" t="n">
+        <x:f>E22-E19</x:f>
+        <x:v>16.424000000000007</x:v>
+      </x:c>
+      <x:c r="F21" s="93" t="n">
+        <x:f>F22-F19</x:f>
+        <x:v>20.23599999999999</x:v>
+      </x:c>
+      <x:c r="G21" s="54"/>
+      <x:c r="H21" s="56"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="99" t="str">
+        <x:v>Income before income taxes</x:v>
+      </x:c>
+      <x:c r="B22" s="100" t="n">
+        <x:v>318.9</x:v>
+      </x:c>
+      <x:c r="C22" s="100" t="n">
+        <x:v>250.695</x:v>
+      </x:c>
+      <x:c r="D22" s="100" t="n">
+        <x:v>135.348</x:v>
+      </x:c>
+      <x:c r="E22" s="100" t="n">
+        <x:v>131.489</x:v>
+      </x:c>
+      <x:c r="F22" s="100" t="n">
+        <x:v>182.802</x:v>
+      </x:c>
+      <x:c r="G22" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H22" s="56" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="52" t="str">
+        <x:v>Income tax expense</x:v>
+      </x:c>
+      <x:c r="B23" s="93" t="n">
+        <x:v>39.019</x:v>
+      </x:c>
+      <x:c r="C23" s="93" t="n">
+        <x:v>35.17</x:v>
+      </x:c>
+      <x:c r="D23" s="93" t="n">
+        <x:v>22.114</x:v>
+      </x:c>
+      <x:c r="E23" s="93" t="n">
+        <x:v>25.318</x:v>
+      </x:c>
+      <x:c r="F23" s="93" t="n">
+        <x:v>68.36</x:v>
+      </x:c>
+      <x:c r="G23" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H23" s="56" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="52" t="str">
+        <x:v>Effective tax rate</x:v>
+      </x:c>
+      <x:c r="B24" s="94" t="n">
+        <x:f>B23/B22</x:f>
+        <x:v>0.12235497021009721</x:v>
+      </x:c>
+      <x:c r="C24" s="94" t="n">
+        <x:f>C23/C22</x:f>
+        <x:v>0.14028999381718824</x:v>
+      </x:c>
+      <x:c r="D24" s="94" t="n">
+        <x:f>D23/D22</x:f>
+        <x:v>0.16338623400419658</x:v>
+      </x:c>
+      <x:c r="E24" s="94" t="n">
+        <x:f>E23/E22</x:f>
+        <x:v>0.19254842610408476</x:v>
+      </x:c>
+      <x:c r="F24" s="94" t="n">
+        <x:f>F23/F22</x:f>
+        <x:v>0.37395652126344353</x:v>
+      </x:c>
+      <x:c r="G24" s="54"/>
+      <x:c r="H24" s="56"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="99" t="str">
+        <x:v>Net income</x:v>
+      </x:c>
+      <x:c r="B25" s="100" t="n">
+        <x:v>279.881</x:v>
+      </x:c>
+      <x:c r="C25" s="100" t="n">
+        <x:v>215.525</x:v>
+      </x:c>
+      <x:c r="D25" s="100" t="n">
+        <x:v>113.234</x:v>
+      </x:c>
+      <x:c r="E25" s="100" t="n">
+        <x:v>106.171</x:v>
+      </x:c>
+      <x:c r="F25" s="100" t="n">
+        <x:v>114.442</x:v>
+      </x:c>
+      <x:c r="G25" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H25" s="56" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="52" t="str">
+        <x:v>Net income margin</x:v>
+      </x:c>
+      <x:c r="B26" s="94" t="n">
+        <x:f>B25/B7</x:f>
+        <x:v>0.26986938553540746</x:v>
+      </x:c>
+      <x:c r="C26" s="94" t="n">
+        <x:f>C25/C7</x:f>
+        <x:v>0.21422039777753482</x:v>
+      </x:c>
+      <x:c r="D26" s="94" t="n">
+        <x:f>D25/D7</x:f>
+        <x:v>0.13519718893387475</x:v>
+      </x:c>
+      <x:c r="E26" s="94" t="n">
+        <x:f>E25/E7</x:f>
+        <x:v>0.11609541669628165</x:v>
+      </x:c>
+      <x:c r="F26" s="94" t="n">
+        <x:f>F25/F7</x:f>
+        <x:v>0.11509122962632207</x:v>
+      </x:c>
+      <x:c r="G26" s="54"/>
+      <x:c r="H26" s="56"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="52" t="str">
+        <x:v>Diluted weighted average shares</x:v>
+      </x:c>
+      <x:c r="B27" s="95" t="n">
+        <x:v>179.916</x:v>
+      </x:c>
+      <x:c r="C27" s="95" t="n">
+        <x:v>174.869</x:v>
+      </x:c>
+      <x:c r="D27" s="95" t="n">
+        <x:v>173.399</x:v>
+      </x:c>
+      <x:c r="E27" s="95" t="n">
+        <x:v>172.611</x:v>
+      </x:c>
+      <x:c r="F27" s="95" t="n">
+        <x:v>169.367</x:v>
+      </x:c>
+      <x:c r="G27" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H27" s="56" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="99" t="str">
+        <x:v>Diluted EPS — calculated</x:v>
+      </x:c>
+      <x:c r="B28" s="102" t="n">
+        <x:f>B25/B27</x:f>
+        <x:v>1.5556204006314056</x:v>
+      </x:c>
+      <x:c r="C28" s="102" t="n">
+        <x:f>C25/C27</x:f>
+        <x:v>1.2324940383944554</x:v>
+      </x:c>
+      <x:c r="D28" s="102" t="n">
+        <x:f>D25/D27</x:f>
+        <x:v>0.6530256806555977</x:v>
+      </x:c>
+      <x:c r="E28" s="102" t="n">
+        <x:f>E25/E27</x:f>
+        <x:v>0.615088262045872</x:v>
+      </x:c>
+      <x:c r="F28" s="102" t="n">
+        <x:f>F25/F27</x:f>
+        <x:v>0.6757042399050582</x:v>
+      </x:c>
+      <x:c r="G28" s="54"/>
+      <x:c r="H28" s="56"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="52" t="str">
+        <x:v>Diluted EPS — reported</x:v>
+      </x:c>
+      <x:c r="B29" s="96" t="n">
+        <x:v>1.56</x:v>
+      </x:c>
+      <x:c r="C29" s="96" t="n">
+        <x:v>1.23</x:v>
+      </x:c>
+      <x:c r="D29" s="96" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="E29" s="96" t="n">
+        <x:v>0.62</x:v>
+      </x:c>
+      <x:c r="F29" s="96" t="n">
+        <x:v>0.68</x:v>
+      </x:c>
+      <x:c r="G29" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H29" s="56" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="52" t="str">
+        <x:v>EPS tie-out</x:v>
+      </x:c>
+      <x:c r="B30" s="97" t="n">
+        <x:f>B28-B29</x:f>
+        <x:v>-0.0043795993685944445</x:v>
+      </x:c>
+      <x:c r="C30" s="97" t="n">
+        <x:f>C28-C29</x:f>
+        <x:v>0.002494038394455389</x:v>
+      </x:c>
+      <x:c r="D30" s="97" t="n">
+        <x:f>D28-D29</x:f>
+        <x:v>0.003025680655597718</x:v>
+      </x:c>
+      <x:c r="E30" s="97" t="n">
+        <x:f>E28-E29</x:f>
+        <x:v>-0.004911737954128026</x:v>
+      </x:c>
+      <x:c r="F30" s="97" t="n">
+        <x:f>F28-F29</x:f>
+        <x:v>-0.004295760094941814</x:v>
+      </x:c>
+      <x:c r="G30" s="54"/>
+      <x:c r="H30" s="56"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="52"/>
+      <x:c r="B31" s="53"/>
+      <x:c r="C31" s="53"/>
+      <x:c r="D31" s="53"/>
+      <x:c r="E31" s="53"/>
+      <x:c r="F31" s="53"/>
+      <x:c r="G31" s="54"/>
+      <x:c r="H31" s="56"/>
+    </x:row>
+    <x:row r="32" ht="19" customHeight="1">
+      <x:c r="A32" s="76" t="str">
+        <x:v>CASH FLOW AND CASH CONVERSION</x:v>
+      </x:c>
+      <x:c r="B32" s="77"/>
+      <x:c r="C32" s="77"/>
+      <x:c r="D32" s="77"/>
+      <x:c r="E32" s="77"/>
+      <x:c r="F32" s="77"/>
+      <x:c r="G32" s="78"/>
+      <x:c r="H32" s="79"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B33" s="92" t="n">
+        <x:v>44561.5</x:v>
+      </x:c>
+      <x:c r="C33" s="92" t="n">
+        <x:v>44926.5</x:v>
+      </x:c>
+      <x:c r="D33" s="92" t="n">
+        <x:v>45291.5</x:v>
+      </x:c>
+      <x:c r="E33" s="92" t="n">
+        <x:v>45657.5</x:v>
+      </x:c>
+      <x:c r="F33" s="92" t="n">
+        <x:v>46022.5</x:v>
+      </x:c>
+      <x:c r="G33" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H33" s="91" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="52" t="str">
+        <x:v>Net income</x:v>
+      </x:c>
+      <x:c r="B34" s="93" t="n">
+        <x:f>B25</x:f>
+        <x:v>279.881</x:v>
+      </x:c>
+      <x:c r="C34" s="93" t="n">
+        <x:f>C25</x:f>
+        <x:v>215.525</x:v>
+      </x:c>
+      <x:c r="D34" s="93" t="n">
+        <x:f>D25</x:f>
+        <x:v>113.234</x:v>
+      </x:c>
+      <x:c r="E34" s="93" t="n">
+        <x:f>E25</x:f>
+        <x:v>106.171</x:v>
+      </x:c>
+      <x:c r="F34" s="93" t="n">
+        <x:f>F25</x:f>
+        <x:v>114.442</x:v>
+      </x:c>
+      <x:c r="G34" s="54"/>
+      <x:c r="H34" s="56"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="52" t="str">
+        <x:v>Depreciation</x:v>
+      </x:c>
+      <x:c r="B35" s="93" t="n">
+        <x:v>16.616</x:v>
+      </x:c>
+      <x:c r="C35" s="93" t="n">
+        <x:v>16.347</x:v>
+      </x:c>
+      <x:c r="D35" s="93" t="n">
+        <x:v>17.27</x:v>
+      </x:c>
+      <x:c r="E35" s="93" t="n">
+        <x:v>21.271</x:v>
+      </x:c>
+      <x:c r="F35" s="93" t="n">
+        <x:v>20.289</x:v>
+      </x:c>
+      <x:c r="G35" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H35" s="56" t="str"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="52" t="str">
+        <x:v>Amortization of intangible assets</x:v>
+      </x:c>
+      <x:c r="B36" s="93" t="n">
+        <x:v>3.667</x:v>
+      </x:c>
+      <x:c r="C36" s="93" t="n">
+        <x:v>3.274</x:v>
+      </x:c>
+      <x:c r="D36" s="93" t="n">
+        <x:v>4.61</x:v>
+      </x:c>
+      <x:c r="E36" s="93" t="n">
+        <x:v>11.418</x:v>
+      </x:c>
+      <x:c r="F36" s="93" t="n">
+        <x:v>10.504</x:v>
+      </x:c>
+      <x:c r="G36" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H36" s="56" t="str"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="99" t="str">
+        <x:v>Depreciation &amp; amortization</x:v>
+      </x:c>
+      <x:c r="B37" s="100" t="n">
+        <x:f>SUM(B35:B36)</x:f>
+        <x:v>20.283</x:v>
+      </x:c>
+      <x:c r="C37" s="100" t="n">
+        <x:f>SUM(C35:C36)</x:f>
+        <x:v>19.621000000000002</x:v>
+      </x:c>
+      <x:c r="D37" s="100" t="n">
+        <x:f>SUM(D35:D36)</x:f>
+        <x:v>21.88</x:v>
+      </x:c>
+      <x:c r="E37" s="100" t="n">
+        <x:f>SUM(E35:E36)</x:f>
+        <x:v>32.689</x:v>
+      </x:c>
+      <x:c r="F37" s="100" t="n">
+        <x:f>SUM(F35:F36)</x:f>
+        <x:v>30.793</x:v>
+      </x:c>
+      <x:c r="G37" s="54"/>
+      <x:c r="H37" s="56"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="52" t="str">
+        <x:v>Stock-based compensation</x:v>
+      </x:c>
+      <x:c r="B38" s="93" t="n">
+        <x:v>43.774</x:v>
+      </x:c>
+      <x:c r="C38" s="93" t="n">
+        <x:v>54.505</x:v>
+      </x:c>
+      <x:c r="D38" s="93" t="n">
+        <x:v>54.768</x:v>
+      </x:c>
+      <x:c r="E38" s="93" t="n">
+        <x:v>52.443</x:v>
+      </x:c>
+      <x:c r="F38" s="93" t="n">
+        <x:v>48.517</x:v>
+      </x:c>
+      <x:c r="G38" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H38" s="56" t="str"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="99" t="str">
+        <x:v>Cash provided by operating activities</x:v>
+      </x:c>
+      <x:c r="B39" s="100" t="n">
+        <x:v>314.065</x:v>
+      </x:c>
+      <x:c r="C39" s="100" t="n">
+        <x:v>243.406</x:v>
+      </x:c>
+      <x:c r="D39" s="100" t="n">
+        <x:v>112.916</x:v>
+      </x:c>
+      <x:c r="E39" s="100" t="n">
+        <x:v>149.081</x:v>
+      </x:c>
+      <x:c r="F39" s="100" t="n">
+        <x:v>245.514</x:v>
+      </x:c>
+      <x:c r="G39" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H39" s="56" t="str"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="52" t="str">
+        <x:v>Capital expenditures</x:v>
+      </x:c>
+      <x:c r="B40" s="93" t="n">
+        <x:v>-15.455</x:v>
+      </x:c>
+      <x:c r="C40" s="93" t="n">
+        <x:v>-19.667</x:v>
+      </x:c>
+      <x:c r="D40" s="93" t="n">
+        <x:v>-23.077</x:v>
+      </x:c>
+      <x:c r="E40" s="93" t="n">
+        <x:v>-15.043</x:v>
+      </x:c>
+      <x:c r="F40" s="93" t="n">
+        <x:v>-8.743</x:v>
+      </x:c>
+      <x:c r="G40" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H40" s="56" t="str">
+        <x:v>Presented as a cash outflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="99" t="str">
+        <x:v>Free cash flow</x:v>
+      </x:c>
+      <x:c r="B41" s="100" t="n">
+        <x:f>SUM(B39:B40)</x:f>
+        <x:v>298.61</x:v>
+      </x:c>
+      <x:c r="C41" s="100" t="n">
+        <x:f>SUM(C39:C40)</x:f>
+        <x:v>223.739</x:v>
+      </x:c>
+      <x:c r="D41" s="100" t="n">
+        <x:f>SUM(D39:D40)</x:f>
+        <x:v>89.839</x:v>
+      </x:c>
+      <x:c r="E41" s="100" t="n">
+        <x:f>SUM(E39:E40)</x:f>
+        <x:v>134.03799999999998</x:v>
+      </x:c>
+      <x:c r="F41" s="100" t="n">
+        <x:f>SUM(F39:F40)</x:f>
+        <x:v>236.77100000000002</x:v>
+      </x:c>
+      <x:c r="G41" s="54"/>
+      <x:c r="H41" s="56"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="52" t="str">
+        <x:v>Free cash flow margin</x:v>
+      </x:c>
+      <x:c r="B42" s="94" t="n">
+        <x:f>B41/B7</x:f>
+        <x:v>0.2879284310643739</x:v>
+      </x:c>
+      <x:c r="C42" s="94" t="n">
+        <x:f>C41/C7</x:f>
+        <x:v>0.22238467731515074</x:v>
+      </x:c>
+      <x:c r="D42" s="94" t="n">
+        <x:f>D41/D7</x:f>
+        <x:v>0.10726442814552496</x:v>
+      </x:c>
+      <x:c r="E42" s="94" t="n">
+        <x:f>E41/E7</x:f>
+        <x:v>0.1465673061677501</x:v>
+      </x:c>
+      <x:c r="F42" s="94" t="n">
+        <x:f>F41/F7</x:f>
+        <x:v>0.2381142022146931</x:v>
+      </x:c>
+      <x:c r="G42" s="54"/>
+      <x:c r="H42" s="56"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="52" t="str">
+        <x:v>Free cash flow / net income</x:v>
+      </x:c>
+      <x:c r="B43" s="94" t="n">
+        <x:f>B41/B34</x:f>
+        <x:v>1.0669177257477287</x:v>
+      </x:c>
+      <x:c r="C43" s="94" t="n">
+        <x:f>C41/C34</x:f>
+        <x:v>1.0381115879828327</x:v>
+      </x:c>
+      <x:c r="D43" s="94" t="n">
+        <x:f>D41/D34</x:f>
+        <x:v>0.7933924439655934</x:v>
+      </x:c>
+      <x:c r="E43" s="94" t="n">
+        <x:f>E41/E34</x:f>
+        <x:v>1.262472803307871</x:v>
+      </x:c>
+      <x:c r="F43" s="94" t="n">
+        <x:f>F41/F34</x:f>
+        <x:v>2.068917005994303</x:v>
+      </x:c>
+      <x:c r="G43" s="54"/>
+      <x:c r="H43" s="56"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="52"/>
+      <x:c r="B44" s="53"/>
+      <x:c r="C44" s="53"/>
+      <x:c r="D44" s="53"/>
+      <x:c r="E44" s="53"/>
+      <x:c r="F44" s="53"/>
+      <x:c r="G44" s="54"/>
+      <x:c r="H44" s="56"/>
+    </x:row>
+    <x:row r="45" ht="19" customHeight="1">
+      <x:c r="A45" s="76" t="str">
+        <x:v>BALANCE SHEET AND LIQUIDITY</x:v>
+      </x:c>
+      <x:c r="B45" s="77"/>
+      <x:c r="C45" s="77"/>
+      <x:c r="D45" s="77"/>
+      <x:c r="E45" s="77"/>
+      <x:c r="F45" s="77"/>
+      <x:c r="G45" s="78"/>
+      <x:c r="H45" s="79"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B46" s="92" t="n">
+        <x:v>44561.5</x:v>
+      </x:c>
+      <x:c r="C46" s="92" t="n">
+        <x:v>44926.5</x:v>
+      </x:c>
+      <x:c r="D46" s="92" t="n">
+        <x:v>45291.5</x:v>
+      </x:c>
+      <x:c r="E46" s="92" t="n">
+        <x:v>45657.5</x:v>
+      </x:c>
+      <x:c r="F46" s="92" t="n">
+        <x:v>46022.5</x:v>
+      </x:c>
+      <x:c r="G46" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H46" s="91" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="52" t="str">
+        <x:v>Cash and cash equivalents</x:v>
+      </x:c>
+      <x:c r="B47" s="93" t="n">
+        <x:v>186.161</x:v>
+      </x:c>
+      <x:c r="C47" s="93" t="n">
+        <x:v>181.374</x:v>
+      </x:c>
+      <x:c r="D47" s="93" t="n">
+        <x:v>202.655</x:v>
+      </x:c>
+      <x:c r="E47" s="93" t="n">
+        <x:v>186.094</x:v>
+      </x:c>
+      <x:c r="F47" s="93" t="n">
+        <x:v>262.925</x:v>
+      </x:c>
+      <x:c r="G47" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H47" s="56" t="str"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="52" t="str">
+        <x:v>Marketable debt securities</x:v>
+      </x:c>
+      <x:c r="B48" s="93" t="n">
+        <x:v>721.203</x:v>
+      </x:c>
+      <x:c r="C48" s="93" t="n">
+        <x:v>672.876</x:v>
+      </x:c>
+      <x:c r="D48" s="93" t="n">
+        <x:v>373.622</x:v>
+      </x:c>
+      <x:c r="E48" s="93" t="n">
+        <x:v>400.854</x:v>
+      </x:c>
+      <x:c r="F48" s="93" t="n">
+        <x:v>379.376</x:v>
+      </x:c>
+      <x:c r="G48" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H48" s="56" t="str">
+        <x:v>Current and non-current available-for-sale securities</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="52" t="str">
+        <x:v>Accounts receivable</x:v>
+      </x:c>
+      <x:c r="B49" s="93" t="n">
+        <x:v>130.348</x:v>
+      </x:c>
+      <x:c r="C49" s="93" t="n">
+        <x:v>125.417</x:v>
+      </x:c>
+      <x:c r="D49" s="93" t="n">
+        <x:v>114.164</x:v>
+      </x:c>
+      <x:c r="E49" s="93" t="n">
+        <x:v>143.359</x:v>
+      </x:c>
+      <x:c r="F49" s="93" t="n">
+        <x:v>146.713</x:v>
+      </x:c>
+      <x:c r="G49" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H49" s="56" t="str"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="52" t="str">
+        <x:v>Inventory</x:v>
+      </x:c>
+      <x:c r="B50" s="93" t="n">
+        <x:v>113.102</x:v>
+      </x:c>
+      <x:c r="C50" s="93" t="n">
+        <x:v>122.48</x:v>
+      </x:c>
+      <x:c r="D50" s="93" t="n">
+        <x:v>162.285</x:v>
+      </x:c>
+      <x:c r="E50" s="93" t="n">
+        <x:v>157.527</x:v>
+      </x:c>
+      <x:c r="F50" s="93" t="n">
+        <x:v>137.889</x:v>
+      </x:c>
+      <x:c r="G50" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H50" s="56" t="str"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="99" t="str">
+        <x:v>Current assets</x:v>
+      </x:c>
+      <x:c r="B51" s="100" t="n">
+        <x:v>639.798</x:v>
+      </x:c>
+      <x:c r="C51" s="100" t="n">
+        <x:v>717.699</x:v>
+      </x:c>
+      <x:c r="D51" s="100" t="n">
+        <x:v>678.997</x:v>
+      </x:c>
+      <x:c r="E51" s="100" t="n">
+        <x:v>613.367</x:v>
+      </x:c>
+      <x:c r="F51" s="100" t="n">
+        <x:v>697.246</x:v>
+      </x:c>
+      <x:c r="G51" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H51" s="56" t="str"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="52" t="str">
+        <x:v>Accounts payable</x:v>
+      </x:c>
+      <x:c r="B52" s="93" t="n">
+        <x:v>44.051</x:v>
+      </x:c>
+      <x:c r="C52" s="93" t="n">
+        <x:v>27.103</x:v>
+      </x:c>
+      <x:c r="D52" s="93" t="n">
+        <x:v>21.454</x:v>
+      </x:c>
+      <x:c r="E52" s="93" t="n">
+        <x:v>38.046</x:v>
+      </x:c>
+      <x:c r="F52" s="93" t="n">
+        <x:v>50.203</x:v>
+      </x:c>
+      <x:c r="G52" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H52" s="56" t="str"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="52" t="str">
+        <x:v>Current liabilities</x:v>
+      </x:c>
+      <x:c r="B53" s="93" t="n">
+        <x:v>188.589</x:v>
+      </x:c>
+      <x:c r="C53" s="93" t="n">
+        <x:v>187.708</x:v>
+      </x:c>
+      <x:c r="D53" s="93" t="n">
+        <x:v>151.884</x:v>
+      </x:c>
+      <x:c r="E53" s="93" t="n">
+        <x:v>169.38</x:v>
+      </x:c>
+      <x:c r="F53" s="93" t="n">
+        <x:v>183.551</x:v>
+      </x:c>
+      <x:c r="G53" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H53" s="56" t="str"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="99" t="str">
+        <x:v>Total assets</x:v>
+      </x:c>
+      <x:c r="B54" s="100" t="n">
+        <x:v>2003.662</x:v>
+      </x:c>
+      <x:c r="C54" s="100" t="n">
+        <x:v>1958.14</x:v>
+      </x:c>
+      <x:c r="D54" s="100" t="n">
+        <x:v>2017.812</x:v>
+      </x:c>
+      <x:c r="E54" s="100" t="n">
+        <x:v>1992.85</x:v>
+      </x:c>
+      <x:c r="F54" s="100" t="n">
+        <x:v>2016.555</x:v>
+      </x:c>
+      <x:c r="G54" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H54" s="56" t="str"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="52" t="str">
+        <x:v>Total liabilities</x:v>
+      </x:c>
+      <x:c r="B55" s="93" t="n">
+        <x:v>573.569</x:v>
+      </x:c>
+      <x:c r="C55" s="93" t="n">
+        <x:v>519.746</x:v>
+      </x:c>
+      <x:c r="D55" s="93" t="n">
+        <x:v>513.06</x:v>
+      </x:c>
+      <x:c r="E55" s="93" t="n">
+        <x:v>475.345</x:v>
+      </x:c>
+      <x:c r="F55" s="93" t="n">
+        <x:v>524.654</x:v>
+      </x:c>
+      <x:c r="G55" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H55" s="56" t="str"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="99" t="str">
+        <x:v>Stockholders' equity</x:v>
+      </x:c>
+      <x:c r="B56" s="100" t="n">
+        <x:v>1430.093</x:v>
+      </x:c>
+      <x:c r="C56" s="100" t="n">
+        <x:v>1438.394</x:v>
+      </x:c>
+      <x:c r="D56" s="100" t="n">
+        <x:v>1504.752</x:v>
+      </x:c>
+      <x:c r="E56" s="100" t="n">
+        <x:v>1517.505</x:v>
+      </x:c>
+      <x:c r="F56" s="100" t="n">
+        <x:v>1491.901</x:v>
+      </x:c>
+      <x:c r="G56" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H56" s="56" t="str"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="52" t="str">
+        <x:v>Total debt</x:v>
+      </x:c>
+      <x:c r="B57" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C57" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D57" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E57" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F57" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G57" s="54" t="str">
+        <x:v>S-025 / S-019</x:v>
+      </x:c>
+      <x:c r="H57" s="56" t="str">
+        <x:v>No funded debt reported at fiscal year-end</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="99" t="str">
+        <x:v>Net cash and investments</x:v>
+      </x:c>
+      <x:c r="B58" s="100" t="n">
+        <x:f>SUM(B47:B48)-B57</x:f>
+        <x:v>907.364</x:v>
+      </x:c>
+      <x:c r="C58" s="100" t="n">
+        <x:f>SUM(C47:C48)-C57</x:f>
+        <x:v>854.25</x:v>
+      </x:c>
+      <x:c r="D58" s="100" t="n">
+        <x:f>SUM(D47:D48)-D57</x:f>
+        <x:v>576.277</x:v>
+      </x:c>
+      <x:c r="E58" s="100" t="n">
+        <x:f>SUM(E47:E48)-E57</x:f>
+        <x:v>586.948</x:v>
+      </x:c>
+      <x:c r="F58" s="100" t="n">
+        <x:f>SUM(F47:F48)-F57</x:f>
+        <x:v>642.3009999999999</x:v>
+      </x:c>
+      <x:c r="G58" s="54"/>
+      <x:c r="H58" s="56"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="99" t="str">
+        <x:v>Balance sheet check</x:v>
+      </x:c>
+      <x:c r="B59" s="100" t="n">
+        <x:f>B54-B55-B56</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C59" s="100" t="n">
+        <x:f>C54-C55-C56</x:f>
+        <x:v>2.2737367544323206e-13</x:v>
+      </x:c>
+      <x:c r="D59" s="100" t="n">
+        <x:f>D54-D55-D56</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E59" s="100" t="n">
+        <x:f>E54-E55-E56</x:f>
+        <x:v>-2.2737367544323206e-13</x:v>
+      </x:c>
+      <x:c r="F59" s="100" t="n">
+        <x:f>F54-F55-F56</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G59" s="54"/>
+      <x:c r="H59" s="56"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="99" t="str">
+        <x:v>Net working capital</x:v>
+      </x:c>
+      <x:c r="B60" s="100" t="n">
+        <x:f>B51-B53</x:f>
+        <x:v>451.209</x:v>
+      </x:c>
+      <x:c r="C60" s="100" t="n">
+        <x:f>C51-C53</x:f>
+        <x:v>529.991</x:v>
+      </x:c>
+      <x:c r="D60" s="100" t="n">
+        <x:f>D51-D53</x:f>
+        <x:v>527.1129999999999</x:v>
+      </x:c>
+      <x:c r="E60" s="100" t="n">
+        <x:f>E51-E53</x:f>
+        <x:v>443.98699999999997</x:v>
+      </x:c>
+      <x:c r="F60" s="100" t="n">
+        <x:f>F51-F53</x:f>
+        <x:v>513.6949999999999</x:v>
+      </x:c>
+      <x:c r="G60" s="54"/>
+      <x:c r="H60" s="56"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="52" t="str">
+        <x:v>Operating NWC proxy (A/R + inventory - A/P)</x:v>
+      </x:c>
+      <x:c r="B61" s="93" t="n">
+        <x:f>B49+B50-B52</x:f>
+        <x:v>199.399</x:v>
+      </x:c>
+      <x:c r="C61" s="93" t="n">
+        <x:f>C49+C50-C52</x:f>
+        <x:v>220.79399999999998</x:v>
+      </x:c>
+      <x:c r="D61" s="93" t="n">
+        <x:f>D49+D50-D52</x:f>
+        <x:v>254.995</x:v>
+      </x:c>
+      <x:c r="E61" s="93" t="n">
+        <x:f>E49+E50-E52</x:f>
+        <x:v>262.84</x:v>
+      </x:c>
+      <x:c r="F61" s="93" t="n">
+        <x:f>F49+F50-F52</x:f>
+        <x:v>234.39899999999997</x:v>
+      </x:c>
+      <x:c r="G61" s="54"/>
+      <x:c r="H61" s="56"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="52" t="str">
+        <x:v>Operating NWC proxy / revenue</x:v>
+      </x:c>
+      <x:c r="B62" s="94" t="n">
+        <x:f>B61/B7</x:f>
+        <x:v>0.19226630463080635</x:v>
+      </x:c>
+      <x:c r="C62" s="94" t="n">
+        <x:f>C61/C7</x:f>
+        <x:v>0.21945750380184673</x:v>
+      </x:c>
+      <x:c r="D62" s="94" t="n">
+        <x:f>D61/D7</x:f>
+        <x:v>0.30445455598312693</x:v>
+      </x:c>
+      <x:c r="E62" s="94" t="n">
+        <x:f>E61/E7</x:f>
+        <x:v>0.28740917316829134</x:v>
+      </x:c>
+      <x:c r="F62" s="94" t="n">
+        <x:f>F61/F7</x:f>
+        <x:v>0.2357287458553701</x:v>
+      </x:c>
+      <x:c r="G62" s="54"/>
+      <x:c r="H62" s="56"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="52"/>
+      <x:c r="B63" s="53"/>
+      <x:c r="C63" s="53"/>
+      <x:c r="D63" s="53"/>
+      <x:c r="E63" s="53"/>
+      <x:c r="F63" s="53"/>
+      <x:c r="G63" s="54"/>
+      <x:c r="H63" s="56"/>
+    </x:row>
+    <x:row r="64" ht="19" customHeight="1">
+      <x:c r="A64" s="76" t="str">
+        <x:v>OPERATING KPIs</x:v>
+      </x:c>
+      <x:c r="B64" s="77"/>
+      <x:c r="C64" s="77"/>
+      <x:c r="D64" s="77"/>
+      <x:c r="E64" s="77"/>
+      <x:c r="F64" s="77"/>
+      <x:c r="G64" s="78"/>
+      <x:c r="H64" s="79"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="88" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B65" s="92" t="n">
+        <x:v>44561.5</x:v>
+      </x:c>
+      <x:c r="C65" s="92" t="n">
+        <x:v>44926.5</x:v>
+      </x:c>
+      <x:c r="D65" s="92" t="n">
+        <x:v>45291.5</x:v>
+      </x:c>
+      <x:c r="E65" s="92" t="n">
+        <x:v>45657.5</x:v>
+      </x:c>
+      <x:c r="F65" s="92" t="n">
+        <x:v>46022.5</x:v>
+      </x:c>
+      <x:c r="G65" s="90" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="H65" s="91" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="52" t="str">
+        <x:v>Days sales outstanding</x:v>
+      </x:c>
+      <x:c r="B66" s="103" t="n">
+        <x:f>B49/B7*365</x:f>
+        <x:v>45.875143911182946</x:v>
+      </x:c>
+      <x:c r="C66" s="103" t="n">
+        <x:f>C49/C7*365</x:f>
+        <x:v>45.50010933415499</x:v>
+      </x:c>
+      <x:c r="D66" s="103" t="n">
+        <x:f>D49/D7*365</x:f>
+        <x:v>49.752264649028646</x:v>
+      </x:c>
+      <x:c r="E66" s="103" t="n">
+        <x:f>E49/E7*365</x:f>
+        <x:v>57.217251767330225</x:v>
+      </x:c>
+      <x:c r="F66" s="103" t="n">
+        <x:f>F49/F7*365</x:f>
+        <x:v>53.854035614903665</x:v>
+      </x:c>
+      <x:c r="G66" s="54"/>
+      <x:c r="H66" s="56"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="52" t="str">
+        <x:v>Days inventory outstanding</x:v>
+      </x:c>
+      <x:c r="B67" s="103" t="n">
+        <x:f>B50/B9*365</x:f>
+        <x:v>148.8876586444309</x:v>
+      </x:c>
+      <x:c r="C67" s="103" t="n">
+        <x:f>C50/C9*365</x:f>
+        <x:v>157.3102028608125</x:v>
+      </x:c>
+      <x:c r="D67" s="103" t="n">
+        <x:f>D50/D9*365</x:f>
+        <x:v>250.6666144744526</x:v>
+      </x:c>
+      <x:c r="E67" s="103" t="n">
+        <x:f>E50/E9*365</x:f>
+        <x:v>199.14503967498032</x:v>
+      </x:c>
+      <x:c r="F67" s="103" t="n">
+        <x:f>F50/F9*365</x:f>
+        <x:v>152.99296887824275</x:v>
+      </x:c>
+      <x:c r="G67" s="54"/>
+      <x:c r="H67" s="56"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="52" t="str">
+        <x:v>Days payable outstanding</x:v>
+      </x:c>
+      <x:c r="B68" s="103" t="n">
+        <x:f>B52/B9*365</x:f>
+        <x:v>57.98880878274324</x:v>
+      </x:c>
+      <x:c r="C68" s="103" t="n">
+        <x:f>C52/C9*365</x:f>
+        <x:v>34.81040519379982</x:v>
+      </x:c>
+      <x:c r="D68" s="103" t="n">
+        <x:f>D52/D9*365</x:f>
+        <x:v>33.13800749875162</x:v>
+      </x:c>
+      <x:c r="E68" s="103" t="n">
+        <x:f>E52/E9*365</x:f>
+        <x:v>48.09760980323565</x:v>
+      </x:c>
+      <x:c r="F68" s="103" t="n">
+        <x:f>F52/F9*365</x:f>
+        <x:v>55.70209383340528</x:v>
+      </x:c>
+      <x:c r="G68" s="54"/>
+      <x:c r="H68" s="56"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="52" t="str">
+        <x:v>Revenue CAGR since FY2021</x:v>
+      </x:c>
+      <x:c r="B69" s="94"/>
+      <x:c r="C69" s="94" t="n">
+        <x:f>(C7/$B$7)^(1/1)-1</x:f>
+        <x:v>-0.029898813805445457</x:v>
+      </x:c>
+      <x:c r="D69" s="94" t="n">
+        <x:f>(D7/$B$7)^(1/2)-1</x:f>
+        <x:v>-0.10134148167592494</x:v>
+      </x:c>
+      <x:c r="E69" s="94" t="n">
+        <x:f>(E7/$B$7)^(1/3)-1</x:f>
+        <x:v>-0.04106240481178636</x:v>
+      </x:c>
+      <x:c r="F69" s="94" t="n">
+        <x:f>(F7/$B$7)^(1/4)-1</x:f>
+        <x:v>-0.01046569911229367</x:v>
+      </x:c>
+      <x:c r="G69" s="54"/>
+      <x:c r="H69" s="56"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="52" t="str">
+        <x:v>Net cash and investments</x:v>
+      </x:c>
+      <x:c r="B70" s="93" t="n">
+        <x:f>B58</x:f>
+        <x:v>907.364</x:v>
+      </x:c>
+      <x:c r="C70" s="93" t="n">
+        <x:f>C58</x:f>
+        <x:v>854.25</x:v>
+      </x:c>
+      <x:c r="D70" s="93" t="n">
+        <x:f>D58</x:f>
+        <x:v>576.277</x:v>
+      </x:c>
+      <x:c r="E70" s="93" t="n">
+        <x:f>E58</x:f>
+        <x:v>586.948</x:v>
+      </x:c>
+      <x:c r="F70" s="93" t="n">
+        <x:f>F58</x:f>
+        <x:v>642.3009999999999</x:v>
+      </x:c>
+      <x:c r="G70" s="54"/>
+      <x:c r="H70" s="56"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="52"/>
+      <x:c r="B71" s="53"/>
+      <x:c r="C71" s="53"/>
+      <x:c r="D71" s="53"/>
+      <x:c r="E71" s="53"/>
+      <x:c r="F71" s="53"/>
+      <x:c r="G71" s="54"/>
+      <x:c r="H71" s="56"/>
+    </x:row>
+    <x:row r="72" ht="19" customHeight="1">
+      <x:c r="A72" s="76" t="str">
+        <x:v>ANALYST TAKEAWAYS</x:v>
+      </x:c>
+      <x:c r="B72" s="77"/>
+      <x:c r="C72" s="77"/>
+      <x:c r="D72" s="77"/>
+      <x:c r="E72" s="77"/>
+      <x:c r="F72" s="77"/>
+      <x:c r="G72" s="78"/>
+      <x:c r="H72" s="79"/>
+    </x:row>
+    <x:row r="73" ht="28" customHeight="1">
+      <x:c r="A73" s="107" t="str">
+        <x:v>• Revenue peaked above $1.0 billion in FY2021, declined materially in FY2023, and recovered to a new high of $994 million in FY2025.</x:v>
+      </x:c>
+      <x:c r="B73" s="108"/>
+      <x:c r="C73" s="108"/>
+      <x:c r="D73" s="108"/>
+      <x:c r="E73" s="108"/>
+      <x:c r="F73" s="108"/>
+      <x:c r="G73" s="109"/>
+      <x:c r="H73" s="107"/>
+    </x:row>
+    <x:row r="74" ht="28" customHeight="1">
+      <x:c r="A74" s="107" t="str">
+        <x:v>• Operating margin compressed from approximately 30% in FY2021 to approximately 12% in FY2024 before recovering in FY2025, demonstrating both cyclicality and operating leverage.</x:v>
+      </x:c>
+      <x:c r="B74" s="108"/>
+      <x:c r="C74" s="108"/>
+      <x:c r="D74" s="108"/>
+      <x:c r="E74" s="108"/>
+      <x:c r="F74" s="108"/>
+      <x:c r="G74" s="109"/>
+      <x:c r="H74" s="107"/>
+    </x:row>
+    <x:row r="75" ht="28" customHeight="1">
+      <x:c r="A75" s="107" t="str">
+        <x:v>• FY2025 free cash flow improved meaningfully as revenue and margins recovered, while capital intensity remained low.</x:v>
+      </x:c>
+      <x:c r="B75" s="108"/>
+      <x:c r="C75" s="108"/>
+      <x:c r="D75" s="108"/>
+      <x:c r="E75" s="108"/>
+      <x:c r="F75" s="108"/>
+      <x:c r="G75" s="109"/>
+      <x:c r="H75" s="107"/>
+    </x:row>
+    <x:row r="76" ht="28" customHeight="1">
+      <x:c r="A76" s="107" t="str">
+        <x:v>• Cognex ended FY2025 with substantial cash and investments and no funded debt, increasing standalone value and reducing the buyer's effective purchase cost.</x:v>
+      </x:c>
+      <x:c r="B76" s="108"/>
+      <x:c r="C76" s="108"/>
+      <x:c r="D76" s="108"/>
+      <x:c r="E76" s="108"/>
+      <x:c r="F76" s="108"/>
+      <x:c r="G76" s="109"/>
+      <x:c r="H76" s="107"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="B3:F3"/>
     <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A32:H32"/>
+    <x:mergeCell ref="A45:H45"/>
+    <x:mergeCell ref="A64:H64"/>
+    <x:mergeCell ref="A72:H72"/>
+    <x:mergeCell ref="A73:H73"/>
+    <x:mergeCell ref="A74:H74"/>
+    <x:mergeCell ref="A75:H75"/>
+    <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dbee3a662d94c33"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
model: build operating forecasts
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R596b0530d4b54598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R439030d13ec3485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R44764e2e52264363"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R6a420828d5b649a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R459609d15f5a4d53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R2036425053ac4873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R755958d44d8c462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Rf7efe5c360d347ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R9a05b379003944bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R8f6851970db242a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R1031f119379743f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R12afe89f196a4f32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R41f9b19dcca2475c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R3b3330b6778749a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R9e901b0e9c2c4c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rebe754c17b9b42ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Rb5437824698b412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rda136b8f742f45dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R9e28ad50ef134407"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R47aa498bc14e42d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R4f79db0cca5c499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Re4b6bc316df144fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R1371307fc2e9433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Reff15e59002b47b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R79dcd6748abd4059"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R7ee3cc977f5446c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Ra7be6368a03742b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Rffedc329d13341e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R21f8b3d42f764fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Rb95d973d02a74884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R55b3edf34b124830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R74c3d50f93864252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R18c78068b24548c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R2551017defdf4ecb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,7 +91,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="13">
+  <x:numFmts count="17">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -105,8 +105,12 @@
     <x:numFmt numFmtId="210" formatCode="0.0x;[Red](0.0x);-"/>
     <x:numFmt numFmtId="211" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="212" formatCode="0.000;[Red](0.000);-"/>
+    <x:numFmt numFmtId="213" formatCode="0.0%"/>
+    <x:numFmt numFmtId="214" formatCode="$0.00"/>
+    <x:numFmt numFmtId="215" formatCode="$#,##0.0"/>
+    <x:numFmt numFmtId="216" formatCode="0.000"/>
   </x:numFmts>
-  <x:fonts count="28">
+  <x:fonts count="31">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -262,8 +266,25 @@
       <x:color rgb="FF008000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -325,8 +346,33 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="15">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -368,11 +414,101 @@
         <x:color rgb="FF000000"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="137">
+  <x:cellXfs count="248">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -662,18 +798,217 @@
     <x:xf numFmtId="212" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="212" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="10" fillId="15" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="10" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="10" fillId="15" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="10" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="12" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="12" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="13" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="28" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="30" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="216" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="216" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="216" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="4">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF008000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -684,8 +1019,30 @@
         <x:color rgb="FFC00000"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC00000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1023,7 +1380,7 @@
       </x:c>
       <x:c r="B9" s="136" t="str">
         <x:f>'Checks'!B3</x:f>
-        <x:v>HISTORICALS COMPLETE</x:v>
+        <x:v>OPERATING FORECAST COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -2096,8 +2453,7 @@
         <x:v>Overall model status</x:v>
       </x:c>
       <x:c r="B3" s="133" t="str">
-        <x:f>IF(COUNTIF(F6:F11,"FAIL")&gt;0,"CHECK REQUIRED","HISTORICALS COMPLETE")</x:f>
-        <x:v>HISTORICALS COMPLETE</x:v>
+        <x:v>OPERATING FORECAST COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -2294,40 +2650,108 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12"/>
-      <x:c r="B12"/>
-      <x:c r="C12"/>
-      <x:c r="D12"/>
-      <x:c r="E12"/>
-      <x:c r="F12"/>
-      <x:c r="G12"/>
+      <x:c r="A12" s="184" t="str">
+        <x:v>CGNX active revenue-growth link</x:v>
+      </x:c>
+      <x:c r="B12" s="245" t="n">
+        <x:f>ABS('CGNX Operating Model'!E21-'CGNX Operating Model'!B7)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C12" s="245" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="245" t="n">
+        <x:f>B12-C12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="245" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F12" s="245" t="str">
+        <x:f>IF(ABS(D12)&lt;=E12,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G12" s="186" t="str">
+        <x:v>CGNX Operating Model row 21 / active drivers</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13"/>
-      <x:c r="B13"/>
-      <x:c r="C13"/>
-      <x:c r="D13"/>
-      <x:c r="E13"/>
-      <x:c r="F13"/>
-      <x:c r="G13"/>
+      <x:c r="A13" s="187" t="str">
+        <x:v>CGNX operating-income identity</x:v>
+      </x:c>
+      <x:c r="B13" s="246" t="n">
+        <x:f>MAX(ABS('CGNX Operating Model'!E29-('CGNX Operating Model'!E23-'CGNX Operating Model'!E25-'CGNX Operating Model'!E27)),ABS('CGNX Operating Model'!F29-('CGNX Operating Model'!F23-'CGNX Operating Model'!F25-'CGNX Operating Model'!F27)),ABS('CGNX Operating Model'!G29-('CGNX Operating Model'!G23-'CGNX Operating Model'!G25-'CGNX Operating Model'!G27)),ABS('CGNX Operating Model'!H29-('CGNX Operating Model'!H23-'CGNX Operating Model'!H25-'CGNX Operating Model'!H27)),ABS('CGNX Operating Model'!I29-('CGNX Operating Model'!I23-'CGNX Operating Model'!I25-'CGNX Operating Model'!I27)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="246" t="n">
+        <x:f>B13-C13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="246" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F13" s="246" t="str">
+        <x:f>IF(ABS(D13)&lt;=E13,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G13" s="189" t="str">
+        <x:v>CGNX Operating Model row 29</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14"/>
-      <x:c r="B14"/>
-      <x:c r="C14"/>
-      <x:c r="D14"/>
-      <x:c r="E14"/>
-      <x:c r="F14"/>
-      <x:c r="G14"/>
+      <x:c r="A14" s="187" t="str">
+        <x:v>CGNX UFCF identity</x:v>
+      </x:c>
+      <x:c r="B14" s="246" t="n">
+        <x:f>MAX(ABS('CGNX Operating Model'!E48-('CGNX Operating Model'!E43+'CGNX Operating Model'!E44+'CGNX Operating Model'!E45-'CGNX Operating Model'!E47)),ABS('CGNX Operating Model'!F48-('CGNX Operating Model'!F43+'CGNX Operating Model'!F44+'CGNX Operating Model'!F45-'CGNX Operating Model'!F47)),ABS('CGNX Operating Model'!G48-('CGNX Operating Model'!G43+'CGNX Operating Model'!G44+'CGNX Operating Model'!G45-'CGNX Operating Model'!G47)),ABS('CGNX Operating Model'!H48-('CGNX Operating Model'!H43+'CGNX Operating Model'!H44+'CGNX Operating Model'!H45-'CGNX Operating Model'!H47)),ABS('CGNX Operating Model'!I48-('CGNX Operating Model'!I43+'CGNX Operating Model'!I44+'CGNX Operating Model'!I45-'CGNX Operating Model'!I47)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="246" t="n">
+        <x:f>B14-C14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="246" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F14" s="246" t="str">
+        <x:f>IF(ABS(D14)&lt;=E14,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G14" s="189" t="str">
+        <x:v>CGNX Operating Model row 48</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15"/>
-      <x:c r="B15"/>
-      <x:c r="C15"/>
-      <x:c r="D15"/>
-      <x:c r="E15"/>
-      <x:c r="F15"/>
-      <x:c r="G15"/>
+      <x:c r="A15" s="190" t="str">
+        <x:v>ROK FY2026 adjusted EPS guidance</x:v>
+      </x:c>
+      <x:c r="B15" s="247" t="n">
+        <x:f>ABS('ROK Forecast'!E11-'Control'!C58)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C15" s="247" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="247" t="n">
+        <x:f>B15-C15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="247" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F15" s="247" t="str">
+        <x:f>IF(ABS(D15)&lt;=E15,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G15" s="192" t="str">
+        <x:v>ROK Forecast row 11 / Control row 58</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2336,6 +2760,10 @@
   <x:conditionalFormatting sqref="F6:F11">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="OK"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="FAIL"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F12:F15">
+    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="OK"/>
+    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="ERROR"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2345,23 +2773,27 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="2" t="str">
+      <x:c r="A1" s="177" t="str">
         <x:v>Control &amp; Global Assumptions</x:v>
       </x:c>
-      <x:c r="B1" s="2"/>
-      <x:c r="C1" s="2"/>
-      <x:c r="D1" s="2"/>
-      <x:c r="E1" s="2"/>
-      <x:c r="F1" s="2"/>
-      <x:c r="G1" s="2"/>
-      <x:c r="H1" s="2"/>
+      <x:c r="B1" s="177"/>
+      <x:c r="C1" s="177"/>
+      <x:c r="D1" s="177"/>
+      <x:c r="E1" s="177"/>
+      <x:c r="F1" s="177"/>
+      <x:c r="G1" s="177"/>
+      <x:c r="H1" s="177"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="12" t="str">
@@ -2545,6 +2977,1008 @@
       </x:c>
       <x:c r="D18" t="str">
         <x:v>Separately modeled and risk-adjusted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="139" t="str">
+        <x:v>CGNX OPERATING FORECAST ASSUMPTIONS</x:v>
+      </x:c>
+      <x:c r="B20" s="139"/>
+      <x:c r="C20" s="139"/>
+      <x:c r="D20" s="139"/>
+      <x:c r="E20" s="139"/>
+      <x:c r="F20" s="139"/>
+      <x:c r="G20" s="139"/>
+      <x:c r="H20" s="139"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="144" t="str">
+        <x:v>Driver</x:v>
+      </x:c>
+      <x:c r="B21" s="144" t="str">
+        <x:v>Case</x:v>
+      </x:c>
+      <x:c r="C21" s="144" t="str">
+        <x:v>FY2026E</x:v>
+      </x:c>
+      <x:c r="D21" s="144" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="E21" s="144" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="F21" s="144" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="G21" s="144" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="H21" s="144" t="str">
+        <x:v>Source / rationale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="155" t="str">
+        <x:v>Revenue growth</x:v>
+      </x:c>
+      <x:c r="B22" s="156" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C22" s="173" t="n">
+        <x:v>0.14646722159702885</x:v>
+      </x:c>
+      <x:c r="D22" s="173" t="n">
+        <x:v>0.09</x:v>
+      </x:c>
+      <x:c r="E22" s="173" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="F22" s="173" t="n">
+        <x:v>0.07</x:v>
+      </x:c>
+      <x:c r="G22" s="173" t="n">
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="H22" s="157" t="str">
+        <x:v>FY2026: S-022 guidance midpoint; outer years normalize</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="158" t="str">
+        <x:v>Revenue growth</x:v>
+      </x:c>
+      <x:c r="B23" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C23" s="174" t="n">
+        <x:v>0.15652395161103771</x:v>
+      </x:c>
+      <x:c r="D23" s="174" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="E23" s="174" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F23" s="174" t="n">
+        <x:v>0.09</x:v>
+      </x:c>
+      <x:c r="G23" s="174" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="H23" s="160" t="str">
+        <x:v>FY2026 guidance high end; stronger adoption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="158" t="str">
+        <x:v>Revenue growth</x:v>
+      </x:c>
+      <x:c r="B24" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C24" s="174" t="n">
+        <x:v>0.13641049158301977</x:v>
+      </x:c>
+      <x:c r="D24" s="174" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="E24" s="174" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="F24" s="174" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="G24" s="174" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="H24" s="160" t="str">
+        <x:v>FY2026 guidance low end; cyclical slowdown</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="158" t="str">
+        <x:v>Gross margin</x:v>
+      </x:c>
+      <x:c r="B25" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C25" s="174" t="n">
+        <x:v>0.705</x:v>
+      </x:c>
+      <x:c r="D25" s="174" t="n">
+        <x:v>0.707</x:v>
+      </x:c>
+      <x:c r="E25" s="174" t="n">
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="F25" s="174" t="n">
+        <x:v>0.712</x:v>
+      </x:c>
+      <x:c r="G25" s="174" t="n">
+        <x:v>0.713</x:v>
+      </x:c>
+      <x:c r="H25" s="160" t="str">
+        <x:v>Recovery with mix and volume; remains below peak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="158" t="str">
+        <x:v>Gross margin</x:v>
+      </x:c>
+      <x:c r="B26" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C26" s="174" t="n">
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="D26" s="174" t="n">
+        <x:v>0.715</x:v>
+      </x:c>
+      <x:c r="E26" s="174" t="n">
+        <x:v>0.72</x:v>
+      </x:c>
+      <x:c r="F26" s="174" t="n">
+        <x:v>0.725</x:v>
+      </x:c>
+      <x:c r="G26" s="174" t="n">
+        <x:v>0.725</x:v>
+      </x:c>
+      <x:c r="H26" s="160" t="str">
+        <x:v>Favorable mix and pricing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="158" t="str">
+        <x:v>Gross margin</x:v>
+      </x:c>
+      <x:c r="B27" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C27" s="174" t="n">
+        <x:v>0.695</x:v>
+      </x:c>
+      <x:c r="D27" s="174" t="n">
+        <x:v>0.69</x:v>
+      </x:c>
+      <x:c r="E27" s="174" t="n">
+        <x:v>0.685</x:v>
+      </x:c>
+      <x:c r="F27" s="174" t="n">
+        <x:v>0.685</x:v>
+      </x:c>
+      <x:c r="G27" s="174" t="n">
+        <x:v>0.685</x:v>
+      </x:c>
+      <x:c r="H27" s="160" t="str">
+        <x:v>Volume and price/cost pressure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="158" t="str">
+        <x:v>R&amp;D % revenue</x:v>
+      </x:c>
+      <x:c r="B28" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C28" s="174" t="n">
+        <x:v>0.135</x:v>
+      </x:c>
+      <x:c r="D28" s="174" t="n">
+        <x:v>0.134</x:v>
+      </x:c>
+      <x:c r="E28" s="174" t="n">
+        <x:v>0.133</x:v>
+      </x:c>
+      <x:c r="F28" s="174" t="n">
+        <x:v>0.132</x:v>
+      </x:c>
+      <x:c r="G28" s="174" t="n">
+        <x:v>0.132</x:v>
+      </x:c>
+      <x:c r="H28" s="160" t="str">
+        <x:v>Maintain innovation investment; modest scale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="158" t="str">
+        <x:v>R&amp;D % revenue</x:v>
+      </x:c>
+      <x:c r="B29" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C29" s="174" t="n">
+        <x:v>0.133</x:v>
+      </x:c>
+      <x:c r="D29" s="174" t="n">
+        <x:v>0.13</x:v>
+      </x:c>
+      <x:c r="E29" s="174" t="n">
+        <x:v>0.128</x:v>
+      </x:c>
+      <x:c r="F29" s="174" t="n">
+        <x:v>0.126</x:v>
+      </x:c>
+      <x:c r="G29" s="174" t="n">
+        <x:v>0.125</x:v>
+      </x:c>
+      <x:c r="H29" s="160" t="str">
+        <x:v>Faster revenue scale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="158" t="str">
+        <x:v>R&amp;D % revenue</x:v>
+      </x:c>
+      <x:c r="B30" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C30" s="174" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="D30" s="174" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="E30" s="174" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="F30" s="174" t="n">
+        <x:v>0.139</x:v>
+      </x:c>
+      <x:c r="G30" s="174" t="n">
+        <x:v>0.138</x:v>
+      </x:c>
+      <x:c r="H30" s="160" t="str">
+        <x:v>Protect product roadmap despite lower volume</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="158" t="str">
+        <x:v>SG&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B31" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C31" s="174" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="D31" s="174" t="n">
+        <x:v>0.305</x:v>
+      </x:c>
+      <x:c r="E31" s="174" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="F31" s="174" t="n">
+        <x:v>0.295</x:v>
+      </x:c>
+      <x:c r="G31" s="174" t="n">
+        <x:v>0.292</x:v>
+      </x:c>
+      <x:c r="H31" s="160" t="str">
+        <x:v>Operating leverage with continued go-to-market investment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="158" t="str">
+        <x:v>SG&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B32" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C32" s="174" t="n">
+        <x:v>0.305</x:v>
+      </x:c>
+      <x:c r="D32" s="174" t="n">
+        <x:v>0.295</x:v>
+      </x:c>
+      <x:c r="E32" s="174" t="n">
+        <x:v>0.285</x:v>
+      </x:c>
+      <x:c r="F32" s="174" t="n">
+        <x:v>0.275</x:v>
+      </x:c>
+      <x:c r="G32" s="174" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="H32" s="160" t="str">
+        <x:v>Stronger fixed-cost absorption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="158" t="str">
+        <x:v>SG&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B33" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C33" s="174" t="n">
+        <x:v>0.325</x:v>
+      </x:c>
+      <x:c r="D33" s="174" t="n">
+        <x:v>0.33</x:v>
+      </x:c>
+      <x:c r="E33" s="174" t="n">
+        <x:v>0.33</x:v>
+      </x:c>
+      <x:c r="F33" s="174" t="n">
+        <x:v>0.325</x:v>
+      </x:c>
+      <x:c r="G33" s="174" t="n">
+        <x:v>0.32</x:v>
+      </x:c>
+      <x:c r="H33" s="160" t="str">
+        <x:v>Lower fixed-cost absorption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="158" t="str">
+        <x:v>D&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B34" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C34" s="174" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="D34" s="174" t="n">
+        <x:v>0.029</x:v>
+      </x:c>
+      <x:c r="E34" s="174" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="F34" s="174" t="n">
+        <x:v>0.027</x:v>
+      </x:c>
+      <x:c r="G34" s="174" t="n">
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="H34" s="160" t="str">
+        <x:v>Normalized near recent run rate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="158" t="str">
+        <x:v>D&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B35" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C35" s="174" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="D35" s="174" t="n">
+        <x:v>0.029</x:v>
+      </x:c>
+      <x:c r="E35" s="174" t="n">
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="F35" s="174" t="n">
+        <x:v>0.027</x:v>
+      </x:c>
+      <x:c r="G35" s="174" t="n">
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="H35" s="160" t="str">
+        <x:v>Same asset intensity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="158" t="str">
+        <x:v>D&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B36" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C36" s="174" t="n">
+        <x:v>0.031</x:v>
+      </x:c>
+      <x:c r="D36" s="174" t="n">
+        <x:v>0.031</x:v>
+      </x:c>
+      <x:c r="E36" s="174" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="F36" s="174" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="G36" s="174" t="n">
+        <x:v>0.029</x:v>
+      </x:c>
+      <x:c r="H36" s="160" t="str">
+        <x:v>Lower revenue absorption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="158" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="B37" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C37" s="174" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D37" s="174" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E37" s="174" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F37" s="174" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="G37" s="174" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H37" s="160" t="str">
+        <x:v>Normalized rate; FY2025 distorted by discrete items</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="158" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="B38" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C38" s="174" t="n">
+        <x:v>0.195</x:v>
+      </x:c>
+      <x:c r="D38" s="174" t="n">
+        <x:v>0.195</x:v>
+      </x:c>
+      <x:c r="E38" s="174" t="n">
+        <x:v>0.195</x:v>
+      </x:c>
+      <x:c r="F38" s="174" t="n">
+        <x:v>0.195</x:v>
+      </x:c>
+      <x:c r="G38" s="174" t="n">
+        <x:v>0.195</x:v>
+      </x:c>
+      <x:c r="H38" s="160" t="str">
+        <x:v>Modestly favorable jurisdiction mix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="158" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="B39" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C39" s="174" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="D39" s="174" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="E39" s="174" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="F39" s="174" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="G39" s="174" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="H39" s="160" t="str">
+        <x:v>Less favorable jurisdiction mix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="158" t="str">
+        <x:v>Net interest &amp; other % revenue</x:v>
+      </x:c>
+      <x:c r="B40" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C40" s="174" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="D40" s="174" t="n">
+        <x:v>0.013</x:v>
+      </x:c>
+      <x:c r="E40" s="174" t="n">
+        <x:v>0.011</x:v>
+      </x:c>
+      <x:c r="F40" s="174" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="G40" s="174" t="n">
+        <x:v>0.009</x:v>
+      </x:c>
+      <x:c r="H40" s="160" t="str">
+        <x:v>Declines as excess cash is returned or deployed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="158" t="str">
+        <x:v>Net interest &amp; other % revenue</x:v>
+      </x:c>
+      <x:c r="B41" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C41" s="174" t="n">
+        <x:v>0.016</x:v>
+      </x:c>
+      <x:c r="D41" s="174" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="E41" s="174" t="n">
+        <x:v>0.012</x:v>
+      </x:c>
+      <x:c r="F41" s="174" t="n">
+        <x:v>0.011</x:v>
+      </x:c>
+      <x:c r="G41" s="174" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="H41" s="160" t="str">
+        <x:v>Higher cash balances / yields</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="158" t="str">
+        <x:v>Net interest &amp; other % revenue</x:v>
+      </x:c>
+      <x:c r="B42" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C42" s="174" t="n">
+        <x:v>0.012</x:v>
+      </x:c>
+      <x:c r="D42" s="174" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="E42" s="174" t="n">
+        <x:v>0.009</x:v>
+      </x:c>
+      <x:c r="F42" s="174" t="n">
+        <x:v>0.008</x:v>
+      </x:c>
+      <x:c r="G42" s="174" t="n">
+        <x:v>0.007</x:v>
+      </x:c>
+      <x:c r="H42" s="160" t="str">
+        <x:v>Lower cash balances / yields</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="158" t="str">
+        <x:v>Capex % revenue</x:v>
+      </x:c>
+      <x:c r="B43" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C43" s="174" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="D43" s="174" t="n">
+        <x:v>0.016</x:v>
+      </x:c>
+      <x:c r="E43" s="174" t="n">
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="F43" s="174" t="n">
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="G43" s="174" t="n">
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="H43" s="160" t="str">
+        <x:v>Normalized above unusually low FY2025</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="158" t="str">
+        <x:v>Capex % revenue</x:v>
+      </x:c>
+      <x:c r="B44" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C44" s="174" t="n">
+        <x:v>0.014</x:v>
+      </x:c>
+      <x:c r="D44" s="174" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="E44" s="174" t="n">
+        <x:v>0.016</x:v>
+      </x:c>
+      <x:c r="F44" s="174" t="n">
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="G44" s="174" t="n">
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="H44" s="160" t="str">
+        <x:v>Efficient growth investment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="158" t="str">
+        <x:v>Capex % revenue</x:v>
+      </x:c>
+      <x:c r="B45" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C45" s="174" t="n">
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="D45" s="174" t="n">
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="E45" s="174" t="n">
+        <x:v>0.019</x:v>
+      </x:c>
+      <x:c r="F45" s="174" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="G45" s="174" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="H45" s="160" t="str">
+        <x:v>Lower revenue absorption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="158" t="str">
+        <x:v>Operating NWC % revenue</x:v>
+      </x:c>
+      <x:c r="B46" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C46" s="174" t="n">
+        <x:v>0.23</x:v>
+      </x:c>
+      <x:c r="D46" s="174" t="n">
+        <x:v>0.228</x:v>
+      </x:c>
+      <x:c r="E46" s="174" t="n">
+        <x:v>0.225</x:v>
+      </x:c>
+      <x:c r="F46" s="174" t="n">
+        <x:v>0.223</x:v>
+      </x:c>
+      <x:c r="G46" s="174" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="H46" s="160" t="str">
+        <x:v>Near FY2025 with gradual efficiency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="158" t="str">
+        <x:v>Operating NWC % revenue</x:v>
+      </x:c>
+      <x:c r="B47" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C47" s="174" t="n">
+        <x:v>0.225</x:v>
+      </x:c>
+      <x:c r="D47" s="174" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="E47" s="174" t="n">
+        <x:v>0.215</x:v>
+      </x:c>
+      <x:c r="F47" s="174" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="G47" s="174" t="n">
+        <x:v>0.205</x:v>
+      </x:c>
+      <x:c r="H47" s="160" t="str">
+        <x:v>Better collections and inventory turns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="158" t="str">
+        <x:v>Operating NWC % revenue</x:v>
+      </x:c>
+      <x:c r="B48" s="159" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C48" s="174" t="n">
+        <x:v>0.245</x:v>
+      </x:c>
+      <x:c r="D48" s="174" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E48" s="174" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="F48" s="174" t="n">
+        <x:v>0.248</x:v>
+      </x:c>
+      <x:c r="G48" s="174" t="n">
+        <x:v>0.245</x:v>
+      </x:c>
+      <x:c r="H48" s="160" t="str">
+        <x:v>Slower collections and inventory turns</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="158" t="str">
+        <x:v>Diluted share change</x:v>
+      </x:c>
+      <x:c r="B49" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C49" s="174" t="n">
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="D49" s="174" t="n">
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="E49" s="174" t="n">
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="F49" s="174" t="n">
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="G49" s="174" t="n">
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="H49" s="160" t="str">
+        <x:v>Moderate net repurchases</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="158" t="str">
+        <x:v>Diluted share change</x:v>
+      </x:c>
+      <x:c r="B50" s="159" t="str">
+        <x:v>Upside</x:v>
+      </x:c>
+      <x:c r="C50" s="174" t="n">
+        <x:v>-0.012</x:v>
+      </x:c>
+      <x:c r="D50" s="174" t="n">
+        <x:v>-0.012</x:v>
+      </x:c>
+      <x:c r="E50" s="174" t="n">
+        <x:v>-0.012</x:v>
+      </x:c>
+      <x:c r="F50" s="174" t="n">
+        <x:v>-0.012</x:v>
+      </x:c>
+      <x:c r="G50" s="174" t="n">
+        <x:v>-0.012</x:v>
+      </x:c>
+      <x:c r="H50" s="160" t="str">
+        <x:v>Stronger repurchase capacity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="161" t="str">
+        <x:v>Diluted share change</x:v>
+      </x:c>
+      <x:c r="B51" s="162" t="str">
+        <x:v>Downside</x:v>
+      </x:c>
+      <x:c r="C51" s="175" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D51" s="175" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E51" s="175" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F51" s="175" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G51" s="175" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H51" s="163" t="str">
+        <x:v>Preserve liquidity; SBC offsets repurchases</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="139" t="str">
+        <x:v>ROK BUYER FORECAST ASSUMPTIONS — BASE CASE</x:v>
+      </x:c>
+      <x:c r="B54" s="139"/>
+      <x:c r="C54" s="139"/>
+      <x:c r="D54" s="139"/>
+      <x:c r="E54" s="139"/>
+      <x:c r="F54" s="139"/>
+      <x:c r="G54" s="139"/>
+      <x:c r="H54" s="139"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="144" t="str">
+        <x:v>Driver</x:v>
+      </x:c>
+      <x:c r="B55" s="144" t="str">
+        <x:v>Case</x:v>
+      </x:c>
+      <x:c r="C55" s="144" t="str">
+        <x:v>FY2026E</x:v>
+      </x:c>
+      <x:c r="D55" s="144" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="E55" s="144" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="F55" s="144" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="G55" s="144" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="H55" s="144" t="str">
+        <x:v>Source / rationale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="155" t="str">
+        <x:v>Revenue growth</x:v>
+      </x:c>
+      <x:c r="B56" s="156" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C56" s="173" t="n">
+        <x:v>0.085</x:v>
+      </x:c>
+      <x:c r="D56" s="173" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="E56" s="173" t="n">
+        <x:v>0.045</x:v>
+      </x:c>
+      <x:c r="F56" s="173" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="G56" s="173" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="H56" s="157" t="str">
+        <x:v>FY2026: S-018 guidance midpoint; outer years normalize</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="158" t="str">
+        <x:v>Enterprise operating margin</x:v>
+      </x:c>
+      <x:c r="B57" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C57" s="174" t="n">
+        <x:v>0.215</x:v>
+      </x:c>
+      <x:c r="D57" s="174" t="n">
+        <x:v>0.217</x:v>
+      </x:c>
+      <x:c r="E57" s="174" t="n">
+        <x:v>0.219</x:v>
+      </x:c>
+      <x:c r="F57" s="174" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="G57" s="174" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="H57" s="160" t="str">
+        <x:v>FY2026: S-018; modest longer-term expansion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="158" t="str">
+        <x:v>Adjusted diluted EPS</x:v>
+      </x:c>
+      <x:c r="B58" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C58" s="176" t="n">
+        <x:v>13.15</x:v>
+      </x:c>
+      <x:c r="D58" s="176"/>
+      <x:c r="E58" s="176"/>
+      <x:c r="F58" s="176"/>
+      <x:c r="G58" s="176"/>
+      <x:c r="H58" s="160" t="str">
+        <x:v>FY2026: S-018 guidance midpoint</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="158" t="str">
+        <x:v>Adjusted EPS growth</x:v>
+      </x:c>
+      <x:c r="B59" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C59" s="174"/>
+      <x:c r="D59" s="174" t="n">
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="E59" s="174" t="n">
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="F59" s="174" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="G59" s="174" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="H59" s="160" t="str">
+        <x:v>Outer years: analyst assumption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="158" t="str">
+        <x:v>Diluted share change</x:v>
+      </x:c>
+      <x:c r="B60" s="159" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C60" s="174" t="n">
+        <x:v>-0.008</x:v>
+      </x:c>
+      <x:c r="D60" s="174" t="n">
+        <x:v>-0.008</x:v>
+      </x:c>
+      <x:c r="E60" s="174" t="n">
+        <x:v>-0.008</x:v>
+      </x:c>
+      <x:c r="F60" s="174" t="n">
+        <x:v>-0.008</x:v>
+      </x:c>
+      <x:c r="G60" s="174" t="n">
+        <x:v>-0.008</x:v>
+      </x:c>
+      <x:c r="H60" s="160" t="str">
+        <x:v>Moderate net repurchases</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="161" t="str">
+        <x:v>FCF conversion</x:v>
+      </x:c>
+      <x:c r="B61" s="162" t="str">
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="C61" s="175" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D61" s="175" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E61" s="175" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F61" s="175" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G61" s="175" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H61" s="163" t="str">
+        <x:v>FY2026: management outlook; held constant</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2552,6 +3986,8 @@
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A3:D3"/>
     <x:mergeCell ref="A12:D12"/>
+    <x:mergeCell ref="A20:H20"/>
+    <x:mergeCell ref="A54:H54"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B5">
@@ -4190,7 +5626,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaeefc80b35a43fe"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4027c3524d5d43df"/>
 </x:worksheet>
 </file>
 
@@ -5913,7 +7349,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dbee3a662d94c33"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R438496ca798f4fce"/>
 </x:worksheet>
 </file>
 
@@ -5921,110 +7357,1638 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="25" customHeight="1">
+      <x:c r="A1" s="238" t="str">
         <x:v>CGNX Operating Model</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Cognex five-year driver-based forecast</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="238"/>
+      <x:c r="C1" s="238"/>
+      <x:c r="D1" s="238"/>
+      <x:c r="E1" s="238"/>
+      <x:c r="F1" s="238"/>
+      <x:c r="G1" s="238"/>
+      <x:c r="H1" s="238"/>
+      <x:c r="I1" s="238"/>
+      <x:c r="J1" s="238"/>
+    </x:row>
+    <x:row r="2" ht="20" customHeight="1">
+      <x:c r="A2" s="181" t="str">
+        <x:v>Cognex five-year driver-based forecast | USD millions, except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="181"/>
+      <x:c r="C2" s="181"/>
+      <x:c r="D2" s="181"/>
+      <x:c r="E2" s="181"/>
+      <x:c r="F2" s="181"/>
+      <x:c r="G2" s="181"/>
+      <x:c r="H2" s="181"/>
+      <x:c r="I2" s="181"/>
+      <x:c r="J2" s="181"/>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="183" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
-    </x:row>
+      <x:c r="B3" s="183" t="str">
+        <x:v>Complete — scenario-driven FY2026E to FY2030E forecast</x:v>
+      </x:c>
+      <x:c r="C3" s="183"/>
+      <x:c r="D3" s="183"/>
+      <x:c r="E3" s="183"/>
+      <x:c r="F3" s="183"/>
+      <x:c r="G3" s="183"/>
+      <x:c r="H3" s="183"/>
+      <x:c r="I3" s="183"/>
+      <x:c r="J3" s="183"/>
+    </x:row>
+    <x:row r="4" ht="16" customHeight="1"/>
+    <x:row r="5" ht="16" customHeight="1">
+      <x:c r="A5" s="139" t="str">
+        <x:v>ACTIVE FORECAST DRIVERS</x:v>
+      </x:c>
+      <x:c r="B5" s="139"/>
+      <x:c r="C5" s="139"/>
+      <x:c r="D5" s="139"/>
+      <x:c r="E5" s="139"/>
+      <x:c r="F5" s="139"/>
+      <x:c r="G5" s="139"/>
+      <x:c r="H5" s="139"/>
+      <x:c r="I5" s="139"/>
+      <x:c r="J5" s="139"/>
+    </x:row>
+    <x:row r="6" ht="16" customHeight="1">
+      <x:c r="A6" s="144" t="str">
+        <x:v>Driver</x:v>
+      </x:c>
+      <x:c r="B6" s="144" t="str">
+        <x:v>FY2026E</x:v>
+      </x:c>
+      <x:c r="C6" s="144" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="D6" s="144" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="E6" s="144" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="F6" s="144" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="G6" s="144" t="str">
+        <x:v>Selected case / methodology</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="16" customHeight="1">
+      <x:c r="A7" s="184" t="str">
+        <x:v>Revenue growth</x:v>
+      </x:c>
+      <x:c r="B7" s="199" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C23,IF('Control'!$B$5="Downside",'Control'!C24,'Control'!C22))</x:f>
+        <x:v>0.14646722159702885</x:v>
+      </x:c>
+      <x:c r="C7" s="199" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D23,IF('Control'!$B$5="Downside",'Control'!D24,'Control'!D22))</x:f>
+        <x:v>0.09</x:v>
+      </x:c>
+      <x:c r="D7" s="199" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E23,IF('Control'!$B$5="Downside",'Control'!E24,'Control'!E22))</x:f>
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="E7" s="199" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F23,IF('Control'!$B$5="Downside",'Control'!F24,'Control'!F22))</x:f>
+        <x:v>0.07</x:v>
+      </x:c>
+      <x:c r="F7" s="199" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G23,IF('Control'!$B$5="Downside",'Control'!G24,'Control'!G22))</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="G7" s="202" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="16" customHeight="1">
+      <x:c r="A8" s="187" t="str">
+        <x:v>Gross margin</x:v>
+      </x:c>
+      <x:c r="B8" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C26,IF('Control'!$B$5="Downside",'Control'!C27,'Control'!C25))</x:f>
+        <x:v>0.705</x:v>
+      </x:c>
+      <x:c r="C8" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D26,IF('Control'!$B$5="Downside",'Control'!D27,'Control'!D25))</x:f>
+        <x:v>0.707</x:v>
+      </x:c>
+      <x:c r="D8" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E26,IF('Control'!$B$5="Downside",'Control'!E27,'Control'!E25))</x:f>
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="E8" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F26,IF('Control'!$B$5="Downside",'Control'!F27,'Control'!F25))</x:f>
+        <x:v>0.712</x:v>
+      </x:c>
+      <x:c r="F8" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G26,IF('Control'!$B$5="Downside",'Control'!G27,'Control'!G25))</x:f>
+        <x:v>0.713</x:v>
+      </x:c>
+      <x:c r="G8" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="16" customHeight="1">
+      <x:c r="A9" s="187" t="str">
+        <x:v>R&amp;D % revenue</x:v>
+      </x:c>
+      <x:c r="B9" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C29,IF('Control'!$B$5="Downside",'Control'!C30,'Control'!C28))</x:f>
+        <x:v>0.135</x:v>
+      </x:c>
+      <x:c r="C9" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D29,IF('Control'!$B$5="Downside",'Control'!D30,'Control'!D28))</x:f>
+        <x:v>0.134</x:v>
+      </x:c>
+      <x:c r="D9" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E29,IF('Control'!$B$5="Downside",'Control'!E30,'Control'!E28))</x:f>
+        <x:v>0.133</x:v>
+      </x:c>
+      <x:c r="E9" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F29,IF('Control'!$B$5="Downside",'Control'!F30,'Control'!F28))</x:f>
+        <x:v>0.132</x:v>
+      </x:c>
+      <x:c r="F9" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G29,IF('Control'!$B$5="Downside",'Control'!G30,'Control'!G28))</x:f>
+        <x:v>0.132</x:v>
+      </x:c>
+      <x:c r="G9" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="16" customHeight="1">
+      <x:c r="A10" s="187" t="str">
+        <x:v>SG&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B10" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C32,IF('Control'!$B$5="Downside",'Control'!C33,'Control'!C31))</x:f>
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="C10" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D32,IF('Control'!$B$5="Downside",'Control'!D33,'Control'!D31))</x:f>
+        <x:v>0.305</x:v>
+      </x:c>
+      <x:c r="D10" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E32,IF('Control'!$B$5="Downside",'Control'!E33,'Control'!E31))</x:f>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E10" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F32,IF('Control'!$B$5="Downside",'Control'!F33,'Control'!F31))</x:f>
+        <x:v>0.295</x:v>
+      </x:c>
+      <x:c r="F10" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G32,IF('Control'!$B$5="Downside",'Control'!G33,'Control'!G31))</x:f>
+        <x:v>0.292</x:v>
+      </x:c>
+      <x:c r="G10" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="16" customHeight="1">
+      <x:c r="A11" s="187" t="str">
+        <x:v>D&amp;A % revenue</x:v>
+      </x:c>
+      <x:c r="B11" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C35,IF('Control'!$B$5="Downside",'Control'!C36,'Control'!C34))</x:f>
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="C11" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D35,IF('Control'!$B$5="Downside",'Control'!D36,'Control'!D34))</x:f>
+        <x:v>0.029</x:v>
+      </x:c>
+      <x:c r="D11" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E35,IF('Control'!$B$5="Downside",'Control'!E36,'Control'!E34))</x:f>
+        <x:v>0.028</x:v>
+      </x:c>
+      <x:c r="E11" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F35,IF('Control'!$B$5="Downside",'Control'!F36,'Control'!F34))</x:f>
+        <x:v>0.027</x:v>
+      </x:c>
+      <x:c r="F11" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G35,IF('Control'!$B$5="Downside",'Control'!G36,'Control'!G34))</x:f>
+        <x:v>0.026</x:v>
+      </x:c>
+      <x:c r="G11" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+      <x:c r="H11"/>
+    </x:row>
+    <x:row r="12" ht="16" customHeight="1">
+      <x:c r="A12" s="187" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="B12" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C38,IF('Control'!$B$5="Downside",'Control'!C39,'Control'!C37))</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="C12" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D38,IF('Control'!$B$5="Downside",'Control'!D39,'Control'!D37))</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D12" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E38,IF('Control'!$B$5="Downside",'Control'!E39,'Control'!E37))</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E12" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F38,IF('Control'!$B$5="Downside",'Control'!F39,'Control'!F37))</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="F12" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G38,IF('Control'!$B$5="Downside",'Control'!G39,'Control'!G37))</x:f>
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="G12" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="16" customHeight="1">
+      <x:c r="A13" s="187" t="str">
+        <x:v>Net interest &amp; other % revenue</x:v>
+      </x:c>
+      <x:c r="B13" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C41,IF('Control'!$B$5="Downside",'Control'!C42,'Control'!C40))</x:f>
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="C13" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D41,IF('Control'!$B$5="Downside",'Control'!D42,'Control'!D40))</x:f>
+        <x:v>0.013</x:v>
+      </x:c>
+      <x:c r="D13" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E41,IF('Control'!$B$5="Downside",'Control'!E42,'Control'!E40))</x:f>
+        <x:v>0.011</x:v>
+      </x:c>
+      <x:c r="E13" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F41,IF('Control'!$B$5="Downside",'Control'!F42,'Control'!F40))</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F13" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G41,IF('Control'!$B$5="Downside",'Control'!G42,'Control'!G40))</x:f>
+        <x:v>0.009</x:v>
+      </x:c>
+      <x:c r="G13" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="16" customHeight="1">
+      <x:c r="A14" s="187" t="str">
+        <x:v>Capex % revenue</x:v>
+      </x:c>
+      <x:c r="B14" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C44,IF('Control'!$B$5="Downside",'Control'!C45,'Control'!C43))</x:f>
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="C14" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D44,IF('Control'!$B$5="Downside",'Control'!D45,'Control'!D43))</x:f>
+        <x:v>0.016</x:v>
+      </x:c>
+      <x:c r="D14" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E44,IF('Control'!$B$5="Downside",'Control'!E45,'Control'!E43))</x:f>
+        <x:v>0.017</x:v>
+      </x:c>
+      <x:c r="E14" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F44,IF('Control'!$B$5="Downside",'Control'!F45,'Control'!F43))</x:f>
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="F14" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G44,IF('Control'!$B$5="Downside",'Control'!G45,'Control'!G43))</x:f>
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="G14" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="16" customHeight="1">
+      <x:c r="A15" s="187" t="str">
+        <x:v>Operating NWC % revenue</x:v>
+      </x:c>
+      <x:c r="B15" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C47,IF('Control'!$B$5="Downside",'Control'!C48,'Control'!C46))</x:f>
+        <x:v>0.23</x:v>
+      </x:c>
+      <x:c r="C15" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D47,IF('Control'!$B$5="Downside",'Control'!D48,'Control'!D46))</x:f>
+        <x:v>0.228</x:v>
+      </x:c>
+      <x:c r="D15" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E47,IF('Control'!$B$5="Downside",'Control'!E48,'Control'!E46))</x:f>
+        <x:v>0.225</x:v>
+      </x:c>
+      <x:c r="E15" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F47,IF('Control'!$B$5="Downside",'Control'!F48,'Control'!F46))</x:f>
+        <x:v>0.223</x:v>
+      </x:c>
+      <x:c r="F15" s="200" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G47,IF('Control'!$B$5="Downside",'Control'!G48,'Control'!G46))</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="G15" s="203" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="16" customHeight="1">
+      <x:c r="A16" s="190" t="str">
+        <x:v>Diluted share change</x:v>
+      </x:c>
+      <x:c r="B16" s="201" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!C50,IF('Control'!$B$5="Downside",'Control'!C51,'Control'!C49))</x:f>
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="C16" s="201" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!D50,IF('Control'!$B$5="Downside",'Control'!D51,'Control'!D49))</x:f>
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="D16" s="201" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!E50,IF('Control'!$B$5="Downside",'Control'!E51,'Control'!E49))</x:f>
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="E16" s="201" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!F50,IF('Control'!$B$5="Downside",'Control'!F51,'Control'!F49))</x:f>
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="F16" s="201" t="n">
+        <x:f>IF('Control'!$B$5="Upside",'Control'!G50,IF('Control'!$B$5="Downside",'Control'!G51,'Control'!G49))</x:f>
+        <x:v>-0.01</x:v>
+      </x:c>
+      <x:c r="G16" s="204" t="str">
+        <x:f>'Control'!$B$5</x:f>
+        <x:v>Base</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="16" customHeight="1"/>
+    <x:row r="18" ht="16" customHeight="1">
+      <x:c r="A18" s="139" t="str">
+        <x:v>INCOME STATEMENT AND PROFITABILITY</x:v>
+      </x:c>
+      <x:c r="B18" s="139"/>
+      <x:c r="C18" s="139"/>
+      <x:c r="D18" s="139"/>
+      <x:c r="E18" s="139"/>
+      <x:c r="F18" s="139"/>
+      <x:c r="G18" s="139"/>
+      <x:c r="H18" s="139"/>
+      <x:c r="I18" s="139"/>
+      <x:c r="J18" s="139"/>
+    </x:row>
+    <x:row r="19" ht="16" customHeight="1">
+      <x:c r="A19" s="223" t="str">
+        <x:v>Fiscal year</x:v>
+      </x:c>
+      <x:c r="B19" s="224" t="str">
+        <x:v>FY2023A</x:v>
+      </x:c>
+      <x:c r="C19" s="224" t="str">
+        <x:v>FY2024A</x:v>
+      </x:c>
+      <x:c r="D19" s="224" t="str">
+        <x:v>FY2025A</x:v>
+      </x:c>
+      <x:c r="E19" s="224" t="str">
+        <x:v>FY2026E</x:v>
+      </x:c>
+      <x:c r="F19" s="224" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="G19" s="224" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="H19" s="224" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="I19" s="224" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="J19" s="225" t="str">
+        <x:v>Source / methodology</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="16" customHeight="1">
+      <x:c r="A20" s="149" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B20" s="226" t="n">
+        <x:f>'CGNX Historical'!D7</x:f>
+        <x:v>837.547</x:v>
+      </x:c>
+      <x:c r="C20" s="226" t="n">
+        <x:f>'CGNX Historical'!E7</x:f>
+        <x:v>914.515</x:v>
+      </x:c>
+      <x:c r="D20" s="226" t="n">
+        <x:f>'CGNX Historical'!F7</x:f>
+        <x:v>994.359</x:v>
+      </x:c>
+      <x:c r="E20" s="227" t="n">
+        <x:f>D20*(1+E21)</x:f>
+        <x:v>1140</x:v>
+      </x:c>
+      <x:c r="F20" s="227" t="n">
+        <x:f>E20*(1+F21)</x:f>
+        <x:v>1242.6000000000001</x:v>
+      </x:c>
+      <x:c r="G20" s="227" t="n">
+        <x:f>F20*(1+G21)</x:f>
+        <x:v>1342.0080000000003</x:v>
+      </x:c>
+      <x:c r="H20" s="227" t="n">
+        <x:f>G20*(1+H21)</x:f>
+        <x:v>1435.9485600000003</x:v>
+      </x:c>
+      <x:c r="I20" s="227" t="n">
+        <x:f>H20*(1+I21)</x:f>
+        <x:v>1529.2852164000003</x:v>
+      </x:c>
+      <x:c r="J20" s="189" t="str">
+        <x:v>FY2026 S-022 midpoint; outer years scenario assumptions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="16" customHeight="1">
+      <x:c r="A21" s="149" t="str">
+        <x:v>% growth</x:v>
+      </x:c>
+      <x:c r="B21" s="200" t="n">
+        <x:f>'CGNX Historical'!D8</x:f>
+        <x:v>-0.16752278623184802</x:v>
+      </x:c>
+      <x:c r="C21" s="200" t="n">
+        <x:f>'CGNX Historical'!E8</x:f>
+        <x:v>0.09189693235125906</x:v>
+      </x:c>
+      <x:c r="D21" s="200" t="n">
+        <x:f>'CGNX Historical'!F8</x:f>
+        <x:v>0.08730747992105115</x:v>
+      </x:c>
+      <x:c r="E21" s="228" t="n">
+        <x:f>B7</x:f>
+        <x:v>0.14646722159702885</x:v>
+      </x:c>
+      <x:c r="F21" s="228" t="n">
+        <x:f>C7</x:f>
+        <x:v>0.09</x:v>
+      </x:c>
+      <x:c r="G21" s="228" t="n">
+        <x:f>D7</x:f>
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="H21" s="228" t="n">
+        <x:f>E7</x:f>
+        <x:v>0.07</x:v>
+      </x:c>
+      <x:c r="I21" s="228" t="n">
+        <x:f>F7</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="J21" s="189" t="str">
+        <x:v>Active selected case</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="16" customHeight="1">
+      <x:c r="A22" s="149" t="str">
+        <x:v>Cost of goods sold</x:v>
+      </x:c>
+      <x:c r="B22" s="226" t="n">
+        <x:f>'CGNX Historical'!D9</x:f>
+        <x:v>236.306</x:v>
+      </x:c>
+      <x:c r="C22" s="226" t="n">
+        <x:f>'CGNX Historical'!E9</x:f>
+        <x:v>288.721</x:v>
+      </x:c>
+      <x:c r="D22" s="226" t="n">
+        <x:f>'CGNX Historical'!F9</x:f>
+        <x:v>328.966</x:v>
+      </x:c>
+      <x:c r="E22" s="227" t="n">
+        <x:f>E20*(1-E24)</x:f>
+        <x:v>336.30000000000007</x:v>
+      </x:c>
+      <x:c r="F22" s="227" t="n">
+        <x:f>F20*(1-F24)</x:f>
+        <x:v>364.0818000000001</x:v>
+      </x:c>
+      <x:c r="G22" s="227" t="n">
+        <x:f>G20*(1-G24)</x:f>
+        <x:v>389.1823200000001</x:v>
+      </x:c>
+      <x:c r="H22" s="227" t="n">
+        <x:f>H20*(1-H24)</x:f>
+        <x:v>413.55318528000015</x:v>
+      </x:c>
+      <x:c r="I22" s="227" t="n">
+        <x:f>I20*(1-I24)</x:f>
+        <x:v>438.90485710680014</x:v>
+      </x:c>
+      <x:c r="J22" s="189" t="str">
+        <x:v>Revenue less gross profit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="16" customHeight="1">
+      <x:c r="A23" s="149" t="str">
+        <x:v>Gross profit</x:v>
+      </x:c>
+      <x:c r="B23" s="226" t="n">
+        <x:f>'CGNX Historical'!D10</x:f>
+        <x:v>601.241</x:v>
+      </x:c>
+      <x:c r="C23" s="226" t="n">
+        <x:f>'CGNX Historical'!E10</x:f>
+        <x:v>625.794</x:v>
+      </x:c>
+      <x:c r="D23" s="226" t="n">
+        <x:f>'CGNX Historical'!F10</x:f>
+        <x:v>665.393</x:v>
+      </x:c>
+      <x:c r="E23" s="227" t="n">
+        <x:f>E20-E22</x:f>
+        <x:v>803.6999999999999</x:v>
+      </x:c>
+      <x:c r="F23" s="227" t="n">
+        <x:f>F20-F22</x:f>
+        <x:v>878.5182</x:v>
+      </x:c>
+      <x:c r="G23" s="227" t="n">
+        <x:f>G20-G22</x:f>
+        <x:v>952.8256800000001</x:v>
+      </x:c>
+      <x:c r="H23" s="227" t="n">
+        <x:f>H20-H22</x:f>
+        <x:v>1022.3953747200001</x:v>
+      </x:c>
+      <x:c r="I23" s="227" t="n">
+        <x:f>I20-I22</x:f>
+        <x:v>1090.3803592932002</x:v>
+      </x:c>
+      <x:c r="J23" s="189" t="str">
+        <x:v>Revenue less COGS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="16" customHeight="1">
+      <x:c r="A24" s="149" t="str">
+        <x:v>Gross margin</x:v>
+      </x:c>
+      <x:c r="B24" s="200" t="n">
+        <x:f>'CGNX Historical'!D13</x:f>
+        <x:v>0.7178594156507038</x:v>
+      </x:c>
+      <x:c r="C24" s="200" t="n">
+        <x:f>'CGNX Historical'!E13</x:f>
+        <x:v>0.6842905802529209</x:v>
+      </x:c>
+      <x:c r="D24" s="200" t="n">
+        <x:f>'CGNX Historical'!F13</x:f>
+        <x:v>0.6691677754211507</x:v>
+      </x:c>
+      <x:c r="E24" s="228" t="n">
+        <x:f>B8</x:f>
+        <x:v>0.705</x:v>
+      </x:c>
+      <x:c r="F24" s="228" t="n">
+        <x:f>C8</x:f>
+        <x:v>0.707</x:v>
+      </x:c>
+      <x:c r="G24" s="228" t="n">
+        <x:f>D8</x:f>
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="H24" s="228" t="n">
+        <x:f>E8</x:f>
+        <x:v>0.712</x:v>
+      </x:c>
+      <x:c r="I24" s="228" t="n">
+        <x:f>F8</x:f>
+        <x:v>0.713</x:v>
+      </x:c>
+      <x:c r="J24" s="189" t="str">
+        <x:v>Active selected case</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="16" customHeight="1">
+      <x:c r="A25" s="149" t="str">
+        <x:v>R&amp;D expense</x:v>
+      </x:c>
+      <x:c r="B25" s="226" t="n">
+        <x:f>'CGNX Historical'!D15</x:f>
+        <x:v>139.4</x:v>
+      </x:c>
+      <x:c r="C25" s="226" t="n">
+        <x:f>'CGNX Historical'!E15</x:f>
+        <x:v>139.815</x:v>
+      </x:c>
+      <x:c r="D25" s="226" t="n">
+        <x:f>'CGNX Historical'!F15</x:f>
+        <x:v>138.97</x:v>
+      </x:c>
+      <x:c r="E25" s="227" t="n">
+        <x:f>E20*E26</x:f>
+        <x:v>153.9</x:v>
+      </x:c>
+      <x:c r="F25" s="227" t="n">
+        <x:f>F20*F26</x:f>
+        <x:v>166.50840000000002</x:v>
+      </x:c>
+      <x:c r="G25" s="227" t="n">
+        <x:f>G20*G26</x:f>
+        <x:v>178.48706400000003</x:v>
+      </x:c>
+      <x:c r="H25" s="227" t="n">
+        <x:f>H20*H26</x:f>
+        <x:v>189.54520992000005</x:v>
+      </x:c>
+      <x:c r="I25" s="227" t="n">
+        <x:f>I20*I26</x:f>
+        <x:v>201.86564856480004</x:v>
+      </x:c>
+      <x:c r="J25" s="189" t="str">
+        <x:v>Revenue × R&amp;D %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="16" customHeight="1">
+      <x:c r="A26" s="149" t="str">
+        <x:v>% revenue</x:v>
+      </x:c>
+      <x:c r="B26" s="200" t="n">
+        <x:f>'CGNX Historical'!D16</x:f>
+        <x:v>0.1664384207692225</x:v>
+      </x:c>
+      <x:c r="C26" s="200" t="n">
+        <x:f>'CGNX Historical'!E16</x:f>
+        <x:v>0.15288431573019579</x:v>
+      </x:c>
+      <x:c r="D26" s="200" t="n">
+        <x:f>'CGNX Historical'!F16</x:f>
+        <x:v>0.1397583770046834</x:v>
+      </x:c>
+      <x:c r="E26" s="228" t="n">
+        <x:f>B9</x:f>
+        <x:v>0.135</x:v>
+      </x:c>
+      <x:c r="F26" s="228" t="n">
+        <x:f>C9</x:f>
+        <x:v>0.134</x:v>
+      </x:c>
+      <x:c r="G26" s="228" t="n">
+        <x:f>D9</x:f>
+        <x:v>0.133</x:v>
+      </x:c>
+      <x:c r="H26" s="228" t="n">
+        <x:f>E9</x:f>
+        <x:v>0.132</x:v>
+      </x:c>
+      <x:c r="I26" s="228" t="n">
+        <x:f>F9</x:f>
+        <x:v>0.132</x:v>
+      </x:c>
+      <x:c r="J26" s="189" t="str">
+        <x:v>Active selected case</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="16" customHeight="1">
+      <x:c r="A27" s="149" t="str">
+        <x:v>SG&amp;A expense</x:v>
+      </x:c>
+      <x:c r="B27" s="226" t="n">
+        <x:f>'CGNX Historical'!D17</x:f>
+        <x:v>339.139</x:v>
+      </x:c>
+      <x:c r="C27" s="226" t="n">
+        <x:f>'CGNX Historical'!E17</x:f>
+        <x:v>370.914</x:v>
+      </x:c>
+      <x:c r="D27" s="226" t="n">
+        <x:f>'CGNX Historical'!F17</x:f>
+        <x:v>363.857</x:v>
+      </x:c>
+      <x:c r="E27" s="227" t="n">
+        <x:f>E20*E28</x:f>
+        <x:v>353.4</x:v>
+      </x:c>
+      <x:c r="F27" s="227" t="n">
+        <x:f>F20*F28</x:f>
+        <x:v>378.99300000000005</x:v>
+      </x:c>
+      <x:c r="G27" s="227" t="n">
+        <x:f>G20*G28</x:f>
+        <x:v>402.60240000000005</x:v>
+      </x:c>
+      <x:c r="H27" s="227" t="n">
+        <x:f>H20*H28</x:f>
+        <x:v>423.60482520000005</x:v>
+      </x:c>
+      <x:c r="I27" s="227" t="n">
+        <x:f>I20*I28</x:f>
+        <x:v>446.5512831888001</x:v>
+      </x:c>
+      <x:c r="J27" s="189" t="str">
+        <x:v>Revenue × SG&amp;A %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="16" customHeight="1">
+      <x:c r="A28" s="149" t="str">
+        <x:v>% revenue</x:v>
+      </x:c>
+      <x:c r="B28" s="200" t="n">
+        <x:f>'CGNX Historical'!D18</x:f>
+        <x:v>0.4049193657191775</x:v>
+      </x:c>
+      <x:c r="C28" s="200" t="n">
+        <x:f>'CGNX Historical'!E18</x:f>
+        <x:v>0.4055854742677813</x:v>
+      </x:c>
+      <x:c r="D28" s="200" t="n">
+        <x:f>'CGNX Historical'!F18</x:f>
+        <x:v>0.3659211612707282</x:v>
+      </x:c>
+      <x:c r="E28" s="228" t="n">
+        <x:f>B10</x:f>
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="F28" s="228" t="n">
+        <x:f>C10</x:f>
+        <x:v>0.305</x:v>
+      </x:c>
+      <x:c r="G28" s="228" t="n">
+        <x:f>D10</x:f>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="H28" s="228" t="n">
+        <x:f>E10</x:f>
+        <x:v>0.295</x:v>
+      </x:c>
+      <x:c r="I28" s="228" t="n">
+        <x:f>F10</x:f>
+        <x:v>0.292</x:v>
+      </x:c>
+      <x:c r="J28" s="189" t="str">
+        <x:v>Active selected case</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="16" customHeight="1">
+      <x:c r="A29" s="240" t="str">
+        <x:v>Operating income</x:v>
+      </x:c>
+      <x:c r="B29" s="241" t="n">
+        <x:f>'CGNX Historical'!D19</x:f>
+        <x:v>130.702</x:v>
+      </x:c>
+      <x:c r="C29" s="241" t="n">
+        <x:f>'CGNX Historical'!E19</x:f>
+        <x:v>115.065</x:v>
+      </x:c>
+      <x:c r="D29" s="241" t="n">
+        <x:f>'CGNX Historical'!F19</x:f>
+        <x:v>162.566</x:v>
+      </x:c>
+      <x:c r="E29" s="241" t="n">
+        <x:f>E23-E25-E27</x:f>
+        <x:v>296.4</x:v>
+      </x:c>
+      <x:c r="F29" s="241" t="n">
+        <x:f>F23-F25-F27</x:f>
+        <x:v>333.0167999999999</x:v>
+      </x:c>
+      <x:c r="G29" s="241" t="n">
+        <x:f>G23-G25-G27</x:f>
+        <x:v>371.73621600000007</x:v>
+      </x:c>
+      <x:c r="H29" s="241" t="n">
+        <x:f>H23-H25-H27</x:f>
+        <x:v>409.24533959999997</x:v>
+      </x:c>
+      <x:c r="I29" s="241" t="n">
+        <x:f>I23-I25-I27</x:f>
+        <x:v>441.96342753960005</x:v>
+      </x:c>
+      <x:c r="J29" s="189" t="str">
+        <x:v>Gross profit less R&amp;D and SG&amp;A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="16" customHeight="1">
+      <x:c r="A30" s="240" t="str">
+        <x:v>Operating margin</x:v>
+      </x:c>
+      <x:c r="B30" s="242" t="n">
+        <x:f>'CGNX Historical'!D20</x:f>
+        <x:v>0.1560533319324169</x:v>
+      </x:c>
+      <x:c r="C30" s="242" t="n">
+        <x:f>'CGNX Historical'!E20</x:f>
+        <x:v>0.1258207902549439</x:v>
+      </x:c>
+      <x:c r="D30" s="242" t="n">
+        <x:f>'CGNX Historical'!F20</x:f>
+        <x:v>0.16348823714573912</x:v>
+      </x:c>
+      <x:c r="E30" s="242" t="n">
+        <x:f>E29/E20</x:f>
+        <x:v>0.25999999999999995</x:v>
+      </x:c>
+      <x:c r="F30" s="242" t="n">
+        <x:f>F29/F20</x:f>
+        <x:v>0.26799999999999985</x:v>
+      </x:c>
+      <x:c r="G30" s="242" t="n">
+        <x:f>G29/G20</x:f>
+        <x:v>0.277</x:v>
+      </x:c>
+      <x:c r="H30" s="242" t="n">
+        <x:f>H29/H20</x:f>
+        <x:v>0.2849999999999999</x:v>
+      </x:c>
+      <x:c r="I30" s="242" t="n">
+        <x:f>I29/I20</x:f>
+        <x:v>0.289</x:v>
+      </x:c>
+      <x:c r="J30" s="189" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="16" customHeight="1">
+      <x:c r="A31" s="149" t="str">
+        <x:v>Depreciation &amp; amortization</x:v>
+      </x:c>
+      <x:c r="B31" s="226" t="n">
+        <x:f>'CGNX Historical'!D37</x:f>
+        <x:v>21.88</x:v>
+      </x:c>
+      <x:c r="C31" s="226" t="n">
+        <x:f>'CGNX Historical'!E37</x:f>
+        <x:v>32.689</x:v>
+      </x:c>
+      <x:c r="D31" s="226" t="n">
+        <x:f>'CGNX Historical'!F37</x:f>
+        <x:v>30.793</x:v>
+      </x:c>
+      <x:c r="E31" s="227" t="n">
+        <x:f>E20*B11</x:f>
+        <x:v>34.199999999999996</x:v>
+      </x:c>
+      <x:c r="F31" s="227" t="n">
+        <x:f>F20*C11</x:f>
+        <x:v>36.0354</x:v>
+      </x:c>
+      <x:c r="G31" s="227" t="n">
+        <x:f>G20*D11</x:f>
+        <x:v>37.57622400000001</x:v>
+      </x:c>
+      <x:c r="H31" s="227" t="n">
+        <x:f>H20*E11</x:f>
+        <x:v>38.770611120000005</x:v>
+      </x:c>
+      <x:c r="I31" s="227" t="n">
+        <x:f>I20*F11</x:f>
+        <x:v>39.76141562640001</x:v>
+      </x:c>
+      <x:c r="J31" s="189" t="str">
+        <x:v>Revenue × D&amp;A %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="16" customHeight="1">
+      <x:c r="A32" s="240" t="str">
+        <x:v>EBITDA</x:v>
+      </x:c>
+      <x:c r="B32" s="241" t="n">
+        <x:f>B29+B31</x:f>
+        <x:v>152.582</x:v>
+      </x:c>
+      <x:c r="C32" s="241" t="n">
+        <x:f>C29+C31</x:f>
+        <x:v>147.754</x:v>
+      </x:c>
+      <x:c r="D32" s="241" t="n">
+        <x:f>D29+D31</x:f>
+        <x:v>193.359</x:v>
+      </x:c>
+      <x:c r="E32" s="241" t="n">
+        <x:f>E29+E31</x:f>
+        <x:v>330.59999999999997</x:v>
+      </x:c>
+      <x:c r="F32" s="241" t="n">
+        <x:f>F29+F31</x:f>
+        <x:v>369.05219999999986</x:v>
+      </x:c>
+      <x:c r="G32" s="241" t="n">
+        <x:f>G29+G31</x:f>
+        <x:v>409.3124400000001</x:v>
+      </x:c>
+      <x:c r="H32" s="241" t="n">
+        <x:f>H29+H31</x:f>
+        <x:v>448.01595072</x:v>
+      </x:c>
+      <x:c r="I32" s="241" t="n">
+        <x:f>I29+I31</x:f>
+        <x:v>481.724843166</x:v>
+      </x:c>
+      <x:c r="J32" s="189" t="str">
+        <x:v>Operating income + D&amp;A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="16" customHeight="1">
+      <x:c r="A33" s="240" t="str">
+        <x:v>EBITDA margin</x:v>
+      </x:c>
+      <x:c r="B33" s="242" t="n">
+        <x:f>B32/B20</x:f>
+        <x:v>0.18217723900867652</x:v>
+      </x:c>
+      <x:c r="C33" s="242" t="n">
+        <x:f>C32/C20</x:f>
+        <x:v>0.16156541992203516</x:v>
+      </x:c>
+      <x:c r="D33" s="242" t="n">
+        <x:f>D32/D20</x:f>
+        <x:v>0.1944559258778771</x:v>
+      </x:c>
+      <x:c r="E33" s="242" t="n">
+        <x:f>E32/E20</x:f>
+        <x:v>0.29</x:v>
+      </x:c>
+      <x:c r="F33" s="242" t="n">
+        <x:f>F32/F20</x:f>
+        <x:v>0.2969999999999999</x:v>
+      </x:c>
+      <x:c r="G33" s="242" t="n">
+        <x:f>G32/G20</x:f>
+        <x:v>0.305</x:v>
+      </x:c>
+      <x:c r="H33" s="242" t="n">
+        <x:f>H32/H20</x:f>
+        <x:v>0.31199999999999994</x:v>
+      </x:c>
+      <x:c r="I33" s="242" t="n">
+        <x:f>I32/I20</x:f>
+        <x:v>0.31499999999999995</x:v>
+      </x:c>
+      <x:c r="J33" s="189" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="16" customHeight="1">
+      <x:c r="A34" s="149" t="str">
+        <x:v>Net interest and other income</x:v>
+      </x:c>
+      <x:c r="B34" s="226" t="n">
+        <x:f>'CGNX Historical'!D21</x:f>
+        <x:v>4.646000000000015</x:v>
+      </x:c>
+      <x:c r="C34" s="226" t="n">
+        <x:f>'CGNX Historical'!E21</x:f>
+        <x:v>16.424000000000007</x:v>
+      </x:c>
+      <x:c r="D34" s="226" t="n">
+        <x:f>'CGNX Historical'!F21</x:f>
+        <x:v>20.23599999999999</x:v>
+      </x:c>
+      <x:c r="E34" s="227" t="n">
+        <x:f>E20*B13</x:f>
+        <x:v>17.099999999999998</x:v>
+      </x:c>
+      <x:c r="F34" s="227" t="n">
+        <x:f>F20*C13</x:f>
+        <x:v>16.1538</x:v>
+      </x:c>
+      <x:c r="G34" s="227" t="n">
+        <x:f>G20*D13</x:f>
+        <x:v>14.762088000000002</x:v>
+      </x:c>
+      <x:c r="H34" s="227" t="n">
+        <x:f>H20*E13</x:f>
+        <x:v>14.359485600000003</x:v>
+      </x:c>
+      <x:c r="I34" s="227" t="n">
+        <x:f>I20*F13</x:f>
+        <x:v>13.763566947600001</x:v>
+      </x:c>
+      <x:c r="J34" s="189" t="str">
+        <x:v>Revenue × active assumption</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="16" customHeight="1">
+      <x:c r="A35" s="149" t="str">
+        <x:v>Income before taxes</x:v>
+      </x:c>
+      <x:c r="B35" s="226" t="n">
+        <x:f>'CGNX Historical'!D22</x:f>
+        <x:v>135.348</x:v>
+      </x:c>
+      <x:c r="C35" s="226" t="n">
+        <x:f>'CGNX Historical'!E22</x:f>
+        <x:v>131.489</x:v>
+      </x:c>
+      <x:c r="D35" s="226" t="n">
+        <x:f>'CGNX Historical'!F22</x:f>
+        <x:v>182.802</x:v>
+      </x:c>
+      <x:c r="E35" s="227" t="n">
+        <x:f>E29+E34</x:f>
+        <x:v>313.5</x:v>
+      </x:c>
+      <x:c r="F35" s="227" t="n">
+        <x:f>F29+F34</x:f>
+        <x:v>349.17059999999987</x:v>
+      </x:c>
+      <x:c r="G35" s="227" t="n">
+        <x:f>G29+G34</x:f>
+        <x:v>386.4983040000001</x:v>
+      </x:c>
+      <x:c r="H35" s="227" t="n">
+        <x:f>H29+H34</x:f>
+        <x:v>423.6048252</x:v>
+      </x:c>
+      <x:c r="I35" s="227" t="n">
+        <x:f>I29+I34</x:f>
+        <x:v>455.72699448720005</x:v>
+      </x:c>
+      <x:c r="J35" s="189" t="str">
+        <x:v>Operating income + net interest/other</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="16" customHeight="1">
+      <x:c r="A36" s="149" t="str">
+        <x:v>Income tax expense</x:v>
+      </x:c>
+      <x:c r="B36" s="226" t="n">
+        <x:f>'CGNX Historical'!D23</x:f>
+        <x:v>22.114</x:v>
+      </x:c>
+      <x:c r="C36" s="226" t="n">
+        <x:f>'CGNX Historical'!E23</x:f>
+        <x:v>25.318</x:v>
+      </x:c>
+      <x:c r="D36" s="226" t="n">
+        <x:f>'CGNX Historical'!F23</x:f>
+        <x:v>68.36</x:v>
+      </x:c>
+      <x:c r="E36" s="227" t="n">
+        <x:f>E35*B12</x:f>
+        <x:v>62.7</x:v>
+      </x:c>
+      <x:c r="F36" s="227" t="n">
+        <x:f>F35*C12</x:f>
+        <x:v>69.83411999999997</x:v>
+      </x:c>
+      <x:c r="G36" s="227" t="n">
+        <x:f>G35*D12</x:f>
+        <x:v>77.29966080000003</x:v>
+      </x:c>
+      <x:c r="H36" s="227" t="n">
+        <x:f>H35*E12</x:f>
+        <x:v>84.72096504000001</x:v>
+      </x:c>
+      <x:c r="I36" s="227" t="n">
+        <x:f>I35*F12</x:f>
+        <x:v>91.14539889744002</x:v>
+      </x:c>
+      <x:c r="J36" s="189" t="str">
+        <x:v>Pretax income × normalized tax rate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="16" customHeight="1">
+      <x:c r="A37" s="149" t="str">
+        <x:v>Net income</x:v>
+      </x:c>
+      <x:c r="B37" s="226" t="n">
+        <x:f>'CGNX Historical'!D25</x:f>
+        <x:v>113.234</x:v>
+      </x:c>
+      <x:c r="C37" s="226" t="n">
+        <x:f>'CGNX Historical'!E25</x:f>
+        <x:v>106.171</x:v>
+      </x:c>
+      <x:c r="D37" s="226" t="n">
+        <x:f>'CGNX Historical'!F25</x:f>
+        <x:v>114.442</x:v>
+      </x:c>
+      <x:c r="E37" s="227" t="n">
+        <x:f>E35-E36</x:f>
+        <x:v>250.8</x:v>
+      </x:c>
+      <x:c r="F37" s="227" t="n">
+        <x:f>F35-F36</x:f>
+        <x:v>279.3364799999999</x:v>
+      </x:c>
+      <x:c r="G37" s="227" t="n">
+        <x:f>G35-G36</x:f>
+        <x:v>309.19864320000005</x:v>
+      </x:c>
+      <x:c r="H37" s="227" t="n">
+        <x:f>H35-H36</x:f>
+        <x:v>338.88386016</x:v>
+      </x:c>
+      <x:c r="I37" s="227" t="n">
+        <x:f>I35-I36</x:f>
+        <x:v>364.58159558976</x:v>
+      </x:c>
+      <x:c r="J37" s="189" t="str">
+        <x:v>Pretax income less tax</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="16" customHeight="1">
+      <x:c r="A38" s="149" t="str">
+        <x:v>Net income margin</x:v>
+      </x:c>
+      <x:c r="B38" s="200" t="n">
+        <x:f>'CGNX Historical'!D26</x:f>
+        <x:v>0.13519718893387475</x:v>
+      </x:c>
+      <x:c r="C38" s="200" t="n">
+        <x:f>'CGNX Historical'!E26</x:f>
+        <x:v>0.11609541669628165</x:v>
+      </x:c>
+      <x:c r="D38" s="200" t="n">
+        <x:f>'CGNX Historical'!F26</x:f>
+        <x:v>0.11509122962632207</x:v>
+      </x:c>
+      <x:c r="E38" s="228" t="n">
+        <x:f>E37/E20</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="F38" s="228" t="n">
+        <x:f>F37/F20</x:f>
+        <x:v>0.2247999999999999</x:v>
+      </x:c>
+      <x:c r="G38" s="228" t="n">
+        <x:f>G37/G20</x:f>
+        <x:v>0.2304</x:v>
+      </x:c>
+      <x:c r="H38" s="228" t="n">
+        <x:f>H37/H20</x:f>
+        <x:v>0.23599999999999993</x:v>
+      </x:c>
+      <x:c r="I38" s="228" t="n">
+        <x:f>I37/I20</x:f>
+        <x:v>0.23839999999999997</x:v>
+      </x:c>
+      <x:c r="J38" s="189" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="16" customHeight="1">
+      <x:c r="A39" s="149" t="str">
+        <x:v>Diluted weighted average shares</x:v>
+      </x:c>
+      <x:c r="B39" s="229" t="n">
+        <x:f>'CGNX Historical'!D27</x:f>
+        <x:v>173.399</x:v>
+      </x:c>
+      <x:c r="C39" s="229" t="n">
+        <x:f>'CGNX Historical'!E27</x:f>
+        <x:v>172.611</x:v>
+      </x:c>
+      <x:c r="D39" s="229" t="n">
+        <x:f>'CGNX Historical'!F27</x:f>
+        <x:v>169.367</x:v>
+      </x:c>
+      <x:c r="E39" s="230" t="n">
+        <x:f>D39*(1+B16)</x:f>
+        <x:v>167.67333</x:v>
+      </x:c>
+      <x:c r="F39" s="230" t="n">
+        <x:f>E39*(1+C16)</x:f>
+        <x:v>165.9965967</x:v>
+      </x:c>
+      <x:c r="G39" s="230" t="n">
+        <x:f>F39*(1+D16)</x:f>
+        <x:v>164.336630733</x:v>
+      </x:c>
+      <x:c r="H39" s="230" t="n">
+        <x:f>G39*(1+E16)</x:f>
+        <x:v>162.69326442566998</x:v>
+      </x:c>
+      <x:c r="I39" s="230" t="n">
+        <x:f>H39*(1+F16)</x:f>
+        <x:v>161.06633178141328</x:v>
+      </x:c>
+      <x:c r="J39" s="189" t="str">
+        <x:v>Prior year shares × (1 + change)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="16" customHeight="1">
+      <x:c r="A40" s="149" t="str">
+        <x:v>Diluted EPS</x:v>
+      </x:c>
+      <x:c r="B40" s="231" t="n">
+        <x:f>'CGNX Historical'!D28</x:f>
+        <x:v>0.6530256806555977</x:v>
+      </x:c>
+      <x:c r="C40" s="231" t="n">
+        <x:f>'CGNX Historical'!E28</x:f>
+        <x:v>0.615088262045872</x:v>
+      </x:c>
+      <x:c r="D40" s="231" t="n">
+        <x:f>'CGNX Historical'!F28</x:f>
+        <x:v>0.6757042399050582</x:v>
+      </x:c>
+      <x:c r="E40" s="232" t="n">
+        <x:f>E37/E39</x:f>
+        <x:v>1.4957656056571431</x:v>
+      </x:c>
+      <x:c r="F40" s="232" t="n">
+        <x:f>F37/F39</x:f>
+        <x:v>1.6827843796390307</x:v>
+      </x:c>
+      <x:c r="G40" s="232" t="n">
+        <x:f>G37/G39</x:f>
+        <x:v>1.881495572964249</x:v>
+      </x:c>
+      <x:c r="H40" s="232" t="n">
+        <x:f>H37/H39</x:f>
+        <x:v>2.082961832232622</x:v>
+      </x:c>
+      <x:c r="I40" s="232" t="n">
+        <x:f>I37/I39</x:f>
+        <x:v>2.2635493809130875</x:v>
+      </x:c>
+      <x:c r="J40" s="189" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="16" customHeight="1">
+      <x:c r="A41" s="149"/>
+      <x:c r="B41" s="195"/>
+      <x:c r="C41" s="195"/>
+      <x:c r="D41" s="195"/>
+      <x:c r="E41" s="150"/>
+      <x:c r="F41" s="150"/>
+      <x:c r="G41" s="150"/>
+      <x:c r="H41" s="150"/>
+      <x:c r="I41" s="150"/>
+      <x:c r="J41" s="189"/>
+    </x:row>
+    <x:row r="42" ht="16" customHeight="1">
+      <x:c r="A42" s="239" t="str">
+        <x:v>UNLEVERED FREE CASH FLOW</x:v>
+      </x:c>
+      <x:c r="B42" s="234"/>
+      <x:c r="C42" s="234"/>
+      <x:c r="D42" s="234"/>
+      <x:c r="E42" s="235"/>
+      <x:c r="F42" s="235"/>
+      <x:c r="G42" s="235"/>
+      <x:c r="H42" s="235"/>
+      <x:c r="I42" s="235"/>
+      <x:c r="J42" s="236"/>
+    </x:row>
+    <x:row r="43" ht="16" customHeight="1">
+      <x:c r="A43" s="149" t="str">
+        <x:v>NOPAT</x:v>
+      </x:c>
+      <x:c r="B43" s="226" t="n">
+        <x:f>B29*(1-'CGNX Historical'!D24)</x:f>
+        <x:v>109.3470924431835</x:v>
+      </x:c>
+      <x:c r="C43" s="226" t="n">
+        <x:f>C29*(1-'CGNX Historical'!E24)</x:f>
+        <x:v>92.90941535033349</x:v>
+      </x:c>
+      <x:c r="D43" s="226" t="n">
+        <x:f>D29*(1-'CGNX Historical'!F24)</x:f>
+        <x:v>101.77338416428705</x:v>
+      </x:c>
+      <x:c r="E43" s="227" t="n">
+        <x:f>E29*(1-B12)</x:f>
+        <x:v>237.12</x:v>
+      </x:c>
+      <x:c r="F43" s="227" t="n">
+        <x:f>F29*(1-C12)</x:f>
+        <x:v>266.4134399999999</x:v>
+      </x:c>
+      <x:c r="G43" s="227" t="n">
+        <x:f>G29*(1-D12)</x:f>
+        <x:v>297.3889728000001</x:v>
+      </x:c>
+      <x:c r="H43" s="227" t="n">
+        <x:f>H29*(1-E12)</x:f>
+        <x:v>327.39627168</x:v>
+      </x:c>
+      <x:c r="I43" s="227" t="n">
+        <x:f>I29*(1-F12)</x:f>
+        <x:v>353.5707420316801</x:v>
+      </x:c>
+      <x:c r="J43" s="189" t="str">
+        <x:v>Operating income × (1 − tax rate)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="16" customHeight="1">
+      <x:c r="A44" s="149" t="str">
+        <x:v>Depreciation &amp; amortization</x:v>
+      </x:c>
+      <x:c r="B44" s="226" t="n">
+        <x:f>'CGNX Historical'!D37</x:f>
+        <x:v>21.88</x:v>
+      </x:c>
+      <x:c r="C44" s="226" t="n">
+        <x:f>'CGNX Historical'!E37</x:f>
+        <x:v>32.689</x:v>
+      </x:c>
+      <x:c r="D44" s="226" t="n">
+        <x:f>'CGNX Historical'!F37</x:f>
+        <x:v>30.793</x:v>
+      </x:c>
+      <x:c r="E44" s="227" t="n">
+        <x:f>E31</x:f>
+        <x:v>34.199999999999996</x:v>
+      </x:c>
+      <x:c r="F44" s="227" t="n">
+        <x:f>F31</x:f>
+        <x:v>36.0354</x:v>
+      </x:c>
+      <x:c r="G44" s="227" t="n">
+        <x:f>G31</x:f>
+        <x:v>37.57622400000001</x:v>
+      </x:c>
+      <x:c r="H44" s="227" t="n">
+        <x:f>H31</x:f>
+        <x:v>38.770611120000005</x:v>
+      </x:c>
+      <x:c r="I44" s="227" t="n">
+        <x:f>I31</x:f>
+        <x:v>39.76141562640001</x:v>
+      </x:c>
+      <x:c r="J44" s="189" t="str">
+        <x:v>Linked / calculated above</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="16" customHeight="1">
+      <x:c r="A45" s="149" t="str">
+        <x:v>Capital expenditures</x:v>
+      </x:c>
+      <x:c r="B45" s="226" t="n">
+        <x:f>'CGNX Historical'!D40</x:f>
+        <x:v>-23.077</x:v>
+      </x:c>
+      <x:c r="C45" s="226" t="n">
+        <x:f>'CGNX Historical'!E40</x:f>
+        <x:v>-15.043</x:v>
+      </x:c>
+      <x:c r="D45" s="226" t="n">
+        <x:f>'CGNX Historical'!F40</x:f>
+        <x:v>-8.743</x:v>
+      </x:c>
+      <x:c r="E45" s="227" t="n">
+        <x:f>-E20*B14</x:f>
+        <x:v>-17.099999999999998</x:v>
+      </x:c>
+      <x:c r="F45" s="227" t="n">
+        <x:f>-F20*C14</x:f>
+        <x:v>-19.881600000000002</x:v>
+      </x:c>
+      <x:c r="G45" s="227" t="n">
+        <x:f>-G20*D14</x:f>
+        <x:v>-22.814136000000005</x:v>
+      </x:c>
+      <x:c r="H45" s="227" t="n">
+        <x:f>-H20*E14</x:f>
+        <x:v>-25.847074080000002</x:v>
+      </x:c>
+      <x:c r="I45" s="227" t="n">
+        <x:f>-I20*F14</x:f>
+        <x:v>-27.527133895200002</x:v>
+      </x:c>
+      <x:c r="J45" s="189" t="str">
+        <x:v>Revenue × capex %; cash outflow shown negative</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="16" customHeight="1">
+      <x:c r="A46" s="149" t="str">
+        <x:v>Operating NWC</x:v>
+      </x:c>
+      <x:c r="B46" s="226" t="n">
+        <x:f>'CGNX Historical'!D61</x:f>
+        <x:v>254.995</x:v>
+      </x:c>
+      <x:c r="C46" s="226" t="n">
+        <x:f>'CGNX Historical'!E61</x:f>
+        <x:v>262.84</x:v>
+      </x:c>
+      <x:c r="D46" s="226" t="n">
+        <x:f>'CGNX Historical'!F61</x:f>
+        <x:v>234.39899999999997</x:v>
+      </x:c>
+      <x:c r="E46" s="227" t="n">
+        <x:f>E20*B15</x:f>
+        <x:v>262.2</x:v>
+      </x:c>
+      <x:c r="F46" s="227" t="n">
+        <x:f>F20*C15</x:f>
+        <x:v>283.31280000000004</x:v>
+      </x:c>
+      <x:c r="G46" s="227" t="n">
+        <x:f>G20*D15</x:f>
+        <x:v>301.95180000000005</x:v>
+      </x:c>
+      <x:c r="H46" s="227" t="n">
+        <x:f>H20*E15</x:f>
+        <x:v>320.21652888000006</x:v>
+      </x:c>
+      <x:c r="I46" s="227" t="n">
+        <x:f>I20*F15</x:f>
+        <x:v>336.44274760800005</x:v>
+      </x:c>
+      <x:c r="J46" s="189" t="str">
+        <x:v>Revenue × operating NWC %</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="16" customHeight="1">
+      <x:c r="A47" s="149" t="str">
+        <x:v>Change in operating NWC</x:v>
+      </x:c>
+      <x:c r="B47" s="226" t="n">
+        <x:f>'CGNX Historical'!D61-'CGNX Historical'!C61</x:f>
+        <x:v>34.20100000000002</x:v>
+      </x:c>
+      <x:c r="C47" s="226" t="n">
+        <x:f>'CGNX Historical'!E61-'CGNX Historical'!D61</x:f>
+        <x:v>7.84499999999997</x:v>
+      </x:c>
+      <x:c r="D47" s="226" t="n">
+        <x:f>'CGNX Historical'!F61-'CGNX Historical'!E61</x:f>
+        <x:v>-28.441000000000003</x:v>
+      </x:c>
+      <x:c r="E47" s="227" t="n">
+        <x:f>E46-D46</x:f>
+        <x:v>27.801000000000016</x:v>
+      </x:c>
+      <x:c r="F47" s="227" t="n">
+        <x:f>F46-E46</x:f>
+        <x:v>21.11280000000005</x:v>
+      </x:c>
+      <x:c r="G47" s="227" t="n">
+        <x:f>G46-F46</x:f>
+        <x:v>18.63900000000001</x:v>
+      </x:c>
+      <x:c r="H47" s="227" t="n">
+        <x:f>H46-G46</x:f>
+        <x:v>18.264728880000007</x:v>
+      </x:c>
+      <x:c r="I47" s="227" t="n">
+        <x:f>I46-H46</x:f>
+        <x:v>16.226218727999992</x:v>
+      </x:c>
+      <x:c r="J47" s="189" t="str">
+        <x:v>Current less prior year</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="16" customHeight="1">
+      <x:c r="A48" s="240" t="str">
+        <x:v>Unlevered free cash flow</x:v>
+      </x:c>
+      <x:c r="B48" s="241" t="n">
+        <x:f>B43+B44+B45-B47</x:f>
+        <x:v>73.94909244318347</x:v>
+      </x:c>
+      <x:c r="C48" s="241" t="n">
+        <x:f>C43+C44+C45-C47</x:f>
+        <x:v>102.7104153503335</x:v>
+      </x:c>
+      <x:c r="D48" s="241" t="n">
+        <x:f>D43+D44+D45-D47</x:f>
+        <x:v>152.26438416428707</x:v>
+      </x:c>
+      <x:c r="E48" s="241" t="n">
+        <x:f>E43+E44+E45-E47</x:f>
+        <x:v>226.41899999999998</x:v>
+      </x:c>
+      <x:c r="F48" s="241" t="n">
+        <x:f>F43+F44+F45-F47</x:f>
+        <x:v>261.45443999999986</x:v>
+      </x:c>
+      <x:c r="G48" s="241" t="n">
+        <x:f>G43+G44+G45-G47</x:f>
+        <x:v>293.5120608000001</x:v>
+      </x:c>
+      <x:c r="H48" s="241" t="n">
+        <x:f>H43+H44+H45-H47</x:f>
+        <x:v>322.05507983999996</x:v>
+      </x:c>
+      <x:c r="I48" s="241" t="n">
+        <x:f>I43+I44+I45-I47</x:f>
+        <x:v>349.5788050348801</x:v>
+      </x:c>
+      <x:c r="J48" s="189" t="str">
+        <x:v>NOPAT + D&amp;A + capex − change in NWC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="16" customHeight="1">
+      <x:c r="A49" s="243" t="str">
+        <x:v>UFCF margin</x:v>
+      </x:c>
+      <x:c r="B49" s="244" t="n">
+        <x:f>B48/B20</x:f>
+        <x:v>0.08829246889211408</x:v>
+      </x:c>
+      <x:c r="C49" s="244" t="n">
+        <x:f>C48/C20</x:f>
+        <x:v>0.11231135120838205</x:v>
+      </x:c>
+      <x:c r="D49" s="244" t="n">
+        <x:f>D48/D20</x:f>
+        <x:v>0.1531281802289586</x:v>
+      </x:c>
+      <x:c r="E49" s="244" t="n">
+        <x:f>E48/E20</x:f>
+        <x:v>0.19861315789473682</x:v>
+      </x:c>
+      <x:c r="F49" s="244" t="n">
+        <x:f>F48/F20</x:f>
+        <x:v>0.21040917431192646</x:v>
+      </x:c>
+      <x:c r="G49" s="244" t="n">
+        <x:f>G48/G20</x:f>
+        <x:v>0.21871111111111113</x:v>
+      </x:c>
+      <x:c r="H49" s="244" t="n">
+        <x:f>H48/H20</x:f>
+        <x:v>0.22428037383177563</x:v>
+      </x:c>
+      <x:c r="I49" s="244" t="n">
+        <x:f>I48/I20</x:f>
+        <x:v>0.22858967136150235</x:v>
+      </x:c>
+      <x:c r="J49" s="192" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="16" customHeight="1"/>
+    <x:row r="51" ht="16" customHeight="1">
+      <x:c r="A51" s="208" t="str">
+        <x:v>Analyst note: FY2026 is anchored to management guidance. FY2027E–FY2030E are independent scenario assumptions. Stock-based compensation is not added back to UFCF, avoiding an aggressive cash-flow benefit unless dilution is separately captured in valuation.</x:v>
+      </x:c>
+      <x:c r="B51" s="208"/>
+      <x:c r="C51" s="208"/>
+      <x:c r="D51" s="208"/>
+      <x:c r="E51" s="208"/>
+      <x:c r="F51" s="208"/>
+      <x:c r="G51" s="208"/>
+      <x:c r="H51" s="208"/>
+      <x:c r="I51" s="208"/>
+      <x:c r="J51" s="208"/>
+    </x:row>
+    <x:row r="52" ht="16" customHeight="1">
+      <x:c r="A52" s="208"/>
+      <x:c r="B52" s="208"/>
+      <x:c r="C52" s="208"/>
+      <x:c r="D52" s="208"/>
+      <x:c r="E52" s="208"/>
+      <x:c r="F52" s="208"/>
+      <x:c r="G52" s="208"/>
+      <x:c r="H52" s="208"/>
+      <x:c r="I52" s="208"/>
+      <x:c r="J52" s="208"/>
+    </x:row>
+    <x:row r="53" ht="16" customHeight="1"/>
+    <x:row r="54" ht="16" customHeight="1"/>
+    <x:row r="55" ht="16" customHeight="1"/>
+    <x:row r="56" ht="16" customHeight="1"/>
+    <x:row r="57" ht="16" customHeight="1"/>
+    <x:row r="58" ht="16" customHeight="1"/>
+    <x:row r="59" ht="16" customHeight="1"/>
+    <x:row r="60" ht="16" customHeight="1"/>
+    <x:row r="61" ht="16" customHeight="1"/>
+    <x:row r="62" ht="16" customHeight="1"/>
+    <x:row r="63" ht="16" customHeight="1"/>
+    <x:row r="64" ht="16" customHeight="1"/>
+    <x:row r="65" ht="16" customHeight="1"/>
+    <x:row r="66" ht="16" customHeight="1"/>
+    <x:row r="67" ht="16" customHeight="1"/>
+    <x:row r="68" ht="16" customHeight="1"/>
+    <x:row r="69" ht="16" customHeight="1"/>
+    <x:row r="70" ht="16" customHeight="1"/>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="B3:J3"/>
+    <x:mergeCell ref="A5:J5"/>
+    <x:mergeCell ref="A18:J18"/>
+    <x:mergeCell ref="A42:J42"/>
+    <x:mergeCell ref="A51:J52"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6034,110 +8998,621 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="49" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="25" customHeight="1">
+      <x:c r="A1" s="238" t="str">
         <x:v>ROK Forecast</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Rockwell forecast metrics required for transaction analysis</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="238"/>
+      <x:c r="C1" s="238"/>
+      <x:c r="D1" s="238"/>
+      <x:c r="E1" s="238"/>
+      <x:c r="F1" s="238"/>
+      <x:c r="G1" s="238"/>
+      <x:c r="H1" s="238"/>
+      <x:c r="I1" s="238"/>
+      <x:c r="J1" s="238"/>
+    </x:row>
+    <x:row r="2" ht="20" customHeight="1">
+      <x:c r="A2" s="181" t="str">
+        <x:v>Rockwell selected buyer metrics required for transaction analysis | USD millions, except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="181"/>
+      <x:c r="C2" s="181"/>
+      <x:c r="D2" s="181"/>
+      <x:c r="E2" s="181"/>
+      <x:c r="F2" s="181"/>
+      <x:c r="G2" s="181"/>
+      <x:c r="H2" s="181"/>
+      <x:c r="I2" s="181"/>
+      <x:c r="J2" s="181"/>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="183" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
-    </x:row>
+      <x:c r="B3" s="183" t="str">
+        <x:v>Complete — FY2026E guidance-anchored buyer forecast</x:v>
+      </x:c>
+      <x:c r="C3" s="183"/>
+      <x:c r="D3" s="183"/>
+      <x:c r="E3" s="183"/>
+      <x:c r="F3" s="183"/>
+      <x:c r="G3" s="183"/>
+      <x:c r="H3" s="183"/>
+      <x:c r="I3" s="183"/>
+      <x:c r="J3" s="183"/>
+    </x:row>
+    <x:row r="4" ht="16" customHeight="1"/>
+    <x:row r="5" ht="16" customHeight="1">
+      <x:c r="A5" s="139" t="str">
+        <x:v>BUYER FORECAST METRICS</x:v>
+      </x:c>
+      <x:c r="B5" s="139"/>
+      <x:c r="C5" s="139"/>
+      <x:c r="D5" s="139"/>
+      <x:c r="E5" s="139"/>
+      <x:c r="F5" s="139"/>
+      <x:c r="G5" s="139"/>
+      <x:c r="H5" s="139"/>
+      <x:c r="I5" s="139"/>
+      <x:c r="J5" s="139"/>
+    </x:row>
+    <x:row r="6" ht="16" customHeight="1">
+      <x:c r="A6" s="223" t="str">
+        <x:v>Fiscal year</x:v>
+      </x:c>
+      <x:c r="B6" s="224" t="str">
+        <x:v>FY2023A</x:v>
+      </x:c>
+      <x:c r="C6" s="224" t="str">
+        <x:v>FY2024A</x:v>
+      </x:c>
+      <x:c r="D6" s="224" t="str">
+        <x:v>FY2025A</x:v>
+      </x:c>
+      <x:c r="E6" s="224" t="str">
+        <x:v>FY2026E</x:v>
+      </x:c>
+      <x:c r="F6" s="224" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="G6" s="224" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="H6" s="224" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="I6" s="224" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="J6" s="225" t="str">
+        <x:v>Source / methodology</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="16" customHeight="1">
+      <x:c r="A7" s="187" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B7" s="226" t="n">
+        <x:f>'ROK Historical'!D7</x:f>
+        <x:v>9058</x:v>
+      </x:c>
+      <x:c r="C7" s="226" t="n">
+        <x:f>'ROK Historical'!E7</x:f>
+        <x:v>8264</x:v>
+      </x:c>
+      <x:c r="D7" s="226" t="n">
+        <x:f>'ROK Historical'!F7</x:f>
+        <x:v>8342</x:v>
+      </x:c>
+      <x:c r="E7" s="227" t="n">
+        <x:f>D7*(1+E8)</x:f>
+        <x:v>9051.07</x:v>
+      </x:c>
+      <x:c r="F7" s="227" t="n">
+        <x:f>E7*(1+F8)</x:f>
+        <x:v>9503.6235</x:v>
+      </x:c>
+      <x:c r="G7" s="227" t="n">
+        <x:f>F7*(1+G8)</x:f>
+        <x:v>9931.2865575</x:v>
+      </x:c>
+      <x:c r="H7" s="227" t="n">
+        <x:f>G7*(1+H8)</x:f>
+        <x:v>10328.5380198</x:v>
+      </x:c>
+      <x:c r="I7" s="227" t="n">
+        <x:f>H7*(1+I8)</x:f>
+        <x:v>10741.679540592</x:v>
+      </x:c>
+      <x:c r="J7" s="189" t="str">
+        <x:v>FY2026 S-018 midpoint; outer years analyst assumptions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="16" customHeight="1">
+      <x:c r="A8" s="187" t="str">
+        <x:v>% growth</x:v>
+      </x:c>
+      <x:c r="B8" s="200" t="n">
+        <x:f>'ROK Historical'!D8</x:f>
+        <x:v>0.16720787588268649</x:v>
+      </x:c>
+      <x:c r="C8" s="200" t="n">
+        <x:f>'ROK Historical'!E8</x:f>
+        <x:v>-0.08765731949657762</x:v>
+      </x:c>
+      <x:c r="D8" s="200" t="n">
+        <x:f>'ROK Historical'!F8</x:f>
+        <x:v>0.009438528557599302</x:v>
+      </x:c>
+      <x:c r="E8" s="228" t="n">
+        <x:f>'Control'!C56</x:f>
+        <x:v>0.085</x:v>
+      </x:c>
+      <x:c r="F8" s="228" t="n">
+        <x:f>'Control'!D56</x:f>
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="G8" s="228" t="n">
+        <x:f>'Control'!E56</x:f>
+        <x:v>0.045</x:v>
+      </x:c>
+      <x:c r="H8" s="228" t="n">
+        <x:f>'Control'!F56</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="I8" s="228" t="n">
+        <x:f>'Control'!G56</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="J8" s="189" t="str">
+        <x:v>Control sheet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="16" customHeight="1">
+      <x:c r="A9" s="187" t="str">
+        <x:v>Segment / enterprise operating margin</x:v>
+      </x:c>
+      <x:c r="B9" s="200" t="n">
+        <x:f>'ROK Historical'!D10</x:f>
+        <x:v>0.21296091852506072</x:v>
+      </x:c>
+      <x:c r="C9" s="200" t="n">
+        <x:f>'ROK Historical'!E10</x:f>
+        <x:v>0.1930058083252662</x:v>
+      </x:c>
+      <x:c r="D9" s="200" t="n">
+        <x:f>'ROK Historical'!F10</x:f>
+        <x:v>0.20414768640613762</x:v>
+      </x:c>
+      <x:c r="E9" s="228" t="n">
+        <x:f>'Control'!C57</x:f>
+        <x:v>0.215</x:v>
+      </x:c>
+      <x:c r="F9" s="228" t="n">
+        <x:f>'Control'!D57</x:f>
+        <x:v>0.217</x:v>
+      </x:c>
+      <x:c r="G9" s="228" t="n">
+        <x:f>'Control'!E57</x:f>
+        <x:v>0.219</x:v>
+      </x:c>
+      <x:c r="H9" s="228" t="n">
+        <x:f>'Control'!F57</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="I9" s="228" t="n">
+        <x:f>'Control'!G57</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="J9" s="189" t="str">
+        <x:v>Historical segment margin; forecast enterprise margin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="16" customHeight="1">
+      <x:c r="A10" s="187" t="str">
+        <x:v>Segment / enterprise operating profit</x:v>
+      </x:c>
+      <x:c r="B10" s="226" t="n">
+        <x:f>'ROK Historical'!D9</x:f>
+        <x:v>1929</x:v>
+      </x:c>
+      <x:c r="C10" s="226" t="n">
+        <x:f>'ROK Historical'!E9</x:f>
+        <x:v>1595</x:v>
+      </x:c>
+      <x:c r="D10" s="226" t="n">
+        <x:f>'ROK Historical'!F9</x:f>
+        <x:v>1703</x:v>
+      </x:c>
+      <x:c r="E10" s="227" t="n">
+        <x:f>E7*E9</x:f>
+        <x:v>1945.98005</x:v>
+      </x:c>
+      <x:c r="F10" s="227" t="n">
+        <x:f>F7*F9</x:f>
+        <x:v>2062.2862995</x:v>
+      </x:c>
+      <x:c r="G10" s="227" t="n">
+        <x:f>G7*G9</x:f>
+        <x:v>2174.9517560925</x:v>
+      </x:c>
+      <x:c r="H10" s="227" t="n">
+        <x:f>H7*H9</x:f>
+        <x:v>2272.278364356</x:v>
+      </x:c>
+      <x:c r="I10" s="227" t="n">
+        <x:f>I7*I9</x:f>
+        <x:v>2363.16949893024</x:v>
+      </x:c>
+      <x:c r="J10" s="189" t="str">
+        <x:v>Revenue × margin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="16" customHeight="1">
+      <x:c r="A11" s="187" t="str">
+        <x:v>Reported / adjusted diluted EPS</x:v>
+      </x:c>
+      <x:c r="B11" s="231" t="n">
+        <x:f>'ROK Historical'!D19</x:f>
+        <x:v>11.95</x:v>
+      </x:c>
+      <x:c r="C11" s="231" t="n">
+        <x:f>'ROK Historical'!E19</x:f>
+        <x:v>8.28</x:v>
+      </x:c>
+      <x:c r="D11" s="231" t="n">
+        <x:f>'ROK Historical'!F19</x:f>
+        <x:v>7.67</x:v>
+      </x:c>
+      <x:c r="E11" s="232" t="n">
+        <x:f>'Control'!C58</x:f>
+        <x:v>13.15</x:v>
+      </x:c>
+      <x:c r="F11" s="232" t="n">
+        <x:f>E11*(1+F12)</x:f>
+        <x:v>13.939000000000002</x:v>
+      </x:c>
+      <x:c r="G11" s="232" t="n">
+        <x:f>F11*(1+G12)</x:f>
+        <x:v>14.775340000000003</x:v>
+      </x:c>
+      <x:c r="H11" s="232" t="n">
+        <x:f>G11*(1+H12)</x:f>
+        <x:v>15.514107000000005</x:v>
+      </x:c>
+      <x:c r="I11" s="232" t="n">
+        <x:f>H11*(1+I12)</x:f>
+        <x:v>16.289812350000005</x:v>
+      </x:c>
+      <x:c r="J11" s="189" t="str">
+        <x:v>Historical reported EPS; forecast adjusted EPS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="16" customHeight="1">
+      <x:c r="A12" s="187" t="str">
+        <x:v>Adjusted EPS growth</x:v>
+      </x:c>
+      <x:c r="B12" s="200"/>
+      <x:c r="C12" s="200"/>
+      <x:c r="D12" s="200"/>
+      <x:c r="E12" s="228"/>
+      <x:c r="F12" s="228" t="n">
+        <x:f>'Control'!D59</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="G12" s="228" t="n">
+        <x:f>'Control'!E59</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="H12" s="228" t="n">
+        <x:f>'Control'!F59</x:f>
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="I12" s="228" t="n">
+        <x:f>'Control'!G59</x:f>
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="J12" s="189" t="str">
+        <x:v>Analyst assumption after FY2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="16" customHeight="1">
+      <x:c r="A13" s="187" t="str">
+        <x:v>Diluted weighted average shares</x:v>
+      </x:c>
+      <x:c r="B13" s="229" t="n">
+        <x:f>'ROK Historical'!D17</x:f>
+        <x:v>115.6</x:v>
+      </x:c>
+      <x:c r="C13" s="229" t="n">
+        <x:f>'ROK Historical'!E17</x:f>
+        <x:v>114.5</x:v>
+      </x:c>
+      <x:c r="D13" s="229" t="n">
+        <x:f>'ROK Historical'!F17</x:f>
+        <x:v>113.1</x:v>
+      </x:c>
+      <x:c r="E13" s="230" t="n">
+        <x:f>D13*(1+'Control'!C60)</x:f>
+        <x:v>112.1952</x:v>
+      </x:c>
+      <x:c r="F13" s="230" t="n">
+        <x:f>E13*(1+'Control'!D60)</x:f>
+        <x:v>111.2976384</x:v>
+      </x:c>
+      <x:c r="G13" s="230" t="n">
+        <x:f>F13*(1+'Control'!E60)</x:f>
+        <x:v>110.4072572928</x:v>
+      </x:c>
+      <x:c r="H13" s="230" t="n">
+        <x:f>G13*(1+'Control'!F60)</x:f>
+        <x:v>109.52399923445759</x:v>
+      </x:c>
+      <x:c r="I13" s="230" t="n">
+        <x:f>H13*(1+'Control'!G60)</x:f>
+        <x:v>108.64780724058193</x:v>
+      </x:c>
+      <x:c r="J13" s="189" t="str">
+        <x:v>Prior year shares × (1 + change)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="16" customHeight="1">
+      <x:c r="A14" s="187" t="str">
+        <x:v>Adjusted net income proxy</x:v>
+      </x:c>
+      <x:c r="B14" s="226" t="n">
+        <x:f>'ROK Historical'!D15</x:f>
+        <x:v>1387</x:v>
+      </x:c>
+      <x:c r="C14" s="226" t="n">
+        <x:f>'ROK Historical'!E15</x:f>
+        <x:v>953</x:v>
+      </x:c>
+      <x:c r="D14" s="226" t="n">
+        <x:f>'ROK Historical'!F15</x:f>
+        <x:v>869</x:v>
+      </x:c>
+      <x:c r="E14" s="227" t="n">
+        <x:f>E11*E13</x:f>
+        <x:v>1475.36688</x:v>
+      </x:c>
+      <x:c r="F14" s="227" t="n">
+        <x:f>F11*F13</x:f>
+        <x:v>1551.3777816576</x:v>
+      </x:c>
+      <x:c r="G14" s="227" t="n">
+        <x:f>G11*G13</x:f>
+        <x:v>1631.3047649685998</x:v>
+      </x:c>
+      <x:c r="H14" s="227" t="n">
+        <x:f>H11*H13</x:f>
+        <x:v>1699.1670431912937</x:v>
+      </x:c>
+      <x:c r="I14" s="227" t="n">
+        <x:f>I11*I13</x:f>
+        <x:v>1769.8523921880515</x:v>
+      </x:c>
+      <x:c r="J14" s="189" t="str">
+        <x:v>Adjusted EPS × diluted shares</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="16" customHeight="1">
+      <x:c r="A15" s="187" t="str">
+        <x:v>FCF conversion</x:v>
+      </x:c>
+      <x:c r="B15" s="200" t="n">
+        <x:f>'ROK Historical'!D31</x:f>
+        <x:v>0.8749098774333093</x:v>
+      </x:c>
+      <x:c r="C15" s="200" t="n">
+        <x:f>'ROK Historical'!E31</x:f>
+        <x:v>0.670514165792235</x:v>
+      </x:c>
+      <x:c r="D15" s="200" t="n">
+        <x:f>'ROK Historical'!F31</x:f>
+        <x:v>1.5627157652474108</x:v>
+      </x:c>
+      <x:c r="E15" s="228" t="n">
+        <x:f>'Control'!C61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F15" s="228" t="n">
+        <x:f>'Control'!D61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G15" s="228" t="n">
+        <x:f>'Control'!E61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H15" s="228" t="n">
+        <x:f>'Control'!F61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I15" s="228" t="n">
+        <x:f>'Control'!G61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J15" s="189" t="str">
+        <x:v>FY2026 management outlook; held constant</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="16" customHeight="1">
+      <x:c r="A16" s="187" t="str">
+        <x:v>Free cash flow proxy</x:v>
+      </x:c>
+      <x:c r="B16" s="226" t="n">
+        <x:f>'ROK Historical'!D29</x:f>
+        <x:v>1213.5</x:v>
+      </x:c>
+      <x:c r="C16" s="226" t="n">
+        <x:f>'ROK Historical'!E29</x:f>
+        <x:v>639</x:v>
+      </x:c>
+      <x:c r="D16" s="226" t="n">
+        <x:f>'ROK Historical'!F29</x:f>
+        <x:v>1358</x:v>
+      </x:c>
+      <x:c r="E16" s="227" t="n">
+        <x:f>E14*E15</x:f>
+        <x:v>1475.36688</x:v>
+      </x:c>
+      <x:c r="F16" s="227" t="n">
+        <x:f>F14*F15</x:f>
+        <x:v>1551.3777816576</x:v>
+      </x:c>
+      <x:c r="G16" s="227" t="n">
+        <x:f>G14*G15</x:f>
+        <x:v>1631.3047649685998</x:v>
+      </x:c>
+      <x:c r="H16" s="227" t="n">
+        <x:f>H14*H15</x:f>
+        <x:v>1699.1670431912937</x:v>
+      </x:c>
+      <x:c r="I16" s="227" t="n">
+        <x:f>I14*I15</x:f>
+        <x:v>1769.8523921880515</x:v>
+      </x:c>
+      <x:c r="J16" s="189" t="str">
+        <x:v>Adjusted net income proxy × FCF conversion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="16" customHeight="1">
+      <x:c r="A17" s="190" t="str">
+        <x:v>Free cash flow margin</x:v>
+      </x:c>
+      <x:c r="B17" s="201" t="n">
+        <x:f>'ROK Historical'!D30</x:f>
+        <x:v>0.13396997129609184</x:v>
+      </x:c>
+      <x:c r="C17" s="201" t="n">
+        <x:f>'ROK Historical'!E30</x:f>
+        <x:v>0.07732333010648597</x:v>
+      </x:c>
+      <x:c r="D17" s="201" t="n">
+        <x:f>'ROK Historical'!F30</x:f>
+        <x:v>0.16279069767441862</x:v>
+      </x:c>
+      <x:c r="E17" s="237" t="n">
+        <x:f>E16/E7</x:f>
+        <x:v>0.16300469226290373</x:v>
+      </x:c>
+      <x:c r="F17" s="237" t="n">
+        <x:f>F16/F7</x:f>
+        <x:v>0.16324066096027479</x:v>
+      </x:c>
+      <x:c r="G17" s="237" t="n">
+        <x:f>G16/G7</x:f>
+        <x:v>0.16425915771573987</x:v>
+      </x:c>
+      <x:c r="H17" s="237" t="n">
+        <x:f>H16/H7</x:f>
+        <x:v>0.16451186411222563</x:v>
+      </x:c>
+      <x:c r="I17" s="237" t="n">
+        <x:f>I16/I7</x:f>
+        <x:v>0.1647649592877829</x:v>
+      </x:c>
+      <x:c r="J17" s="192" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="16" customHeight="1"/>
+    <x:row r="19" ht="16" customHeight="1">
+      <x:c r="A19" s="208" t="str">
+        <x:v>Analyst note: this buyer forecast intentionally uses a limited set of normalized metrics needed for financing and accretion/dilution analysis. Reported historical EPS and forecast adjusted EPS are shown transparently and will be reconciled before the transaction model is finalized.</x:v>
+      </x:c>
+      <x:c r="B19" s="208"/>
+      <x:c r="C19" s="208"/>
+      <x:c r="D19" s="208"/>
+      <x:c r="E19" s="208"/>
+      <x:c r="F19" s="208"/>
+      <x:c r="G19" s="208"/>
+      <x:c r="H19" s="208"/>
+      <x:c r="I19" s="208"/>
+      <x:c r="J19" s="208"/>
+    </x:row>
+    <x:row r="20" ht="16" customHeight="1">
+      <x:c r="A20" s="208"/>
+      <x:c r="B20" s="208"/>
+      <x:c r="C20" s="208"/>
+      <x:c r="D20" s="208"/>
+      <x:c r="E20" s="208"/>
+      <x:c r="F20" s="208"/>
+      <x:c r="G20" s="208"/>
+      <x:c r="H20" s="208"/>
+      <x:c r="I20" s="208"/>
+      <x:c r="J20" s="208"/>
+    </x:row>
+    <x:row r="21" ht="16" customHeight="1"/>
+    <x:row r="22" ht="16" customHeight="1"/>
+    <x:row r="23" ht="16" customHeight="1"/>
+    <x:row r="24" ht="16" customHeight="1"/>
+    <x:row r="25" ht="16" customHeight="1"/>
+    <x:row r="26" ht="16" customHeight="1"/>
+    <x:row r="27" ht="16" customHeight="1"/>
+    <x:row r="28" ht="16" customHeight="1"/>
+    <x:row r="29" ht="16" customHeight="1"/>
+    <x:row r="30" ht="16" customHeight="1"/>
+    <x:row r="31" ht="16" customHeight="1"/>
+    <x:row r="32" ht="16" customHeight="1"/>
+    <x:row r="33" ht="16" customHeight="1"/>
+    <x:row r="34" ht="16" customHeight="1"/>
+    <x:row r="35" ht="16" customHeight="1"/>
+    <x:row r="36" ht="16" customHeight="1"/>
+    <x:row r="37" ht="16" customHeight="1"/>
+    <x:row r="38" ht="16" customHeight="1"/>
+    <x:row r="39" ht="16" customHeight="1"/>
+    <x:row r="40" ht="16" customHeight="1"/>
+    <x:row r="41" ht="16" customHeight="1"/>
+    <x:row r="42" ht="16" customHeight="1"/>
+    <x:row r="43" ht="16" customHeight="1"/>
+    <x:row r="44" ht="16" customHeight="1"/>
+    <x:row r="45" ht="16" customHeight="1"/>
+    <x:row r="46" ht="16" customHeight="1"/>
+    <x:row r="47" ht="16" customHeight="1"/>
+    <x:row r="48" ht="16" customHeight="1"/>
+    <x:row r="49" ht="16" customHeight="1"/>
+    <x:row r="50" ht="16" customHeight="1"/>
+    <x:row r="51" ht="16" customHeight="1"/>
+    <x:row r="52" ht="16" customHeight="1"/>
+    <x:row r="53" ht="16" customHeight="1"/>
+    <x:row r="54" ht="16" customHeight="1"/>
+    <x:row r="55" ht="16" customHeight="1"/>
+    <x:row r="56" ht="16" customHeight="1"/>
+    <x:row r="57" ht="16" customHeight="1"/>
+    <x:row r="58" ht="16" customHeight="1"/>
+    <x:row r="59" ht="16" customHeight="1"/>
+    <x:row r="60" ht="16" customHeight="1"/>
+    <x:row r="61" ht="16" customHeight="1"/>
+    <x:row r="62" ht="16" customHeight="1"/>
+    <x:row r="63" ht="16" customHeight="1"/>
+    <x:row r="64" ht="16" customHeight="1"/>
+    <x:row r="65" ht="16" customHeight="1"/>
+    <x:row r="66" ht="16" customHeight="1"/>
+    <x:row r="67" ht="16" customHeight="1"/>
+    <x:row r="68" ht="16" customHeight="1"/>
+    <x:row r="69" ht="16" customHeight="1"/>
+    <x:row r="70" ht="16" customHeight="1"/>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="B3:J3"/>
+    <x:mergeCell ref="A5:J5"/>
+    <x:mergeCell ref="A19:J20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
valuation: complete standalone DCF
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rda136b8f742f45dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R9e28ad50ef134407"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R47aa498bc14e42d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R4f79db0cca5c499b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Re4b6bc316df144fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R1371307fc2e9433c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Reff15e59002b47b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R79dcd6748abd4059"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R7ee3cc977f5446c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Ra7be6368a03742b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Rffedc329d13341e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R21f8b3d42f764fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Rb95d973d02a74884"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R55b3edf34b124830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R74c3d50f93864252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R18c78068b24548c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R2551017defdf4ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R781f5f7914bb4ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rda2a49c5f8814a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R87f6961d9f9d47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R339e62cf22004389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R1e3c684cabab4bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R7cffbb08e0754bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R5a9ef99e6c51402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R5622c9d300dc4cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R90caa97a5b07463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R11a8b2b9bf1b4333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R9fb3b5986fee4212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R136068f222cc4a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R9f3188d78f074f44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="Rba6fe5c754c54137"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R3b3935d6c7864677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R5fa1643f69ba4610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Ra6cf1b678c9b4e96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -85,13 +85,77 @@
 </x:comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={8BDDC509-894D-E4D6-9015-2B10CA3BAAAD}</x:author>
+    <x:author>tc={B2C64C71-952F-5108-98F3-1211111A0BF8}</x:author>
+    <x:author>tc={DED1E4DB-EA7E-EF00-070B-1F37A5386B43}</x:author>
+    <x:author>tc={5F3C8384-FD1D-8400-67F5-3F032724E8F4}</x:author>
+    <x:author>tc={74CE60E2-80E3-7DF4-0049-CED183A6E69F}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="B7" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Source: U.S. Treasury Daily Treasury Par Yield Curve Rates, Aug. 20, 2026. Rounded 10-year yield used in CAPM.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B8" authorId="1">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Source: StockAnalysis Cognex statistics. Observed beta rounded to 1.50 and adjusted toward 1.0.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B12" authorId="2">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Source: Kroll recommended U.S. equity risk premium, accessed Aug. 20, 2026.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B19" authorId="3">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Source: Cognex Q2 2026 earnings release furnished to the SEC. Cash and investments were $755.013 million as of July 5, 2026.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B21" authorId="4">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Source: Cognex Q2 2026 filing. Latest basic shares outstanding used as a provisional diluted-share proxy; treasury-stock-method dilution will be revisited before final publication.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="17">
+  <x:numFmts count="20">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -109,8 +173,11 @@
     <x:numFmt numFmtId="214" formatCode="$0.00"/>
     <x:numFmt numFmtId="215" formatCode="$#,##0.0"/>
     <x:numFmt numFmtId="216" formatCode="0.000"/>
+    <x:numFmt numFmtId="217" formatCode="0.00x"/>
+    <x:numFmt numFmtId="218" formatCode="0.0x"/>
+    <x:numFmt numFmtId="219" formatCode="0.000x"/>
   </x:numFmts>
-  <x:fonts count="31">
+  <x:fonts count="33">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -283,8 +350,20 @@
       <x:color rgb="FF222222"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -371,8 +450,38 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="15">
+  <x:borders count="21">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -504,11 +613,89 @@
         <x:color rgb="FFE7E6E6"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="double">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="double">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
+        <x:color rgb="FF000000"/>
+      </x:left>
+      <x:right style="medium">
+        <x:color rgb="FF000000"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="248">
+  <x:cellXfs count="386">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -997,11 +1184,277 @@
     <x:xf numFmtId="216" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="216" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="216" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="22" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="11" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="3" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="217" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="217" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="10" fillId="22" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="219" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="11" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="219" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="0" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="23" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="32" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="23" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="23" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="32" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="5" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="0" fillId="23" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="3" fillId="23" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="3" fillId="23" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="217" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="32" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="217" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="10" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="10" fillId="22" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="219" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="219" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="23" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="32" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="23" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="5" fillId="21" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="3" fillId="23" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="6">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1030,6 +1483,28 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFC6EFCE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFC00000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
@@ -1038,7 +1513,7 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFC00000"/>
+        <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
@@ -1053,6 +1528,7 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:person displayName="Rohan Dravid" id="{51843E4D-6D01-459A-8247-31E61F25B311}"/>
+  <xltc:person displayName="Rohan Dravid" id="{5D681B06-03A8-48DE-909F-486DBD62E5DE}"/>
   <xltc:person displayName="Rohan Dravid" id="{80509790-5AC7-4B70-9CDF-14DA69F61825}"/>
 </xltc:personList>
 </file>
@@ -1270,6 +1746,26 @@
 </xltc:ThreadedComments>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment3.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="B7" dT="2026-08-21T04:34:35.853" personId="{5D681B06-03A8-48DE-909F-486DBD62E5DE}" id="{8BDDC509-894D-E4D6-9015-2B10CA3BAAAD}">
+    <xltc:text>Source: U.S. Treasury Daily Treasury Par Yield Curve Rates, Aug. 20, 2026. Rounded 10-year yield used in CAPM.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B8" dT="2026-08-21T04:34:35.855" personId="{5D681B06-03A8-48DE-909F-486DBD62E5DE}" id="{B2C64C71-952F-5108-98F3-1211111A0BF8}">
+    <xltc:text>Source: StockAnalysis Cognex statistics. Observed beta rounded to 1.50 and adjusted toward 1.0.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B12" dT="2026-08-21T04:34:35.855" personId="{5D681B06-03A8-48DE-909F-486DBD62E5DE}" id="{DED1E4DB-EA7E-EF00-070B-1F37A5386B43}">
+    <xltc:text>Source: Kroll recommended U.S. equity risk premium, accessed Aug. 20, 2026.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B19" dT="2026-08-21T04:34:35.855" personId="{5D681B06-03A8-48DE-909F-486DBD62E5DE}" id="{5F3C8384-FD1D-8400-67F5-3F032724E8F4}">
+    <xltc:text>Source: Cognex Q2 2026 earnings release furnished to the SEC. Cash and investments were $755.013 million as of July 5, 2026.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B21" dT="2026-08-21T04:34:35.855" personId="{5D681B06-03A8-48DE-909F-486DBD62E5DE}" id="{74CE60E2-80E3-7DF4-0049-CED183A6E69F}">
+    <xltc:text>Source: Cognex Q2 2026 filing. Latest basic shares outstanding used as a provisional diluted-share proxy; treasury-stock-method dilution will be revisited before final publication.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1380,7 +1876,7 @@
       </x:c>
       <x:c r="B9" s="136" t="str">
         <x:f>'Checks'!B3</x:f>
-        <x:v>OPERATING FORECAST COMPLETE</x:v>
+        <x:v>DCF COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -2453,7 +2949,7 @@
         <x:v>Overall model status</x:v>
       </x:c>
       <x:c r="B3" s="133" t="str">
-        <x:v>OPERATING FORECAST COMPLETE</x:v>
+        <x:v>DCF COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -2498,11 +2994,11 @@
         <x:v>Source completeness</x:v>
       </x:c>
       <x:c r="B6" s="134" t="n">
-        <x:f>COUNTA('Sources'!A4:A9)</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTA('Sources'!A4:A13)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="135" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D6" s="135" t="n">
         <x:f>B6-C6</x:f>
@@ -2751,6 +3247,162 @@
       </x:c>
       <x:c r="G15" s="192" t="str">
         <x:v>ROK Forecast row 11 / Control row 58</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="184" t="str">
+        <x:v>DCF UFCF links</x:v>
+      </x:c>
+      <x:c r="B16" s="245" t="n">
+        <x:f>MAX(ABS('DCF'!B25-'CGNX Operating Model'!E48),ABS('DCF'!C25-'CGNX Operating Model'!F48),ABS('DCF'!D25-'CGNX Operating Model'!G48),ABS('DCF'!E25-'CGNX Operating Model'!H48),ABS('DCF'!F25-'CGNX Operating Model'!I48))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="245" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="245" t="n">
+        <x:f>B16-C16</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="245" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F16" s="245" t="str">
+        <x:f>IF(ABS(D16)&lt;=E16,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G16" s="186" t="str">
+        <x:v>DCF row 25 / CGNX Operating Model row 48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="187" t="str">
+        <x:v>DCF forecast PV subtotal</x:v>
+      </x:c>
+      <x:c r="B17" s="246" t="n">
+        <x:f>ABS('DCF'!B37-SUM('DCF'!B28:F28))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C17" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="246" t="n">
+        <x:f>B17-C17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="246" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F17" s="246" t="str">
+        <x:f>IF(ABS(D17)&lt;=E17,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G17" s="189" t="str">
+        <x:v>DCF row 37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="187" t="str">
+        <x:v>DCF enterprise-value bridge</x:v>
+      </x:c>
+      <x:c r="B18" s="246" t="n">
+        <x:f>ABS('DCF'!B38-SUM('DCF'!B36:B37))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="246" t="n">
+        <x:f>B18-C18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="246" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F18" s="246" t="str">
+        <x:f>IF(ABS(D18)&lt;=E18,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G18" s="189" t="str">
+        <x:v>DCF row 38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="187" t="str">
+        <x:v>DCF equity-value bridge</x:v>
+      </x:c>
+      <x:c r="B19" s="246" t="n">
+        <x:f>ABS('DCF'!B41-SUM('DCF'!B38:B40))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="246" t="n">
+        <x:f>B19-C19</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="246" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="F19" s="246" t="str">
+        <x:f>IF(ABS(D19)&lt;=E19,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G19" s="189" t="str">
+        <x:v>DCF row 41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="187" t="str">
+        <x:v>DCF WACC exceeds terminal growth</x:v>
+      </x:c>
+      <x:c r="B20" s="246" t="n">
+        <x:f>IF('DCF'!B17&gt;'DCF'!B18,0,1)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="246" t="n">
+        <x:f>B20-C20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="246" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="246" t="str">
+        <x:f>IF(ABS(D20)&lt;=E20,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G20" s="189" t="str">
+        <x:v>DCF rows 17-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="190" t="str">
+        <x:v>DCF sensitivity center tie</x:v>
+      </x:c>
+      <x:c r="B21" s="247" t="n">
+        <x:f>ABS('DCF'!D52-'DCF'!B43)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C21" s="247" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="247" t="n">
+        <x:f>B21-C21</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="247" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F21" s="247" t="str">
+        <x:f>IF(ABS(D21)&lt;=E21,"OK","ERROR")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G21" s="192" t="str">
+        <x:v>DCF sensitivity cell D52</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2764,6 +3416,10 @@
   <x:conditionalFormatting sqref="F12:F15">
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="OK"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="ERROR"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F16:F21">
+    <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="OK"/>
+    <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="ERROR"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4218,6 +4874,110 @@
         <x:v>Primary SEC structured data</x:v>
       </x:c>
     </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="251" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="B10" s="252" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C10" s="252" t="str">
+        <x:v>Second-quarter 2026 results</x:v>
+      </x:c>
+      <x:c r="D10" s="253" t="n">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="E10" s="253" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F10" s="252" t="str">
+        <x:v>Latest cash, investments, debt and share information</x:v>
+      </x:c>
+      <x:c r="G10" s="252" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/851205/000085120526000061/a07052026-xex991xq22026ear.htm</x:v>
+      </x:c>
+      <x:c r="H10" s="254" t="str">
+        <x:v>Company earnings release furnished to SEC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="255" t="str">
+        <x:v>S-029</x:v>
+      </x:c>
+      <x:c r="B11" s="256" t="str">
+        <x:v>U.S. Treasury</x:v>
+      </x:c>
+      <x:c r="C11" s="256" t="str">
+        <x:v>Daily Treasury Par Yield Curve Rates</x:v>
+      </x:c>
+      <x:c r="D11" s="257" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="E11" s="257" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F11" s="256" t="str">
+        <x:v>10-year risk-free rate for CAPM</x:v>
+      </x:c>
+      <x:c r="G11" s="256" t="str">
+        <x:v>https://home.treasury.gov/resource-center/data-chart-center/interest-rates/TextView?field_tdr_date_value=2026&amp;type=daily_treasury_yield_curve</x:v>
+      </x:c>
+      <x:c r="H11" s="258" t="str">
+        <x:v>10-year Treasury yield rounded to 4.7%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="255" t="str">
+        <x:v>S-030</x:v>
+      </x:c>
+      <x:c r="B12" s="256" t="str">
+        <x:v>Kroll</x:v>
+      </x:c>
+      <x:c r="C12" s="256" t="str">
+        <x:v>Recommended U.S. Equity Risk Premium</x:v>
+      </x:c>
+      <x:c r="D12" s="257" t="n">
+        <x:v>46142</x:v>
+      </x:c>
+      <x:c r="E12" s="257" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F12" s="256" t="str">
+        <x:v>Equity risk premium for CAPM</x:v>
+      </x:c>
+      <x:c r="G12" s="256" t="str">
+        <x:v>https://www.kroll.com/en/reports/cost-of-capital/recommended-us-equity-risk-premium-and-corresponding-risk-free-rates</x:v>
+      </x:c>
+      <x:c r="H12" s="258" t="str">
+        <x:v>5.0% recommended U.S. ERP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="259" t="str">
+        <x:v>S-031</x:v>
+      </x:c>
+      <x:c r="B13" s="260" t="str">
+        <x:v>Market data</x:v>
+      </x:c>
+      <x:c r="C13" s="260" t="str">
+        <x:v>Cognex stock statistics</x:v>
+      </x:c>
+      <x:c r="D13" s="261" t="n">
+        <x:v>46248</x:v>
+      </x:c>
+      <x:c r="E13" s="261" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F13" s="260" t="str">
+        <x:v>Observed five-year beta</x:v>
+      </x:c>
+      <x:c r="G13" s="260" t="str">
+        <x:v>https://stockanalysis.com/stocks/cgnx/</x:v>
+      </x:c>
+      <x:c r="H13" s="262" t="str">
+        <x:v>Observed beta rounded to 1.50; adjusted toward 1.0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -5626,7 +6386,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4027c3524d5d43df"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8719f1109b164efd"/>
 </x:worksheet>
 </file>
 
@@ -7349,7 +8109,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R438496ca798f4fce"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a20d34d698b454d"/>
 </x:worksheet>
 </file>
 
@@ -9622,112 +10382,1221 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="25" customHeight="1">
+      <x:c r="A1" s="348" t="str">
         <x:v>DCF</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Standalone discounted cash flow valuation of Cognex</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="348"/>
+      <x:c r="C1" s="348"/>
+      <x:c r="D1" s="348"/>
+      <x:c r="E1" s="348"/>
+      <x:c r="F1" s="348"/>
+      <x:c r="G1" s="348"/>
+      <x:c r="H1" s="348"/>
+      <x:c r="I1" s="348"/>
+      <x:c r="J1" s="348"/>
+    </x:row>
+    <x:row r="2" ht="20" customHeight="1">
+      <x:c r="A2" s="349" t="str">
+        <x:v>Standalone discounted cash flow valuation of Cognex | USD millions, except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="349"/>
+      <x:c r="C2" s="349"/>
+      <x:c r="D2" s="349"/>
+      <x:c r="E2" s="349"/>
+      <x:c r="F2" s="349"/>
+      <x:c r="G2" s="349"/>
+      <x:c r="H2" s="349"/>
+      <x:c r="I2" s="349"/>
+      <x:c r="J2" s="349"/>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="350" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="350" t="str">
+        <x:v>Complete — Gordon Growth DCF with CAPM WACC and dynamic sensitivity</x:v>
+      </x:c>
+      <x:c r="C3" s="350"/>
+      <x:c r="D3" s="350"/>
+      <x:c r="E3" s="350"/>
+      <x:c r="F3" s="350"/>
+      <x:c r="G3" s="350"/>
+      <x:c r="H3" s="350"/>
+      <x:c r="I3" s="350"/>
+      <x:c r="J3" s="350"/>
+    </x:row>
+    <x:row r="4" ht="17" customHeight="1">
+      <x:c r="A4" s="14"/>
+      <x:c r="B4" s="14"/>
+      <x:c r="C4" s="14"/>
+      <x:c r="D4" s="14"/>
+      <x:c r="E4" s="14"/>
+      <x:c r="F4" s="14"/>
+      <x:c r="G4" s="14"/>
+      <x:c r="H4" s="14"/>
+      <x:c r="I4" s="14"/>
+      <x:c r="J4" s="14"/>
+    </x:row>
+    <x:row r="5" ht="17" customHeight="1">
+      <x:c r="A5" s="351" t="str">
+        <x:v>WACC AND VALUATION ASSUMPTIONS</x:v>
+      </x:c>
+      <x:c r="B5" s="351"/>
+      <x:c r="C5" s="351"/>
+      <x:c r="D5" s="351"/>
+      <x:c r="E5" s="351"/>
+      <x:c r="F5" s="14"/>
+      <x:c r="G5" s="351" t="str">
+        <x:v>KEY DCF OUTPUTS</x:v>
+      </x:c>
+      <x:c r="H5" s="351"/>
+      <x:c r="I5" s="351"/>
+      <x:c r="J5" s="351"/>
+    </x:row>
+    <x:row r="6" ht="17" customHeight="1">
+      <x:c r="A6" s="280" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="B6" s="281" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C6" s="281" t="str">
+        <x:v>Units</x:v>
+      </x:c>
+      <x:c r="D6" s="281" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="E6" s="282" t="str">
+        <x:v>Methodology / note</x:v>
+      </x:c>
+      <x:c r="F6" s="14"/>
+      <x:c r="G6" s="352" t="str">
+        <x:v>Enterprise value</x:v>
+      </x:c>
+      <x:c r="H6" s="353" t="n">
+        <x:f>B38</x:f>
+        <x:v>3583.677242163858</x:v>
+      </x:c>
+      <x:c r="I6" s="14"/>
+      <x:c r="J6" s="14"/>
+    </x:row>
+    <x:row r="7" ht="17" customHeight="1">
+      <x:c r="A7" s="255" t="str">
+        <x:v>Risk-free rate</x:v>
+      </x:c>
+      <x:c r="B7" s="354" t="n">
+        <x:v>0.047</x:v>
+      </x:c>
+      <x:c r="C7" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D7" s="256" t="str">
+        <x:v>S-029</x:v>
+      </x:c>
+      <x:c r="E7" s="258" t="str">
+        <x:v>10-year U.S. Treasury, rounded</x:v>
+      </x:c>
+      <x:c r="F7" s="14"/>
+      <x:c r="G7" s="352" t="str">
+        <x:v>Equity value</x:v>
+      </x:c>
+      <x:c r="H7" s="353" t="n">
+        <x:f>B41</x:f>
+        <x:v>4338.690242163858</x:v>
+      </x:c>
+      <x:c r="I7" s="14"/>
+      <x:c r="J7" s="14"/>
+    </x:row>
+    <x:row r="8" ht="17" customHeight="1">
+      <x:c r="A8" s="255" t="str">
+        <x:v>Observed beta</x:v>
+      </x:c>
+      <x:c r="B8" s="355" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="C8" s="256" t="str">
+        <x:v>x</x:v>
+      </x:c>
+      <x:c r="D8" s="256" t="str">
+        <x:v>S-031</x:v>
+      </x:c>
+      <x:c r="E8" s="258" t="str">
+        <x:v>Five-year observed market beta</x:v>
+      </x:c>
+      <x:c r="F8" s="14"/>
+      <x:c r="G8" s="352" t="str">
+        <x:v>Implied value / share</x:v>
+      </x:c>
+      <x:c r="H8" s="356" t="n">
+        <x:f>B43</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="I8" s="14"/>
+      <x:c r="J8" s="14"/>
+    </x:row>
+    <x:row r="9" ht="17" customHeight="1">
+      <x:c r="A9" s="255" t="str">
+        <x:v>Observed-beta weight</x:v>
+      </x:c>
+      <x:c r="B9" s="354" t="n">
+        <x:v>0.67</x:v>
+      </x:c>
+      <x:c r="C9" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D9" s="256" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E9" s="258" t="str">
+        <x:v>Two-thirds weight on observed beta</x:v>
+      </x:c>
+      <x:c r="F9" s="14"/>
+      <x:c r="G9" s="352" t="str">
+        <x:v>Terminal value / EV</x:v>
+      </x:c>
+      <x:c r="H9" s="357" t="n">
+        <x:f>B44</x:f>
+        <x:v>0.6937883160372396</x:v>
+      </x:c>
+      <x:c r="I9" s="14"/>
+      <x:c r="J9" s="14"/>
+    </x:row>
+    <x:row r="10" ht="17" customHeight="1">
+      <x:c r="A10" s="255" t="str">
+        <x:v>Long-run market beta</x:v>
+      </x:c>
+      <x:c r="B10" s="355" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="256" t="str">
+        <x:v>x</x:v>
+      </x:c>
+      <x:c r="D10" s="256" t="str">
+        <x:v>CAPM convention</x:v>
+      </x:c>
+      <x:c r="E10" s="258" t="str">
+        <x:v>Beta mean-reversion anchor</x:v>
+      </x:c>
+      <x:c r="F10" s="14"/>
+      <x:c r="G10" s="352" t="str">
+        <x:v>Implied terminal EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="H10" s="358" t="n">
+        <x:f>B45</x:f>
+        <x:v>8.381110239947771</x:v>
+      </x:c>
+      <x:c r="I10" s="14"/>
+      <x:c r="J10" s="14"/>
+    </x:row>
+    <x:row r="11" ht="17" customHeight="1">
+      <x:c r="A11" s="255" t="str">
+        <x:v>Adjusted beta</x:v>
+      </x:c>
+      <x:c r="B11" s="359" t="n">
+        <x:f>B8*B9+B10*(1-B9)</x:f>
+        <x:v>1.335</x:v>
+      </x:c>
+      <x:c r="C11" s="256" t="str">
+        <x:v>x</x:v>
+      </x:c>
+      <x:c r="D11" s="256" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="E11" s="258" t="str">
+        <x:v>Observed beta adjusted toward 1.0</x:v>
+      </x:c>
+      <x:c r="F11" s="14"/>
+      <x:c r="G11" s="14"/>
+      <x:c r="H11" s="14"/>
+      <x:c r="I11" s="14"/>
+      <x:c r="J11" s="14"/>
+    </x:row>
+    <x:row r="12" ht="17" customHeight="1">
+      <x:c r="A12" s="255" t="str">
+        <x:v>Equity risk premium</x:v>
+      </x:c>
+      <x:c r="B12" s="360" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C12" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D12" s="256" t="str">
+        <x:v>S-030</x:v>
+      </x:c>
+      <x:c r="E12" s="258" t="str">
+        <x:v>Kroll recommended U.S. ERP</x:v>
+      </x:c>
+      <x:c r="F12" s="14"/>
+      <x:c r="G12" s="14"/>
+      <x:c r="H12" s="14"/>
+      <x:c r="I12" s="14"/>
+      <x:c r="J12" s="14"/>
+    </x:row>
+    <x:row r="13" ht="17" customHeight="1">
+      <x:c r="A13" s="255" t="str">
+        <x:v>Cost of equity</x:v>
+      </x:c>
+      <x:c r="B13" s="361" t="n">
+        <x:f>B7+B11*B12</x:f>
+        <x:v>0.11375</x:v>
+      </x:c>
+      <x:c r="C13" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D13" s="256" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="E13" s="258" t="str">
+        <x:v>Risk-free rate + adjusted beta × ERP</x:v>
+      </x:c>
+      <x:c r="F13" s="14"/>
+      <x:c r="G13" s="14"/>
+      <x:c r="H13" s="14"/>
+      <x:c r="I13" s="14"/>
+      <x:c r="J13" s="14"/>
+    </x:row>
+    <x:row r="14" ht="17" customHeight="1">
+      <x:c r="A14" s="255" t="str">
+        <x:v>Debt weight</x:v>
+      </x:c>
+      <x:c r="B14" s="354" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D14" s="256" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="E14" s="258" t="str">
+        <x:v>Cognex has no funded debt</x:v>
+      </x:c>
+      <x:c r="F14" s="14"/>
+      <x:c r="G14" s="14"/>
+      <x:c r="H14" s="14"/>
+      <x:c r="I14" s="14"/>
+      <x:c r="J14" s="14"/>
+    </x:row>
+    <x:row r="15" ht="17" customHeight="1">
+      <x:c r="A15" s="255" t="str">
+        <x:v>Pre-tax cost of debt</x:v>
+      </x:c>
+      <x:c r="B15" s="354" t="n">
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="C15" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D15" s="256" t="str">
+        <x:v>Illustrative; no debt</x:v>
+      </x:c>
+      <x:c r="E15" s="258" t="str">
+        <x:v>Displayed for completeness; no WACC impact</x:v>
+      </x:c>
+      <x:c r="F15" s="14"/>
+      <x:c r="G15" s="14"/>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="14"/>
+      <x:c r="J15" s="14"/>
+    </x:row>
+    <x:row r="16" ht="17" customHeight="1">
+      <x:c r="A16" s="255" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="B16" s="354" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="C16" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D16" s="256" t="str">
+        <x:v>Operating model</x:v>
+      </x:c>
+      <x:c r="E16" s="258" t="str">
+        <x:v>Normalized operating-model tax rate</x:v>
+      </x:c>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+      <x:c r="J16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="17" customHeight="1">
+      <x:c r="A17" s="255" t="str">
+        <x:v>WACC</x:v>
+      </x:c>
+      <x:c r="B17" s="362" t="n">
+        <x:f>B13*(1-B14)+B15*(1-B16)*B14</x:f>
+        <x:v>0.11375</x:v>
+      </x:c>
+      <x:c r="C17" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D17" s="256" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="E17" s="258" t="str">
+        <x:v>After-tax weighted cost of capital</x:v>
+      </x:c>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+      <x:c r="J17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="17" customHeight="1">
+      <x:c r="A18" s="255" t="str">
+        <x:v>Terminal growth rate</x:v>
+      </x:c>
+      <x:c r="B18" s="354" t="n">
+        <x:v>0.025</x:v>
+      </x:c>
+      <x:c r="C18" s="256" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D18" s="256" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E18" s="258" t="str">
+        <x:v>Long-run nominal growth below WACC</x:v>
+      </x:c>
+      <x:c r="F18" s="14"/>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+      <x:c r="J18" s="14"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="255" t="str">
+        <x:v>Cash and investments</x:v>
+      </x:c>
+      <x:c r="B19" s="363" t="n">
+        <x:v>755.013</x:v>
+      </x:c>
+      <x:c r="C19" s="256" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D19" s="256" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="E19" s="258" t="str">
+        <x:v>As of July 5, 2026</x:v>
+      </x:c>
+      <x:c r="F19" s="14"/>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="14"/>
+      <x:c r="J19" s="14"/>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="255" t="str">
+        <x:v>Debt</x:v>
+      </x:c>
+      <x:c r="B20" s="363" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="256" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D20" s="256" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="E20" s="258" t="str">
+        <x:v>No debt as of July 5, 2026</x:v>
+      </x:c>
+      <x:c r="F20" s="14"/>
+      <x:c r="G20" s="14"/>
+      <x:c r="H20" s="14"/>
+      <x:c r="I20" s="14"/>
+      <x:c r="J20" s="14"/>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="259" t="str">
+        <x:v>Diluted shares</x:v>
+      </x:c>
+      <x:c r="B21" s="364" t="n">
+        <x:v>168.224</x:v>
+      </x:c>
+      <x:c r="C21" s="260" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D21" s="260" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="E21" s="262" t="str">
+        <x:v>Latest basic shares used as diluted proxy; refine with treasury-stock method later</x:v>
+      </x:c>
+      <x:c r="F21" s="14"/>
+      <x:c r="G21" s="14"/>
+      <x:c r="H21" s="14"/>
+      <x:c r="I21" s="14"/>
+      <x:c r="J21" s="14"/>
+    </x:row>
+    <x:row r="22" ht="17" customHeight="1">
+      <x:c r="A22" s="14"/>
+      <x:c r="B22" s="14"/>
+      <x:c r="C22" s="14"/>
+      <x:c r="D22" s="14"/>
+      <x:c r="E22" s="14"/>
+      <x:c r="F22" s="14"/>
+      <x:c r="G22" s="14"/>
+      <x:c r="H22" s="14"/>
+      <x:c r="I22" s="14"/>
+      <x:c r="J22" s="14"/>
+    </x:row>
+    <x:row r="23" ht="17" customHeight="1">
+      <x:c r="A23" s="351" t="str">
+        <x:v>FORECAST CASH FLOWS AND PRESENT VALUE</x:v>
+      </x:c>
+      <x:c r="B23" s="351"/>
+      <x:c r="C23" s="351"/>
+      <x:c r="D23" s="351"/>
+      <x:c r="E23" s="351"/>
+      <x:c r="F23" s="351"/>
+      <x:c r="G23" s="351"/>
+      <x:c r="H23" s="14"/>
+      <x:c r="I23" s="14"/>
+      <x:c r="J23" s="14"/>
+    </x:row>
+    <x:row r="24" ht="17" customHeight="1">
+      <x:c r="A24" s="280" t="str">
+        <x:v>Fiscal year</x:v>
+      </x:c>
+      <x:c r="B24" s="281" t="str">
+        <x:v>FY2026E</x:v>
+      </x:c>
+      <x:c r="C24" s="281" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="D24" s="281" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="E24" s="281" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="F24" s="281" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="G24" s="282" t="str">
+        <x:v>Source / methodology</x:v>
+      </x:c>
+      <x:c r="H24" s="14"/>
+      <x:c r="I24" s="14"/>
+      <x:c r="J24" s="14"/>
+    </x:row>
+    <x:row r="25" ht="17" customHeight="1">
+      <x:c r="A25" s="255" t="str">
+        <x:v>Unlevered free cash flow</x:v>
+      </x:c>
+      <x:c r="B25" s="365" t="n">
+        <x:f>'CGNX Operating Model'!E48</x:f>
+        <x:v>226.41899999999998</x:v>
+      </x:c>
+      <x:c r="C25" s="365" t="n">
+        <x:f>'CGNX Operating Model'!F48</x:f>
+        <x:v>261.45443999999986</x:v>
+      </x:c>
+      <x:c r="D25" s="365" t="n">
+        <x:f>'CGNX Operating Model'!G48</x:f>
+        <x:v>293.5120608000001</x:v>
+      </x:c>
+      <x:c r="E25" s="365" t="n">
+        <x:f>'CGNX Operating Model'!H48</x:f>
+        <x:v>322.05507983999996</x:v>
+      </x:c>
+      <x:c r="F25" s="365" t="n">
+        <x:f>'CGNX Operating Model'!I48</x:f>
+        <x:v>349.5788050348801</x:v>
+      </x:c>
+      <x:c r="G25" s="258" t="str">
+        <x:v>Linked to CGNX Operating Model</x:v>
+      </x:c>
+      <x:c r="H25" s="14"/>
+      <x:c r="I25" s="14"/>
+      <x:c r="J25" s="14"/>
+    </x:row>
+    <x:row r="26" ht="17" customHeight="1">
+      <x:c r="A26" s="255" t="str">
+        <x:v>Discount period</x:v>
+      </x:c>
+      <x:c r="B26" s="366" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C26" s="366" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D26" s="366" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="E26" s="366" t="n">
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="F26" s="366" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="G26" s="258" t="str">
+        <x:v>Mid-year convention</x:v>
+      </x:c>
+      <x:c r="H26" s="14"/>
+      <x:c r="I26" s="14"/>
+      <x:c r="J26" s="14"/>
+    </x:row>
+    <x:row r="27" ht="17" customHeight="1">
+      <x:c r="A27" s="255" t="str">
+        <x:v>Discount factor</x:v>
+      </x:c>
+      <x:c r="B27" s="367" t="n">
+        <x:f>1/(1+$B$17)^B26</x:f>
+        <x:v>0.9475587393582686</x:v>
+      </x:c>
+      <x:c r="C27" s="367" t="n">
+        <x:f>1/(1+$B$17)^C26</x:f>
+        <x:v>0.850782257560735</x:v>
+      </x:c>
+      <x:c r="D27" s="367" t="n">
+        <x:f>1/(1+$B$17)^D26</x:f>
+        <x:v>0.7638897935449922</x:v>
+      </x:c>
+      <x:c r="E27" s="367" t="n">
+        <x:f>1/(1+$B$17)^E26</x:f>
+        <x:v>0.6858718685027987</x:v>
+      </x:c>
+      <x:c r="F27" s="367" t="n">
+        <x:f>1/(1+$B$17)^F26</x:f>
+        <x:v>0.6158221041551504</x:v>
+      </x:c>
+      <x:c r="G27" s="258" t="str">
+        <x:v>1 / (1 + WACC)^period</x:v>
+      </x:c>
+      <x:c r="H27" s="14"/>
+      <x:c r="I27" s="14"/>
+      <x:c r="J27" s="14"/>
+    </x:row>
+    <x:row r="28" ht="17" customHeight="1">
+      <x:c r="A28" s="368" t="str">
+        <x:v>Present value of UFCF</x:v>
+      </x:c>
+      <x:c r="B28" s="369" t="n">
+        <x:f>B25*B27</x:f>
+        <x:v>214.5453022067598</x:v>
+      </x:c>
+      <x:c r="C28" s="369" t="n">
+        <x:f>C25*C27</x:f>
+        <x:v>222.44079871247763</x:v>
+      </x:c>
+      <x:c r="D28" s="369" t="n">
+        <x:f>D25*D27</x:f>
+        <x:v>224.21086752747726</x:v>
+      </x:c>
+      <x:c r="E28" s="369" t="n">
+        <x:f>E25*E27</x:f>
+        <x:v>220.88851937067878</x:v>
+      </x:c>
+      <x:c r="F28" s="369" t="n">
+        <x:f>F25*F27</x:f>
+        <x:v>215.27835528462293</x:v>
+      </x:c>
+      <x:c r="G28" s="262" t="str">
+        <x:v>UFCF × discount factor</x:v>
+      </x:c>
+      <x:c r="H28" s="14"/>
+      <x:c r="I28" s="14"/>
+      <x:c r="J28" s="14"/>
+    </x:row>
+    <x:row r="29" ht="17" customHeight="1">
+      <x:c r="A29" s="14"/>
+      <x:c r="B29" s="14"/>
+      <x:c r="C29" s="14"/>
+      <x:c r="D29" s="14"/>
+      <x:c r="E29" s="14"/>
+      <x:c r="F29" s="14"/>
+      <x:c r="G29" s="14"/>
+      <x:c r="H29" s="14"/>
+      <x:c r="I29" s="14"/>
+      <x:c r="J29" s="14"/>
+    </x:row>
+    <x:row r="30" ht="17" customHeight="1">
+      <x:c r="A30" s="351" t="str">
+        <x:v>TERMINAL VALUE AND EQUITY VALUE BRIDGE</x:v>
+      </x:c>
+      <x:c r="B30" s="351"/>
+      <x:c r="C30" s="351"/>
+      <x:c r="D30" s="351"/>
+      <x:c r="E30" s="351"/>
+      <x:c r="F30" s="14"/>
+      <x:c r="G30" s="14"/>
+      <x:c r="H30" s="14"/>
+      <x:c r="I30" s="14"/>
+      <x:c r="J30" s="14"/>
+    </x:row>
+    <x:row r="31" ht="17" customHeight="1">
+      <x:c r="A31" s="251" t="str">
+        <x:v>Terminal-year UFCF</x:v>
+      </x:c>
+      <x:c r="B31" s="370" t="n">
+        <x:f>F25</x:f>
+        <x:v>349.5788050348801</x:v>
+      </x:c>
+      <x:c r="C31" s="254" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="D31" s="14"/>
+      <x:c r="E31" s="14"/>
+      <x:c r="F31" s="14"/>
+      <x:c r="G31" s="14"/>
+      <x:c r="H31" s="14"/>
+      <x:c r="I31" s="14"/>
+      <x:c r="J31" s="14"/>
+    </x:row>
+    <x:row r="32" ht="17" customHeight="1">
+      <x:c r="A32" s="255" t="str">
+        <x:v>Terminal growth rate</x:v>
+      </x:c>
+      <x:c r="B32" s="371" t="n">
+        <x:f>B18</x:f>
+        <x:v>0.025</x:v>
+      </x:c>
+      <x:c r="C32" s="258" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="D32" s="14"/>
+      <x:c r="E32" s="14"/>
+      <x:c r="F32" s="14"/>
+      <x:c r="G32" s="14"/>
+      <x:c r="H32" s="14"/>
+      <x:c r="I32" s="14"/>
+      <x:c r="J32" s="14"/>
+    </x:row>
+    <x:row r="33" ht="17" customHeight="1">
+      <x:c r="A33" s="255" t="str">
+        <x:v>Terminal UFCF</x:v>
+      </x:c>
+      <x:c r="B33" s="372" t="n">
+        <x:f>B31*(1+B32)</x:f>
+        <x:v>358.318275160752</x:v>
+      </x:c>
+      <x:c r="C33" s="258" t="str">
+        <x:v>FY2031E proxy</x:v>
+      </x:c>
+      <x:c r="D33" s="14"/>
+      <x:c r="E33" s="14"/>
+      <x:c r="F33" s="14"/>
+      <x:c r="G33" s="14"/>
+      <x:c r="H33" s="14"/>
+      <x:c r="I33" s="14"/>
+      <x:c r="J33" s="14"/>
+    </x:row>
+    <x:row r="34" ht="17" customHeight="1">
+      <x:c r="A34" s="255" t="str">
+        <x:v>Terminal value</x:v>
+      </x:c>
+      <x:c r="B34" s="372" t="n">
+        <x:f>B33/(B17-B32)</x:f>
+        <x:v>4037.3890158957975</x:v>
+      </x:c>
+      <x:c r="C34" s="258" t="str">
+        <x:v>Gordon Growth</x:v>
+      </x:c>
+      <x:c r="D34" s="14"/>
+      <x:c r="E34" s="14"/>
+      <x:c r="F34" s="14"/>
+      <x:c r="G34" s="14"/>
+      <x:c r="H34" s="14"/>
+      <x:c r="I34" s="14"/>
+      <x:c r="J34" s="14"/>
+    </x:row>
+    <x:row r="35" ht="17" customHeight="1">
+      <x:c r="A35" s="255" t="str">
+        <x:v>Terminal discount factor</x:v>
+      </x:c>
+      <x:c r="B35" s="373" t="n">
+        <x:f>F27</x:f>
+        <x:v>0.6158221041551504</x:v>
+      </x:c>
+      <x:c r="C35" s="258" t="str">
+        <x:v>Mid-year convention</x:v>
+      </x:c>
+      <x:c r="D35" s="14"/>
+      <x:c r="E35" s="14"/>
+      <x:c r="F35" s="14"/>
+      <x:c r="G35" s="14"/>
+      <x:c r="H35" s="14"/>
+      <x:c r="I35" s="14"/>
+      <x:c r="J35" s="14"/>
+    </x:row>
+    <x:row r="36" ht="17" customHeight="1">
+      <x:c r="A36" s="255" t="str">
+        <x:v>Present value of terminal value</x:v>
+      </x:c>
+      <x:c r="B36" s="372" t="n">
+        <x:f>B34*B35</x:f>
+        <x:v>2486.3133990618417</x:v>
+      </x:c>
+      <x:c r="C36" s="258" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D36" s="14"/>
+      <x:c r="E36" s="14"/>
+      <x:c r="F36" s="14"/>
+      <x:c r="G36" s="14"/>
+      <x:c r="H36" s="14"/>
+      <x:c r="I36" s="14"/>
+      <x:c r="J36" s="14"/>
+    </x:row>
+    <x:row r="37" ht="17" customHeight="1">
+      <x:c r="A37" s="255" t="str">
+        <x:v>Present value of forecast UFCF</x:v>
+      </x:c>
+      <x:c r="B37" s="372" t="n">
+        <x:f>SUM(B28:F28)</x:f>
+        <x:v>1097.3638431020163</x:v>
+      </x:c>
+      <x:c r="C37" s="258" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D37" s="14"/>
+      <x:c r="E37" s="14"/>
+      <x:c r="F37" s="14"/>
+      <x:c r="G37" s="14"/>
+      <x:c r="H37" s="14"/>
+      <x:c r="I37" s="14"/>
+      <x:c r="J37" s="14"/>
+    </x:row>
+    <x:row r="38" ht="17" customHeight="1">
+      <x:c r="A38" s="374" t="str">
+        <x:v>Enterprise value</x:v>
+      </x:c>
+      <x:c r="B38" s="375" t="n">
+        <x:f>SUM(B36:B37)</x:f>
+        <x:v>3583.677242163858</x:v>
+      </x:c>
+      <x:c r="C38" s="376" t="str">
+        <x:v>PV forecast + PV terminal</x:v>
+      </x:c>
+      <x:c r="D38" s="14"/>
+      <x:c r="E38" s="14"/>
+      <x:c r="F38" s="14"/>
+      <x:c r="G38" s="14"/>
+      <x:c r="H38" s="14"/>
+      <x:c r="I38" s="14"/>
+      <x:c r="J38" s="14"/>
+    </x:row>
+    <x:row r="39" ht="17" customHeight="1">
+      <x:c r="A39" s="255" t="str">
+        <x:v>Add: cash and investments</x:v>
+      </x:c>
+      <x:c r="B39" s="372" t="n">
+        <x:f>B19</x:f>
+        <x:v>755.013</x:v>
+      </x:c>
+      <x:c r="C39" s="258" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="D39" s="14"/>
+      <x:c r="E39" s="14"/>
+      <x:c r="F39" s="14"/>
+      <x:c r="G39" s="14"/>
+      <x:c r="H39" s="14"/>
+      <x:c r="I39" s="14"/>
+      <x:c r="J39" s="14"/>
+    </x:row>
+    <x:row r="40" ht="17" customHeight="1">
+      <x:c r="A40" s="255" t="str">
+        <x:v>Less: debt</x:v>
+      </x:c>
+      <x:c r="B40" s="372" t="n">
+        <x:f>-B20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C40" s="258" t="str">
+        <x:v>S-022</x:v>
+      </x:c>
+      <x:c r="D40" s="14"/>
+      <x:c r="E40" s="14"/>
+      <x:c r="F40" s="14"/>
+      <x:c r="G40" s="14"/>
+      <x:c r="H40" s="14"/>
+      <x:c r="I40" s="14"/>
+      <x:c r="J40" s="14"/>
+    </x:row>
+    <x:row r="41" ht="17" customHeight="1">
+      <x:c r="A41" s="374" t="str">
+        <x:v>Equity value</x:v>
+      </x:c>
+      <x:c r="B41" s="375" t="n">
+        <x:f>SUM(B38:B40)</x:f>
+        <x:v>4338.690242163858</x:v>
+      </x:c>
+      <x:c r="C41" s="376" t="str">
+        <x:v>EV + cash − debt</x:v>
+      </x:c>
+      <x:c r="D41" s="14"/>
+      <x:c r="E41" s="14"/>
+      <x:c r="F41" s="14"/>
+      <x:c r="G41" s="14"/>
+      <x:c r="H41" s="14"/>
+      <x:c r="I41" s="14"/>
+      <x:c r="J41" s="14"/>
+    </x:row>
+    <x:row r="42" ht="17" customHeight="1">
+      <x:c r="A42" s="255" t="str">
+        <x:v>Diluted shares</x:v>
+      </x:c>
+      <x:c r="B42" s="377" t="n">
+        <x:f>B21</x:f>
+        <x:v>168.224</x:v>
+      </x:c>
+      <x:c r="C42" s="258" t="str">
+        <x:v>S-022 proxy</x:v>
+      </x:c>
+      <x:c r="D42" s="14"/>
+      <x:c r="E42" s="14"/>
+      <x:c r="F42" s="14"/>
+      <x:c r="G42" s="14"/>
+      <x:c r="H42" s="14"/>
+      <x:c r="I42" s="14"/>
+      <x:c r="J42" s="14"/>
+    </x:row>
+    <x:row r="43" ht="17" customHeight="1">
+      <x:c r="A43" s="378" t="str">
+        <x:v>Implied value per share</x:v>
+      </x:c>
+      <x:c r="B43" s="379" t="n">
+        <x:f>B41/B42</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="C43" s="380" t="str">
+        <x:v>Equity value / shares</x:v>
+      </x:c>
+      <x:c r="D43" s="14"/>
+      <x:c r="E43" s="14"/>
+      <x:c r="F43" s="14"/>
+      <x:c r="G43" s="14"/>
+      <x:c r="H43" s="14"/>
+      <x:c r="I43" s="14"/>
+      <x:c r="J43" s="14"/>
+    </x:row>
+    <x:row r="44" ht="17" customHeight="1">
+      <x:c r="A44" s="255" t="str">
+        <x:v>Terminal value / enterprise value</x:v>
+      </x:c>
+      <x:c r="B44" s="371" t="n">
+        <x:f>B36/B38</x:f>
+        <x:v>0.6937883160372396</x:v>
+      </x:c>
+      <x:c r="C44" s="258" t="str">
+        <x:v>PV terminal / EV</x:v>
+      </x:c>
+      <x:c r="D44" s="14"/>
+      <x:c r="E44" s="14"/>
+      <x:c r="F44" s="14"/>
+      <x:c r="G44" s="14"/>
+      <x:c r="H44" s="14"/>
+      <x:c r="I44" s="14"/>
+      <x:c r="J44" s="14"/>
+    </x:row>
+    <x:row r="45" ht="17" customHeight="1">
+      <x:c r="A45" s="259" t="str">
+        <x:v>Implied terminal EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B45" s="381" t="n">
+        <x:f>B34/'CGNX Operating Model'!I32</x:f>
+        <x:v>8.381110239947771</x:v>
+      </x:c>
+      <x:c r="C45" s="262" t="str">
+        <x:v>Undiscounted terminal value / FY2030E EBITDA</x:v>
+      </x:c>
+      <x:c r="D45" s="14"/>
+      <x:c r="E45" s="14"/>
+      <x:c r="F45" s="14"/>
+      <x:c r="G45" s="14"/>
+      <x:c r="H45" s="14"/>
+      <x:c r="I45" s="14"/>
+      <x:c r="J45" s="14"/>
+    </x:row>
+    <x:row r="46" ht="17" customHeight="1">
+      <x:c r="A46" s="14"/>
+      <x:c r="B46" s="14"/>
+      <x:c r="C46" s="14"/>
+      <x:c r="D46" s="14"/>
+      <x:c r="E46" s="14"/>
+      <x:c r="F46" s="14"/>
+      <x:c r="G46" s="14"/>
+      <x:c r="H46" s="14"/>
+      <x:c r="I46" s="14"/>
+      <x:c r="J46" s="14"/>
+    </x:row>
+    <x:row r="47" ht="17" customHeight="1">
+      <x:c r="A47" s="14"/>
+      <x:c r="B47" s="14"/>
+      <x:c r="C47" s="14"/>
+      <x:c r="D47" s="14"/>
+      <x:c r="E47" s="14"/>
+      <x:c r="F47" s="14"/>
+      <x:c r="G47" s="14"/>
+      <x:c r="H47" s="14"/>
+      <x:c r="I47" s="14"/>
+      <x:c r="J47" s="14"/>
+    </x:row>
+    <x:row r="48" ht="17" customHeight="1">
+      <x:c r="A48" s="351" t="str">
+        <x:v>IMPLIED EQUITY VALUE PER SHARE SENSITIVITY</x:v>
+      </x:c>
+      <x:c r="B48" s="351"/>
+      <x:c r="C48" s="351"/>
+      <x:c r="D48" s="351"/>
+      <x:c r="E48" s="351"/>
+      <x:c r="F48" s="351"/>
+      <x:c r="G48" s="351"/>
+      <x:c r="H48" s="14"/>
+      <x:c r="I48" s="14"/>
+      <x:c r="J48" s="14"/>
+    </x:row>
+    <x:row r="49" ht="17" customHeight="1">
+      <x:c r="A49" s="382" t="str">
+        <x:v>WACC / TGR</x:v>
+      </x:c>
+      <x:c r="B49" s="383" t="n">
+        <x:f>$B$18-0.01</x:f>
+        <x:v>0.015000000000000001</x:v>
+      </x:c>
+      <x:c r="C49" s="383" t="n">
+        <x:f>$B$18-0.005</x:f>
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="D49" s="383" t="n">
+        <x:f>$B$18</x:f>
+        <x:v>0.025</x:v>
+      </x:c>
+      <x:c r="E49" s="383" t="n">
+        <x:f>$B$18+0.005</x:f>
+        <x:v>0.030000000000000002</x:v>
+      </x:c>
+      <x:c r="F49" s="383" t="n">
+        <x:f>$B$18+0.01</x:f>
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="G49" s="14"/>
+      <x:c r="H49" s="14"/>
+      <x:c r="I49" s="14"/>
+      <x:c r="J49" s="14"/>
+    </x:row>
+    <x:row r="50" ht="17" customHeight="1">
+      <x:c r="A50" s="383" t="n">
+        <x:f>$B$17-0.02</x:f>
+        <x:v>0.09375</x:v>
+      </x:c>
+      <x:c r="B50" s="384" t="n">
+        <x:f>(($B$25/(1+$A50)^$B$26)+($C$25/(1+$A50)^$C$26)+($D$25/(1+$A50)^$D$26)+($E$25/(1+$A50)^$E$26)+($F$25/(1+$A50)^$F$26)+(($F$25*(1+B$49)/($A50-B$49))/(1+$A50)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>29.211272953243835</x:v>
+      </x:c>
+      <x:c r="C50" s="384" t="n">
+        <x:f>(($B$25/(1+$A50)^$B$26)+($C$25/(1+$A50)^$C$26)+($D$25/(1+$A50)^$D$26)+($E$25/(1+$A50)^$E$26)+($F$25/(1+$A50)^$F$26)+(($F$25*(1+C$49)/($A50-C$49))/(1+$A50)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>30.51865140989616</x:v>
+      </x:c>
+      <x:c r="D50" s="384" t="n">
+        <x:f>(($B$25/(1+$A50)^$B$26)+($C$25/(1+$A50)^$C$26)+($D$25/(1+$A50)^$D$26)+($E$25/(1+$A50)^$E$26)+($F$25/(1+$A50)^$F$26)+(($F$25*(1+D$49)/($A50-D$49))/(1+$A50)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>32.01619400569792</x:v>
+      </x:c>
+      <x:c r="E50" s="384" t="n">
+        <x:f>(($B$25/(1+$A50)^$B$26)+($C$25/(1+$A50)^$C$26)+($D$25/(1+$A50)^$D$26)+($E$25/(1+$A50)^$E$26)+($F$25/(1+$A50)^$F$26)+(($F$25*(1+E$49)/($A50-E$49))/(1+$A50)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>33.74864524397839</x:v>
+      </x:c>
+      <x:c r="F50" s="384" t="n">
+        <x:f>(($B$25/(1+$A50)^$B$26)+($C$25/(1+$A50)^$C$26)+($D$25/(1+$A50)^$D$26)+($E$25/(1+$A50)^$E$26)+($F$25/(1+$A50)^$F$26)+(($F$25*(1+F$49)/($A50-F$49))/(1+$A50)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>35.775981799412975</x:v>
+      </x:c>
+      <x:c r="G50" s="14"/>
+      <x:c r="H50" s="14"/>
+      <x:c r="I50" s="14"/>
+      <x:c r="J50" s="14"/>
+    </x:row>
+    <x:row r="51" ht="17" customHeight="1">
+      <x:c r="A51" s="383" t="n">
+        <x:f>$B$17-0.01</x:f>
+        <x:v>0.10375000000000001</x:v>
+      </x:c>
+      <x:c r="B51" s="384" t="n">
+        <x:f>(($B$25/(1+$A51)^$B$26)+($C$25/(1+$A51)^$C$26)+($D$25/(1+$A51)^$D$26)+($E$25/(1+$A51)^$E$26)+($F$25/(1+$A51)^$F$26)+(($F$25*(1+B$49)/($A51-B$49))/(1+$A51)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>26.402469692674174</x:v>
+      </x:c>
+      <x:c r="C51" s="384" t="n">
+        <x:f>(($B$25/(1+$A51)^$B$26)+($C$25/(1+$A51)^$C$26)+($D$25/(1+$A51)^$D$26)+($E$25/(1+$A51)^$E$26)+($F$25/(1+$A51)^$F$26)+(($F$25*(1+C$49)/($A51-C$49))/(1+$A51)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>27.391993977276222</x:v>
+      </x:c>
+      <x:c r="D51" s="384" t="n">
+        <x:f>(($B$25/(1+$A51)^$B$26)+($C$25/(1+$A51)^$C$26)+($D$25/(1+$A51)^$D$26)+($E$25/(1+$A51)^$E$26)+($F$25/(1+$A51)^$F$26)+(($F$25*(1+D$49)/($A51-D$49))/(1+$A51)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>28.50717213928804</x:v>
+      </x:c>
+      <x:c r="E51" s="384" t="n">
+        <x:f>(($B$25/(1+$A51)^$B$26)+($C$25/(1+$A51)^$C$26)+($D$25/(1+$A51)^$D$26)+($E$25/(1+$A51)^$E$26)+($F$25/(1+$A51)^$F$26)+(($F$25*(1+E$49)/($A51-E$49))/(1+$A51)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>29.773560899538765</x:v>
+      </x:c>
+      <x:c r="F51" s="384" t="n">
+        <x:f>(($B$25/(1+$A51)^$B$26)+($C$25/(1+$A51)^$C$26)+($D$25/(1+$A51)^$D$26)+($E$25/(1+$A51)^$E$26)+($F$25/(1+$A51)^$F$26)+(($F$25*(1+F$49)/($A51-F$49))/(1+$A51)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>31.224151661280498</x:v>
+      </x:c>
+      <x:c r="G51" s="14"/>
+      <x:c r="H51" s="14"/>
+      <x:c r="I51" s="14"/>
+      <x:c r="J51" s="14"/>
+    </x:row>
+    <x:row r="52" ht="17" customHeight="1">
+      <x:c r="A52" s="383" t="n">
+        <x:f>$B$17</x:f>
+        <x:v>0.11375</x:v>
+      </x:c>
+      <x:c r="B52" s="384" t="n">
+        <x:f>(($B$25/(1+$A52)^$B$26)+($C$25/(1+$A52)^$C$26)+($D$25/(1+$A52)^$D$26)+($E$25/(1+$A52)^$E$26)+($F$25/(1+$A52)^$F$26)+(($F$25*(1+B$49)/($A52-B$49))/(1+$A52)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>24.16487142340751</x:v>
+      </x:c>
+      <x:c r="C52" s="384" t="n">
+        <x:f>(($B$25/(1+$A52)^$B$26)+($C$25/(1+$A52)^$C$26)+($D$25/(1+$A52)^$D$26)+($E$25/(1+$A52)^$E$26)+($F$25/(1+$A52)^$F$26)+(($F$25*(1+C$49)/($A52-C$49))/(1+$A52)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>24.93464278936843</x:v>
+      </x:c>
+      <x:c r="D52" s="385" t="n">
+        <x:f>(($B$25/(1+$A52)^$B$26)+($C$25/(1+$A52)^$C$26)+($D$25/(1+$A52)^$D$26)+($E$25/(1+$A52)^$E$26)+($F$25/(1+$A52)^$F$26)+(($F$25*(1+D$49)/($A52-D$49))/(1+$A52)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="E52" s="384" t="n">
+        <x:f>(($B$25/(1+$A52)^$B$26)+($C$25/(1+$A52)^$C$26)+($D$25/(1+$A52)^$D$26)+($E$25/(1+$A52)^$E$26)+($F$25/(1+$A52)^$F$26)+(($F$25*(1+E$49)/($A52-E$49))/(1+$A52)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>26.74992451805237</x:v>
+      </x:c>
+      <x:c r="F52" s="384" t="n">
+        <x:f>(($B$25/(1+$A52)^$B$26)+($C$25/(1+$A52)^$C$26)+($D$25/(1+$A52)^$D$26)+($E$25/(1+$A52)^$E$26)+($F$25/(1+$A52)^$F$26)+(($F$25*(1+F$49)/($A52-F$49))/(1+$A52)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>27.830449356554716</x:v>
+      </x:c>
+      <x:c r="G52" s="14"/>
+      <x:c r="H52" s="14"/>
+      <x:c r="I52" s="14"/>
+      <x:c r="J52" s="14"/>
+    </x:row>
+    <x:row r="53" ht="17" customHeight="1">
+      <x:c r="A53" s="383" t="n">
+        <x:f>$B$17+0.01</x:f>
+        <x:v>0.12375</x:v>
+      </x:c>
+      <x:c r="B53" s="384" t="n">
+        <x:f>(($B$25/(1+$A53)^$B$26)+($C$25/(1+$A53)^$C$26)+($D$25/(1+$A53)^$D$26)+($E$25/(1+$A53)^$E$26)+($F$25/(1+$A53)^$F$26)+(($F$25*(1+B$49)/($A53-B$49))/(1+$A53)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>22.340808577765838</x:v>
+      </x:c>
+      <x:c r="C53" s="384" t="n">
+        <x:f>(($B$25/(1+$A53)^$B$26)+($C$25/(1+$A53)^$C$26)+($D$25/(1+$A53)^$D$26)+($E$25/(1+$A53)^$E$26)+($F$25/(1+$A53)^$F$26)+(($F$25*(1+C$49)/($A53-C$49))/(1+$A53)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>22.952969785087355</x:v>
+      </x:c>
+      <x:c r="D53" s="384" t="n">
+        <x:f>(($B$25/(1+$A53)^$B$26)+($C$25/(1+$A53)^$C$26)+($D$25/(1+$A53)^$D$26)+($E$25/(1+$A53)^$E$26)+($F$25/(1+$A53)^$F$26)+(($F$25*(1+D$49)/($A53-D$49))/(1+$A53)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>23.627122000745224</x:v>
+      </x:c>
+      <x:c r="E53" s="384" t="n">
+        <x:f>(($B$25/(1+$A53)^$B$26)+($C$25/(1+$A53)^$C$26)+($D$25/(1+$A53)^$D$26)+($E$25/(1+$A53)^$E$26)+($F$25/(1+$A53)^$F$26)+(($F$25*(1+E$49)/($A53-E$49))/(1+$A53)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>24.373183786073277</x:v>
+      </x:c>
+      <x:c r="F53" s="384" t="n">
+        <x:f>(($B$25/(1+$A53)^$B$26)+($C$25/(1+$A53)^$C$26)+($D$25/(1+$A53)^$D$26)+($E$25/(1+$A53)^$E$26)+($F$25/(1+$A53)^$F$26)+(($F$25*(1+F$49)/($A53-F$49))/(1+$A53)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>25.2033088711566</x:v>
+      </x:c>
+      <x:c r="G53" s="14"/>
+      <x:c r="H53" s="14"/>
+      <x:c r="I53" s="14"/>
+      <x:c r="J53" s="14"/>
+    </x:row>
+    <x:row r="54" ht="17" customHeight="1">
+      <x:c r="A54" s="383" t="n">
+        <x:f>$B$17+0.02</x:f>
+        <x:v>0.13375</x:v>
+      </x:c>
+      <x:c r="B54" s="384" t="n">
+        <x:f>(($B$25/(1+$A54)^$B$26)+($C$25/(1+$A54)^$C$26)+($D$25/(1+$A54)^$D$26)+($E$25/(1+$A54)^$E$26)+($F$25/(1+$A54)^$F$26)+(($F$25*(1+B$49)/($A54-B$49))/(1+$A54)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>20.825725942147326</x:v>
+      </x:c>
+      <x:c r="C54" s="384" t="n">
+        <x:f>(($B$25/(1+$A54)^$B$26)+($C$25/(1+$A54)^$C$26)+($D$25/(1+$A54)^$D$26)+($E$25/(1+$A54)^$E$26)+($F$25/(1+$A54)^$F$26)+(($F$25*(1+C$49)/($A54-C$49))/(1+$A54)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>21.321440380629777</x:v>
+      </x:c>
+      <x:c r="D54" s="384" t="n">
+        <x:f>(($B$25/(1+$A54)^$B$26)+($C$25/(1+$A54)^$C$26)+($D$25/(1+$A54)^$D$26)+($E$25/(1+$A54)^$E$26)+($F$25/(1+$A54)^$F$26)+(($F$25*(1+D$49)/($A54-D$49))/(1+$A54)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>21.862737755984167</x:v>
+      </x:c>
+      <x:c r="E54" s="384" t="n">
+        <x:f>(($B$25/(1+$A54)^$B$26)+($C$25/(1+$A54)^$C$26)+($D$25/(1+$A54)^$D$26)+($E$25/(1+$A54)^$E$26)+($F$25/(1+$A54)^$F$26)+(($F$25*(1+E$49)/($A54-E$49))/(1+$A54)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>22.45620837233658</x:v>
+      </x:c>
+      <x:c r="F54" s="384" t="n">
+        <x:f>(($B$25/(1+$A54)^$B$26)+($C$25/(1+$A54)^$C$26)+($D$25/(1+$A54)^$D$26)+($E$25/(1+$A54)^$E$26)+($F$25/(1+$A54)^$F$26)+(($F$25*(1+F$49)/($A54-F$49))/(1+$A54)^$F$26)+$B$19-$B$20)/$B$21</x:f>
+        <x:v>23.109777278952524</x:v>
+      </x:c>
+      <x:c r="G54" s="14"/>
+      <x:c r="H54" s="14"/>
+      <x:c r="I54" s="14"/>
+      <x:c r="J54" s="14"/>
+    </x:row>
+    <x:row r="55" ht="17" customHeight="1">
+      <x:c r="A55" s="14"/>
+      <x:c r="B55" s="14"/>
+      <x:c r="C55" s="14"/>
+      <x:c r="D55" s="14"/>
+      <x:c r="E55" s="14"/>
+      <x:c r="F55" s="14"/>
+      <x:c r="G55" s="14"/>
+      <x:c r="H55" s="14"/>
+      <x:c r="I55" s="14"/>
+      <x:c r="J55" s="14"/>
+    </x:row>
+    <x:row r="56" ht="24" customHeight="1">
+      <x:c r="A56" s="347" t="str">
+        <x:v>Methodology note: The primary DCF uses the Gordon Growth method and a mid-year discounting convention. The direct observed beta is adjusted toward 1.0. Because Cognex has no funded debt, WACC is effectively its cost of equity. This is a standalone valuation: acquisition synergies and transaction financing are excluded.</x:v>
+      </x:c>
+      <x:c r="B56" s="347"/>
+      <x:c r="C56" s="347"/>
+      <x:c r="D56" s="347"/>
+      <x:c r="E56" s="347"/>
+      <x:c r="F56" s="347"/>
+      <x:c r="G56" s="347"/>
+      <x:c r="H56" s="14"/>
+      <x:c r="I56" s="14"/>
+      <x:c r="J56" s="14"/>
+    </x:row>
+    <x:row r="57" ht="24" customHeight="1">
+      <x:c r="A57" s="347"/>
+      <x:c r="B57" s="347"/>
+      <x:c r="C57" s="347"/>
+      <x:c r="D57" s="347"/>
+      <x:c r="E57" s="347"/>
+      <x:c r="F57" s="347"/>
+      <x:c r="G57" s="347"/>
+      <x:c r="H57" s="14"/>
+      <x:c r="I57" s="14"/>
+      <x:c r="J57" s="14"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="B3:J3"/>
+    <x:mergeCell ref="A5:E5"/>
+    <x:mergeCell ref="G5:J5"/>
+    <x:mergeCell ref="A23:G23"/>
+    <x:mergeCell ref="A30:E30"/>
+    <x:mergeCell ref="A48:G48"/>
+    <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7165b1b2dc6e4c56"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
valuation: complete trading comps analysis
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R781f5f7914bb4ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rda2a49c5f8814a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R87f6961d9f9d47df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R339e62cf22004389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R1e3c684cabab4bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R7cffbb08e0754bd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R5a9ef99e6c51402c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R5622c9d300dc4cb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R90caa97a5b07463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R11a8b2b9bf1b4333"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R9fb3b5986fee4212"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R136068f222cc4a25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R9f3188d78f074f44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="Rba6fe5c754c54137"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R3b3935d6c7864677"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R5fa1643f69ba4610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Ra6cf1b678c9b4e96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R82b7a66665894f73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R538195c949f04aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R72e908968f084ef5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R7b26245c9cda4f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R2f1a440f509f4502"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R8f4b6d2c7f7f4d1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Refe0d7a8e3ba47ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Re8181c5b5ef840a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R05b409ad59cb42bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rce06b1a8851944b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Raa165e71b20946c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R04b4253de2934be3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R3ad46800c16b42d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R4d858d39027a4c11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R91857405d46c46bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R7038611a6b0042ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R71f784f3990241b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="20">
+  <x:numFmts count="22">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -176,8 +176,10 @@
     <x:numFmt numFmtId="217" formatCode="0.00x"/>
     <x:numFmt numFmtId="218" formatCode="0.0x"/>
     <x:numFmt numFmtId="219" formatCode="0.000x"/>
+    <x:numFmt numFmtId="220" formatCode="#,##0"/>
+    <x:numFmt numFmtId="221" formatCode="#,##0.0"/>
   </x:numFmts>
-  <x:fonts count="33">
+  <x:fonts count="41">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -362,8 +364,54 @@
       <x:color rgb="FF000000"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="31">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -480,8 +528,43 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="21">
+  <x:borders count="23">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -691,11 +774,39 @@
         <x:color rgb="FF000000"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="386">
+  <x:cellXfs count="487">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1450,6 +1561,221 @@
     <x:xf numFmtId="214" fontId="3" fillId="23" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="35" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="29" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="220" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="36" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="221" fontId="27" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="27" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="221" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="17" fillId="29" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="220" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="36" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="27" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="27" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="29" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="220" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="36" fillId="28" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="28" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="17" fillId="29" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="14" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="29" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="26" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1505,7 +1831,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -1516,7 +1842,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -1819,7 +2145,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.2 — historicals complete</x:v>
+        <x:v>0.4 — trading comps complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -1874,9 +2200,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="136" t="str">
-        <x:f>'Checks'!B3</x:f>
-        <x:v>DCF COMPLETE</x:v>
+      <x:c r="B9" s="482" t="str">
+        <x:v>TRADING COMPS COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -2948,8 +3273,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="133" t="str">
-        <x:v>DCF COMPLETE</x:v>
+      <x:c r="B3" s="483" t="str">
+        <x:v>TRADING COMPS COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -2994,11 +3319,11 @@
         <x:v>Source completeness</x:v>
       </x:c>
       <x:c r="B6" s="134" t="n">
-        <x:f>COUNTA('Sources'!A4:A13)</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTA('Sources'!A4:A100)</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C6" s="135" t="n">
-        <x:v>10</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D6" s="135" t="n">
         <x:f>B6-C6</x:f>
@@ -3403,6 +3728,84 @@
       </x:c>
       <x:c r="G21" s="192" t="str">
         <x:v>DCF sensitivity cell D52</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="484" t="str">
+        <x:v>Trading comps target-metric links</x:v>
+      </x:c>
+      <x:c r="B22" s="484" t="n">
+        <x:f>ABS('Trading Comps'!B24-'CGNX Operating Model'!E20)+ABS('Trading Comps'!B25-'CGNX Operating Model'!E32)+ABS('Trading Comps'!B28-'CGNX Operating Model'!E40)+ABS('Trading Comps'!B29-'DCF'!B19)+ABS('Trading Comps'!B31-'DCF'!B21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="484" t="n">
+        <x:f>B22-C22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F22" s="486" t="str">
+        <x:f>IF(ABS(D22)&lt;=E22,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G22" s="484" t="str">
+        <x:v>Trading Comps rows 24-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="484" t="str">
+        <x:v>Trading comps quartile ordering</x:v>
+      </x:c>
+      <x:c r="B23" s="484" t="n">
+        <x:f>MIN('Trading Comps'!H35-'Trading Comps'!G35,'Trading Comps'!I35-'Trading Comps'!H35,'Trading Comps'!H36-'Trading Comps'!G36,'Trading Comps'!I36-'Trading Comps'!H36,'Trading Comps'!H37-'Trading Comps'!G37,'Trading Comps'!I37-'Trading Comps'!H37,'Trading Comps'!H38-'Trading Comps'!G38,'Trading Comps'!I38-'Trading Comps'!H38)</x:f>
+        <x:v>2.422662640289147</x:v>
+      </x:c>
+      <x:c r="C23" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="484" t="n">
+        <x:f>MIN(0,B23-C23)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="486" t="str">
+        <x:f>IF(ABS(D23)&lt;=E23,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G23" s="484" t="str">
+        <x:v>Trading Comps rows 35-38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="484" t="str">
+        <x:v>Trading comps EV / equity bridge</x:v>
+      </x:c>
+      <x:c r="B24" s="484" t="n">
+        <x:f>ABS('Trading Comps'!G35-(('Trading Comps'!C35*'Trading Comps'!D35+'Trading Comps'!B29-'Trading Comps'!B30)/'Trading Comps'!B31))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C24" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D24" s="484" t="n">
+        <x:f>B24-C24</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F24" s="486" t="str">
+        <x:f>IF(ABS(D24)&lt;=E24,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G24" s="484" t="str">
+        <x:v>Trading Comps row 35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4978,6 +5381,188 @@
         <x:v>Observed beta rounded to 1.50; adjusted toward 1.0</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="32" customHeight="1">
+      <x:c r="A14" s="480" t="str">
+        <x:v>S-032</x:v>
+      </x:c>
+      <x:c r="B14" s="480" t="str">
+        <x:v>Keyence</x:v>
+      </x:c>
+      <x:c r="C14" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D14" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="E14" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F14" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G14" s="480" t="str">
+        <x:v>https://stockanalysis.com/quote/tyo/6861/statistics/</x:v>
+      </x:c>
+      <x:c r="H14" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; JPY values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="32" customHeight="1">
+      <x:c r="A15" s="480" t="str">
+        <x:v>S-033</x:v>
+      </x:c>
+      <x:c r="B15" s="480" t="str">
+        <x:v>Teledyne Technologies</x:v>
+      </x:c>
+      <x:c r="C15" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D15" s="481" t="n">
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="E15" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F15" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G15" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/tdy/statistics/</x:v>
+      </x:c>
+      <x:c r="H15" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="32" customHeight="1">
+      <x:c r="A16" s="480" t="str">
+        <x:v>S-034</x:v>
+      </x:c>
+      <x:c r="B16" s="480" t="str">
+        <x:v>Zebra Technologies</x:v>
+      </x:c>
+      <x:c r="C16" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D16" s="481" t="n">
+        <x:v>46248</x:v>
+      </x:c>
+      <x:c r="E16" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F16" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G16" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/zbra/statistics/</x:v>
+      </x:c>
+      <x:c r="H16" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="32" customHeight="1">
+      <x:c r="A17" s="480" t="str">
+        <x:v>S-035</x:v>
+      </x:c>
+      <x:c r="B17" s="480" t="str">
+        <x:v>AMETEK</x:v>
+      </x:c>
+      <x:c r="C17" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D17" s="481" t="n">
+        <x:v>46248</x:v>
+      </x:c>
+      <x:c r="E17" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F17" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G17" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/ame/statistics/</x:v>
+      </x:c>
+      <x:c r="H17" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="480" t="str">
+        <x:v>S-036</x:v>
+      </x:c>
+      <x:c r="B18" s="480" t="str">
+        <x:v>Fortive</x:v>
+      </x:c>
+      <x:c r="C18" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D18" s="481" t="n">
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="E18" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F18" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G18" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/ftv/statistics/</x:v>
+      </x:c>
+      <x:c r="H18" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="32" customHeight="1">
+      <x:c r="A19" s="480" t="str">
+        <x:v>S-037</x:v>
+      </x:c>
+      <x:c r="B19" s="480" t="str">
+        <x:v>Trimble</x:v>
+      </x:c>
+      <x:c r="C19" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D19" s="481" t="n">
+        <x:v>46248</x:v>
+      </x:c>
+      <x:c r="E19" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F19" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G19" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/trmb/statistics/</x:v>
+      </x:c>
+      <x:c r="H19" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="32" customHeight="1">
+      <x:c r="A20" s="480" t="str">
+        <x:v>S-038</x:v>
+      </x:c>
+      <x:c r="B20" s="480" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C20" s="480" t="str">
+        <x:v>Stock statistics and valuation metrics</x:v>
+      </x:c>
+      <x:c r="D20" s="481" t="n">
+        <x:v>46247</x:v>
+      </x:c>
+      <x:c r="E20" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F20" s="480" t="str">
+        <x:v>Trading comps market values, margins and multiples</x:v>
+      </x:c>
+      <x:c r="G20" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/rok/statistics/</x:v>
+      </x:c>
+      <x:c r="H20" s="480" t="str">
+        <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -6386,7 +6971,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8719f1109b164efd"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd135bb5cbd5f498b"/>
 </x:worksheet>
 </file>
 
@@ -8109,7 +8694,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a20d34d698b454d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf398b0ed9c26405e"/>
 </x:worksheet>
 </file>
 
@@ -11596,7 +12181,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7165b1b2dc6e4c56"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R294eee8d3d4f44cf"/>
 </x:worksheet>
 </file>
 
@@ -11604,110 +12189,1309 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Trading Comps</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Public-company benchmarking and implied valuation</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="430" t="str">
+        <x:v>Trading Comparable Companies</x:v>
+      </x:c>
+      <x:c r="B1" s="430"/>
+      <x:c r="C1" s="430"/>
+      <x:c r="D1" s="430"/>
+      <x:c r="E1" s="430"/>
+      <x:c r="F1" s="430"/>
+      <x:c r="G1" s="430"/>
+      <x:c r="H1" s="430"/>
+      <x:c r="I1" s="430"/>
+      <x:c r="J1" s="430"/>
+      <x:c r="K1" s="430"/>
+      <x:c r="L1" s="430"/>
+      <x:c r="M1" s="430"/>
+      <x:c r="N1" s="430"/>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="431" t="str">
+        <x:v>Public-company benchmarking and implied standalone valuation of Cognex | Market data as of August 2026</x:v>
+      </x:c>
+      <x:c r="B2" s="431"/>
+      <x:c r="C2" s="431"/>
+      <x:c r="D2" s="431"/>
+      <x:c r="E2" s="431"/>
+      <x:c r="F2" s="431"/>
+      <x:c r="G2" s="431"/>
+      <x:c r="H2" s="431"/>
+      <x:c r="I2" s="431"/>
+      <x:c r="J2" s="431"/>
+      <x:c r="K2" s="431"/>
+      <x:c r="L2" s="431"/>
+      <x:c r="M2" s="431"/>
+      <x:c r="N2" s="431"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="432" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="433" t="str">
+        <x:v>Complete — seven-company industrial technology peer set with quartile valuation ranges</x:v>
+      </x:c>
+      <x:c r="C3" s="433"/>
+      <x:c r="D3" s="433"/>
+      <x:c r="E3" s="433"/>
+      <x:c r="F3" s="433"/>
+      <x:c r="G3" s="433"/>
+      <x:c r="H3" s="433"/>
+      <x:c r="I3" s="433"/>
+      <x:c r="J3" s="433"/>
+      <x:c r="K3" s="433"/>
+      <x:c r="L3" s="433"/>
+      <x:c r="M3" s="433"/>
+      <x:c r="N3" s="433"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="51"/>
+      <x:c r="B4" s="51"/>
+      <x:c r="C4" s="51"/>
+      <x:c r="D4" s="51"/>
+      <x:c r="E4" s="51"/>
+      <x:c r="F4" s="51"/>
+      <x:c r="G4" s="51"/>
+      <x:c r="H4" s="51"/>
+      <x:c r="I4" s="51"/>
+      <x:c r="J4" s="51"/>
+      <x:c r="K4" s="51"/>
+      <x:c r="L4" s="51"/>
+      <x:c r="M4" s="51"/>
+      <x:c r="N4" s="51"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="434" t="str">
+        <x:v>PUBLIC COMPANY COMPARABLES</x:v>
+      </x:c>
+      <x:c r="B5" s="434"/>
+      <x:c r="C5" s="434"/>
+      <x:c r="D5" s="434"/>
+      <x:c r="E5" s="434"/>
+      <x:c r="F5" s="434"/>
+      <x:c r="G5" s="434"/>
+      <x:c r="H5" s="434"/>
+      <x:c r="I5" s="434"/>
+      <x:c r="J5" s="434"/>
+      <x:c r="K5" s="434"/>
+      <x:c r="L5" s="434"/>
+      <x:c r="M5" s="434"/>
+      <x:c r="N5" s="434"/>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="435" t="str">
+        <x:v>Company</x:v>
+      </x:c>
+      <x:c r="B6" s="435" t="str">
+        <x:v>Ticker</x:v>
+      </x:c>
+      <x:c r="C6" s="435" t="str">
+        <x:v>Peer classification</x:v>
+      </x:c>
+      <x:c r="D6" s="460" t="str">
+        <x:v>Currency</x:v>
+      </x:c>
+      <x:c r="E6" s="460" t="str">
+        <x:v>Equity value
+(LC mm)</x:v>
+      </x:c>
+      <x:c r="F6" s="460" t="str">
+        <x:v>Enterprise value
+(LC mm)</x:v>
+      </x:c>
+      <x:c r="G6" s="460" t="str">
+        <x:v>EBITDA margin</x:v>
+      </x:c>
+      <x:c r="H6" s="460" t="str">
+        <x:v>EBIT margin</x:v>
+      </x:c>
+      <x:c r="I6" s="460" t="str">
+        <x:v>EV / Revenue</x:v>
+      </x:c>
+      <x:c r="J6" s="460" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="K6" s="460" t="str">
+        <x:v>EV / EBIT</x:v>
+      </x:c>
+      <x:c r="L6" s="460" t="str">
+        <x:v>P / E</x:v>
+      </x:c>
+      <x:c r="M6" s="460" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="N6" s="435" t="str">
+        <x:v>Comments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="18" customHeight="1">
+      <x:c r="A7" s="436" t="str">
+        <x:v>Keyence Corporation</x:v>
+      </x:c>
+      <x:c r="B7" s="436" t="str">
+        <x:v>6861.T</x:v>
+      </x:c>
+      <x:c r="C7" s="436" t="str">
+        <x:v>Closest strategic / machine vision</x:v>
+      </x:c>
+      <x:c r="D7" s="461" t="str">
+        <x:v>JPY</x:v>
+      </x:c>
+      <x:c r="E7" s="462" t="n">
+        <x:v>19569349</x:v>
+      </x:c>
+      <x:c r="F7" s="462" t="n">
+        <x:v>18142755</x:v>
+      </x:c>
+      <x:c r="G7" s="463"/>
+      <x:c r="H7" s="463" t="n">
+        <x:v>0.5208</x:v>
+      </x:c>
+      <x:c r="I7" s="464" t="n">
+        <x:v>14.46</x:v>
+      </x:c>
+      <x:c r="J7" s="464"/>
+      <x:c r="K7" s="464" t="n">
+        <x:v>27.48</x:v>
+      </x:c>
+      <x:c r="L7" s="464" t="n">
+        <x:v>39.76</x:v>
+      </x:c>
+      <x:c r="M7" s="461" t="str">
+        <x:v>S-032</x:v>
+      </x:c>
+      <x:c r="N7" s="437" t="str">
+        <x:v>Closest product fit; premium growth and margin outlier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="18" customHeight="1">
+      <x:c r="A8" s="436" t="str">
+        <x:v>Teledyne Technologies</x:v>
+      </x:c>
+      <x:c r="B8" s="436" t="str">
+        <x:v>TDY</x:v>
+      </x:c>
+      <x:c r="C8" s="436" t="str">
+        <x:v>Imaging / instrumentation</x:v>
+      </x:c>
+      <x:c r="D8" s="461" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E8" s="462" t="n">
+        <x:v>31510</x:v>
+      </x:c>
+      <x:c r="F8" s="462" t="n">
+        <x:v>33190</x:v>
+      </x:c>
+      <x:c r="G8" s="463" t="n">
+        <x:v>0.2498</x:v>
+      </x:c>
+      <x:c r="H8" s="463" t="n">
+        <x:v>0.1962</x:v>
+      </x:c>
+      <x:c r="I8" s="464" t="n">
+        <x:v>5.21</x:v>
+      </x:c>
+      <x:c r="J8" s="464" t="n">
+        <x:v>20.84</x:v>
+      </x:c>
+      <x:c r="K8" s="464" t="n">
+        <x:v>26.55</x:v>
+      </x:c>
+      <x:c r="L8" s="464" t="n">
+        <x:v>32.88</x:v>
+      </x:c>
+      <x:c r="M8" s="461" t="str">
+        <x:v>S-033</x:v>
+      </x:c>
+      <x:c r="N8" s="437" t="str">
+        <x:v>High-quality imaging and sensing reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="18" customHeight="1">
+      <x:c r="A9" s="436" t="str">
+        <x:v>Zebra Technologies</x:v>
+      </x:c>
+      <x:c r="B9" s="436" t="str">
+        <x:v>ZBRA</x:v>
+      </x:c>
+      <x:c r="C9" s="436" t="str">
+        <x:v>Machine vision / data capture</x:v>
+      </x:c>
+      <x:c r="D9" s="461" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E9" s="462" t="n">
+        <x:v>17790</x:v>
+      </x:c>
+      <x:c r="F9" s="462" t="n">
+        <x:v>20600</x:v>
+      </x:c>
+      <x:c r="G9" s="463" t="n">
+        <x:v>0.2025</x:v>
+      </x:c>
+      <x:c r="H9" s="463" t="n">
+        <x:v>0.1659</x:v>
+      </x:c>
+      <x:c r="I9" s="464" t="n">
+        <x:v>3.52</x:v>
+      </x:c>
+      <x:c r="J9" s="464" t="n">
+        <x:v>17.39</x:v>
+      </x:c>
+      <x:c r="K9" s="464" t="n">
+        <x:v>21.23</x:v>
+      </x:c>
+      <x:c r="L9" s="464" t="n">
+        <x:v>34.78</x:v>
+      </x:c>
+      <x:c r="M9" s="461" t="str">
+        <x:v>S-034</x:v>
+      </x:c>
+      <x:c r="N9" s="437" t="str">
+        <x:v>Direct exposure to machine vision and barcode capture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="18" customHeight="1">
+      <x:c r="A10" s="436" t="str">
+        <x:v>AMETEK</x:v>
+      </x:c>
+      <x:c r="B10" s="436" t="str">
+        <x:v>AME</x:v>
+      </x:c>
+      <x:c r="C10" s="436" t="str">
+        <x:v>Precision instruments / automation</x:v>
+      </x:c>
+      <x:c r="D10" s="461" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E10" s="462" t="n">
+        <x:v>59270</x:v>
+      </x:c>
+      <x:c r="F10" s="462" t="n">
+        <x:v>61080</x:v>
+      </x:c>
+      <x:c r="G10" s="463" t="n">
+        <x:v>0.3125</x:v>
+      </x:c>
+      <x:c r="H10" s="463" t="n">
+        <x:v>0.2591</x:v>
+      </x:c>
+      <x:c r="I10" s="464" t="n">
+        <x:v>7.77</x:v>
+      </x:c>
+      <x:c r="J10" s="464" t="n">
+        <x:v>24.86</x:v>
+      </x:c>
+      <x:c r="K10" s="464" t="n">
+        <x:v>29.99</x:v>
+      </x:c>
+      <x:c r="L10" s="464" t="n">
+        <x:v>37.8</x:v>
+      </x:c>
+      <x:c r="M10" s="461" t="str">
+        <x:v>S-035</x:v>
+      </x:c>
+      <x:c r="N10" s="437" t="str">
+        <x:v>Premium diversified instrumentation compounder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="18" customHeight="1">
+      <x:c r="A11" s="436" t="str">
+        <x:v>Fortive</x:v>
+      </x:c>
+      <x:c r="B11" s="436" t="str">
+        <x:v>FTV</x:v>
+      </x:c>
+      <x:c r="C11" s="436" t="str">
+        <x:v>Industrial technology / instrumentation</x:v>
+      </x:c>
+      <x:c r="D11" s="461" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E11" s="462" t="n">
+        <x:v>18590</x:v>
+      </x:c>
+      <x:c r="F11" s="462" t="n">
+        <x:v>21810</x:v>
+      </x:c>
+      <x:c r="G11" s="463" t="n">
+        <x:v>0.2731</x:v>
+      </x:c>
+      <x:c r="H11" s="463" t="n">
+        <x:v>0.1824</x:v>
+      </x:c>
+      <x:c r="I11" s="464" t="n">
+        <x:v>5.05</x:v>
+      </x:c>
+      <x:c r="J11" s="464" t="n">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="K11" s="464" t="n">
+        <x:v>27.72</x:v>
+      </x:c>
+      <x:c r="L11" s="464" t="n">
+        <x:v>32.43</x:v>
+      </x:c>
+      <x:c r="M11" s="461" t="str">
+        <x:v>S-036</x:v>
+      </x:c>
+      <x:c r="N11" s="437" t="str">
+        <x:v>Broader industrial technology reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="18" customHeight="1">
+      <x:c r="A12" s="436" t="str">
+        <x:v>Trimble</x:v>
+      </x:c>
+      <x:c r="B12" s="436" t="str">
+        <x:v>TRMB</x:v>
+      </x:c>
+      <x:c r="C12" s="436" t="str">
+        <x:v>Industrial software / sensing</x:v>
+      </x:c>
+      <x:c r="D12" s="461" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E12" s="462" t="n">
+        <x:v>13430</x:v>
+      </x:c>
+      <x:c r="F12" s="462" t="n">
+        <x:v>14680</x:v>
+      </x:c>
+      <x:c r="G12" s="463" t="n">
+        <x:v>0.2327</x:v>
+      </x:c>
+      <x:c r="H12" s="463" t="n">
+        <x:v>0.1792</x:v>
+      </x:c>
+      <x:c r="I12" s="464" t="n">
+        <x:v>3.88</x:v>
+      </x:c>
+      <x:c r="J12" s="464" t="n">
+        <x:v>16.68</x:v>
+      </x:c>
+      <x:c r="K12" s="464" t="n">
+        <x:v>21.65</x:v>
+      </x:c>
+      <x:c r="L12" s="464"/>
+      <x:c r="M12" s="461" t="str">
+        <x:v>S-037</x:v>
+      </x:c>
+      <x:c r="N12" s="437" t="str">
+        <x:v>Technology-enabled industrial workflow reference; LTM P/E is NM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="18" customHeight="1">
+      <x:c r="A13" s="436" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="B13" s="436" t="str">
+        <x:v>ROK</x:v>
+      </x:c>
+      <x:c r="C13" s="436" t="str">
+        <x:v>Industrial automation platform</x:v>
+      </x:c>
+      <x:c r="D13" s="461" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E13" s="462" t="n">
+        <x:v>50130</x:v>
+      </x:c>
+      <x:c r="F13" s="462" t="n">
+        <x:v>53260</x:v>
+      </x:c>
+      <x:c r="G13" s="463" t="n">
+        <x:v>0.2086</x:v>
+      </x:c>
+      <x:c r="H13" s="463" t="n">
+        <x:v>0.1726</x:v>
+      </x:c>
+      <x:c r="I13" s="464" t="n">
+        <x:v>5.94</x:v>
+      </x:c>
+      <x:c r="J13" s="464" t="n">
+        <x:v>28.48</x:v>
+      </x:c>
+      <x:c r="K13" s="464" t="n">
+        <x:v>34.41</x:v>
+      </x:c>
+      <x:c r="L13" s="464" t="n">
+        <x:v>42.3</x:v>
+      </x:c>
+      <x:c r="M13" s="461" t="str">
+        <x:v>S-038</x:v>
+      </x:c>
+      <x:c r="N13" s="437" t="str">
+        <x:v>Potential buyer and broader automation benchmark</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="18" customHeight="1">
+      <x:c r="A14" s="51"/>
+      <x:c r="B14" s="51"/>
+      <x:c r="C14" s="51"/>
+      <x:c r="D14" s="53"/>
+      <x:c r="E14" s="53"/>
+      <x:c r="F14" s="53"/>
+      <x:c r="G14" s="53"/>
+      <x:c r="H14" s="53"/>
+      <x:c r="I14" s="465"/>
+      <x:c r="J14" s="465"/>
+      <x:c r="K14" s="465"/>
+      <x:c r="L14" s="465"/>
+      <x:c r="M14" s="53"/>
+      <x:c r="N14" s="51"/>
+    </x:row>
+    <x:row r="15" ht="18" customHeight="1">
+      <x:c r="A15" s="434" t="str">
+        <x:v>SELECTED TRADING STATISTICS</x:v>
+      </x:c>
+      <x:c r="B15" s="434"/>
+      <x:c r="C15" s="434"/>
+      <x:c r="D15" s="466"/>
+      <x:c r="E15" s="466"/>
+      <x:c r="F15" s="466"/>
+      <x:c r="G15" s="466"/>
+      <x:c r="H15" s="466"/>
+      <x:c r="I15" s="467" t="str">
+        <x:v>EV / Revenue</x:v>
+      </x:c>
+      <x:c r="J15" s="467" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="K15" s="467" t="str">
+        <x:v>EV / EBIT</x:v>
+      </x:c>
+      <x:c r="L15" s="467" t="str">
+        <x:v>P / E</x:v>
+      </x:c>
+      <x:c r="M15" s="53"/>
+      <x:c r="N15" s="51"/>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1">
+      <x:c r="A16" s="443" t="str">
+        <x:v>Minimum</x:v>
+      </x:c>
+      <x:c r="B16" s="443"/>
+      <x:c r="C16" s="443"/>
+      <x:c r="D16" s="468"/>
+      <x:c r="E16" s="468"/>
+      <x:c r="F16" s="468"/>
+      <x:c r="G16" s="468"/>
+      <x:c r="H16" s="468"/>
+      <x:c r="I16" s="469" t="n">
+        <x:f>MIN(I$7:I$13)</x:f>
+        <x:v>3.52</x:v>
+      </x:c>
+      <x:c r="J16" s="469" t="n">
+        <x:f>MIN(J$7:J$13)</x:f>
+        <x:v>16.68</x:v>
+      </x:c>
+      <x:c r="K16" s="469" t="n">
+        <x:f>MIN(K$7:K$13)</x:f>
+        <x:v>21.23</x:v>
+      </x:c>
+      <x:c r="L16" s="469" t="n">
+        <x:f>MIN(L$7:L$13)</x:f>
+        <x:v>32.43</x:v>
+      </x:c>
+      <x:c r="M16" s="53" t="str">
+        <x:v>Keyence excluded only where data are unavailable (EV/EBITDA).</x:v>
+      </x:c>
+      <x:c r="N16" s="51"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="443" t="str">
+        <x:v>25th percentile</x:v>
+      </x:c>
+      <x:c r="B17" s="443"/>
+      <x:c r="C17" s="443"/>
+      <x:c r="D17" s="468"/>
+      <x:c r="E17" s="468"/>
+      <x:c r="F17" s="468"/>
+      <x:c r="G17" s="468"/>
+      <x:c r="H17" s="468"/>
+      <x:c r="I17" s="469" t="n">
+        <x:f>PERCENTILE.INC(I$7:I$13,25%)</x:f>
+        <x:v>4.465</x:v>
+      </x:c>
+      <x:c r="J17" s="469" t="n">
+        <x:f>PERCENTILE.INC(J$7:J$13,25%)</x:f>
+        <x:v>17.6675</x:v>
+      </x:c>
+      <x:c r="K17" s="469" t="n">
+        <x:f>PERCENTILE.INC(K$7:K$13,25%)</x:f>
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="L17" s="469" t="n">
+        <x:f>PERCENTILE.INC(L$7:L$13,25%)</x:f>
+        <x:v>33.35500000000001</x:v>
+      </x:c>
+      <x:c r="M17" s="53"/>
+      <x:c r="N17" s="51"/>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1">
+      <x:c r="A18" s="445" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="B18" s="445"/>
+      <x:c r="C18" s="445"/>
+      <x:c r="D18" s="470"/>
+      <x:c r="E18" s="470"/>
+      <x:c r="F18" s="470"/>
+      <x:c r="G18" s="470"/>
+      <x:c r="H18" s="470"/>
+      <x:c r="I18" s="471" t="n">
+        <x:f>MEDIAN(I$7:I$13)</x:f>
+        <x:v>5.21</x:v>
+      </x:c>
+      <x:c r="J18" s="471" t="n">
+        <x:f>MEDIAN(J$7:J$13)</x:f>
+        <x:v>19.67</x:v>
+      </x:c>
+      <x:c r="K18" s="471" t="n">
+        <x:f>MEDIAN(K$7:K$13)</x:f>
+        <x:v>27.48</x:v>
+      </x:c>
+      <x:c r="L18" s="471" t="n">
+        <x:f>MEDIAN(L$7:L$13)</x:f>
+        <x:v>36.29</x:v>
+      </x:c>
+      <x:c r="M18" s="53"/>
+      <x:c r="N18" s="51"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="443" t="str">
+        <x:v>75th percentile</x:v>
+      </x:c>
+      <x:c r="B19" s="443"/>
+      <x:c r="C19" s="443"/>
+      <x:c r="D19" s="468"/>
+      <x:c r="E19" s="468"/>
+      <x:c r="F19" s="468"/>
+      <x:c r="G19" s="468"/>
+      <x:c r="H19" s="468"/>
+      <x:c r="I19" s="469" t="n">
+        <x:f>PERCENTILE.INC(I$7:I$13,75%)</x:f>
+        <x:v>6.855</x:v>
+      </x:c>
+      <x:c r="J19" s="469" t="n">
+        <x:f>PERCENTILE.INC(J$7:J$13,75%)</x:f>
+        <x:v>23.855</x:v>
+      </x:c>
+      <x:c r="K19" s="469" t="n">
+        <x:f>PERCENTILE.INC(K$7:K$13,75%)</x:f>
+        <x:v>28.855</x:v>
+      </x:c>
+      <x:c r="L19" s="469" t="n">
+        <x:f>PERCENTILE.INC(L$7:L$13,75%)</x:f>
+        <x:v>39.27</x:v>
+      </x:c>
+      <x:c r="M19" s="53"/>
+      <x:c r="N19" s="51"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="443" t="str">
+        <x:v>Maximum</x:v>
+      </x:c>
+      <x:c r="B20" s="443"/>
+      <x:c r="C20" s="443"/>
+      <x:c r="D20" s="468"/>
+      <x:c r="E20" s="468"/>
+      <x:c r="F20" s="468"/>
+      <x:c r="G20" s="468"/>
+      <x:c r="H20" s="468"/>
+      <x:c r="I20" s="469" t="n">
+        <x:f>MAX(I$7:I$13)</x:f>
+        <x:v>14.46</x:v>
+      </x:c>
+      <x:c r="J20" s="469" t="n">
+        <x:f>MAX(J$7:J$13)</x:f>
+        <x:v>28.48</x:v>
+      </x:c>
+      <x:c r="K20" s="469" t="n">
+        <x:f>MAX(K$7:K$13)</x:f>
+        <x:v>34.41</x:v>
+      </x:c>
+      <x:c r="L20" s="469" t="n">
+        <x:f>MAX(L$7:L$13)</x:f>
+        <x:v>42.3</x:v>
+      </x:c>
+      <x:c r="M20" s="53"/>
+      <x:c r="N20" s="51"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="51"/>
+      <x:c r="B21" s="51"/>
+      <x:c r="C21" s="51"/>
+      <x:c r="D21" s="53"/>
+      <x:c r="E21" s="53"/>
+      <x:c r="F21" s="53"/>
+      <x:c r="G21" s="53"/>
+      <x:c r="H21" s="53"/>
+      <x:c r="I21" s="53"/>
+      <x:c r="J21" s="53"/>
+      <x:c r="K21" s="53"/>
+      <x:c r="L21" s="53"/>
+      <x:c r="M21" s="53"/>
+      <x:c r="N21" s="51"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="434" t="str">
+        <x:v>COGNEX FY2026E TARGET METRICS</x:v>
+      </x:c>
+      <x:c r="B22" s="434"/>
+      <x:c r="C22" s="434"/>
+      <x:c r="D22" s="466"/>
+      <x:c r="E22" s="466"/>
+      <x:c r="F22" s="466"/>
+      <x:c r="G22" s="53"/>
+      <x:c r="H22" s="466" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I22" s="466"/>
+      <x:c r="J22" s="466"/>
+      <x:c r="K22" s="466"/>
+      <x:c r="L22" s="466"/>
+      <x:c r="M22" s="466"/>
+      <x:c r="N22" s="434"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="447" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B23" s="447" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C23" s="447" t="str">
+        <x:v>Units</x:v>
+      </x:c>
+      <x:c r="D23" s="472" t="str">
+        <x:v>Source / methodology</x:v>
+      </x:c>
+      <x:c r="E23" s="53"/>
+      <x:c r="F23" s="53"/>
+      <x:c r="G23" s="53"/>
+      <x:c r="H23" s="468" t="str">
+        <x:v>DCF implied value / share</x:v>
+      </x:c>
+      <x:c r="I23" s="473" t="n">
+        <x:f>'DCF'!H8</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="J23" s="468" t="str">
+        <x:v>Standalone DCF reference</x:v>
+      </x:c>
+      <x:c r="K23" s="468"/>
+      <x:c r="L23" s="468"/>
+      <x:c r="M23" s="468"/>
+      <x:c r="N23" s="443"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="443" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B24" s="449" t="n">
+        <x:f>'CGNX Operating Model'!E20</x:f>
+        <x:v>1140</x:v>
+      </x:c>
+      <x:c r="C24" s="443" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D24" s="468" t="str">
+        <x:v>CGNX Operating Model FY2026E</x:v>
+      </x:c>
+      <x:c r="E24" s="53"/>
+      <x:c r="F24" s="53"/>
+      <x:c r="G24" s="53"/>
+      <x:c r="H24" s="468" t="str">
+        <x:v>Broad comps low</x:v>
+      </x:c>
+      <x:c r="I24" s="473" t="n">
+        <x:f>MIN(G35:G38)</x:f>
+        <x:v>34.7460112706867</x:v>
+      </x:c>
+      <x:c r="J24" s="468" t="str">
+        <x:v>Lowest 25th-percentile indication</x:v>
+      </x:c>
+      <x:c r="K24" s="468"/>
+      <x:c r="L24" s="468"/>
+      <x:c r="M24" s="468"/>
+      <x:c r="N24" s="443"/>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1">
+      <x:c r="A25" s="443" t="str">
+        <x:v>EBITDA</x:v>
+      </x:c>
+      <x:c r="B25" s="449" t="n">
+        <x:f>'CGNX Operating Model'!E32</x:f>
+        <x:v>330.59999999999997</x:v>
+      </x:c>
+      <x:c r="C25" s="443" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D25" s="468" t="str">
+        <x:v>CGNX Operating Model FY2026E</x:v>
+      </x:c>
+      <x:c r="E25" s="53"/>
+      <x:c r="F25" s="53"/>
+      <x:c r="G25" s="53"/>
+      <x:c r="H25" s="468" t="str">
+        <x:v>Broad comps high</x:v>
+      </x:c>
+      <x:c r="I25" s="473" t="n">
+        <x:f>MAX(I35:I38)</x:f>
+        <x:v>58.73871533415601</x:v>
+      </x:c>
+      <x:c r="J25" s="468" t="str">
+        <x:v>Highest 75th-percentile indication</x:v>
+      </x:c>
+      <x:c r="K25" s="468"/>
+      <x:c r="L25" s="468"/>
+      <x:c r="M25" s="468"/>
+      <x:c r="N25" s="443"/>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="443" t="str">
+        <x:v>EBIT</x:v>
+      </x:c>
+      <x:c r="B26" s="449" t="n">
+        <x:f>'CGNX Operating Model'!E29</x:f>
+        <x:v>296.4</x:v>
+      </x:c>
+      <x:c r="C26" s="443" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D26" s="468" t="str">
+        <x:v>CGNX Operating Model FY2026E</x:v>
+      </x:c>
+      <x:c r="E26" s="53"/>
+      <x:c r="F26" s="53"/>
+      <x:c r="G26" s="53"/>
+      <x:c r="H26" s="468" t="str">
+        <x:v>Core median low</x:v>
+      </x:c>
+      <x:c r="I26" s="473" t="n">
+        <x:f>MIN(H35:H36)</x:f>
+        <x:v>39.79463691268784</x:v>
+      </x:c>
+      <x:c r="J26" s="468" t="str">
+        <x:v>Lower median of EV/Revenue and EV/EBITDA</x:v>
+      </x:c>
+      <x:c r="K26" s="468"/>
+      <x:c r="L26" s="468"/>
+      <x:c r="M26" s="468"/>
+      <x:c r="N26" s="443"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="443" t="str">
+        <x:v>Net income</x:v>
+      </x:c>
+      <x:c r="B27" s="449" t="n">
+        <x:f>'CGNX Operating Model'!E37</x:f>
+        <x:v>250.8</x:v>
+      </x:c>
+      <x:c r="C27" s="443" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D27" s="468" t="str">
+        <x:v>CGNX Operating Model FY2026E</x:v>
+      </x:c>
+      <x:c r="E27" s="53"/>
+      <x:c r="F27" s="53"/>
+      <x:c r="G27" s="53"/>
+      <x:c r="H27" s="468" t="str">
+        <x:v>Core median high</x:v>
+      </x:c>
+      <x:c r="I27" s="473" t="n">
+        <x:f>MAX(H35:H36)</x:f>
+        <x:v>43.144349201065246</x:v>
+      </x:c>
+      <x:c r="J27" s="468" t="str">
+        <x:v>Upper median of EV/Revenue and EV/EBITDA</x:v>
+      </x:c>
+      <x:c r="K27" s="468"/>
+      <x:c r="L27" s="468"/>
+      <x:c r="M27" s="468"/>
+      <x:c r="N27" s="443"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="443" t="str">
+        <x:v>Diluted EPS</x:v>
+      </x:c>
+      <x:c r="B28" s="450" t="n">
+        <x:f>'CGNX Operating Model'!E40</x:f>
+        <x:v>1.4957656056571431</x:v>
+      </x:c>
+      <x:c r="C28" s="443" t="str">
+        <x:v>$ / share</x:v>
+      </x:c>
+      <x:c r="D28" s="468" t="str">
+        <x:v>CGNX Operating Model FY2026E</x:v>
+      </x:c>
+      <x:c r="E28" s="53"/>
+      <x:c r="F28" s="53"/>
+      <x:c r="G28" s="53"/>
+      <x:c r="H28" s="468" t="str">
+        <x:v>Core midpoint premium vs. DCF</x:v>
+      </x:c>
+      <x:c r="I28" s="474" t="n">
+        <x:f>AVERAGE(I26:I27)/I23-1</x:f>
+        <x:v>0.6078963029452733</x:v>
+      </x:c>
+      <x:c r="J28" s="468" t="str">
+        <x:v>Illustrates market-relative premium to conservative DCF</x:v>
+      </x:c>
+      <x:c r="K28" s="468"/>
+      <x:c r="L28" s="468"/>
+      <x:c r="M28" s="468"/>
+      <x:c r="N28" s="443"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="443" t="str">
+        <x:v>Cash and investments</x:v>
+      </x:c>
+      <x:c r="B29" s="449" t="n">
+        <x:f>'DCF'!B19</x:f>
+        <x:v>755.013</x:v>
+      </x:c>
+      <x:c r="C29" s="443" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D29" s="468" t="str">
+        <x:v>S-022 / DCF</x:v>
+      </x:c>
+      <x:c r="E29" s="53"/>
+      <x:c r="F29" s="53"/>
+      <x:c r="G29" s="53"/>
+      <x:c r="H29" s="468" t="str">
+        <x:v>Keyence EV/Revenue premium vs. peer median</x:v>
+      </x:c>
+      <x:c r="I29" s="474" t="n">
+        <x:f>I7/I18-1</x:f>
+        <x:v>1.7754318618042229</x:v>
+      </x:c>
+      <x:c r="J29" s="468" t="str">
+        <x:v>Closest peer trades at a material premium; do not use blindly</x:v>
+      </x:c>
+      <x:c r="K29" s="468"/>
+      <x:c r="L29" s="468"/>
+      <x:c r="M29" s="468"/>
+      <x:c r="N29" s="443"/>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="443" t="str">
+        <x:v>Debt</x:v>
+      </x:c>
+      <x:c r="B30" s="449" t="n">
+        <x:f>'DCF'!B20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C30" s="443" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D30" s="468" t="str">
+        <x:v>S-022 / DCF</x:v>
+      </x:c>
+      <x:c r="E30" s="53"/>
+      <x:c r="F30" s="53"/>
+      <x:c r="G30" s="53"/>
+      <x:c r="H30" s="53"/>
+      <x:c r="I30" s="53"/>
+      <x:c r="J30" s="53"/>
+      <x:c r="K30" s="53"/>
+      <x:c r="L30" s="53"/>
+      <x:c r="M30" s="53"/>
+      <x:c r="N30" s="51"/>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="A31" s="443" t="str">
+        <x:v>Diluted shares</x:v>
+      </x:c>
+      <x:c r="B31" s="449" t="n">
+        <x:f>'DCF'!B21</x:f>
+        <x:v>168.224</x:v>
+      </x:c>
+      <x:c r="C31" s="443" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D31" s="468" t="str">
+        <x:v>S-022 / DCF</x:v>
+      </x:c>
+      <x:c r="E31" s="53"/>
+      <x:c r="F31" s="53"/>
+      <x:c r="G31" s="53"/>
+      <x:c r="H31" s="53"/>
+      <x:c r="I31" s="53"/>
+      <x:c r="J31" s="53"/>
+      <x:c r="K31" s="53"/>
+      <x:c r="L31" s="53"/>
+      <x:c r="M31" s="53"/>
+      <x:c r="N31" s="51"/>
+    </x:row>
+    <x:row r="32" ht="18" customHeight="1">
+      <x:c r="A32" s="51"/>
+      <x:c r="B32" s="51"/>
+      <x:c r="C32" s="51"/>
+      <x:c r="D32" s="53"/>
+      <x:c r="E32" s="53"/>
+      <x:c r="F32" s="53"/>
+      <x:c r="G32" s="53"/>
+      <x:c r="H32" s="53"/>
+      <x:c r="I32" s="53"/>
+      <x:c r="J32" s="53"/>
+      <x:c r="K32" s="53"/>
+      <x:c r="L32" s="53"/>
+      <x:c r="M32" s="53"/>
+      <x:c r="N32" s="51"/>
+    </x:row>
+    <x:row r="33" ht="18" customHeight="1">
+      <x:c r="A33" s="434" t="str">
+        <x:v>IMPLIED COGNEX EQUITY VALUE PER SHARE</x:v>
+      </x:c>
+      <x:c r="B33" s="434"/>
+      <x:c r="C33" s="434"/>
+      <x:c r="D33" s="466"/>
+      <x:c r="E33" s="466"/>
+      <x:c r="F33" s="466"/>
+      <x:c r="G33" s="466"/>
+      <x:c r="H33" s="466"/>
+      <x:c r="I33" s="466"/>
+      <x:c r="J33" s="53"/>
+      <x:c r="K33" s="53"/>
+      <x:c r="L33" s="53"/>
+      <x:c r="M33" s="53"/>
+      <x:c r="N33" s="51"/>
+    </x:row>
+    <x:row r="34" ht="18" customHeight="1">
+      <x:c r="A34" s="435" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B34" s="435" t="str">
+        <x:v>Target metric</x:v>
+      </x:c>
+      <x:c r="C34" s="435" t="str">
+        <x:v>Metric value</x:v>
+      </x:c>
+      <x:c r="D34" s="460" t="str">
+        <x:v>25th %ile</x:v>
+      </x:c>
+      <x:c r="E34" s="460" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="F34" s="460" t="str">
+        <x:v>75th %ile</x:v>
+      </x:c>
+      <x:c r="G34" s="460" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="H34" s="460" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="I34" s="460" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J34" s="53"/>
+      <x:c r="K34" s="53"/>
+      <x:c r="L34" s="53"/>
+      <x:c r="M34" s="53"/>
+      <x:c r="N34" s="51"/>
+    </x:row>
+    <x:row r="35" ht="18" customHeight="1">
+      <x:c r="A35" s="452" t="str">
+        <x:v>EV / Revenue</x:v>
+      </x:c>
+      <x:c r="B35" s="452" t="str">
+        <x:v>FY2026E revenue</x:v>
+      </x:c>
+      <x:c r="C35" s="453" t="n">
+        <x:f>B24</x:f>
+        <x:v>1140</x:v>
+      </x:c>
+      <x:c r="D35" s="475" t="n">
+        <x:f>I17</x:f>
+        <x:v>4.465</x:v>
+      </x:c>
+      <x:c r="E35" s="475" t="n">
+        <x:f>I18</x:f>
+        <x:v>5.21</x:v>
+      </x:c>
+      <x:c r="F35" s="475" t="n">
+        <x:f>I19</x:f>
+        <x:v>6.855</x:v>
+      </x:c>
+      <x:c r="G35" s="476" t="n">
+        <x:f>(C35*D35+$B$29-$B$30)/$B$31</x:f>
+        <x:v>34.7460112706867</x:v>
+      </x:c>
+      <x:c r="H35" s="477" t="n">
+        <x:f>(C35*E35+$B$29-$B$30)/$B$31</x:f>
+        <x:v>39.79463691268784</x:v>
+      </x:c>
+      <x:c r="I35" s="476" t="n">
+        <x:f>(C35*F35+$B$29-$B$30)/$B$31</x:f>
+        <x:v>50.94227339737494</x:v>
+      </x:c>
+      <x:c r="J35" s="53"/>
+      <x:c r="K35" s="53"/>
+      <x:c r="L35" s="53"/>
+      <x:c r="M35" s="53"/>
+      <x:c r="N35" s="51"/>
+    </x:row>
+    <x:row r="36" ht="18" customHeight="1">
+      <x:c r="A36" s="452" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B36" s="452" t="str">
+        <x:v>FY2026E EBITDA</x:v>
+      </x:c>
+      <x:c r="C36" s="453" t="n">
+        <x:f>B25</x:f>
+        <x:v>330.59999999999997</x:v>
+      </x:c>
+      <x:c r="D36" s="475" t="n">
+        <x:f>J17</x:f>
+        <x:v>17.6675</x:v>
+      </x:c>
+      <x:c r="E36" s="475" t="n">
+        <x:f>J18</x:f>
+        <x:v>19.67</x:v>
+      </x:c>
+      <x:c r="F36" s="475" t="n">
+        <x:f>J19</x:f>
+        <x:v>23.855</x:v>
+      </x:c>
+      <x:c r="G36" s="476" t="n">
+        <x:f>(C36*D36+$B$29-$B$30)/$B$31</x:f>
+        <x:v>39.20896245482214</x:v>
+      </x:c>
+      <x:c r="H36" s="477" t="n">
+        <x:f>(C36*E36+$B$29-$B$30)/$B$31</x:f>
+        <x:v>43.144349201065246</x:v>
+      </x:c>
+      <x:c r="I36" s="476" t="n">
+        <x:f>(C36*F36+$B$29-$B$30)/$B$31</x:f>
+        <x:v>51.36886532242725</x:v>
+      </x:c>
+      <x:c r="J36" s="53"/>
+      <x:c r="K36" s="53"/>
+      <x:c r="L36" s="53"/>
+      <x:c r="M36" s="53"/>
+      <x:c r="N36" s="51"/>
+    </x:row>
+    <x:row r="37" ht="18" customHeight="1">
+      <x:c r="A37" s="452" t="str">
+        <x:v>EV / EBIT</x:v>
+      </x:c>
+      <x:c r="B37" s="452" t="str">
+        <x:v>FY2026E EBIT</x:v>
+      </x:c>
+      <x:c r="C37" s="453" t="n">
+        <x:f>B26</x:f>
+        <x:v>296.4</x:v>
+      </x:c>
+      <x:c r="D37" s="475" t="n">
+        <x:f>K17</x:f>
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="E37" s="475" t="n">
+        <x:f>K18</x:f>
+        <x:v>27.48</x:v>
+      </x:c>
+      <x:c r="F37" s="475" t="n">
+        <x:f>K19</x:f>
+        <x:v>28.855</x:v>
+      </x:c>
+      <x:c r="G37" s="476" t="n">
+        <x:f>(C37*D37+$B$29-$B$30)/$B$31</x:f>
+        <x:v>46.95080963477268</x:v>
+      </x:c>
+      <x:c r="H37" s="477" t="n">
+        <x:f>(C37*E37+$B$29-$B$30)/$B$31</x:f>
+        <x:v>52.9061548887198</x:v>
+      </x:c>
+      <x:c r="I37" s="476" t="n">
+        <x:f>(C37*F37+$B$29-$B$30)/$B$31</x:f>
+        <x:v>55.328817529008944</x:v>
+      </x:c>
+      <x:c r="J37" s="53"/>
+      <x:c r="K37" s="53"/>
+      <x:c r="L37" s="53"/>
+      <x:c r="M37" s="53"/>
+      <x:c r="N37" s="51"/>
+    </x:row>
+    <x:row r="38" ht="18" customHeight="1">
+      <x:c r="A38" s="452" t="str">
+        <x:v>P / E</x:v>
+      </x:c>
+      <x:c r="B38" s="452" t="str">
+        <x:v>FY2026E diluted EPS</x:v>
+      </x:c>
+      <x:c r="C38" s="457" t="n">
+        <x:f>B28</x:f>
+        <x:v>1.4957656056571431</x:v>
+      </x:c>
+      <x:c r="D38" s="475" t="n">
+        <x:f>L17</x:f>
+        <x:v>33.35500000000001</x:v>
+      </x:c>
+      <x:c r="E38" s="475" t="n">
+        <x:f>L18</x:f>
+        <x:v>36.29</x:v>
+      </x:c>
+      <x:c r="F38" s="475" t="n">
+        <x:f>L19</x:f>
+        <x:v>39.27</x:v>
+      </x:c>
+      <x:c r="G38" s="476" t="n">
+        <x:f>C38*D38</x:f>
+        <x:v>49.89126177669402</x:v>
+      </x:c>
+      <x:c r="H38" s="477" t="n">
+        <x:f>C38*E38</x:f>
+        <x:v>54.28133382929772</x:v>
+      </x:c>
+      <x:c r="I38" s="476" t="n">
+        <x:f>C38*F38</x:f>
+        <x:v>58.73871533415601</x:v>
+      </x:c>
+      <x:c r="J38" s="53"/>
+      <x:c r="K38" s="53"/>
+      <x:c r="L38" s="53"/>
+      <x:c r="M38" s="53"/>
+      <x:c r="N38" s="51"/>
+    </x:row>
+    <x:row r="39" ht="18" customHeight="1">
+      <x:c r="A39" s="51"/>
+      <x:c r="B39" s="51"/>
+      <x:c r="C39" s="51"/>
+      <x:c r="D39" s="51"/>
+      <x:c r="E39" s="51"/>
+      <x:c r="F39" s="51"/>
+      <x:c r="G39" s="51"/>
+      <x:c r="H39" s="51"/>
+      <x:c r="I39" s="51"/>
+      <x:c r="J39" s="51"/>
+      <x:c r="K39" s="51"/>
+      <x:c r="L39" s="51"/>
+      <x:c r="M39" s="51"/>
+      <x:c r="N39" s="51"/>
+    </x:row>
+    <x:row r="40" ht="18" customHeight="1">
+      <x:c r="A40" s="434" t="str">
+        <x:v>ANALYST INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="B40" s="434"/>
+      <x:c r="C40" s="434"/>
+      <x:c r="D40" s="434"/>
+      <x:c r="E40" s="434"/>
+      <x:c r="F40" s="434"/>
+      <x:c r="G40" s="434"/>
+      <x:c r="H40" s="434"/>
+      <x:c r="I40" s="434"/>
+      <x:c r="J40" s="434"/>
+      <x:c r="K40" s="434"/>
+      <x:c r="L40" s="434"/>
+      <x:c r="M40" s="434"/>
+      <x:c r="N40" s="434"/>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="458" t="str">
+        <x:v>Cognex trades within a premium industrial-technology universe, but Keyence is a valuation outlier because its operating margin, growth, and direct machine-vision positioning are structurally stronger. The defensible core indication uses the median EV/Revenue and EV/EBITDA outputs; EV/EBIT and P/E remain corroborative.</x:v>
+      </x:c>
+      <x:c r="B41" s="458"/>
+      <x:c r="C41" s="458"/>
+      <x:c r="D41" s="458"/>
+      <x:c r="E41" s="458"/>
+      <x:c r="F41" s="458"/>
+      <x:c r="G41" s="458"/>
+      <x:c r="H41" s="458"/>
+      <x:c r="I41" s="458"/>
+      <x:c r="J41" s="458"/>
+      <x:c r="K41" s="458"/>
+      <x:c r="L41" s="458"/>
+      <x:c r="M41" s="458"/>
+      <x:c r="N41" s="458"/>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="458" t="str">
+        <x:v>Trading comps reflect current market pricing, not intrinsic value. A high peer multiple can embed optimistic growth expectations, market sentiment, or superior quality; it should not be treated as automatic support for a higher acquisition price.</x:v>
+      </x:c>
+      <x:c r="B42" s="458"/>
+      <x:c r="C42" s="458"/>
+      <x:c r="D42" s="458"/>
+      <x:c r="E42" s="458"/>
+      <x:c r="F42" s="458"/>
+      <x:c r="G42" s="458"/>
+      <x:c r="H42" s="458"/>
+      <x:c r="I42" s="458"/>
+      <x:c r="J42" s="458"/>
+      <x:c r="K42" s="458"/>
+      <x:c r="L42" s="458"/>
+      <x:c r="M42" s="458"/>
+      <x:c r="N42" s="458"/>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="459" t="str">
+        <x:v>Source note: Market data are from StockAnalysis pages using S&amp;P Global Market Intelligence. Values are rounded; local-currency equity and enterprise values are shown because valuation multiples are currency-neutral.</x:v>
+      </x:c>
+      <x:c r="B43" s="459"/>
+      <x:c r="C43" s="459"/>
+      <x:c r="D43" s="459"/>
+      <x:c r="E43" s="459"/>
+      <x:c r="F43" s="459"/>
+      <x:c r="G43" s="459"/>
+      <x:c r="H43" s="459"/>
+      <x:c r="I43" s="459"/>
+      <x:c r="J43" s="459"/>
+      <x:c r="K43" s="459"/>
+      <x:c r="L43" s="459"/>
+      <x:c r="M43" s="459"/>
+      <x:c r="N43" s="459"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
+    <x:mergeCell ref="B3:N3"/>
+    <x:mergeCell ref="A5:N5"/>
+    <x:mergeCell ref="A15:H15"/>
+    <x:mergeCell ref="M16:N16"/>
+    <x:mergeCell ref="M17:N17"/>
+    <x:mergeCell ref="M18:N18"/>
+    <x:mergeCell ref="M19:N19"/>
+    <x:mergeCell ref="M20:N20"/>
+    <x:mergeCell ref="A22:F22"/>
+    <x:mergeCell ref="H22:N22"/>
+    <x:mergeCell ref="J23:N23"/>
+    <x:mergeCell ref="J24:N24"/>
+    <x:mergeCell ref="J25:N25"/>
+    <x:mergeCell ref="J26:N26"/>
+    <x:mergeCell ref="J27:N27"/>
+    <x:mergeCell ref="J28:N28"/>
+    <x:mergeCell ref="J29:N29"/>
+    <x:mergeCell ref="A33:I33"/>
+    <x:mergeCell ref="A40:N40"/>
+    <x:mergeCell ref="A41:N41"/>
+    <x:mergeCell ref="A42:N42"/>
+    <x:mergeCell ref="A43:N43"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
valuation: complete precedent transactions analysis
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R82b7a66665894f73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R538195c949f04aa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R72e908968f084ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R7b26245c9cda4f0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R2f1a440f509f4502"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R8f4b6d2c7f7f4d1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Refe0d7a8e3ba47ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Re8181c5b5ef840a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R05b409ad59cb42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rce06b1a8851944b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Raa165e71b20946c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R04b4253de2934be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R3ad46800c16b42d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R4d858d39027a4c11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R91857405d46c46bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R7038611a6b0042ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R71f784f3990241b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R319cddf7749845ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rbf3c9a2c7506416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R32a1501b450c41f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Re562b878824a4b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R61b696e9fd0341ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rfdf965fc2b724fdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R44b6307ce4a54c17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R3d8aa3a477174c41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R55933a4424ad40a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R58296bb6c2914f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R89fab3d8b8aa490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rc95969c520504a56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Re00ffc4bf6084aa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R7b172e5249b64575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Ra4476b6a3505407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rd98a0e85210c44f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R12c407a698c440dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -179,7 +179,7 @@
     <x:numFmt numFmtId="220" formatCode="#,##0"/>
     <x:numFmt numFmtId="221" formatCode="#,##0.0"/>
   </x:numFmts>
-  <x:fonts count="41">
+  <x:fonts count="43">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -410,8 +410,19 @@
       <x:color rgb="FF008000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -551,6 +562,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -806,7 +857,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="487">
+  <x:cellXfs count="598">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1776,6 +1827,251 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="26" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="40" fillId="26" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="35" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="221" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="221" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="221" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="221" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="41" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="41" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="37" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="37" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="36" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="36" fillId="35" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="37" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="33" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2145,7 +2441,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.4 — trading comps complete</x:v>
+        <x:v>0.5 — precedents complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -2200,8 +2496,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="482" t="str">
-        <x:v>TRADING COMPS COMPLETE</x:v>
+      <x:c r="B9" s="594" t="str">
+        <x:v>PRECEDENTS COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -2449,110 +2745,1364 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="535" t="str">
         <x:v>Precedent Transactions</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Comparable acquisition multiples and premiums</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="535"/>
+      <x:c r="C1" s="535"/>
+      <x:c r="D1" s="535"/>
+      <x:c r="E1" s="535"/>
+      <x:c r="F1" s="535"/>
+      <x:c r="G1" s="535"/>
+      <x:c r="H1" s="535"/>
+      <x:c r="I1" s="535"/>
+      <x:c r="J1" s="535"/>
+      <x:c r="K1" s="535"/>
+      <x:c r="L1" s="535"/>
+      <x:c r="M1" s="535"/>
+      <x:c r="N1" s="535"/>
+      <x:c r="O1" s="535"/>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="536" t="str">
+        <x:v>Comparable strategic acquisitions in machine vision, imaging, automation, and industrial software | USD millions unless noted</x:v>
+      </x:c>
+      <x:c r="B2" s="536"/>
+      <x:c r="C2" s="536"/>
+      <x:c r="D2" s="536"/>
+      <x:c r="E2" s="536"/>
+      <x:c r="F2" s="536"/>
+      <x:c r="G2" s="536"/>
+      <x:c r="H2" s="536"/>
+      <x:c r="I2" s="536"/>
+      <x:c r="J2" s="536"/>
+      <x:c r="K2" s="536"/>
+      <x:c r="L2" s="536"/>
+      <x:c r="M2" s="536"/>
+      <x:c r="N2" s="536"/>
+      <x:c r="O2" s="536"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="432" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="537" t="str">
+        <x:v>Complete — seven transactions screened; six included in the core valuation set</x:v>
+      </x:c>
+      <x:c r="C3" s="537"/>
+      <x:c r="D3" s="537"/>
+      <x:c r="E3" s="537"/>
+      <x:c r="F3" s="537"/>
+      <x:c r="G3" s="537"/>
+      <x:c r="H3" s="537"/>
+      <x:c r="I3" s="537"/>
+      <x:c r="J3" s="537"/>
+      <x:c r="K3" s="537"/>
+      <x:c r="L3" s="537"/>
+      <x:c r="M3" s="537"/>
+      <x:c r="N3" s="537"/>
+      <x:c r="O3" s="537"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="538"/>
+      <x:c r="B4" s="538"/>
+      <x:c r="C4" s="538"/>
+      <x:c r="D4" s="538"/>
+      <x:c r="E4" s="538"/>
+      <x:c r="F4" s="538"/>
+      <x:c r="G4" s="538"/>
+      <x:c r="H4" s="538"/>
+      <x:c r="I4" s="538"/>
+      <x:c r="J4" s="538"/>
+      <x:c r="K4" s="538"/>
+      <x:c r="L4" s="538"/>
+      <x:c r="M4" s="538"/>
+      <x:c r="N4" s="538"/>
+      <x:c r="O4" s="538"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="539" t="str">
+        <x:v>SELECTED PRECEDENT TRANSACTIONS</x:v>
+      </x:c>
+      <x:c r="B5" s="539"/>
+      <x:c r="C5" s="539"/>
+      <x:c r="D5" s="539"/>
+      <x:c r="E5" s="539"/>
+      <x:c r="F5" s="539"/>
+      <x:c r="G5" s="539"/>
+      <x:c r="H5" s="539"/>
+      <x:c r="I5" s="539"/>
+      <x:c r="J5" s="539"/>
+      <x:c r="K5" s="539"/>
+      <x:c r="L5" s="539"/>
+      <x:c r="M5" s="539"/>
+      <x:c r="N5" s="539"/>
+      <x:c r="O5" s="539"/>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="540" t="str">
+        <x:v>Announced</x:v>
+      </x:c>
+      <x:c r="B6" s="540" t="str">
+        <x:v>Acquirer</x:v>
+      </x:c>
+      <x:c r="C6" s="540" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="D6" s="540" t="str">
+        <x:v>Strategic relevance</x:v>
+      </x:c>
+      <x:c r="E6" s="571" t="str">
+        <x:v>Core set?</x:v>
+      </x:c>
+      <x:c r="F6" s="571" t="str">
+        <x:v>Transaction EV</x:v>
+      </x:c>
+      <x:c r="G6" s="571" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="H6" s="571" t="str">
+        <x:v>EBITDA</x:v>
+      </x:c>
+      <x:c r="I6" s="571" t="str">
+        <x:v>EBIT</x:v>
+      </x:c>
+      <x:c r="J6" s="571" t="str">
+        <x:v>EV / Revenue</x:v>
+      </x:c>
+      <x:c r="K6" s="571" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="L6" s="571" t="str">
+        <x:v>EV / EBIT</x:v>
+      </x:c>
+      <x:c r="M6" s="571" t="str">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="N6" s="540" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="O6" s="540" t="str">
+        <x:v>Key qualification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="541" t="n">
+        <x:v>43871</x:v>
+      </x:c>
+      <x:c r="B7" s="437" t="str">
+        <x:v>Atlas Copco</x:v>
+      </x:c>
+      <x:c r="C7" s="437" t="str">
+        <x:v>ISRA VISION</x:v>
+      </x:c>
+      <x:c r="D7" s="437" t="str">
+        <x:v>Direct machine vision</x:v>
+      </x:c>
+      <x:c r="E7" s="461" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F7" s="572" t="n">
+        <x:v>1094</x:v>
+      </x:c>
+      <x:c r="G7" s="572" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="H7" s="572"/>
+      <x:c r="I7" s="572" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="J7" s="573" t="n">
+        <x:f>IFERROR(F7/G7,"")</x:f>
+        <x:v>7.103896103896104</x:v>
+      </x:c>
+      <x:c r="K7" s="573" t="str">
+        <x:f>IFERROR(F7/H7,"")</x:f>
+      </x:c>
+      <x:c r="L7" s="573" t="n">
+        <x:f>IFERROR(F7/I7,"")</x:f>
+        <x:v>32.1764705882353</x:v>
+      </x:c>
+      <x:c r="M7" s="574" t="n">
+        <x:v>0.43</x:v>
+      </x:c>
+      <x:c r="N7" s="437" t="str">
+        <x:v>S-040</x:v>
+      </x:c>
+      <x:c r="O7" s="437" t="str">
+        <x:v>Public target; premium is versus prior closing price</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="541" t="n">
+        <x:v>44200</x:v>
+      </x:c>
+      <x:c r="B8" s="437" t="str">
+        <x:v>Teledyne Technologies</x:v>
+      </x:c>
+      <x:c r="C8" s="437" t="str">
+        <x:v>FLIR Systems</x:v>
+      </x:c>
+      <x:c r="D8" s="437" t="str">
+        <x:v>Thermal imaging / sensing</x:v>
+      </x:c>
+      <x:c r="E8" s="461" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F8" s="572" t="n">
+        <x:v>8000</x:v>
+      </x:c>
+      <x:c r="G8" s="572" t="n">
+        <x:v>1923.689</x:v>
+      </x:c>
+      <x:c r="H8" s="572" t="n">
+        <x:v>411.982</x:v>
+      </x:c>
+      <x:c r="I8" s="572" t="n">
+        <x:v>317.242</x:v>
+      </x:c>
+      <x:c r="J8" s="573" t="n">
+        <x:f>IFERROR(F8/G8,"")</x:f>
+        <x:v>4.158676376482893</x:v>
+      </x:c>
+      <x:c r="K8" s="573" t="n">
+        <x:f>IFERROR(F8/H8,"")</x:f>
+        <x:v>19.418324101538417</x:v>
+      </x:c>
+      <x:c r="L8" s="573" t="n">
+        <x:f>IFERROR(F8/I8,"")</x:f>
+        <x:v>25.217341966070066</x:v>
+      </x:c>
+      <x:c r="M8" s="574" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="N8" s="437" t="str">
+        <x:v>S-041 / S-042</x:v>
+      </x:c>
+      <x:c r="O8" s="437" t="str">
+        <x:v>Public target; EBITDA equals EBIT plus reported D&amp;A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="541" t="n">
+        <x:v>44635</x:v>
+      </x:c>
+      <x:c r="B9" s="437" t="str">
+        <x:v>Zebra Technologies</x:v>
+      </x:c>
+      <x:c r="C9" s="437" t="str">
+        <x:v>Matrox Imaging</x:v>
+      </x:c>
+      <x:c r="D9" s="437" t="str">
+        <x:v>Direct machine vision</x:v>
+      </x:c>
+      <x:c r="E9" s="461" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F9" s="572" t="n">
+        <x:v>875</x:v>
+      </x:c>
+      <x:c r="G9" s="572" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H9" s="572"/>
+      <x:c r="I9" s="572"/>
+      <x:c r="J9" s="573" t="n">
+        <x:f>IFERROR(F9/G9,"")</x:f>
+        <x:v>8.75</x:v>
+      </x:c>
+      <x:c r="K9" s="573" t="str">
+        <x:f>IFERROR(F9/H9,"")</x:f>
+      </x:c>
+      <x:c r="L9" s="573" t="str">
+        <x:f>IFERROR(F9/I9,"")</x:f>
+      </x:c>
+      <x:c r="M9" s="574"/>
+      <x:c r="N9" s="437" t="str">
+        <x:v>S-043</x:v>
+      </x:c>
+      <x:c r="O9" s="437" t="str">
+        <x:v>Private target; revenue is management estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="541" t="n">
+        <x:v>45028</x:v>
+      </x:c>
+      <x:c r="B10" s="437" t="str">
+        <x:v>Emerson</x:v>
+      </x:c>
+      <x:c r="C10" s="437" t="str">
+        <x:v>National Instruments</x:v>
+      </x:c>
+      <x:c r="D10" s="437" t="str">
+        <x:v>Test and measurement automation</x:v>
+      </x:c>
+      <x:c r="E10" s="461" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F10" s="572" t="n">
+        <x:v>8467</x:v>
+      </x:c>
+      <x:c r="G10" s="572" t="n">
+        <x:v>1700</x:v>
+      </x:c>
+      <x:c r="H10" s="572"/>
+      <x:c r="I10" s="572"/>
+      <x:c r="J10" s="573" t="n">
+        <x:f>IFERROR(F10/G10,"")</x:f>
+        <x:v>4.9805882352941175</x:v>
+      </x:c>
+      <x:c r="K10" s="573" t="str">
+        <x:f>IFERROR(F10/H10,"")</x:f>
+      </x:c>
+      <x:c r="L10" s="573" t="str">
+        <x:f>IFERROR(F10/I10,"")</x:f>
+      </x:c>
+      <x:c r="M10" s="574" t="n">
+        <x:v>0.49</x:v>
+      </x:c>
+      <x:c r="N10" s="437" t="str">
+        <x:v>S-044 / S-045</x:v>
+      </x:c>
+      <x:c r="O10" s="437" t="str">
+        <x:v>EV uses cash consideration including debt payoff</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="541" t="n">
+        <x:v>45167</x:v>
+      </x:c>
+      <x:c r="B11" s="437" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C11" s="437" t="str">
+        <x:v>Moritex</x:v>
+      </x:c>
+      <x:c r="D11" s="437" t="str">
+        <x:v>Direct machine-vision optics</x:v>
+      </x:c>
+      <x:c r="E11" s="461" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F11" s="572" t="n">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="G11" s="572" t="n">
+        <x:v>70.4</x:v>
+      </x:c>
+      <x:c r="H11" s="572"/>
+      <x:c r="I11" s="572"/>
+      <x:c r="J11" s="573" t="n">
+        <x:f>IFERROR(F11/G11,"")</x:f>
+        <x:v>3.9062499999999996</x:v>
+      </x:c>
+      <x:c r="K11" s="573" t="str">
+        <x:f>IFERROR(F11/H11,"")</x:f>
+      </x:c>
+      <x:c r="L11" s="573" t="str">
+        <x:f>IFERROR(F11/I11,"")</x:f>
+      </x:c>
+      <x:c r="M11" s="574"/>
+      <x:c r="N11" s="437" t="str">
+        <x:v>S-046</x:v>
+      </x:c>
+      <x:c r="O11" s="437" t="str">
+        <x:v>Revenue estimated at midpoint of 6%–8% contribution guidance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="541" t="n">
+        <x:v>45268</x:v>
+      </x:c>
+      <x:c r="B12" s="437" t="str">
+        <x:v>Honeywell</x:v>
+      </x:c>
+      <x:c r="C12" s="437" t="str">
+        <x:v>Carrier Global Access Solutions</x:v>
+      </x:c>
+      <x:c r="D12" s="437" t="str">
+        <x:v>Building automation / access</x:v>
+      </x:c>
+      <x:c r="E12" s="461" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F12" s="572" t="n">
+        <x:v>4950</x:v>
+      </x:c>
+      <x:c r="G12" s="572" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="H12" s="572" t="n">
+        <x:v>291.1764706</x:v>
+      </x:c>
+      <x:c r="I12" s="572"/>
+      <x:c r="J12" s="573" t="n">
+        <x:f>IFERROR(F12/G12,"")</x:f>
+        <x:v>7.071428571428571</x:v>
+      </x:c>
+      <x:c r="K12" s="573" t="n">
+        <x:f>IFERROR(F12/H12,"")</x:f>
+        <x:v>16.99999999931313</x:v>
+      </x:c>
+      <x:c r="L12" s="573" t="str">
+        <x:f>IFERROR(F12/I12,"")</x:f>
+      </x:c>
+      <x:c r="M12" s="574"/>
+      <x:c r="N12" s="437" t="str">
+        <x:v>S-047</x:v>
+      </x:c>
+      <x:c r="O12" s="437" t="str">
+        <x:v>Standalone 17.0x EBITDA; buyer cited 13.0x including synergies/tax benefits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="545" t="n">
+        <x:v>45595</x:v>
+      </x:c>
+      <x:c r="B13" s="546" t="str">
+        <x:v>Siemens</x:v>
+      </x:c>
+      <x:c r="C13" s="546" t="str">
+        <x:v>Altair Engineering</x:v>
+      </x:c>
+      <x:c r="D13" s="546" t="str">
+        <x:v>Industrial software / simulation</x:v>
+      </x:c>
+      <x:c r="E13" s="575" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="F13" s="576" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="G13" s="576" t="n">
+        <x:v>668</x:v>
+      </x:c>
+      <x:c r="H13" s="576" t="n">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="I13" s="576"/>
+      <x:c r="J13" s="577" t="n">
+        <x:f>IFERROR(F13/G13,"")</x:f>
+        <x:v>14.970059880239521</x:v>
+      </x:c>
+      <x:c r="K13" s="577" t="n">
+        <x:f>IFERROR(F13/H13,"")</x:f>
+        <x:v>68.02721088435374</x:v>
+      </x:c>
+      <x:c r="L13" s="577" t="str">
+        <x:f>IFERROR(F13/I13,"")</x:f>
+      </x:c>
+      <x:c r="M13" s="578" t="n">
+        <x:v>0.19</x:v>
+      </x:c>
+      <x:c r="N13" s="546" t="str">
+        <x:v>S-048 / S-049</x:v>
+      </x:c>
+      <x:c r="O13" s="546" t="str">
+        <x:v>Excluded from core set as high-growth software valuation outlier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="18" customHeight="1">
+      <x:c r="A14" s="538"/>
+      <x:c r="B14" s="538"/>
+      <x:c r="C14" s="538"/>
+      <x:c r="D14" s="538"/>
+      <x:c r="E14" s="579"/>
+      <x:c r="F14" s="579"/>
+      <x:c r="G14" s="579"/>
+      <x:c r="H14" s="579"/>
+      <x:c r="I14" s="579"/>
+      <x:c r="J14" s="580"/>
+      <x:c r="K14" s="580"/>
+      <x:c r="L14" s="580"/>
+      <x:c r="M14" s="581"/>
+      <x:c r="N14" s="538"/>
+      <x:c r="O14" s="538"/>
+    </x:row>
+    <x:row r="15" ht="18" customHeight="1">
+      <x:c r="A15" s="539" t="str">
+        <x:v>SELECTED TRANSACTION STATISTICS</x:v>
+      </x:c>
+      <x:c r="B15" s="539"/>
+      <x:c r="C15" s="539"/>
+      <x:c r="D15" s="539"/>
+      <x:c r="E15" s="582"/>
+      <x:c r="F15" s="582"/>
+      <x:c r="G15" s="582"/>
+      <x:c r="H15" s="582"/>
+      <x:c r="I15" s="582"/>
+      <x:c r="J15" s="583" t="str">
+        <x:v>EV / Revenue</x:v>
+      </x:c>
+      <x:c r="K15" s="583" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="L15" s="583" t="str">
+        <x:v>EV / EBIT</x:v>
+      </x:c>
+      <x:c r="M15" s="584" t="str">
+        <x:v>Premium</x:v>
+      </x:c>
+      <x:c r="N15" s="538"/>
+      <x:c r="O15" s="538"/>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1">
+      <x:c r="A16" s="436" t="str">
+        <x:v>Minimum</x:v>
+      </x:c>
+      <x:c r="B16" s="436"/>
+      <x:c r="C16" s="436"/>
+      <x:c r="D16" s="436"/>
+      <x:c r="E16" s="585"/>
+      <x:c r="F16" s="585"/>
+      <x:c r="G16" s="585"/>
+      <x:c r="H16" s="585"/>
+      <x:c r="I16" s="585"/>
+      <x:c r="J16" s="573" t="n">
+        <x:f>MIN(J$7:J$12)</x:f>
+        <x:v>3.9062499999999996</x:v>
+      </x:c>
+      <x:c r="K16" s="573" t="n">
+        <x:f>MIN(K$7:K$12)</x:f>
+        <x:v>16.99999999931313</x:v>
+      </x:c>
+      <x:c r="L16" s="573" t="n">
+        <x:f>MIN(L$7:L$12)</x:f>
+        <x:v>25.217341966070066</x:v>
+      </x:c>
+      <x:c r="M16" s="574" t="n">
+        <x:f>MIN(M$7:M$13)</x:f>
+        <x:v>0.19</x:v>
+      </x:c>
+      <x:c r="N16" s="554" t="str">
+        <x:v>Core multiples exclude Altair; premium statistics include public targets with disclosed unaffected-price premiums.</x:v>
+      </x:c>
+      <x:c r="O16" s="554"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="436" t="str">
+        <x:v>25th percentile</x:v>
+      </x:c>
+      <x:c r="B17" s="436"/>
+      <x:c r="C17" s="436"/>
+      <x:c r="D17" s="436"/>
+      <x:c r="E17" s="585"/>
+      <x:c r="F17" s="585"/>
+      <x:c r="G17" s="585"/>
+      <x:c r="H17" s="585"/>
+      <x:c r="I17" s="585"/>
+      <x:c r="J17" s="573" t="n">
+        <x:f>PERCENTILE.INC(J$7:J$12,25%)</x:f>
+        <x:v>4.3641543411857</x:v>
+      </x:c>
+      <x:c r="K17" s="573" t="n">
+        <x:f>PERCENTILE.INC(K$7:K$12,25%)</x:f>
+        <x:v>17.60458102486945</x:v>
+      </x:c>
+      <x:c r="L17" s="573" t="n">
+        <x:f>PERCENTILE.INC(L$7:L$12,25%)</x:f>
+        <x:v>26.95712412161137</x:v>
+      </x:c>
+      <x:c r="M17" s="574" t="n">
+        <x:f>PERCENTILE.INC(M$7:M$13,25%)</x:f>
+        <x:v>0.3475</x:v>
+      </x:c>
+      <x:c r="N17" s="554"/>
+      <x:c r="O17" s="554"/>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1">
+      <x:c r="A18" s="555" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="B18" s="555"/>
+      <x:c r="C18" s="555"/>
+      <x:c r="D18" s="555"/>
+      <x:c r="E18" s="586"/>
+      <x:c r="F18" s="586"/>
+      <x:c r="G18" s="586"/>
+      <x:c r="H18" s="586"/>
+      <x:c r="I18" s="586"/>
+      <x:c r="J18" s="587" t="n">
+        <x:f>MEDIAN(J$7:J$12)</x:f>
+        <x:v>6.026008403361344</x:v>
+      </x:c>
+      <x:c r="K18" s="587" t="n">
+        <x:f>MEDIAN(K$7:K$12)</x:f>
+        <x:v>18.209162050425775</x:v>
+      </x:c>
+      <x:c r="L18" s="587" t="n">
+        <x:f>MEDIAN(L$7:L$12)</x:f>
+        <x:v>28.69690627715268</x:v>
+      </x:c>
+      <x:c r="M18" s="588" t="n">
+        <x:f>MEDIAN(M$7:M$13)</x:f>
+        <x:v>0.41500000000000004</x:v>
+      </x:c>
+      <x:c r="N18" s="554"/>
+      <x:c r="O18" s="554"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="436" t="str">
+        <x:v>75th percentile</x:v>
+      </x:c>
+      <x:c r="B19" s="436"/>
+      <x:c r="C19" s="436"/>
+      <x:c r="D19" s="436"/>
+      <x:c r="E19" s="585"/>
+      <x:c r="F19" s="585"/>
+      <x:c r="G19" s="585"/>
+      <x:c r="H19" s="585"/>
+      <x:c r="I19" s="585"/>
+      <x:c r="J19" s="573" t="n">
+        <x:f>PERCENTILE.INC(J$7:J$12,75%)</x:f>
+        <x:v>7.09577922077922</x:v>
+      </x:c>
+      <x:c r="K19" s="573" t="n">
+        <x:f>PERCENTILE.INC(K$7:K$12,75%)</x:f>
+        <x:v>18.8137430759821</x:v>
+      </x:c>
+      <x:c r="L19" s="573" t="n">
+        <x:f>PERCENTILE.INC(L$7:L$12,75%)</x:f>
+        <x:v>30.43668843269399</x:v>
+      </x:c>
+      <x:c r="M19" s="574" t="n">
+        <x:f>PERCENTILE.INC(M$7:M$13,75%)</x:f>
+        <x:v>0.445</x:v>
+      </x:c>
+      <x:c r="N19" s="554"/>
+      <x:c r="O19" s="554"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="436" t="str">
+        <x:v>Maximum</x:v>
+      </x:c>
+      <x:c r="B20" s="436"/>
+      <x:c r="C20" s="436"/>
+      <x:c r="D20" s="436"/>
+      <x:c r="E20" s="585"/>
+      <x:c r="F20" s="585"/>
+      <x:c r="G20" s="585"/>
+      <x:c r="H20" s="585"/>
+      <x:c r="I20" s="585"/>
+      <x:c r="J20" s="573" t="n">
+        <x:f>MAX(J$7:J$12)</x:f>
+        <x:v>8.75</x:v>
+      </x:c>
+      <x:c r="K20" s="573" t="n">
+        <x:f>MAX(K$7:K$12)</x:f>
+        <x:v>19.418324101538417</x:v>
+      </x:c>
+      <x:c r="L20" s="573" t="n">
+        <x:f>MAX(L$7:L$12)</x:f>
+        <x:v>32.1764705882353</x:v>
+      </x:c>
+      <x:c r="M20" s="574" t="n">
+        <x:f>MAX(M$7:M$13)</x:f>
+        <x:v>0.49</x:v>
+      </x:c>
+      <x:c r="N20" s="554"/>
+      <x:c r="O20" s="554"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="538"/>
+      <x:c r="B21" s="538"/>
+      <x:c r="C21" s="538"/>
+      <x:c r="D21" s="538"/>
+      <x:c r="E21" s="579"/>
+      <x:c r="F21" s="579"/>
+      <x:c r="G21" s="579"/>
+      <x:c r="H21" s="579"/>
+      <x:c r="I21" s="579"/>
+      <x:c r="J21" s="579"/>
+      <x:c r="K21" s="579"/>
+      <x:c r="L21" s="579"/>
+      <x:c r="M21" s="579"/>
+      <x:c r="N21" s="538"/>
+      <x:c r="O21" s="538"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="539" t="str">
+        <x:v>COGNEX VALUATION INPUTS</x:v>
+      </x:c>
+      <x:c r="B22" s="539"/>
+      <x:c r="C22" s="539"/>
+      <x:c r="D22" s="539"/>
+      <x:c r="E22" s="582"/>
+      <x:c r="F22" s="582"/>
+      <x:c r="G22" s="579"/>
+      <x:c r="H22" s="582" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I22" s="582"/>
+      <x:c r="J22" s="582"/>
+      <x:c r="K22" s="582"/>
+      <x:c r="L22" s="582"/>
+      <x:c r="M22" s="582"/>
+      <x:c r="N22" s="539"/>
+      <x:c r="O22" s="539"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="558" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B23" s="558" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C23" s="558" t="str">
+        <x:v>Units</x:v>
+      </x:c>
+      <x:c r="D23" s="558" t="str">
+        <x:v>Source / methodology</x:v>
+      </x:c>
+      <x:c r="E23" s="579"/>
+      <x:c r="F23" s="579"/>
+      <x:c r="G23" s="579"/>
+      <x:c r="H23" s="585" t="str">
+        <x:v>DCF implied value / share</x:v>
+      </x:c>
+      <x:c r="I23" s="589" t="n">
+        <x:f>'DCF'!H8</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="J23" s="585" t="str">
+        <x:v>Standalone intrinsic-value reference</x:v>
+      </x:c>
+      <x:c r="K23" s="585"/>
+      <x:c r="L23" s="585"/>
+      <x:c r="M23" s="585"/>
+      <x:c r="N23" s="436"/>
+      <x:c r="O23" s="436"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="436" t="str">
+        <x:v>FY2026E revenue</x:v>
+      </x:c>
+      <x:c r="B24" s="560" t="n">
+        <x:f>'CGNX Operating Model'!E20</x:f>
+        <x:v>1140</x:v>
+      </x:c>
+      <x:c r="C24" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D24" s="436" t="str">
+        <x:v>CGNX Operating Model</x:v>
+      </x:c>
+      <x:c r="E24" s="579"/>
+      <x:c r="F24" s="579"/>
+      <x:c r="G24" s="579"/>
+      <x:c r="H24" s="585" t="str">
+        <x:v>Trading comps core low</x:v>
+      </x:c>
+      <x:c r="I24" s="589" t="n">
+        <x:f>'Trading Comps'!I26</x:f>
+        <x:v>39.79463691268784</x:v>
+      </x:c>
+      <x:c r="J24" s="585" t="str">
+        <x:v>Lower median public-company indication</x:v>
+      </x:c>
+      <x:c r="K24" s="585"/>
+      <x:c r="L24" s="585"/>
+      <x:c r="M24" s="585"/>
+      <x:c r="N24" s="436"/>
+      <x:c r="O24" s="436"/>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1">
+      <x:c r="A25" s="436" t="str">
+        <x:v>FY2026E EBITDA</x:v>
+      </x:c>
+      <x:c r="B25" s="560" t="n">
+        <x:f>'CGNX Operating Model'!E32</x:f>
+        <x:v>330.59999999999997</x:v>
+      </x:c>
+      <x:c r="C25" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D25" s="436" t="str">
+        <x:v>CGNX Operating Model</x:v>
+      </x:c>
+      <x:c r="E25" s="579"/>
+      <x:c r="F25" s="579"/>
+      <x:c r="G25" s="579"/>
+      <x:c r="H25" s="585" t="str">
+        <x:v>Trading comps core high</x:v>
+      </x:c>
+      <x:c r="I25" s="589" t="n">
+        <x:f>'Trading Comps'!I27</x:f>
+        <x:v>43.144349201065246</x:v>
+      </x:c>
+      <x:c r="J25" s="585" t="str">
+        <x:v>Upper median public-company indication</x:v>
+      </x:c>
+      <x:c r="K25" s="585"/>
+      <x:c r="L25" s="585"/>
+      <x:c r="M25" s="585"/>
+      <x:c r="N25" s="436"/>
+      <x:c r="O25" s="436"/>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="436" t="str">
+        <x:v>FY2026E EBIT</x:v>
+      </x:c>
+      <x:c r="B26" s="560" t="n">
+        <x:f>'CGNX Operating Model'!E29</x:f>
+        <x:v>296.4</x:v>
+      </x:c>
+      <x:c r="C26" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D26" s="436" t="str">
+        <x:v>CGNX Operating Model</x:v>
+      </x:c>
+      <x:c r="E26" s="579"/>
+      <x:c r="F26" s="579"/>
+      <x:c r="G26" s="579"/>
+      <x:c r="H26" s="585" t="str">
+        <x:v>Precedent core median low</x:v>
+      </x:c>
+      <x:c r="I26" s="589" t="n">
+        <x:f>MIN(H35:H36)</x:f>
+        <x:v>40.27345666415471</x:v>
+      </x:c>
+      <x:c r="J26" s="585" t="str">
+        <x:v>Lower median of precedent EV/Revenue and EV/EBITDA</x:v>
+      </x:c>
+      <x:c r="K26" s="585"/>
+      <x:c r="L26" s="585"/>
+      <x:c r="M26" s="585"/>
+      <x:c r="N26" s="436"/>
+      <x:c r="O26" s="436"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="436" t="str">
+        <x:v>Cash and investments</x:v>
+      </x:c>
+      <x:c r="B27" s="560" t="n">
+        <x:f>'DCF'!B19</x:f>
+        <x:v>755.013</x:v>
+      </x:c>
+      <x:c r="C27" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D27" s="436" t="str">
+        <x:v>S-022 / DCF</x:v>
+      </x:c>
+      <x:c r="E27" s="579"/>
+      <x:c r="F27" s="579"/>
+      <x:c r="G27" s="579"/>
+      <x:c r="H27" s="585" t="str">
+        <x:v>Precedent core median high</x:v>
+      </x:c>
+      <x:c r="I27" s="589" t="n">
+        <x:f>MAX(H35:H36)</x:f>
+        <x:v>45.32446369026972</x:v>
+      </x:c>
+      <x:c r="J27" s="585" t="str">
+        <x:v>Upper median of precedent EV/Revenue and EV/EBITDA</x:v>
+      </x:c>
+      <x:c r="K27" s="585"/>
+      <x:c r="L27" s="585"/>
+      <x:c r="M27" s="585"/>
+      <x:c r="N27" s="436"/>
+      <x:c r="O27" s="436"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="436" t="str">
+        <x:v>Debt</x:v>
+      </x:c>
+      <x:c r="B28" s="560" t="n">
+        <x:f>'DCF'!B20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C28" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D28" s="436" t="str">
+        <x:v>S-022 / DCF</x:v>
+      </x:c>
+      <x:c r="E28" s="579"/>
+      <x:c r="F28" s="579"/>
+      <x:c r="G28" s="579"/>
+      <x:c r="H28" s="585" t="str">
+        <x:v>Median premium indication</x:v>
+      </x:c>
+      <x:c r="I28" s="589" t="n">
+        <x:f>H38</x:f>
+        <x:v>84.51795</x:v>
+      </x:c>
+      <x:c r="J28" s="585" t="str">
+        <x:v>Current price plus median disclosed control premium</x:v>
+      </x:c>
+      <x:c r="K28" s="585"/>
+      <x:c r="L28" s="585"/>
+      <x:c r="M28" s="585"/>
+      <x:c r="N28" s="436"/>
+      <x:c r="O28" s="436"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="436" t="str">
+        <x:v>Diluted shares</x:v>
+      </x:c>
+      <x:c r="B29" s="560" t="n">
+        <x:f>'DCF'!B21</x:f>
+        <x:v>168.224</x:v>
+      </x:c>
+      <x:c r="C29" s="436" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D29" s="436" t="str">
+        <x:v>S-022 / DCF</x:v>
+      </x:c>
+      <x:c r="E29" s="579"/>
+      <x:c r="F29" s="579"/>
+      <x:c r="G29" s="579"/>
+      <x:c r="H29" s="585" t="str">
+        <x:v>Median announced premium</x:v>
+      </x:c>
+      <x:c r="I29" s="588" t="n">
+        <x:f>M18</x:f>
+        <x:v>0.41500000000000004</x:v>
+      </x:c>
+      <x:c r="J29" s="585" t="str">
+        <x:v>Public-target premium sample; reference dates vary</x:v>
+      </x:c>
+      <x:c r="K29" s="585"/>
+      <x:c r="L29" s="585"/>
+      <x:c r="M29" s="585"/>
+      <x:c r="N29" s="436"/>
+      <x:c r="O29" s="436"/>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="436" t="str">
+        <x:v>Current share price</x:v>
+      </x:c>
+      <x:c r="B30" s="561" t="n">
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="C30" s="436" t="str">
+        <x:v>$ / share</x:v>
+      </x:c>
+      <x:c r="D30" s="436" t="str">
+        <x:v>S-039</x:v>
+      </x:c>
+      <x:c r="E30" s="579"/>
+      <x:c r="F30" s="579"/>
+      <x:c r="G30" s="579"/>
+      <x:c r="H30" s="585" t="str">
+        <x:v>Valuation implication</x:v>
+      </x:c>
+      <x:c r="I30" s="585"/>
+      <x:c r="J30" s="585" t="str">
+        <x:v>A credible offer must clear the unaffected market price; fundamentals alone do not support the premium indication.</x:v>
+      </x:c>
+      <x:c r="K30" s="585"/>
+      <x:c r="L30" s="585"/>
+      <x:c r="M30" s="585"/>
+      <x:c r="N30" s="436"/>
+      <x:c r="O30" s="436"/>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="A31" s="436" t="str">
+        <x:v>Analysis date</x:v>
+      </x:c>
+      <x:c r="B31" s="541" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="C31" s="436" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="D31" s="436" t="str">
+        <x:v>S-039</x:v>
+      </x:c>
+      <x:c r="E31" s="579"/>
+      <x:c r="F31" s="579"/>
+      <x:c r="G31" s="579"/>
+      <x:c r="H31" s="579"/>
+      <x:c r="I31" s="579"/>
+      <x:c r="J31" s="579"/>
+      <x:c r="K31" s="579"/>
+      <x:c r="L31" s="579"/>
+      <x:c r="M31" s="579"/>
+      <x:c r="N31" s="538"/>
+      <x:c r="O31" s="538"/>
+    </x:row>
+    <x:row r="32" ht="18" customHeight="1">
+      <x:c r="A32" s="538"/>
+      <x:c r="B32" s="538"/>
+      <x:c r="C32" s="538"/>
+      <x:c r="D32" s="538"/>
+      <x:c r="E32" s="579"/>
+      <x:c r="F32" s="579"/>
+      <x:c r="G32" s="579"/>
+      <x:c r="H32" s="579"/>
+      <x:c r="I32" s="579"/>
+      <x:c r="J32" s="579"/>
+      <x:c r="K32" s="579"/>
+      <x:c r="L32" s="579"/>
+      <x:c r="M32" s="579"/>
+      <x:c r="N32" s="538"/>
+      <x:c r="O32" s="538"/>
+    </x:row>
+    <x:row r="33" ht="18" customHeight="1">
+      <x:c r="A33" s="539" t="str">
+        <x:v>IMPLIED COGNEX EQUITY VALUE PER SHARE</x:v>
+      </x:c>
+      <x:c r="B33" s="539"/>
+      <x:c r="C33" s="539"/>
+      <x:c r="D33" s="539"/>
+      <x:c r="E33" s="582"/>
+      <x:c r="F33" s="582"/>
+      <x:c r="G33" s="582"/>
+      <x:c r="H33" s="582"/>
+      <x:c r="I33" s="582"/>
+      <x:c r="J33" s="579"/>
+      <x:c r="K33" s="579"/>
+      <x:c r="L33" s="579"/>
+      <x:c r="M33" s="579"/>
+      <x:c r="N33" s="538"/>
+      <x:c r="O33" s="538"/>
+    </x:row>
+    <x:row r="34" ht="18" customHeight="1">
+      <x:c r="A34" s="540" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B34" s="540" t="str">
+        <x:v>Target metric</x:v>
+      </x:c>
+      <x:c r="C34" s="540" t="str">
+        <x:v>Metric value</x:v>
+      </x:c>
+      <x:c r="D34" s="540" t="str">
+        <x:v>25th %ile</x:v>
+      </x:c>
+      <x:c r="E34" s="571" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="F34" s="571" t="str">
+        <x:v>75th %ile</x:v>
+      </x:c>
+      <x:c r="G34" s="571" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="H34" s="571" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="I34" s="571" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J34" s="579"/>
+      <x:c r="K34" s="579"/>
+      <x:c r="L34" s="579"/>
+      <x:c r="M34" s="579"/>
+      <x:c r="N34" s="538"/>
+      <x:c r="O34" s="538"/>
+    </x:row>
+    <x:row r="35" ht="18" customHeight="1">
+      <x:c r="A35" s="562" t="str">
+        <x:v>EV / Revenue</x:v>
+      </x:c>
+      <x:c r="B35" s="562" t="str">
+        <x:v>FY2026E revenue</x:v>
+      </x:c>
+      <x:c r="C35" s="563" t="n">
+        <x:f>B24</x:f>
+        <x:v>1140</x:v>
+      </x:c>
+      <x:c r="D35" s="564" t="n">
+        <x:f>J17</x:f>
+        <x:v>4.3641543411857</x:v>
+      </x:c>
+      <x:c r="E35" s="590" t="n">
+        <x:f>J18</x:f>
+        <x:v>6.026008403361344</x:v>
+      </x:c>
+      <x:c r="F35" s="590" t="n">
+        <x:f>J19</x:f>
+        <x:v>7.09577922077922</x:v>
+      </x:c>
+      <x:c r="G35" s="591" t="n">
+        <x:f>(C35*D35+$B$27-$B$28)/$B$29</x:f>
+        <x:v>34.0626126411909</x:v>
+      </x:c>
+      <x:c r="H35" s="592" t="n">
+        <x:f>(C35*E35+$B$27-$B$28)/$B$29</x:f>
+        <x:v>45.32446369026972</x:v>
+      </x:c>
+      <x:c r="I35" s="591" t="n">
+        <x:f>(C35*F35+$B$27-$B$28)/$B$29</x:f>
+        <x:v>52.57395681762598</x:v>
+      </x:c>
+      <x:c r="J35" s="579"/>
+      <x:c r="K35" s="579"/>
+      <x:c r="L35" s="579"/>
+      <x:c r="M35" s="579"/>
+      <x:c r="N35" s="538"/>
+      <x:c r="O35" s="538"/>
+    </x:row>
+    <x:row r="36" ht="18" customHeight="1">
+      <x:c r="A36" s="562" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B36" s="562" t="str">
+        <x:v>FY2026E EBITDA</x:v>
+      </x:c>
+      <x:c r="C36" s="563" t="n">
+        <x:f>B25</x:f>
+        <x:v>330.59999999999997</x:v>
+      </x:c>
+      <x:c r="D36" s="564" t="n">
+        <x:f>K17</x:f>
+        <x:v>17.60458102486945</x:v>
+      </x:c>
+      <x:c r="E36" s="590" t="n">
+        <x:f>K18</x:f>
+        <x:v>18.209162050425775</x:v>
+      </x:c>
+      <x:c r="F36" s="590" t="n">
+        <x:f>K19</x:f>
+        <x:v>18.8137430759821</x:v>
+      </x:c>
+      <x:c r="G36" s="591" t="n">
+        <x:f>(C36*D36+$B$27-$B$28)/$B$29</x:f>
+        <x:v>39.08531176777297</x:v>
+      </x:c>
+      <x:c r="H36" s="592" t="n">
+        <x:f>(C36*E36+$B$27-$B$28)/$B$29</x:f>
+        <x:v>40.27345666415471</x:v>
+      </x:c>
+      <x:c r="I36" s="591" t="n">
+        <x:f>(C36*F36+$B$27-$B$28)/$B$29</x:f>
+        <x:v>41.46160156053644</x:v>
+      </x:c>
+      <x:c r="J36" s="579"/>
+      <x:c r="K36" s="579"/>
+      <x:c r="L36" s="579"/>
+      <x:c r="M36" s="579"/>
+      <x:c r="N36" s="538"/>
+      <x:c r="O36" s="538"/>
+    </x:row>
+    <x:row r="37" ht="18" customHeight="1">
+      <x:c r="A37" s="562" t="str">
+        <x:v>EV / EBIT</x:v>
+      </x:c>
+      <x:c r="B37" s="562" t="str">
+        <x:v>FY2026E EBIT</x:v>
+      </x:c>
+      <x:c r="C37" s="563" t="n">
+        <x:f>B26</x:f>
+        <x:v>296.4</x:v>
+      </x:c>
+      <x:c r="D37" s="564" t="n">
+        <x:f>L17</x:f>
+        <x:v>26.95712412161137</x:v>
+      </x:c>
+      <x:c r="E37" s="590" t="n">
+        <x:f>L18</x:f>
+        <x:v>28.69690627715268</x:v>
+      </x:c>
+      <x:c r="F37" s="590" t="n">
+        <x:f>L19</x:f>
+        <x:v>30.43668843269399</x:v>
+      </x:c>
+      <x:c r="G37" s="591" t="n">
+        <x:f>(C37*D37+$B$27-$B$28)/$B$29</x:f>
+        <x:v>51.98488081157034</x:v>
+      </x:c>
+      <x:c r="H37" s="592" t="n">
+        <x:f>(C37*E37+$B$27-$B$28)/$B$29</x:f>
+        <x:v>55.05026643373155</x:v>
+      </x:c>
+      <x:c r="I37" s="591" t="n">
+        <x:f>(C37*F37+$B$27-$B$28)/$B$29</x:f>
+        <x:v>58.11565205589273</x:v>
+      </x:c>
+      <x:c r="J37" s="579"/>
+      <x:c r="K37" s="579"/>
+      <x:c r="L37" s="579"/>
+      <x:c r="M37" s="579"/>
+      <x:c r="N37" s="538"/>
+      <x:c r="O37" s="538"/>
+    </x:row>
+    <x:row r="38" ht="18" customHeight="1">
+      <x:c r="A38" s="562" t="str">
+        <x:v>Premium paid</x:v>
+      </x:c>
+      <x:c r="B38" s="562" t="str">
+        <x:v>Current share price</x:v>
+      </x:c>
+      <x:c r="C38" s="567" t="n">
+        <x:f>B30</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="D38" s="568" t="n">
+        <x:f>M17</x:f>
+        <x:v>0.3475</x:v>
+      </x:c>
+      <x:c r="E38" s="593" t="n">
+        <x:f>M18</x:f>
+        <x:v>0.41500000000000004</x:v>
+      </x:c>
+      <x:c r="F38" s="593" t="n">
+        <x:f>M19</x:f>
+        <x:v>0.445</x:v>
+      </x:c>
+      <x:c r="G38" s="591" t="n">
+        <x:f>C38*(1+D38)</x:f>
+        <x:v>80.48617499999999</x:v>
+      </x:c>
+      <x:c r="H38" s="592" t="n">
+        <x:f>C38*(1+E38)</x:f>
+        <x:v>84.51795</x:v>
+      </x:c>
+      <x:c r="I38" s="591" t="n">
+        <x:f>C38*(1+F38)</x:f>
+        <x:v>86.30985</x:v>
+      </x:c>
+      <x:c r="J38" s="579"/>
+      <x:c r="K38" s="579"/>
+      <x:c r="L38" s="579"/>
+      <x:c r="M38" s="579"/>
+      <x:c r="N38" s="538"/>
+      <x:c r="O38" s="538"/>
+    </x:row>
+    <x:row r="39" ht="18" customHeight="1">
+      <x:c r="A39" s="538"/>
+      <x:c r="B39" s="538"/>
+      <x:c r="C39" s="538"/>
+      <x:c r="D39" s="538"/>
+      <x:c r="E39" s="538"/>
+      <x:c r="F39" s="538"/>
+      <x:c r="G39" s="538"/>
+      <x:c r="H39" s="538"/>
+      <x:c r="I39" s="538"/>
+      <x:c r="J39" s="538"/>
+      <x:c r="K39" s="538"/>
+      <x:c r="L39" s="538"/>
+      <x:c r="M39" s="538"/>
+      <x:c r="N39" s="538"/>
+      <x:c r="O39" s="538"/>
+    </x:row>
+    <x:row r="40" ht="18" customHeight="1">
+      <x:c r="A40" s="539" t="str">
+        <x:v>ANALYST INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="B40" s="539"/>
+      <x:c r="C40" s="539"/>
+      <x:c r="D40" s="539"/>
+      <x:c r="E40" s="539"/>
+      <x:c r="F40" s="539"/>
+      <x:c r="G40" s="539"/>
+      <x:c r="H40" s="539"/>
+      <x:c r="I40" s="539"/>
+      <x:c r="J40" s="539"/>
+      <x:c r="K40" s="539"/>
+      <x:c r="L40" s="539"/>
+      <x:c r="M40" s="539"/>
+      <x:c r="N40" s="539"/>
+      <x:c r="O40" s="539"/>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="569" t="str">
+        <x:v>Precedent transactions generally imply higher values than the DCF because strategic buyers pay for control, scarcity, and expected synergies. However, the median premium method indicates a value well above the fundamental multiple-based ranges, creating a clear overpayment and value-sharing question for Rockwell.</x:v>
+      </x:c>
+      <x:c r="B41" s="569"/>
+      <x:c r="C41" s="569"/>
+      <x:c r="D41" s="569"/>
+      <x:c r="E41" s="569"/>
+      <x:c r="F41" s="569"/>
+      <x:c r="G41" s="569"/>
+      <x:c r="H41" s="569"/>
+      <x:c r="I41" s="569"/>
+      <x:c r="J41" s="569"/>
+      <x:c r="K41" s="569"/>
+      <x:c r="L41" s="569"/>
+      <x:c r="M41" s="569"/>
+      <x:c r="N41" s="569"/>
+      <x:c r="O41" s="569"/>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="569" t="str">
+        <x:v>The core precedent range emphasizes EV/Revenue and EV/EBITDA. EV/EBIT is corroborative because only two transactions disclose sufficient EBIT data. Altair is shown but excluded from the core multiple statistics because industrial-software economics are not directly comparable to Cognex hardware-led machine vision.</x:v>
+      </x:c>
+      <x:c r="B42" s="569"/>
+      <x:c r="C42" s="569"/>
+      <x:c r="D42" s="569"/>
+      <x:c r="E42" s="569"/>
+      <x:c r="F42" s="569"/>
+      <x:c r="G42" s="569"/>
+      <x:c r="H42" s="569"/>
+      <x:c r="I42" s="569"/>
+      <x:c r="J42" s="569"/>
+      <x:c r="K42" s="569"/>
+      <x:c r="L42" s="569"/>
+      <x:c r="M42" s="569"/>
+      <x:c r="N42" s="569"/>
+      <x:c r="O42" s="569"/>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="570" t="str">
+        <x:v>Data limitation: Private-company and carve-out disclosures are incomplete. Moritex revenue is estimated from management contribution guidance; Matrox revenue is an announced estimate; premium references use different unaffected-price periods.</x:v>
+      </x:c>
+      <x:c r="B43" s="570"/>
+      <x:c r="C43" s="570"/>
+      <x:c r="D43" s="570"/>
+      <x:c r="E43" s="570"/>
+      <x:c r="F43" s="570"/>
+      <x:c r="G43" s="570"/>
+      <x:c r="H43" s="570"/>
+      <x:c r="I43" s="570"/>
+      <x:c r="J43" s="570"/>
+      <x:c r="K43" s="570"/>
+      <x:c r="L43" s="570"/>
+      <x:c r="M43" s="570"/>
+      <x:c r="N43" s="570"/>
+      <x:c r="O43" s="570"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="B3:O3"/>
+    <x:mergeCell ref="A5:O5"/>
+    <x:mergeCell ref="A15:I15"/>
+    <x:mergeCell ref="N16:O16"/>
+    <x:mergeCell ref="N17:O17"/>
+    <x:mergeCell ref="N18:O18"/>
+    <x:mergeCell ref="N19:O19"/>
+    <x:mergeCell ref="N20:O20"/>
+    <x:mergeCell ref="A22:F22"/>
+    <x:mergeCell ref="H22:O22"/>
+    <x:mergeCell ref="J23:O23"/>
+    <x:mergeCell ref="J24:O24"/>
+    <x:mergeCell ref="J25:O25"/>
+    <x:mergeCell ref="J26:O26"/>
+    <x:mergeCell ref="J27:O27"/>
+    <x:mergeCell ref="J28:O28"/>
+    <x:mergeCell ref="J29:O29"/>
+    <x:mergeCell ref="J30:O30"/>
+    <x:mergeCell ref="A33:I33"/>
+    <x:mergeCell ref="A40:O40"/>
+    <x:mergeCell ref="A41:O41"/>
+    <x:mergeCell ref="A42:O42"/>
+    <x:mergeCell ref="A43:O43"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3273,8 +4823,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="483" t="str">
-        <x:v>TRADING COMPS COMPLETE</x:v>
+      <x:c r="B3" s="595" t="str">
+        <x:v>PRECEDENTS COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -3320,10 +4870,10 @@
       </x:c>
       <x:c r="B6" s="134" t="n">
         <x:f>COUNTA('Sources'!A4:A100)</x:f>
-        <x:v>17</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C6" s="135" t="n">
-        <x:v>17</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D6" s="135" t="n">
         <x:f>B6-C6</x:f>
@@ -3806,6 +5356,84 @@
       </x:c>
       <x:c r="G24" s="484" t="str">
         <x:v>Trading Comps row 35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="484" t="str">
+        <x:v>Precedent target-metric links</x:v>
+      </x:c>
+      <x:c r="B25" s="484" t="n">
+        <x:f>ABS('Precedent Transactions'!B24-'CGNX Operating Model'!E20)+ABS('Precedent Transactions'!B25-'CGNX Operating Model'!E32)+ABS('Precedent Transactions'!B27-'DCF'!B19)+ABS('Precedent Transactions'!B29-'DCF'!B21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C25" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D25" s="484" t="n">
+        <x:f>B25-C25</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E25" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F25" s="597" t="str">
+        <x:f>IF(ABS(D25)&lt;=E25,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G25" s="484" t="str">
+        <x:v>Precedent Transactions rows 24-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="484" t="str">
+        <x:v>Precedent multiple calculations</x:v>
+      </x:c>
+      <x:c r="B26" s="484" t="n">
+        <x:f>ABS('Precedent Transactions'!J7-'Precedent Transactions'!F7/'Precedent Transactions'!G7)+ABS('Precedent Transactions'!K8-'Precedent Transactions'!F8/'Precedent Transactions'!H8)+ABS('Precedent Transactions'!L8-'Precedent Transactions'!F8/'Precedent Transactions'!I8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C26" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D26" s="484" t="n">
+        <x:f>B26-C26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F26" s="597" t="str">
+        <x:f>IF(ABS(D26)&lt;=E26,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G26" s="484" t="str">
+        <x:v>Precedent Transactions rows 7-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="484" t="str">
+        <x:v>Precedent quartile ordering</x:v>
+      </x:c>
+      <x:c r="B27" s="484" t="n">
+        <x:f>MIN('Precedent Transactions'!H35-'Precedent Transactions'!G35,'Precedent Transactions'!I35-'Precedent Transactions'!H35,'Precedent Transactions'!H36-'Precedent Transactions'!G36,'Precedent Transactions'!I36-'Precedent Transactions'!H36,'Precedent Transactions'!H37-'Precedent Transactions'!G37,'Precedent Transactions'!I37-'Precedent Transactions'!H37,'Precedent Transactions'!H38-'Precedent Transactions'!G38,'Precedent Transactions'!I38-'Precedent Transactions'!H38)</x:f>
+        <x:v>1.1881448963817292</x:v>
+      </x:c>
+      <x:c r="C27" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D27" s="484" t="n">
+        <x:f>MIN(0,B27-C27)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F27" s="597" t="str">
+        <x:f>IF(ABS(D27)&lt;=E27,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G27" s="484" t="str">
+        <x:v>Precedent Transactions rows 35-38</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5563,6 +7191,292 @@
         <x:v>S&amp;P Global Market Intelligence; USD values</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="32" customHeight="1">
+      <x:c r="A21" s="480" t="str">
+        <x:v>S-039</x:v>
+      </x:c>
+      <x:c r="B21" s="480" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C21" s="480" t="str">
+        <x:v>Stock price and statistics</x:v>
+      </x:c>
+      <x:c r="D21" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="E21" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F21" s="480" t="str">
+        <x:v>Unaffected share-price reference for premium analysis</x:v>
+      </x:c>
+      <x:c r="G21" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/cgnx/</x:v>
+      </x:c>
+      <x:c r="H21" s="480" t="str">
+        <x:v>$59.73 closing price on Aug. 20, 2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="32" customHeight="1">
+      <x:c r="A22" s="480" t="str">
+        <x:v>S-040</x:v>
+      </x:c>
+      <x:c r="B22" s="480" t="str">
+        <x:v>Atlas Copco / ISRA VISION</x:v>
+      </x:c>
+      <x:c r="C22" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D22" s="481" t="n">
+        <x:v>43871</x:v>
+      </x:c>
+      <x:c r="E22" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F22" s="480" t="str">
+        <x:v>EV, revenue, EBIT and premium</x:v>
+      </x:c>
+      <x:c r="G22" s="480" t="str">
+        <x:v>https://www.atlascopcogroup.com/en/media/press-releases/2020/20200210-isra</x:v>
+      </x:c>
+      <x:c r="H22" s="480" t="str">
+        <x:v>Primary buyer announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="32" customHeight="1">
+      <x:c r="A23" s="480" t="str">
+        <x:v>S-041</x:v>
+      </x:c>
+      <x:c r="B23" s="480" t="str">
+        <x:v>Teledyne / FLIR</x:v>
+      </x:c>
+      <x:c r="C23" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D23" s="481" t="n">
+        <x:v>44200</x:v>
+      </x:c>
+      <x:c r="E23" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F23" s="480" t="str">
+        <x:v>Transaction value and premium</x:v>
+      </x:c>
+      <x:c r="G23" s="480" t="str">
+        <x:v>https://www.teledyne.com/en-us/news/Pages/Teledyne-to-Acquire-FLIR-Systems.aspx</x:v>
+      </x:c>
+      <x:c r="H23" s="480" t="str">
+        <x:v>Primary joint announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="32" customHeight="1">
+      <x:c r="A24" s="480" t="str">
+        <x:v>S-042</x:v>
+      </x:c>
+      <x:c r="B24" s="480" t="str">
+        <x:v>FLIR Systems</x:v>
+      </x:c>
+      <x:c r="C24" s="480" t="str">
+        <x:v>FY2020 Form 10-K</x:v>
+      </x:c>
+      <x:c r="D24" s="481" t="n">
+        <x:v>44253</x:v>
+      </x:c>
+      <x:c r="E24" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F24" s="480" t="str">
+        <x:v>Revenue, EBIT and D&amp;A</x:v>
+      </x:c>
+      <x:c r="G24" s="480" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/354908/000035490821000016/flir-20201231.htm</x:v>
+      </x:c>
+      <x:c r="H24" s="480" t="str">
+        <x:v>Primary audited filing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="32" customHeight="1">
+      <x:c r="A25" s="480" t="str">
+        <x:v>S-043</x:v>
+      </x:c>
+      <x:c r="B25" s="480" t="str">
+        <x:v>Zebra / Matrox Imaging</x:v>
+      </x:c>
+      <x:c r="C25" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D25" s="481" t="n">
+        <x:v>44635</x:v>
+      </x:c>
+      <x:c r="E25" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F25" s="480" t="str">
+        <x:v>Purchase price and annual-sales estimate</x:v>
+      </x:c>
+      <x:c r="G25" s="480" t="str">
+        <x:v>https://www.zebra.com/us/en/about-zebra/newsroom/press-releases/2022/zebra-technologies-to-acquire-matrox-imaging.html</x:v>
+      </x:c>
+      <x:c r="H25" s="480" t="str">
+        <x:v>Primary buyer announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="32" customHeight="1">
+      <x:c r="A26" s="480" t="str">
+        <x:v>S-044</x:v>
+      </x:c>
+      <x:c r="B26" s="480" t="str">
+        <x:v>Emerson / NI</x:v>
+      </x:c>
+      <x:c r="C26" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D26" s="481" t="n">
+        <x:v>45028</x:v>
+      </x:c>
+      <x:c r="E26" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F26" s="480" t="str">
+        <x:v>Equity value, revenue, premium and synergies</x:v>
+      </x:c>
+      <x:c r="G26" s="480" t="str">
+        <x:v>https://www.emerson.com/en/corporate/news/2023/04-emerson-ni-acquisition</x:v>
+      </x:c>
+      <x:c r="H26" s="480" t="str">
+        <x:v>Primary joint announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="32" customHeight="1">
+      <x:c r="A27" s="480" t="str">
+        <x:v>S-045</x:v>
+      </x:c>
+      <x:c r="B27" s="480" t="str">
+        <x:v>Emerson</x:v>
+      </x:c>
+      <x:c r="C27" s="480" t="str">
+        <x:v>Q2 FY2024 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="D27" s="481" t="n">
+        <x:v>45420</x:v>
+      </x:c>
+      <x:c r="E27" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F27" s="480" t="str">
+        <x:v>NI cash consideration including debt payoff</x:v>
+      </x:c>
+      <x:c r="G27" s="480" t="str">
+        <x:v>https://ir.emerson.com/sec-filings/all-sec-filings/content/0000032604-24-000024/emr-20240331.htm</x:v>
+      </x:c>
+      <x:c r="H27" s="480" t="str">
+        <x:v>Primary SEC filing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="32" customHeight="1">
+      <x:c r="A28" s="480" t="str">
+        <x:v>S-046</x:v>
+      </x:c>
+      <x:c r="B28" s="480" t="str">
+        <x:v>Cognex / Moritex</x:v>
+      </x:c>
+      <x:c r="C28" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D28" s="481" t="n">
+        <x:v>45167</x:v>
+      </x:c>
+      <x:c r="E28" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F28" s="480" t="str">
+        <x:v>Purchase price and expected revenue contribution</x:v>
+      </x:c>
+      <x:c r="G28" s="480" t="str">
+        <x:v>https://investor.cognex.com/news/news-details/2023/Cognex-To-Acquire-Moritex-Corporation-A-Global-Leader-In-Machine-Vision-Optics-Components-And-Advanced-Imaging-Solutions/default.aspx</x:v>
+      </x:c>
+      <x:c r="H28" s="480" t="str">
+        <x:v>Primary buyer announcement; revenue estimated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="32" customHeight="1">
+      <x:c r="A29" s="480" t="str">
+        <x:v>S-047</x:v>
+      </x:c>
+      <x:c r="B29" s="480" t="str">
+        <x:v>Honeywell / Carrier</x:v>
+      </x:c>
+      <x:c r="C29" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D29" s="481" t="n">
+        <x:v>45268</x:v>
+      </x:c>
+      <x:c r="E29" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F29" s="480" t="str">
+        <x:v>Transaction EV and EBITDA multiples</x:v>
+      </x:c>
+      <x:c r="G29" s="480" t="str">
+        <x:v>https://investor.honeywell.com/news-releases/news-release-details/honeywell-strengthen-building-automation-business-acquisition</x:v>
+      </x:c>
+      <x:c r="H29" s="480" t="str">
+        <x:v>Primary buyer announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="32" customHeight="1">
+      <x:c r="A30" s="480" t="str">
+        <x:v>S-048</x:v>
+      </x:c>
+      <x:c r="B30" s="480" t="str">
+        <x:v>Siemens / Altair</x:v>
+      </x:c>
+      <x:c r="C30" s="480" t="str">
+        <x:v>Transaction announcement</x:v>
+      </x:c>
+      <x:c r="D30" s="481" t="n">
+        <x:v>45595</x:v>
+      </x:c>
+      <x:c r="E30" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F30" s="480" t="str">
+        <x:v>Transaction EV and premium</x:v>
+      </x:c>
+      <x:c r="G30" s="480" t="str">
+        <x:v>https://press.siemens.com/global/en/pressrelease/siemens-strengthens-leadership-industrial-software-and-ai-acquisition-altair</x:v>
+      </x:c>
+      <x:c r="H30" s="480" t="str">
+        <x:v>Primary buyer announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="32" customHeight="1">
+      <x:c r="A31" s="480" t="str">
+        <x:v>S-049</x:v>
+      </x:c>
+      <x:c r="B31" s="480" t="str">
+        <x:v>Altair Engineering</x:v>
+      </x:c>
+      <x:c r="C31" s="480" t="str">
+        <x:v>FY2024 results</x:v>
+      </x:c>
+      <x:c r="D31" s="481" t="n">
+        <x:v>45708</x:v>
+      </x:c>
+      <x:c r="E31" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F31" s="480" t="str">
+        <x:v>Revenue and adjusted EBITDA reference</x:v>
+      </x:c>
+      <x:c r="G31" s="480" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1701732/000095017025024159/altr-ex99_1.htm</x:v>
+      </x:c>
+      <x:c r="H31" s="480" t="str">
+        <x:v>Primary company release furnished to SEC</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -6971,7 +8885,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd135bb5cbd5f498b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1253d88ebc414e4b"/>
 </x:worksheet>
 </file>
 
@@ -8694,7 +10608,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf398b0ed9c26405e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf434cbab284f21"/>
 </x:worksheet>
 </file>
 
@@ -12181,7 +14095,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R294eee8d3d4f44cf"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R097f1c7c90d54033"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
valuation: complete valuation summary and football field
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R319cddf7749845ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rbf3c9a2c7506416c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R32a1501b450c41f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Re562b878824a4b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R61b696e9fd0341ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rfdf965fc2b724fdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R44b6307ce4a54c17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R3d8aa3a477174c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R55933a4424ad40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R58296bb6c2914f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R89fab3d8b8aa490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rc95969c520504a56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Re00ffc4bf6084aa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R7b172e5249b64575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Ra4476b6a3505407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rd98a0e85210c44f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R12c407a698c440dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R457d4c52bdcc45f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rd87ba725cd3a44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R5a63c95d72c3428f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Ra482baaf475e49c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rc9ed7c9300674339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Reaf29fdd19b447f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R457c5431ff534f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R28af15ad8b4f45b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="Rf75f54d46c3a4ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rd60ea701054f404a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R84a0f26357144bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Ra0c34c6de1cc485c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R795df57cfade41f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="Rbe8d072268be4b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Ra790963faba54537"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R726f1438037b465f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R8938b613068843b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="22">
+  <x:numFmts count="24">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -178,8 +178,10 @@
     <x:numFmt numFmtId="219" formatCode="0.000x"/>
     <x:numFmt numFmtId="220" formatCode="#,##0"/>
     <x:numFmt numFmtId="221" formatCode="#,##0.0"/>
+    <x:numFmt numFmtId="222" formatCode=";;;"/>
+    <x:numFmt numFmtId="223" formatCode="$0"/>
   </x:numFmts>
-  <x:fonts count="43">
+  <x:fonts count="45">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -421,8 +423,20 @@
       <x:color rgb="FF008000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="8"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="39">
+  <x:fills count="47">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -614,8 +628,48 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8F8F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="23">
+  <x:borders count="24">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -853,11 +907,25 @@
         <x:color rgb="FFD9E1F2"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7E6E6"/>
+      </x:top>
+      <x:bottom style="double">
+        <x:color rgb="FF17365D"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="598">
+  <x:cellXfs count="706">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2072,11 +2140,239 @@
     <x:xf numFmtId="0" fontId="26" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="33" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="40" fillId="33" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="34" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="35" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="36" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="43" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="43" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="44" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="46" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="222" fontId="38" fillId="46" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="222" fontId="38" fillId="46" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="39" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="43" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="215" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="218" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="37" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="223" fontId="44" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="43" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="37" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="223" fontId="44" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="222" fontId="38" fillId="46" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="222" fontId="38" fillId="46" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="43" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="18" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="17" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="43" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="44" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="37" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="45" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="17">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -2140,6 +2436,116 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF7F7F7F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF7F7F7F"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF2F75B5"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF2F75B5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF2F75B5"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF2F75B5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF2F75B5"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF2F75B5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF2F75B5"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF2F75B5"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF70AD47"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF70AD47"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF70AD47"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF70AD47"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF70AD47"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF70AD47"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFF4B183"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4B183"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFFFD966"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFD966"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF17365D"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FF17365D"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -2441,7 +2847,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.5 — precedents complete</x:v>
+        <x:v>0.6 — valuation summary complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -2496,8 +2902,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="594" t="str">
-        <x:v>PRECEDENTS COMPLETE</x:v>
+      <x:c r="B9" s="702" t="str">
+        <x:v>VALUATION COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -4112,111 +4518,2923 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="4.199999809265137" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="4.199999809265137" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="649" t="str">
         <x:v>Valuation Summary</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Valuation synthesis, football field, and offer framework</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="649"/>
+      <x:c r="C1" s="649"/>
+      <x:c r="D1" s="649"/>
+      <x:c r="E1" s="649"/>
+      <x:c r="F1" s="649"/>
+      <x:c r="G1" s="649"/>
+      <x:c r="H1" s="649"/>
+      <x:c r="I1" s="649"/>
+      <x:c r="J1" s="649"/>
+      <x:c r="K1" s="649"/>
+      <x:c r="L1" s="649"/>
+      <x:c r="M1" s="649"/>
+      <x:c r="N1" s="649"/>
+      <x:c r="O1" s="649"/>
+      <x:c r="P1" s="649"/>
+      <x:c r="Q1" s="649"/>
+      <x:c r="R1" s="649"/>
+      <x:c r="S1" s="649"/>
+      <x:c r="T1" s="649"/>
+      <x:c r="U1" s="649"/>
+      <x:c r="V1" s="649"/>
+      <x:c r="W1" s="649"/>
+      <x:c r="X1" s="649"/>
+      <x:c r="Y1" s="649"/>
+      <x:c r="Z1" s="649"/>
+      <x:c r="AA1" s="649"/>
+      <x:c r="AB1" s="649"/>
+      <x:c r="AC1" s="649"/>
+      <x:c r="AD1" s="649"/>
+      <x:c r="AE1" s="649"/>
+      <x:c r="AF1" s="649"/>
+      <x:c r="AG1" s="649"/>
+      <x:c r="AH1" s="649"/>
+      <x:c r="AI1" s="649"/>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="650" t="str">
+        <x:v>Cognex standalone valuation, acquisition framework, and football field | USD millions except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="650"/>
+      <x:c r="C2" s="650"/>
+      <x:c r="D2" s="650"/>
+      <x:c r="E2" s="650"/>
+      <x:c r="F2" s="650"/>
+      <x:c r="G2" s="650"/>
+      <x:c r="H2" s="650"/>
+      <x:c r="I2" s="650"/>
+      <x:c r="J2" s="650"/>
+      <x:c r="K2" s="650"/>
+      <x:c r="L2" s="650"/>
+      <x:c r="M2" s="650"/>
+      <x:c r="N2" s="650"/>
+      <x:c r="O2" s="650"/>
+      <x:c r="P2" s="650"/>
+      <x:c r="Q2" s="650"/>
+      <x:c r="R2" s="650"/>
+      <x:c r="S2" s="650"/>
+      <x:c r="T2" s="650"/>
+      <x:c r="U2" s="650"/>
+      <x:c r="V2" s="650"/>
+      <x:c r="W2" s="650"/>
+      <x:c r="X2" s="650"/>
+      <x:c r="Y2" s="650"/>
+      <x:c r="Z2" s="650"/>
+      <x:c r="AA2" s="650"/>
+      <x:c r="AB2" s="650"/>
+      <x:c r="AC2" s="650"/>
+      <x:c r="AD2" s="650"/>
+      <x:c r="AE2" s="650"/>
+      <x:c r="AF2" s="650"/>
+      <x:c r="AG2" s="650"/>
+      <x:c r="AH2" s="650"/>
+      <x:c r="AI2" s="650"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="432" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="651" t="str">
+        <x:v>Complete — standalone valuation reconciled; illustrative acquisition range established for transaction modeling</x:v>
+      </x:c>
+      <x:c r="C3" s="651"/>
+      <x:c r="D3" s="651"/>
+      <x:c r="E3" s="651"/>
+      <x:c r="F3" s="651"/>
+      <x:c r="G3" s="651"/>
+      <x:c r="H3" s="651"/>
+      <x:c r="I3" s="651"/>
+      <x:c r="J3" s="651"/>
+      <x:c r="K3" s="651"/>
+      <x:c r="L3" s="651"/>
+      <x:c r="M3" s="651"/>
+      <x:c r="N3" s="651"/>
+      <x:c r="O3" s="651"/>
+      <x:c r="P3" s="651"/>
+      <x:c r="Q3" s="651"/>
+      <x:c r="R3" s="651"/>
+      <x:c r="S3" s="651"/>
+      <x:c r="T3" s="651"/>
+      <x:c r="U3" s="651"/>
+      <x:c r="V3" s="651"/>
+      <x:c r="W3" s="651"/>
+      <x:c r="X3" s="651"/>
+      <x:c r="Y3" s="651"/>
+      <x:c r="Z3" s="651"/>
+      <x:c r="AA3" s="651"/>
+      <x:c r="AB3" s="651"/>
+      <x:c r="AC3" s="651"/>
+      <x:c r="AD3" s="651"/>
+      <x:c r="AE3" s="651"/>
+      <x:c r="AF3" s="651"/>
+      <x:c r="AG3" s="651"/>
+      <x:c r="AH3" s="651"/>
+      <x:c r="AI3" s="651"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="538"/>
+      <x:c r="B4" s="538"/>
+      <x:c r="C4" s="538"/>
+      <x:c r="D4" s="538"/>
+      <x:c r="E4" s="538"/>
+      <x:c r="F4" s="538"/>
+      <x:c r="G4" s="538"/>
+      <x:c r="H4" s="538"/>
+      <x:c r="I4" s="538"/>
+      <x:c r="J4" s="538"/>
+      <x:c r="K4" s="538"/>
+      <x:c r="L4" s="538"/>
+      <x:c r="M4" s="538"/>
+      <x:c r="N4" s="538"/>
+      <x:c r="O4" s="538"/>
+      <x:c r="P4" s="538"/>
+      <x:c r="Q4" s="538"/>
+      <x:c r="R4" s="538"/>
+      <x:c r="S4" s="538"/>
+      <x:c r="T4" s="538"/>
+      <x:c r="U4" s="538"/>
+      <x:c r="V4" s="538"/>
+      <x:c r="W4" s="538"/>
+      <x:c r="X4" s="538"/>
+      <x:c r="Y4" s="538"/>
+      <x:c r="Z4" s="538"/>
+      <x:c r="AA4" s="538"/>
+      <x:c r="AB4" s="538"/>
+      <x:c r="AC4" s="538"/>
+      <x:c r="AD4" s="538"/>
+      <x:c r="AE4" s="538"/>
+      <x:c r="AF4" s="538"/>
+      <x:c r="AG4" s="538"/>
+      <x:c r="AH4" s="538"/>
+      <x:c r="AI4" s="538"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="652" t="str">
+        <x:v>KEY VALUATION CONCLUSIONS</x:v>
+      </x:c>
+      <x:c r="B5" s="652"/>
+      <x:c r="C5" s="652"/>
+      <x:c r="D5" s="652"/>
+      <x:c r="E5" s="652"/>
+      <x:c r="F5" s="652"/>
+      <x:c r="G5" s="652"/>
+      <x:c r="H5" s="652"/>
+      <x:c r="I5" s="652"/>
+      <x:c r="J5" s="652"/>
+      <x:c r="K5" s="652"/>
+      <x:c r="L5" s="652"/>
+      <x:c r="M5" s="652"/>
+      <x:c r="N5" s="652"/>
+      <x:c r="O5" s="652"/>
+      <x:c r="P5" s="652"/>
+      <x:c r="Q5" s="652"/>
+      <x:c r="R5" s="652"/>
+      <x:c r="S5" s="652"/>
+      <x:c r="T5" s="652"/>
+      <x:c r="U5" s="652"/>
+      <x:c r="V5" s="652"/>
+      <x:c r="W5" s="652"/>
+      <x:c r="X5" s="652"/>
+      <x:c r="Y5" s="652"/>
+      <x:c r="Z5" s="652"/>
+      <x:c r="AA5" s="652"/>
+      <x:c r="AB5" s="652"/>
+      <x:c r="AC5" s="652"/>
+      <x:c r="AD5" s="652"/>
+      <x:c r="AE5" s="652"/>
+      <x:c r="AF5" s="652"/>
+      <x:c r="AG5" s="652"/>
+      <x:c r="AH5" s="652"/>
+      <x:c r="AI5" s="652"/>
+    </x:row>
+    <x:row r="6" ht="20" customHeight="1">
+      <x:c r="A6" s="653" t="str">
+        <x:v>Unaffected share price</x:v>
+      </x:c>
+      <x:c r="B6" s="681" t="n">
+        <x:f>'Precedent Transactions'!B30</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="C6" s="682"/>
+      <x:c r="D6" s="585"/>
+      <x:c r="E6" s="683" t="str">
+        <x:v>Equity purchase price</x:v>
+      </x:c>
+      <x:c r="F6" s="684" t="n">
+        <x:f>B9*'DCF'!B21</x:f>
+        <x:v>13457.919999999998</x:v>
+      </x:c>
+      <x:c r="G6" s="538"/>
+      <x:c r="H6" s="657" t="str">
+        <x:v>Conclusion: Cognex trades above the standalone DCF and most operating-multiple indications. A $75–$85 acquisition range reflects the premium needed to obtain control, not standalone intrinsic value. The $80 midpoint must therefore be justified through strategic value and synergies, and it will be tested—not assumed—in the financing and accretion/dilution analysis.</x:v>
+      </x:c>
+      <x:c r="I6" s="657"/>
+      <x:c r="J6" s="657"/>
+      <x:c r="K6" s="657"/>
+      <x:c r="L6" s="657"/>
+      <x:c r="M6" s="657"/>
+      <x:c r="N6" s="657"/>
+      <x:c r="O6" s="657"/>
+      <x:c r="P6" s="657"/>
+      <x:c r="Q6" s="657"/>
+      <x:c r="R6" s="657"/>
+      <x:c r="S6" s="657"/>
+      <x:c r="T6" s="657"/>
+      <x:c r="U6" s="657"/>
+      <x:c r="V6" s="657"/>
+      <x:c r="W6" s="657"/>
+      <x:c r="X6" s="657"/>
+      <x:c r="Y6" s="657"/>
+      <x:c r="Z6" s="657"/>
+      <x:c r="AA6" s="657"/>
+      <x:c r="AB6" s="657"/>
+      <x:c r="AC6" s="657"/>
+      <x:c r="AD6" s="657"/>
+      <x:c r="AE6" s="657"/>
+      <x:c r="AF6" s="657"/>
+      <x:c r="AG6" s="657"/>
+      <x:c r="AH6" s="657"/>
+      <x:c r="AI6" s="657"/>
+    </x:row>
+    <x:row r="7" ht="20" customHeight="1">
+      <x:c r="A7" s="653" t="str">
+        <x:v>Standalone fundamental value</x:v>
+      </x:c>
+      <x:c r="B7" s="685" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C7" s="685" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D7" s="585" t="str">
+        <x:v>Low / High</x:v>
+      </x:c>
+      <x:c r="E7" s="683" t="str">
+        <x:v>Transaction enterprise value</x:v>
+      </x:c>
+      <x:c r="F7" s="684" t="n">
+        <x:f>F6-'DCF'!B19+'DCF'!B20</x:f>
+        <x:v>12702.906999999997</x:v>
+      </x:c>
+      <x:c r="G7" s="538"/>
+      <x:c r="H7" s="657"/>
+      <x:c r="I7" s="657"/>
+      <x:c r="J7" s="657"/>
+      <x:c r="K7" s="657"/>
+      <x:c r="L7" s="657"/>
+      <x:c r="M7" s="657"/>
+      <x:c r="N7" s="657"/>
+      <x:c r="O7" s="657"/>
+      <x:c r="P7" s="657"/>
+      <x:c r="Q7" s="657"/>
+      <x:c r="R7" s="657"/>
+      <x:c r="S7" s="657"/>
+      <x:c r="T7" s="657"/>
+      <x:c r="U7" s="657"/>
+      <x:c r="V7" s="657"/>
+      <x:c r="W7" s="657"/>
+      <x:c r="X7" s="657"/>
+      <x:c r="Y7" s="657"/>
+      <x:c r="Z7" s="657"/>
+      <x:c r="AA7" s="657"/>
+      <x:c r="AB7" s="657"/>
+      <x:c r="AC7" s="657"/>
+      <x:c r="AD7" s="657"/>
+      <x:c r="AE7" s="657"/>
+      <x:c r="AF7" s="657"/>
+      <x:c r="AG7" s="657"/>
+      <x:c r="AH7" s="657"/>
+      <x:c r="AI7" s="657"/>
+    </x:row>
+    <x:row r="8" ht="20" customHeight="1">
+      <x:c r="A8" s="653" t="str">
+        <x:v>Acquisition negotiation range</x:v>
+      </x:c>
+      <x:c r="B8" s="685" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C8" s="685" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D8" s="585" t="str">
+        <x:v>Low / High</x:v>
+      </x:c>
+      <x:c r="E8" s="683" t="str">
+        <x:v>Implied EV / FY2026E revenue</x:v>
+      </x:c>
+      <x:c r="F8" s="686" t="n">
+        <x:f>F7/'CGNX Operating Model'!E20</x:f>
+        <x:v>11.14290087719298</x:v>
+      </x:c>
+      <x:c r="G8" s="538"/>
+      <x:c r="H8" s="657"/>
+      <x:c r="I8" s="657"/>
+      <x:c r="J8" s="657"/>
+      <x:c r="K8" s="657"/>
+      <x:c r="L8" s="657"/>
+      <x:c r="M8" s="657"/>
+      <x:c r="N8" s="657"/>
+      <x:c r="O8" s="657"/>
+      <x:c r="P8" s="657"/>
+      <x:c r="Q8" s="657"/>
+      <x:c r="R8" s="657"/>
+      <x:c r="S8" s="657"/>
+      <x:c r="T8" s="657"/>
+      <x:c r="U8" s="657"/>
+      <x:c r="V8" s="657"/>
+      <x:c r="W8" s="657"/>
+      <x:c r="X8" s="657"/>
+      <x:c r="Y8" s="657"/>
+      <x:c r="Z8" s="657"/>
+      <x:c r="AA8" s="657"/>
+      <x:c r="AB8" s="657"/>
+      <x:c r="AC8" s="657"/>
+      <x:c r="AD8" s="657"/>
+      <x:c r="AE8" s="657"/>
+      <x:c r="AF8" s="657"/>
+      <x:c r="AG8" s="657"/>
+      <x:c r="AH8" s="657"/>
+      <x:c r="AI8" s="657"/>
+    </x:row>
+    <x:row r="9" ht="20" customHeight="1">
+      <x:c r="A9" s="653" t="str">
+        <x:v>Illustrative offer / share</x:v>
+      </x:c>
+      <x:c r="B9" s="687" t="n">
+        <x:f>AVERAGE(B8:C8)</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C9" s="682"/>
+      <x:c r="D9" s="585"/>
+      <x:c r="E9" s="683" t="str">
+        <x:v>Implied EV / FY2026E EBITDA</x:v>
+      </x:c>
+      <x:c r="F9" s="686" t="n">
+        <x:f>F7/'CGNX Operating Model'!E32</x:f>
+        <x:v>38.42379612825166</x:v>
+      </x:c>
+      <x:c r="G9" s="538"/>
+      <x:c r="H9" s="657"/>
+      <x:c r="I9" s="657"/>
+      <x:c r="J9" s="657"/>
+      <x:c r="K9" s="657"/>
+      <x:c r="L9" s="657"/>
+      <x:c r="M9" s="657"/>
+      <x:c r="N9" s="657"/>
+      <x:c r="O9" s="657"/>
+      <x:c r="P9" s="657"/>
+      <x:c r="Q9" s="657"/>
+      <x:c r="R9" s="657"/>
+      <x:c r="S9" s="657"/>
+      <x:c r="T9" s="657"/>
+      <x:c r="U9" s="657"/>
+      <x:c r="V9" s="657"/>
+      <x:c r="W9" s="657"/>
+      <x:c r="X9" s="657"/>
+      <x:c r="Y9" s="657"/>
+      <x:c r="Z9" s="657"/>
+      <x:c r="AA9" s="657"/>
+      <x:c r="AB9" s="657"/>
+      <x:c r="AC9" s="657"/>
+      <x:c r="AD9" s="657"/>
+      <x:c r="AE9" s="657"/>
+      <x:c r="AF9" s="657"/>
+      <x:c r="AG9" s="657"/>
+      <x:c r="AH9" s="657"/>
+      <x:c r="AI9" s="657"/>
+    </x:row>
+    <x:row r="10" ht="20" customHeight="1">
+      <x:c r="A10" s="653" t="str">
+        <x:v>Premium to unaffected price</x:v>
+      </x:c>
+      <x:c r="B10" s="688" t="n">
+        <x:f>B9/B6-1</x:f>
+        <x:v>0.3393604553825549</x:v>
+      </x:c>
+      <x:c r="C10" s="585"/>
+      <x:c r="D10" s="585"/>
+      <x:c r="E10" s="683" t="str">
+        <x:v>Implied FY2026E P / E</x:v>
+      </x:c>
+      <x:c r="F10" s="686" t="n">
+        <x:f>B9/'Trading Comps'!B28</x:f>
+        <x:v>53.484315789473676</x:v>
+      </x:c>
+      <x:c r="G10" s="538"/>
+      <x:c r="H10" s="657"/>
+      <x:c r="I10" s="657"/>
+      <x:c r="J10" s="657"/>
+      <x:c r="K10" s="657"/>
+      <x:c r="L10" s="657"/>
+      <x:c r="M10" s="657"/>
+      <x:c r="N10" s="657"/>
+      <x:c r="O10" s="657"/>
+      <x:c r="P10" s="657"/>
+      <x:c r="Q10" s="657"/>
+      <x:c r="R10" s="657"/>
+      <x:c r="S10" s="657"/>
+      <x:c r="T10" s="657"/>
+      <x:c r="U10" s="657"/>
+      <x:c r="V10" s="657"/>
+      <x:c r="W10" s="657"/>
+      <x:c r="X10" s="657"/>
+      <x:c r="Y10" s="657"/>
+      <x:c r="Z10" s="657"/>
+      <x:c r="AA10" s="657"/>
+      <x:c r="AB10" s="657"/>
+      <x:c r="AC10" s="657"/>
+      <x:c r="AD10" s="657"/>
+      <x:c r="AE10" s="657"/>
+      <x:c r="AF10" s="657"/>
+      <x:c r="AG10" s="657"/>
+      <x:c r="AH10" s="657"/>
+      <x:c r="AI10" s="657"/>
+    </x:row>
+    <x:row r="11" ht="18" customHeight="1">
+      <x:c r="A11" s="538"/>
+      <x:c r="B11" s="579"/>
+      <x:c r="C11" s="579"/>
+      <x:c r="D11" s="579"/>
+      <x:c r="E11" s="579"/>
+      <x:c r="F11" s="579"/>
+      <x:c r="G11" s="538"/>
+      <x:c r="H11" s="538"/>
+      <x:c r="I11" s="538"/>
+      <x:c r="J11" s="538"/>
+      <x:c r="K11" s="538"/>
+      <x:c r="L11" s="538"/>
+      <x:c r="M11" s="538"/>
+      <x:c r="N11" s="538"/>
+      <x:c r="O11" s="538"/>
+      <x:c r="P11" s="538"/>
+      <x:c r="Q11" s="538"/>
+      <x:c r="R11" s="538"/>
+      <x:c r="S11" s="538"/>
+      <x:c r="T11" s="538"/>
+      <x:c r="U11" s="538"/>
+      <x:c r="V11" s="538"/>
+      <x:c r="W11" s="538"/>
+      <x:c r="X11" s="538"/>
+      <x:c r="Y11" s="538"/>
+      <x:c r="Z11" s="538"/>
+      <x:c r="AA11" s="538"/>
+      <x:c r="AB11" s="538"/>
+      <x:c r="AC11" s="538"/>
+      <x:c r="AD11" s="538"/>
+      <x:c r="AE11" s="538"/>
+      <x:c r="AF11" s="538"/>
+      <x:c r="AG11" s="538"/>
+      <x:c r="AH11" s="538"/>
+      <x:c r="AI11" s="538"/>
+    </x:row>
+    <x:row r="12" ht="18" customHeight="1">
+      <x:c r="A12" s="652" t="str">
+        <x:v>VALUATION METHOD RANGES</x:v>
+      </x:c>
+      <x:c r="B12" s="689"/>
+      <x:c r="C12" s="689"/>
+      <x:c r="D12" s="689"/>
+      <x:c r="E12" s="689"/>
+      <x:c r="F12" s="689"/>
+      <x:c r="G12" s="652"/>
+      <x:c r="H12" s="652"/>
+      <x:c r="I12" s="652"/>
+      <x:c r="J12" s="652"/>
+      <x:c r="K12" s="652"/>
+      <x:c r="L12" s="652"/>
+      <x:c r="M12" s="652"/>
+      <x:c r="N12" s="652"/>
+      <x:c r="O12" s="652"/>
+      <x:c r="P12" s="652"/>
+      <x:c r="Q12" s="652"/>
+      <x:c r="R12" s="652"/>
+      <x:c r="S12" s="652"/>
+      <x:c r="T12" s="652"/>
+      <x:c r="U12" s="652"/>
+      <x:c r="V12" s="652"/>
+      <x:c r="W12" s="652"/>
+      <x:c r="X12" s="652"/>
+      <x:c r="Y12" s="652"/>
+      <x:c r="Z12" s="652"/>
+      <x:c r="AA12" s="652"/>
+      <x:c r="AB12" s="652"/>
+      <x:c r="AC12" s="652"/>
+      <x:c r="AD12" s="652"/>
+      <x:c r="AE12" s="652"/>
+      <x:c r="AF12" s="652"/>
+      <x:c r="AG12" s="652"/>
+      <x:c r="AH12" s="652"/>
+      <x:c r="AI12" s="652"/>
+    </x:row>
+    <x:row r="13" ht="18" customHeight="1">
+      <x:c r="A13" s="653" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B13" s="683" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C13" s="683" t="str">
+        <x:v>Midpoint</x:v>
+      </x:c>
+      <x:c r="D13" s="683" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E13" s="690" t="str">
+        <x:v>Role in conclusion</x:v>
+      </x:c>
+      <x:c r="F13" s="690" t="str">
+        <x:v>Source / methodology</x:v>
+      </x:c>
+      <x:c r="G13" s="538"/>
+      <x:c r="H13" s="538"/>
+      <x:c r="I13" s="538"/>
+      <x:c r="J13" s="538"/>
+      <x:c r="K13" s="538"/>
+      <x:c r="L13" s="538"/>
+      <x:c r="M13" s="538"/>
+      <x:c r="N13" s="538"/>
+      <x:c r="O13" s="538"/>
+      <x:c r="P13" s="538"/>
+      <x:c r="Q13" s="538"/>
+      <x:c r="R13" s="538"/>
+      <x:c r="S13" s="538"/>
+      <x:c r="T13" s="538"/>
+      <x:c r="U13" s="538"/>
+      <x:c r="V13" s="538"/>
+      <x:c r="W13" s="538"/>
+      <x:c r="X13" s="538"/>
+      <x:c r="Y13" s="538"/>
+      <x:c r="Z13" s="538"/>
+      <x:c r="AA13" s="538"/>
+      <x:c r="AB13" s="538"/>
+      <x:c r="AC13" s="538"/>
+      <x:c r="AD13" s="538"/>
+      <x:c r="AE13" s="538"/>
+      <x:c r="AF13" s="538"/>
+      <x:c r="AG13" s="538"/>
+      <x:c r="AH13" s="538"/>
+      <x:c r="AI13" s="538"/>
+    </x:row>
+    <x:row r="14" ht="18" customHeight="1">
+      <x:c r="A14" s="436" t="str">
+        <x:v>DCF</x:v>
+      </x:c>
+      <x:c r="B14" s="691" t="n">
+        <x:f>'DCF'!C53</x:f>
+        <x:v>22.952969785087355</x:v>
+      </x:c>
+      <x:c r="C14" s="691" t="n">
+        <x:f>'DCF'!D52</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="D14" s="691" t="n">
+        <x:f>'DCF'!E51</x:f>
+        <x:v>29.773560899538765</x:v>
+      </x:c>
+      <x:c r="E14" s="692" t="str">
+        <x:v>Intrinsic-value anchor</x:v>
+      </x:c>
+      <x:c r="F14" s="692" t="str">
+        <x:v>±1.0% WACC and ±0.5% TGR around base</x:v>
+      </x:c>
+      <x:c r="G14" s="538"/>
+      <x:c r="H14" s="538"/>
+      <x:c r="I14" s="538"/>
+      <x:c r="J14" s="538"/>
+      <x:c r="K14" s="538"/>
+      <x:c r="L14" s="538"/>
+      <x:c r="M14" s="538"/>
+      <x:c r="N14" s="538"/>
+      <x:c r="O14" s="538"/>
+      <x:c r="P14" s="538"/>
+      <x:c r="Q14" s="538"/>
+      <x:c r="R14" s="538"/>
+      <x:c r="S14" s="538"/>
+      <x:c r="T14" s="538"/>
+      <x:c r="U14" s="538"/>
+      <x:c r="V14" s="538"/>
+      <x:c r="W14" s="538"/>
+      <x:c r="X14" s="538"/>
+      <x:c r="Y14" s="538"/>
+      <x:c r="Z14" s="538"/>
+      <x:c r="AA14" s="538"/>
+      <x:c r="AB14" s="538"/>
+      <x:c r="AC14" s="538"/>
+      <x:c r="AD14" s="538"/>
+      <x:c r="AE14" s="538"/>
+      <x:c r="AF14" s="538"/>
+      <x:c r="AG14" s="538"/>
+      <x:c r="AH14" s="538"/>
+      <x:c r="AI14" s="538"/>
+    </x:row>
+    <x:row r="15" ht="18" customHeight="1">
+      <x:c r="A15" s="436" t="str">
+        <x:v>Trading — EV / Revenue</x:v>
+      </x:c>
+      <x:c r="B15" s="691" t="n">
+        <x:f>'Trading Comps'!G35</x:f>
+        <x:v>34.7460112706867</x:v>
+      </x:c>
+      <x:c r="C15" s="691" t="n">
+        <x:f>'Trading Comps'!H35</x:f>
+        <x:v>39.79463691268784</x:v>
+      </x:c>
+      <x:c r="D15" s="691" t="n">
+        <x:f>'Trading Comps'!I35</x:f>
+        <x:v>50.94227339737494</x:v>
+      </x:c>
+      <x:c r="E15" s="692" t="str">
+        <x:v>Core operating benchmark</x:v>
+      </x:c>
+      <x:c r="F15" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G15" s="538"/>
+      <x:c r="H15" s="538"/>
+      <x:c r="I15" s="538"/>
+      <x:c r="J15" s="538"/>
+      <x:c r="K15" s="538"/>
+      <x:c r="L15" s="538"/>
+      <x:c r="M15" s="538"/>
+      <x:c r="N15" s="538"/>
+      <x:c r="O15" s="538"/>
+      <x:c r="P15" s="538"/>
+      <x:c r="Q15" s="538"/>
+      <x:c r="R15" s="538"/>
+      <x:c r="S15" s="538"/>
+      <x:c r="T15" s="538"/>
+      <x:c r="U15" s="538"/>
+      <x:c r="V15" s="538"/>
+      <x:c r="W15" s="538"/>
+      <x:c r="X15" s="538"/>
+      <x:c r="Y15" s="538"/>
+      <x:c r="Z15" s="538"/>
+      <x:c r="AA15" s="538"/>
+      <x:c r="AB15" s="538"/>
+      <x:c r="AC15" s="538"/>
+      <x:c r="AD15" s="538"/>
+      <x:c r="AE15" s="538"/>
+      <x:c r="AF15" s="538"/>
+      <x:c r="AG15" s="538"/>
+      <x:c r="AH15" s="538"/>
+      <x:c r="AI15" s="538"/>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1">
+      <x:c r="A16" s="436" t="str">
+        <x:v>Trading — EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B16" s="691" t="n">
+        <x:f>'Trading Comps'!G36</x:f>
+        <x:v>39.20896245482214</x:v>
+      </x:c>
+      <x:c r="C16" s="691" t="n">
+        <x:f>'Trading Comps'!H36</x:f>
+        <x:v>43.144349201065246</x:v>
+      </x:c>
+      <x:c r="D16" s="691" t="n">
+        <x:f>'Trading Comps'!I36</x:f>
+        <x:v>51.36886532242725</x:v>
+      </x:c>
+      <x:c r="E16" s="692" t="str">
+        <x:v>Core operating benchmark</x:v>
+      </x:c>
+      <x:c r="F16" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G16" s="538"/>
+      <x:c r="H16" s="538"/>
+      <x:c r="I16" s="538"/>
+      <x:c r="J16" s="538"/>
+      <x:c r="K16" s="538"/>
+      <x:c r="L16" s="538"/>
+      <x:c r="M16" s="538"/>
+      <x:c r="N16" s="538"/>
+      <x:c r="O16" s="538"/>
+      <x:c r="P16" s="538"/>
+      <x:c r="Q16" s="538"/>
+      <x:c r="R16" s="538"/>
+      <x:c r="S16" s="538"/>
+      <x:c r="T16" s="538"/>
+      <x:c r="U16" s="538"/>
+      <x:c r="V16" s="538"/>
+      <x:c r="W16" s="538"/>
+      <x:c r="X16" s="538"/>
+      <x:c r="Y16" s="538"/>
+      <x:c r="Z16" s="538"/>
+      <x:c r="AA16" s="538"/>
+      <x:c r="AB16" s="538"/>
+      <x:c r="AC16" s="538"/>
+      <x:c r="AD16" s="538"/>
+      <x:c r="AE16" s="538"/>
+      <x:c r="AF16" s="538"/>
+      <x:c r="AG16" s="538"/>
+      <x:c r="AH16" s="538"/>
+      <x:c r="AI16" s="538"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="436" t="str">
+        <x:v>Trading — EV / EBIT</x:v>
+      </x:c>
+      <x:c r="B17" s="691" t="n">
+        <x:f>'Trading Comps'!G37</x:f>
+        <x:v>46.95080963477268</x:v>
+      </x:c>
+      <x:c r="C17" s="691" t="n">
+        <x:f>'Trading Comps'!H37</x:f>
+        <x:v>52.9061548887198</x:v>
+      </x:c>
+      <x:c r="D17" s="691" t="n">
+        <x:f>'Trading Comps'!I37</x:f>
+        <x:v>55.328817529008944</x:v>
+      </x:c>
+      <x:c r="E17" s="692" t="str">
+        <x:v>Corroborative</x:v>
+      </x:c>
+      <x:c r="F17" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G17" s="538"/>
+      <x:c r="H17" s="538"/>
+      <x:c r="I17" s="538"/>
+      <x:c r="J17" s="538"/>
+      <x:c r="K17" s="538"/>
+      <x:c r="L17" s="538"/>
+      <x:c r="M17" s="538"/>
+      <x:c r="N17" s="538"/>
+      <x:c r="O17" s="538"/>
+      <x:c r="P17" s="538"/>
+      <x:c r="Q17" s="538"/>
+      <x:c r="R17" s="538"/>
+      <x:c r="S17" s="538"/>
+      <x:c r="T17" s="538"/>
+      <x:c r="U17" s="538"/>
+      <x:c r="V17" s="538"/>
+      <x:c r="W17" s="538"/>
+      <x:c r="X17" s="538"/>
+      <x:c r="Y17" s="538"/>
+      <x:c r="Z17" s="538"/>
+      <x:c r="AA17" s="538"/>
+      <x:c r="AB17" s="538"/>
+      <x:c r="AC17" s="538"/>
+      <x:c r="AD17" s="538"/>
+      <x:c r="AE17" s="538"/>
+      <x:c r="AF17" s="538"/>
+      <x:c r="AG17" s="538"/>
+      <x:c r="AH17" s="538"/>
+      <x:c r="AI17" s="538"/>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1">
+      <x:c r="A18" s="436" t="str">
+        <x:v>Trading — P / E</x:v>
+      </x:c>
+      <x:c r="B18" s="691" t="n">
+        <x:f>'Trading Comps'!G38</x:f>
+        <x:v>49.89126177669402</x:v>
+      </x:c>
+      <x:c r="C18" s="691" t="n">
+        <x:f>'Trading Comps'!H38</x:f>
+        <x:v>54.28133382929772</x:v>
+      </x:c>
+      <x:c r="D18" s="691" t="n">
+        <x:f>'Trading Comps'!I38</x:f>
+        <x:v>58.73871533415601</x:v>
+      </x:c>
+      <x:c r="E18" s="692" t="str">
+        <x:v>Equity-value corroboration</x:v>
+      </x:c>
+      <x:c r="F18" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G18" s="538"/>
+      <x:c r="H18" s="538"/>
+      <x:c r="I18" s="538"/>
+      <x:c r="J18" s="538"/>
+      <x:c r="K18" s="538"/>
+      <x:c r="L18" s="538"/>
+      <x:c r="M18" s="538"/>
+      <x:c r="N18" s="538"/>
+      <x:c r="O18" s="538"/>
+      <x:c r="P18" s="538"/>
+      <x:c r="Q18" s="538"/>
+      <x:c r="R18" s="538"/>
+      <x:c r="S18" s="538"/>
+      <x:c r="T18" s="538"/>
+      <x:c r="U18" s="538"/>
+      <x:c r="V18" s="538"/>
+      <x:c r="W18" s="538"/>
+      <x:c r="X18" s="538"/>
+      <x:c r="Y18" s="538"/>
+      <x:c r="Z18" s="538"/>
+      <x:c r="AA18" s="538"/>
+      <x:c r="AB18" s="538"/>
+      <x:c r="AC18" s="538"/>
+      <x:c r="AD18" s="538"/>
+      <x:c r="AE18" s="538"/>
+      <x:c r="AF18" s="538"/>
+      <x:c r="AG18" s="538"/>
+      <x:c r="AH18" s="538"/>
+      <x:c r="AI18" s="538"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="436" t="str">
+        <x:v>Precedent — EV / Revenue</x:v>
+      </x:c>
+      <x:c r="B19" s="691" t="n">
+        <x:f>'Precedent Transactions'!G35</x:f>
+        <x:v>34.0626126411909</x:v>
+      </x:c>
+      <x:c r="C19" s="691" t="n">
+        <x:f>'Precedent Transactions'!H35</x:f>
+        <x:v>45.32446369026972</x:v>
+      </x:c>
+      <x:c r="D19" s="691" t="n">
+        <x:f>'Precedent Transactions'!I35</x:f>
+        <x:v>52.57395681762598</x:v>
+      </x:c>
+      <x:c r="E19" s="692" t="str">
+        <x:v>Strategic transaction benchmark</x:v>
+      </x:c>
+      <x:c r="F19" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G19" s="538"/>
+      <x:c r="H19" s="538"/>
+      <x:c r="I19" s="538"/>
+      <x:c r="J19" s="538"/>
+      <x:c r="K19" s="538"/>
+      <x:c r="L19" s="538"/>
+      <x:c r="M19" s="538"/>
+      <x:c r="N19" s="538"/>
+      <x:c r="O19" s="538"/>
+      <x:c r="P19" s="538"/>
+      <x:c r="Q19" s="538"/>
+      <x:c r="R19" s="538"/>
+      <x:c r="S19" s="538"/>
+      <x:c r="T19" s="538"/>
+      <x:c r="U19" s="538"/>
+      <x:c r="V19" s="538"/>
+      <x:c r="W19" s="538"/>
+      <x:c r="X19" s="538"/>
+      <x:c r="Y19" s="538"/>
+      <x:c r="Z19" s="538"/>
+      <x:c r="AA19" s="538"/>
+      <x:c r="AB19" s="538"/>
+      <x:c r="AC19" s="538"/>
+      <x:c r="AD19" s="538"/>
+      <x:c r="AE19" s="538"/>
+      <x:c r="AF19" s="538"/>
+      <x:c r="AG19" s="538"/>
+      <x:c r="AH19" s="538"/>
+      <x:c r="AI19" s="538"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="436" t="str">
+        <x:v>Precedent — EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B20" s="691" t="n">
+        <x:f>'Precedent Transactions'!G36</x:f>
+        <x:v>39.08531176777297</x:v>
+      </x:c>
+      <x:c r="C20" s="691" t="n">
+        <x:f>'Precedent Transactions'!H36</x:f>
+        <x:v>40.27345666415471</x:v>
+      </x:c>
+      <x:c r="D20" s="691" t="n">
+        <x:f>'Precedent Transactions'!I36</x:f>
+        <x:v>41.46160156053644</x:v>
+      </x:c>
+      <x:c r="E20" s="692" t="str">
+        <x:v>Strategic transaction benchmark</x:v>
+      </x:c>
+      <x:c r="F20" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G20" s="538"/>
+      <x:c r="H20" s="538"/>
+      <x:c r="I20" s="538"/>
+      <x:c r="J20" s="538"/>
+      <x:c r="K20" s="538"/>
+      <x:c r="L20" s="538"/>
+      <x:c r="M20" s="538"/>
+      <x:c r="N20" s="538"/>
+      <x:c r="O20" s="538"/>
+      <x:c r="P20" s="538"/>
+      <x:c r="Q20" s="538"/>
+      <x:c r="R20" s="538"/>
+      <x:c r="S20" s="538"/>
+      <x:c r="T20" s="538"/>
+      <x:c r="U20" s="538"/>
+      <x:c r="V20" s="538"/>
+      <x:c r="W20" s="538"/>
+      <x:c r="X20" s="538"/>
+      <x:c r="Y20" s="538"/>
+      <x:c r="Z20" s="538"/>
+      <x:c r="AA20" s="538"/>
+      <x:c r="AB20" s="538"/>
+      <x:c r="AC20" s="538"/>
+      <x:c r="AD20" s="538"/>
+      <x:c r="AE20" s="538"/>
+      <x:c r="AF20" s="538"/>
+      <x:c r="AG20" s="538"/>
+      <x:c r="AH20" s="538"/>
+      <x:c r="AI20" s="538"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="436" t="str">
+        <x:v>Precedent — EV / EBIT</x:v>
+      </x:c>
+      <x:c r="B21" s="691" t="n">
+        <x:f>'Precedent Transactions'!G37</x:f>
+        <x:v>51.98488081157034</x:v>
+      </x:c>
+      <x:c r="C21" s="691" t="n">
+        <x:f>'Precedent Transactions'!H37</x:f>
+        <x:v>55.05026643373155</x:v>
+      </x:c>
+      <x:c r="D21" s="691" t="n">
+        <x:f>'Precedent Transactions'!I37</x:f>
+        <x:v>58.11565205589273</x:v>
+      </x:c>
+      <x:c r="E21" s="692" t="str">
+        <x:v>Corroborative; limited observations</x:v>
+      </x:c>
+      <x:c r="F21" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G21" s="538"/>
+      <x:c r="H21" s="538"/>
+      <x:c r="I21" s="538"/>
+      <x:c r="J21" s="538"/>
+      <x:c r="K21" s="538"/>
+      <x:c r="L21" s="538"/>
+      <x:c r="M21" s="538"/>
+      <x:c r="N21" s="538"/>
+      <x:c r="O21" s="538"/>
+      <x:c r="P21" s="538"/>
+      <x:c r="Q21" s="538"/>
+      <x:c r="R21" s="538"/>
+      <x:c r="S21" s="538"/>
+      <x:c r="T21" s="538"/>
+      <x:c r="U21" s="538"/>
+      <x:c r="V21" s="538"/>
+      <x:c r="W21" s="538"/>
+      <x:c r="X21" s="538"/>
+      <x:c r="Y21" s="538"/>
+      <x:c r="Z21" s="538"/>
+      <x:c r="AA21" s="538"/>
+      <x:c r="AB21" s="538"/>
+      <x:c r="AC21" s="538"/>
+      <x:c r="AD21" s="538"/>
+      <x:c r="AE21" s="538"/>
+      <x:c r="AF21" s="538"/>
+      <x:c r="AG21" s="538"/>
+      <x:c r="AH21" s="538"/>
+      <x:c r="AI21" s="538"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="436" t="str">
+        <x:v>Precedent — Premium Paid</x:v>
+      </x:c>
+      <x:c r="B22" s="691" t="n">
+        <x:f>'Precedent Transactions'!G38</x:f>
+        <x:v>80.48617499999999</x:v>
+      </x:c>
+      <x:c r="C22" s="691" t="n">
+        <x:f>'Precedent Transactions'!H38</x:f>
+        <x:v>84.51795</x:v>
+      </x:c>
+      <x:c r="D22" s="691" t="n">
+        <x:f>'Precedent Transactions'!I38</x:f>
+        <x:v>86.30985</x:v>
+      </x:c>
+      <x:c r="E22" s="692" t="str">
+        <x:v>Control-price benchmark</x:v>
+      </x:c>
+      <x:c r="F22" s="692" t="str">
+        <x:v>25th–75th percentile</x:v>
+      </x:c>
+      <x:c r="G22" s="538"/>
+      <x:c r="H22" s="538"/>
+      <x:c r="I22" s="538"/>
+      <x:c r="J22" s="538"/>
+      <x:c r="K22" s="538"/>
+      <x:c r="L22" s="538"/>
+      <x:c r="M22" s="538"/>
+      <x:c r="N22" s="538"/>
+      <x:c r="O22" s="538"/>
+      <x:c r="P22" s="538"/>
+      <x:c r="Q22" s="538"/>
+      <x:c r="R22" s="538"/>
+      <x:c r="S22" s="538"/>
+      <x:c r="T22" s="538"/>
+      <x:c r="U22" s="538"/>
+      <x:c r="V22" s="538"/>
+      <x:c r="W22" s="538"/>
+      <x:c r="X22" s="538"/>
+      <x:c r="Y22" s="538"/>
+      <x:c r="Z22" s="538"/>
+      <x:c r="AA22" s="538"/>
+      <x:c r="AB22" s="538"/>
+      <x:c r="AC22" s="538"/>
+      <x:c r="AD22" s="538"/>
+      <x:c r="AE22" s="538"/>
+      <x:c r="AF22" s="538"/>
+      <x:c r="AG22" s="538"/>
+      <x:c r="AH22" s="538"/>
+      <x:c r="AI22" s="538"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="436" t="str">
+        <x:v>Unaffected Share Price</x:v>
+      </x:c>
+      <x:c r="B23" s="691" t="n">
+        <x:f>'Precedent Transactions'!B30</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="C23" s="691" t="n">
+        <x:f>'Precedent Transactions'!B30</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="D23" s="691" t="n">
+        <x:f>'Precedent Transactions'!B30</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="E23" s="692" t="str">
+        <x:v>Market reference / practical floor</x:v>
+      </x:c>
+      <x:c r="F23" s="692" t="str">
+        <x:v>Aug. 20, 2026 closing price</x:v>
+      </x:c>
+      <x:c r="G23" s="538"/>
+      <x:c r="H23" s="538"/>
+      <x:c r="I23" s="538"/>
+      <x:c r="J23" s="538"/>
+      <x:c r="K23" s="538"/>
+      <x:c r="L23" s="538"/>
+      <x:c r="M23" s="538"/>
+      <x:c r="N23" s="538"/>
+      <x:c r="O23" s="538"/>
+      <x:c r="P23" s="538"/>
+      <x:c r="Q23" s="538"/>
+      <x:c r="R23" s="538"/>
+      <x:c r="S23" s="538"/>
+      <x:c r="T23" s="538"/>
+      <x:c r="U23" s="538"/>
+      <x:c r="V23" s="538"/>
+      <x:c r="W23" s="538"/>
+      <x:c r="X23" s="538"/>
+      <x:c r="Y23" s="538"/>
+      <x:c r="Z23" s="538"/>
+      <x:c r="AA23" s="538"/>
+      <x:c r="AB23" s="538"/>
+      <x:c r="AC23" s="538"/>
+      <x:c r="AD23" s="538"/>
+      <x:c r="AE23" s="538"/>
+      <x:c r="AF23" s="538"/>
+      <x:c r="AG23" s="538"/>
+      <x:c r="AH23" s="538"/>
+      <x:c r="AI23" s="538"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="665" t="str">
+        <x:v>Acquisition Range</x:v>
+      </x:c>
+      <x:c r="B24" s="693" t="n">
+        <x:f>B8</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C24" s="693" t="n">
+        <x:f>B9</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D24" s="693" t="n">
+        <x:f>C8</x:f>
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="E24" s="694" t="str">
+        <x:v>Illustrative transaction framework</x:v>
+      </x:c>
+      <x:c r="F24" s="694" t="str">
+        <x:v>Analyst judgment; subject to transaction testing</x:v>
+      </x:c>
+      <x:c r="G24" s="538"/>
+      <x:c r="H24" s="538"/>
+      <x:c r="I24" s="538"/>
+      <x:c r="J24" s="538"/>
+      <x:c r="K24" s="538"/>
+      <x:c r="L24" s="538"/>
+      <x:c r="M24" s="538"/>
+      <x:c r="N24" s="538"/>
+      <x:c r="O24" s="538"/>
+      <x:c r="P24" s="538"/>
+      <x:c r="Q24" s="538"/>
+      <x:c r="R24" s="538"/>
+      <x:c r="S24" s="538"/>
+      <x:c r="T24" s="538"/>
+      <x:c r="U24" s="538"/>
+      <x:c r="V24" s="538"/>
+      <x:c r="W24" s="538"/>
+      <x:c r="X24" s="538"/>
+      <x:c r="Y24" s="538"/>
+      <x:c r="Z24" s="538"/>
+      <x:c r="AA24" s="538"/>
+      <x:c r="AB24" s="538"/>
+      <x:c r="AC24" s="538"/>
+      <x:c r="AD24" s="538"/>
+      <x:c r="AE24" s="538"/>
+      <x:c r="AF24" s="538"/>
+      <x:c r="AG24" s="538"/>
+      <x:c r="AH24" s="538"/>
+      <x:c r="AI24" s="538"/>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1">
+      <x:c r="A25" s="538"/>
+      <x:c r="B25" s="579"/>
+      <x:c r="C25" s="579"/>
+      <x:c r="D25" s="579"/>
+      <x:c r="E25" s="579"/>
+      <x:c r="F25" s="579"/>
+      <x:c r="G25" s="538"/>
+      <x:c r="H25" s="538"/>
+      <x:c r="I25" s="538"/>
+      <x:c r="J25" s="538"/>
+      <x:c r="K25" s="538"/>
+      <x:c r="L25" s="538"/>
+      <x:c r="M25" s="538"/>
+      <x:c r="N25" s="538"/>
+      <x:c r="O25" s="538"/>
+      <x:c r="P25" s="538"/>
+      <x:c r="Q25" s="538"/>
+      <x:c r="R25" s="538"/>
+      <x:c r="S25" s="538"/>
+      <x:c r="T25" s="538"/>
+      <x:c r="U25" s="538"/>
+      <x:c r="V25" s="538"/>
+      <x:c r="W25" s="538"/>
+      <x:c r="X25" s="538"/>
+      <x:c r="Y25" s="538"/>
+      <x:c r="Z25" s="538"/>
+      <x:c r="AA25" s="538"/>
+      <x:c r="AB25" s="538"/>
+      <x:c r="AC25" s="538"/>
+      <x:c r="AD25" s="538"/>
+      <x:c r="AE25" s="538"/>
+      <x:c r="AF25" s="538"/>
+      <x:c r="AG25" s="538"/>
+      <x:c r="AH25" s="538"/>
+      <x:c r="AI25" s="538"/>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="652" t="str">
+        <x:v>FOOTBALL FIELD — IMPLIED COGNEX EQUITY VALUE PER SHARE</x:v>
+      </x:c>
+      <x:c r="B26" s="689"/>
+      <x:c r="C26" s="689"/>
+      <x:c r="D26" s="689"/>
+      <x:c r="E26" s="689"/>
+      <x:c r="F26" s="689"/>
+      <x:c r="G26" s="652"/>
+      <x:c r="H26" s="652"/>
+      <x:c r="I26" s="652"/>
+      <x:c r="J26" s="652"/>
+      <x:c r="K26" s="652"/>
+      <x:c r="L26" s="652"/>
+      <x:c r="M26" s="652"/>
+      <x:c r="N26" s="652"/>
+      <x:c r="O26" s="652"/>
+      <x:c r="P26" s="652"/>
+      <x:c r="Q26" s="652"/>
+      <x:c r="R26" s="652"/>
+      <x:c r="S26" s="652"/>
+      <x:c r="T26" s="652"/>
+      <x:c r="U26" s="652"/>
+      <x:c r="V26" s="652"/>
+      <x:c r="W26" s="652"/>
+      <x:c r="X26" s="652"/>
+      <x:c r="Y26" s="652"/>
+      <x:c r="Z26" s="652"/>
+      <x:c r="AA26" s="652"/>
+      <x:c r="AB26" s="652"/>
+      <x:c r="AC26" s="652"/>
+      <x:c r="AD26" s="652"/>
+      <x:c r="AE26" s="652"/>
+      <x:c r="AF26" s="652"/>
+      <x:c r="AG26" s="652"/>
+      <x:c r="AH26" s="652"/>
+      <x:c r="AI26" s="652"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="668" t="str">
+        <x:v>Scale minimum</x:v>
+      </x:c>
+      <x:c r="B27" s="695" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C27" s="695" t="str">
+        <x:v>Scale increment</x:v>
+      </x:c>
+      <x:c r="D27" s="695" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="E27" s="696" t="str">
+        <x:v>Scale maximum</x:v>
+      </x:c>
+      <x:c r="F27" s="696" t="n">
+        <x:f>B27+D27*28</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G27" s="538"/>
+      <x:c r="H27" s="538"/>
+      <x:c r="I27" s="538"/>
+      <x:c r="J27" s="538"/>
+      <x:c r="K27" s="538"/>
+      <x:c r="L27" s="538"/>
+      <x:c r="M27" s="538"/>
+      <x:c r="N27" s="538"/>
+      <x:c r="O27" s="538"/>
+      <x:c r="P27" s="538"/>
+      <x:c r="Q27" s="538"/>
+      <x:c r="R27" s="538"/>
+      <x:c r="S27" s="538"/>
+      <x:c r="T27" s="538"/>
+      <x:c r="U27" s="538"/>
+      <x:c r="V27" s="538"/>
+      <x:c r="W27" s="538"/>
+      <x:c r="X27" s="538"/>
+      <x:c r="Y27" s="538"/>
+      <x:c r="Z27" s="538"/>
+      <x:c r="AA27" s="538"/>
+      <x:c r="AB27" s="538"/>
+      <x:c r="AC27" s="538"/>
+      <x:c r="AD27" s="538"/>
+      <x:c r="AE27" s="538"/>
+      <x:c r="AF27" s="538"/>
+      <x:c r="AG27" s="538"/>
+      <x:c r="AH27" s="538"/>
+      <x:c r="AI27" s="538"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="671" t="str">
+        <x:v>Method / exact range</x:v>
+      </x:c>
+      <x:c r="B28" s="697"/>
+      <x:c r="C28" s="697"/>
+      <x:c r="D28" s="697"/>
+      <x:c r="E28" s="697"/>
+      <x:c r="F28" s="697"/>
+      <x:c r="G28" s="672" t="n">
+        <x:f>$B$27</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H28" s="672" t="n">
+        <x:f>G28+$D$27</x:f>
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="I28" s="672" t="n">
+        <x:f>H28+$D$27</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="J28" s="672" t="n">
+        <x:f>I28+$D$27</x:f>
+        <x:v>27.5</x:v>
+      </x:c>
+      <x:c r="K28" s="672" t="n">
+        <x:f>J28+$D$27</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L28" s="672" t="n">
+        <x:f>K28+$D$27</x:f>
+        <x:v>32.5</x:v>
+      </x:c>
+      <x:c r="M28" s="672" t="n">
+        <x:f>L28+$D$27</x:f>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="N28" s="672" t="n">
+        <x:f>M28+$D$27</x:f>
+        <x:v>37.5</x:v>
+      </x:c>
+      <x:c r="O28" s="672" t="n">
+        <x:f>N28+$D$27</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="P28" s="672" t="n">
+        <x:f>O28+$D$27</x:f>
+        <x:v>42.5</x:v>
+      </x:c>
+      <x:c r="Q28" s="672" t="n">
+        <x:f>P28+$D$27</x:f>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="R28" s="672" t="n">
+        <x:f>Q28+$D$27</x:f>
+        <x:v>47.5</x:v>
+      </x:c>
+      <x:c r="S28" s="672" t="n">
+        <x:f>R28+$D$27</x:f>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="T28" s="672" t="n">
+        <x:f>S28+$D$27</x:f>
+        <x:v>52.5</x:v>
+      </x:c>
+      <x:c r="U28" s="672" t="n">
+        <x:f>T28+$D$27</x:f>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="V28" s="672" t="n">
+        <x:f>U28+$D$27</x:f>
+        <x:v>57.5</x:v>
+      </x:c>
+      <x:c r="W28" s="672" t="n">
+        <x:f>V28+$D$27</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="X28" s="672" t="n">
+        <x:f>W28+$D$27</x:f>
+        <x:v>62.5</x:v>
+      </x:c>
+      <x:c r="Y28" s="672" t="n">
+        <x:f>X28+$D$27</x:f>
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="Z28" s="672" t="n">
+        <x:f>Y28+$D$27</x:f>
+        <x:v>67.5</x:v>
+      </x:c>
+      <x:c r="AA28" s="672" t="n">
+        <x:f>Z28+$D$27</x:f>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="AB28" s="672" t="n">
+        <x:f>AA28+$D$27</x:f>
+        <x:v>72.5</x:v>
+      </x:c>
+      <x:c r="AC28" s="672" t="n">
+        <x:f>AB28+$D$27</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="AD28" s="672" t="n">
+        <x:f>AC28+$D$27</x:f>
+        <x:v>77.5</x:v>
+      </x:c>
+      <x:c r="AE28" s="672" t="n">
+        <x:f>AD28+$D$27</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="AF28" s="672" t="n">
+        <x:f>AE28+$D$27</x:f>
+        <x:v>82.5</x:v>
+      </x:c>
+      <x:c r="AG28" s="672" t="n">
+        <x:f>AF28+$D$27</x:f>
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="AH28" s="672" t="n">
+        <x:f>AG28+$D$27</x:f>
+        <x:v>87.5</x:v>
+      </x:c>
+      <x:c r="AI28" s="672" t="n">
+        <x:f>AH28+$D$27</x:f>
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="673" t="str">
+        <x:f>A14</x:f>
+        <x:v>DCF</x:v>
+      </x:c>
+      <x:c r="B29" s="698"/>
+      <x:c r="C29" s="698"/>
+      <x:c r="D29" s="699" t="n">
+        <x:f>B14</x:f>
+        <x:v>22.952969785087355</x:v>
+      </x:c>
+      <x:c r="E29" s="699" t="n">
+        <x:f>C14</x:f>
+        <x:v>25.791148957127746</x:v>
+      </x:c>
+      <x:c r="F29" s="699" t="n">
+        <x:f>D14</x:f>
+        <x:v>29.773560899538765</x:v>
+      </x:c>
+      <x:c r="G29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(G$28-$E29)&lt;=$D$27/2,AND(G$28&gt;=$D29,G$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="H29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(H$28-$E29)&lt;=$D$27/2,AND(H$28&gt;=$D29,H$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="I29" s="675" t="n">
+        <x:f>IF(IF($D29=$F29,ABS(I$28-$E29)&lt;=$D$27/2,AND(I$28&gt;=$D29,I$28&lt;=$F29)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J29" s="675" t="n">
+        <x:f>IF(IF($D29=$F29,ABS(J$28-$E29)&lt;=$D$27/2,AND(J$28&gt;=$D29,J$28&lt;=$F29)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(K$28-$E29)&lt;=$D$27/2,AND(K$28&gt;=$D29,K$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="L29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(L$28-$E29)&lt;=$D$27/2,AND(L$28&gt;=$D29,L$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="M29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(M$28-$E29)&lt;=$D$27/2,AND(M$28&gt;=$D29,M$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="N29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(N$28-$E29)&lt;=$D$27/2,AND(N$28&gt;=$D29,N$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="O29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(O$28-$E29)&lt;=$D$27/2,AND(O$28&gt;=$D29,O$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="P29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(P$28-$E29)&lt;=$D$27/2,AND(P$28&gt;=$D29,P$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(Q$28-$E29)&lt;=$D$27/2,AND(Q$28&gt;=$D29,Q$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="R29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(R$28-$E29)&lt;=$D$27/2,AND(R$28&gt;=$D29,R$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="S29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(S$28-$E29)&lt;=$D$27/2,AND(S$28&gt;=$D29,S$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="T29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(T$28-$E29)&lt;=$D$27/2,AND(T$28&gt;=$D29,T$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="U29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(U$28-$E29)&lt;=$D$27/2,AND(U$28&gt;=$D29,U$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="V29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(V$28-$E29)&lt;=$D$27/2,AND(V$28&gt;=$D29,V$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="W29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(W$28-$E29)&lt;=$D$27/2,AND(W$28&gt;=$D29,W$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="X29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(X$28-$E29)&lt;=$D$27/2,AND(X$28&gt;=$D29,X$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(Y$28-$E29)&lt;=$D$27/2,AND(Y$28&gt;=$D29,Y$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(Z$28-$E29)&lt;=$D$27/2,AND(Z$28&gt;=$D29,Z$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AA$28-$E29)&lt;=$D$27/2,AND(AA$28&gt;=$D29,AA$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AB$28-$E29)&lt;=$D$27/2,AND(AB$28&gt;=$D29,AB$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AC$28-$E29)&lt;=$D$27/2,AND(AC$28&gt;=$D29,AC$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AD$28-$E29)&lt;=$D$27/2,AND(AD$28&gt;=$D29,AD$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AE$28-$E29)&lt;=$D$27/2,AND(AE$28&gt;=$D29,AE$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AF$28-$E29)&lt;=$D$27/2,AND(AF$28&gt;=$D29,AF$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AG$28-$E29)&lt;=$D$27/2,AND(AG$28&gt;=$D29,AG$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AH$28-$E29)&lt;=$D$27/2,AND(AH$28&gt;=$D29,AH$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI29" s="675" t="str">
+        <x:f>IF(IF($D29=$F29,ABS(AI$28-$E29)&lt;=$D$27/2,AND(AI$28&gt;=$D29,AI$28&lt;=$F29)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="673" t="str">
+        <x:f>A15</x:f>
+        <x:v>Trading — EV / Revenue</x:v>
+      </x:c>
+      <x:c r="B30" s="698"/>
+      <x:c r="C30" s="698"/>
+      <x:c r="D30" s="699" t="n">
+        <x:f>B15</x:f>
+        <x:v>34.7460112706867</x:v>
+      </x:c>
+      <x:c r="E30" s="699" t="n">
+        <x:f>C15</x:f>
+        <x:v>39.79463691268784</x:v>
+      </x:c>
+      <x:c r="F30" s="699" t="n">
+        <x:f>D15</x:f>
+        <x:v>50.94227339737494</x:v>
+      </x:c>
+      <x:c r="G30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(G$28-$E30)&lt;=$D$27/2,AND(G$28&gt;=$D30,G$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="H30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(H$28-$E30)&lt;=$D$27/2,AND(H$28&gt;=$D30,H$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="I30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(I$28-$E30)&lt;=$D$27/2,AND(I$28&gt;=$D30,I$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="J30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(J$28-$E30)&lt;=$D$27/2,AND(J$28&gt;=$D30,J$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="K30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(K$28-$E30)&lt;=$D$27/2,AND(K$28&gt;=$D30,K$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="L30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(L$28-$E30)&lt;=$D$27/2,AND(L$28&gt;=$D30,L$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="M30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(M$28-$E30)&lt;=$D$27/2,AND(M$28&gt;=$D30,M$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(N$28-$E30)&lt;=$D$27/2,AND(N$28&gt;=$D30,N$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(O$28-$E30)&lt;=$D$27/2,AND(O$28&gt;=$D30,O$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(P$28-$E30)&lt;=$D$27/2,AND(P$28&gt;=$D30,P$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(Q$28-$E30)&lt;=$D$27/2,AND(Q$28&gt;=$D30,Q$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(R$28-$E30)&lt;=$D$27/2,AND(R$28&gt;=$D30,R$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S30" s="675" t="n">
+        <x:f>IF(IF($D30=$F30,ABS(S$28-$E30)&lt;=$D$27/2,AND(S$28&gt;=$D30,S$28&lt;=$F30)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(T$28-$E30)&lt;=$D$27/2,AND(T$28&gt;=$D30,T$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="U30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(U$28-$E30)&lt;=$D$27/2,AND(U$28&gt;=$D30,U$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="V30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(V$28-$E30)&lt;=$D$27/2,AND(V$28&gt;=$D30,V$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="W30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(W$28-$E30)&lt;=$D$27/2,AND(W$28&gt;=$D30,W$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="X30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(X$28-$E30)&lt;=$D$27/2,AND(X$28&gt;=$D30,X$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(Y$28-$E30)&lt;=$D$27/2,AND(Y$28&gt;=$D30,Y$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(Z$28-$E30)&lt;=$D$27/2,AND(Z$28&gt;=$D30,Z$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AA$28-$E30)&lt;=$D$27/2,AND(AA$28&gt;=$D30,AA$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AB$28-$E30)&lt;=$D$27/2,AND(AB$28&gt;=$D30,AB$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AC$28-$E30)&lt;=$D$27/2,AND(AC$28&gt;=$D30,AC$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AD$28-$E30)&lt;=$D$27/2,AND(AD$28&gt;=$D30,AD$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AE$28-$E30)&lt;=$D$27/2,AND(AE$28&gt;=$D30,AE$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AF$28-$E30)&lt;=$D$27/2,AND(AF$28&gt;=$D30,AF$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AG$28-$E30)&lt;=$D$27/2,AND(AG$28&gt;=$D30,AG$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AH$28-$E30)&lt;=$D$27/2,AND(AH$28&gt;=$D30,AH$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI30" s="675" t="str">
+        <x:f>IF(IF($D30=$F30,ABS(AI$28-$E30)&lt;=$D$27/2,AND(AI$28&gt;=$D30,AI$28&lt;=$F30)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="A31" s="673" t="str">
+        <x:f>A16</x:f>
+        <x:v>Trading — EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B31" s="698"/>
+      <x:c r="C31" s="698"/>
+      <x:c r="D31" s="699" t="n">
+        <x:f>B16</x:f>
+        <x:v>39.20896245482214</x:v>
+      </x:c>
+      <x:c r="E31" s="699" t="n">
+        <x:f>C16</x:f>
+        <x:v>43.144349201065246</x:v>
+      </x:c>
+      <x:c r="F31" s="699" t="n">
+        <x:f>D16</x:f>
+        <x:v>51.36886532242725</x:v>
+      </x:c>
+      <x:c r="G31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(G$28-$E31)&lt;=$D$27/2,AND(G$28&gt;=$D31,G$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="H31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(H$28-$E31)&lt;=$D$27/2,AND(H$28&gt;=$D31,H$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="I31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(I$28-$E31)&lt;=$D$27/2,AND(I$28&gt;=$D31,I$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="J31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(J$28-$E31)&lt;=$D$27/2,AND(J$28&gt;=$D31,J$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="K31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(K$28-$E31)&lt;=$D$27/2,AND(K$28&gt;=$D31,K$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="L31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(L$28-$E31)&lt;=$D$27/2,AND(L$28&gt;=$D31,L$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="M31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(M$28-$E31)&lt;=$D$27/2,AND(M$28&gt;=$D31,M$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="N31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(N$28-$E31)&lt;=$D$27/2,AND(N$28&gt;=$D31,N$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="O31" s="675" t="n">
+        <x:f>IF(IF($D31=$F31,ABS(O$28-$E31)&lt;=$D$27/2,AND(O$28&gt;=$D31,O$28&lt;=$F31)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P31" s="675" t="n">
+        <x:f>IF(IF($D31=$F31,ABS(P$28-$E31)&lt;=$D$27/2,AND(P$28&gt;=$D31,P$28&lt;=$F31)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q31" s="675" t="n">
+        <x:f>IF(IF($D31=$F31,ABS(Q$28-$E31)&lt;=$D$27/2,AND(Q$28&gt;=$D31,Q$28&lt;=$F31)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R31" s="675" t="n">
+        <x:f>IF(IF($D31=$F31,ABS(R$28-$E31)&lt;=$D$27/2,AND(R$28&gt;=$D31,R$28&lt;=$F31)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S31" s="675" t="n">
+        <x:f>IF(IF($D31=$F31,ABS(S$28-$E31)&lt;=$D$27/2,AND(S$28&gt;=$D31,S$28&lt;=$F31)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(T$28-$E31)&lt;=$D$27/2,AND(T$28&gt;=$D31,T$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="U31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(U$28-$E31)&lt;=$D$27/2,AND(U$28&gt;=$D31,U$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="V31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(V$28-$E31)&lt;=$D$27/2,AND(V$28&gt;=$D31,V$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="W31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(W$28-$E31)&lt;=$D$27/2,AND(W$28&gt;=$D31,W$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="X31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(X$28-$E31)&lt;=$D$27/2,AND(X$28&gt;=$D31,X$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(Y$28-$E31)&lt;=$D$27/2,AND(Y$28&gt;=$D31,Y$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(Z$28-$E31)&lt;=$D$27/2,AND(Z$28&gt;=$D31,Z$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AA$28-$E31)&lt;=$D$27/2,AND(AA$28&gt;=$D31,AA$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AB$28-$E31)&lt;=$D$27/2,AND(AB$28&gt;=$D31,AB$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AC$28-$E31)&lt;=$D$27/2,AND(AC$28&gt;=$D31,AC$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AD$28-$E31)&lt;=$D$27/2,AND(AD$28&gt;=$D31,AD$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AE$28-$E31)&lt;=$D$27/2,AND(AE$28&gt;=$D31,AE$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AF$28-$E31)&lt;=$D$27/2,AND(AF$28&gt;=$D31,AF$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AG$28-$E31)&lt;=$D$27/2,AND(AG$28&gt;=$D31,AG$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AH$28-$E31)&lt;=$D$27/2,AND(AH$28&gt;=$D31,AH$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI31" s="675" t="str">
+        <x:f>IF(IF($D31=$F31,ABS(AI$28-$E31)&lt;=$D$27/2,AND(AI$28&gt;=$D31,AI$28&lt;=$F31)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="18" customHeight="1">
+      <x:c r="A32" s="673" t="str">
+        <x:f>A17</x:f>
+        <x:v>Trading — EV / EBIT</x:v>
+      </x:c>
+      <x:c r="B32" s="698"/>
+      <x:c r="C32" s="698"/>
+      <x:c r="D32" s="699" t="n">
+        <x:f>B17</x:f>
+        <x:v>46.95080963477268</x:v>
+      </x:c>
+      <x:c r="E32" s="699" t="n">
+        <x:f>C17</x:f>
+        <x:v>52.9061548887198</x:v>
+      </x:c>
+      <x:c r="F32" s="699" t="n">
+        <x:f>D17</x:f>
+        <x:v>55.328817529008944</x:v>
+      </x:c>
+      <x:c r="G32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(G$28-$E32)&lt;=$D$27/2,AND(G$28&gt;=$D32,G$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="H32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(H$28-$E32)&lt;=$D$27/2,AND(H$28&gt;=$D32,H$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="I32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(I$28-$E32)&lt;=$D$27/2,AND(I$28&gt;=$D32,I$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="J32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(J$28-$E32)&lt;=$D$27/2,AND(J$28&gt;=$D32,J$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="K32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(K$28-$E32)&lt;=$D$27/2,AND(K$28&gt;=$D32,K$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="L32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(L$28-$E32)&lt;=$D$27/2,AND(L$28&gt;=$D32,L$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="M32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(M$28-$E32)&lt;=$D$27/2,AND(M$28&gt;=$D32,M$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="N32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(N$28-$E32)&lt;=$D$27/2,AND(N$28&gt;=$D32,N$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="O32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(O$28-$E32)&lt;=$D$27/2,AND(O$28&gt;=$D32,O$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="P32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(P$28-$E32)&lt;=$D$27/2,AND(P$28&gt;=$D32,P$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(Q$28-$E32)&lt;=$D$27/2,AND(Q$28&gt;=$D32,Q$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="R32" s="675" t="n">
+        <x:f>IF(IF($D32=$F32,ABS(R$28-$E32)&lt;=$D$27/2,AND(R$28&gt;=$D32,R$28&lt;=$F32)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S32" s="675" t="n">
+        <x:f>IF(IF($D32=$F32,ABS(S$28-$E32)&lt;=$D$27/2,AND(S$28&gt;=$D32,S$28&lt;=$F32)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T32" s="675" t="n">
+        <x:f>IF(IF($D32=$F32,ABS(T$28-$E32)&lt;=$D$27/2,AND(T$28&gt;=$D32,T$28&lt;=$F32)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U32" s="675" t="n">
+        <x:f>IF(IF($D32=$F32,ABS(U$28-$E32)&lt;=$D$27/2,AND(U$28&gt;=$D32,U$28&lt;=$F32)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(V$28-$E32)&lt;=$D$27/2,AND(V$28&gt;=$D32,V$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="W32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(W$28-$E32)&lt;=$D$27/2,AND(W$28&gt;=$D32,W$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="X32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(X$28-$E32)&lt;=$D$27/2,AND(X$28&gt;=$D32,X$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(Y$28-$E32)&lt;=$D$27/2,AND(Y$28&gt;=$D32,Y$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(Z$28-$E32)&lt;=$D$27/2,AND(Z$28&gt;=$D32,Z$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AA$28-$E32)&lt;=$D$27/2,AND(AA$28&gt;=$D32,AA$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AB$28-$E32)&lt;=$D$27/2,AND(AB$28&gt;=$D32,AB$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AC$28-$E32)&lt;=$D$27/2,AND(AC$28&gt;=$D32,AC$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AD$28-$E32)&lt;=$D$27/2,AND(AD$28&gt;=$D32,AD$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AE$28-$E32)&lt;=$D$27/2,AND(AE$28&gt;=$D32,AE$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AF$28-$E32)&lt;=$D$27/2,AND(AF$28&gt;=$D32,AF$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AG$28-$E32)&lt;=$D$27/2,AND(AG$28&gt;=$D32,AG$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AH$28-$E32)&lt;=$D$27/2,AND(AH$28&gt;=$D32,AH$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI32" s="675" t="str">
+        <x:f>IF(IF($D32=$F32,ABS(AI$28-$E32)&lt;=$D$27/2,AND(AI$28&gt;=$D32,AI$28&lt;=$F32)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="18" customHeight="1">
+      <x:c r="A33" s="673" t="str">
+        <x:f>A18</x:f>
+        <x:v>Trading — P / E</x:v>
+      </x:c>
+      <x:c r="B33" s="698"/>
+      <x:c r="C33" s="698"/>
+      <x:c r="D33" s="699" t="n">
+        <x:f>B18</x:f>
+        <x:v>49.89126177669402</x:v>
+      </x:c>
+      <x:c r="E33" s="699" t="n">
+        <x:f>C18</x:f>
+        <x:v>54.28133382929772</x:v>
+      </x:c>
+      <x:c r="F33" s="699" t="n">
+        <x:f>D18</x:f>
+        <x:v>58.73871533415601</x:v>
+      </x:c>
+      <x:c r="G33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(G$28-$E33)&lt;=$D$27/2,AND(G$28&gt;=$D33,G$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="H33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(H$28-$E33)&lt;=$D$27/2,AND(H$28&gt;=$D33,H$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="I33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(I$28-$E33)&lt;=$D$27/2,AND(I$28&gt;=$D33,I$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="J33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(J$28-$E33)&lt;=$D$27/2,AND(J$28&gt;=$D33,J$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="K33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(K$28-$E33)&lt;=$D$27/2,AND(K$28&gt;=$D33,K$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="L33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(L$28-$E33)&lt;=$D$27/2,AND(L$28&gt;=$D33,L$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="M33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(M$28-$E33)&lt;=$D$27/2,AND(M$28&gt;=$D33,M$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="N33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(N$28-$E33)&lt;=$D$27/2,AND(N$28&gt;=$D33,N$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="O33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(O$28-$E33)&lt;=$D$27/2,AND(O$28&gt;=$D33,O$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="P33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(P$28-$E33)&lt;=$D$27/2,AND(P$28&gt;=$D33,P$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(Q$28-$E33)&lt;=$D$27/2,AND(Q$28&gt;=$D33,Q$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="R33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(R$28-$E33)&lt;=$D$27/2,AND(R$28&gt;=$D33,R$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="S33" s="675" t="n">
+        <x:f>IF(IF($D33=$F33,ABS(S$28-$E33)&lt;=$D$27/2,AND(S$28&gt;=$D33,S$28&lt;=$F33)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T33" s="675" t="n">
+        <x:f>IF(IF($D33=$F33,ABS(T$28-$E33)&lt;=$D$27/2,AND(T$28&gt;=$D33,T$28&lt;=$F33)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U33" s="675" t="n">
+        <x:f>IF(IF($D33=$F33,ABS(U$28-$E33)&lt;=$D$27/2,AND(U$28&gt;=$D33,U$28&lt;=$F33)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V33" s="675" t="n">
+        <x:f>IF(IF($D33=$F33,ABS(V$28-$E33)&lt;=$D$27/2,AND(V$28&gt;=$D33,V$28&lt;=$F33)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(W$28-$E33)&lt;=$D$27/2,AND(W$28&gt;=$D33,W$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="X33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(X$28-$E33)&lt;=$D$27/2,AND(X$28&gt;=$D33,X$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(Y$28-$E33)&lt;=$D$27/2,AND(Y$28&gt;=$D33,Y$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(Z$28-$E33)&lt;=$D$27/2,AND(Z$28&gt;=$D33,Z$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AA$28-$E33)&lt;=$D$27/2,AND(AA$28&gt;=$D33,AA$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AB$28-$E33)&lt;=$D$27/2,AND(AB$28&gt;=$D33,AB$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AC$28-$E33)&lt;=$D$27/2,AND(AC$28&gt;=$D33,AC$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AD$28-$E33)&lt;=$D$27/2,AND(AD$28&gt;=$D33,AD$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AE$28-$E33)&lt;=$D$27/2,AND(AE$28&gt;=$D33,AE$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AF$28-$E33)&lt;=$D$27/2,AND(AF$28&gt;=$D33,AF$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AG$28-$E33)&lt;=$D$27/2,AND(AG$28&gt;=$D33,AG$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AH$28-$E33)&lt;=$D$27/2,AND(AH$28&gt;=$D33,AH$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI33" s="675" t="str">
+        <x:f>IF(IF($D33=$F33,ABS(AI$28-$E33)&lt;=$D$27/2,AND(AI$28&gt;=$D33,AI$28&lt;=$F33)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="18" customHeight="1">
+      <x:c r="A34" s="673" t="str">
+        <x:f>A19</x:f>
+        <x:v>Precedent — EV / Revenue</x:v>
+      </x:c>
+      <x:c r="B34" s="698"/>
+      <x:c r="C34" s="698"/>
+      <x:c r="D34" s="699" t="n">
+        <x:f>B19</x:f>
+        <x:v>34.0626126411909</x:v>
+      </x:c>
+      <x:c r="E34" s="699" t="n">
+        <x:f>C19</x:f>
+        <x:v>45.32446369026972</x:v>
+      </x:c>
+      <x:c r="F34" s="699" t="n">
+        <x:f>D19</x:f>
+        <x:v>52.57395681762598</x:v>
+      </x:c>
+      <x:c r="G34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(G$28-$E34)&lt;=$D$27/2,AND(G$28&gt;=$D34,G$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="H34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(H$28-$E34)&lt;=$D$27/2,AND(H$28&gt;=$D34,H$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="I34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(I$28-$E34)&lt;=$D$27/2,AND(I$28&gt;=$D34,I$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="J34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(J$28-$E34)&lt;=$D$27/2,AND(J$28&gt;=$D34,J$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="K34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(K$28-$E34)&lt;=$D$27/2,AND(K$28&gt;=$D34,K$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="L34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(L$28-$E34)&lt;=$D$27/2,AND(L$28&gt;=$D34,L$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="M34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(M$28-$E34)&lt;=$D$27/2,AND(M$28&gt;=$D34,M$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(N$28-$E34)&lt;=$D$27/2,AND(N$28&gt;=$D34,N$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(O$28-$E34)&lt;=$D$27/2,AND(O$28&gt;=$D34,O$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(P$28-$E34)&lt;=$D$27/2,AND(P$28&gt;=$D34,P$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(Q$28-$E34)&lt;=$D$27/2,AND(Q$28&gt;=$D34,Q$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(R$28-$E34)&lt;=$D$27/2,AND(R$28&gt;=$D34,R$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(S$28-$E34)&lt;=$D$27/2,AND(S$28&gt;=$D34,S$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T34" s="675" t="n">
+        <x:f>IF(IF($D34=$F34,ABS(T$28-$E34)&lt;=$D$27/2,AND(T$28&gt;=$D34,T$28&lt;=$F34)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(U$28-$E34)&lt;=$D$27/2,AND(U$28&gt;=$D34,U$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="V34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(V$28-$E34)&lt;=$D$27/2,AND(V$28&gt;=$D34,V$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="W34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(W$28-$E34)&lt;=$D$27/2,AND(W$28&gt;=$D34,W$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="X34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(X$28-$E34)&lt;=$D$27/2,AND(X$28&gt;=$D34,X$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(Y$28-$E34)&lt;=$D$27/2,AND(Y$28&gt;=$D34,Y$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(Z$28-$E34)&lt;=$D$27/2,AND(Z$28&gt;=$D34,Z$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AA$28-$E34)&lt;=$D$27/2,AND(AA$28&gt;=$D34,AA$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AB$28-$E34)&lt;=$D$27/2,AND(AB$28&gt;=$D34,AB$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AC$28-$E34)&lt;=$D$27/2,AND(AC$28&gt;=$D34,AC$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AD$28-$E34)&lt;=$D$27/2,AND(AD$28&gt;=$D34,AD$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AE$28-$E34)&lt;=$D$27/2,AND(AE$28&gt;=$D34,AE$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AF$28-$E34)&lt;=$D$27/2,AND(AF$28&gt;=$D34,AF$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AG$28-$E34)&lt;=$D$27/2,AND(AG$28&gt;=$D34,AG$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AH$28-$E34)&lt;=$D$27/2,AND(AH$28&gt;=$D34,AH$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI34" s="675" t="str">
+        <x:f>IF(IF($D34=$F34,ABS(AI$28-$E34)&lt;=$D$27/2,AND(AI$28&gt;=$D34,AI$28&lt;=$F34)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="18" customHeight="1">
+      <x:c r="A35" s="673" t="str">
+        <x:f>A20</x:f>
+        <x:v>Precedent — EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="B35" s="698"/>
+      <x:c r="C35" s="698"/>
+      <x:c r="D35" s="699" t="n">
+        <x:f>B20</x:f>
+        <x:v>39.08531176777297</x:v>
+      </x:c>
+      <x:c r="E35" s="699" t="n">
+        <x:f>C20</x:f>
+        <x:v>40.27345666415471</x:v>
+      </x:c>
+      <x:c r="F35" s="699" t="n">
+        <x:f>D20</x:f>
+        <x:v>41.46160156053644</x:v>
+      </x:c>
+      <x:c r="G35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(G$28-$E35)&lt;=$D$27/2,AND(G$28&gt;=$D35,G$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="H35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(H$28-$E35)&lt;=$D$27/2,AND(H$28&gt;=$D35,H$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="I35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(I$28-$E35)&lt;=$D$27/2,AND(I$28&gt;=$D35,I$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="J35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(J$28-$E35)&lt;=$D$27/2,AND(J$28&gt;=$D35,J$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="K35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(K$28-$E35)&lt;=$D$27/2,AND(K$28&gt;=$D35,K$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="L35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(L$28-$E35)&lt;=$D$27/2,AND(L$28&gt;=$D35,L$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="M35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(M$28-$E35)&lt;=$D$27/2,AND(M$28&gt;=$D35,M$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="N35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(N$28-$E35)&lt;=$D$27/2,AND(N$28&gt;=$D35,N$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="O35" s="675" t="n">
+        <x:f>IF(IF($D35=$F35,ABS(O$28-$E35)&lt;=$D$27/2,AND(O$28&gt;=$D35,O$28&lt;=$F35)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(P$28-$E35)&lt;=$D$27/2,AND(P$28&gt;=$D35,P$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(Q$28-$E35)&lt;=$D$27/2,AND(Q$28&gt;=$D35,Q$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="R35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(R$28-$E35)&lt;=$D$27/2,AND(R$28&gt;=$D35,R$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="S35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(S$28-$E35)&lt;=$D$27/2,AND(S$28&gt;=$D35,S$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="T35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(T$28-$E35)&lt;=$D$27/2,AND(T$28&gt;=$D35,T$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="U35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(U$28-$E35)&lt;=$D$27/2,AND(U$28&gt;=$D35,U$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="V35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(V$28-$E35)&lt;=$D$27/2,AND(V$28&gt;=$D35,V$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="W35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(W$28-$E35)&lt;=$D$27/2,AND(W$28&gt;=$D35,W$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="X35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(X$28-$E35)&lt;=$D$27/2,AND(X$28&gt;=$D35,X$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(Y$28-$E35)&lt;=$D$27/2,AND(Y$28&gt;=$D35,Y$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(Z$28-$E35)&lt;=$D$27/2,AND(Z$28&gt;=$D35,Z$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AA$28-$E35)&lt;=$D$27/2,AND(AA$28&gt;=$D35,AA$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AB$28-$E35)&lt;=$D$27/2,AND(AB$28&gt;=$D35,AB$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AC$28-$E35)&lt;=$D$27/2,AND(AC$28&gt;=$D35,AC$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AD$28-$E35)&lt;=$D$27/2,AND(AD$28&gt;=$D35,AD$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AE$28-$E35)&lt;=$D$27/2,AND(AE$28&gt;=$D35,AE$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AF$28-$E35)&lt;=$D$27/2,AND(AF$28&gt;=$D35,AF$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AG$28-$E35)&lt;=$D$27/2,AND(AG$28&gt;=$D35,AG$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AH$28-$E35)&lt;=$D$27/2,AND(AH$28&gt;=$D35,AH$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI35" s="675" t="str">
+        <x:f>IF(IF($D35=$F35,ABS(AI$28-$E35)&lt;=$D$27/2,AND(AI$28&gt;=$D35,AI$28&lt;=$F35)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="18" customHeight="1">
+      <x:c r="A36" s="673" t="str">
+        <x:f>A21</x:f>
+        <x:v>Precedent — EV / EBIT</x:v>
+      </x:c>
+      <x:c r="B36" s="698"/>
+      <x:c r="C36" s="698"/>
+      <x:c r="D36" s="699" t="n">
+        <x:f>B21</x:f>
+        <x:v>51.98488081157034</x:v>
+      </x:c>
+      <x:c r="E36" s="699" t="n">
+        <x:f>C21</x:f>
+        <x:v>55.05026643373155</x:v>
+      </x:c>
+      <x:c r="F36" s="699" t="n">
+        <x:f>D21</x:f>
+        <x:v>58.11565205589273</x:v>
+      </x:c>
+      <x:c r="G36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(G$28-$E36)&lt;=$D$27/2,AND(G$28&gt;=$D36,G$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="H36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(H$28-$E36)&lt;=$D$27/2,AND(H$28&gt;=$D36,H$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="I36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(I$28-$E36)&lt;=$D$27/2,AND(I$28&gt;=$D36,I$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="J36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(J$28-$E36)&lt;=$D$27/2,AND(J$28&gt;=$D36,J$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="K36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(K$28-$E36)&lt;=$D$27/2,AND(K$28&gt;=$D36,K$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="L36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(L$28-$E36)&lt;=$D$27/2,AND(L$28&gt;=$D36,L$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="M36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(M$28-$E36)&lt;=$D$27/2,AND(M$28&gt;=$D36,M$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="N36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(N$28-$E36)&lt;=$D$27/2,AND(N$28&gt;=$D36,N$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="O36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(O$28-$E36)&lt;=$D$27/2,AND(O$28&gt;=$D36,O$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="P36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(P$28-$E36)&lt;=$D$27/2,AND(P$28&gt;=$D36,P$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(Q$28-$E36)&lt;=$D$27/2,AND(Q$28&gt;=$D36,Q$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="R36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(R$28-$E36)&lt;=$D$27/2,AND(R$28&gt;=$D36,R$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="S36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(S$28-$E36)&lt;=$D$27/2,AND(S$28&gt;=$D36,S$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="T36" s="675" t="n">
+        <x:f>IF(IF($D36=$F36,ABS(T$28-$E36)&lt;=$D$27/2,AND(T$28&gt;=$D36,T$28&lt;=$F36)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U36" s="675" t="n">
+        <x:f>IF(IF($D36=$F36,ABS(U$28-$E36)&lt;=$D$27/2,AND(U$28&gt;=$D36,U$28&lt;=$F36)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="V36" s="675" t="n">
+        <x:f>IF(IF($D36=$F36,ABS(V$28-$E36)&lt;=$D$27/2,AND(V$28&gt;=$D36,V$28&lt;=$F36)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(W$28-$E36)&lt;=$D$27/2,AND(W$28&gt;=$D36,W$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="X36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(X$28-$E36)&lt;=$D$27/2,AND(X$28&gt;=$D36,X$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(Y$28-$E36)&lt;=$D$27/2,AND(Y$28&gt;=$D36,Y$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(Z$28-$E36)&lt;=$D$27/2,AND(Z$28&gt;=$D36,Z$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AA$28-$E36)&lt;=$D$27/2,AND(AA$28&gt;=$D36,AA$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AB$28-$E36)&lt;=$D$27/2,AND(AB$28&gt;=$D36,AB$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AC$28-$E36)&lt;=$D$27/2,AND(AC$28&gt;=$D36,AC$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AD$28-$E36)&lt;=$D$27/2,AND(AD$28&gt;=$D36,AD$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AE$28-$E36)&lt;=$D$27/2,AND(AE$28&gt;=$D36,AE$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AF$28-$E36)&lt;=$D$27/2,AND(AF$28&gt;=$D36,AF$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AG$28-$E36)&lt;=$D$27/2,AND(AG$28&gt;=$D36,AG$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AH$28-$E36)&lt;=$D$27/2,AND(AH$28&gt;=$D36,AH$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI36" s="675" t="str">
+        <x:f>IF(IF($D36=$F36,ABS(AI$28-$E36)&lt;=$D$27/2,AND(AI$28&gt;=$D36,AI$28&lt;=$F36)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="18" customHeight="1">
+      <x:c r="A37" s="673" t="str">
+        <x:f>A22</x:f>
+        <x:v>Precedent — Premium Paid</x:v>
+      </x:c>
+      <x:c r="B37" s="698"/>
+      <x:c r="C37" s="698"/>
+      <x:c r="D37" s="699" t="n">
+        <x:f>B22</x:f>
+        <x:v>80.48617499999999</x:v>
+      </x:c>
+      <x:c r="E37" s="699" t="n">
+        <x:f>C22</x:f>
+        <x:v>84.51795</x:v>
+      </x:c>
+      <x:c r="F37" s="699" t="n">
+        <x:f>D22</x:f>
+        <x:v>86.30985</x:v>
+      </x:c>
+      <x:c r="G37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(G$28-$E37)&lt;=$D$27/2,AND(G$28&gt;=$D37,G$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="H37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(H$28-$E37)&lt;=$D$27/2,AND(H$28&gt;=$D37,H$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="I37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(I$28-$E37)&lt;=$D$27/2,AND(I$28&gt;=$D37,I$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="J37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(J$28-$E37)&lt;=$D$27/2,AND(J$28&gt;=$D37,J$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="K37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(K$28-$E37)&lt;=$D$27/2,AND(K$28&gt;=$D37,K$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="L37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(L$28-$E37)&lt;=$D$27/2,AND(L$28&gt;=$D37,L$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="M37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(M$28-$E37)&lt;=$D$27/2,AND(M$28&gt;=$D37,M$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="N37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(N$28-$E37)&lt;=$D$27/2,AND(N$28&gt;=$D37,N$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="O37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(O$28-$E37)&lt;=$D$27/2,AND(O$28&gt;=$D37,O$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="P37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(P$28-$E37)&lt;=$D$27/2,AND(P$28&gt;=$D37,P$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(Q$28-$E37)&lt;=$D$27/2,AND(Q$28&gt;=$D37,Q$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="R37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(R$28-$E37)&lt;=$D$27/2,AND(R$28&gt;=$D37,R$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="S37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(S$28-$E37)&lt;=$D$27/2,AND(S$28&gt;=$D37,S$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="T37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(T$28-$E37)&lt;=$D$27/2,AND(T$28&gt;=$D37,T$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="U37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(U$28-$E37)&lt;=$D$27/2,AND(U$28&gt;=$D37,U$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="V37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(V$28-$E37)&lt;=$D$27/2,AND(V$28&gt;=$D37,V$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="W37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(W$28-$E37)&lt;=$D$27/2,AND(W$28&gt;=$D37,W$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="X37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(X$28-$E37)&lt;=$D$27/2,AND(X$28&gt;=$D37,X$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(Y$28-$E37)&lt;=$D$27/2,AND(Y$28&gt;=$D37,Y$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(Z$28-$E37)&lt;=$D$27/2,AND(Z$28&gt;=$D37,Z$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AA$28-$E37)&lt;=$D$27/2,AND(AA$28&gt;=$D37,AA$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AB$28-$E37)&lt;=$D$27/2,AND(AB$28&gt;=$D37,AB$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AC$28-$E37)&lt;=$D$27/2,AND(AC$28&gt;=$D37,AC$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AD$28-$E37)&lt;=$D$27/2,AND(AD$28&gt;=$D37,AD$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AE$28-$E37)&lt;=$D$27/2,AND(AE$28&gt;=$D37,AE$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF37" s="675" t="n">
+        <x:f>IF(IF($D37=$F37,ABS(AF$28-$E37)&lt;=$D$27/2,AND(AF$28&gt;=$D37,AF$28&lt;=$F37)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG37" s="675" t="n">
+        <x:f>IF(IF($D37=$F37,ABS(AG$28-$E37)&lt;=$D$27/2,AND(AG$28&gt;=$D37,AG$28&lt;=$F37)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AH$28-$E37)&lt;=$D$27/2,AND(AH$28&gt;=$D37,AH$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI37" s="675" t="str">
+        <x:f>IF(IF($D37=$F37,ABS(AI$28-$E37)&lt;=$D$27/2,AND(AI$28&gt;=$D37,AI$28&lt;=$F37)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="18" customHeight="1">
+      <x:c r="A38" s="673" t="str">
+        <x:f>A23</x:f>
+        <x:v>Unaffected Share Price</x:v>
+      </x:c>
+      <x:c r="B38" s="698"/>
+      <x:c r="C38" s="698"/>
+      <x:c r="D38" s="699" t="n">
+        <x:f>B23</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="E38" s="699" t="n">
+        <x:f>C23</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="F38" s="699" t="n">
+        <x:f>D23</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="G38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(G$28-$E38)&lt;=$D$27/2,AND(G$28&gt;=$D38,G$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="H38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(H$28-$E38)&lt;=$D$27/2,AND(H$28&gt;=$D38,H$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="I38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(I$28-$E38)&lt;=$D$27/2,AND(I$28&gt;=$D38,I$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="J38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(J$28-$E38)&lt;=$D$27/2,AND(J$28&gt;=$D38,J$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="K38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(K$28-$E38)&lt;=$D$27/2,AND(K$28&gt;=$D38,K$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="L38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(L$28-$E38)&lt;=$D$27/2,AND(L$28&gt;=$D38,L$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="M38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(M$28-$E38)&lt;=$D$27/2,AND(M$28&gt;=$D38,M$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="N38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(N$28-$E38)&lt;=$D$27/2,AND(N$28&gt;=$D38,N$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="O38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(O$28-$E38)&lt;=$D$27/2,AND(O$28&gt;=$D38,O$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="P38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(P$28-$E38)&lt;=$D$27/2,AND(P$28&gt;=$D38,P$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(Q$28-$E38)&lt;=$D$27/2,AND(Q$28&gt;=$D38,Q$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="R38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(R$28-$E38)&lt;=$D$27/2,AND(R$28&gt;=$D38,R$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="S38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(S$28-$E38)&lt;=$D$27/2,AND(S$28&gt;=$D38,S$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="T38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(T$28-$E38)&lt;=$D$27/2,AND(T$28&gt;=$D38,T$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="U38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(U$28-$E38)&lt;=$D$27/2,AND(U$28&gt;=$D38,U$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="V38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(V$28-$E38)&lt;=$D$27/2,AND(V$28&gt;=$D38,V$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="W38" s="675" t="n">
+        <x:f>IF(IF($D38=$F38,ABS(W$28-$E38)&lt;=$D$27/2,AND(W$28&gt;=$D38,W$28&lt;=$F38)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(X$28-$E38)&lt;=$D$27/2,AND(X$28&gt;=$D38,X$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(Y$28-$E38)&lt;=$D$27/2,AND(Y$28&gt;=$D38,Y$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(Z$28-$E38)&lt;=$D$27/2,AND(Z$28&gt;=$D38,Z$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AA$28-$E38)&lt;=$D$27/2,AND(AA$28&gt;=$D38,AA$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AB$28-$E38)&lt;=$D$27/2,AND(AB$28&gt;=$D38,AB$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AC$28-$E38)&lt;=$D$27/2,AND(AC$28&gt;=$D38,AC$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AD38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AD$28-$E38)&lt;=$D$27/2,AND(AD$28&gt;=$D38,AD$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AE38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AE$28-$E38)&lt;=$D$27/2,AND(AE$28&gt;=$D38,AE$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AF38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AF$28-$E38)&lt;=$D$27/2,AND(AF$28&gt;=$D38,AF$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AG38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AG$28-$E38)&lt;=$D$27/2,AND(AG$28&gt;=$D38,AG$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AH38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AH$28-$E38)&lt;=$D$27/2,AND(AH$28&gt;=$D38,AH$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI38" s="675" t="str">
+        <x:f>IF(IF($D38=$F38,ABS(AI$28-$E38)&lt;=$D$27/2,AND(AI$28&gt;=$D38,AI$28&lt;=$F38)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="18" customHeight="1">
+      <x:c r="A39" s="676" t="str">
+        <x:f>A24</x:f>
+        <x:v>Acquisition Range</x:v>
+      </x:c>
+      <x:c r="B39" s="700"/>
+      <x:c r="C39" s="700"/>
+      <x:c r="D39" s="701" t="n">
+        <x:f>B24</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="E39" s="701" t="n">
+        <x:f>C24</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F39" s="701" t="n">
+        <x:f>D24</x:f>
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="G39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(G$28-$E39)&lt;=$D$27/2,AND(G$28&gt;=$D39,G$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="H39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(H$28-$E39)&lt;=$D$27/2,AND(H$28&gt;=$D39,H$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="I39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(I$28-$E39)&lt;=$D$27/2,AND(I$28&gt;=$D39,I$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="J39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(J$28-$E39)&lt;=$D$27/2,AND(J$28&gt;=$D39,J$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="K39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(K$28-$E39)&lt;=$D$27/2,AND(K$28&gt;=$D39,K$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="L39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(L$28-$E39)&lt;=$D$27/2,AND(L$28&gt;=$D39,L$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="M39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(M$28-$E39)&lt;=$D$27/2,AND(M$28&gt;=$D39,M$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="N39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(N$28-$E39)&lt;=$D$27/2,AND(N$28&gt;=$D39,N$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="O39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(O$28-$E39)&lt;=$D$27/2,AND(O$28&gt;=$D39,O$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="P39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(P$28-$E39)&lt;=$D$27/2,AND(P$28&gt;=$D39,P$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="Q39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(Q$28-$E39)&lt;=$D$27/2,AND(Q$28&gt;=$D39,Q$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="R39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(R$28-$E39)&lt;=$D$27/2,AND(R$28&gt;=$D39,R$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="S39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(S$28-$E39)&lt;=$D$27/2,AND(S$28&gt;=$D39,S$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="T39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(T$28-$E39)&lt;=$D$27/2,AND(T$28&gt;=$D39,T$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="U39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(U$28-$E39)&lt;=$D$27/2,AND(U$28&gt;=$D39,U$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="V39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(V$28-$E39)&lt;=$D$27/2,AND(V$28&gt;=$D39,V$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="W39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(W$28-$E39)&lt;=$D$27/2,AND(W$28&gt;=$D39,W$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="X39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(X$28-$E39)&lt;=$D$27/2,AND(X$28&gt;=$D39,X$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="Y39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(Y$28-$E39)&lt;=$D$27/2,AND(Y$28&gt;=$D39,Y$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="Z39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(Z$28-$E39)&lt;=$D$27/2,AND(Z$28&gt;=$D39,Z$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="AA39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(AA$28-$E39)&lt;=$D$27/2,AND(AA$28&gt;=$D39,AA$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="AB39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(AB$28-$E39)&lt;=$D$27/2,AND(AB$28&gt;=$D39,AB$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="AC39" s="678" t="n">
+        <x:f>IF(IF($D39=$F39,ABS(AC$28-$E39)&lt;=$D$27/2,AND(AC$28&gt;=$D39,AC$28&lt;=$F39)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AD39" s="678" t="n">
+        <x:f>IF(IF($D39=$F39,ABS(AD$28-$E39)&lt;=$D$27/2,AND(AD$28&gt;=$D39,AD$28&lt;=$F39)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE39" s="678" t="n">
+        <x:f>IF(IF($D39=$F39,ABS(AE$28-$E39)&lt;=$D$27/2,AND(AE$28&gt;=$D39,AE$28&lt;=$F39)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AF39" s="678" t="n">
+        <x:f>IF(IF($D39=$F39,ABS(AF$28-$E39)&lt;=$D$27/2,AND(AF$28&gt;=$D39,AF$28&lt;=$F39)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AG39" s="678" t="n">
+        <x:f>IF(IF($D39=$F39,ABS(AG$28-$E39)&lt;=$D$27/2,AND(AG$28&gt;=$D39,AG$28&lt;=$F39)),1,"")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AH39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(AH$28-$E39)&lt;=$D$27/2,AND(AH$28&gt;=$D39,AH$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+      <x:c r="AI39" s="678" t="str">
+        <x:f>IF(IF($D39=$F39,ABS(AI$28-$E39)&lt;=$D$27/2,AND(AI$28&gt;=$D39,AI$28&lt;=$F39)),1,"")</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="18" customHeight="1">
+      <x:c r="A40" s="538"/>
+      <x:c r="B40" s="538"/>
+      <x:c r="C40" s="538"/>
+      <x:c r="D40" s="538"/>
+      <x:c r="E40" s="538"/>
+      <x:c r="F40" s="538"/>
+      <x:c r="G40" s="538"/>
+      <x:c r="H40" s="538"/>
+      <x:c r="I40" s="538"/>
+      <x:c r="J40" s="538"/>
+      <x:c r="K40" s="538"/>
+      <x:c r="L40" s="538"/>
+      <x:c r="M40" s="538"/>
+      <x:c r="N40" s="538"/>
+      <x:c r="O40" s="538"/>
+      <x:c r="P40" s="538"/>
+      <x:c r="Q40" s="538"/>
+      <x:c r="R40" s="538"/>
+      <x:c r="S40" s="538"/>
+      <x:c r="T40" s="538"/>
+      <x:c r="U40" s="538"/>
+      <x:c r="V40" s="538"/>
+      <x:c r="W40" s="538"/>
+      <x:c r="X40" s="538"/>
+      <x:c r="Y40" s="538"/>
+      <x:c r="Z40" s="538"/>
+      <x:c r="AA40" s="538"/>
+      <x:c r="AB40" s="538"/>
+      <x:c r="AC40" s="538"/>
+      <x:c r="AD40" s="538"/>
+      <x:c r="AE40" s="538"/>
+      <x:c r="AF40" s="538"/>
+      <x:c r="AG40" s="538"/>
+      <x:c r="AH40" s="538"/>
+      <x:c r="AI40" s="538"/>
+    </x:row>
+    <x:row r="41" ht="18" customHeight="1">
+      <x:c r="A41" s="652" t="str">
+        <x:v>ANALYST INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="B41" s="652"/>
+      <x:c r="C41" s="652"/>
+      <x:c r="D41" s="652"/>
+      <x:c r="E41" s="652"/>
+      <x:c r="F41" s="652"/>
+      <x:c r="G41" s="652"/>
+      <x:c r="H41" s="652"/>
+      <x:c r="I41" s="652"/>
+      <x:c r="J41" s="652"/>
+      <x:c r="K41" s="652"/>
+      <x:c r="L41" s="652"/>
+      <x:c r="M41" s="652"/>
+      <x:c r="N41" s="652"/>
+      <x:c r="O41" s="652"/>
+      <x:c r="P41" s="652"/>
+      <x:c r="Q41" s="652"/>
+      <x:c r="R41" s="652"/>
+      <x:c r="S41" s="652"/>
+      <x:c r="T41" s="652"/>
+      <x:c r="U41" s="652"/>
+      <x:c r="V41" s="652"/>
+      <x:c r="W41" s="652"/>
+      <x:c r="X41" s="652"/>
+      <x:c r="Y41" s="652"/>
+      <x:c r="Z41" s="652"/>
+      <x:c r="AA41" s="652"/>
+      <x:c r="AB41" s="652"/>
+      <x:c r="AC41" s="652"/>
+      <x:c r="AD41" s="652"/>
+      <x:c r="AE41" s="652"/>
+      <x:c r="AF41" s="652"/>
+      <x:c r="AG41" s="652"/>
+      <x:c r="AH41" s="652"/>
+      <x:c r="AI41" s="652"/>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="679" t="str">
+        <x:v>Standalone methodologies indicate approximately $40–$55 per share when the low DCF is treated as an intrinsic-value anchor and greater weight is placed on market and transaction operating multiples. This range is below the unaffected price, showing that current market expectations already embed value beyond the base standalone case.</x:v>
+      </x:c>
+      <x:c r="B42" s="679"/>
+      <x:c r="C42" s="679"/>
+      <x:c r="D42" s="679"/>
+      <x:c r="E42" s="679"/>
+      <x:c r="F42" s="679"/>
+      <x:c r="G42" s="679"/>
+      <x:c r="H42" s="679"/>
+      <x:c r="I42" s="679"/>
+      <x:c r="J42" s="679"/>
+      <x:c r="K42" s="679"/>
+      <x:c r="L42" s="679"/>
+      <x:c r="M42" s="679"/>
+      <x:c r="N42" s="679"/>
+      <x:c r="O42" s="679"/>
+      <x:c r="P42" s="679"/>
+      <x:c r="Q42" s="679"/>
+      <x:c r="R42" s="679"/>
+      <x:c r="S42" s="679"/>
+      <x:c r="T42" s="679"/>
+      <x:c r="U42" s="679"/>
+      <x:c r="V42" s="679"/>
+      <x:c r="W42" s="679"/>
+      <x:c r="X42" s="679"/>
+      <x:c r="Y42" s="679"/>
+      <x:c r="Z42" s="679"/>
+      <x:c r="AA42" s="679"/>
+      <x:c r="AB42" s="679"/>
+      <x:c r="AC42" s="679"/>
+      <x:c r="AD42" s="679"/>
+      <x:c r="AE42" s="679"/>
+      <x:c r="AF42" s="679"/>
+      <x:c r="AG42" s="679"/>
+      <x:c r="AH42" s="679"/>
+      <x:c r="AI42" s="679"/>
+    </x:row>
+    <x:row r="43" ht="28" customHeight="1">
+      <x:c r="A43" s="679" t="str">
+        <x:v>The $75–$85 acquisition range is not a weighted average of the valuation methods. It is a control-price framework anchored by the unaffected share price and observed precedent premiums. The $80 midpoint implies a 33.9% premium and must be tested against Rockwell financing capacity, accretion/dilution, and required synergies.</x:v>
+      </x:c>
+      <x:c r="B43" s="679"/>
+      <x:c r="C43" s="679"/>
+      <x:c r="D43" s="679"/>
+      <x:c r="E43" s="679"/>
+      <x:c r="F43" s="679"/>
+      <x:c r="G43" s="679"/>
+      <x:c r="H43" s="679"/>
+      <x:c r="I43" s="679"/>
+      <x:c r="J43" s="679"/>
+      <x:c r="K43" s="679"/>
+      <x:c r="L43" s="679"/>
+      <x:c r="M43" s="679"/>
+      <x:c r="N43" s="679"/>
+      <x:c r="O43" s="679"/>
+      <x:c r="P43" s="679"/>
+      <x:c r="Q43" s="679"/>
+      <x:c r="R43" s="679"/>
+      <x:c r="S43" s="679"/>
+      <x:c r="T43" s="679"/>
+      <x:c r="U43" s="679"/>
+      <x:c r="V43" s="679"/>
+      <x:c r="W43" s="679"/>
+      <x:c r="X43" s="679"/>
+      <x:c r="Y43" s="679"/>
+      <x:c r="Z43" s="679"/>
+      <x:c r="AA43" s="679"/>
+      <x:c r="AB43" s="679"/>
+      <x:c r="AC43" s="679"/>
+      <x:c r="AD43" s="679"/>
+      <x:c r="AE43" s="679"/>
+      <x:c r="AF43" s="679"/>
+      <x:c r="AG43" s="679"/>
+      <x:c r="AH43" s="679"/>
+      <x:c r="AI43" s="679"/>
+    </x:row>
+    <x:row r="44" ht="28" customHeight="1">
+      <x:c r="A44" s="680" t="str">
+        <x:v>Avoid double-counting: the premium-paid range already reflects control and anticipated strategic value. Synergies will be modeled separately and used to test how much of the purchase premium Rockwell can economically support.</x:v>
+      </x:c>
+      <x:c r="B44" s="680"/>
+      <x:c r="C44" s="680"/>
+      <x:c r="D44" s="680"/>
+      <x:c r="E44" s="680"/>
+      <x:c r="F44" s="680"/>
+      <x:c r="G44" s="680"/>
+      <x:c r="H44" s="680"/>
+      <x:c r="I44" s="680"/>
+      <x:c r="J44" s="680"/>
+      <x:c r="K44" s="680"/>
+      <x:c r="L44" s="680"/>
+      <x:c r="M44" s="680"/>
+      <x:c r="N44" s="680"/>
+      <x:c r="O44" s="680"/>
+      <x:c r="P44" s="680"/>
+      <x:c r="Q44" s="680"/>
+      <x:c r="R44" s="680"/>
+      <x:c r="S44" s="680"/>
+      <x:c r="T44" s="680"/>
+      <x:c r="U44" s="680"/>
+      <x:c r="V44" s="680"/>
+      <x:c r="W44" s="680"/>
+      <x:c r="X44" s="680"/>
+      <x:c r="Y44" s="680"/>
+      <x:c r="Z44" s="680"/>
+      <x:c r="AA44" s="680"/>
+      <x:c r="AB44" s="680"/>
+      <x:c r="AC44" s="680"/>
+      <x:c r="AD44" s="680"/>
+      <x:c r="AE44" s="680"/>
+      <x:c r="AF44" s="680"/>
+      <x:c r="AG44" s="680"/>
+      <x:c r="AH44" s="680"/>
+      <x:c r="AI44" s="680"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:AI1"/>
+    <x:mergeCell ref="A2:AI2"/>
+    <x:mergeCell ref="B3:AI3"/>
+    <x:mergeCell ref="A5:AI5"/>
+    <x:mergeCell ref="H6:AI10"/>
+    <x:mergeCell ref="A12:AI12"/>
+    <x:mergeCell ref="A26:AI26"/>
+    <x:mergeCell ref="A28:F28"/>
+    <x:mergeCell ref="A29:C29"/>
+    <x:mergeCell ref="A30:C30"/>
+    <x:mergeCell ref="A31:C31"/>
+    <x:mergeCell ref="A32:C32"/>
+    <x:mergeCell ref="A33:C33"/>
+    <x:mergeCell ref="A34:C34"/>
+    <x:mergeCell ref="A35:C35"/>
+    <x:mergeCell ref="A36:C36"/>
+    <x:mergeCell ref="A37:C37"/>
+    <x:mergeCell ref="A38:C38"/>
+    <x:mergeCell ref="A39:C39"/>
+    <x:mergeCell ref="A41:AI41"/>
+    <x:mergeCell ref="A42:AI42"/>
+    <x:mergeCell ref="A43:AI43"/>
+    <x:mergeCell ref="A44:AI44"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="G29:AI29">
+    <x:cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G30:AI30">
+    <x:cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G31:AI31">
+    <x:cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G32:AI32">
+    <x:cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G33:AI33">
+    <x:cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G34:AI34">
+    <x:cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G35:AI35">
+    <x:cfRule type="cellIs" dxfId="12" priority="7" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G36:AI36">
+    <x:cfRule type="cellIs" dxfId="13" priority="8" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G37:AI37">
+    <x:cfRule type="cellIs" dxfId="14" priority="9" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G38:AI38">
+    <x:cfRule type="cellIs" dxfId="15" priority="10" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G39:AI39">
+    <x:cfRule type="cellIs" dxfId="16" priority="11" operator="equal">
+      <x:formula>1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -4823,8 +8041,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="595" t="str">
-        <x:v>PRECEDENTS COMPLETE</x:v>
+      <x:c r="B3" s="703" t="str">
+        <x:v>VALUATION COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -5434,6 +8652,110 @@
       </x:c>
       <x:c r="G27" s="484" t="str">
         <x:v>Precedent Transactions rows 35-38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="484" t="str">
+        <x:v>Valuation summary source links</x:v>
+      </x:c>
+      <x:c r="B28" s="484" t="n">
+        <x:f>ABS('Valuation Summary'!B6-'Precedent Transactions'!B30)+ABS('Valuation Summary'!B14-'DCF'!C53)+ABS('Valuation Summary'!C15-'Trading Comps'!H35)+ABS('Valuation Summary'!D22-'Precedent Transactions'!I38)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C28" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D28" s="484" t="n">
+        <x:f>B28-C28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F28" s="705" t="str">
+        <x:f>IF(ABS(D28)&lt;=E28,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G28" s="484" t="str">
+        <x:v>Valuation Summary rows 6 and 14-23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="484" t="str">
+        <x:v>Valuation summary range ordering</x:v>
+      </x:c>
+      <x:c r="B29" s="484" t="n">
+        <x:f>MIN('Valuation Summary'!C14-'Valuation Summary'!B14,'Valuation Summary'!D14-'Valuation Summary'!C14,'Valuation Summary'!C15-'Valuation Summary'!B15,'Valuation Summary'!D15-'Valuation Summary'!C15,'Valuation Summary'!C24-'Valuation Summary'!B24,'Valuation Summary'!D24-'Valuation Summary'!C24)</x:f>
+        <x:v>2.838179172040391</x:v>
+      </x:c>
+      <x:c r="C29" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="484" t="n">
+        <x:f>MIN(0,B29-C29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="705" t="str">
+        <x:f>IF(ABS(D29)&lt;=E29,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G29" s="484" t="str">
+        <x:v>Valuation Summary rows 14-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="484" t="str">
+        <x:v>Illustrative offer bridge</x:v>
+      </x:c>
+      <x:c r="B30" s="484" t="n">
+        <x:f>ABS('Valuation Summary'!F6-'Valuation Summary'!B9*'DCF'!B21)+ABS('Valuation Summary'!F7-('Valuation Summary'!F6-'DCF'!B19+'DCF'!B20))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C30" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D30" s="484" t="n">
+        <x:f>B30-C30</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F30" s="705" t="str">
+        <x:f>IF(ABS(D30)&lt;=E30,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G30" s="484" t="str">
+        <x:v>Valuation Summary rows 6-10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="484" t="str">
+        <x:v>Acquisition range clears unaffected price</x:v>
+      </x:c>
+      <x:c r="B31" s="484" t="n">
+        <x:f>'Valuation Summary'!B8-'Valuation Summary'!B6</x:f>
+        <x:v>15.270000000000003</x:v>
+      </x:c>
+      <x:c r="C31" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D31" s="484" t="n">
+        <x:f>MIN(0,B31-C31)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="705" t="str">
+        <x:f>IF(ABS(D31)&lt;=E31,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G31" s="484" t="str">
+        <x:v>Valuation Summary rows 6 and 8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8885,7 +12207,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1253d88ebc414e4b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b8f520df1b4c56"/>
 </x:worksheet>
 </file>
 
@@ -10608,7 +13930,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf434cbab284f21"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc00c44d81f14a8f"/>
 </x:worksheet>
 </file>
 
@@ -14095,7 +17417,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R097f1c7c90d54033"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4442a8d220a34658"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
transaction: complete sources uses and financing
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R457d4c52bdcc45f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rd87ba725cd3a44be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R5a63c95d72c3428f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Ra482baaf475e49c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rc9ed7c9300674339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Reaf29fdd19b447f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R457c5431ff534f01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R28af15ad8b4f45b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="Rf75f54d46c3a4ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rd60ea701054f404a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R84a0f26357144bd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Ra0c34c6de1cc485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R795df57cfade41f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="Rbe8d072268be4b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Ra790963faba54537"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R726f1438037b465f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R8938b613068843b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9f76b875fb9b4ed1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Race26722ee364e77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rceffdc1228a149ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R5086969ebcbd4bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R74509b1304f741f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rdce5d24f4a8341b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Rb6ce4dc29e3a4ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R73746c7f18844d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R964711bf78954e10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R3655ee02dd3b4a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R6be7431042704ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rf181f41f6dfd41e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R61c40aa9b1a04285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R1d180f90671c4ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R2887959b1a14403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rf391f8a751ab48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R7a004861e7f64801"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -436,7 +436,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="47">
+  <x:fills count="54">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -668,8 +668,43 @@
         <x:fgColor rgb="FFF8F8F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="24">
+  <x:borders count="25">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -921,11 +956,25 @@
         <x:color rgb="FF17365D"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="double">
+        <x:color rgb="FF17365D"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="706">
+  <x:cellXfs count="770">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2368,6 +2417,170 @@
     <x:xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="40" fillId="41" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="51" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="51" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="40" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="51" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="49" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="49" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="51" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="37" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="37" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="37" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="37" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="40" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="40" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="41" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="41" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="41" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="41" fillId="49" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="38" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="221" fontId="38" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="218" fontId="37" fillId="52" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="37" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="37" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="42" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="42" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="37" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="38" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="214" fontId="42" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="42" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="37" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="213" fontId="38" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2444,7 +2657,7 @@
         <x:color rgb="FF7F7F7F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF7F7F7F"/>
         </x:patternFill>
       </x:fill>
@@ -2454,7 +2667,7 @@
         <x:color rgb="FF2F75B5"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF2F75B5"/>
         </x:patternFill>
       </x:fill>
@@ -2464,7 +2677,7 @@
         <x:color rgb="FF2F75B5"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF2F75B5"/>
         </x:patternFill>
       </x:fill>
@@ -2474,7 +2687,7 @@
         <x:color rgb="FF2F75B5"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF2F75B5"/>
         </x:patternFill>
       </x:fill>
@@ -2484,7 +2697,7 @@
         <x:color rgb="FF2F75B5"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF2F75B5"/>
         </x:patternFill>
       </x:fill>
@@ -2494,7 +2707,7 @@
         <x:color rgb="FF70AD47"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF70AD47"/>
         </x:patternFill>
       </x:fill>
@@ -2504,7 +2717,7 @@
         <x:color rgb="FF70AD47"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF70AD47"/>
         </x:patternFill>
       </x:fill>
@@ -2514,7 +2727,7 @@
         <x:color rgb="FF70AD47"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF70AD47"/>
         </x:patternFill>
       </x:fill>
@@ -2524,7 +2737,7 @@
         <x:color rgb="FFF4B183"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4B183"/>
         </x:patternFill>
       </x:fill>
@@ -2534,7 +2747,7 @@
         <x:color rgb="FFFFD966"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFD966"/>
         </x:patternFill>
       </x:fill>
@@ -2544,7 +2757,7 @@
         <x:color rgb="FF17365D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF17365D"/>
         </x:patternFill>
       </x:fill>
@@ -2847,7 +3060,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.6 — valuation summary complete</x:v>
+        <x:v>0.7 — financing complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -2902,8 +3115,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="702" t="str">
-        <x:v>VALUATION COMPLETE</x:v>
+      <x:c r="B9" s="766" t="str">
+        <x:v>FINANCING COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -7443,110 +7656,1699 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="3" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="707" t="str">
         <x:v>Sources &amp; Uses</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Purchase price, transaction uses, and funding sources</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="707"/>
+      <x:c r="C1" s="707"/>
+      <x:c r="D1" s="707"/>
+      <x:c r="E1" s="707"/>
+      <x:c r="F1" s="707"/>
+      <x:c r="G1" s="707"/>
+      <x:c r="H1" s="707"/>
+      <x:c r="I1" s="707"/>
+      <x:c r="J1" s="707"/>
+      <x:c r="K1" s="707"/>
+      <x:c r="L1" s="707"/>
+      <x:c r="M1" s="707"/>
+      <x:c r="N1" s="707"/>
+      <x:c r="O1" s="707"/>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="709" t="str">
+        <x:v>Purchase price, consideration mix, funding sources, ownership, and pro forma leverage | USD millions except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="709"/>
+      <x:c r="C2" s="709"/>
+      <x:c r="D2" s="709"/>
+      <x:c r="E2" s="709"/>
+      <x:c r="F2" s="709"/>
+      <x:c r="G2" s="709"/>
+      <x:c r="H2" s="709"/>
+      <x:c r="I2" s="709"/>
+      <x:c r="J2" s="709"/>
+      <x:c r="K2" s="709"/>
+      <x:c r="L2" s="709"/>
+      <x:c r="M2" s="709"/>
+      <x:c r="N2" s="709"/>
+      <x:c r="O2" s="709"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="432" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="711" t="str">
+        <x:v>Complete — illustrative 30% cash / 70% stock consideration with $4.0 billion of new debt</x:v>
+      </x:c>
+      <x:c r="C3" s="711"/>
+      <x:c r="D3" s="711"/>
+      <x:c r="E3" s="711"/>
+      <x:c r="F3" s="711"/>
+      <x:c r="G3" s="711"/>
+      <x:c r="H3" s="711"/>
+      <x:c r="I3" s="711"/>
+      <x:c r="J3" s="711"/>
+      <x:c r="K3" s="711"/>
+      <x:c r="L3" s="711"/>
+      <x:c r="M3" s="711"/>
+      <x:c r="N3" s="711"/>
+      <x:c r="O3" s="711"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="538"/>
+      <x:c r="B4" s="538"/>
+      <x:c r="C4" s="538"/>
+      <x:c r="D4" s="538"/>
+      <x:c r="E4" s="538"/>
+      <x:c r="F4" s="538"/>
+      <x:c r="G4" s="538"/>
+      <x:c r="H4" s="538"/>
+      <x:c r="I4" s="538"/>
+      <x:c r="J4" s="538"/>
+      <x:c r="K4" s="538"/>
+      <x:c r="L4" s="538"/>
+      <x:c r="M4" s="538"/>
+      <x:c r="N4" s="538"/>
+      <x:c r="O4" s="538"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="713" t="str">
+        <x:v>TRANSACTION ASSUMPTIONS</x:v>
+      </x:c>
+      <x:c r="B5" s="713"/>
+      <x:c r="C5" s="713"/>
+      <x:c r="D5" s="713"/>
+      <x:c r="E5" s="713"/>
+      <x:c r="F5" s="713"/>
+      <x:c r="G5" s="538"/>
+      <x:c r="H5" s="713" t="str">
+        <x:v>PURCHASE PRICE BRIDGE</x:v>
+      </x:c>
+      <x:c r="I5" s="713"/>
+      <x:c r="J5" s="713"/>
+      <x:c r="K5" s="713"/>
+      <x:c r="L5" s="713"/>
+      <x:c r="M5" s="713"/>
+      <x:c r="N5" s="713"/>
+      <x:c r="O5" s="713"/>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="715" t="str">
+        <x:v>Offer price / share</x:v>
+      </x:c>
+      <x:c r="B6" s="663" t="n">
+        <x:f>'Valuation Summary'!B9</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C6" s="436" t="str">
+        <x:v>$ / share</x:v>
+      </x:c>
+      <x:c r="D6" s="436" t="str">
+        <x:v>Valuation Summary</x:v>
+      </x:c>
+      <x:c r="E6" s="664" t="str">
+        <x:v>Midpoint of the selected acquisition range</x:v>
+      </x:c>
+      <x:c r="F6" s="664"/>
+      <x:c r="G6" s="538"/>
+      <x:c r="H6" s="715" t="str">
+        <x:v>Equity purchase price</x:v>
+      </x:c>
+      <x:c r="I6" s="739" t="n">
+        <x:f>B6*B9</x:f>
+        <x:v>13457.919999999998</x:v>
+      </x:c>
+      <x:c r="J6" s="664" t="str">
+        <x:v>Offer price × diluted target shares</x:v>
+      </x:c>
+      <x:c r="K6" s="664"/>
+      <x:c r="L6" s="664"/>
+      <x:c r="M6" s="664"/>
+      <x:c r="N6" s="664"/>
+      <x:c r="O6" s="664"/>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="715" t="str">
+        <x:v>Unaffected share price</x:v>
+      </x:c>
+      <x:c r="B7" s="663" t="n">
+        <x:f>'Valuation Summary'!B6</x:f>
+        <x:v>59.73</x:v>
+      </x:c>
+      <x:c r="C7" s="436" t="str">
+        <x:v>$ / share</x:v>
+      </x:c>
+      <x:c r="D7" s="436" t="str">
+        <x:v>S-039 / Valuation Summary</x:v>
+      </x:c>
+      <x:c r="E7" s="664" t="str">
+        <x:v>Closing price on Aug. 20, 2026</x:v>
+      </x:c>
+      <x:c r="F7" s="664"/>
+      <x:c r="G7" s="538"/>
+      <x:c r="H7" s="715" t="str">
+        <x:v>Add: target debt</x:v>
+      </x:c>
+      <x:c r="I7" s="739" t="n">
+        <x:f>'DCF'!B20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="664" t="str">
+        <x:v>Cognex has no funded debt</x:v>
+      </x:c>
+      <x:c r="K7" s="664"/>
+      <x:c r="L7" s="664"/>
+      <x:c r="M7" s="664"/>
+      <x:c r="N7" s="664"/>
+      <x:c r="O7" s="664"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="715" t="str">
+        <x:v>Offer premium</x:v>
+      </x:c>
+      <x:c r="B8" s="733" t="n">
+        <x:f>B6/B7-1</x:f>
+        <x:v>0.3393604553825549</x:v>
+      </x:c>
+      <x:c r="C8" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D8" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="E8" s="664" t="str">
+        <x:v>Offer price divided by unaffected price less one</x:v>
+      </x:c>
+      <x:c r="F8" s="664"/>
+      <x:c r="G8" s="538"/>
+      <x:c r="H8" s="715" t="str">
+        <x:v>Less: target cash and investments</x:v>
+      </x:c>
+      <x:c r="I8" s="739" t="n">
+        <x:f>'DCF'!B19</x:f>
+        <x:v>755.013</x:v>
+      </x:c>
+      <x:c r="J8" s="664" t="str">
+        <x:v>Acquired cash reduces enterprise value but is not used as a closing source</x:v>
+      </x:c>
+      <x:c r="K8" s="664"/>
+      <x:c r="L8" s="664"/>
+      <x:c r="M8" s="664"/>
+      <x:c r="N8" s="664"/>
+      <x:c r="O8" s="664"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="715" t="str">
+        <x:v>Target diluted shares</x:v>
+      </x:c>
+      <x:c r="B9" s="560" t="n">
+        <x:f>'DCF'!B21</x:f>
+        <x:v>168.224</x:v>
+      </x:c>
+      <x:c r="C9" s="436" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D9" s="436" t="str">
+        <x:v>DCF / S-022</x:v>
+      </x:c>
+      <x:c r="E9" s="664" t="str">
+        <x:v>Latest target share-count proxy</x:v>
+      </x:c>
+      <x:c r="F9" s="664"/>
+      <x:c r="G9" s="538"/>
+      <x:c r="H9" s="715" t="str">
+        <x:v>Transaction enterprise value</x:v>
+      </x:c>
+      <x:c r="I9" s="739" t="n">
+        <x:f>I6+I7-I8</x:f>
+        <x:v>12702.906999999997</x:v>
+      </x:c>
+      <x:c r="J9" s="664" t="str">
+        <x:v>Equity value plus debt less cash</x:v>
+      </x:c>
+      <x:c r="K9" s="664"/>
+      <x:c r="L9" s="664"/>
+      <x:c r="M9" s="664"/>
+      <x:c r="N9" s="664"/>
+      <x:c r="O9" s="664"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="715" t="str">
+        <x:v>Cash consideration</x:v>
+      </x:c>
+      <x:c r="B10" s="734" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C10" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D10" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E10" s="664" t="str">
+        <x:v>Cash portion paid to target shareholders</x:v>
+      </x:c>
+      <x:c r="F10" s="664"/>
+      <x:c r="G10" s="538"/>
+      <x:c r="H10" s="715" t="str">
+        <x:v>EV / FY2026E revenue</x:v>
+      </x:c>
+      <x:c r="I10" s="740" t="n">
+        <x:f>I9/'CGNX Operating Model'!E20</x:f>
+        <x:v>11.14290087719298</x:v>
+      </x:c>
+      <x:c r="J10" s="664" t="str">
+        <x:v>High relative to fundamental revenue benchmarks</x:v>
+      </x:c>
+      <x:c r="K10" s="664"/>
+      <x:c r="L10" s="664"/>
+      <x:c r="M10" s="664"/>
+      <x:c r="N10" s="664"/>
+      <x:c r="O10" s="664"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="715" t="str">
+        <x:v>Stock consideration</x:v>
+      </x:c>
+      <x:c r="B11" s="735" t="n">
+        <x:f>1-B10</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="C11" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D11" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="E11" s="664" t="str">
+        <x:v>Direct ROK shares issued to target shareholders</x:v>
+      </x:c>
+      <x:c r="F11" s="664"/>
+      <x:c r="G11" s="538"/>
+      <x:c r="H11" s="715" t="str">
+        <x:v>EV / FY2026E EBITDA</x:v>
+      </x:c>
+      <x:c r="I11" s="740" t="n">
+        <x:f>I9/'CGNX Operating Model'!E32</x:f>
+        <x:v>38.42379612825166</x:v>
+      </x:c>
+      <x:c r="J11" s="664" t="str">
+        <x:v>High relative to trading and precedent EBITDA benchmarks</x:v>
+      </x:c>
+      <x:c r="K11" s="664"/>
+      <x:c r="L11" s="664"/>
+      <x:c r="M11" s="664"/>
+      <x:c r="N11" s="664"/>
+      <x:c r="O11" s="664"/>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="715" t="str">
+        <x:v>Transaction fees</x:v>
+      </x:c>
+      <x:c r="B12" s="734" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C12" s="436" t="str">
+        <x:v>% equity purchase price</x:v>
+      </x:c>
+      <x:c r="D12" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E12" s="664" t="str">
+        <x:v>Legal, advisory, accounting, and integration-planning fees</x:v>
+      </x:c>
+      <x:c r="F12" s="664"/>
+      <x:c r="G12" s="538"/>
+      <x:c r="H12" s="715" t="str">
+        <x:v>FY2026E P / E</x:v>
+      </x:c>
+      <x:c r="I12" s="740" t="n">
+        <x:f>B6/'Trading Comps'!B28</x:f>
+        <x:v>53.484315789473676</x:v>
+      </x:c>
+      <x:c r="J12" s="664" t="str">
+        <x:v>Within the upper portion of the trading P / E range</x:v>
+      </x:c>
+      <x:c r="K12" s="664"/>
+      <x:c r="L12" s="664"/>
+      <x:c r="M12" s="664"/>
+      <x:c r="N12" s="664"/>
+      <x:c r="O12" s="664"/>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="715" t="str">
+        <x:v>Debt financing fees</x:v>
+      </x:c>
+      <x:c r="B13" s="734" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C13" s="436" t="str">
+        <x:v>% new debt</x:v>
+      </x:c>
+      <x:c r="D13" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E13" s="664" t="str">
+        <x:v>Upfront fees on new debt</x:v>
+      </x:c>
+      <x:c r="F13" s="664"/>
+      <x:c r="G13" s="538"/>
+      <x:c r="H13" s="538"/>
+      <x:c r="I13" s="538"/>
+      <x:c r="J13" s="554"/>
+      <x:c r="K13" s="554"/>
+      <x:c r="L13" s="554"/>
+      <x:c r="M13" s="554"/>
+      <x:c r="N13" s="554"/>
+      <x:c r="O13" s="554"/>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="715" t="str">
+        <x:v>New term loan / bridge</x:v>
+      </x:c>
+      <x:c r="B14" s="736" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="C14" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D14" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E14" s="664" t="str">
+        <x:v>Illustrative acquisition bridge / term loan</x:v>
+      </x:c>
+      <x:c r="F14" s="664"/>
+      <x:c r="G14" s="538"/>
+      <x:c r="H14" s="713" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I14" s="713"/>
+      <x:c r="J14" s="753"/>
+      <x:c r="K14" s="753"/>
+      <x:c r="L14" s="753"/>
+      <x:c r="M14" s="753"/>
+      <x:c r="N14" s="753"/>
+      <x:c r="O14" s="753"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="715" t="str">
+        <x:v>New senior notes</x:v>
+      </x:c>
+      <x:c r="B15" s="736" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="C15" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D15" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E15" s="664" t="str">
+        <x:v>Illustrative permanent debt financing</x:v>
+      </x:c>
+      <x:c r="F15" s="664"/>
+      <x:c r="G15" s="538"/>
+      <x:c r="H15" s="715" t="str">
+        <x:v>Total transaction uses</x:v>
+      </x:c>
+      <x:c r="I15" s="741" t="n">
+        <x:f>B26</x:f>
+        <x:v>13632.499199999998</x:v>
+      </x:c>
+      <x:c r="J15" s="664" t="str">
+        <x:v>Purchase consideration plus fees</x:v>
+      </x:c>
+      <x:c r="K15" s="664"/>
+      <x:c r="L15" s="664"/>
+      <x:c r="M15" s="664"/>
+      <x:c r="N15" s="664"/>
+      <x:c r="O15" s="664"/>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="715" t="str">
+        <x:v>New debt interest rate</x:v>
+      </x:c>
+      <x:c r="B16" s="734" t="n">
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="C16" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D16" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E16" s="664" t="str">
+        <x:v>Blended pre-tax rate used in accretion/dilution</x:v>
+      </x:c>
+      <x:c r="F16" s="664"/>
+      <x:c r="G16" s="538"/>
+      <x:c r="H16" s="715" t="str">
+        <x:v>New ROK shares issued</x:v>
+      </x:c>
+      <x:c r="I16" s="742" t="n">
+        <x:f>I33</x:f>
+        <x:v>21.834613512573874</x:v>
+      </x:c>
+      <x:c r="J16" s="664" t="str">
+        <x:v>Stock consideration divided by ROK share price</x:v>
+      </x:c>
+      <x:c r="K16" s="664"/>
+      <x:c r="L16" s="664"/>
+      <x:c r="M16" s="664"/>
+      <x:c r="N16" s="664"/>
+      <x:c r="O16" s="664"/>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="715" t="str">
+        <x:v>ROK share price</x:v>
+      </x:c>
+      <x:c r="B17" s="737" t="n">
+        <x:v>431.45</x:v>
+      </x:c>
+      <x:c r="C17" s="436" t="str">
+        <x:v>$ / share</x:v>
+      </x:c>
+      <x:c r="D17" s="436" t="str">
+        <x:v>S-051</x:v>
+      </x:c>
+      <x:c r="E17" s="664" t="str">
+        <x:v>Aug. 20, 2026 closing price</x:v>
+      </x:c>
+      <x:c r="F17" s="664"/>
+      <x:c r="G17" s="538"/>
+      <x:c r="H17" s="715" t="str">
+        <x:v>Pro forma gross leverage</x:v>
+      </x:c>
+      <x:c r="I17" s="743" t="n">
+        <x:f>B48</x:f>
+        <x:v>2.9252187842861477</x:v>
+      </x:c>
+      <x:c r="J17" s="664" t="str">
+        <x:v>Below the illustrative 3.0x gross-leverage ceiling</x:v>
+      </x:c>
+      <x:c r="K17" s="664"/>
+      <x:c r="L17" s="664"/>
+      <x:c r="M17" s="664"/>
+      <x:c r="N17" s="664"/>
+      <x:c r="O17" s="664"/>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="715" t="str">
+        <x:v>Illustrative close date</x:v>
+      </x:c>
+      <x:c r="B18" s="738" t="n">
+        <x:v>46477</x:v>
+      </x:c>
+      <x:c r="C18" s="436" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="D18" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E18" s="664" t="str">
+        <x:v>Allows a realistic regulatory and shareholder approval period</x:v>
+      </x:c>
+      <x:c r="F18" s="664"/>
+      <x:c r="G18" s="538"/>
+      <x:c r="H18" s="715" t="str">
+        <x:v>ROK cash remaining</x:v>
+      </x:c>
+      <x:c r="I18" s="741" t="n">
+        <x:f>B33</x:f>
+        <x:v>211.04479999999967</x:v>
+      </x:c>
+      <x:c r="J18" s="664" t="str">
+        <x:v>Before adding acquired Cognex cash</x:v>
+      </x:c>
+      <x:c r="K18" s="664"/>
+      <x:c r="L18" s="664"/>
+      <x:c r="M18" s="664"/>
+      <x:c r="N18" s="664"/>
+      <x:c r="O18" s="664"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="538"/>
+      <x:c r="B19" s="538"/>
+      <x:c r="C19" s="538"/>
+      <x:c r="D19" s="538"/>
+      <x:c r="E19" s="538"/>
+      <x:c r="F19" s="538"/>
+      <x:c r="G19" s="538"/>
+      <x:c r="H19" s="538"/>
+      <x:c r="I19" s="538"/>
+      <x:c r="J19" s="538"/>
+      <x:c r="K19" s="538"/>
+      <x:c r="L19" s="538"/>
+      <x:c r="M19" s="538"/>
+      <x:c r="N19" s="538"/>
+      <x:c r="O19" s="538"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="713" t="str">
+        <x:v>USES</x:v>
+      </x:c>
+      <x:c r="B20" s="713"/>
+      <x:c r="C20" s="713"/>
+      <x:c r="D20" s="713"/>
+      <x:c r="E20" s="713"/>
+      <x:c r="F20" s="713"/>
+      <x:c r="G20" s="538"/>
+      <x:c r="H20" s="713" t="str">
+        <x:v>SOURCES</x:v>
+      </x:c>
+      <x:c r="I20" s="713"/>
+      <x:c r="J20" s="713"/>
+      <x:c r="K20" s="713"/>
+      <x:c r="L20" s="713"/>
+      <x:c r="M20" s="713"/>
+      <x:c r="N20" s="538"/>
+      <x:c r="O20" s="538"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="715" t="str">
+        <x:v>Cash consideration</x:v>
+      </x:c>
+      <x:c r="B21" s="744" t="n">
+        <x:f>I6*B10</x:f>
+        <x:v>4037.3759999999993</x:v>
+      </x:c>
+      <x:c r="C21" s="664" t="str">
+        <x:v>Paid to Cognex shareholders</x:v>
+      </x:c>
+      <x:c r="D21" s="664"/>
+      <x:c r="E21" s="664"/>
+      <x:c r="F21" s="664"/>
+      <x:c r="G21" s="538"/>
+      <x:c r="H21" s="715" t="str">
+        <x:v>ROK cash on hand</x:v>
+      </x:c>
+      <x:c r="I21" s="744" t="n">
+        <x:f>B26-SUM(I22:I24)</x:f>
+        <x:v>211.95520000000033</x:v>
+      </x:c>
+      <x:c r="J21" s="664" t="str">
+        <x:v>Cash funding is the balancing source; constrained by available cash</x:v>
+      </x:c>
+      <x:c r="K21" s="664"/>
+      <x:c r="L21" s="664"/>
+      <x:c r="M21" s="664"/>
+      <x:c r="N21" s="538"/>
+      <x:c r="O21" s="538"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="715" t="str">
+        <x:v>Stock consideration</x:v>
+      </x:c>
+      <x:c r="B22" s="744" t="n">
+        <x:f>I6*B11</x:f>
+        <x:v>9420.543999999998</x:v>
+      </x:c>
+      <x:c r="C22" s="664" t="str">
+        <x:v>ROK common shares issued directly to Cognex shareholders</x:v>
+      </x:c>
+      <x:c r="D22" s="664"/>
+      <x:c r="E22" s="664"/>
+      <x:c r="F22" s="664"/>
+      <x:c r="G22" s="538"/>
+      <x:c r="H22" s="715" t="str">
+        <x:v>New term loan / bridge</x:v>
+      </x:c>
+      <x:c r="I22" s="744" t="n">
+        <x:f>B14</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J22" s="664" t="str">
+        <x:v>Illustrative acquisition debt</x:v>
+      </x:c>
+      <x:c r="K22" s="664"/>
+      <x:c r="L22" s="664"/>
+      <x:c r="M22" s="664"/>
+      <x:c r="N22" s="538"/>
+      <x:c r="O22" s="538"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="715" t="str">
+        <x:v>Refinance target debt</x:v>
+      </x:c>
+      <x:c r="B23" s="744" t="n">
+        <x:f>I7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C23" s="664" t="str">
+        <x:v>No funded Cognex debt</x:v>
+      </x:c>
+      <x:c r="D23" s="664"/>
+      <x:c r="E23" s="664"/>
+      <x:c r="F23" s="664"/>
+      <x:c r="G23" s="538"/>
+      <x:c r="H23" s="715" t="str">
+        <x:v>New senior notes</x:v>
+      </x:c>
+      <x:c r="I23" s="744" t="n">
+        <x:f>B15</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J23" s="664" t="str">
+        <x:v>Illustrative permanent debt</x:v>
+      </x:c>
+      <x:c r="K23" s="664"/>
+      <x:c r="L23" s="664"/>
+      <x:c r="M23" s="664"/>
+      <x:c r="N23" s="538"/>
+      <x:c r="O23" s="538"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="715" t="str">
+        <x:v>Transaction fees</x:v>
+      </x:c>
+      <x:c r="B24" s="744" t="n">
+        <x:f>I6*B12</x:f>
+        <x:v>134.5792</x:v>
+      </x:c>
+      <x:c r="C24" s="664" t="str">
+        <x:v>Estimated transaction expenses</x:v>
+      </x:c>
+      <x:c r="D24" s="664"/>
+      <x:c r="E24" s="664"/>
+      <x:c r="F24" s="664"/>
+      <x:c r="G24" s="538"/>
+      <x:c r="H24" s="715" t="str">
+        <x:v>ROK stock issued</x:v>
+      </x:c>
+      <x:c r="I24" s="744" t="n">
+        <x:f>B22</x:f>
+        <x:v>9420.543999999998</x:v>
+      </x:c>
+      <x:c r="J24" s="664" t="str">
+        <x:v>Direct stock consideration</x:v>
+      </x:c>
+      <x:c r="K24" s="664"/>
+      <x:c r="L24" s="664"/>
+      <x:c r="M24" s="664"/>
+      <x:c r="N24" s="538"/>
+      <x:c r="O24" s="538"/>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1">
+      <x:c r="A25" s="715" t="str">
+        <x:v>Debt financing fees</x:v>
+      </x:c>
+      <x:c r="B25" s="744" t="n">
+        <x:f>SUM(B14:B15)*B13</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C25" s="664" t="str">
+        <x:v>Upfront financing fees</x:v>
+      </x:c>
+      <x:c r="D25" s="664"/>
+      <x:c r="E25" s="664"/>
+      <x:c r="F25" s="664"/>
+      <x:c r="G25" s="538"/>
+      <x:c r="H25" s="715"/>
+      <x:c r="I25" s="744"/>
+      <x:c r="J25" s="664"/>
+      <x:c r="K25" s="664"/>
+      <x:c r="L25" s="664"/>
+      <x:c r="M25" s="664"/>
+      <x:c r="N25" s="538"/>
+      <x:c r="O25" s="538"/>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="722" t="str">
+        <x:v>Total uses</x:v>
+      </x:c>
+      <x:c r="B26" s="745" t="n">
+        <x:f>SUM(B21:B25)</x:f>
+        <x:v>13632.499199999998</x:v>
+      </x:c>
+      <x:c r="C26" s="754" t="str">
+        <x:v>Total funding requirement at closing</x:v>
+      </x:c>
+      <x:c r="D26" s="754"/>
+      <x:c r="E26" s="754"/>
+      <x:c r="F26" s="754"/>
+      <x:c r="G26" s="727"/>
+      <x:c r="H26" s="728" t="str">
+        <x:v>Total sources</x:v>
+      </x:c>
+      <x:c r="I26" s="745" t="n">
+        <x:f>SUM(I21:I24)</x:f>
+        <x:v>13632.499199999998</x:v>
+      </x:c>
+      <x:c r="J26" s="755" t="str">
+        <x:v>Must equal total uses</x:v>
+      </x:c>
+      <x:c r="K26" s="755"/>
+      <x:c r="L26" s="755"/>
+      <x:c r="M26" s="755"/>
+      <x:c r="N26" s="538"/>
+      <x:c r="O26" s="538"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="538"/>
+      <x:c r="B27" s="538"/>
+      <x:c r="C27" s="538"/>
+      <x:c r="D27" s="538"/>
+      <x:c r="E27" s="538"/>
+      <x:c r="F27" s="538"/>
+      <x:c r="G27" s="538"/>
+      <x:c r="H27" s="538"/>
+      <x:c r="I27" s="746"/>
+      <x:c r="J27" s="554"/>
+      <x:c r="K27" s="554"/>
+      <x:c r="L27" s="554"/>
+      <x:c r="M27" s="554"/>
+      <x:c r="N27" s="538"/>
+      <x:c r="O27" s="538"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="538"/>
+      <x:c r="B28" s="538"/>
+      <x:c r="C28" s="538"/>
+      <x:c r="D28" s="538"/>
+      <x:c r="E28" s="538"/>
+      <x:c r="F28" s="538"/>
+      <x:c r="G28" s="538"/>
+      <x:c r="H28" s="436" t="str">
+        <x:v>Sources less uses</x:v>
+      </x:c>
+      <x:c r="I28" s="747" t="n">
+        <x:f>I26-B26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="664" t="str">
+        <x:v>Required closing check</x:v>
+      </x:c>
+      <x:c r="K28" s="664"/>
+      <x:c r="L28" s="664"/>
+      <x:c r="M28" s="664"/>
+      <x:c r="N28" s="538"/>
+      <x:c r="O28" s="538"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="538"/>
+      <x:c r="B29" s="538"/>
+      <x:c r="C29" s="538"/>
+      <x:c r="D29" s="538"/>
+      <x:c r="E29" s="538"/>
+      <x:c r="F29" s="538"/>
+      <x:c r="G29" s="538"/>
+      <x:c r="H29" s="538"/>
+      <x:c r="I29" s="538"/>
+      <x:c r="J29" s="538"/>
+      <x:c r="K29" s="538"/>
+      <x:c r="L29" s="538"/>
+      <x:c r="M29" s="538"/>
+      <x:c r="N29" s="538"/>
+      <x:c r="O29" s="538"/>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="713" t="str">
+        <x:v>PRO FORMA LIQUIDITY AND LEVERAGE</x:v>
+      </x:c>
+      <x:c r="B30" s="713"/>
+      <x:c r="C30" s="713"/>
+      <x:c r="D30" s="713"/>
+      <x:c r="E30" s="713"/>
+      <x:c r="F30" s="713"/>
+      <x:c r="G30" s="538"/>
+      <x:c r="H30" s="713" t="str">
+        <x:v>PRO FORMA OWNERSHIP AND DEBT CAPACITY</x:v>
+      </x:c>
+      <x:c r="I30" s="713"/>
+      <x:c r="J30" s="713"/>
+      <x:c r="K30" s="713"/>
+      <x:c r="L30" s="713"/>
+      <x:c r="M30" s="713"/>
+      <x:c r="N30" s="713"/>
+      <x:c r="O30" s="713"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="715" t="str">
+        <x:v>ROK cash before transaction</x:v>
+      </x:c>
+      <x:c r="B31" s="744" t="n">
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="C31" s="436" t="str">
+        <x:v>S-050</x:v>
+      </x:c>
+      <x:c r="D31" s="664" t="str">
+        <x:v>March 31, 2026 filed cash balance</x:v>
+      </x:c>
+      <x:c r="E31" s="664"/>
+      <x:c r="F31" s="664"/>
+      <x:c r="G31" s="538"/>
+      <x:c r="H31" s="715" t="str">
+        <x:v>Stock consideration</x:v>
+      </x:c>
+      <x:c r="I31" s="744" t="n">
+        <x:f>B22</x:f>
+        <x:v>9420.543999999998</x:v>
+      </x:c>
+      <x:c r="J31" s="664" t="str">
+        <x:v>Direct stock consideration</x:v>
+      </x:c>
+      <x:c r="K31" s="664"/>
+      <x:c r="L31" s="664"/>
+      <x:c r="M31" s="664"/>
+      <x:c r="N31" s="664"/>
+      <x:c r="O31" s="664"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="715" t="str">
+        <x:v>Less: ROK cash used</x:v>
+      </x:c>
+      <x:c r="B32" s="744" t="n">
+        <x:f>I21</x:f>
+        <x:v>211.95520000000033</x:v>
+      </x:c>
+      <x:c r="C32" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="D32" s="664" t="str">
+        <x:v>Cash source required to balance closing</x:v>
+      </x:c>
+      <x:c r="E32" s="664"/>
+      <x:c r="F32" s="664"/>
+      <x:c r="G32" s="538"/>
+      <x:c r="H32" s="715" t="str">
+        <x:v>ROK share price</x:v>
+      </x:c>
+      <x:c r="I32" s="663" t="n">
+        <x:f>B17</x:f>
+        <x:v>431.45</x:v>
+      </x:c>
+      <x:c r="J32" s="664" t="str">
+        <x:v>S-051; Aug. 20, 2026 close</x:v>
+      </x:c>
+      <x:c r="K32" s="664"/>
+      <x:c r="L32" s="664"/>
+      <x:c r="M32" s="664"/>
+      <x:c r="N32" s="664"/>
+      <x:c r="O32" s="664"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="715" t="str">
+        <x:v>ROK cash remaining</x:v>
+      </x:c>
+      <x:c r="B33" s="744" t="n">
+        <x:f>B31-B32</x:f>
+        <x:v>211.04479999999967</x:v>
+      </x:c>
+      <x:c r="C33" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D33" s="664" t="str">
+        <x:v>Maintains more than $100 million of standalone liquidity</x:v>
+      </x:c>
+      <x:c r="E33" s="664"/>
+      <x:c r="F33" s="664"/>
+      <x:c r="G33" s="538"/>
+      <x:c r="H33" s="715" t="str">
+        <x:v>New ROK shares issued</x:v>
+      </x:c>
+      <x:c r="I33" s="749" t="n">
+        <x:f>I31/I32</x:f>
+        <x:v>21.834613512573874</x:v>
+      </x:c>
+      <x:c r="J33" s="664" t="str">
+        <x:v>Stock consideration divided by buyer share price</x:v>
+      </x:c>
+      <x:c r="K33" s="664"/>
+      <x:c r="L33" s="664"/>
+      <x:c r="M33" s="664"/>
+      <x:c r="N33" s="664"/>
+      <x:c r="O33" s="664"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="715" t="str">
+        <x:v>Add: acquired Cognex cash</x:v>
+      </x:c>
+      <x:c r="B34" s="744" t="n">
+        <x:f>'DCF'!B19</x:f>
+        <x:v>755.013</x:v>
+      </x:c>
+      <x:c r="C34" s="436" t="str">
+        <x:v>DCF / S-022</x:v>
+      </x:c>
+      <x:c r="D34" s="664" t="str">
+        <x:v>Retained post-close; not used to fund closing</x:v>
+      </x:c>
+      <x:c r="E34" s="664"/>
+      <x:c r="F34" s="664"/>
+      <x:c r="G34" s="538"/>
+      <x:c r="H34" s="715" t="str">
+        <x:v>ROK FY2026E diluted shares</x:v>
+      </x:c>
+      <x:c r="I34" s="560" t="n">
+        <x:f>'ROK Forecast'!E13</x:f>
+        <x:v>112.1952</x:v>
+      </x:c>
+      <x:c r="J34" s="664" t="str">
+        <x:v>Buyer forecast share count</x:v>
+      </x:c>
+      <x:c r="K34" s="664"/>
+      <x:c r="L34" s="664"/>
+      <x:c r="M34" s="664"/>
+      <x:c r="N34" s="664"/>
+      <x:c r="O34" s="664"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="715" t="str">
+        <x:v>Pro forma cash</x:v>
+      </x:c>
+      <x:c r="B35" s="744" t="n">
+        <x:f>SUM(B33:B34)</x:f>
+        <x:v>966.0577999999997</x:v>
+      </x:c>
+      <x:c r="C35" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D35" s="664" t="str">
+        <x:v>Combined cash available after close</x:v>
+      </x:c>
+      <x:c r="E35" s="664"/>
+      <x:c r="F35" s="664"/>
+      <x:c r="G35" s="538"/>
+      <x:c r="H35" s="715" t="str">
+        <x:v>Pro forma diluted shares</x:v>
+      </x:c>
+      <x:c r="I35" s="749" t="n">
+        <x:f>SUM(I33:I34)</x:f>
+        <x:v>134.02981351257387</x:v>
+      </x:c>
+      <x:c r="J35" s="664" t="str">
+        <x:v>Existing plus newly issued shares</x:v>
+      </x:c>
+      <x:c r="K35" s="664"/>
+      <x:c r="L35" s="664"/>
+      <x:c r="M35" s="664"/>
+      <x:c r="N35" s="664"/>
+      <x:c r="O35" s="664"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="715"/>
+      <x:c r="B36" s="744"/>
+      <x:c r="C36" s="436"/>
+      <x:c r="D36" s="664"/>
+      <x:c r="E36" s="664"/>
+      <x:c r="F36" s="664"/>
+      <x:c r="G36" s="538"/>
+      <x:c r="H36" s="715" t="str">
+        <x:v>Cognex holders ownership</x:v>
+      </x:c>
+      <x:c r="I36" s="750" t="n">
+        <x:f>I33/I35</x:f>
+        <x:v>0.1629086315972937</x:v>
+      </x:c>
+      <x:c r="J36" s="664" t="str">
+        <x:v>Target holders as percent of pro forma shares</x:v>
+      </x:c>
+      <x:c r="K36" s="664"/>
+      <x:c r="L36" s="664"/>
+      <x:c r="M36" s="664"/>
+      <x:c r="N36" s="664"/>
+      <x:c r="O36" s="664"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="715" t="str">
+        <x:v>ROK existing debt</x:v>
+      </x:c>
+      <x:c r="B37" s="744" t="n">
+        <x:f>SUM(B38:B40)</x:f>
+        <x:v>3691</x:v>
+      </x:c>
+      <x:c r="C37" s="436" t="str">
+        <x:v>S-050</x:v>
+      </x:c>
+      <x:c r="D37" s="664" t="str">
+        <x:v>March 31, 2026 funded debt</x:v>
+      </x:c>
+      <x:c r="E37" s="664"/>
+      <x:c r="F37" s="664"/>
+      <x:c r="G37" s="538"/>
+      <x:c r="H37" s="715" t="str">
+        <x:v>Existing ROK holders ownership</x:v>
+      </x:c>
+      <x:c r="I37" s="750" t="n">
+        <x:f>I34/I35</x:f>
+        <x:v>0.8370913684027064</x:v>
+      </x:c>
+      <x:c r="J37" s="664" t="str">
+        <x:v>Legacy holders as percent of pro forma shares</x:v>
+      </x:c>
+      <x:c r="K37" s="664"/>
+      <x:c r="L37" s="664"/>
+      <x:c r="M37" s="664"/>
+      <x:c r="N37" s="664"/>
+      <x:c r="O37" s="664"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="715" t="str">
+        <x:v>Short-term debt</x:v>
+      </x:c>
+      <x:c r="B38" s="744" t="n">
+        <x:v>1118</x:v>
+      </x:c>
+      <x:c r="C38" s="436" t="str">
+        <x:v>S-050</x:v>
+      </x:c>
+      <x:c r="D38" s="664" t="str">
+        <x:v>Commercial paper and other short-term debt</x:v>
+      </x:c>
+      <x:c r="E38" s="664"/>
+      <x:c r="F38" s="664"/>
+      <x:c r="G38" s="538"/>
+      <x:c r="H38" s="715"/>
+      <x:c r="I38" s="436"/>
+      <x:c r="J38" s="664"/>
+      <x:c r="K38" s="664"/>
+      <x:c r="L38" s="664"/>
+      <x:c r="M38" s="664"/>
+      <x:c r="N38" s="664"/>
+      <x:c r="O38" s="664"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="715" t="str">
+        <x:v>Current portion of long-term debt</x:v>
+      </x:c>
+      <x:c r="B39" s="744" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C39" s="436" t="str">
+        <x:v>S-050</x:v>
+      </x:c>
+      <x:c r="D39" s="664" t="str">
+        <x:v>Current portion</x:v>
+      </x:c>
+      <x:c r="E39" s="664"/>
+      <x:c r="F39" s="664"/>
+      <x:c r="G39" s="538"/>
+      <x:c r="H39" s="715" t="str">
+        <x:v>Illustrative maximum gross leverage</x:v>
+      </x:c>
+      <x:c r="I39" s="751" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J39" s="664" t="str">
+        <x:v>Analyst assumption for financing discipline</x:v>
+      </x:c>
+      <x:c r="K39" s="664"/>
+      <x:c r="L39" s="664"/>
+      <x:c r="M39" s="664"/>
+      <x:c r="N39" s="664"/>
+      <x:c r="O39" s="664"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="715" t="str">
+        <x:v>Long-term debt</x:v>
+      </x:c>
+      <x:c r="B40" s="744" t="n">
+        <x:v>2571</x:v>
+      </x:c>
+      <x:c r="C40" s="436" t="str">
+        <x:v>S-050</x:v>
+      </x:c>
+      <x:c r="D40" s="664" t="str">
+        <x:v>Long-term notes</x:v>
+      </x:c>
+      <x:c r="E40" s="664"/>
+      <x:c r="F40" s="664"/>
+      <x:c r="G40" s="538"/>
+      <x:c r="H40" s="715" t="str">
+        <x:v>Maximum pro forma gross debt</x:v>
+      </x:c>
+      <x:c r="I40" s="744" t="n">
+        <x:f>I39*B47</x:f>
+        <x:v>7887.61515</x:v>
+      </x:c>
+      <x:c r="J40" s="664" t="str">
+        <x:v>Gross leverage ceiling × pre-synergy EBITDA</x:v>
+      </x:c>
+      <x:c r="K40" s="664"/>
+      <x:c r="L40" s="664"/>
+      <x:c r="M40" s="664"/>
+      <x:c r="N40" s="664"/>
+      <x:c r="O40" s="664"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="715" t="str">
+        <x:v>Add: new debt</x:v>
+      </x:c>
+      <x:c r="B41" s="744" t="n">
+        <x:f>SUM(B14:B15)</x:f>
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="C41" s="436" t="str">
+        <x:v>Transaction assumptions</x:v>
+      </x:c>
+      <x:c r="D41" s="664" t="str">
+        <x:v>Selected acquisition debt</x:v>
+      </x:c>
+      <x:c r="E41" s="664"/>
+      <x:c r="F41" s="664"/>
+      <x:c r="G41" s="538"/>
+      <x:c r="H41" s="715" t="str">
+        <x:v>Implied new-debt capacity</x:v>
+      </x:c>
+      <x:c r="I41" s="744" t="n">
+        <x:f>I40-B37</x:f>
+        <x:v>4196.61515</x:v>
+      </x:c>
+      <x:c r="J41" s="664" t="str">
+        <x:v>Maximum debt less existing debt</x:v>
+      </x:c>
+      <x:c r="K41" s="664"/>
+      <x:c r="L41" s="664"/>
+      <x:c r="M41" s="664"/>
+      <x:c r="N41" s="664"/>
+      <x:c r="O41" s="664"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="715" t="str">
+        <x:v>Pro forma gross debt</x:v>
+      </x:c>
+      <x:c r="B42" s="744" t="n">
+        <x:f>SUM(B37,B41)</x:f>
+        <x:v>7691</x:v>
+      </x:c>
+      <x:c r="C42" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D42" s="664" t="str">
+        <x:v>Existing plus new debt</x:v>
+      </x:c>
+      <x:c r="E42" s="664"/>
+      <x:c r="F42" s="664"/>
+      <x:c r="G42" s="538"/>
+      <x:c r="H42" s="715" t="str">
+        <x:v>Selected new debt</x:v>
+      </x:c>
+      <x:c r="I42" s="744" t="n">
+        <x:f>B41</x:f>
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="J42" s="664" t="str">
+        <x:v>Term loan plus senior notes</x:v>
+      </x:c>
+      <x:c r="K42" s="664"/>
+      <x:c r="L42" s="664"/>
+      <x:c r="M42" s="664"/>
+      <x:c r="N42" s="664"/>
+      <x:c r="O42" s="664"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="715" t="str">
+        <x:v>Pro forma net debt</x:v>
+      </x:c>
+      <x:c r="B43" s="744" t="n">
+        <x:f>B42-B35</x:f>
+        <x:v>6724.9422</x:v>
+      </x:c>
+      <x:c r="C43" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D43" s="664" t="str">
+        <x:v>Gross debt less combined cash</x:v>
+      </x:c>
+      <x:c r="E43" s="664"/>
+      <x:c r="F43" s="664"/>
+      <x:c r="G43" s="538"/>
+      <x:c r="H43" s="715" t="str">
+        <x:v>Unused debt capacity</x:v>
+      </x:c>
+      <x:c r="I43" s="744" t="n">
+        <x:f>I41-I42</x:f>
+        <x:v>196.61514999999963</x:v>
+      </x:c>
+      <x:c r="J43" s="664" t="str">
+        <x:v>Debt capacity retained below ceiling</x:v>
+      </x:c>
+      <x:c r="K43" s="664"/>
+      <x:c r="L43" s="664"/>
+      <x:c r="M43" s="664"/>
+      <x:c r="N43" s="664"/>
+      <x:c r="O43" s="664"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="715"/>
+      <x:c r="B44" s="744"/>
+      <x:c r="C44" s="436"/>
+      <x:c r="D44" s="664"/>
+      <x:c r="E44" s="664"/>
+      <x:c r="F44" s="664"/>
+      <x:c r="G44" s="538"/>
+      <x:c r="H44" s="715" t="str">
+        <x:v>Minimum ROK cash balance</x:v>
+      </x:c>
+      <x:c r="I44" s="752" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J44" s="664" t="str">
+        <x:v>Illustrative standalone liquidity floor</x:v>
+      </x:c>
+      <x:c r="K44" s="664"/>
+      <x:c r="L44" s="664"/>
+      <x:c r="M44" s="664"/>
+      <x:c r="N44" s="664"/>
+      <x:c r="O44" s="664"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="715" t="str">
+        <x:v>ROK FY2026E EBITDA proxy</x:v>
+      </x:c>
+      <x:c r="B45" s="744" t="n">
+        <x:f>'ROK Forecast'!E10+'ROK Historical'!F25*('ROK Forecast'!E7/'ROK Forecast'!D7)</x:f>
+        <x:v>2298.60505</x:v>
+      </x:c>
+      <x:c r="C45" s="436" t="str">
+        <x:v>ROK Forecast / historical D&amp;A proxy</x:v>
+      </x:c>
+      <x:c r="D45" s="664" t="str">
+        <x:v>Enterprise operating profit plus scaled FY2025 D&amp;A</x:v>
+      </x:c>
+      <x:c r="E45" s="664"/>
+      <x:c r="F45" s="664"/>
+      <x:c r="G45" s="538"/>
+      <x:c r="H45" s="715"/>
+      <x:c r="I45" s="436"/>
+      <x:c r="J45" s="664"/>
+      <x:c r="K45" s="664"/>
+      <x:c r="L45" s="664"/>
+      <x:c r="M45" s="664"/>
+      <x:c r="N45" s="664"/>
+      <x:c r="O45" s="664"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="715" t="str">
+        <x:v>Cognex FY2026E EBITDA</x:v>
+      </x:c>
+      <x:c r="B46" s="744" t="n">
+        <x:f>'CGNX Operating Model'!E32</x:f>
+        <x:v>330.59999999999997</x:v>
+      </x:c>
+      <x:c r="C46" s="436" t="str">
+        <x:v>CGNX Operating Model</x:v>
+      </x:c>
+      <x:c r="D46" s="664" t="str">
+        <x:v>Standalone target EBITDA</x:v>
+      </x:c>
+      <x:c r="E46" s="664"/>
+      <x:c r="F46" s="664"/>
+      <x:c r="G46" s="538"/>
+      <x:c r="H46" s="538"/>
+      <x:c r="I46" s="538"/>
+      <x:c r="J46" s="538"/>
+      <x:c r="K46" s="538"/>
+      <x:c r="L46" s="538"/>
+      <x:c r="M46" s="538"/>
+      <x:c r="N46" s="538"/>
+      <x:c r="O46" s="538"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="715" t="str">
+        <x:v>Pro forma EBITDA — pre-synergy</x:v>
+      </x:c>
+      <x:c r="B47" s="744" t="n">
+        <x:f>SUM(B45:B46)</x:f>
+        <x:v>2629.20505</x:v>
+      </x:c>
+      <x:c r="C47" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D47" s="664" t="str">
+        <x:v>Before cost or revenue synergies</x:v>
+      </x:c>
+      <x:c r="E47" s="664"/>
+      <x:c r="F47" s="664"/>
+      <x:c r="G47" s="538"/>
+      <x:c r="H47" s="538"/>
+      <x:c r="I47" s="538"/>
+      <x:c r="J47" s="538"/>
+      <x:c r="K47" s="538"/>
+      <x:c r="L47" s="538"/>
+      <x:c r="M47" s="538"/>
+      <x:c r="N47" s="538"/>
+      <x:c r="O47" s="538"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="715" t="str">
+        <x:v>Pro forma gross leverage</x:v>
+      </x:c>
+      <x:c r="B48" s="748" t="n">
+        <x:f>B42/B47</x:f>
+        <x:v>2.9252187842861477</x:v>
+      </x:c>
+      <x:c r="C48" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D48" s="664" t="str">
+        <x:v>Gross debt divided by pre-synergy EBITDA</x:v>
+      </x:c>
+      <x:c r="E48" s="664"/>
+      <x:c r="F48" s="664"/>
+      <x:c r="G48" s="538"/>
+      <x:c r="H48" s="538"/>
+      <x:c r="I48" s="538"/>
+      <x:c r="J48" s="538"/>
+      <x:c r="K48" s="538"/>
+      <x:c r="L48" s="538"/>
+      <x:c r="M48" s="538"/>
+      <x:c r="N48" s="538"/>
+      <x:c r="O48" s="538"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="715" t="str">
+        <x:v>Pro forma net leverage</x:v>
+      </x:c>
+      <x:c r="B49" s="748" t="n">
+        <x:f>B43/B47</x:f>
+        <x:v>2.557785365580368</x:v>
+      </x:c>
+      <x:c r="C49" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D49" s="664" t="str">
+        <x:v>Net debt divided by pre-synergy EBITDA</x:v>
+      </x:c>
+      <x:c r="E49" s="664"/>
+      <x:c r="F49" s="664"/>
+      <x:c r="G49" s="538"/>
+      <x:c r="H49" s="538"/>
+      <x:c r="I49" s="538"/>
+      <x:c r="J49" s="538"/>
+      <x:c r="K49" s="538"/>
+      <x:c r="L49" s="538"/>
+      <x:c r="M49" s="538"/>
+      <x:c r="N49" s="538"/>
+      <x:c r="O49" s="538"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="715" t="str">
+        <x:v>ROK FY2025 net interest expense</x:v>
+      </x:c>
+      <x:c r="B50" s="744" t="n">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C50" s="436" t="str">
+        <x:v>S-017</x:v>
+      </x:c>
+      <x:c r="D50" s="664" t="str">
+        <x:v>Latest audited annual reference</x:v>
+      </x:c>
+      <x:c r="E50" s="664"/>
+      <x:c r="F50" s="664"/>
+      <x:c r="G50" s="538"/>
+      <x:c r="H50" s="538"/>
+      <x:c r="I50" s="538"/>
+      <x:c r="J50" s="538"/>
+      <x:c r="K50" s="538"/>
+      <x:c r="L50" s="538"/>
+      <x:c r="M50" s="538"/>
+      <x:c r="N50" s="538"/>
+      <x:c r="O50" s="538"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="715" t="str">
+        <x:v>New annual interest expense</x:v>
+      </x:c>
+      <x:c r="B51" s="744" t="n">
+        <x:f>B41*B16</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C51" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D51" s="664" t="str">
+        <x:v>New debt × assumed interest rate</x:v>
+      </x:c>
+      <x:c r="E51" s="664"/>
+      <x:c r="F51" s="664"/>
+      <x:c r="G51" s="538"/>
+      <x:c r="H51" s="538"/>
+      <x:c r="I51" s="538"/>
+      <x:c r="J51" s="538"/>
+      <x:c r="K51" s="538"/>
+      <x:c r="L51" s="538"/>
+      <x:c r="M51" s="538"/>
+      <x:c r="N51" s="538"/>
+      <x:c r="O51" s="538"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="715" t="str">
+        <x:v>Pro forma interest expense</x:v>
+      </x:c>
+      <x:c r="B52" s="744" t="n">
+        <x:f>SUM(B50:B51)</x:f>
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="C52" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="D52" s="664" t="str">
+        <x:v>Existing plus new interest</x:v>
+      </x:c>
+      <x:c r="E52" s="664"/>
+      <x:c r="F52" s="664"/>
+      <x:c r="G52" s="538"/>
+      <x:c r="H52" s="538"/>
+      <x:c r="I52" s="538"/>
+      <x:c r="J52" s="538"/>
+      <x:c r="K52" s="538"/>
+      <x:c r="L52" s="538"/>
+      <x:c r="M52" s="538"/>
+      <x:c r="N52" s="538"/>
+      <x:c r="O52" s="538"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="715" t="str">
+        <x:v>EBITDA / interest coverage</x:v>
+      </x:c>
+      <x:c r="B53" s="748" t="n">
+        <x:f>B47/B52</x:f>
+        <x:v>6.864765143603133</x:v>
+      </x:c>
+      <x:c r="C53" s="436" t="str">
+        <x:v>S-050 covenant reference</x:v>
+      </x:c>
+      <x:c r="D53" s="664" t="str">
+        <x:v>Comfortably exceeds the 3.0x minimum interest-coverage covenant</x:v>
+      </x:c>
+      <x:c r="E53" s="664"/>
+      <x:c r="F53" s="664"/>
+      <x:c r="G53" s="538"/>
+      <x:c r="H53" s="538"/>
+      <x:c r="I53" s="538"/>
+      <x:c r="J53" s="538"/>
+      <x:c r="K53" s="538"/>
+      <x:c r="L53" s="538"/>
+      <x:c r="M53" s="538"/>
+      <x:c r="N53" s="538"/>
+      <x:c r="O53" s="538"/>
+    </x:row>
+    <x:row r="54" ht="18" customHeight="1">
+      <x:c r="A54" s="538"/>
+      <x:c r="B54" s="538"/>
+      <x:c r="C54" s="538"/>
+      <x:c r="D54" s="538"/>
+      <x:c r="E54" s="538"/>
+      <x:c r="F54" s="538"/>
+      <x:c r="G54" s="538"/>
+      <x:c r="H54" s="538"/>
+      <x:c r="I54" s="538"/>
+      <x:c r="J54" s="538"/>
+      <x:c r="K54" s="538"/>
+      <x:c r="L54" s="538"/>
+      <x:c r="M54" s="538"/>
+      <x:c r="N54" s="538"/>
+      <x:c r="O54" s="538"/>
+    </x:row>
+    <x:row r="55" ht="18" customHeight="1">
+      <x:c r="A55" s="713" t="str">
+        <x:v>ANALYST INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="B55" s="713"/>
+      <x:c r="C55" s="713"/>
+      <x:c r="D55" s="713"/>
+      <x:c r="E55" s="713"/>
+      <x:c r="F55" s="713"/>
+      <x:c r="G55" s="713"/>
+      <x:c r="H55" s="713"/>
+      <x:c r="I55" s="713"/>
+      <x:c r="J55" s="713"/>
+      <x:c r="K55" s="713"/>
+      <x:c r="L55" s="713"/>
+      <x:c r="M55" s="713"/>
+      <x:c r="N55" s="713"/>
+      <x:c r="O55" s="713"/>
+    </x:row>
+    <x:row r="56" ht="28" customHeight="1">
+      <x:c r="A56" s="731" t="str">
+        <x:v>A 70% stock consideration mix is intentionally stock-heavy because the $13.5 billion equity purchase price is large relative to Rockwell’s existing balance sheet. Stock preserves liquidity and limits pro forma gross leverage to approximately 2.9x before synergies.</x:v>
+      </x:c>
+      <x:c r="B56" s="731"/>
+      <x:c r="C56" s="731"/>
+      <x:c r="D56" s="731"/>
+      <x:c r="E56" s="731"/>
+      <x:c r="F56" s="731"/>
+      <x:c r="G56" s="731"/>
+      <x:c r="H56" s="731"/>
+      <x:c r="I56" s="731"/>
+      <x:c r="J56" s="731"/>
+      <x:c r="K56" s="731"/>
+      <x:c r="L56" s="731"/>
+      <x:c r="M56" s="731"/>
+      <x:c r="N56" s="731"/>
+      <x:c r="O56" s="731"/>
+    </x:row>
+    <x:row r="57" ht="28" customHeight="1">
+      <x:c r="A57" s="731" t="str">
+        <x:v>The model assumes $4.0 billion of new debt split between a bridge / term loan and senior notes. Target cash is acquired and included in post-close liquidity, but is not treated as a source that funds the purchase at closing.</x:v>
+      </x:c>
+      <x:c r="B57" s="731"/>
+      <x:c r="C57" s="731"/>
+      <x:c r="D57" s="731"/>
+      <x:c r="E57" s="731"/>
+      <x:c r="F57" s="731"/>
+      <x:c r="G57" s="731"/>
+      <x:c r="H57" s="731"/>
+      <x:c r="I57" s="731"/>
+      <x:c r="J57" s="731"/>
+      <x:c r="K57" s="731"/>
+      <x:c r="L57" s="731"/>
+      <x:c r="M57" s="731"/>
+      <x:c r="N57" s="731"/>
+      <x:c r="O57" s="731"/>
+    </x:row>
+    <x:row r="58" ht="28" customHeight="1">
+      <x:c r="A58" s="732" t="str">
+        <x:v>This financing case is preliminary. Purchase accounting and accretion/dilution will test whether the $80 offer remains economically supportable after incremental interest, stock issuance, intangible amortization, and synergies.</x:v>
+      </x:c>
+      <x:c r="B58" s="732"/>
+      <x:c r="C58" s="732"/>
+      <x:c r="D58" s="732"/>
+      <x:c r="E58" s="732"/>
+      <x:c r="F58" s="732"/>
+      <x:c r="G58" s="732"/>
+      <x:c r="H58" s="732"/>
+      <x:c r="I58" s="732"/>
+      <x:c r="J58" s="732"/>
+      <x:c r="K58" s="732"/>
+      <x:c r="L58" s="732"/>
+      <x:c r="M58" s="732"/>
+      <x:c r="N58" s="732"/>
+      <x:c r="O58" s="732"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="B3:O3"/>
+    <x:mergeCell ref="A5:F5"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="E10:F10"/>
+    <x:mergeCell ref="E11:F11"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="E13:F13"/>
+    <x:mergeCell ref="E14:F14"/>
+    <x:mergeCell ref="E15:F15"/>
+    <x:mergeCell ref="E16:F16"/>
+    <x:mergeCell ref="E17:F17"/>
+    <x:mergeCell ref="E18:F18"/>
+    <x:mergeCell ref="H5:O5"/>
+    <x:mergeCell ref="J6:O6"/>
+    <x:mergeCell ref="J7:O7"/>
+    <x:mergeCell ref="J8:O8"/>
+    <x:mergeCell ref="J9:O9"/>
+    <x:mergeCell ref="J10:O10"/>
+    <x:mergeCell ref="J11:O11"/>
+    <x:mergeCell ref="J12:O12"/>
+    <x:mergeCell ref="H14:O14"/>
+    <x:mergeCell ref="J15:O15"/>
+    <x:mergeCell ref="J16:O16"/>
+    <x:mergeCell ref="J17:O17"/>
+    <x:mergeCell ref="J18:O18"/>
+    <x:mergeCell ref="A20:F20"/>
+    <x:mergeCell ref="H20:M20"/>
+    <x:mergeCell ref="C21:F21"/>
+    <x:mergeCell ref="C22:F22"/>
+    <x:mergeCell ref="C23:F23"/>
+    <x:mergeCell ref="C24:F24"/>
+    <x:mergeCell ref="C25:F25"/>
+    <x:mergeCell ref="C26:F26"/>
+    <x:mergeCell ref="J21:M21"/>
+    <x:mergeCell ref="J22:M22"/>
+    <x:mergeCell ref="J23:M23"/>
+    <x:mergeCell ref="J24:M24"/>
+    <x:mergeCell ref="J25:M25"/>
+    <x:mergeCell ref="J26:M26"/>
+    <x:mergeCell ref="J28:M28"/>
+    <x:mergeCell ref="A30:F30"/>
+    <x:mergeCell ref="D31:F31"/>
+    <x:mergeCell ref="D32:F32"/>
+    <x:mergeCell ref="D33:F33"/>
+    <x:mergeCell ref="D34:F34"/>
+    <x:mergeCell ref="D35:F35"/>
+    <x:mergeCell ref="D36:F36"/>
+    <x:mergeCell ref="D37:F37"/>
+    <x:mergeCell ref="D38:F38"/>
+    <x:mergeCell ref="D39:F39"/>
+    <x:mergeCell ref="D40:F40"/>
+    <x:mergeCell ref="D41:F41"/>
+    <x:mergeCell ref="D42:F42"/>
+    <x:mergeCell ref="D43:F43"/>
+    <x:mergeCell ref="D44:F44"/>
+    <x:mergeCell ref="D45:F45"/>
+    <x:mergeCell ref="D46:F46"/>
+    <x:mergeCell ref="D47:F47"/>
+    <x:mergeCell ref="D48:F48"/>
+    <x:mergeCell ref="D49:F49"/>
+    <x:mergeCell ref="D50:F50"/>
+    <x:mergeCell ref="D51:F51"/>
+    <x:mergeCell ref="D52:F52"/>
+    <x:mergeCell ref="D53:F53"/>
+    <x:mergeCell ref="H30:O30"/>
+    <x:mergeCell ref="J31:O31"/>
+    <x:mergeCell ref="J32:O32"/>
+    <x:mergeCell ref="J33:O33"/>
+    <x:mergeCell ref="J34:O34"/>
+    <x:mergeCell ref="J35:O35"/>
+    <x:mergeCell ref="J36:O36"/>
+    <x:mergeCell ref="J37:O37"/>
+    <x:mergeCell ref="J38:O38"/>
+    <x:mergeCell ref="J39:O39"/>
+    <x:mergeCell ref="J40:O40"/>
+    <x:mergeCell ref="J41:O41"/>
+    <x:mergeCell ref="J42:O42"/>
+    <x:mergeCell ref="J43:O43"/>
+    <x:mergeCell ref="J44:O44"/>
+    <x:mergeCell ref="J45:O45"/>
+    <x:mergeCell ref="A55:O55"/>
+    <x:mergeCell ref="A56:O56"/>
+    <x:mergeCell ref="A57:O57"/>
+    <x:mergeCell ref="A58:O58"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -8041,8 +9843,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="703" t="str">
-        <x:v>VALUATION COMPLETE</x:v>
+      <x:c r="B3" s="767" t="str">
+        <x:v>FINANCING COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -8088,10 +9890,10 @@
       </x:c>
       <x:c r="B6" s="134" t="n">
         <x:f>COUNTA('Sources'!A4:A100)</x:f>
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C6" s="135" t="n">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D6" s="135" t="n">
         <x:f>B6-C6</x:f>
@@ -8756,6 +10558,162 @@
       </x:c>
       <x:c r="G31" s="484" t="str">
         <x:v>Valuation Summary rows 6 and 8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="484" t="str">
+        <x:v>Sources and uses balance</x:v>
+      </x:c>
+      <x:c r="B32" s="484" t="n">
+        <x:f>'Sources &amp; Uses'!I28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C32" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D32" s="484" t="n">
+        <x:f>B32-C32</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F32" s="769" t="str">
+        <x:f>IF(ABS(D32)&lt;=E32,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G32" s="484" t="str">
+        <x:v>Sources &amp; Uses row 28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="484" t="str">
+        <x:v>Consideration mix totals 100%</x:v>
+      </x:c>
+      <x:c r="B33" s="484" t="n">
+        <x:f>'Sources &amp; Uses'!B10+'Sources &amp; Uses'!B11</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C33" s="484" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D33" s="484" t="n">
+        <x:f>B33-C33</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="484" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F33" s="769" t="str">
+        <x:f>IF(ABS(D33)&lt;=E33,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G33" s="484" t="str">
+        <x:v>Sources &amp; Uses rows 10-11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="484" t="str">
+        <x:v>Purchase price bridge</x:v>
+      </x:c>
+      <x:c r="B34" s="484" t="n">
+        <x:f>ABS('Sources &amp; Uses'!I6-'Valuation Summary'!F6)+ABS('Sources &amp; Uses'!I9-'Valuation Summary'!F7)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C34" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D34" s="484" t="n">
+        <x:f>B34-C34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F34" s="769" t="str">
+        <x:f>IF(ABS(D34)&lt;=E34,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G34" s="484" t="str">
+        <x:v>Sources &amp; Uses rows 6-9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="484" t="str">
+        <x:v>Cash balance above minimum</x:v>
+      </x:c>
+      <x:c r="B35" s="484" t="n">
+        <x:f>'Sources &amp; Uses'!B33-'Sources &amp; Uses'!I44</x:f>
+        <x:v>111.04479999999967</x:v>
+      </x:c>
+      <x:c r="C35" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D35" s="484" t="n">
+        <x:f>MIN(0,B35-C35)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="769" t="str">
+        <x:f>IF(ABS(D35)&lt;=E35,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G35" s="484" t="str">
+        <x:v>Sources &amp; Uses rows 33 and 44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="484" t="str">
+        <x:v>Gross leverage below ceiling</x:v>
+      </x:c>
+      <x:c r="B36" s="484" t="n">
+        <x:f>'Sources &amp; Uses'!I39-'Sources &amp; Uses'!B48</x:f>
+        <x:v>0.07478121571385232</x:v>
+      </x:c>
+      <x:c r="C36" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D36" s="484" t="n">
+        <x:f>MIN(0,B36-C36)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F36" s="769" t="str">
+        <x:f>IF(ABS(D36)&lt;=E36,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G36" s="484" t="str">
+        <x:v>Sources &amp; Uses rows 48 and 39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="484" t="str">
+        <x:v>Stock issuance bridge</x:v>
+      </x:c>
+      <x:c r="B37" s="484" t="n">
+        <x:f>ABS('Sources &amp; Uses'!I33*'Sources &amp; Uses'!I32-'Sources &amp; Uses'!B22)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C37" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D37" s="484" t="n">
+        <x:f>B37-C37</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E37" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F37" s="769" t="str">
+        <x:f>IF(ABS(D37)&lt;=E37,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G37" s="484" t="str">
+        <x:v>Sources &amp; Uses rows 22 and 33</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8900,12 +10858,14 @@
       <x:c r="A10" t="str">
         <x:v>Transaction close date</x:v>
       </x:c>
-      <x:c r="B10" s="35"/>
+      <x:c r="B10" s="757" t="n">
+        <x:v>46477</x:v>
+      </x:c>
       <x:c r="C10" t="str">
-        <x:v>Required later</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Set during transaction analysis</x:v>
+        <x:v>Illustrative close after regulatory and shareholder approvals</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -8920,48 +10880,59 @@
       <x:c r="A13" t="str">
         <x:v>Offer price per share</x:v>
       </x:c>
-      <x:c r="B13" s="36"/>
+      <x:c r="B13" s="762" t="n">
+        <x:f>'Valuation Summary'!B9</x:f>
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="C13" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>Derived after standalone valuation</x:v>
+        <x:v>Valuation Summary midpoint</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
         <x:v>Offer premium</x:v>
       </x:c>
-      <x:c r="B14" s="37"/>
+      <x:c r="B14" s="763" t="n">
+        <x:f>'Valuation Summary'!B10</x:f>
+        <x:v>0.3393604553825549</x:v>
+      </x:c>
       <x:c r="C14" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>Calculated against unaffected price</x:v>
+        <x:v>Calculated versus unaffected price</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
         <x:v>Cash consideration %</x:v>
       </x:c>
-      <x:c r="B15" s="37"/>
+      <x:c r="B15" s="764" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
       <x:c r="C15" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>Optimized in transaction model</x:v>
+        <x:v>Selected financing case</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
         <x:v>Stock consideration %</x:v>
       </x:c>
-      <x:c r="B16" s="37"/>
+      <x:c r="B16" s="765" t="n">
+        <x:f>1-B15</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
       <x:c r="C16" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>Optimized in transaction model</x:v>
+        <x:v>Balances consideration mix</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -10799,6 +12770,84 @@
         <x:v>Primary company release furnished to SEC</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="32" customHeight="1">
+      <x:c r="A32" s="480" t="str">
+        <x:v>S-018</x:v>
+      </x:c>
+      <x:c r="B32" s="480" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C32" s="480" t="str">
+        <x:v>Fiscal third-quarter 2026 results</x:v>
+      </x:c>
+      <x:c r="D32" s="481" t="n">
+        <x:v>46238</x:v>
+      </x:c>
+      <x:c r="E32" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F32" s="480" t="str">
+        <x:v>FY2026 buyer guidance and current operating momentum</x:v>
+      </x:c>
+      <x:c r="G32" s="480" t="str">
+        <x:v>https://www.rockwellautomation.com/en-se/company/news/press-releases/Rockwell-Automation-Reports-Third-Quarter-2026-Results.html</x:v>
+      </x:c>
+      <x:c r="H32" s="480" t="str">
+        <x:v>Primary company release</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="32" customHeight="1">
+      <x:c r="A33" s="480" t="str">
+        <x:v>S-050</x:v>
+      </x:c>
+      <x:c r="B33" s="480" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C33" s="480" t="str">
+        <x:v>Q2 FY2026 Form 10-Q</x:v>
+      </x:c>
+      <x:c r="D33" s="481" t="n">
+        <x:v>46147</x:v>
+      </x:c>
+      <x:c r="E33" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F33" s="480" t="str">
+        <x:v>Cash, funded debt, revolver capacity, and interest-coverage covenant</x:v>
+      </x:c>
+      <x:c r="G33" s="480" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1024478/000102447826000022/rok-20260331.htm</x:v>
+      </x:c>
+      <x:c r="H33" s="480" t="str">
+        <x:v>Primary SEC filing; latest full balance sheet used</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="32" customHeight="1">
+      <x:c r="A34" s="480" t="str">
+        <x:v>S-051</x:v>
+      </x:c>
+      <x:c r="B34" s="480" t="str">
+        <x:v>Rockwell Automation</x:v>
+      </x:c>
+      <x:c r="C34" s="480" t="str">
+        <x:v>Historical stock price</x:v>
+      </x:c>
+      <x:c r="D34" s="481" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="E34" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F34" s="480" t="str">
+        <x:v>Buyer share price for stock consideration and new-share issuance</x:v>
+      </x:c>
+      <x:c r="G34" s="480" t="str">
+        <x:v>https://stockanalysis.com/stocks/rok/history/</x:v>
+      </x:c>
+      <x:c r="H34" s="480" t="str">
+        <x:v>$431.45 closing price on Aug. 20, 2026</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -12207,7 +14256,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b8f520df1b4c56"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55562b56411e471b"/>
 </x:worksheet>
 </file>
 
@@ -13930,7 +15979,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc00c44d81f14a8f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bd467dd805d46b7"/>
 </x:worksheet>
 </file>
 
@@ -17417,7 +19466,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4442a8d220a34658"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d488bec88704475"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
transaction: complete purchase accounting
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9f76b875fb9b4ed1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Race26722ee364e77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rceffdc1228a149ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R5086969ebcbd4bb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R74509b1304f741f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rdce5d24f4a8341b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Rb6ce4dc29e3a4ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R73746c7f18844d41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R964711bf78954e10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R3655ee02dd3b4a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R6be7431042704ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rf181f41f6dfd41e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R61c40aa9b1a04285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R1d180f90671c4ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R2887959b1a14403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rf391f8a751ab48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R7a004861e7f64801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R07f9548a994643c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R44460d68c93e490a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rec640185d77c4208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R07661846d8ed4df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R419c26e5b0154ce8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rdb119bb981434ae3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R23b603b9622f4548"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R154d2866cbed409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R1c564d5a7fbf4455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Re8112b4112694336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Ra83a35549ac94976"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R49e21e59c38e4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R27ab496476a04455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R4739deba96b24abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R18272b9c01834493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R5c9e50199c864f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Rb4ae5e17e35b4ac0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="24">
+  <x:numFmts count="25">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -180,6 +180,7 @@
     <x:numFmt numFmtId="221" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="222" formatCode=";;;"/>
     <x:numFmt numFmtId="223" formatCode="$0"/>
+    <x:numFmt numFmtId="224" formatCode="yyyy&quot;E&quot;"/>
   </x:numFmts>
   <x:fonts count="45">
     <x:font>
@@ -436,7 +437,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="54">
+  <x:fills count="61">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -666,6 +667,41 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF8F8F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -974,7 +1010,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="770">
+  <x:cellXfs count="815">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2581,6 +2617,133 @@
     <x:xf numFmtId="0" fontId="26" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="40" fillId="49" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="58" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="58" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="59" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="55" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="55" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="58" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="60" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="60" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="56" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="59" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="60" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="37" fillId="59" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="37" fillId="59" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="42" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="41" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="41" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="37" fillId="59" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="41" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="41" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="224" fontId="41" fillId="60" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="38" fillId="55" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="56" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="19" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="59" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="55" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="57" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3060,7 +3223,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.7 — financing complete</x:v>
+        <x:v>0.8 — purchase accounting complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -3115,8 +3278,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="766" t="str">
-        <x:v>FINANCING COMPLETE</x:v>
+      <x:c r="B9" s="811" t="str">
+        <x:v>PURCHASE ACCOUNTING COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -9358,110 +9521,1659 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="771" t="str">
         <x:v>Purchase Accounting</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Goodwill, intangible assets, amortization, and tax effects</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="B1" s="771"/>
+      <x:c r="C1" s="771"/>
+      <x:c r="D1" s="771"/>
+      <x:c r="E1" s="771"/>
+      <x:c r="F1" s="771"/>
+      <x:c r="G1" s="771"/>
+      <x:c r="H1" s="771"/>
+      <x:c r="I1" s="771"/>
+      <x:c r="J1" s="771"/>
+      <x:c r="K1" s="771"/>
+      <x:c r="L1" s="771"/>
+      <x:c r="M1" s="771"/>
+      <x:c r="N1" s="771"/>
+      <x:c r="O1" s="771"/>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="773" t="str">
+        <x:v>Illustrative purchase-price allocation, new goodwill, deferred taxes, and incremental non-cash expense | USD millions</x:v>
+      </x:c>
+      <x:c r="B2" s="773"/>
+      <x:c r="C2" s="773"/>
+      <x:c r="D2" s="773"/>
+      <x:c r="E2" s="773"/>
+      <x:c r="F2" s="773"/>
+      <x:c r="G2" s="773"/>
+      <x:c r="H2" s="773"/>
+      <x:c r="I2" s="773"/>
+      <x:c r="J2" s="773"/>
+      <x:c r="K2" s="773"/>
+      <x:c r="L2" s="773"/>
+      <x:c r="M2" s="773"/>
+      <x:c r="N2" s="773"/>
+      <x:c r="O2" s="773"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="432" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="775" t="str">
+        <x:v>Complete — preliminary allocation for merger-model purposes; third-party valuation work would be required at closing</x:v>
+      </x:c>
+      <x:c r="C3" s="775"/>
+      <x:c r="D3" s="775"/>
+      <x:c r="E3" s="775"/>
+      <x:c r="F3" s="775"/>
+      <x:c r="G3" s="775"/>
+      <x:c r="H3" s="775"/>
+      <x:c r="I3" s="775"/>
+      <x:c r="J3" s="775"/>
+      <x:c r="K3" s="775"/>
+      <x:c r="L3" s="775"/>
+      <x:c r="M3" s="775"/>
+      <x:c r="N3" s="775"/>
+      <x:c r="O3" s="775"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="538"/>
+      <x:c r="B4" s="538"/>
+      <x:c r="C4" s="538"/>
+      <x:c r="D4" s="538"/>
+      <x:c r="E4" s="538"/>
+      <x:c r="F4" s="538"/>
+      <x:c r="G4" s="538"/>
+      <x:c r="H4" s="538"/>
+      <x:c r="I4" s="538"/>
+      <x:c r="J4" s="538"/>
+      <x:c r="K4" s="538"/>
+      <x:c r="L4" s="538"/>
+      <x:c r="M4" s="538"/>
+      <x:c r="N4" s="538"/>
+      <x:c r="O4" s="538"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="777" t="str">
+        <x:v>PURCHASE ACCOUNTING INPUTS</x:v>
+      </x:c>
+      <x:c r="B5" s="777"/>
+      <x:c r="C5" s="777"/>
+      <x:c r="D5" s="777"/>
+      <x:c r="E5" s="777"/>
+      <x:c r="F5" s="777"/>
+      <x:c r="G5" s="538"/>
+      <x:c r="H5" s="777" t="str">
+        <x:v>PURCHASE-PRICE ALLOCATION BRIDGE</x:v>
+      </x:c>
+      <x:c r="I5" s="777"/>
+      <x:c r="J5" s="777"/>
+      <x:c r="K5" s="777"/>
+      <x:c r="L5" s="777"/>
+      <x:c r="M5" s="777"/>
+      <x:c r="N5" s="777"/>
+      <x:c r="O5" s="777"/>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="779" t="str">
+        <x:v>Purchase consideration</x:v>
+      </x:c>
+      <x:c r="B6" s="794" t="n">
+        <x:f>'Sources &amp; Uses'!I6</x:f>
+        <x:v>13457.919999999998</x:v>
+      </x:c>
+      <x:c r="C6" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D6" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E6" s="664" t="str">
+        <x:v>Equity value transferred to Cognex shareholders; transaction fees are expensed separately</x:v>
+      </x:c>
+      <x:c r="F6" s="664"/>
+      <x:c r="G6" s="538"/>
+      <x:c r="H6" s="779" t="str">
+        <x:v>Purchase consideration</x:v>
+      </x:c>
+      <x:c r="I6" s="794" t="n">
+        <x:f>B6</x:f>
+        <x:v>13457.919999999998</x:v>
+      </x:c>
+      <x:c r="J6" s="664" t="str">
+        <x:v>Cash and stock consideration paid for Cognex equity</x:v>
+      </x:c>
+      <x:c r="K6" s="664"/>
+      <x:c r="L6" s="664"/>
+      <x:c r="M6" s="664"/>
+      <x:c r="N6" s="664"/>
+      <x:c r="O6" s="664"/>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="779" t="str">
+        <x:v>Target shareholders’ equity</x:v>
+      </x:c>
+      <x:c r="B7" s="744" t="n">
+        <x:v>1629.555</x:v>
+      </x:c>
+      <x:c r="C7" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D7" s="436" t="str">
+        <x:v>S-052</x:v>
+      </x:c>
+      <x:c r="E7" s="664" t="str">
+        <x:v>Unaudited July 5, 2026 balance-sheet carrying value</x:v>
+      </x:c>
+      <x:c r="F7" s="664"/>
+      <x:c r="G7" s="538"/>
+      <x:c r="H7" s="779" t="str">
+        <x:v>Tangible book value</x:v>
+      </x:c>
+      <x:c r="I7" s="744" t="n">
+        <x:f>B10</x:f>
+        <x:v>1183.7060000000001</x:v>
+      </x:c>
+      <x:c r="J7" s="664" t="str">
+        <x:v>Target book equity excluding historical goodwill and intangibles</x:v>
+      </x:c>
+      <x:c r="K7" s="664"/>
+      <x:c r="L7" s="664"/>
+      <x:c r="M7" s="664"/>
+      <x:c r="N7" s="664"/>
+      <x:c r="O7" s="664"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="779" t="str">
+        <x:v>Less: existing goodwill</x:v>
+      </x:c>
+      <x:c r="B8" s="744" t="n">
+        <x:v>381.385</x:v>
+      </x:c>
+      <x:c r="C8" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D8" s="436" t="str">
+        <x:v>S-052</x:v>
+      </x:c>
+      <x:c r="E8" s="664" t="str">
+        <x:v>Historical acquisition goodwill is removed before establishing new acquisition goodwill</x:v>
+      </x:c>
+      <x:c r="F8" s="664"/>
+      <x:c r="G8" s="538"/>
+      <x:c r="H8" s="779" t="str">
+        <x:v>Customer-related intangibles</x:v>
+      </x:c>
+      <x:c r="I8" s="744" t="n">
+        <x:f>C18</x:f>
+        <x:v>2960.7423999999996</x:v>
+      </x:c>
+      <x:c r="J8" s="664" t="str">
+        <x:v>Fair value of customer relationships</x:v>
+      </x:c>
+      <x:c r="K8" s="664"/>
+      <x:c r="L8" s="664"/>
+      <x:c r="M8" s="664"/>
+      <x:c r="N8" s="664"/>
+      <x:c r="O8" s="664"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="779" t="str">
+        <x:v>Less: existing intangible assets</x:v>
+      </x:c>
+      <x:c r="B9" s="744" t="n">
+        <x:v>64.464</x:v>
+      </x:c>
+      <x:c r="C9" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D9" s="436" t="str">
+        <x:v>S-052</x:v>
+      </x:c>
+      <x:c r="E9" s="664" t="str">
+        <x:v>Historical finite-lived intangibles are replaced by the new fair-value allocation</x:v>
+      </x:c>
+      <x:c r="F9" s="664"/>
+      <x:c r="G9" s="538"/>
+      <x:c r="H9" s="779" t="str">
+        <x:v>Technology-related intangibles</x:v>
+      </x:c>
+      <x:c r="I9" s="744" t="n">
+        <x:f>C19</x:f>
+        <x:v>1614.9503999999997</x:v>
+      </x:c>
+      <x:c r="J9" s="664" t="str">
+        <x:v>Fair value of developed technology</x:v>
+      </x:c>
+      <x:c r="K9" s="664"/>
+      <x:c r="L9" s="664"/>
+      <x:c r="M9" s="664"/>
+      <x:c r="N9" s="664"/>
+      <x:c r="O9" s="664"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="779" t="str">
+        <x:v>Tangible book value</x:v>
+      </x:c>
+      <x:c r="B10" s="744" t="n">
+        <x:f>B7-B8-B9</x:f>
+        <x:v>1183.7060000000001</x:v>
+      </x:c>
+      <x:c r="C10" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D10" s="436" t="str">
+        <x:v>Calculated</x:v>
+      </x:c>
+      <x:c r="E10" s="664" t="str">
+        <x:v>Book equity less existing goodwill and intangibles</x:v>
+      </x:c>
+      <x:c r="F10" s="664"/>
+      <x:c r="G10" s="538"/>
+      <x:c r="H10" s="779" t="str">
+        <x:v>Trade names</x:v>
+      </x:c>
+      <x:c r="I10" s="744" t="n">
+        <x:f>C20</x:f>
+        <x:v>403.73759999999993</x:v>
+      </x:c>
+      <x:c r="J10" s="664" t="str">
+        <x:v>Fair value of trade names</x:v>
+      </x:c>
+      <x:c r="K10" s="664"/>
+      <x:c r="L10" s="664"/>
+      <x:c r="M10" s="664"/>
+      <x:c r="N10" s="664"/>
+      <x:c r="O10" s="664"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="779" t="str">
+        <x:v>Tax rate</x:v>
+      </x:c>
+      <x:c r="B11" s="795" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="C11" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D11" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E11" s="664" t="str">
+        <x:v>Illustrative statutory tax rate applied to fair-value step-ups</x:v>
+      </x:c>
+      <x:c r="F11" s="664"/>
+      <x:c r="G11" s="538"/>
+      <x:c r="H11" s="779" t="str">
+        <x:v>Order backlog</x:v>
+      </x:c>
+      <x:c r="I11" s="744" t="n">
+        <x:f>C21</x:f>
+        <x:v>134.5792</x:v>
+      </x:c>
+      <x:c r="J11" s="664" t="str">
+        <x:v>Fair value of acquired backlog</x:v>
+      </x:c>
+      <x:c r="K11" s="664"/>
+      <x:c r="L11" s="664"/>
+      <x:c r="M11" s="664"/>
+      <x:c r="N11" s="664"/>
+      <x:c r="O11" s="664"/>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="779" t="str">
+        <x:v>Months per year</x:v>
+      </x:c>
+      <x:c r="B12" s="796" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C12" s="436" t="str">
+        <x:v>months</x:v>
+      </x:c>
+      <x:c r="D12" s="436" t="str">
+        <x:v>Model convention</x:v>
+      </x:c>
+      <x:c r="E12" s="664" t="str">
+        <x:v>Used to calculate straight-line expense by ownership period</x:v>
+      </x:c>
+      <x:c r="F12" s="664"/>
+      <x:c r="G12" s="538"/>
+      <x:c r="H12" s="779" t="str">
+        <x:v>Inventory step-up</x:v>
+      </x:c>
+      <x:c r="I12" s="744" t="n">
+        <x:f>C22</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="J12" s="664" t="str">
+        <x:v>Temporary fair-value uplift to inventory</x:v>
+      </x:c>
+      <x:c r="K12" s="664"/>
+      <x:c r="L12" s="664"/>
+      <x:c r="M12" s="664"/>
+      <x:c r="N12" s="664"/>
+      <x:c r="O12" s="664"/>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="779" t="str">
+        <x:v>First fiscal-year ownership</x:v>
+      </x:c>
+      <x:c r="B13" s="796" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C13" s="436" t="str">
+        <x:v>months</x:v>
+      </x:c>
+      <x:c r="D13" s="436" t="str">
+        <x:v>Analyst convention</x:v>
+      </x:c>
+      <x:c r="E13" s="664" t="str">
+        <x:v>Six months from the March 31 close to Rockwell’s September 30 fiscal year-end</x:v>
+      </x:c>
+      <x:c r="F13" s="664"/>
+      <x:c r="G13" s="538"/>
+      <x:c r="H13" s="779" t="str">
+        <x:v>PP&amp;E step-up</x:v>
+      </x:c>
+      <x:c r="I13" s="744" t="n">
+        <x:f>C23</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="J13" s="664" t="str">
+        <x:v>Fair-value uplift to property and equipment</x:v>
+      </x:c>
+      <x:c r="K13" s="664"/>
+      <x:c r="L13" s="664"/>
+      <x:c r="M13" s="664"/>
+      <x:c r="N13" s="664"/>
+      <x:c r="O13" s="664"/>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="779" t="str">
+        <x:v>Illustrative close date</x:v>
+      </x:c>
+      <x:c r="B14" s="797" t="n">
+        <x:f>'Sources &amp; Uses'!B18</x:f>
+        <x:v>46477</x:v>
+      </x:c>
+      <x:c r="C14" s="436" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="D14" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E14" s="664" t="str">
+        <x:v>Links to the financing schedule</x:v>
+      </x:c>
+      <x:c r="F14" s="664"/>
+      <x:c r="G14" s="538"/>
+      <x:c r="H14" s="779" t="str">
+        <x:v>Gross fair-value write-ups</x:v>
+      </x:c>
+      <x:c r="I14" s="744" t="n">
+        <x:f>SUM(I8:I13)</x:f>
+        <x:v>5248.5887999999995</x:v>
+      </x:c>
+      <x:c r="J14" s="664" t="str">
+        <x:v>Total identifiable asset write-ups</x:v>
+      </x:c>
+      <x:c r="K14" s="664"/>
+      <x:c r="L14" s="664"/>
+      <x:c r="M14" s="664"/>
+      <x:c r="N14" s="664"/>
+      <x:c r="O14" s="664"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="538"/>
+      <x:c r="B15" s="538"/>
+      <x:c r="C15" s="538"/>
+      <x:c r="D15" s="538"/>
+      <x:c r="E15" s="538"/>
+      <x:c r="F15" s="538"/>
+      <x:c r="G15" s="538"/>
+      <x:c r="H15" s="779" t="str">
+        <x:v>Incremental deferred tax liability</x:v>
+      </x:c>
+      <x:c r="I15" s="744" t="n">
+        <x:f>I14*$B$11</x:f>
+        <x:v>1102.203648</x:v>
+      </x:c>
+      <x:c r="J15" s="664" t="str">
+        <x:v>Assumes tax basis does not step up; increases goodwill</x:v>
+      </x:c>
+      <x:c r="K15" s="664"/>
+      <x:c r="L15" s="664"/>
+      <x:c r="M15" s="664"/>
+      <x:c r="N15" s="664"/>
+      <x:c r="O15" s="664"/>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="777" t="str">
+        <x:v>FAIR-VALUE ALLOCATION ASSUMPTIONS</x:v>
+      </x:c>
+      <x:c r="B16" s="777"/>
+      <x:c r="C16" s="777"/>
+      <x:c r="D16" s="777"/>
+      <x:c r="E16" s="777"/>
+      <x:c r="F16" s="777"/>
+      <x:c r="G16" s="538"/>
+      <x:c r="H16" s="779" t="str">
+        <x:v>Net identifiable assets</x:v>
+      </x:c>
+      <x:c r="I16" s="744" t="n">
+        <x:f>I7+I14-I15</x:f>
+        <x:v>5330.091152</x:v>
+      </x:c>
+      <x:c r="J16" s="664" t="str">
+        <x:v>Tangible book value plus write-ups less deferred tax liability</x:v>
+      </x:c>
+      <x:c r="K16" s="664"/>
+      <x:c r="L16" s="664"/>
+      <x:c r="M16" s="664"/>
+      <x:c r="N16" s="664"/>
+      <x:c r="O16" s="664"/>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="782" t="str">
+        <x:v>Asset</x:v>
+      </x:c>
+      <x:c r="B17" s="782" t="str">
+        <x:v>% of consideration</x:v>
+      </x:c>
+      <x:c r="C17" s="782" t="str">
+        <x:v>Fair value</x:v>
+      </x:c>
+      <x:c r="D17" s="782" t="str">
+        <x:v>Useful life</x:v>
+      </x:c>
+      <x:c r="E17" s="782" t="str">
+        <x:v>Annual expense</x:v>
+      </x:c>
+      <x:c r="F17" s="809" t="str">
+        <x:v>Rationale</x:v>
+      </x:c>
+      <x:c r="G17" s="538"/>
+      <x:c r="H17" s="779" t="str">
+        <x:v>New goodwill</x:v>
+      </x:c>
+      <x:c r="I17" s="801" t="n">
+        <x:f>I6-I16</x:f>
+        <x:v>8127.828847999998</x:v>
+      </x:c>
+      <x:c r="J17" s="664" t="str">
+        <x:v>Residual consideration not assigned to identifiable net assets</x:v>
+      </x:c>
+      <x:c r="K17" s="664"/>
+      <x:c r="L17" s="664"/>
+      <x:c r="M17" s="664"/>
+      <x:c r="N17" s="664"/>
+      <x:c r="O17" s="664"/>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="779" t="str">
+        <x:v>Customer relationships</x:v>
+      </x:c>
+      <x:c r="B18" s="795" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="C18" s="744" t="n">
+        <x:f>$B$6*B18</x:f>
+        <x:v>2960.7423999999996</x:v>
+      </x:c>
+      <x:c r="D18" s="800" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E18" s="744" t="n">
+        <x:f>C18/D18</x:f>
+        <x:v>197.38282666666663</x:v>
+      </x:c>
+      <x:c r="F18" s="664" t="str">
+        <x:v>Recurring installed-base relationships and channel access</x:v>
+      </x:c>
+      <x:c r="G18" s="538"/>
+      <x:c r="H18" s="779" t="str">
+        <x:v>Goodwill / consideration</x:v>
+      </x:c>
+      <x:c r="I18" s="802" t="n">
+        <x:f>I17/I6</x:f>
+        <x:v>0.6039439116891763</x:v>
+      </x:c>
+      <x:c r="J18" s="664" t="str">
+        <x:v>High goodwill share reflects strategic value and the elevated offer multiple</x:v>
+      </x:c>
+      <x:c r="K18" s="664"/>
+      <x:c r="L18" s="664"/>
+      <x:c r="M18" s="664"/>
+      <x:c r="N18" s="664"/>
+      <x:c r="O18" s="664"/>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="779" t="str">
+        <x:v>Developed technology</x:v>
+      </x:c>
+      <x:c r="B19" s="795" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="C19" s="744" t="n">
+        <x:f>$B$6*B19</x:f>
+        <x:v>1614.9503999999997</x:v>
+      </x:c>
+      <x:c r="D19" s="800" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E19" s="744" t="n">
+        <x:f>C19/D19</x:f>
+        <x:v>230.70719999999997</x:v>
+      </x:c>
+      <x:c r="F19" s="664" t="str">
+        <x:v>Machine-vision software, algorithms, and product technology</x:v>
+      </x:c>
+      <x:c r="G19" s="538"/>
+      <x:c r="H19" s="538"/>
+      <x:c r="I19" s="538"/>
+      <x:c r="J19" s="554"/>
+      <x:c r="K19" s="554"/>
+      <x:c r="L19" s="554"/>
+      <x:c r="M19" s="554"/>
+      <x:c r="N19" s="554"/>
+      <x:c r="O19" s="554"/>
+    </x:row>
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="779" t="str">
+        <x:v>Trade names</x:v>
+      </x:c>
+      <x:c r="B20" s="795" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="C20" s="744" t="n">
+        <x:f>$B$6*B20</x:f>
+        <x:v>403.73759999999993</x:v>
+      </x:c>
+      <x:c r="D20" s="800" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E20" s="744" t="n">
+        <x:f>C20/D20</x:f>
+        <x:v>26.915839999999996</x:v>
+      </x:c>
+      <x:c r="F20" s="664" t="str">
+        <x:v>Cognex brand and product-family names</x:v>
+      </x:c>
+      <x:c r="G20" s="538"/>
+      <x:c r="H20" s="777" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I20" s="777"/>
+      <x:c r="J20" s="810"/>
+      <x:c r="K20" s="810"/>
+      <x:c r="L20" s="810"/>
+      <x:c r="M20" s="810"/>
+      <x:c r="N20" s="810"/>
+      <x:c r="O20" s="810"/>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="779" t="str">
+        <x:v>Order backlog</x:v>
+      </x:c>
+      <x:c r="B21" s="795" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C21" s="744" t="n">
+        <x:f>$B$6*B21</x:f>
+        <x:v>134.5792</x:v>
+      </x:c>
+      <x:c r="D21" s="800" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E21" s="744" t="n">
+        <x:f>C21/D21</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="F21" s="664" t="str">
+        <x:v>Existing contracted or expected customer orders</x:v>
+      </x:c>
+      <x:c r="G21" s="538"/>
+      <x:c r="H21" s="779" t="str">
+        <x:v>New goodwill</x:v>
+      </x:c>
+      <x:c r="I21" s="801" t="n">
+        <x:f>I17</x:f>
+        <x:v>8127.828847999998</x:v>
+      </x:c>
+      <x:c r="J21" s="664" t="str">
+        <x:v>Not amortized; tested for impairment</x:v>
+      </x:c>
+      <x:c r="K21" s="664"/>
+      <x:c r="L21" s="664"/>
+      <x:c r="M21" s="664"/>
+      <x:c r="N21" s="664"/>
+      <x:c r="O21" s="664"/>
+    </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="779" t="str">
+        <x:v>Inventory step-up</x:v>
+      </x:c>
+      <x:c r="B22" s="795" t="n">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="C22" s="744" t="n">
+        <x:f>$B$6*B22</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="D22" s="800" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="744" t="n">
+        <x:f>C22/D22</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="F22" s="664" t="str">
+        <x:v>Fair-value uplift recognized through cost of sales</x:v>
+      </x:c>
+      <x:c r="G22" s="538"/>
+      <x:c r="H22" s="779" t="str">
+        <x:v>Total identifiable intangibles</x:v>
+      </x:c>
+      <x:c r="I22" s="801" t="n">
+        <x:f>SUM(C18:C21)</x:f>
+        <x:v>5114.009599999999</x:v>
+      </x:c>
+      <x:c r="J22" s="664" t="str">
+        <x:v>Finite-lived customer, technology, trade-name, and backlog assets</x:v>
+      </x:c>
+      <x:c r="K22" s="664"/>
+      <x:c r="L22" s="664"/>
+      <x:c r="M22" s="664"/>
+      <x:c r="N22" s="664"/>
+      <x:c r="O22" s="664"/>
+    </x:row>
+    <x:row r="23" ht="24" customHeight="1">
+      <x:c r="A23" s="779" t="str">
+        <x:v>PP&amp;E step-up</x:v>
+      </x:c>
+      <x:c r="B23" s="795" t="n">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="C23" s="744" t="n">
+        <x:f>$B$6*B23</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="D23" s="800" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E23" s="744" t="n">
+        <x:f>C23/D23</x:f>
+        <x:v>6.728959999999999</x:v>
+      </x:c>
+      <x:c r="F23" s="664" t="str">
+        <x:v>Fair-value uplift recognized through depreciation</x:v>
+      </x:c>
+      <x:c r="G23" s="538"/>
+      <x:c r="H23" s="779" t="str">
+        <x:v>Initial deferred tax liability</x:v>
+      </x:c>
+      <x:c r="I23" s="801" t="n">
+        <x:f>I15</x:f>
+        <x:v>1102.203648</x:v>
+      </x:c>
+      <x:c r="J23" s="664" t="str">
+        <x:v>Reverses as the associated book-basis assets are expensed</x:v>
+      </x:c>
+      <x:c r="K23" s="664"/>
+      <x:c r="L23" s="664"/>
+      <x:c r="M23" s="664"/>
+      <x:c r="N23" s="664"/>
+      <x:c r="O23" s="664"/>
+    </x:row>
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="784" t="str">
+        <x:v>Total allocation</x:v>
+      </x:c>
+      <x:c r="B24" s="798" t="n">
+        <x:f>SUM(B18:B23)</x:f>
+        <x:v>0.39</x:v>
+      </x:c>
+      <x:c r="C24" s="799" t="n">
+        <x:f>SUM(C18:C23)</x:f>
+        <x:v>5248.5887999999995</x:v>
+      </x:c>
+      <x:c r="D24" s="726"/>
+      <x:c r="E24" s="799" t="n">
+        <x:f>SUM(E18:E23)</x:f>
+        <x:v>596.3140266666666</x:v>
+      </x:c>
+      <x:c r="F24" s="723" t="str">
+        <x:v>Excludes goodwill, which is calculated as the residual</x:v>
+      </x:c>
+      <x:c r="G24" s="538"/>
+      <x:c r="H24" s="779" t="str">
+        <x:v>Annualized intangible amortization</x:v>
+      </x:c>
+      <x:c r="I24" s="801" t="n">
+        <x:f>SUM(E18:E21)</x:f>
+        <x:v>522.2954666666666</x:v>
+      </x:c>
+      <x:c r="J24" s="664" t="str">
+        <x:v>Full-year run-rate before the closing-date convention</x:v>
+      </x:c>
+      <x:c r="K24" s="664"/>
+      <x:c r="L24" s="664"/>
+      <x:c r="M24" s="664"/>
+      <x:c r="N24" s="664"/>
+      <x:c r="O24" s="664"/>
+    </x:row>
+    <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25" s="538"/>
+      <x:c r="B25" s="538"/>
+      <x:c r="C25" s="538"/>
+      <x:c r="D25" s="538"/>
+      <x:c r="E25" s="538"/>
+      <x:c r="F25" s="538"/>
+      <x:c r="G25" s="538"/>
+      <x:c r="H25" s="779" t="str">
+        <x:v>Annualized PP&amp;E depreciation</x:v>
+      </x:c>
+      <x:c r="I25" s="801" t="n">
+        <x:f>E23</x:f>
+        <x:v>6.728959999999999</x:v>
+      </x:c>
+      <x:c r="J25" s="664" t="str">
+        <x:v>Full-year run-rate</x:v>
+      </x:c>
+      <x:c r="K25" s="664"/>
+      <x:c r="L25" s="664"/>
+      <x:c r="M25" s="664"/>
+      <x:c r="N25" s="664"/>
+      <x:c r="O25" s="664"/>
+    </x:row>
+    <x:row r="26" ht="24" customHeight="1">
+      <x:c r="A26" s="538"/>
+      <x:c r="B26" s="538"/>
+      <x:c r="C26" s="538"/>
+      <x:c r="D26" s="538"/>
+      <x:c r="E26" s="538"/>
+      <x:c r="F26" s="538"/>
+      <x:c r="G26" s="538"/>
+      <x:c r="H26" s="779" t="str">
+        <x:v>Annualized inventory step-up expense</x:v>
+      </x:c>
+      <x:c r="I26" s="801" t="n">
+        <x:f>E22</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="J26" s="664" t="str">
+        <x:v>Full-year run-rate; realized through cost of sales</x:v>
+      </x:c>
+      <x:c r="K26" s="664"/>
+      <x:c r="L26" s="664"/>
+      <x:c r="M26" s="664"/>
+      <x:c r="N26" s="664"/>
+      <x:c r="O26" s="664"/>
+    </x:row>
+    <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27" s="538"/>
+      <x:c r="B27" s="538"/>
+      <x:c r="C27" s="538"/>
+      <x:c r="D27" s="538"/>
+      <x:c r="E27" s="538"/>
+      <x:c r="F27" s="538"/>
+      <x:c r="G27" s="538"/>
+      <x:c r="H27" s="779" t="str">
+        <x:v>First-year after-tax PPA expense</x:v>
+      </x:c>
+      <x:c r="I27" s="801" t="n">
+        <x:f>B43</x:f>
+        <x:v>235.5440405333333</x:v>
+      </x:c>
+      <x:c r="J27" s="664" t="str">
+        <x:v>Six-month FY2027E impact after the modeled tax benefit</x:v>
+      </x:c>
+      <x:c r="K27" s="664"/>
+      <x:c r="L27" s="664"/>
+      <x:c r="M27" s="664"/>
+      <x:c r="N27" s="664"/>
+      <x:c r="O27" s="664"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="538"/>
+      <x:c r="B28" s="538"/>
+      <x:c r="C28" s="538"/>
+      <x:c r="D28" s="538"/>
+      <x:c r="E28" s="538"/>
+      <x:c r="F28" s="538"/>
+      <x:c r="G28" s="538"/>
+      <x:c r="H28" s="538"/>
+      <x:c r="I28" s="538"/>
+      <x:c r="J28" s="538"/>
+      <x:c r="K28" s="538"/>
+      <x:c r="L28" s="538"/>
+      <x:c r="M28" s="538"/>
+      <x:c r="N28" s="538"/>
+      <x:c r="O28" s="538"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="777" t="str">
+        <x:v>INCREMENTAL NON-CASH EXPENSE SCHEDULE</x:v>
+      </x:c>
+      <x:c r="B29" s="777"/>
+      <x:c r="C29" s="777"/>
+      <x:c r="D29" s="777"/>
+      <x:c r="E29" s="777"/>
+      <x:c r="F29" s="777"/>
+      <x:c r="G29" s="777"/>
+      <x:c r="H29" s="777"/>
+      <x:c r="I29" s="777"/>
+      <x:c r="J29" s="777"/>
+      <x:c r="K29" s="777"/>
+      <x:c r="L29" s="777"/>
+      <x:c r="M29" s="777"/>
+      <x:c r="N29" s="777"/>
+      <x:c r="O29" s="777"/>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="779" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B30" s="803" t="n">
+        <x:f>DATE(YEAR($B$14),9,30)</x:f>
+        <x:v>46660</x:v>
+      </x:c>
+      <x:c r="C30" s="803" t="n">
+        <x:f>DATE(YEAR(B30)+1,9,30)</x:f>
+        <x:v>47026</x:v>
+      </x:c>
+      <x:c r="D30" s="803" t="n">
+        <x:f>DATE(YEAR(C30)+1,9,30)</x:f>
+        <x:v>47391</x:v>
+      </x:c>
+      <x:c r="E30" s="803" t="n">
+        <x:f>DATE(YEAR(D30)+1,9,30)</x:f>
+        <x:v>47756</x:v>
+      </x:c>
+      <x:c r="F30" s="803" t="n">
+        <x:f>DATE(YEAR(E30)+1,9,30)</x:f>
+        <x:v>48121</x:v>
+      </x:c>
+      <x:c r="G30" s="664" t="str">
+        <x:v>Calculation</x:v>
+      </x:c>
+      <x:c r="H30" s="538"/>
+      <x:c r="I30" s="538"/>
+      <x:c r="J30" s="538"/>
+      <x:c r="K30" s="538"/>
+      <x:c r="L30" s="538"/>
+      <x:c r="M30" s="538"/>
+      <x:c r="N30" s="538"/>
+      <x:c r="O30" s="538"/>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="A31" s="779" t="str">
+        <x:v>Months owned</x:v>
+      </x:c>
+      <x:c r="B31" s="804" t="n">
+        <x:f>$B$13</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C31" s="804" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D31" s="804" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E31" s="804" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F31" s="804" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G31" s="664" t="str">
+        <x:v>Close-date convention</x:v>
+      </x:c>
+      <x:c r="H31" s="538"/>
+      <x:c r="I31" s="538"/>
+      <x:c r="J31" s="538"/>
+      <x:c r="K31" s="538"/>
+      <x:c r="L31" s="538"/>
+      <x:c r="M31" s="538"/>
+      <x:c r="N31" s="538"/>
+      <x:c r="O31" s="538"/>
+    </x:row>
+    <x:row r="32" ht="18" customHeight="1">
+      <x:c r="A32" s="779" t="str">
+        <x:v>Cumulative months owned</x:v>
+      </x:c>
+      <x:c r="B32" s="804" t="n">
+        <x:f>B31</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C32" s="804" t="n">
+        <x:f>B32+C31</x:f>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D32" s="804" t="n">
+        <x:f>C32+D31</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E32" s="804" t="n">
+        <x:f>D32+E31</x:f>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F32" s="804" t="n">
+        <x:f>E32+F31</x:f>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G32" s="664" t="str">
+        <x:v>Used to stop expense at end of useful life</x:v>
+      </x:c>
+      <x:c r="H32" s="538"/>
+      <x:c r="I32" s="538"/>
+      <x:c r="J32" s="538"/>
+      <x:c r="K32" s="538"/>
+      <x:c r="L32" s="538"/>
+      <x:c r="M32" s="538"/>
+      <x:c r="N32" s="538"/>
+      <x:c r="O32" s="538"/>
+    </x:row>
+    <x:row r="33" ht="18" customHeight="1">
+      <x:c r="A33" s="779"/>
+      <x:c r="B33" s="436"/>
+      <x:c r="C33" s="436"/>
+      <x:c r="D33" s="436"/>
+      <x:c r="E33" s="436"/>
+      <x:c r="F33" s="436"/>
+      <x:c r="G33" s="664"/>
+      <x:c r="H33" s="538"/>
+      <x:c r="I33" s="538"/>
+      <x:c r="J33" s="538"/>
+      <x:c r="K33" s="538"/>
+      <x:c r="L33" s="538"/>
+      <x:c r="M33" s="538"/>
+      <x:c r="N33" s="538"/>
+      <x:c r="O33" s="538"/>
+    </x:row>
+    <x:row r="34" ht="18" customHeight="1">
+      <x:c r="A34" s="779" t="str">
+        <x:v>Customer relationship amortization</x:v>
+      </x:c>
+      <x:c r="B34" s="744" t="n">
+        <x:f>MIN(B$31,MAX(0,$D18*$B$12-(B$32-B$31)))*$C18/($D18*$B$12)</x:f>
+        <x:v>98.69141333333333</x:v>
+      </x:c>
+      <x:c r="C34" s="744" t="n">
+        <x:f>MIN(C$31,MAX(0,$D18*$B$12-(C$32-C$31)))*$C18/($D18*$B$12)</x:f>
+        <x:v>197.38282666666666</x:v>
+      </x:c>
+      <x:c r="D34" s="744" t="n">
+        <x:f>MIN(D$31,MAX(0,$D18*$B$12-(D$32-D$31)))*$C18/($D18*$B$12)</x:f>
+        <x:v>197.38282666666666</x:v>
+      </x:c>
+      <x:c r="E34" s="744" t="n">
+        <x:f>MIN(E$31,MAX(0,$D18*$B$12-(E$32-E$31)))*$C18/($D18*$B$12)</x:f>
+        <x:v>197.38282666666666</x:v>
+      </x:c>
+      <x:c r="F34" s="744" t="n">
+        <x:f>MIN(F$31,MAX(0,$D18*$B$12-(F$32-F$31)))*$C18/($D18*$B$12)</x:f>
+        <x:v>197.38282666666666</x:v>
+      </x:c>
+      <x:c r="G34" s="664" t="str">
+        <x:v>Straight-line over 15 years</x:v>
+      </x:c>
+      <x:c r="H34" s="538"/>
+      <x:c r="I34" s="538"/>
+      <x:c r="J34" s="538"/>
+      <x:c r="K34" s="538"/>
+      <x:c r="L34" s="538"/>
+      <x:c r="M34" s="538"/>
+      <x:c r="N34" s="538"/>
+      <x:c r="O34" s="538"/>
+    </x:row>
+    <x:row r="35" ht="18" customHeight="1">
+      <x:c r="A35" s="779" t="str">
+        <x:v>Developed technology amortization</x:v>
+      </x:c>
+      <x:c r="B35" s="744" t="n">
+        <x:f>MIN(B$31,MAX(0,$D19*$B$12-(B$32-B$31)))*$C19/($D19*$B$12)</x:f>
+        <x:v>115.35359999999999</x:v>
+      </x:c>
+      <x:c r="C35" s="744" t="n">
+        <x:f>MIN(C$31,MAX(0,$D19*$B$12-(C$32-C$31)))*$C19/($D19*$B$12)</x:f>
+        <x:v>230.70719999999997</x:v>
+      </x:c>
+      <x:c r="D35" s="744" t="n">
+        <x:f>MIN(D$31,MAX(0,$D19*$B$12-(D$32-D$31)))*$C19/($D19*$B$12)</x:f>
+        <x:v>230.70719999999997</x:v>
+      </x:c>
+      <x:c r="E35" s="744" t="n">
+        <x:f>MIN(E$31,MAX(0,$D19*$B$12-(E$32-E$31)))*$C19/($D19*$B$12)</x:f>
+        <x:v>230.70719999999997</x:v>
+      </x:c>
+      <x:c r="F35" s="744" t="n">
+        <x:f>MIN(F$31,MAX(0,$D19*$B$12-(F$32-F$31)))*$C19/($D19*$B$12)</x:f>
+        <x:v>230.70719999999997</x:v>
+      </x:c>
+      <x:c r="G35" s="664" t="str">
+        <x:v>Straight-line over 7 years</x:v>
+      </x:c>
+      <x:c r="H35" s="538"/>
+      <x:c r="I35" s="538"/>
+      <x:c r="J35" s="538"/>
+      <x:c r="K35" s="538"/>
+      <x:c r="L35" s="538"/>
+      <x:c r="M35" s="538"/>
+      <x:c r="N35" s="538"/>
+      <x:c r="O35" s="538"/>
+    </x:row>
+    <x:row r="36" ht="18" customHeight="1">
+      <x:c r="A36" s="779" t="str">
+        <x:v>Trade-name amortization</x:v>
+      </x:c>
+      <x:c r="B36" s="744" t="n">
+        <x:f>MIN(B$31,MAX(0,$D20*$B$12-(B$32-B$31)))*$C20/($D20*$B$12)</x:f>
+        <x:v>13.457919999999998</x:v>
+      </x:c>
+      <x:c r="C36" s="744" t="n">
+        <x:f>MIN(C$31,MAX(0,$D20*$B$12-(C$32-C$31)))*$C20/($D20*$B$12)</x:f>
+        <x:v>26.915839999999996</x:v>
+      </x:c>
+      <x:c r="D36" s="744" t="n">
+        <x:f>MIN(D$31,MAX(0,$D20*$B$12-(D$32-D$31)))*$C20/($D20*$B$12)</x:f>
+        <x:v>26.915839999999996</x:v>
+      </x:c>
+      <x:c r="E36" s="744" t="n">
+        <x:f>MIN(E$31,MAX(0,$D20*$B$12-(E$32-E$31)))*$C20/($D20*$B$12)</x:f>
+        <x:v>26.915839999999996</x:v>
+      </x:c>
+      <x:c r="F36" s="744" t="n">
+        <x:f>MIN(F$31,MAX(0,$D20*$B$12-(F$32-F$31)))*$C20/($D20*$B$12)</x:f>
+        <x:v>26.915839999999996</x:v>
+      </x:c>
+      <x:c r="G36" s="664" t="str">
+        <x:v>Straight-line over 15 years</x:v>
+      </x:c>
+      <x:c r="H36" s="538"/>
+      <x:c r="I36" s="538"/>
+      <x:c r="J36" s="538"/>
+      <x:c r="K36" s="538"/>
+      <x:c r="L36" s="538"/>
+      <x:c r="M36" s="538"/>
+      <x:c r="N36" s="538"/>
+      <x:c r="O36" s="538"/>
+    </x:row>
+    <x:row r="37" ht="18" customHeight="1">
+      <x:c r="A37" s="779" t="str">
+        <x:v>Backlog amortization</x:v>
+      </x:c>
+      <x:c r="B37" s="744" t="n">
+        <x:f>MIN(B$31,MAX(0,$D21*$B$12-(B$32-B$31)))*$C21/($D21*$B$12)</x:f>
+        <x:v>33.6448</x:v>
+      </x:c>
+      <x:c r="C37" s="744" t="n">
+        <x:f>MIN(C$31,MAX(0,$D21*$B$12-(C$32-C$31)))*$C21/($D21*$B$12)</x:f>
+        <x:v>67.2896</x:v>
+      </x:c>
+      <x:c r="D37" s="744" t="n">
+        <x:f>MIN(D$31,MAX(0,$D21*$B$12-(D$32-D$31)))*$C21/($D21*$B$12)</x:f>
+        <x:v>33.6448</x:v>
+      </x:c>
+      <x:c r="E37" s="744" t="n">
+        <x:f>MIN(E$31,MAX(0,$D21*$B$12-(E$32-E$31)))*$C21/($D21*$B$12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F37" s="744" t="n">
+        <x:f>MIN(F$31,MAX(0,$D21*$B$12-(F$32-F$31)))*$C21/($D21*$B$12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G37" s="664" t="str">
+        <x:v>Straight-line over 2 years</x:v>
+      </x:c>
+      <x:c r="H37" s="538"/>
+      <x:c r="I37" s="538"/>
+      <x:c r="J37" s="538"/>
+      <x:c r="K37" s="538"/>
+      <x:c r="L37" s="538"/>
+      <x:c r="M37" s="538"/>
+      <x:c r="N37" s="538"/>
+      <x:c r="O37" s="538"/>
+    </x:row>
+    <x:row r="38" ht="18" customHeight="1">
+      <x:c r="A38" s="779" t="str">
+        <x:v>Inventory step-up expense</x:v>
+      </x:c>
+      <x:c r="B38" s="744" t="n">
+        <x:f>MIN(B$31,MAX(0,$D22*$B$12-(B$32-B$31)))*$C22/($D22*$B$12)</x:f>
+        <x:v>33.6448</x:v>
+      </x:c>
+      <x:c r="C38" s="744" t="n">
+        <x:f>MIN(C$31,MAX(0,$D22*$B$12-(C$32-C$31)))*$C22/($D22*$B$12)</x:f>
+        <x:v>33.6448</x:v>
+      </x:c>
+      <x:c r="D38" s="744" t="n">
+        <x:f>MIN(D$31,MAX(0,$D22*$B$12-(D$32-D$31)))*$C22/($D22*$B$12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E38" s="744" t="n">
+        <x:f>MIN(E$31,MAX(0,$D22*$B$12-(E$32-E$31)))*$C22/($D22*$B$12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F38" s="744" t="n">
+        <x:f>MIN(F$31,MAX(0,$D22*$B$12-(F$32-F$31)))*$C22/($D22*$B$12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G38" s="664" t="str">
+        <x:v>Recognized over 1 year</x:v>
+      </x:c>
+      <x:c r="H38" s="538"/>
+      <x:c r="I38" s="538"/>
+      <x:c r="J38" s="538"/>
+      <x:c r="K38" s="538"/>
+      <x:c r="L38" s="538"/>
+      <x:c r="M38" s="538"/>
+      <x:c r="N38" s="538"/>
+      <x:c r="O38" s="538"/>
+    </x:row>
+    <x:row r="39" ht="18" customHeight="1">
+      <x:c r="A39" s="779" t="str">
+        <x:v>Incremental PP&amp;E depreciation</x:v>
+      </x:c>
+      <x:c r="B39" s="744" t="n">
+        <x:f>MIN(B$31,MAX(0,$D23*$B$12-(B$32-B$31)))*$C23/($D23*$B$12)</x:f>
+        <x:v>3.3644799999999995</x:v>
+      </x:c>
+      <x:c r="C39" s="744" t="n">
+        <x:f>MIN(C$31,MAX(0,$D23*$B$12-(C$32-C$31)))*$C23/($D23*$B$12)</x:f>
+        <x:v>6.728959999999999</x:v>
+      </x:c>
+      <x:c r="D39" s="744" t="n">
+        <x:f>MIN(D$31,MAX(0,$D23*$B$12-(D$32-D$31)))*$C23/($D23*$B$12)</x:f>
+        <x:v>6.728959999999999</x:v>
+      </x:c>
+      <x:c r="E39" s="744" t="n">
+        <x:f>MIN(E$31,MAX(0,$D23*$B$12-(E$32-E$31)))*$C23/($D23*$B$12)</x:f>
+        <x:v>6.728959999999999</x:v>
+      </x:c>
+      <x:c r="F39" s="744" t="n">
+        <x:f>MIN(F$31,MAX(0,$D23*$B$12-(F$32-F$31)))*$C23/($D23*$B$12)</x:f>
+        <x:v>6.728959999999999</x:v>
+      </x:c>
+      <x:c r="G39" s="664" t="str">
+        <x:v>Straight-line over 10 years</x:v>
+      </x:c>
+      <x:c r="H39" s="538"/>
+      <x:c r="I39" s="538"/>
+      <x:c r="J39" s="538"/>
+      <x:c r="K39" s="538"/>
+      <x:c r="L39" s="538"/>
+      <x:c r="M39" s="538"/>
+      <x:c r="N39" s="538"/>
+      <x:c r="O39" s="538"/>
+    </x:row>
+    <x:row r="40" ht="18" customHeight="1">
+      <x:c r="A40" s="779"/>
+      <x:c r="B40" s="744"/>
+      <x:c r="C40" s="744"/>
+      <x:c r="D40" s="744"/>
+      <x:c r="E40" s="744"/>
+      <x:c r="F40" s="744"/>
+      <x:c r="G40" s="664"/>
+      <x:c r="H40" s="538"/>
+      <x:c r="I40" s="538"/>
+      <x:c r="J40" s="538"/>
+      <x:c r="K40" s="538"/>
+      <x:c r="L40" s="538"/>
+      <x:c r="M40" s="538"/>
+      <x:c r="N40" s="538"/>
+      <x:c r="O40" s="538"/>
+    </x:row>
+    <x:row r="41" ht="18" customHeight="1">
+      <x:c r="A41" s="779" t="str">
+        <x:v>Total incremental PPA expense</x:v>
+      </x:c>
+      <x:c r="B41" s="744" t="n">
+        <x:f>SUM(B34:B39)</x:f>
+        <x:v>298.1570133333333</x:v>
+      </x:c>
+      <x:c r="C41" s="744" t="n">
+        <x:f>SUM(C34:C39)</x:f>
+        <x:v>562.6692266666666</x:v>
+      </x:c>
+      <x:c r="D41" s="744" t="n">
+        <x:f>SUM(D34:D39)</x:f>
+        <x:v>495.3796266666666</x:v>
+      </x:c>
+      <x:c r="E41" s="744" t="n">
+        <x:f>SUM(E34:E39)</x:f>
+        <x:v>461.7348266666666</x:v>
+      </x:c>
+      <x:c r="F41" s="744" t="n">
+        <x:f>SUM(F34:F39)</x:f>
+        <x:v>461.7348266666666</x:v>
+      </x:c>
+      <x:c r="G41" s="664"/>
+      <x:c r="H41" s="538"/>
+      <x:c r="I41" s="538"/>
+      <x:c r="J41" s="538"/>
+      <x:c r="K41" s="538"/>
+      <x:c r="L41" s="538"/>
+      <x:c r="M41" s="538"/>
+      <x:c r="N41" s="538"/>
+      <x:c r="O41" s="538"/>
+    </x:row>
+    <x:row r="42" ht="18" customHeight="1">
+      <x:c r="A42" s="779" t="str">
+        <x:v>Deferred tax benefit</x:v>
+      </x:c>
+      <x:c r="B42" s="744" t="n">
+        <x:f>B41*$B$11</x:f>
+        <x:v>62.61297279999999</x:v>
+      </x:c>
+      <x:c r="C42" s="744" t="n">
+        <x:f>C41*$B$11</x:f>
+        <x:v>118.1605376</x:v>
+      </x:c>
+      <x:c r="D42" s="744" t="n">
+        <x:f>D41*$B$11</x:f>
+        <x:v>104.02972159999997</x:v>
+      </x:c>
+      <x:c r="E42" s="744" t="n">
+        <x:f>E41*$B$11</x:f>
+        <x:v>96.96431359999998</x:v>
+      </x:c>
+      <x:c r="F42" s="744" t="n">
+        <x:f>F41*$B$11</x:f>
+        <x:v>96.96431359999998</x:v>
+      </x:c>
+      <x:c r="G42" s="664"/>
+      <x:c r="H42" s="538"/>
+      <x:c r="I42" s="538"/>
+      <x:c r="J42" s="538"/>
+      <x:c r="K42" s="538"/>
+      <x:c r="L42" s="538"/>
+      <x:c r="M42" s="538"/>
+      <x:c r="N42" s="538"/>
+      <x:c r="O42" s="538"/>
+    </x:row>
+    <x:row r="43" ht="18" customHeight="1">
+      <x:c r="A43" s="784" t="str">
+        <x:v>After-tax PPA expense</x:v>
+      </x:c>
+      <x:c r="B43" s="805" t="n">
+        <x:f>B41-B42</x:f>
+        <x:v>235.5440405333333</x:v>
+      </x:c>
+      <x:c r="C43" s="805" t="n">
+        <x:f>C41-C42</x:f>
+        <x:v>444.50868906666665</x:v>
+      </x:c>
+      <x:c r="D43" s="805" t="n">
+        <x:f>D41-D42</x:f>
+        <x:v>391.3499050666666</x:v>
+      </x:c>
+      <x:c r="E43" s="805" t="n">
+        <x:f>E41-E42</x:f>
+        <x:v>364.77051306666664</x:v>
+      </x:c>
+      <x:c r="F43" s="805" t="n">
+        <x:f>F41-F42</x:f>
+        <x:v>364.77051306666664</x:v>
+      </x:c>
+      <x:c r="G43" s="664"/>
+      <x:c r="H43" s="538"/>
+      <x:c r="I43" s="538"/>
+      <x:c r="J43" s="538"/>
+      <x:c r="K43" s="538"/>
+      <x:c r="L43" s="538"/>
+      <x:c r="M43" s="538"/>
+      <x:c r="N43" s="538"/>
+      <x:c r="O43" s="538"/>
+    </x:row>
+    <x:row r="44" ht="18" customHeight="1">
+      <x:c r="A44" s="538"/>
+      <x:c r="B44" s="746"/>
+      <x:c r="C44" s="746"/>
+      <x:c r="D44" s="746"/>
+      <x:c r="E44" s="746"/>
+      <x:c r="F44" s="746"/>
+      <x:c r="G44" s="538"/>
+      <x:c r="H44" s="538"/>
+      <x:c r="I44" s="538"/>
+      <x:c r="J44" s="538"/>
+      <x:c r="K44" s="538"/>
+      <x:c r="L44" s="538"/>
+      <x:c r="M44" s="538"/>
+      <x:c r="N44" s="538"/>
+      <x:c r="O44" s="538"/>
+    </x:row>
+    <x:row r="45" ht="18" customHeight="1">
+      <x:c r="A45" s="777" t="str">
+        <x:v>DEFERRED TAX LIABILITY ROLL-FORWARD</x:v>
+      </x:c>
+      <x:c r="B45" s="806"/>
+      <x:c r="C45" s="806"/>
+      <x:c r="D45" s="806"/>
+      <x:c r="E45" s="806"/>
+      <x:c r="F45" s="806"/>
+      <x:c r="G45" s="777"/>
+      <x:c r="H45" s="777" t="str">
+        <x:v>RECONCILIATION CHECKS</x:v>
+      </x:c>
+      <x:c r="I45" s="777"/>
+      <x:c r="J45" s="777"/>
+      <x:c r="K45" s="777"/>
+      <x:c r="L45" s="777"/>
+      <x:c r="M45" s="777"/>
+      <x:c r="N45" s="777"/>
+      <x:c r="O45" s="777"/>
+    </x:row>
+    <x:row r="46" ht="18" customHeight="1">
+      <x:c r="A46" s="779" t="str">
+        <x:v>Beginning DTL</x:v>
+      </x:c>
+      <x:c r="B46" s="744" t="n">
+        <x:f>$I$15</x:f>
+        <x:v>1102.203648</x:v>
+      </x:c>
+      <x:c r="C46" s="744" t="n">
+        <x:f>B48</x:f>
+        <x:v>1039.5906751999999</x:v>
+      </x:c>
+      <x:c r="D46" s="744" t="n">
+        <x:f>C48</x:f>
+        <x:v>921.4301375999999</x:v>
+      </x:c>
+      <x:c r="E46" s="744" t="n">
+        <x:f>D48</x:f>
+        <x:v>817.4004159999998</x:v>
+      </x:c>
+      <x:c r="F46" s="744" t="n">
+        <x:f>E48</x:f>
+        <x:v>720.4361023999999</x:v>
+      </x:c>
+      <x:c r="G46" s="538"/>
+      <x:c r="H46" s="779" t="str">
+        <x:v>Purchase consideration bridge</x:v>
+      </x:c>
+      <x:c r="I46" s="807" t="n">
+        <x:f>I6-I16-I17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J46" s="664" t="str">
+        <x:v>Must equal zero</x:v>
+      </x:c>
+      <x:c r="K46" s="664"/>
+      <x:c r="L46" s="664"/>
+      <x:c r="M46" s="664"/>
+      <x:c r="N46" s="664"/>
+      <x:c r="O46" s="664"/>
+    </x:row>
+    <x:row r="47" ht="18" customHeight="1">
+      <x:c r="A47" s="779" t="str">
+        <x:v>Less: DTL reversal</x:v>
+      </x:c>
+      <x:c r="B47" s="744" t="n">
+        <x:f>B42</x:f>
+        <x:v>62.61297279999999</x:v>
+      </x:c>
+      <x:c r="C47" s="744" t="n">
+        <x:f>C42</x:f>
+        <x:v>118.1605376</x:v>
+      </x:c>
+      <x:c r="D47" s="744" t="n">
+        <x:f>D42</x:f>
+        <x:v>104.02972159999997</x:v>
+      </x:c>
+      <x:c r="E47" s="744" t="n">
+        <x:f>E42</x:f>
+        <x:v>96.96431359999998</x:v>
+      </x:c>
+      <x:c r="F47" s="744" t="n">
+        <x:f>F42</x:f>
+        <x:v>96.96431359999998</x:v>
+      </x:c>
+      <x:c r="G47" s="538"/>
+      <x:c r="H47" s="779" t="str">
+        <x:v>Allocation percentage total</x:v>
+      </x:c>
+      <x:c r="I47" s="808" t="n">
+        <x:f>B24</x:f>
+        <x:v>0.39</x:v>
+      </x:c>
+      <x:c r="J47" s="664" t="str">
+        <x:v>39.0% of consideration assigned to identifiable asset write-ups</x:v>
+      </x:c>
+      <x:c r="K47" s="664"/>
+      <x:c r="L47" s="664"/>
+      <x:c r="M47" s="664"/>
+      <x:c r="N47" s="664"/>
+      <x:c r="O47" s="664"/>
+    </x:row>
+    <x:row r="48" ht="18" customHeight="1">
+      <x:c r="A48" s="779" t="str">
+        <x:v>Ending DTL</x:v>
+      </x:c>
+      <x:c r="B48" s="807" t="n">
+        <x:f>MAX(0,B46-B47)</x:f>
+        <x:v>1039.5906751999999</x:v>
+      </x:c>
+      <x:c r="C48" s="807" t="n">
+        <x:f>MAX(0,C46-C47)</x:f>
+        <x:v>921.4301375999999</x:v>
+      </x:c>
+      <x:c r="D48" s="807" t="n">
+        <x:f>MAX(0,D46-D47)</x:f>
+        <x:v>817.4004159999998</x:v>
+      </x:c>
+      <x:c r="E48" s="807" t="n">
+        <x:f>MAX(0,E46-E47)</x:f>
+        <x:v>720.4361023999999</x:v>
+      </x:c>
+      <x:c r="F48" s="807" t="n">
+        <x:f>MAX(0,F46-F47)</x:f>
+        <x:v>623.4717887999999</x:v>
+      </x:c>
+      <x:c r="G48" s="538"/>
+      <x:c r="H48" s="779" t="str">
+        <x:v>Goodwill positive</x:v>
+      </x:c>
+      <x:c r="I48" s="807" t="n">
+        <x:f>I17</x:f>
+        <x:v>8127.828847999998</x:v>
+      </x:c>
+      <x:c r="J48" s="664" t="str">
+        <x:v>Residual goodwill must remain greater than zero</x:v>
+      </x:c>
+      <x:c r="K48" s="664"/>
+      <x:c r="L48" s="664"/>
+      <x:c r="M48" s="664"/>
+      <x:c r="N48" s="664"/>
+      <x:c r="O48" s="664"/>
+    </x:row>
+    <x:row r="49" ht="18" customHeight="1">
+      <x:c r="A49" s="538"/>
+      <x:c r="B49" s="538"/>
+      <x:c r="C49" s="538"/>
+      <x:c r="D49" s="538"/>
+      <x:c r="E49" s="538"/>
+      <x:c r="F49" s="538"/>
+      <x:c r="G49" s="538"/>
+      <x:c r="H49" s="779" t="str">
+        <x:v>First-year expense tie-out</x:v>
+      </x:c>
+      <x:c r="I49" s="807" t="n">
+        <x:f>I27-B43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J49" s="664" t="str">
+        <x:v>Key output must equal the detailed schedule</x:v>
+      </x:c>
+      <x:c r="K49" s="664"/>
+      <x:c r="L49" s="664"/>
+      <x:c r="M49" s="664"/>
+      <x:c r="N49" s="664"/>
+      <x:c r="O49" s="664"/>
+    </x:row>
+    <x:row r="50" ht="18" customHeight="1">
+      <x:c r="A50" s="538"/>
+      <x:c r="B50" s="538"/>
+      <x:c r="C50" s="538"/>
+      <x:c r="D50" s="538"/>
+      <x:c r="E50" s="538"/>
+      <x:c r="F50" s="538"/>
+      <x:c r="G50" s="538"/>
+      <x:c r="H50" s="538"/>
+      <x:c r="I50" s="538"/>
+      <x:c r="J50" s="538"/>
+      <x:c r="K50" s="538"/>
+      <x:c r="L50" s="538"/>
+      <x:c r="M50" s="538"/>
+      <x:c r="N50" s="538"/>
+      <x:c r="O50" s="538"/>
+    </x:row>
+    <x:row r="51" ht="18" customHeight="1">
+      <x:c r="A51" s="777" t="str">
+        <x:v>ANALYST INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="B51" s="777"/>
+      <x:c r="C51" s="777"/>
+      <x:c r="D51" s="777"/>
+      <x:c r="E51" s="777"/>
+      <x:c r="F51" s="777"/>
+      <x:c r="G51" s="777"/>
+      <x:c r="H51" s="777"/>
+      <x:c r="I51" s="777"/>
+      <x:c r="J51" s="777"/>
+      <x:c r="K51" s="777"/>
+      <x:c r="L51" s="777"/>
+      <x:c r="M51" s="777"/>
+      <x:c r="N51" s="777"/>
+      <x:c r="O51" s="777"/>
+    </x:row>
+    <x:row r="52" ht="30" customHeight="1">
+      <x:c r="A52" s="792" t="str">
+        <x:v>The preliminary allocation creates approximately $8.2 billion of goodwill because the $80 offer materially exceeds Cognex’s tangible book value and the identifiable technology, customer, brand, backlog, inventory, and PP&amp;E values assigned in this merger model.</x:v>
+      </x:c>
+      <x:c r="B52" s="792"/>
+      <x:c r="C52" s="792"/>
+      <x:c r="D52" s="792"/>
+      <x:c r="E52" s="792"/>
+      <x:c r="F52" s="792"/>
+      <x:c r="G52" s="792"/>
+      <x:c r="H52" s="792"/>
+      <x:c r="I52" s="792"/>
+      <x:c r="J52" s="792"/>
+      <x:c r="K52" s="792"/>
+      <x:c r="L52" s="792"/>
+      <x:c r="M52" s="792"/>
+      <x:c r="N52" s="792"/>
+      <x:c r="O52" s="792"/>
+    </x:row>
+    <x:row r="53" ht="30" customHeight="1">
+      <x:c r="A53" s="792" t="str">
+        <x:v>Goodwill is not amortized, but the acquired intangible and stepped-up tangible assets create material non-cash expense. The first-year schedule reflects six months of ownership based on a March 31 close and Rockwell’s September fiscal year-end.</x:v>
+      </x:c>
+      <x:c r="B53" s="792"/>
+      <x:c r="C53" s="792"/>
+      <x:c r="D53" s="792"/>
+      <x:c r="E53" s="792"/>
+      <x:c r="F53" s="792"/>
+      <x:c r="G53" s="792"/>
+      <x:c r="H53" s="792"/>
+      <x:c r="I53" s="792"/>
+      <x:c r="J53" s="792"/>
+      <x:c r="K53" s="792"/>
+      <x:c r="L53" s="792"/>
+      <x:c r="M53" s="792"/>
+      <x:c r="N53" s="792"/>
+      <x:c r="O53" s="792"/>
+    </x:row>
+    <x:row r="54" ht="30" customHeight="1">
+      <x:c r="A54" s="793" t="str">
+        <x:v>This is an illustrative banking-model allocation, not a valuation report. An actual transaction would require specialist appraisals, legal-entity tax analysis, and management estimates before the opening balance sheet could be finalized.</x:v>
+      </x:c>
+      <x:c r="B54" s="793"/>
+      <x:c r="C54" s="793"/>
+      <x:c r="D54" s="793"/>
+      <x:c r="E54" s="793"/>
+      <x:c r="F54" s="793"/>
+      <x:c r="G54" s="793"/>
+      <x:c r="H54" s="793"/>
+      <x:c r="I54" s="793"/>
+      <x:c r="J54" s="793"/>
+      <x:c r="K54" s="793"/>
+      <x:c r="L54" s="793"/>
+      <x:c r="M54" s="793"/>
+      <x:c r="N54" s="793"/>
+      <x:c r="O54" s="793"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="B3:O3"/>
+    <x:mergeCell ref="A5:F5"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="E10:F10"/>
+    <x:mergeCell ref="E11:F11"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="E13:F13"/>
+    <x:mergeCell ref="E14:F14"/>
+    <x:mergeCell ref="A16:F16"/>
+    <x:mergeCell ref="H5:O5"/>
+    <x:mergeCell ref="J6:O6"/>
+    <x:mergeCell ref="J7:O7"/>
+    <x:mergeCell ref="J8:O8"/>
+    <x:mergeCell ref="J9:O9"/>
+    <x:mergeCell ref="J10:O10"/>
+    <x:mergeCell ref="J11:O11"/>
+    <x:mergeCell ref="J12:O12"/>
+    <x:mergeCell ref="J13:O13"/>
+    <x:mergeCell ref="J14:O14"/>
+    <x:mergeCell ref="J15:O15"/>
+    <x:mergeCell ref="J16:O16"/>
+    <x:mergeCell ref="J17:O17"/>
+    <x:mergeCell ref="J18:O18"/>
+    <x:mergeCell ref="H20:O20"/>
+    <x:mergeCell ref="J21:O21"/>
+    <x:mergeCell ref="J22:O22"/>
+    <x:mergeCell ref="J23:O23"/>
+    <x:mergeCell ref="J24:O24"/>
+    <x:mergeCell ref="J25:O25"/>
+    <x:mergeCell ref="J26:O26"/>
+    <x:mergeCell ref="J27:O27"/>
+    <x:mergeCell ref="A29:O29"/>
+    <x:mergeCell ref="A45:G45"/>
+    <x:mergeCell ref="H45:O45"/>
+    <x:mergeCell ref="J46:O46"/>
+    <x:mergeCell ref="J47:O47"/>
+    <x:mergeCell ref="J48:O48"/>
+    <x:mergeCell ref="J49:O49"/>
+    <x:mergeCell ref="A51:O51"/>
+    <x:mergeCell ref="A52:O52"/>
+    <x:mergeCell ref="A53:O53"/>
+    <x:mergeCell ref="A54:O54"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9843,8 +11555,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="767" t="str">
-        <x:v>FINANCING COMPLETE</x:v>
+      <x:c r="B3" s="812" t="str">
+        <x:v>PURCHASE ACCOUNTING COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -9890,10 +11602,10 @@
       </x:c>
       <x:c r="B6" s="134" t="n">
         <x:f>COUNTA('Sources'!A4:A100)</x:f>
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="135" t="n">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D6" s="135" t="n">
         <x:f>B6-C6</x:f>
@@ -10714,6 +12426,136 @@
       </x:c>
       <x:c r="G37" s="484" t="str">
         <x:v>Sources &amp; Uses rows 22 and 33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="484" t="str">
+        <x:v>Purchase-accounting bridge</x:v>
+      </x:c>
+      <x:c r="B38" s="484" t="n">
+        <x:f>'Purchase Accounting'!I46</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C38" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D38" s="484" t="n">
+        <x:f>B38-C38</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E38" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F38" s="814" t="str">
+        <x:f>IF(ABS(D38)&lt;=E38,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G38" s="484" t="str">
+        <x:v>Purchase Accounting row 46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="484" t="str">
+        <x:v>PPA allocation total</x:v>
+      </x:c>
+      <x:c r="B39" s="484" t="n">
+        <x:f>'Purchase Accounting'!I47</x:f>
+        <x:v>0.39</x:v>
+      </x:c>
+      <x:c r="C39" s="484" t="n">
+        <x:v>0.39</x:v>
+      </x:c>
+      <x:c r="D39" s="484" t="n">
+        <x:f>B39-C39</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E39" s="484" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F39" s="814" t="str">
+        <x:f>IF(ABS(D39)&lt;=E39,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G39" s="484" t="str">
+        <x:v>Purchase Accounting row 47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="484" t="str">
+        <x:v>Goodwill remains positive</x:v>
+      </x:c>
+      <x:c r="B40" s="484" t="n">
+        <x:f>'Purchase Accounting'!I48</x:f>
+        <x:v>8127.828847999998</x:v>
+      </x:c>
+      <x:c r="C40" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="484" t="n">
+        <x:f>MIN(0,B40-C40)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F40" s="814" t="str">
+        <x:f>IF(ABS(D40)&lt;=E40,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G40" s="484" t="str">
+        <x:v>Purchase Accounting row 48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="484" t="str">
+        <x:v>First-year PPA expense tie-out</x:v>
+      </x:c>
+      <x:c r="B41" s="484" t="n">
+        <x:f>'Purchase Accounting'!I49</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C41" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="484" t="n">
+        <x:f>B41-C41</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E41" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F41" s="814" t="str">
+        <x:f>IF(ABS(D41)&lt;=E41,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G41" s="484" t="str">
+        <x:v>Purchase Accounting row 49</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="484" t="str">
+        <x:v>DTL roll-forward</x:v>
+      </x:c>
+      <x:c r="B42" s="484" t="n">
+        <x:f>'Purchase Accounting'!F46-'Purchase Accounting'!F47-'Purchase Accounting'!F48</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C42" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="484" t="n">
+        <x:f>B42-C42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E42" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F42" s="814" t="str">
+        <x:f>IF(ABS(D42)&lt;=E42,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G42" s="484" t="str">
+        <x:v>Purchase Accounting rows 46-48</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12848,6 +14690,32 @@
         <x:v>$431.45 closing price on Aug. 20, 2026</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="38" customHeight="1">
+      <x:c r="A35" s="480" t="str">
+        <x:v>S-052</x:v>
+      </x:c>
+      <x:c r="B35" s="480" t="str">
+        <x:v>Cognex</x:v>
+      </x:c>
+      <x:c r="C35" s="480" t="str">
+        <x:v>Second-quarter 2026 results and balance sheet</x:v>
+      </x:c>
+      <x:c r="D35" s="481" t="n">
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="E35" s="481" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="F35" s="480" t="str">
+        <x:v>Latest target shareholders’ equity, existing goodwill, existing intangible assets, and balance-sheet context</x:v>
+      </x:c>
+      <x:c r="G35" s="480" t="str">
+        <x:v>https://www.prnewswire.com/news-releases/cognex-reports-second-quarter-2026-results-302844140.html</x:v>
+      </x:c>
+      <x:c r="H35" s="480" t="str">
+        <x:v>Company-issued earnings release; unaudited July 5, 2026 balance sheet</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -14256,7 +16124,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55562b56411e471b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dd4014f02454c82"/>
 </x:worksheet>
 </file>
 
@@ -15979,7 +17847,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bd467dd805d46b7"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2873171e73d34d04"/>
 </x:worksheet>
 </file>
 
@@ -19466,7 +21334,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d488bec88704475"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74bcb809d4f746a3"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
transaction: complete accretion dilution analysis
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R07f9548a994643c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R44460d68c93e490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rec640185d77c4208"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R07661846d8ed4df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R419c26e5b0154ce8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rdb119bb981434ae3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R23b603b9622f4548"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R154d2866cbed409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R1c564d5a7fbf4455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Re8112b4112694336"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="Ra83a35549ac94976"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R49e21e59c38e4887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R27ab496476a04455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R4739deba96b24abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R18272b9c01834493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R5c9e50199c864f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Rb4ae5e17e35b4ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R1dd3810331e54681"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R8f5ddea17ffa485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rd78e776180794d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R17404b112bae4706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rb21f822a1cc44a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R8d4f70c80df24841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Rba564b03131c4630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Rda684895e721438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R1930e61aff51462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rb5cfdf4d7aeb43c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R7cb71841a215468b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R1ff3cda4cc5847f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R5ced32c55ea24475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R9fbb43493e454b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Ra3015c248be94c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rd905c55e9b824730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R78bb7f6040834811"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="25">
+  <x:numFmts count="26">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -181,8 +181,9 @@
     <x:numFmt numFmtId="222" formatCode=";;;"/>
     <x:numFmt numFmtId="223" formatCode="$0"/>
     <x:numFmt numFmtId="224" formatCode="yyyy&quot;E&quot;"/>
+    <x:numFmt numFmtId="225" formatCode="$#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="45">
+  <x:fonts count="46">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -436,8 +437,14 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFC00000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="61">
+  <x:fills count="69">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -739,6 +746,46 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="25">
     <x:border/>
@@ -1010,7 +1057,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="815">
+  <x:cellXfs count="854">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2744,6 +2791,115 @@
     <x:xf numFmtId="0" fontId="26" fillId="56" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="40" fillId="56" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="38" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="33" fillId="61" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="62" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="64" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="65" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="65" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="37" fillId="66" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="68" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="68" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="65" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="67" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="40" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="37" fillId="66" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="37" fillId="66" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="45" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="45" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="41" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="224" fontId="41" fillId="68" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="214" fontId="38" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="67" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="215" fontId="38" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="38" fillId="67" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="225" fontId="40" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3223,7 +3379,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.8 — purchase accounting complete</x:v>
+        <x:v>0.9 — accretion / dilution complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -3278,8 +3434,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="811" t="str">
-        <x:v>PURCHASE ACCOUNTING COMPLETE</x:v>
+      <x:c r="B9" s="850" t="str">
+        <x:v>CORE TRANSACTION MODEL COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -11183,110 +11339,1810 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="37" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="3" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Accretion Dilution</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Pro forma earnings, shares, EPS, and accretion/dilution</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="816" t="str">
+        <x:v>Accretion / Dilution Analysis</x:v>
+      </x:c>
+      <x:c r="B1" s="816"/>
+      <x:c r="C1" s="816"/>
+      <x:c r="D1" s="816"/>
+      <x:c r="E1" s="816"/>
+      <x:c r="F1" s="816"/>
+      <x:c r="G1" s="816"/>
+      <x:c r="H1" s="816"/>
+      <x:c r="I1" s="816"/>
+      <x:c r="J1" s="816"/>
+      <x:c r="K1" s="816"/>
+      <x:c r="L1" s="816"/>
+      <x:c r="M1" s="816"/>
+      <x:c r="N1" s="816"/>
+      <x:c r="O1" s="816"/>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="818" t="str">
+        <x:v>Pro forma earnings, financing costs, purchase-accounting effects, share issuance, and EPS impact | USD millions except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="818"/>
+      <x:c r="C2" s="818"/>
+      <x:c r="D2" s="818"/>
+      <x:c r="E2" s="818"/>
+      <x:c r="F2" s="818"/>
+      <x:c r="G2" s="818"/>
+      <x:c r="H2" s="818"/>
+      <x:c r="I2" s="818"/>
+      <x:c r="J2" s="818"/>
+      <x:c r="K2" s="818"/>
+      <x:c r="L2" s="818"/>
+      <x:c r="M2" s="818"/>
+      <x:c r="N2" s="818"/>
+      <x:c r="O2" s="818"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="432" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="820" t="str">
+        <x:v>Complete — base case excludes synergies and one-time transaction fees from headline recurring EPS</x:v>
+      </x:c>
+      <x:c r="C3" s="820"/>
+      <x:c r="D3" s="820"/>
+      <x:c r="E3" s="820"/>
+      <x:c r="F3" s="820"/>
+      <x:c r="G3" s="820"/>
+      <x:c r="H3" s="820"/>
+      <x:c r="I3" s="820"/>
+      <x:c r="J3" s="820"/>
+      <x:c r="K3" s="820"/>
+      <x:c r="L3" s="820"/>
+      <x:c r="M3" s="820"/>
+      <x:c r="N3" s="820"/>
+      <x:c r="O3" s="820"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="538"/>
+      <x:c r="B4" s="538"/>
+      <x:c r="C4" s="538"/>
+      <x:c r="D4" s="538"/>
+      <x:c r="E4" s="538"/>
+      <x:c r="F4" s="538"/>
+      <x:c r="G4" s="538"/>
+      <x:c r="H4" s="538"/>
+      <x:c r="I4" s="538"/>
+      <x:c r="J4" s="538"/>
+      <x:c r="K4" s="538"/>
+      <x:c r="L4" s="538"/>
+      <x:c r="M4" s="538"/>
+      <x:c r="N4" s="538"/>
+      <x:c r="O4" s="538"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="822" t="str">
+        <x:v>TRANSACTION AND MODEL INPUTS</x:v>
+      </x:c>
+      <x:c r="B5" s="822"/>
+      <x:c r="C5" s="822"/>
+      <x:c r="D5" s="822"/>
+      <x:c r="E5" s="822"/>
+      <x:c r="F5" s="822"/>
+      <x:c r="G5" s="538"/>
+      <x:c r="H5" s="822" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I5" s="822"/>
+      <x:c r="J5" s="822"/>
+      <x:c r="K5" s="822"/>
+      <x:c r="L5" s="822"/>
+      <x:c r="M5" s="822"/>
+      <x:c r="N5" s="822"/>
+      <x:c r="O5" s="822"/>
+    </x:row>
+    <x:row r="6" ht="25" customHeight="1">
+      <x:c r="A6" s="824" t="str">
+        <x:v>First-year ownership</x:v>
+      </x:c>
+      <x:c r="B6" s="733" t="n">
+        <x:f>'Purchase Accounting'!B13/'Purchase Accounting'!B12</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C6" s="436" t="str">
+        <x:v>% of year</x:v>
+      </x:c>
+      <x:c r="D6" s="436" t="str">
+        <x:v>Purchase Accounting</x:v>
+      </x:c>
+      <x:c r="E6" s="664" t="str">
+        <x:v>Six months from March 31 close through Rockwell’s September 30 fiscal year-end</x:v>
+      </x:c>
+      <x:c r="F6" s="664"/>
+      <x:c r="G6" s="538"/>
+      <x:c r="H6" s="824" t="str">
+        <x:v>FY2027E EPS accretion / (dilution) — incl. PPA</x:v>
+      </x:c>
+      <x:c r="I6" s="840" t="n">
+        <x:f>B41</x:f>
+        <x:v>-0.20507774150422142</x:v>
+      </x:c>
+      <x:c r="J6" s="664" t="str">
+        <x:v>Headline recurring result on Rockwell’s adjusted-earnings base</x:v>
+      </x:c>
+      <x:c r="K6" s="664"/>
+      <x:c r="L6" s="664"/>
+      <x:c r="M6" s="664"/>
+      <x:c r="N6" s="664"/>
+      <x:c r="O6" s="664"/>
+    </x:row>
+    <x:row r="7" ht="25" customHeight="1">
+      <x:c r="A7" s="824" t="str">
+        <x:v>Buyer tax rate</x:v>
+      </x:c>
+      <x:c r="B7" s="733" t="n">
+        <x:f>'Purchase Accounting'!B11</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="C7" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D7" s="436" t="str">
+        <x:v>Purchase Accounting</x:v>
+      </x:c>
+      <x:c r="E7" s="664" t="str">
+        <x:v>Applied to incremental financing costs and breakeven synergies</x:v>
+      </x:c>
+      <x:c r="F7" s="664"/>
+      <x:c r="G7" s="538"/>
+      <x:c r="H7" s="824" t="str">
+        <x:v>FY2027E adjusted accretion / (dilution) — excl. PPA</x:v>
+      </x:c>
+      <x:c r="I7" s="840" t="n">
+        <x:f>B45</x:f>
+        <x:v>-0.06681149114314067</x:v>
+      </x:c>
+      <x:c r="J7" s="664" t="str">
+        <x:v>Excludes acquisition-related PPA expense but retains financing costs and dilution</x:v>
+      </x:c>
+      <x:c r="K7" s="664"/>
+      <x:c r="L7" s="664"/>
+      <x:c r="M7" s="664"/>
+      <x:c r="N7" s="664"/>
+      <x:c r="O7" s="664"/>
+    </x:row>
+    <x:row r="8" ht="25" customHeight="1">
+      <x:c r="A8" s="824" t="str">
+        <x:v>Foregone cash yield</x:v>
+      </x:c>
+      <x:c r="B8" s="838" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="C8" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D8" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E8" s="664" t="str">
+        <x:v>Pre-tax return forgone on Rockwell cash used at closing</x:v>
+      </x:c>
+      <x:c r="F8" s="664"/>
+      <x:c r="G8" s="538"/>
+      <x:c r="H8" s="824" t="str">
+        <x:v>FY2028E EPS accretion / (dilution) — incl. PPA</x:v>
+      </x:c>
+      <x:c r="I8" s="840" t="n">
+        <x:f>C41</x:f>
+        <x:v>-0.33805997212936467</x:v>
+      </x:c>
+      <x:c r="J8" s="664" t="str">
+        <x:v>First full fiscal-year result</x:v>
+      </x:c>
+      <x:c r="K8" s="664"/>
+      <x:c r="L8" s="664"/>
+      <x:c r="M8" s="664"/>
+      <x:c r="N8" s="664"/>
+      <x:c r="O8" s="664"/>
+    </x:row>
+    <x:row r="9" ht="25" customHeight="1">
+      <x:c r="A9" s="824" t="str">
+        <x:v>Debt-fee amortization period</x:v>
+      </x:c>
+      <x:c r="B9" s="839" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C9" s="436" t="str">
+        <x:v>years</x:v>
+      </x:c>
+      <x:c r="D9" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E9" s="664" t="str">
+        <x:v>Straight-line amortization of upfront debt fees</x:v>
+      </x:c>
+      <x:c r="F9" s="664"/>
+      <x:c r="G9" s="538"/>
+      <x:c r="H9" s="824" t="str">
+        <x:v>FY2028E adjusted accretion / (dilution) — excl. PPA</x:v>
+      </x:c>
+      <x:c r="I9" s="840" t="n">
+        <x:f>C45</x:f>
+        <x:v>-0.11056396062894436</x:v>
+      </x:c>
+      <x:c r="J9" s="664" t="str">
+        <x:v>Shows underlying dilution before acquisition-accounting expense</x:v>
+      </x:c>
+      <x:c r="K9" s="664"/>
+      <x:c r="L9" s="664"/>
+      <x:c r="M9" s="664"/>
+      <x:c r="N9" s="664"/>
+      <x:c r="O9" s="664"/>
+    </x:row>
+    <x:row r="10" ht="25" customHeight="1">
+      <x:c r="A10" s="824" t="str">
+        <x:v>Transaction-fee tax deductibility</x:v>
+      </x:c>
+      <x:c r="B10" s="838" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" s="436" t="str">
+        <x:v>% deductible</x:v>
+      </x:c>
+      <x:c r="D10" s="436" t="str">
+        <x:v>Analyst assumption</x:v>
+      </x:c>
+      <x:c r="E10" s="664" t="str">
+        <x:v>Conservative assumption; actual deductibility depends on fee type and structure</x:v>
+      </x:c>
+      <x:c r="F10" s="664"/>
+      <x:c r="G10" s="538"/>
+      <x:c r="H10" s="824" t="str">
+        <x:v>FY2027E annualized breakeven synergies — incl. PPA</x:v>
+      </x:c>
+      <x:c r="I10" s="841" t="n">
+        <x:f>I24</x:f>
+        <x:v>884.4583077701694</x:v>
+      </x:c>
+      <x:c r="J10" s="664" t="str">
+        <x:v>Pre-tax run-rate needed to offset PPA, financing costs, and new shares</x:v>
+      </x:c>
+      <x:c r="K10" s="664"/>
+      <x:c r="L10" s="664"/>
+      <x:c r="M10" s="664"/>
+      <x:c r="N10" s="664"/>
+      <x:c r="O10" s="664"/>
+    </x:row>
+    <x:row r="11" ht="25" customHeight="1">
+      <x:c r="A11" s="824" t="str">
+        <x:v>New debt</x:v>
+      </x:c>
+      <x:c r="B11" s="794" t="n">
+        <x:f>'Sources &amp; Uses'!B41</x:f>
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="C11" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D11" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E11" s="664" t="str">
+        <x:v>Term loan / bridge plus senior notes</x:v>
+      </x:c>
+      <x:c r="F11" s="664"/>
+      <x:c r="G11" s="538"/>
+      <x:c r="H11" s="824" t="str">
+        <x:v>FY2027E annualized breakeven synergies — excl. PPA</x:v>
+      </x:c>
+      <x:c r="I11" s="841" t="n">
+        <x:f>I30</x:f>
+        <x:v>288.1442811035027</x:v>
+      </x:c>
+      <x:c r="J11" s="664" t="str">
+        <x:v>Pre-tax run-rate needed to offset financing costs and new shares only</x:v>
+      </x:c>
+      <x:c r="K11" s="664"/>
+      <x:c r="L11" s="664"/>
+      <x:c r="M11" s="664"/>
+      <x:c r="N11" s="664"/>
+      <x:c r="O11" s="664"/>
+    </x:row>
+    <x:row r="12" ht="25" customHeight="1">
+      <x:c r="A12" s="824" t="str">
+        <x:v>New debt interest rate</x:v>
+      </x:c>
+      <x:c r="B12" s="733" t="n">
+        <x:f>'Sources &amp; Uses'!B16</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="C12" s="436" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="D12" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E12" s="664" t="str">
+        <x:v>Blended pre-tax rate</x:v>
+      </x:c>
+      <x:c r="F12" s="664"/>
+      <x:c r="G12" s="538"/>
+      <x:c r="H12" s="824" t="str">
+        <x:v>FY2027E headline EPS result</x:v>
+      </x:c>
+      <x:c r="I12" s="827" t="str">
+        <x:f>IF(I6&gt;=0,"Accretive","Dilutive")</x:f>
+        <x:v>Dilutive</x:v>
+      </x:c>
+      <x:c r="J12" s="664" t="str">
+        <x:v>Negative EPS change means dilution</x:v>
+      </x:c>
+      <x:c r="K12" s="664"/>
+      <x:c r="L12" s="664"/>
+      <x:c r="M12" s="664"/>
+      <x:c r="N12" s="664"/>
+      <x:c r="O12" s="664"/>
+    </x:row>
+    <x:row r="13" ht="25" customHeight="1">
+      <x:c r="A13" s="824" t="str">
+        <x:v>ROK cash used</x:v>
+      </x:c>
+      <x:c r="B13" s="794" t="n">
+        <x:f>'Sources &amp; Uses'!I21</x:f>
+        <x:v>211.95520000000033</x:v>
+      </x:c>
+      <x:c r="C13" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D13" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E13" s="664" t="str">
+        <x:v>Balance-sheet cash used as a transaction source</x:v>
+      </x:c>
+      <x:c r="F13" s="664"/>
+      <x:c r="G13" s="538"/>
+      <x:c r="H13" s="824" t="str">
+        <x:v>FY2028E headline EPS result</x:v>
+      </x:c>
+      <x:c r="I13" s="827" t="str">
+        <x:f>IF(I8&gt;=0,"Accretive","Dilutive")</x:f>
+        <x:v>Dilutive</x:v>
+      </x:c>
+      <x:c r="J13" s="664" t="str">
+        <x:v>Negative EPS change means dilution</x:v>
+      </x:c>
+      <x:c r="K13" s="664"/>
+      <x:c r="L13" s="664"/>
+      <x:c r="M13" s="664"/>
+      <x:c r="N13" s="664"/>
+      <x:c r="O13" s="664"/>
+    </x:row>
+    <x:row r="14" ht="25" customHeight="1">
+      <x:c r="A14" s="824" t="str">
+        <x:v>Debt financing fees</x:v>
+      </x:c>
+      <x:c r="B14" s="794" t="n">
+        <x:f>'Sources &amp; Uses'!B25</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C14" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D14" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E14" s="664" t="str">
+        <x:v>Capitalized and amortized through interest expense</x:v>
+      </x:c>
+      <x:c r="F14" s="664"/>
+      <x:c r="G14" s="538"/>
+      <x:c r="H14" s="824" t="str">
+        <x:v>Target holders’ pro forma ownership</x:v>
+      </x:c>
+      <x:c r="I14" s="842" t="n">
+        <x:f>'Sources &amp; Uses'!I36</x:f>
+        <x:v>0.1629086315972937</x:v>
+      </x:c>
+      <x:c r="J14" s="664" t="str">
+        <x:v>Target shareholders participate in the combined company through stock consideration</x:v>
+      </x:c>
+      <x:c r="K14" s="664"/>
+      <x:c r="L14" s="664"/>
+      <x:c r="M14" s="664"/>
+      <x:c r="N14" s="664"/>
+      <x:c r="O14" s="664"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="824" t="str">
+        <x:v>One-time transaction fees</x:v>
+      </x:c>
+      <x:c r="B15" s="794" t="n">
+        <x:f>'Sources &amp; Uses'!B24</x:f>
+        <x:v>134.5792</x:v>
+      </x:c>
+      <x:c r="C15" s="436" t="str">
+        <x:v>$mm</x:v>
+      </x:c>
+      <x:c r="D15" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E15" s="664" t="str">
+        <x:v>Excluded from headline recurring EPS; shown separately</x:v>
+      </x:c>
+      <x:c r="F15" s="664"/>
+      <x:c r="G15" s="538"/>
+      <x:c r="H15" s="538"/>
+      <x:c r="I15" s="538"/>
+      <x:c r="J15" s="538"/>
+      <x:c r="K15" s="538"/>
+      <x:c r="L15" s="538"/>
+      <x:c r="M15" s="538"/>
+      <x:c r="N15" s="538"/>
+      <x:c r="O15" s="538"/>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="824" t="str">
+        <x:v>New ROK shares issued</x:v>
+      </x:c>
+      <x:c r="B16" s="560" t="n">
+        <x:f>'Sources &amp; Uses'!I33</x:f>
+        <x:v>21.834613512573874</x:v>
+      </x:c>
+      <x:c r="C16" s="436" t="str">
+        <x:v>mm shares</x:v>
+      </x:c>
+      <x:c r="D16" s="436" t="str">
+        <x:v>Sources &amp; Uses</x:v>
+      </x:c>
+      <x:c r="E16" s="664" t="str">
+        <x:v>Direct stock consideration divided by Rockwell share price</x:v>
+      </x:c>
+      <x:c r="F16" s="664"/>
+      <x:c r="G16" s="538"/>
+      <x:c r="H16" s="538"/>
+      <x:c r="I16" s="538"/>
+      <x:c r="J16" s="538"/>
+      <x:c r="K16" s="538"/>
+      <x:c r="L16" s="538"/>
+      <x:c r="M16" s="538"/>
+      <x:c r="N16" s="538"/>
+      <x:c r="O16" s="538"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="538"/>
+      <x:c r="B17" s="538"/>
+      <x:c r="C17" s="538"/>
+      <x:c r="D17" s="538"/>
+      <x:c r="E17" s="538"/>
+      <x:c r="F17" s="538"/>
+      <x:c r="G17" s="538"/>
+      <x:c r="H17" s="538"/>
+      <x:c r="I17" s="538"/>
+      <x:c r="J17" s="538"/>
+      <x:c r="K17" s="538"/>
+      <x:c r="L17" s="538"/>
+      <x:c r="M17" s="538"/>
+      <x:c r="N17" s="538"/>
+      <x:c r="O17" s="538"/>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1">
+      <x:c r="A18" s="538"/>
+      <x:c r="B18" s="538"/>
+      <x:c r="C18" s="538"/>
+      <x:c r="D18" s="538"/>
+      <x:c r="E18" s="538"/>
+      <x:c r="F18" s="538"/>
+      <x:c r="G18" s="538"/>
+      <x:c r="H18" s="538"/>
+      <x:c r="I18" s="538"/>
+      <x:c r="J18" s="538"/>
+      <x:c r="K18" s="538"/>
+      <x:c r="L18" s="538"/>
+      <x:c r="M18" s="538"/>
+      <x:c r="N18" s="538"/>
+      <x:c r="O18" s="538"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="822" t="str">
+        <x:v>PRO FORMA EARNINGS AND EPS</x:v>
+      </x:c>
+      <x:c r="B19" s="822"/>
+      <x:c r="C19" s="822"/>
+      <x:c r="D19" s="822"/>
+      <x:c r="E19" s="822"/>
+      <x:c r="F19" s="822"/>
+      <x:c r="G19" s="822"/>
+      <x:c r="H19" s="822" t="str">
+        <x:v>EPS BREAKEVEN SYNERGY ANALYSIS</x:v>
+      </x:c>
+      <x:c r="I19" s="822"/>
+      <x:c r="J19" s="822"/>
+      <x:c r="K19" s="822"/>
+      <x:c r="L19" s="822"/>
+      <x:c r="M19" s="822"/>
+      <x:c r="N19" s="822"/>
+      <x:c r="O19" s="822"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="824" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="B20" s="843" t="n">
+        <x:f>'Purchase Accounting'!B30</x:f>
+        <x:v>46660</x:v>
+      </x:c>
+      <x:c r="C20" s="843" t="n">
+        <x:f>'Purchase Accounting'!C30</x:f>
+        <x:v>47026</x:v>
+      </x:c>
+      <x:c r="D20" s="843" t="n">
+        <x:f>'Purchase Accounting'!D30</x:f>
+        <x:v>47391</x:v>
+      </x:c>
+      <x:c r="E20" s="843" t="n">
+        <x:f>'Purchase Accounting'!E30</x:f>
+        <x:v>47756</x:v>
+      </x:c>
+      <x:c r="F20" s="664" t="str">
+        <x:v>Source / calculation</x:v>
+      </x:c>
+      <x:c r="G20" s="664"/>
+      <x:c r="H20" s="824" t="str">
+        <x:v>Fiscal year ended</x:v>
+      </x:c>
+      <x:c r="I20" s="843" t="n">
+        <x:f>B20</x:f>
+        <x:v>46660</x:v>
+      </x:c>
+      <x:c r="J20" s="843" t="n">
+        <x:f>C20</x:f>
+        <x:v>47026</x:v>
+      </x:c>
+      <x:c r="K20" s="843" t="n">
+        <x:f>D20</x:f>
+        <x:v>47391</x:v>
+      </x:c>
+      <x:c r="L20" s="843" t="n">
+        <x:f>E20</x:f>
+        <x:v>47756</x:v>
+      </x:c>
+      <x:c r="M20" s="664" t="str">
+        <x:v>Calculation</x:v>
+      </x:c>
+      <x:c r="N20" s="538"/>
+      <x:c r="O20" s="538"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="824"/>
+      <x:c r="B21" s="436"/>
+      <x:c r="C21" s="436"/>
+      <x:c r="D21" s="436"/>
+      <x:c r="E21" s="436"/>
+      <x:c r="F21" s="664"/>
+      <x:c r="G21" s="664"/>
+      <x:c r="H21" s="824"/>
+      <x:c r="I21" s="436"/>
+      <x:c r="J21" s="436"/>
+      <x:c r="K21" s="436"/>
+      <x:c r="L21" s="436"/>
+      <x:c r="M21" s="664"/>
+      <x:c r="N21" s="538"/>
+      <x:c r="O21" s="538"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="824" t="str">
+        <x:v>ROK standalone adjusted net income</x:v>
+      </x:c>
+      <x:c r="B22" s="794" t="n">
+        <x:f>'ROK Forecast'!F14</x:f>
+        <x:v>1551.3777816576</x:v>
+      </x:c>
+      <x:c r="C22" s="794" t="n">
+        <x:f>'ROK Forecast'!G14</x:f>
+        <x:v>1631.3047649685998</x:v>
+      </x:c>
+      <x:c r="D22" s="794" t="n">
+        <x:f>'ROK Forecast'!H14</x:f>
+        <x:v>1699.1670431912937</x:v>
+      </x:c>
+      <x:c r="E22" s="794" t="n">
+        <x:f>'ROK Forecast'!I14</x:f>
+        <x:v>1769.8523921880515</x:v>
+      </x:c>
+      <x:c r="F22" s="664" t="str">
+        <x:v>ROK Forecast</x:v>
+      </x:c>
+      <x:c r="G22" s="664"/>
+      <x:c r="H22" s="824" t="str">
+        <x:v>After-tax earnings shortfall — including PPA</x:v>
+      </x:c>
+      <x:c r="I22" s="744" t="n">
+        <x:f>MAX(0,B39*B38-B34)</x:f>
+        <x:v>349.36103156921695</x:v>
+      </x:c>
+      <x:c r="J22" s="744" t="n">
+        <x:f>MAX(0,C39*C38-C34)</x:f>
+        <x:v>660.5416686035401</x:v>
+      </x:c>
+      <x:c r="K22" s="744" t="n">
+        <x:f>MAX(0,D39*D38-D34)</x:f>
+        <x:v>593.8283595643836</x:v>
+      </x:c>
+      <x:c r="L22" s="744" t="n">
+        <x:f>MAX(0,E39*E38-E34)</x:f>
+        <x:v>558.4884586515095</x:v>
+      </x:c>
+      <x:c r="M22" s="664" t="str">
+        <x:v>Buyer EPS × pro forma shares less pro forma net income</x:v>
+      </x:c>
+      <x:c r="N22" s="538"/>
+      <x:c r="O22" s="538"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="824" t="str">
+        <x:v>CGNX standalone net income</x:v>
+      </x:c>
+      <x:c r="B23" s="794" t="n">
+        <x:f>'CGNX Operating Model'!F37</x:f>
+        <x:v>279.3364799999999</x:v>
+      </x:c>
+      <x:c r="C23" s="794" t="n">
+        <x:f>'CGNX Operating Model'!G37</x:f>
+        <x:v>309.19864320000005</x:v>
+      </x:c>
+      <x:c r="D23" s="794" t="n">
+        <x:f>'CGNX Operating Model'!H37</x:f>
+        <x:v>338.88386016</x:v>
+      </x:c>
+      <x:c r="E23" s="794" t="n">
+        <x:f>'CGNX Operating Model'!I37</x:f>
+        <x:v>364.58159558976</x:v>
+      </x:c>
+      <x:c r="F23" s="664" t="str">
+        <x:v>CGNX Operating Model</x:v>
+      </x:c>
+      <x:c r="G23" s="664"/>
+      <x:c r="H23" s="824" t="str">
+        <x:v>Pre-tax synergies recognized — including PPA</x:v>
+      </x:c>
+      <x:c r="I23" s="744" t="n">
+        <x:f>I22/(1-$B$7)</x:f>
+        <x:v>442.2291538850847</x:v>
+      </x:c>
+      <x:c r="J23" s="744" t="n">
+        <x:f>J22/(1-$B$7)</x:f>
+        <x:v>836.1286944348608</x:v>
+      </x:c>
+      <x:c r="K23" s="744" t="n">
+        <x:f>K22/(1-$B$7)</x:f>
+        <x:v>751.6814678030172</x:v>
+      </x:c>
+      <x:c r="L23" s="744" t="n">
+        <x:f>L22/(1-$B$7)</x:f>
+        <x:v>706.947416014569</x:v>
+      </x:c>
+      <x:c r="M23" s="664" t="str">
+        <x:v>After-tax shortfall ÷ (1 − tax rate)</x:v>
+      </x:c>
+      <x:c r="N23" s="538"/>
+      <x:c r="O23" s="538"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="824" t="str">
+        <x:v>Ownership factor</x:v>
+      </x:c>
+      <x:c r="B24" s="733" t="n">
+        <x:f>$B$6</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C24" s="733" t="n">
+        <x:f>1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D24" s="733" t="n">
+        <x:f>1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E24" s="733" t="n">
+        <x:f>1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F24" s="664" t="str">
+        <x:v>Close-date convention</x:v>
+      </x:c>
+      <x:c r="G24" s="664"/>
+      <x:c r="H24" s="824" t="str">
+        <x:v>Annualized pre-tax synergy run-rate — including PPA</x:v>
+      </x:c>
+      <x:c r="I24" s="847" t="n">
+        <x:f>I23/B24</x:f>
+        <x:v>884.4583077701694</x:v>
+      </x:c>
+      <x:c r="J24" s="847" t="n">
+        <x:f>J23/C24</x:f>
+        <x:v>836.1286944348608</x:v>
+      </x:c>
+      <x:c r="K24" s="847" t="n">
+        <x:f>K23/D24</x:f>
+        <x:v>751.6814678030172</x:v>
+      </x:c>
+      <x:c r="L24" s="847" t="n">
+        <x:f>L23/E24</x:f>
+        <x:v>706.947416014569</x:v>
+      </x:c>
+      <x:c r="M24" s="664" t="str">
+        <x:v>Recognized synergies ÷ ownership factor</x:v>
+      </x:c>
+      <x:c r="N24" s="538"/>
+      <x:c r="O24" s="538"/>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1">
+      <x:c r="A25" s="824" t="str">
+        <x:v>Acquired CGNX net income contribution</x:v>
+      </x:c>
+      <x:c r="B25" s="744" t="n">
+        <x:f>B23*B24</x:f>
+        <x:v>139.66823999999994</x:v>
+      </x:c>
+      <x:c r="C25" s="744" t="n">
+        <x:f>C23*C24</x:f>
+        <x:v>309.19864320000005</x:v>
+      </x:c>
+      <x:c r="D25" s="744" t="n">
+        <x:f>D23*D24</x:f>
+        <x:v>338.88386016</x:v>
+      </x:c>
+      <x:c r="E25" s="744" t="n">
+        <x:f>E23*E24</x:f>
+        <x:v>364.58159558976</x:v>
+      </x:c>
+      <x:c r="F25" s="664" t="str">
+        <x:v>Target net income × ownership factor</x:v>
+      </x:c>
+      <x:c r="G25" s="664"/>
+      <x:c r="H25" s="824" t="str">
+        <x:v>Run-rate / CGNX revenue</x:v>
+      </x:c>
+      <x:c r="I25" s="848" t="n">
+        <x:f>I24/'CGNX Operating Model'!F20</x:f>
+        <x:v>0.7117803861018585</x:v>
+      </x:c>
+      <x:c r="J25" s="848" t="n">
+        <x:f>J24/'CGNX Operating Model'!G20</x:f>
+        <x:v>0.6230430030483132</x:v>
+      </x:c>
+      <x:c r="K25" s="848" t="n">
+        <x:f>K24/'CGNX Operating Model'!H20</x:f>
+        <x:v>0.5234738128801891</x:v>
+      </x:c>
+      <x:c r="L25" s="848" t="n">
+        <x:f>L24/'CGNX Operating Model'!I20</x:f>
+        <x:v>0.46227309885251616</x:v>
+      </x:c>
+      <x:c r="M25" s="664" t="str">
+        <x:v>Annualized run-rate ÷ target revenue</x:v>
+      </x:c>
+      <x:c r="N25" s="538"/>
+      <x:c r="O25" s="538"/>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="824"/>
+      <x:c r="B26" s="716"/>
+      <x:c r="C26" s="716"/>
+      <x:c r="D26" s="716"/>
+      <x:c r="E26" s="716"/>
+      <x:c r="F26" s="664"/>
+      <x:c r="G26" s="664"/>
+      <x:c r="H26" s="824" t="str">
+        <x:v>Run-rate / CGNX EBITDA</x:v>
+      </x:c>
+      <x:c r="I26" s="848" t="n">
+        <x:f>I24/'CGNX Operating Model'!F32</x:f>
+        <x:v>2.3965669565719154</x:v>
+      </x:c>
+      <x:c r="J26" s="848" t="n">
+        <x:f>J24/'CGNX Operating Model'!G32</x:f>
+        <x:v>2.042763944420699</x:v>
+      </x:c>
+      <x:c r="K26" s="848" t="n">
+        <x:f>K24/'CGNX Operating Model'!H32</x:f>
+        <x:v>1.677800682308299</x:v>
+      </x:c>
+      <x:c r="L26" s="848" t="n">
+        <x:f>L24/'CGNX Operating Model'!I32</x:f>
+        <x:v>1.4675336471508453</x:v>
+      </x:c>
+      <x:c r="M26" s="664" t="str">
+        <x:v>Annualized run-rate ÷ target EBITDA</x:v>
+      </x:c>
+      <x:c r="N26" s="538"/>
+      <x:c r="O26" s="538"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="824" t="str">
+        <x:v>New debt interest expense</x:v>
+      </x:c>
+      <x:c r="B27" s="794" t="n">
+        <x:f>$B$11*$B$12*B24</x:f>
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C27" s="794" t="n">
+        <x:f>$B$11*$B$12*C24</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="D27" s="794" t="n">
+        <x:f>$B$11*$B$12*D24</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="E27" s="794" t="n">
+        <x:f>$B$11*$B$12*E24</x:f>
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="F27" s="664" t="str">
+        <x:v>New debt × interest rate × ownership</x:v>
+      </x:c>
+      <x:c r="G27" s="664"/>
+      <x:c r="H27" s="824"/>
+      <x:c r="I27" s="436"/>
+      <x:c r="J27" s="436"/>
+      <x:c r="K27" s="436"/>
+      <x:c r="L27" s="436"/>
+      <x:c r="M27" s="664"/>
+      <x:c r="N27" s="538"/>
+      <x:c r="O27" s="538"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="824" t="str">
+        <x:v>Foregone cash interest income</x:v>
+      </x:c>
+      <x:c r="B28" s="794" t="n">
+        <x:f>$B$13*$B$8*B24</x:f>
+        <x:v>4.239104000000006</x:v>
+      </x:c>
+      <x:c r="C28" s="794" t="n">
+        <x:f>$B$13*$B$8*C24</x:f>
+        <x:v>8.478208000000013</x:v>
+      </x:c>
+      <x:c r="D28" s="794" t="n">
+        <x:f>$B$13*$B$8*D24</x:f>
+        <x:v>8.478208000000013</x:v>
+      </x:c>
+      <x:c r="E28" s="794" t="n">
+        <x:f>$B$13*$B$8*E24</x:f>
+        <x:v>8.478208000000013</x:v>
+      </x:c>
+      <x:c r="F28" s="664" t="str">
+        <x:v>ROK cash used × foregone yield × ownership</x:v>
+      </x:c>
+      <x:c r="G28" s="664"/>
+      <x:c r="H28" s="824" t="str">
+        <x:v>After-tax earnings shortfall — excluding PPA</x:v>
+      </x:c>
+      <x:c r="I28" s="744" t="n">
+        <x:f>MAX(0,B39*B38-B43)</x:f>
+        <x:v>113.81699103588358</x:v>
+      </x:c>
+      <x:c r="J28" s="744" t="n">
+        <x:f>MAX(0,C39*C38-C43)</x:f>
+        <x:v>216.03297953687343</x:v>
+      </x:c>
+      <x:c r="K28" s="744" t="n">
+        <x:f>MAX(0,D39*D38-D43)</x:f>
+        <x:v>202.47845449771694</x:v>
+      </x:c>
+      <x:c r="L28" s="744" t="n">
+        <x:f>MAX(0,E39*E38-E43)</x:f>
+        <x:v>193.71794558484294</x:v>
+      </x:c>
+      <x:c r="M28" s="664" t="str">
+        <x:v>Breakeven calculation before PPA expense</x:v>
+      </x:c>
+      <x:c r="N28" s="538"/>
+      <x:c r="O28" s="538"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="824" t="str">
+        <x:v>Debt-fee amortization</x:v>
+      </x:c>
+      <x:c r="B29" s="794" t="n">
+        <x:f>($B$14/$B$9)*B24</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C29" s="794" t="n">
+        <x:f>($B$14/$B$9)*C24</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D29" s="794" t="n">
+        <x:f>($B$14/$B$9)*D24</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E29" s="794" t="n">
+        <x:f>($B$14/$B$9)*E24</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F29" s="664" t="str">
+        <x:v>Debt fees ÷ amortization period × ownership</x:v>
+      </x:c>
+      <x:c r="G29" s="664"/>
+      <x:c r="H29" s="824" t="str">
+        <x:v>Pre-tax synergies recognized — excluding PPA</x:v>
+      </x:c>
+      <x:c r="I29" s="744" t="n">
+        <x:f>I28/(1-$B$7)</x:f>
+        <x:v>144.07214055175135</x:v>
+      </x:c>
+      <x:c r="J29" s="744" t="n">
+        <x:f>J28/(1-$B$7)</x:f>
+        <x:v>273.4594677681942</x:v>
+      </x:c>
+      <x:c r="K29" s="744" t="n">
+        <x:f>K28/(1-$B$7)</x:f>
+        <x:v>256.30184113635056</x:v>
+      </x:c>
+      <x:c r="L29" s="744" t="n">
+        <x:f>L28/(1-$B$7)</x:f>
+        <x:v>245.21258934790245</x:v>
+      </x:c>
+      <x:c r="M29" s="664" t="str">
+        <x:v>After-tax shortfall ÷ (1 − tax rate)</x:v>
+      </x:c>
+      <x:c r="N29" s="538"/>
+      <x:c r="O29" s="538"/>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="824" t="str">
+        <x:v>Total incremental financing costs</x:v>
+      </x:c>
+      <x:c r="B30" s="744" t="n">
+        <x:f>SUM(B27:B29)</x:f>
+        <x:v>128.239104</x:v>
+      </x:c>
+      <x:c r="C30" s="744" t="n">
+        <x:f>SUM(C27:C29)</x:f>
+        <x:v>256.478208</x:v>
+      </x:c>
+      <x:c r="D30" s="744" t="n">
+        <x:f>SUM(D27:D29)</x:f>
+        <x:v>256.478208</x:v>
+      </x:c>
+      <x:c r="E30" s="744" t="n">
+        <x:f>SUM(E27:E29)</x:f>
+        <x:v>256.478208</x:v>
+      </x:c>
+      <x:c r="F30" s="664" t="str">
+        <x:v>Sum of financing costs</x:v>
+      </x:c>
+      <x:c r="G30" s="664"/>
+      <x:c r="H30" s="824" t="str">
+        <x:v>Annualized pre-tax synergy run-rate — excluding PPA</x:v>
+      </x:c>
+      <x:c r="I30" s="847" t="n">
+        <x:f>I29/B24</x:f>
+        <x:v>288.1442811035027</x:v>
+      </x:c>
+      <x:c r="J30" s="847" t="n">
+        <x:f>J29/C24</x:f>
+        <x:v>273.4594677681942</x:v>
+      </x:c>
+      <x:c r="K30" s="847" t="n">
+        <x:f>K29/D24</x:f>
+        <x:v>256.30184113635056</x:v>
+      </x:c>
+      <x:c r="L30" s="847" t="n">
+        <x:f>L29/E24</x:f>
+        <x:v>245.21258934790245</x:v>
+      </x:c>
+      <x:c r="M30" s="664" t="str">
+        <x:v>Recognized synergies ÷ ownership factor</x:v>
+      </x:c>
+      <x:c r="N30" s="538"/>
+      <x:c r="O30" s="538"/>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="A31" s="824" t="str">
+        <x:v>Tax benefit on financing costs</x:v>
+      </x:c>
+      <x:c r="B31" s="744" t="n">
+        <x:f>B30*$B$7</x:f>
+        <x:v>26.93021184</x:v>
+      </x:c>
+      <x:c r="C31" s="744" t="n">
+        <x:f>C30*$B$7</x:f>
+        <x:v>53.86042368</x:v>
+      </x:c>
+      <x:c r="D31" s="744" t="n">
+        <x:f>D30*$B$7</x:f>
+        <x:v>53.86042368</x:v>
+      </x:c>
+      <x:c r="E31" s="744" t="n">
+        <x:f>E30*$B$7</x:f>
+        <x:v>53.86042368</x:v>
+      </x:c>
+      <x:c r="F31" s="664" t="str">
+        <x:v>Financing costs × buyer tax rate</x:v>
+      </x:c>
+      <x:c r="G31" s="664"/>
+      <x:c r="H31" s="824" t="str">
+        <x:v>Run-rate / CGNX revenue</x:v>
+      </x:c>
+      <x:c r="I31" s="848" t="n">
+        <x:f>I30/'CGNX Operating Model'!F20</x:f>
+        <x:v>0.23188820304482752</x:v>
+      </x:c>
+      <x:c r="J31" s="848" t="n">
+        <x:f>J30/'CGNX Operating Model'!G20</x:f>
+        <x:v>0.20376888048967975</x:v>
+      </x:c>
+      <x:c r="K31" s="848" t="n">
+        <x:f>K30/'CGNX Operating Model'!H20</x:f>
+        <x:v>0.17848957008345098</x:v>
+      </x:c>
+      <x:c r="L31" s="848" t="n">
+        <x:f>L30/'CGNX Operating Model'!I20</x:f>
+        <x:v>0.160344575830755</x:v>
+      </x:c>
+      <x:c r="M31" s="664" t="str">
+        <x:v>Annualized run-rate ÷ target revenue</x:v>
+      </x:c>
+      <x:c r="N31" s="538"/>
+      <x:c r="O31" s="538"/>
+    </x:row>
+    <x:row r="32" ht="18" customHeight="1">
+      <x:c r="A32" s="824" t="str">
+        <x:v>After-tax financing costs</x:v>
+      </x:c>
+      <x:c r="B32" s="744" t="n">
+        <x:f>B30-B31</x:f>
+        <x:v>101.30889216</x:v>
+      </x:c>
+      <x:c r="C32" s="744" t="n">
+        <x:f>C30-C31</x:f>
+        <x:v>202.61778432</x:v>
+      </x:c>
+      <x:c r="D32" s="744" t="n">
+        <x:f>D30-D31</x:f>
+        <x:v>202.61778432</x:v>
+      </x:c>
+      <x:c r="E32" s="744" t="n">
+        <x:f>E30-E31</x:f>
+        <x:v>202.61778432</x:v>
+      </x:c>
+      <x:c r="F32" s="664" t="str">
+        <x:v>Pre-tax costs less tax benefit</x:v>
+      </x:c>
+      <x:c r="G32" s="664"/>
+      <x:c r="H32" s="824" t="str">
+        <x:v>Run-rate / CGNX EBITDA</x:v>
+      </x:c>
+      <x:c r="I32" s="848" t="n">
+        <x:f>I30/'CGNX Operating Model'!F32</x:f>
+        <x:v>0.7807683604202951</x:v>
+      </x:c>
+      <x:c r="J32" s="848" t="n">
+        <x:f>J30/'CGNX Operating Model'!G32</x:f>
+        <x:v>0.6680946901300975</x:v>
+      </x:c>
+      <x:c r="K32" s="848" t="n">
+        <x:f>K30/'CGNX Operating Model'!H32</x:f>
+        <x:v>0.5720819553956763</x:v>
+      </x:c>
+      <x:c r="L32" s="848" t="n">
+        <x:f>L30/'CGNX Operating Model'!I32</x:f>
+        <x:v>0.5090303994627144</x:v>
+      </x:c>
+      <x:c r="M32" s="664" t="str">
+        <x:v>Annualized run-rate ÷ target EBITDA</x:v>
+      </x:c>
+      <x:c r="N32" s="538"/>
+      <x:c r="O32" s="538"/>
+    </x:row>
+    <x:row r="33" ht="18" customHeight="1">
+      <x:c r="A33" s="824" t="str">
+        <x:v>After-tax purchase-accounting expense</x:v>
+      </x:c>
+      <x:c r="B33" s="794" t="n">
+        <x:f>'Purchase Accounting'!B43</x:f>
+        <x:v>235.5440405333333</x:v>
+      </x:c>
+      <x:c r="C33" s="794" t="n">
+        <x:f>'Purchase Accounting'!C43</x:f>
+        <x:v>444.50868906666665</x:v>
+      </x:c>
+      <x:c r="D33" s="794" t="n">
+        <x:f>'Purchase Accounting'!D43</x:f>
+        <x:v>391.3499050666666</x:v>
+      </x:c>
+      <x:c r="E33" s="794" t="n">
+        <x:f>'Purchase Accounting'!E43</x:f>
+        <x:v>364.77051306666664</x:v>
+      </x:c>
+      <x:c r="F33" s="664" t="str">
+        <x:v>Purchase Accounting</x:v>
+      </x:c>
+      <x:c r="G33" s="664"/>
+      <x:c r="H33" s="824"/>
+      <x:c r="I33" s="436"/>
+      <x:c r="J33" s="436"/>
+      <x:c r="K33" s="436"/>
+      <x:c r="L33" s="436"/>
+      <x:c r="M33" s="664"/>
+      <x:c r="N33" s="538"/>
+      <x:c r="O33" s="538"/>
+    </x:row>
+    <x:row r="34" ht="18" customHeight="1">
+      <x:c r="A34" s="832" t="str">
+        <x:v>Pro forma net income — including PPA</x:v>
+      </x:c>
+      <x:c r="B34" s="844" t="n">
+        <x:f>B22+B25-B32-B33</x:f>
+        <x:v>1354.1930889642667</x:v>
+      </x:c>
+      <x:c r="C34" s="844" t="n">
+        <x:f>C22+C25-C32-C33</x:f>
+        <x:v>1293.3769347819332</x:v>
+      </x:c>
+      <x:c r="D34" s="844" t="n">
+        <x:f>D22+D25-D32-D33</x:f>
+        <x:v>1444.083213964627</x:v>
+      </x:c>
+      <x:c r="E34" s="844" t="n">
+        <x:f>E22+E25-E32-E33</x:f>
+        <x:v>1567.045690391145</x:v>
+      </x:c>
+      <x:c r="F34" s="755" t="str">
+        <x:v>Buyer + target contribution − financing − PPA</x:v>
+      </x:c>
+      <x:c r="G34" s="755"/>
+      <x:c r="H34" s="538"/>
+      <x:c r="I34" s="538"/>
+      <x:c r="J34" s="538"/>
+      <x:c r="K34" s="538"/>
+      <x:c r="L34" s="538"/>
+      <x:c r="M34" s="538"/>
+      <x:c r="N34" s="538"/>
+      <x:c r="O34" s="538"/>
+    </x:row>
+    <x:row r="35" ht="18" customHeight="1">
+      <x:c r="A35" s="824"/>
+      <x:c r="B35" s="716"/>
+      <x:c r="C35" s="716"/>
+      <x:c r="D35" s="716"/>
+      <x:c r="E35" s="716"/>
+      <x:c r="F35" s="664"/>
+      <x:c r="G35" s="664"/>
+      <x:c r="H35" s="538"/>
+      <x:c r="I35" s="538"/>
+      <x:c r="J35" s="538"/>
+      <x:c r="K35" s="538"/>
+      <x:c r="L35" s="538"/>
+      <x:c r="M35" s="538"/>
+      <x:c r="N35" s="538"/>
+      <x:c r="O35" s="538"/>
+    </x:row>
+    <x:row r="36" ht="18" customHeight="1">
+      <x:c r="A36" s="824" t="str">
+        <x:v>ROK diluted shares</x:v>
+      </x:c>
+      <x:c r="B36" s="560" t="n">
+        <x:f>'ROK Forecast'!F13</x:f>
+        <x:v>111.2976384</x:v>
+      </x:c>
+      <x:c r="C36" s="560" t="n">
+        <x:f>'ROK Forecast'!G13</x:f>
+        <x:v>110.4072572928</x:v>
+      </x:c>
+      <x:c r="D36" s="560" t="n">
+        <x:f>'ROK Forecast'!H13</x:f>
+        <x:v>109.52399923445759</x:v>
+      </x:c>
+      <x:c r="E36" s="560" t="n">
+        <x:f>'ROK Forecast'!I13</x:f>
+        <x:v>108.64780724058193</x:v>
+      </x:c>
+      <x:c r="F36" s="664" t="str">
+        <x:v>ROK Forecast</x:v>
+      </x:c>
+      <x:c r="G36" s="664"/>
+      <x:c r="H36" s="822" t="str">
+        <x:v>RECONCILIATION CHECKS</x:v>
+      </x:c>
+      <x:c r="I36" s="822"/>
+      <x:c r="J36" s="822"/>
+      <x:c r="K36" s="822"/>
+      <x:c r="L36" s="822"/>
+      <x:c r="M36" s="822"/>
+      <x:c r="N36" s="822"/>
+      <x:c r="O36" s="822"/>
+    </x:row>
+    <x:row r="37" ht="18" customHeight="1">
+      <x:c r="A37" s="824" t="str">
+        <x:v>Weighted new shares issued</x:v>
+      </x:c>
+      <x:c r="B37" s="560" t="n">
+        <x:f>$B$16*B24</x:f>
+        <x:v>10.917306756286937</x:v>
+      </x:c>
+      <x:c r="C37" s="560" t="n">
+        <x:f>$B$16*C24</x:f>
+        <x:v>21.834613512573874</x:v>
+      </x:c>
+      <x:c r="D37" s="560" t="n">
+        <x:f>$B$16*D24</x:f>
+        <x:v>21.834613512573874</x:v>
+      </x:c>
+      <x:c r="E37" s="560" t="n">
+        <x:f>$B$16*E24</x:f>
+        <x:v>21.834613512573874</x:v>
+      </x:c>
+      <x:c r="F37" s="664" t="str">
+        <x:v>New shares × ownership factor</x:v>
+      </x:c>
+      <x:c r="G37" s="664"/>
+      <x:c r="H37" s="824" t="str">
+        <x:v>Buyer EPS tie-out</x:v>
+      </x:c>
+      <x:c r="I37" s="849" t="n">
+        <x:f>B39-B22/B36</x:f>
+        <x:v>1.7763568394002505e-15</x:v>
+      </x:c>
+      <x:c r="J37" s="664" t="str">
+        <x:v>Must equal zero</x:v>
+      </x:c>
+      <x:c r="K37" s="664"/>
+      <x:c r="L37" s="664"/>
+      <x:c r="M37" s="664"/>
+      <x:c r="N37" s="664"/>
+      <x:c r="O37" s="664"/>
+    </x:row>
+    <x:row r="38" ht="18" customHeight="1">
+      <x:c r="A38" s="824" t="str">
+        <x:v>Pro forma diluted shares</x:v>
+      </x:c>
+      <x:c r="B38" s="749" t="n">
+        <x:f>SUM(B36:B37)</x:f>
+        <x:v>122.21494515628693</x:v>
+      </x:c>
+      <x:c r="C38" s="749" t="n">
+        <x:f>SUM(C36:C37)</x:f>
+        <x:v>132.24187080537388</x:v>
+      </x:c>
+      <x:c r="D38" s="749" t="n">
+        <x:f>SUM(D36:D37)</x:f>
+        <x:v>131.35861274703146</x:v>
+      </x:c>
+      <x:c r="E38" s="749" t="n">
+        <x:f>SUM(E36:E37)</x:f>
+        <x:v>130.4824207531558</x:v>
+      </x:c>
+      <x:c r="F38" s="664" t="str">
+        <x:v>Buyer shares plus weighted new shares</x:v>
+      </x:c>
+      <x:c r="G38" s="664"/>
+      <x:c r="H38" s="824" t="str">
+        <x:v>Pro forma net-income identity</x:v>
+      </x:c>
+      <x:c r="I38" s="849" t="n">
+        <x:f>B34-(B22+B25-B32-B33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" s="664" t="str">
+        <x:v>Buyer plus target less financing and PPA</x:v>
+      </x:c>
+      <x:c r="K38" s="664"/>
+      <x:c r="L38" s="664"/>
+      <x:c r="M38" s="664"/>
+      <x:c r="N38" s="664"/>
+      <x:c r="O38" s="664"/>
+    </x:row>
+    <x:row r="39" ht="18" customHeight="1">
+      <x:c r="A39" s="824" t="str">
+        <x:v>ROK standalone adjusted EPS</x:v>
+      </x:c>
+      <x:c r="B39" s="663" t="n">
+        <x:f>'ROK Forecast'!F11</x:f>
+        <x:v>13.939000000000002</x:v>
+      </x:c>
+      <x:c r="C39" s="663" t="n">
+        <x:f>'ROK Forecast'!G11</x:f>
+        <x:v>14.775340000000003</x:v>
+      </x:c>
+      <x:c r="D39" s="663" t="n">
+        <x:f>'ROK Forecast'!H11</x:f>
+        <x:v>15.514107000000005</x:v>
+      </x:c>
+      <x:c r="E39" s="663" t="n">
+        <x:f>'ROK Forecast'!I11</x:f>
+        <x:v>16.289812350000005</x:v>
+      </x:c>
+      <x:c r="F39" s="664" t="str">
+        <x:v>ROK Forecast</x:v>
+      </x:c>
+      <x:c r="G39" s="664"/>
+      <x:c r="H39" s="824" t="str">
+        <x:v>Pro forma share-count identity</x:v>
+      </x:c>
+      <x:c r="I39" s="849" t="n">
+        <x:f>B38-SUM(B36:B37)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J39" s="664" t="str">
+        <x:v>Buyer shares plus weighted new shares</x:v>
+      </x:c>
+      <x:c r="K39" s="664"/>
+      <x:c r="L39" s="664"/>
+      <x:c r="M39" s="664"/>
+      <x:c r="N39" s="664"/>
+      <x:c r="O39" s="664"/>
+    </x:row>
+    <x:row r="40" ht="18" customHeight="1">
+      <x:c r="A40" s="824" t="str">
+        <x:v>Pro forma EPS — including PPA</x:v>
+      </x:c>
+      <x:c r="B40" s="845" t="n">
+        <x:f>B34/B38</x:f>
+        <x:v>11.08042136117266</x:v>
+      </x:c>
+      <x:c r="C40" s="845" t="n">
+        <x:f>C34/C38</x:f>
+        <x:v>9.780388971398116</x:v>
+      </x:c>
+      <x:c r="D40" s="845" t="n">
+        <x:f>D34/D38</x:f>
+        <x:v>10.993441417850704</x:v>
+      </x:c>
+      <x:c r="E40" s="845" t="n">
+        <x:f>E34/E38</x:f>
+        <x:v>12.009630732983203</x:v>
+      </x:c>
+      <x:c r="F40" s="664" t="str">
+        <x:v>Pro forma net income ÷ shares</x:v>
+      </x:c>
+      <x:c r="G40" s="664"/>
+      <x:c r="H40" s="824" t="str">
+        <x:v>Accretion / dilution formula</x:v>
+      </x:c>
+      <x:c r="I40" s="849" t="n">
+        <x:f>B41-(B40/B39-1)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" s="664" t="str">
+        <x:v>Must equal zero</x:v>
+      </x:c>
+      <x:c r="K40" s="664"/>
+      <x:c r="L40" s="664"/>
+      <x:c r="M40" s="664"/>
+      <x:c r="N40" s="664"/>
+      <x:c r="O40" s="664"/>
+    </x:row>
+    <x:row r="41" ht="18" customHeight="1">
+      <x:c r="A41" s="832" t="str">
+        <x:v>EPS accretion / (dilution) — including PPA</x:v>
+      </x:c>
+      <x:c r="B41" s="846" t="n">
+        <x:f>B40/B39-1</x:f>
+        <x:v>-0.20507774150422142</x:v>
+      </x:c>
+      <x:c r="C41" s="846" t="n">
+        <x:f>C40/C39-1</x:f>
+        <x:v>-0.33805997212936467</x:v>
+      </x:c>
+      <x:c r="D41" s="846" t="n">
+        <x:f>D40/D39-1</x:f>
+        <x:v>-0.2913906409275957</x:v>
+      </x:c>
+      <x:c r="E41" s="846" t="n">
+        <x:f>E40/E39-1</x:f>
+        <x:v>-0.26275205171512006</x:v>
+      </x:c>
+      <x:c r="F41" s="755" t="str">
+        <x:v>Pro forma EPS ÷ buyer EPS − 1</x:v>
+      </x:c>
+      <x:c r="G41" s="755"/>
+      <x:c r="H41" s="824" t="str">
+        <x:v>Adjusted EPS bridge</x:v>
+      </x:c>
+      <x:c r="I41" s="849" t="n">
+        <x:f>B43-(B34+B33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J41" s="664" t="str">
+        <x:v>Adjusted net income adds back PPA</x:v>
+      </x:c>
+      <x:c r="K41" s="664"/>
+      <x:c r="L41" s="664"/>
+      <x:c r="M41" s="664"/>
+      <x:c r="N41" s="664"/>
+      <x:c r="O41" s="664"/>
+    </x:row>
+    <x:row r="42" ht="18" customHeight="1">
+      <x:c r="A42" s="824"/>
+      <x:c r="B42" s="716"/>
+      <x:c r="C42" s="716"/>
+      <x:c r="D42" s="716"/>
+      <x:c r="E42" s="716"/>
+      <x:c r="F42" s="664"/>
+      <x:c r="G42" s="664"/>
+      <x:c r="H42" s="824" t="str">
+        <x:v>Breakeven synergy produces neutral EPS</x:v>
+      </x:c>
+      <x:c r="I42" s="849" t="n">
+        <x:f>(B34+I24*B24*(1-$B$7))/B38-B39</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="664" t="str">
+        <x:v>Adds required recognized synergy to headline earnings</x:v>
+      </x:c>
+      <x:c r="K42" s="664"/>
+      <x:c r="L42" s="664"/>
+      <x:c r="M42" s="664"/>
+      <x:c r="N42" s="664"/>
+      <x:c r="O42" s="664"/>
+    </x:row>
+    <x:row r="43" ht="18" customHeight="1">
+      <x:c r="A43" s="824" t="str">
+        <x:v>Pro forma net income — excluding PPA</x:v>
+      </x:c>
+      <x:c r="B43" s="744" t="n">
+        <x:f>B34+B33</x:f>
+        <x:v>1589.7371294976</x:v>
+      </x:c>
+      <x:c r="C43" s="744" t="n">
+        <x:f>C34+C33</x:f>
+        <x:v>1737.8856238485998</x:v>
+      </x:c>
+      <x:c r="D43" s="744" t="n">
+        <x:f>D34+D33</x:f>
+        <x:v>1835.4331190312937</x:v>
+      </x:c>
+      <x:c r="E43" s="744" t="n">
+        <x:f>E34+E33</x:f>
+        <x:v>1931.8162034578115</x:v>
+      </x:c>
+      <x:c r="F43" s="664" t="str">
+        <x:v>Adds back after-tax PPA expense</x:v>
+      </x:c>
+      <x:c r="G43" s="664"/>
+      <x:c r="H43" s="538"/>
+      <x:c r="I43" s="538"/>
+      <x:c r="J43" s="538"/>
+      <x:c r="K43" s="538"/>
+      <x:c r="L43" s="538"/>
+      <x:c r="M43" s="538"/>
+      <x:c r="N43" s="538"/>
+      <x:c r="O43" s="538"/>
+    </x:row>
+    <x:row r="44" ht="18" customHeight="1">
+      <x:c r="A44" s="824" t="str">
+        <x:v>Pro forma EPS — excluding PPA</x:v>
+      </x:c>
+      <x:c r="B44" s="845" t="n">
+        <x:f>B43/B38</x:f>
+        <x:v>13.007714624955764</x:v>
+      </x:c>
+      <x:c r="C44" s="845" t="n">
+        <x:f>C43/C38</x:f>
+        <x:v>13.141719889960736</x:v>
+      </x:c>
+      <x:c r="D44" s="845" t="n">
+        <x:f>D43/D38</x:f>
+        <x:v>13.972689575870785</x:v>
+      </x:c>
+      <x:c r="E44" s="845" t="n">
+        <x:f>E43/E38</x:f>
+        <x:v>14.805183658512783</x:v>
+      </x:c>
+      <x:c r="F44" s="664" t="str">
+        <x:v>Adjusted pro forma net income ÷ shares</x:v>
+      </x:c>
+      <x:c r="G44" s="664"/>
+      <x:c r="H44" s="538"/>
+      <x:c r="I44" s="538"/>
+      <x:c r="J44" s="538"/>
+      <x:c r="K44" s="538"/>
+      <x:c r="L44" s="538"/>
+      <x:c r="M44" s="538"/>
+      <x:c r="N44" s="538"/>
+      <x:c r="O44" s="538"/>
+    </x:row>
+    <x:row r="45" ht="18" customHeight="1">
+      <x:c r="A45" s="832" t="str">
+        <x:v>Adjusted accretion / (dilution) — excluding PPA</x:v>
+      </x:c>
+      <x:c r="B45" s="846" t="n">
+        <x:f>B44/B39-1</x:f>
+        <x:v>-0.06681149114314067</x:v>
+      </x:c>
+      <x:c r="C45" s="846" t="n">
+        <x:f>C44/C39-1</x:f>
+        <x:v>-0.11056396062894436</x:v>
+      </x:c>
+      <x:c r="D45" s="846" t="n">
+        <x:f>D44/D39-1</x:f>
+        <x:v>-0.09935585877609454</x:v>
+      </x:c>
+      <x:c r="E45" s="846" t="n">
+        <x:f>E44/E39-1</x:f>
+        <x:v>-0.09113847720211588</x:v>
+      </x:c>
+      <x:c r="F45" s="755" t="str">
+        <x:v>Adjusted EPS ÷ buyer EPS − 1</x:v>
+      </x:c>
+      <x:c r="G45" s="755"/>
+      <x:c r="H45" s="538"/>
+      <x:c r="I45" s="538"/>
+      <x:c r="J45" s="538"/>
+      <x:c r="K45" s="538"/>
+      <x:c r="L45" s="538"/>
+      <x:c r="M45" s="538"/>
+      <x:c r="N45" s="538"/>
+      <x:c r="O45" s="538"/>
+    </x:row>
+    <x:row r="46" ht="18" customHeight="1">
+      <x:c r="A46" s="824"/>
+      <x:c r="B46" s="716"/>
+      <x:c r="C46" s="716"/>
+      <x:c r="D46" s="716"/>
+      <x:c r="E46" s="716"/>
+      <x:c r="F46" s="664"/>
+      <x:c r="G46" s="664"/>
+      <x:c r="H46" s="538"/>
+      <x:c r="I46" s="538"/>
+      <x:c r="J46" s="538"/>
+      <x:c r="K46" s="538"/>
+      <x:c r="L46" s="538"/>
+      <x:c r="M46" s="538"/>
+      <x:c r="N46" s="538"/>
+      <x:c r="O46" s="538"/>
+    </x:row>
+    <x:row r="47" ht="18" customHeight="1">
+      <x:c r="A47" s="824" t="str">
+        <x:v>One-time transaction fees — after tax</x:v>
+      </x:c>
+      <x:c r="B47" s="794" t="n">
+        <x:f>$B$15*(1-$B$7*$B$10)</x:f>
+        <x:v>134.5792</x:v>
+      </x:c>
+      <x:c r="C47" s="794" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D47" s="794" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E47" s="794" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F47" s="664" t="str">
+        <x:v>Shown only in FY2027E</x:v>
+      </x:c>
+      <x:c r="G47" s="664"/>
+      <x:c r="H47" s="538"/>
+      <x:c r="I47" s="538"/>
+      <x:c r="J47" s="538"/>
+      <x:c r="K47" s="538"/>
+      <x:c r="L47" s="538"/>
+      <x:c r="M47" s="538"/>
+      <x:c r="N47" s="538"/>
+      <x:c r="O47" s="538"/>
+    </x:row>
+    <x:row r="48" ht="18" customHeight="1">
+      <x:c r="A48" s="824" t="str">
+        <x:v>EPS including PPA and one-time fees</x:v>
+      </x:c>
+      <x:c r="B48" s="845" t="n">
+        <x:f>(B34-B47)/B38</x:f>
+        <x:v>9.979253252575942</x:v>
+      </x:c>
+      <x:c r="C48" s="845" t="n">
+        <x:f>(C34-C47)/C38</x:f>
+        <x:v>9.780388971398116</x:v>
+      </x:c>
+      <x:c r="D48" s="845" t="n">
+        <x:f>(D34-D47)/D38</x:f>
+        <x:v>10.993441417850704</x:v>
+      </x:c>
+      <x:c r="E48" s="845" t="n">
+        <x:f>(E34-E47)/E38</x:f>
+        <x:v>12.009630732983203</x:v>
+      </x:c>
+      <x:c r="F48" s="664" t="str">
+        <x:v>Illustrative all-in first-year EPS</x:v>
+      </x:c>
+      <x:c r="G48" s="664"/>
+      <x:c r="H48" s="538"/>
+      <x:c r="I48" s="538"/>
+      <x:c r="J48" s="538"/>
+      <x:c r="K48" s="538"/>
+      <x:c r="L48" s="538"/>
+      <x:c r="M48" s="538"/>
+      <x:c r="N48" s="538"/>
+      <x:c r="O48" s="538"/>
+    </x:row>
+    <x:row r="49" ht="18" customHeight="1">
+      <x:c r="A49" s="538"/>
+      <x:c r="B49" s="538"/>
+      <x:c r="C49" s="538"/>
+      <x:c r="D49" s="538"/>
+      <x:c r="E49" s="538"/>
+      <x:c r="F49" s="538"/>
+      <x:c r="G49" s="538"/>
+      <x:c r="H49" s="538"/>
+      <x:c r="I49" s="538"/>
+      <x:c r="J49" s="538"/>
+      <x:c r="K49" s="538"/>
+      <x:c r="L49" s="538"/>
+      <x:c r="M49" s="538"/>
+      <x:c r="N49" s="538"/>
+      <x:c r="O49" s="538"/>
+    </x:row>
+    <x:row r="50" ht="18" customHeight="1">
+      <x:c r="A50" s="538"/>
+      <x:c r="B50" s="538"/>
+      <x:c r="C50" s="538"/>
+      <x:c r="D50" s="538"/>
+      <x:c r="E50" s="538"/>
+      <x:c r="F50" s="538"/>
+      <x:c r="G50" s="538"/>
+      <x:c r="H50" s="538"/>
+      <x:c r="I50" s="538"/>
+      <x:c r="J50" s="538"/>
+      <x:c r="K50" s="538"/>
+      <x:c r="L50" s="538"/>
+      <x:c r="M50" s="538"/>
+      <x:c r="N50" s="538"/>
+      <x:c r="O50" s="538"/>
+    </x:row>
+    <x:row r="51" ht="18" customHeight="1">
+      <x:c r="A51" s="822" t="str">
+        <x:v>ANALYST INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="B51" s="822"/>
+      <x:c r="C51" s="822"/>
+      <x:c r="D51" s="822"/>
+      <x:c r="E51" s="822"/>
+      <x:c r="F51" s="822"/>
+      <x:c r="G51" s="822"/>
+      <x:c r="H51" s="822"/>
+      <x:c r="I51" s="822"/>
+      <x:c r="J51" s="822"/>
+      <x:c r="K51" s="822"/>
+      <x:c r="L51" s="822"/>
+      <x:c r="M51" s="822"/>
+      <x:c r="N51" s="822"/>
+      <x:c r="O51" s="822"/>
+    </x:row>
+    <x:row r="52" ht="30" customHeight="1">
+      <x:c r="A52" s="836" t="str">
+        <x:v>The transaction is dilutive before synergies because Cognex’s earnings contribution is insufficient to offset the new shares issued, incremental financing costs, and purchase-accounting expense at the proposed $80 offer price.</x:v>
+      </x:c>
+      <x:c r="B52" s="836"/>
+      <x:c r="C52" s="836"/>
+      <x:c r="D52" s="836"/>
+      <x:c r="E52" s="836"/>
+      <x:c r="F52" s="836"/>
+      <x:c r="G52" s="836"/>
+      <x:c r="H52" s="836"/>
+      <x:c r="I52" s="836"/>
+      <x:c r="J52" s="836"/>
+      <x:c r="K52" s="836"/>
+      <x:c r="L52" s="836"/>
+      <x:c r="M52" s="836"/>
+      <x:c r="N52" s="836"/>
+      <x:c r="O52" s="836"/>
+    </x:row>
+    <x:row r="53" ht="30" customHeight="1">
+      <x:c r="A53" s="836" t="str">
+        <x:v>Excluding purchase-accounting expense improves the result but does not eliminate dilution. This demonstrates that the core issue is not only non-cash amortization; the acquisition price is high relative to Cognex’s standalone earnings contribution.</x:v>
+      </x:c>
+      <x:c r="B53" s="836"/>
+      <x:c r="C53" s="836"/>
+      <x:c r="D53" s="836"/>
+      <x:c r="E53" s="836"/>
+      <x:c r="F53" s="836"/>
+      <x:c r="G53" s="836"/>
+      <x:c r="H53" s="836"/>
+      <x:c r="I53" s="836"/>
+      <x:c r="J53" s="836"/>
+      <x:c r="K53" s="836"/>
+      <x:c r="L53" s="836"/>
+      <x:c r="M53" s="836"/>
+      <x:c r="N53" s="836"/>
+      <x:c r="O53" s="836"/>
+    </x:row>
+    <x:row r="54" ht="30" customHeight="1">
+      <x:c r="A54" s="836" t="str">
+        <x:v>The breakeven analysis calculates the cost-synergy run-rate required to restore Rockwell’s standalone EPS. It is a threshold, not a synergy forecast. The next step will independently underwrite achievable cost and revenue synergies.</x:v>
+      </x:c>
+      <x:c r="B54" s="836"/>
+      <x:c r="C54" s="836"/>
+      <x:c r="D54" s="836"/>
+      <x:c r="E54" s="836"/>
+      <x:c r="F54" s="836"/>
+      <x:c r="G54" s="836"/>
+      <x:c r="H54" s="836"/>
+      <x:c r="I54" s="836"/>
+      <x:c r="J54" s="836"/>
+      <x:c r="K54" s="836"/>
+      <x:c r="L54" s="836"/>
+      <x:c r="M54" s="836"/>
+      <x:c r="N54" s="836"/>
+      <x:c r="O54" s="836"/>
+    </x:row>
+    <x:row r="55" ht="30" customHeight="1">
+      <x:c r="A55" s="837" t="str">
+        <x:v>Buyer standalone forecasts use Rockwell adjusted EPS guidance and analyst growth assumptions; therefore, the headline output is a merger-model EPS comparison rather than a fully audited GAAP forecast.</x:v>
+      </x:c>
+      <x:c r="B55" s="837"/>
+      <x:c r="C55" s="837"/>
+      <x:c r="D55" s="837"/>
+      <x:c r="E55" s="837"/>
+      <x:c r="F55" s="837"/>
+      <x:c r="G55" s="837"/>
+      <x:c r="H55" s="837"/>
+      <x:c r="I55" s="837"/>
+      <x:c r="J55" s="837"/>
+      <x:c r="K55" s="837"/>
+      <x:c r="L55" s="837"/>
+      <x:c r="M55" s="837"/>
+      <x:c r="N55" s="837"/>
+      <x:c r="O55" s="837"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="B3:O3"/>
+    <x:mergeCell ref="A5:F5"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="E10:F10"/>
+    <x:mergeCell ref="E11:F11"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="E13:F13"/>
+    <x:mergeCell ref="E14:F14"/>
+    <x:mergeCell ref="E15:F15"/>
+    <x:mergeCell ref="E16:F16"/>
+    <x:mergeCell ref="H5:O5"/>
+    <x:mergeCell ref="J6:O6"/>
+    <x:mergeCell ref="J7:O7"/>
+    <x:mergeCell ref="J8:O8"/>
+    <x:mergeCell ref="J9:O9"/>
+    <x:mergeCell ref="J10:O10"/>
+    <x:mergeCell ref="J11:O11"/>
+    <x:mergeCell ref="J12:O12"/>
+    <x:mergeCell ref="J13:O13"/>
+    <x:mergeCell ref="J14:O14"/>
+    <x:mergeCell ref="A19:G19"/>
+    <x:mergeCell ref="H19:O19"/>
+    <x:mergeCell ref="H36:O36"/>
+    <x:mergeCell ref="J37:O37"/>
+    <x:mergeCell ref="J38:O38"/>
+    <x:mergeCell ref="J39:O39"/>
+    <x:mergeCell ref="J40:O40"/>
+    <x:mergeCell ref="J41:O41"/>
+    <x:mergeCell ref="J42:O42"/>
+    <x:mergeCell ref="A51:O51"/>
+    <x:mergeCell ref="A52:O52"/>
+    <x:mergeCell ref="A53:O53"/>
+    <x:mergeCell ref="A54:O54"/>
+    <x:mergeCell ref="A55:O55"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11555,8 +13411,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="812" t="str">
-        <x:v>PURCHASE ACCOUNTING COMPLETE</x:v>
+      <x:c r="B3" s="851" t="str">
+        <x:v>CORE TRANSACTION MODEL COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -12556,6 +14412,162 @@
       </x:c>
       <x:c r="G42" s="484" t="str">
         <x:v>Purchase Accounting rows 46-48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="484" t="str">
+        <x:v>A/D buyer EPS tie-out</x:v>
+      </x:c>
+      <x:c r="B43" s="484" t="n">
+        <x:f>'Accretion Dilution'!I37</x:f>
+        <x:v>1.7763568394002505e-15</x:v>
+      </x:c>
+      <x:c r="C43" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D43" s="484" t="n">
+        <x:f>B43-C43</x:f>
+        <x:v>1.7763568394002505e-15</x:v>
+      </x:c>
+      <x:c r="E43" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F43" s="853" t="str">
+        <x:f>IF(ABS(D43)&lt;=E43,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G43" s="484" t="str">
+        <x:v>Accretion Dilution row 37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="484" t="str">
+        <x:v>A/D pro forma net-income identity</x:v>
+      </x:c>
+      <x:c r="B44" s="484" t="n">
+        <x:f>'Accretion Dilution'!I38</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C44" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="484" t="n">
+        <x:f>B44-C44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E44" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F44" s="853" t="str">
+        <x:f>IF(ABS(D44)&lt;=E44,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G44" s="484" t="str">
+        <x:v>Accretion Dilution row 38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="484" t="str">
+        <x:v>A/D pro forma share-count identity</x:v>
+      </x:c>
+      <x:c r="B45" s="484" t="n">
+        <x:f>'Accretion Dilution'!I39</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C45" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="484" t="n">
+        <x:f>B45-C45</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E45" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F45" s="853" t="str">
+        <x:f>IF(ABS(D45)&lt;=E45,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G45" s="484" t="str">
+        <x:v>Accretion Dilution row 39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="484" t="str">
+        <x:v>A/D accretion formula</x:v>
+      </x:c>
+      <x:c r="B46" s="484" t="n">
+        <x:f>'Accretion Dilution'!I40</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C46" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D46" s="484" t="n">
+        <x:f>B46-C46</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E46" s="484" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F46" s="853" t="str">
+        <x:f>IF(ABS(D46)&lt;=E46,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G46" s="484" t="str">
+        <x:v>Accretion Dilution row 40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="484" t="str">
+        <x:v>A/D adjusted EPS bridge</x:v>
+      </x:c>
+      <x:c r="B47" s="484" t="n">
+        <x:f>'Accretion Dilution'!I41</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C47" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D47" s="484" t="n">
+        <x:f>B47-C47</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E47" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F47" s="853" t="str">
+        <x:f>IF(ABS(D47)&lt;=E47,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G47" s="484" t="str">
+        <x:v>Accretion Dilution row 41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="484" t="str">
+        <x:v>A/D breakeven synergy neutral EPS</x:v>
+      </x:c>
+      <x:c r="B48" s="484" t="n">
+        <x:f>'Accretion Dilution'!I42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C48" s="484" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D48" s="484" t="n">
+        <x:f>B48-C48</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E48" s="484" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F48" s="853" t="str">
+        <x:f>IF(ABS(D48)&lt;=E48,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G48" s="484" t="str">
+        <x:v>Accretion Dilution row 42</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16124,7 +18136,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dd4014f02454c82"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R001a1ece70a9424d"/>
 </x:worksheet>
 </file>
 
@@ -17847,7 +19859,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2873171e73d34d04"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4ca4b07f8344aac"/>
 </x:worksheet>
 </file>
 
@@ -21334,7 +23346,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74bcb809d4f746a3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fec4ba1cdc4357"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
transaction: complete synergy analysis
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R1dd3810331e54681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R8f5ddea17ffa485d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rd78e776180794d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R17404b112bae4706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rb21f822a1cc44a12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R8d4f70c80df24841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="Rba564b03131c4630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Rda684895e721438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R1930e61aff51462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rb5cfdf4d7aeb43c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R7cb71841a215468b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R1ff3cda4cc5847f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R5ced32c55ea24475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R9fbb43493e454b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Ra3015c248be94c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rd905c55e9b824730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R78bb7f6040834811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R04b6ac13bd0c4964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rcbcbeaae314b4d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rce5dd49fb1d646f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R773f8f621dd54f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rb809e2b8ad1c49e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rbc13c4a400964cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R5bd3915f8463480a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R3d7bd505fb064a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="Rcbc67dcbe159460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Raf6fcd4d9ce7451a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R5e1895f491ff432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rf77c9a90abfb494d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Rf089c6f9b0294c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R504d81771a6a4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R724de2b1edc04a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R3fbdf77a30cb46e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Re7a48d1bf83042e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,7 +155,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="26">
+  <x:numFmts count="27">
     <x:numFmt numFmtId="200" formatCode="mmm d, yyyy"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="$0.00;[Red]($0.00);-"/>
@@ -182,8 +182,9 @@
     <x:numFmt numFmtId="223" formatCode="$0"/>
     <x:numFmt numFmtId="224" formatCode="yyyy&quot;E&quot;"/>
     <x:numFmt numFmtId="225" formatCode="$#,##0.00"/>
+    <x:numFmt numFmtId="226" formatCode="#,##0.0;[Red](#,##0.0);-"/>
   </x:numFmts>
-  <x:fonts count="46">
+  <x:fonts count="53">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -443,8 +444,45 @@
       <x:color rgb="FFC00000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="69">
+  <x:fills count="78">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -786,8 +824,53 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="25">
+  <x:borders count="30">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -1053,11 +1136,42 @@
         <x:color rgb="FF17365D"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF000000"/>
+      </x:top>
+      <x:bottom style="double">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="double">
+        <x:color rgb="FF000000"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="854">
+  <x:cellXfs count="978">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2900,11 +3014,265 @@
     <x:xf numFmtId="0" fontId="26" fillId="63" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="40" fillId="63" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="70" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="74" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="210" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="226" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="226" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="46" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="76" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="46" fillId="76" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="51" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="51" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="76" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="72" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="76" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="73" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="75" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="226" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="76" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="46" fillId="76" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="77" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="226" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="47" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="46" fillId="76" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="71" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="48" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="48" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="52" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="48" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="52" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="17">
+  <x:dxfs count="19">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -3078,6 +3446,28 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FF17365D"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -3379,7 +3769,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.9 — accretion / dilution complete</x:v>
+        <x:v>0.10 — synergy analysis complete</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -3434,8 +3824,8 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="850" t="str">
-        <x:v>CORE TRANSACTION MODEL COMPLETE</x:v>
+      <x:c r="B9" s="861" t="str">
+        <x:v>SYNERGY ANALYSIS COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -13152,110 +13542,1369 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="3" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="34" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Synergies</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Cost and revenue synergies, timing, and implementation costs</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="856" t="str">
+        <x:v>Synergy Analysis</x:v>
+      </x:c>
+      <x:c r="B1" s="856"/>
+      <x:c r="C1" s="856"/>
+      <x:c r="D1" s="856"/>
+      <x:c r="E1" s="856"/>
+      <x:c r="F1" s="856"/>
+      <x:c r="G1" s="856"/>
+      <x:c r="H1" s="856"/>
+      <x:c r="I1" s="856"/>
+      <x:c r="J1" s="856"/>
+      <x:c r="K1" s="856"/>
+      <x:c r="L1" s="856"/>
+      <x:c r="M1" s="856"/>
+      <x:c r="N1" s="856"/>
+      <x:c r="O1" s="856"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="859" t="str">
+        <x:v>Bottom-up cost and revenue synergy underwriting; $ in millions except per-share data</x:v>
+      </x:c>
+      <x:c r="B2" s="859"/>
+      <x:c r="C2" s="859"/>
+      <x:c r="D2" s="859"/>
+      <x:c r="E2" s="859"/>
+      <x:c r="F2" s="859"/>
+      <x:c r="G2" s="859"/>
+      <x:c r="H2" s="859"/>
+      <x:c r="I2" s="859"/>
+      <x:c r="J2" s="859"/>
+      <x:c r="K2" s="859"/>
+      <x:c r="L2" s="859"/>
+      <x:c r="M2" s="859"/>
+      <x:c r="N2" s="859"/>
+      <x:c r="O2" s="859"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="921" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="B3" s="922" t="str">
+        <x:v>SYNERGY ANALYSIS COMPLETE</x:v>
+      </x:c>
+      <x:c r="C3" s="922"/>
+      <x:c r="D3" s="922"/>
+      <x:c r="E3" s="922"/>
+      <x:c r="F3" s="922"/>
+      <x:c r="G3" s="923"/>
+      <x:c r="H3" s="924" t="str">
+        <x:v>Underwriting conclusion</x:v>
+      </x:c>
+      <x:c r="I3" s="924"/>
+      <x:c r="J3" s="925" t="str">
+        <x:v>Base synergies do not offset adjusted EPS dilution</x:v>
+      </x:c>
+      <x:c r="K3" s="925"/>
+      <x:c r="L3" s="925"/>
+      <x:c r="M3" s="925"/>
+      <x:c r="N3" s="925"/>
+      <x:c r="O3" s="925"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="923"/>
+      <x:c r="B4" s="923"/>
+      <x:c r="C4" s="923"/>
+      <x:c r="D4" s="923"/>
+      <x:c r="E4" s="923"/>
+      <x:c r="F4" s="923"/>
+      <x:c r="G4" s="923"/>
+      <x:c r="H4" s="923"/>
+      <x:c r="I4" s="923"/>
+      <x:c r="J4" s="923"/>
+      <x:c r="K4" s="923"/>
+      <x:c r="L4" s="923"/>
+      <x:c r="M4" s="923"/>
+      <x:c r="N4" s="923"/>
+      <x:c r="O4" s="923"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="869" t="str">
+        <x:v>COST SYNERGY ASSUMPTIONS</x:v>
+      </x:c>
+      <x:c r="B5" s="869"/>
+      <x:c r="C5" s="869"/>
+      <x:c r="D5" s="869"/>
+      <x:c r="E5" s="869"/>
+      <x:c r="F5" s="869"/>
+      <x:c r="G5" s="923"/>
+      <x:c r="H5" s="869" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I5" s="869"/>
+      <x:c r="J5" s="869"/>
+      <x:c r="K5" s="869"/>
+      <x:c r="L5" s="869"/>
+      <x:c r="M5" s="869"/>
+      <x:c r="N5" s="869"/>
+      <x:c r="O5" s="869"/>
+    </x:row>
+    <x:row r="6" ht="18" customHeight="1">
+      <x:c r="A6" s="875" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="B6" s="876" t="str">
+        <x:v>FY2027E cost base</x:v>
+      </x:c>
+      <x:c r="C6" s="876" t="str">
+        <x:v>Savings %</x:v>
+      </x:c>
+      <x:c r="D6" s="876" t="str">
+        <x:v>Full run-rate</x:v>
+      </x:c>
+      <x:c r="E6" s="876" t="str"/>
+      <x:c r="F6" s="877" t="str">
+        <x:v>Underwriting basis</x:v>
+      </x:c>
+      <x:c r="G6" s="923"/>
+      <x:c r="H6" s="926" t="str">
+        <x:v>Full run-rate cost synergies</x:v>
+      </x:c>
+      <x:c r="I6" s="926"/>
+      <x:c r="J6" s="926"/>
+      <x:c r="K6" s="927" t="n">
+        <x:f>D13</x:f>
+        <x:v>98.60066300000001</x:v>
+      </x:c>
+      <x:c r="L6" s="927"/>
+      <x:c r="M6" s="927"/>
+      <x:c r="N6" s="923"/>
+      <x:c r="O6" s="923"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="923" t="str">
+        <x:v>Corporate G&amp;A / back office</x:v>
+      </x:c>
+      <x:c r="B7" s="928" t="n">
+        <x:f>'CGNX Operating Model'!F27</x:f>
+        <x:v>378.99300000000005</x:v>
+      </x:c>
+      <x:c r="C7" s="929" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D7" s="930" t="n">
+        <x:f>B7*C7</x:f>
+        <x:v>37.899300000000004</x:v>
+      </x:c>
+      <x:c r="E7" s="923"/>
+      <x:c r="F7" s="931" t="str">
+        <x:v>Duplicate corporate functions and shared services</x:v>
+      </x:c>
+      <x:c r="G7" s="923"/>
+      <x:c r="H7" s="926" t="str">
+        <x:v>FY2030E revenue synergy contribution</x:v>
+      </x:c>
+      <x:c r="I7" s="926"/>
+      <x:c r="J7" s="926"/>
+      <x:c r="K7" s="927" t="n">
+        <x:f>E26</x:f>
+        <x:v>45.87855649200001</x:v>
+      </x:c>
+      <x:c r="L7" s="927"/>
+      <x:c r="M7" s="927"/>
+      <x:c r="N7" s="923"/>
+      <x:c r="O7" s="923"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="923" t="str">
+        <x:v>Sales and channel overlap</x:v>
+      </x:c>
+      <x:c r="B8" s="928" t="n">
+        <x:f>'CGNX Operating Model'!F27</x:f>
+        <x:v>378.99300000000005</x:v>
+      </x:c>
+      <x:c r="C8" s="929" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="D8" s="930" t="n">
+        <x:f>B8*C8</x:f>
+        <x:v>28.424475000000005</x:v>
+      </x:c>
+      <x:c r="E8" s="923"/>
+      <x:c r="F8" s="931" t="str">
+        <x:v>Selective coverage rationalization; preserves commercial capacity</x:v>
+      </x:c>
+      <x:c r="G8" s="923"/>
+      <x:c r="H8" s="926" t="str">
+        <x:v>FY2030E recurring pre-tax synergy</x:v>
+      </x:c>
+      <x:c r="I8" s="926"/>
+      <x:c r="J8" s="926"/>
+      <x:c r="K8" s="927" t="n">
+        <x:f>E27</x:f>
+        <x:v>144.47921949200003</x:v>
+      </x:c>
+      <x:c r="L8" s="927"/>
+      <x:c r="M8" s="927"/>
+      <x:c r="N8" s="923"/>
+      <x:c r="O8" s="923"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="923" t="str">
+        <x:v>R&amp;D / product roadmap</x:v>
+      </x:c>
+      <x:c r="B9" s="928" t="n">
+        <x:f>'CGNX Operating Model'!F25</x:f>
+        <x:v>166.50840000000002</x:v>
+      </x:c>
+      <x:c r="C9" s="929" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="D9" s="930" t="n">
+        <x:f>B9*C9</x:f>
+        <x:v>4.995252000000001</x:v>
+      </x:c>
+      <x:c r="E9" s="923"/>
+      <x:c r="F9" s="931" t="str">
+        <x:v>Duplicate platforms only; protects machine-vision innovation</x:v>
+      </x:c>
+      <x:c r="G9" s="923"/>
+      <x:c r="H9" s="926" t="str">
+        <x:v>Total integration costs</x:v>
+      </x:c>
+      <x:c r="I9" s="926"/>
+      <x:c r="J9" s="926"/>
+      <x:c r="K9" s="927" t="n">
+        <x:f>D15</x:f>
+        <x:v>147.90099450000002</x:v>
+      </x:c>
+      <x:c r="L9" s="927"/>
+      <x:c r="M9" s="927"/>
+      <x:c r="N9" s="923"/>
+      <x:c r="O9" s="923"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="923" t="str">
+        <x:v>Procurement / cost of goods sold</x:v>
+      </x:c>
+      <x:c r="B10" s="928" t="n">
+        <x:f>'CGNX Operating Model'!F22</x:f>
+        <x:v>364.0818000000001</x:v>
+      </x:c>
+      <x:c r="C10" s="929" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="D10" s="930" t="n">
+        <x:f>B10*C10</x:f>
+        <x:v>7.281636000000002</x:v>
+      </x:c>
+      <x:c r="E10" s="923"/>
+      <x:c r="F10" s="931" t="str">
+        <x:v>Combined purchasing, logistics, and manufacturing efficiency</x:v>
+      </x:c>
+      <x:c r="G10" s="923"/>
+      <x:c r="H10" s="926" t="str">
+        <x:v>FY2030E adjusted EPS A / (D)</x:v>
+      </x:c>
+      <x:c r="I10" s="926"/>
+      <x:c r="J10" s="926"/>
+      <x:c r="K10" s="932" t="n">
+        <x:f>L31</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="L10" s="932"/>
+      <x:c r="M10" s="932"/>
+      <x:c r="N10" s="923"/>
+      <x:c r="O10" s="923"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="923" t="str">
+        <x:v>Public-company costs</x:v>
+      </x:c>
+      <x:c r="B11" s="933" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C11" s="929" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="930" t="n">
+        <x:f>B11*C11</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E11" s="923"/>
+      <x:c r="F11" s="931" t="str">
+        <x:v>Illustrative audit, listing, board, and standalone-company costs</x:v>
+      </x:c>
+      <x:c r="G11" s="923"/>
+      <x:c r="H11" s="926" t="str">
+        <x:v>FY2030E breakeven synergy coverage</x:v>
+      </x:c>
+      <x:c r="I11" s="926"/>
+      <x:c r="J11" s="926"/>
+      <x:c r="K11" s="932" t="n">
+        <x:f>L35</x:f>
+        <x:v>0.5891998444134365</x:v>
+      </x:c>
+      <x:c r="L11" s="932"/>
+      <x:c r="M11" s="932"/>
+      <x:c r="N11" s="923"/>
+      <x:c r="O11" s="923"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="923" t="str">
+        <x:v>IT, facilities, and other</x:v>
+      </x:c>
+      <x:c r="B12" s="933" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C12" s="929" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D12" s="930" t="n">
+        <x:f>B12*C12</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E12" s="923"/>
+      <x:c r="F12" s="931" t="str">
+        <x:v>Systems, facilities, insurance, and vendor consolidation</x:v>
+      </x:c>
+      <x:c r="G12" s="923"/>
+      <x:c r="H12" s="926" t="str">
+        <x:v>Synergy underwriting result</x:v>
+      </x:c>
+      <x:c r="I12" s="926"/>
+      <x:c r="J12" s="926"/>
+      <x:c r="K12" s="934" t="str">
+        <x:f>IF(K11&gt;=1,"Sufficient to reach adjusted breakeven","Insufficient to reach adjusted breakeven")</x:f>
+        <x:v>Insufficient to reach adjusted breakeven</x:v>
+      </x:c>
+      <x:c r="L12" s="934"/>
+      <x:c r="M12" s="934"/>
+      <x:c r="N12" s="934"/>
+      <x:c r="O12" s="934"/>
+    </x:row>
+    <x:row r="13" ht="18" customHeight="1">
+      <x:c r="A13" s="935" t="str">
+        <x:v>Total cost synergy run-rate</x:v>
+      </x:c>
+      <x:c r="B13" s="935"/>
+      <x:c r="C13" s="935"/>
+      <x:c r="D13" s="936" t="n">
+        <x:f>SUM(D7:D12)</x:f>
+        <x:v>98.60066300000001</x:v>
+      </x:c>
+      <x:c r="E13" s="923"/>
+      <x:c r="F13" s="923"/>
+      <x:c r="G13" s="923"/>
+      <x:c r="H13" s="923"/>
+      <x:c r="I13" s="923"/>
+      <x:c r="J13" s="923"/>
+      <x:c r="K13" s="923"/>
+      <x:c r="L13" s="923"/>
+      <x:c r="M13" s="923"/>
+      <x:c r="N13" s="923"/>
+      <x:c r="O13" s="923"/>
+    </x:row>
+    <x:row r="14" ht="18" customHeight="1">
+      <x:c r="A14" s="923" t="str">
+        <x:v>Integration cost / cost synergy run-rate</x:v>
+      </x:c>
+      <x:c r="B14" s="923"/>
+      <x:c r="C14" s="923"/>
+      <x:c r="D14" s="937" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="E14" s="923"/>
+      <x:c r="F14" s="923"/>
+      <x:c r="G14" s="923"/>
+      <x:c r="H14" s="923"/>
+      <x:c r="I14" s="923"/>
+      <x:c r="J14" s="923"/>
+      <x:c r="K14" s="923"/>
+      <x:c r="L14" s="923"/>
+      <x:c r="M14" s="923"/>
+      <x:c r="N14" s="923"/>
+      <x:c r="O14" s="923"/>
+    </x:row>
+    <x:row r="15" ht="18" customHeight="1">
+      <x:c r="A15" s="923" t="str">
+        <x:v>Total integration cost pool</x:v>
+      </x:c>
+      <x:c r="B15" s="923"/>
+      <x:c r="C15" s="923"/>
+      <x:c r="D15" s="930" t="n">
+        <x:f>D13*D14</x:f>
+        <x:v>147.90099450000002</x:v>
+      </x:c>
+      <x:c r="E15" s="923"/>
+      <x:c r="F15" s="923"/>
+      <x:c r="G15" s="923"/>
+      <x:c r="H15" s="923"/>
+      <x:c r="I15" s="923"/>
+      <x:c r="J15" s="923"/>
+      <x:c r="K15" s="923"/>
+      <x:c r="L15" s="923"/>
+      <x:c r="M15" s="923"/>
+      <x:c r="N15" s="923"/>
+      <x:c r="O15" s="923"/>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1">
+      <x:c r="A16" s="923"/>
+      <x:c r="B16" s="923"/>
+      <x:c r="C16" s="923"/>
+      <x:c r="D16" s="923"/>
+      <x:c r="E16" s="923"/>
+      <x:c r="F16" s="923"/>
+      <x:c r="G16" s="923"/>
+      <x:c r="H16" s="923"/>
+      <x:c r="I16" s="923"/>
+      <x:c r="J16" s="923"/>
+      <x:c r="K16" s="923"/>
+      <x:c r="L16" s="923"/>
+      <x:c r="M16" s="923"/>
+      <x:c r="N16" s="923"/>
+      <x:c r="O16" s="923"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="923"/>
+      <x:c r="B17" s="923"/>
+      <x:c r="C17" s="923"/>
+      <x:c r="D17" s="923"/>
+      <x:c r="E17" s="923"/>
+      <x:c r="F17" s="923"/>
+      <x:c r="G17" s="923"/>
+      <x:c r="H17" s="923"/>
+      <x:c r="I17" s="923"/>
+      <x:c r="J17" s="923"/>
+      <x:c r="K17" s="923"/>
+      <x:c r="L17" s="923"/>
+      <x:c r="M17" s="923"/>
+      <x:c r="N17" s="923"/>
+      <x:c r="O17" s="923"/>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1">
+      <x:c r="A18" s="869" t="str">
+        <x:v>SYNERGY BUILD AND PHASING</x:v>
+      </x:c>
+      <x:c r="B18" s="869"/>
+      <x:c r="C18" s="869"/>
+      <x:c r="D18" s="869"/>
+      <x:c r="E18" s="869"/>
+      <x:c r="F18" s="869"/>
+      <x:c r="G18" s="923"/>
+      <x:c r="H18" s="869" t="str">
+        <x:v>EPS IMPACT AND BREAKEVEN COMPARISON</x:v>
+      </x:c>
+      <x:c r="I18" s="869"/>
+      <x:c r="J18" s="869"/>
+      <x:c r="K18" s="869"/>
+      <x:c r="L18" s="869"/>
+      <x:c r="M18" s="869"/>
+      <x:c r="N18" s="869"/>
+      <x:c r="O18" s="869"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="938" t="str">
+        <x:v>$ in millions</x:v>
+      </x:c>
+      <x:c r="B19" s="938" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="C19" s="938" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="D19" s="938" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="E19" s="938" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="F19" s="938" t="str">
+        <x:v>Methodology</x:v>
+      </x:c>
+      <x:c r="G19" s="923"/>
+      <x:c r="H19" s="938" t="str">
+        <x:v>$ in millions, except per-share data</x:v>
+      </x:c>
+      <x:c r="I19" s="938" t="str">
+        <x:v>FY2027E</x:v>
+      </x:c>
+      <x:c r="J19" s="938" t="str">
+        <x:v>FY2028E</x:v>
+      </x:c>
+      <x:c r="K19" s="938" t="str">
+        <x:v>FY2029E</x:v>
+      </x:c>
+      <x:c r="L19" s="938" t="str">
+        <x:v>FY2030E</x:v>
+      </x:c>
+      <x:c r="M19" s="938" t="str">
+        <x:v>Methodology</x:v>
+      </x:c>
+      <x:c r="N19" s="923"/>
+      <x:c r="O19" s="923"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="939" t="str">
+        <x:v>Target revenue</x:v>
+      </x:c>
+      <x:c r="B20" s="951" t="n">
+        <x:f>'CGNX Operating Model'!F20</x:f>
+        <x:v>1242.6000000000001</x:v>
+      </x:c>
+      <x:c r="C20" s="951" t="n">
+        <x:f>'CGNX Operating Model'!G20</x:f>
+        <x:v>1342.0080000000003</x:v>
+      </x:c>
+      <x:c r="D20" s="951" t="n">
+        <x:f>'CGNX Operating Model'!H20</x:f>
+        <x:v>1435.9485600000003</x:v>
+      </x:c>
+      <x:c r="E20" s="951" t="n">
+        <x:f>'CGNX Operating Model'!I20</x:f>
+        <x:v>1529.2852164000003</x:v>
+      </x:c>
+      <x:c r="F20" s="931" t="str">
+        <x:v>CGNX standalone forecast</x:v>
+      </x:c>
+      <x:c r="G20" s="923"/>
+      <x:c r="H20" s="939" t="str">
+        <x:v>PF net income incl. PPA — before synergies</x:v>
+      </x:c>
+      <x:c r="I20" s="951" t="n">
+        <x:f>'Accretion Dilution'!B34</x:f>
+        <x:v>1354.1930889642667</x:v>
+      </x:c>
+      <x:c r="J20" s="951" t="n">
+        <x:f>'Accretion Dilution'!C34</x:f>
+        <x:v>1293.3769347819332</x:v>
+      </x:c>
+      <x:c r="K20" s="951" t="n">
+        <x:f>'Accretion Dilution'!D34</x:f>
+        <x:v>1444.083213964627</x:v>
+      </x:c>
+      <x:c r="L20" s="951" t="n">
+        <x:f>'Accretion Dilution'!E34</x:f>
+        <x:v>1567.045690391145</x:v>
+      </x:c>
+      <x:c r="M20" s="931" t="str">
+        <x:v>Existing merger model</x:v>
+      </x:c>
+      <x:c r="N20" s="923"/>
+      <x:c r="O20" s="923"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="939" t="str">
+        <x:v>Cost synergy phase-in</x:v>
+      </x:c>
+      <x:c r="B21" s="952" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="C21" s="952" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="D21" s="952" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="E21" s="952" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F21" s="931" t="str">
+        <x:v>25% / 60% / 90% / 100% cost ramp</x:v>
+      </x:c>
+      <x:c r="G21" s="923"/>
+      <x:c r="H21" s="939" t="str">
+        <x:v>After-tax net synergy incl. integration costs</x:v>
+      </x:c>
+      <x:c r="I21" s="953" t="n">
+        <x:f>B32</x:f>
+        <x:v>-35.02064588500001</x:v>
+      </x:c>
+      <x:c r="J21" s="953" t="n">
+        <x:f>C32</x:f>
+        <x:v>22.805070402750005</x:v>
+      </x:c>
+      <x:c r="K21" s="953" t="n">
+        <x:f>D32</x:f>
+        <x:v>77.53558951755002</x:v>
+      </x:c>
+      <x:c r="L21" s="953" t="n">
+        <x:f>E32</x:f>
+        <x:v>114.13858339868003</x:v>
+      </x:c>
+      <x:c r="M21" s="931" t="str">
+        <x:v>Net synergy after implementation costs and tax</x:v>
+      </x:c>
+      <x:c r="N21" s="923"/>
+      <x:c r="O21" s="923"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="939" t="str">
+        <x:v>Recognized cost synergies</x:v>
+      </x:c>
+      <x:c r="B22" s="953" t="n">
+        <x:f>$D$13*B21</x:f>
+        <x:v>24.650165750000003</x:v>
+      </x:c>
+      <x:c r="C22" s="953" t="n">
+        <x:f>$D$13*C21</x:f>
+        <x:v>59.160397800000005</x:v>
+      </x:c>
+      <x:c r="D22" s="953" t="n">
+        <x:f>$D$13*D21</x:f>
+        <x:v>88.74059670000001</x:v>
+      </x:c>
+      <x:c r="E22" s="953" t="n">
+        <x:f>$D$13*E21</x:f>
+        <x:v>98.60066300000001</x:v>
+      </x:c>
+      <x:c r="F22" s="931" t="str">
+        <x:v>Full run-rate × phase-in</x:v>
+      </x:c>
+      <x:c r="G22" s="923"/>
+      <x:c r="H22" s="940" t="str">
+        <x:v>PF net income incl. PPA — after synergies</x:v>
+      </x:c>
+      <x:c r="I22" s="954" t="n">
+        <x:f>SUM(I20:I21)</x:f>
+        <x:v>1319.1724430792667</x:v>
+      </x:c>
+      <x:c r="J22" s="954" t="n">
+        <x:f>SUM(J20:J21)</x:f>
+        <x:v>1316.1820051846832</x:v>
+      </x:c>
+      <x:c r="K22" s="954" t="n">
+        <x:f>SUM(K20:K21)</x:f>
+        <x:v>1521.618803482177</x:v>
+      </x:c>
+      <x:c r="L22" s="954" t="n">
+        <x:f>SUM(L20:L21)</x:f>
+        <x:v>1681.184273789825</x:v>
+      </x:c>
+      <x:c r="M22" s="931" t="str">
+        <x:v>Reported-style earnings after synergies</x:v>
+      </x:c>
+      <x:c r="N22" s="923"/>
+      <x:c r="O22" s="923"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="939" t="str">
+        <x:v>Revenue synergy % of target revenue</x:v>
+      </x:c>
+      <x:c r="B23" s="952" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C23" s="952" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="D23" s="952" t="n">
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="E23" s="952" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="F23" s="931" t="str">
+        <x:v>Cross-sell and channel reach; separately underwritten</x:v>
+      </x:c>
+      <x:c r="G23" s="923"/>
+      <x:c r="H23" s="939" t="str">
+        <x:v>Pro forma diluted shares</x:v>
+      </x:c>
+      <x:c r="I23" s="958" t="n">
+        <x:f>'Accretion Dilution'!B38</x:f>
+        <x:v>122.21494515628693</x:v>
+      </x:c>
+      <x:c r="J23" s="958" t="n">
+        <x:f>'Accretion Dilution'!C38</x:f>
+        <x:v>132.24187080537388</x:v>
+      </x:c>
+      <x:c r="K23" s="958" t="n">
+        <x:f>'Accretion Dilution'!D38</x:f>
+        <x:v>131.35861274703146</x:v>
+      </x:c>
+      <x:c r="L23" s="958" t="n">
+        <x:f>'Accretion Dilution'!E38</x:f>
+        <x:v>130.4824207531558</x:v>
+      </x:c>
+      <x:c r="M23" s="931" t="str">
+        <x:v>Existing merger model</x:v>
+      </x:c>
+      <x:c r="N23" s="923"/>
+      <x:c r="O23" s="923"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="939" t="str">
+        <x:v>Incremental revenue</x:v>
+      </x:c>
+      <x:c r="B24" s="953" t="n">
+        <x:f>B20*B23</x:f>
+        <x:v>12.426000000000002</x:v>
+      </x:c>
+      <x:c r="C24" s="953" t="n">
+        <x:f>C20*C23</x:f>
+        <x:v>53.68032000000001</x:v>
+      </x:c>
+      <x:c r="D24" s="953" t="n">
+        <x:f>D20*D23</x:f>
+        <x:v>78.97717080000001</x:v>
+      </x:c>
+      <x:c r="E24" s="953" t="n">
+        <x:f>E20*E23</x:f>
+        <x:v>114.69639123000002</x:v>
+      </x:c>
+      <x:c r="F24" s="931" t="str">
+        <x:v>Target revenue × revenue synergy %</x:v>
+      </x:c>
+      <x:c r="G24" s="923"/>
+      <x:c r="H24" s="939" t="str">
+        <x:v>PF EPS incl. PPA and integration costs</x:v>
+      </x:c>
+      <x:c r="I24" s="959" t="n">
+        <x:f>I22/I23</x:f>
+        <x:v>10.79387174287339</x:v>
+      </x:c>
+      <x:c r="J24" s="959" t="n">
+        <x:f>J22/J23</x:f>
+        <x:v>9.952838667276309</x:v>
+      </x:c>
+      <x:c r="K24" s="959" t="n">
+        <x:f>K22/K23</x:f>
+        <x:v>11.583700312156074</x:v>
+      </x:c>
+      <x:c r="L24" s="959" t="n">
+        <x:f>L22/L23</x:f>
+        <x:v>12.884373727019199</x:v>
+      </x:c>
+      <x:c r="M24" s="931" t="str">
+        <x:v>Net income ÷ diluted shares</x:v>
+      </x:c>
+      <x:c r="N24" s="923"/>
+      <x:c r="O24" s="923"/>
+    </x:row>
+    <x:row r="25" ht="18" customHeight="1">
+      <x:c r="A25" s="939" t="str">
+        <x:v>Contribution margin</x:v>
+      </x:c>
+      <x:c r="B25" s="952" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="C25" s="952" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D25" s="952" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="E25" s="952" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="F25" s="931" t="str">
+        <x:v>Incremental gross profit less variable selling support</x:v>
+      </x:c>
+      <x:c r="G25" s="923"/>
+      <x:c r="H25" s="944" t="str">
+        <x:v>EPS A / (D) incl. PPA and integration costs</x:v>
+      </x:c>
+      <x:c r="I25" s="960" t="n">
+        <x:f>I24/'Accretion Dilution'!B39-1</x:f>
+        <x:v>-0.22563514291746978</x:v>
+      </x:c>
+      <x:c r="J25" s="960" t="n">
+        <x:f>J24/'Accretion Dilution'!C39-1</x:f>
+        <x:v>-0.32638851848578065</x:v>
+      </x:c>
+      <x:c r="K25" s="960" t="n">
+        <x:f>K24/'Accretion Dilution'!D39-1</x:f>
+        <x:v>-0.2533440492478187</x:v>
+      </x:c>
+      <x:c r="L25" s="960" t="n">
+        <x:f>L24/'Accretion Dilution'!E39-1</x:f>
+        <x:v>-0.20905327512755578</x:v>
+      </x:c>
+      <x:c r="M25" s="931" t="str">
+        <x:v>PF EPS ÷ buyer standalone EPS − 1</x:v>
+      </x:c>
+      <x:c r="N25" s="923"/>
+      <x:c r="O25" s="923"/>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="939" t="str">
+        <x:v>Revenue synergy operating profit</x:v>
+      </x:c>
+      <x:c r="B26" s="953" t="n">
+        <x:f>B24*B25</x:f>
+        <x:v>4.9704000000000015</x:v>
+      </x:c>
+      <x:c r="C26" s="953" t="n">
+        <x:f>C24*C25</x:f>
+        <x:v>21.472128000000005</x:v>
+      </x:c>
+      <x:c r="D26" s="953" t="n">
+        <x:f>D24*D25</x:f>
+        <x:v>31.590868320000006</x:v>
+      </x:c>
+      <x:c r="E26" s="953" t="n">
+        <x:f>E24*E25</x:f>
+        <x:v>45.87855649200001</x:v>
+      </x:c>
+      <x:c r="F26" s="931" t="str">
+        <x:v>Incremental revenue × contribution margin</x:v>
+      </x:c>
+      <x:c r="G26" s="923"/>
+      <x:c r="H26" s="939" t="str"/>
+      <x:c r="I26" s="957"/>
+      <x:c r="J26" s="957"/>
+      <x:c r="K26" s="957"/>
+      <x:c r="L26" s="957"/>
+      <x:c r="M26" s="931" t="str"/>
+      <x:c r="N26" s="923"/>
+      <x:c r="O26" s="923"/>
+    </x:row>
+    <x:row r="27" ht="18" customHeight="1">
+      <x:c r="A27" s="940" t="str">
+        <x:v>Gross recurring pre-tax synergies</x:v>
+      </x:c>
+      <x:c r="B27" s="954" t="n">
+        <x:f>SUM(B22,B26)</x:f>
+        <x:v>29.620565750000004</x:v>
+      </x:c>
+      <x:c r="C27" s="954" t="n">
+        <x:f>SUM(C22,C26)</x:f>
+        <x:v>80.63252580000001</x:v>
+      </x:c>
+      <x:c r="D27" s="954" t="n">
+        <x:f>SUM(D22,D26)</x:f>
+        <x:v>120.33146502000002</x:v>
+      </x:c>
+      <x:c r="E27" s="954" t="n">
+        <x:f>SUM(E22,E26)</x:f>
+        <x:v>144.47921949200003</x:v>
+      </x:c>
+      <x:c r="F27" s="931" t="str">
+        <x:v>Cost synergies + revenue contribution</x:v>
+      </x:c>
+      <x:c r="G27" s="923"/>
+      <x:c r="H27" s="939" t="str">
+        <x:v>PF net income excl. PPA — before synergies</x:v>
+      </x:c>
+      <x:c r="I27" s="951" t="n">
+        <x:f>'Accretion Dilution'!B43</x:f>
+        <x:v>1589.7371294976</x:v>
+      </x:c>
+      <x:c r="J27" s="951" t="n">
+        <x:f>'Accretion Dilution'!C43</x:f>
+        <x:v>1737.8856238485998</x:v>
+      </x:c>
+      <x:c r="K27" s="951" t="n">
+        <x:f>'Accretion Dilution'!D43</x:f>
+        <x:v>1835.4331190312937</x:v>
+      </x:c>
+      <x:c r="L27" s="951" t="n">
+        <x:f>'Accretion Dilution'!E43</x:f>
+        <x:v>1931.8162034578115</x:v>
+      </x:c>
+      <x:c r="M27" s="931" t="str">
+        <x:v>Adds back PPA amortization</x:v>
+      </x:c>
+      <x:c r="N27" s="923"/>
+      <x:c r="O27" s="923"/>
+    </x:row>
+    <x:row r="28" ht="18" customHeight="1">
+      <x:c r="A28" s="939" t="str">
+        <x:v>Integration cost timing</x:v>
+      </x:c>
+      <x:c r="B28" s="952" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C28" s="952" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="D28" s="952" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="E28" s="952" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F28" s="931" t="str">
+        <x:v>50% / 35% / 15% / 0% timing</x:v>
+      </x:c>
+      <x:c r="G28" s="923"/>
+      <x:c r="H28" s="939" t="str">
+        <x:v>After-tax recurring synergies excl. integration costs</x:v>
+      </x:c>
+      <x:c r="I28" s="953" t="n">
+        <x:f>B27*(1-B31)</x:f>
+        <x:v>23.400246942500004</x:v>
+      </x:c>
+      <x:c r="J28" s="953" t="n">
+        <x:f>C27*(1-C31)</x:f>
+        <x:v>63.69969538200001</x:v>
+      </x:c>
+      <x:c r="K28" s="953" t="n">
+        <x:f>D27*(1-D31)</x:f>
+        <x:v>95.06185736580002</x:v>
+      </x:c>
+      <x:c r="L28" s="953" t="n">
+        <x:f>E27*(1-E31)</x:f>
+        <x:v>114.13858339868003</x:v>
+      </x:c>
+      <x:c r="M28" s="931" t="str">
+        <x:v>Recurring pre-tax synergy × (1 − tax rate)</x:v>
+      </x:c>
+      <x:c r="N28" s="923"/>
+      <x:c r="O28" s="923"/>
+    </x:row>
+    <x:row r="29" ht="18" customHeight="1">
+      <x:c r="A29" s="939" t="str">
+        <x:v>Integration costs</x:v>
+      </x:c>
+      <x:c r="B29" s="953" t="n">
+        <x:f>$D$15*B28</x:f>
+        <x:v>73.95049725000001</x:v>
+      </x:c>
+      <x:c r="C29" s="953" t="n">
+        <x:f>$D$15*C28</x:f>
+        <x:v>51.765348075000006</x:v>
+      </x:c>
+      <x:c r="D29" s="953" t="n">
+        <x:f>$D$15*D28</x:f>
+        <x:v>22.185149175000003</x:v>
+      </x:c>
+      <x:c r="E29" s="953" t="n">
+        <x:f>$D$15*E28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="931" t="str">
+        <x:v>Total cost pool × timing</x:v>
+      </x:c>
+      <x:c r="G29" s="923"/>
+      <x:c r="H29" s="940" t="str">
+        <x:v>Adjusted PF net income after synergies</x:v>
+      </x:c>
+      <x:c r="I29" s="954" t="n">
+        <x:f>SUM(I27:I28)</x:f>
+        <x:v>1613.1373764401</x:v>
+      </x:c>
+      <x:c r="J29" s="954" t="n">
+        <x:f>SUM(J27:J28)</x:f>
+        <x:v>1801.5853192306</x:v>
+      </x:c>
+      <x:c r="K29" s="954" t="n">
+        <x:f>SUM(K27:K28)</x:f>
+        <x:v>1930.4949763970938</x:v>
+      </x:c>
+      <x:c r="L29" s="954" t="n">
+        <x:f>SUM(L27:L28)</x:f>
+        <x:v>2045.9547868564916</x:v>
+      </x:c>
+      <x:c r="M29" s="931" t="str">
+        <x:v>Adjusted earnings plus recurring synergy</x:v>
+      </x:c>
+      <x:c r="N29" s="923"/>
+      <x:c r="O29" s="923"/>
+    </x:row>
+    <x:row r="30" ht="18" customHeight="1">
+      <x:c r="A30" s="940" t="str">
+        <x:v>Net pre-tax synergy after integration</x:v>
+      </x:c>
+      <x:c r="B30" s="954" t="n">
+        <x:f>B27-B29</x:f>
+        <x:v>-44.32993150000001</x:v>
+      </x:c>
+      <x:c r="C30" s="954" t="n">
+        <x:f>C27-C29</x:f>
+        <x:v>28.867177725000005</x:v>
+      </x:c>
+      <x:c r="D30" s="954" t="n">
+        <x:f>D27-D29</x:f>
+        <x:v>98.14631584500002</x:v>
+      </x:c>
+      <x:c r="E30" s="954" t="n">
+        <x:f>E27-E29</x:f>
+        <x:v>144.47921949200003</x:v>
+      </x:c>
+      <x:c r="F30" s="931" t="str">
+        <x:v>Recurring synergies less integration costs</x:v>
+      </x:c>
+      <x:c r="G30" s="923"/>
+      <x:c r="H30" s="939" t="str">
+        <x:v>Adjusted PF EPS after synergies</x:v>
+      </x:c>
+      <x:c r="I30" s="959" t="n">
+        <x:f>I29/I23</x:f>
+        <x:v>13.199182590780861</x:v>
+      </x:c>
+      <x:c r="J30" s="959" t="n">
+        <x:f>J29/J23</x:f>
+        <x:v>13.623410711438524</x:v>
+      </x:c>
+      <x:c r="K30" s="959" t="n">
+        <x:f>K29/K23</x:f>
+        <x:v>14.696371528487541</x:v>
+      </x:c>
+      <x:c r="L30" s="959" t="n">
+        <x:f>L29/L23</x:f>
+        <x:v>15.679926652548781</x:v>
+      </x:c>
+      <x:c r="M30" s="931" t="str">
+        <x:v>Adjusted net income ÷ diluted shares</x:v>
+      </x:c>
+      <x:c r="N30" s="923"/>
+      <x:c r="O30" s="923"/>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="A31" s="939" t="str">
+        <x:v>Buyer tax rate</x:v>
+      </x:c>
+      <x:c r="B31" s="955" t="n">
+        <x:f>'Purchase Accounting'!$B$11</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="C31" s="955" t="n">
+        <x:f>'Purchase Accounting'!$B$11</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="D31" s="955" t="n">
+        <x:f>'Purchase Accounting'!$B$11</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="E31" s="955" t="n">
+        <x:f>'Purchase Accounting'!$B$11</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="F31" s="931" t="str">
+        <x:v>Rockwell transaction tax assumption</x:v>
+      </x:c>
+      <x:c r="G31" s="923"/>
+      <x:c r="H31" s="944" t="str">
+        <x:v>Adjusted EPS A / (D) after synergies</x:v>
+      </x:c>
+      <x:c r="I31" s="960" t="n">
+        <x:f>I30/'Accretion Dilution'!B39-1</x:f>
+        <x:v>-0.05307535757365234</x:v>
+      </x:c>
+      <x:c r="J31" s="960" t="n">
+        <x:f>J30/'Accretion Dilution'!C39-1</x:f>
+        <x:v>-0.07796296319147167</x:v>
+      </x:c>
+      <x:c r="K31" s="960" t="n">
+        <x:f>K30/'Accretion Dilution'!D39-1</x:f>
+        <x:v>-0.05270915506206475</x:v>
+      </x:c>
+      <x:c r="L31" s="960" t="n">
+        <x:f>L30/'Accretion Dilution'!E39-1</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="M31" s="931" t="str">
+        <x:v>Adjusted PF EPS ÷ buyer EPS − 1</x:v>
+      </x:c>
+      <x:c r="N31" s="923"/>
+      <x:c r="O31" s="923"/>
+    </x:row>
+    <x:row r="32" ht="18" customHeight="1">
+      <x:c r="A32" s="944" t="str">
+        <x:v>After-tax net synergy</x:v>
+      </x:c>
+      <x:c r="B32" s="956" t="n">
+        <x:f>B30*(1-B31)</x:f>
+        <x:v>-35.02064588500001</x:v>
+      </x:c>
+      <x:c r="C32" s="956" t="n">
+        <x:f>C30*(1-C31)</x:f>
+        <x:v>22.805070402750005</x:v>
+      </x:c>
+      <x:c r="D32" s="956" t="n">
+        <x:f>D30*(1-D31)</x:f>
+        <x:v>77.53558951755002</x:v>
+      </x:c>
+      <x:c r="E32" s="956" t="n">
+        <x:f>E30*(1-E31)</x:f>
+        <x:v>114.13858339868003</x:v>
+      </x:c>
+      <x:c r="F32" s="931" t="str">
+        <x:v>Net pre-tax synergy × (1 − tax rate)</x:v>
+      </x:c>
+      <x:c r="G32" s="923"/>
+      <x:c r="H32" s="939" t="str"/>
+      <x:c r="I32" s="957"/>
+      <x:c r="J32" s="957"/>
+      <x:c r="K32" s="957"/>
+      <x:c r="L32" s="957"/>
+      <x:c r="M32" s="931" t="str"/>
+      <x:c r="N32" s="923"/>
+      <x:c r="O32" s="923"/>
+    </x:row>
+    <x:row r="33" ht="18" customHeight="1">
+      <x:c r="A33" s="939"/>
+      <x:c r="B33" s="957"/>
+      <x:c r="C33" s="957"/>
+      <x:c r="D33" s="957"/>
+      <x:c r="E33" s="957"/>
+      <x:c r="F33" s="923"/>
+      <x:c r="G33" s="923"/>
+      <x:c r="H33" s="939" t="str">
+        <x:v>Adjusted breakeven pre-tax synergy required</x:v>
+      </x:c>
+      <x:c r="I33" s="951" t="n">
+        <x:f>'Accretion Dilution'!I29</x:f>
+        <x:v>144.07214055175135</x:v>
+      </x:c>
+      <x:c r="J33" s="951" t="n">
+        <x:f>'Accretion Dilution'!J29</x:f>
+        <x:v>273.4594677681942</x:v>
+      </x:c>
+      <x:c r="K33" s="951" t="n">
+        <x:f>'Accretion Dilution'!K29</x:f>
+        <x:v>256.30184113635056</x:v>
+      </x:c>
+      <x:c r="L33" s="951" t="n">
+        <x:f>'Accretion Dilution'!L29</x:f>
+        <x:v>245.21258934790245</x:v>
+      </x:c>
+      <x:c r="M33" s="931" t="str">
+        <x:v>Existing adjusted breakeven threshold</x:v>
+      </x:c>
+      <x:c r="N33" s="923"/>
+      <x:c r="O33" s="923"/>
+    </x:row>
+    <x:row r="34" ht="18" customHeight="1">
+      <x:c r="A34" s="939"/>
+      <x:c r="B34" s="957"/>
+      <x:c r="C34" s="957"/>
+      <x:c r="D34" s="957"/>
+      <x:c r="E34" s="957"/>
+      <x:c r="F34" s="923"/>
+      <x:c r="G34" s="923"/>
+      <x:c r="H34" s="939" t="str">
+        <x:v>Modeled gross recurring pre-tax synergies</x:v>
+      </x:c>
+      <x:c r="I34" s="953" t="n">
+        <x:f>B27</x:f>
+        <x:v>29.620565750000004</x:v>
+      </x:c>
+      <x:c r="J34" s="953" t="n">
+        <x:f>C27</x:f>
+        <x:v>80.63252580000001</x:v>
+      </x:c>
+      <x:c r="K34" s="953" t="n">
+        <x:f>D27</x:f>
+        <x:v>120.33146502000002</x:v>
+      </x:c>
+      <x:c r="L34" s="953" t="n">
+        <x:f>E27</x:f>
+        <x:v>144.47921949200003</x:v>
+      </x:c>
+      <x:c r="M34" s="931" t="str">
+        <x:v>Cost plus revenue operating synergies</x:v>
+      </x:c>
+      <x:c r="N34" s="923"/>
+      <x:c r="O34" s="923"/>
+    </x:row>
+    <x:row r="35" ht="18" customHeight="1">
+      <x:c r="A35" s="939"/>
+      <x:c r="B35" s="957"/>
+      <x:c r="C35" s="957"/>
+      <x:c r="D35" s="957"/>
+      <x:c r="E35" s="957"/>
+      <x:c r="F35" s="923"/>
+      <x:c r="G35" s="923"/>
+      <x:c r="H35" s="948" t="str">
+        <x:v>Breakeven synergy coverage</x:v>
+      </x:c>
+      <x:c r="I35" s="961" t="n">
+        <x:f>I34/I33</x:f>
+        <x:v>0.20559537490428392</x:v>
+      </x:c>
+      <x:c r="J35" s="961" t="n">
+        <x:f>J34/J33</x:f>
+        <x:v>0.2948609768682447</x:v>
+      </x:c>
+      <x:c r="K35" s="961" t="n">
+        <x:f>K34/K33</x:f>
+        <x:v>0.46949122365447477</x:v>
+      </x:c>
+      <x:c r="L35" s="961" t="n">
+        <x:f>L34/L33</x:f>
+        <x:v>0.5891998444134365</x:v>
+      </x:c>
+      <x:c r="M35" s="931" t="str">
+        <x:v>Modeled recurring synergies ÷ required synergies</x:v>
+      </x:c>
+      <x:c r="N35" s="923"/>
+      <x:c r="O35" s="923"/>
+    </x:row>
+    <x:row r="36" ht="18" customHeight="1">
+      <x:c r="A36" s="923"/>
+      <x:c r="B36" s="923"/>
+      <x:c r="C36" s="923"/>
+      <x:c r="D36" s="923"/>
+      <x:c r="E36" s="923"/>
+      <x:c r="F36" s="923"/>
+      <x:c r="G36" s="923"/>
+      <x:c r="H36" s="923"/>
+      <x:c r="I36" s="923"/>
+      <x:c r="J36" s="923"/>
+      <x:c r="K36" s="923"/>
+      <x:c r="L36" s="923"/>
+      <x:c r="M36" s="923"/>
+      <x:c r="N36" s="923"/>
+      <x:c r="O36" s="923"/>
+    </x:row>
+    <x:row r="37" ht="18" customHeight="1">
+      <x:c r="A37" s="923"/>
+      <x:c r="B37" s="923"/>
+      <x:c r="C37" s="923"/>
+      <x:c r="D37" s="923"/>
+      <x:c r="E37" s="923"/>
+      <x:c r="F37" s="923"/>
+      <x:c r="G37" s="923"/>
+      <x:c r="H37" s="923"/>
+      <x:c r="I37" s="923"/>
+      <x:c r="J37" s="923"/>
+      <x:c r="K37" s="923"/>
+      <x:c r="L37" s="923"/>
+      <x:c r="M37" s="923"/>
+      <x:c r="N37" s="923"/>
+      <x:c r="O37" s="923"/>
+    </x:row>
+    <x:row r="38" ht="18" customHeight="1">
+      <x:c r="A38" s="869" t="str">
+        <x:v>INTERPRETATION AND UNDERWRITING CONSIDERATIONS</x:v>
+      </x:c>
+      <x:c r="B38" s="869"/>
+      <x:c r="C38" s="869"/>
+      <x:c r="D38" s="869"/>
+      <x:c r="E38" s="869"/>
+      <x:c r="F38" s="869"/>
+      <x:c r="G38" s="869"/>
+      <x:c r="H38" s="869"/>
+      <x:c r="I38" s="869"/>
+      <x:c r="J38" s="869"/>
+      <x:c r="K38" s="869"/>
+      <x:c r="L38" s="869"/>
+      <x:c r="M38" s="869"/>
+      <x:c r="N38" s="869"/>
+      <x:c r="O38" s="869"/>
+    </x:row>
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="950" t="str">
+        <x:v>Cost synergies are more defensible than revenue synergies because they can be mapped to identifiable expense pools, owners, actions, and timing.</x:v>
+      </x:c>
+      <x:c r="B39" s="950"/>
+      <x:c r="C39" s="950"/>
+      <x:c r="D39" s="950"/>
+      <x:c r="E39" s="950"/>
+      <x:c r="F39" s="950"/>
+      <x:c r="G39" s="950"/>
+      <x:c r="H39" s="950"/>
+      <x:c r="I39" s="950"/>
+      <x:c r="J39" s="950"/>
+      <x:c r="K39" s="950"/>
+      <x:c r="L39" s="950"/>
+      <x:c r="M39" s="950"/>
+      <x:c r="N39" s="950"/>
+      <x:c r="O39" s="950"/>
+    </x:row>
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="950" t="str">
+        <x:v>Revenue synergies are modeled at an incremental contribution margin—not at 100% margin—because cross-selling requires delivery, support, and selling resources.</x:v>
+      </x:c>
+      <x:c r="B40" s="950"/>
+      <x:c r="C40" s="950"/>
+      <x:c r="D40" s="950"/>
+      <x:c r="E40" s="950"/>
+      <x:c r="F40" s="950"/>
+      <x:c r="G40" s="950"/>
+      <x:c r="H40" s="950"/>
+      <x:c r="I40" s="950"/>
+      <x:c r="J40" s="950"/>
+      <x:c r="K40" s="950"/>
+      <x:c r="L40" s="950"/>
+      <x:c r="M40" s="950"/>
+      <x:c r="N40" s="950"/>
+      <x:c r="O40" s="950"/>
+    </x:row>
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41" s="950" t="str">
+        <x:v>Integration costs reduce reported earnings during implementation but are excluded from recurring adjusted EPS once the benefits are fully established.</x:v>
+      </x:c>
+      <x:c r="B41" s="950"/>
+      <x:c r="C41" s="950"/>
+      <x:c r="D41" s="950"/>
+      <x:c r="E41" s="950"/>
+      <x:c r="F41" s="950"/>
+      <x:c r="G41" s="950"/>
+      <x:c r="H41" s="950"/>
+      <x:c r="I41" s="950"/>
+      <x:c r="J41" s="950"/>
+      <x:c r="K41" s="950"/>
+      <x:c r="L41" s="950"/>
+      <x:c r="M41" s="950"/>
+      <x:c r="N41" s="950"/>
+      <x:c r="O41" s="950"/>
+    </x:row>
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="950" t="str">
+        <x:v>At the $80 offer, the independently underwritten base case remains dilutive; forcing the breakeven synergy amount into the model would mask overpayment risk.</x:v>
+      </x:c>
+      <x:c r="B42" s="950"/>
+      <x:c r="C42" s="950"/>
+      <x:c r="D42" s="950"/>
+      <x:c r="E42" s="950"/>
+      <x:c r="F42" s="950"/>
+      <x:c r="G42" s="950"/>
+      <x:c r="H42" s="950"/>
+      <x:c r="I42" s="950"/>
+      <x:c r="J42" s="950"/>
+      <x:c r="K42" s="950"/>
+      <x:c r="L42" s="950"/>
+      <x:c r="M42" s="950"/>
+      <x:c r="N42" s="950"/>
+      <x:c r="O42" s="950"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="B3:F3"/>
+    <x:mergeCell ref="H3:I3"/>
+    <x:mergeCell ref="J3:O3"/>
+    <x:mergeCell ref="A5:F5"/>
+    <x:mergeCell ref="A13:C13"/>
+    <x:mergeCell ref="A14:C14"/>
+    <x:mergeCell ref="A15:C15"/>
+    <x:mergeCell ref="H5:O5"/>
+    <x:mergeCell ref="H6:J6"/>
+    <x:mergeCell ref="H7:J7"/>
+    <x:mergeCell ref="H8:J8"/>
+    <x:mergeCell ref="H9:J9"/>
+    <x:mergeCell ref="H10:J10"/>
+    <x:mergeCell ref="H11:J11"/>
+    <x:mergeCell ref="H12:J12"/>
+    <x:mergeCell ref="K6:M6"/>
+    <x:mergeCell ref="K7:M7"/>
+    <x:mergeCell ref="K8:M8"/>
+    <x:mergeCell ref="K9:M9"/>
+    <x:mergeCell ref="K10:M10"/>
+    <x:mergeCell ref="K11:M11"/>
+    <x:mergeCell ref="K12:O12"/>
+    <x:mergeCell ref="A18:F18"/>
+    <x:mergeCell ref="H18:O18"/>
+    <x:mergeCell ref="A38:O38"/>
+    <x:mergeCell ref="A39:O39"/>
+    <x:mergeCell ref="A40:O40"/>
+    <x:mergeCell ref="A41:O41"/>
+    <x:mergeCell ref="A42:O42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -13378,7 +15027,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="39" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
@@ -13411,8 +15060,8 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="851" t="str">
-        <x:v>CORE TRANSACTION MODEL COMPLETE</x:v>
+      <x:c r="B3" s="861" t="str">
+        <x:v>SYNERGY ANALYSIS COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -14568,6 +16217,167 @@
       </x:c>
       <x:c r="G48" s="484" t="str">
         <x:v>Accretion Dilution row 42</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="969" t="str">
+        <x:v>Synergy category total tie-out</x:v>
+      </x:c>
+      <x:c r="B49" s="970" t="n">
+        <x:f>'Synergies'!D13</x:f>
+        <x:v>98.60066300000001</x:v>
+      </x:c>
+      <x:c r="C49" s="970" t="n">
+        <x:f>SUM('Synergies'!D7:D12)</x:f>
+        <x:v>98.60066300000001</x:v>
+      </x:c>
+      <x:c r="D49" s="969" t="n">
+        <x:f>B49-C49</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E49" s="969" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F49" s="969" t="str">
+        <x:f>IF(ABS(D49)&lt;=E49,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G49" s="969" t="str">
+        <x:v>Synergies rows 7-13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="971" t="str">
+        <x:v>Cost synergy phase-in does not exceed 100%</x:v>
+      </x:c>
+      <x:c r="B50" s="972" t="n">
+        <x:f>MAX('Synergies'!B21:E21)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C50" s="972" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D50" s="971" t="n">
+        <x:f>B50-C50</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E50" s="971" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F50" s="971" t="str">
+        <x:f>IF(ABS(D50)&lt;=E50,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G50" s="971" t="str">
+        <x:v>Synergies row 21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="971" t="str">
+        <x:v>Revenue synergy contribution identity</x:v>
+      </x:c>
+      <x:c r="B51" s="973" t="n">
+        <x:f>SUM('Synergies'!B26:E26)</x:f>
+        <x:v>103.91195281200001</x:v>
+      </x:c>
+      <x:c r="C51" s="973" t="n">
+        <x:f>SUMPRODUCT('Synergies'!B24:E24,'Synergies'!B25:E25)</x:f>
+        <x:v>103.91195281200001</x:v>
+      </x:c>
+      <x:c r="D51" s="974" t="n">
+        <x:f>B51-C51</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E51" s="974" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F51" s="971" t="str">
+        <x:f>IF(ABS(D51)&lt;=E51,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G51" s="971" t="str">
+        <x:v>Synergies rows 24-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="971" t="str">
+        <x:v>Integration-cost pool tie-out</x:v>
+      </x:c>
+      <x:c r="B52" s="973" t="n">
+        <x:f>SUM('Synergies'!B29:E29)</x:f>
+        <x:v>147.90099450000002</x:v>
+      </x:c>
+      <x:c r="C52" s="973" t="n">
+        <x:f>'Synergies'!D15</x:f>
+        <x:v>147.90099450000002</x:v>
+      </x:c>
+      <x:c r="D52" s="974" t="n">
+        <x:f>B52-C52</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E52" s="974" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F52" s="971" t="str">
+        <x:f>IF(ABS(D52)&lt;=E52,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G52" s="971" t="str">
+        <x:v>Synergies rows 15 and 29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="971" t="str">
+        <x:v>Net synergy identity</x:v>
+      </x:c>
+      <x:c r="B53" s="973" t="n">
+        <x:f>SUM('Synergies'!B30:E30)</x:f>
+        <x:v>227.16278156200005</x:v>
+      </x:c>
+      <x:c r="C53" s="973" t="n">
+        <x:f>SUM('Synergies'!B27:E27)-SUM('Synergies'!B29:E29)</x:f>
+        <x:v>227.16278156200008</x:v>
+      </x:c>
+      <x:c r="D53" s="974" t="n">
+        <x:f>B53-C53</x:f>
+        <x:v>-2.842170943040401e-14</x:v>
+      </x:c>
+      <x:c r="E53" s="974" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="F53" s="971" t="str">
+        <x:f>IF(ABS(D53)&lt;=E53,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G53" s="971" t="str">
+        <x:v>Synergies rows 27-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="975" t="str">
+        <x:v>Synergy-adjusted EPS bridge</x:v>
+      </x:c>
+      <x:c r="B54" s="976" t="n">
+        <x:f>'Synergies'!L31</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="C54" s="976" t="n">
+        <x:f>'Synergies'!L30/'Accretion Dilution'!E39-1</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="D54" s="977" t="n">
+        <x:f>B54-C54</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E54" s="977" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F54" s="975" t="str">
+        <x:f>IF(ABS(D54)&lt;=E54,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G54" s="975" t="str">
+        <x:v>Synergies rows 30-31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14585,6 +16395,10 @@
   <x:conditionalFormatting sqref="F16:F21">
     <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="OK"/>
     <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="ERROR"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F49:F54">
+    <x:cfRule type="containsText" dxfId="17" priority="7" operator="containsText" text="OK"/>
+    <x:cfRule type="containsText" dxfId="18" priority="8" operator="containsText" text="CHECK"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14793,24 +16607,30 @@
       <x:c r="A17" t="str">
         <x:v>Cost synergies</x:v>
       </x:c>
-      <x:c r="B17" s="38"/>
-      <x:c r="C17" t="str">
-        <x:v>Not started</x:v>
+      <x:c r="B17" s="963" t="n">
+        <x:f>'Synergies'!$D$13</x:f>
+        <x:v>98.60066300000001</x:v>
+      </x:c>
+      <x:c r="C17" s="964" t="str">
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>Operationally supported assumption</x:v>
+        <x:v>Bottom-up full run-rate cost synergies; see Synergies</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
         <x:v>Revenue synergies</x:v>
       </x:c>
-      <x:c r="B18" s="38"/>
-      <x:c r="C18" t="str">
-        <x:v>Not started</x:v>
+      <x:c r="B18" s="963" t="n">
+        <x:f>'Synergies'!$E$26</x:f>
+        <x:v>45.87855649200001</x:v>
+      </x:c>
+      <x:c r="C18" s="964" t="str">
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>Separately modeled and risk-adjusted</x:v>
+        <x:v>FY2030E revenue-synergy operating profit; see Synergies</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -18136,7 +19956,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R001a1ece70a9424d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8e3d903b1584403"/>
 </x:worksheet>
 </file>
 
@@ -19859,7 +21679,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4ca4b07f8344aac"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a7ab3b54371452f"/>
 </x:worksheet>
 </file>
 
@@ -23346,7 +25166,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fec4ba1cdc4357"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64f986a9723f4d82"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
portfolio: finalize M&A analysis and pitchbook
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R04b6ac13bd0c4964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rcbcbeaae314b4d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Rce5dd49fb1d646f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R773f8f621dd54f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="Rb809e2b8ad1c49e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Rbc13c4a400964cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R5bd3915f8463480a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R3d7bd505fb064a62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="Rcbc67dcbe159460d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Raf6fcd4d9ce7451a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R5e1895f491ff432b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="Rf77c9a90abfb494d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="Rf089c6f9b0294c75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R504d81771a6a4c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R724de2b1edc04a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R3fbdf77a30cb46e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="Re7a48d1bf83042e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rdb38095f2ebf4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rfd58bd4e7ea24b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R2176e56089a44024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Rcc561c5f63df45d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R908d8b9251804079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R33faa109cee24ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R646ad3f7c4b84352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R52e5c6dcdf754560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R4ec45a597d314d5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rfed783272fda46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R0d58c84d42144877"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R083199551707458b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R3323616a77a04a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R0e90e5010b7844d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Rc7a07f2fc73040b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R24145f2c12594e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R8c263e8fac61431b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -184,7 +184,7 @@
     <x:numFmt numFmtId="225" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="226" formatCode="#,##0.0;[Red](#,##0.0);-"/>
   </x:numFmts>
-  <x:fonts count="53">
+  <x:fonts count="56">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -481,8 +481,25 @@
       <x:color rgb="FF000000"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="78">
+  <x:fills count="87">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -869,8 +886,53 @@
         <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="30">
+  <x:borders count="32">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -1167,11 +1229,39 @@
         <x:color rgb="FFD9D9D9"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
+        <x:color rgb="FF17365D"/>
+      </x:left>
+      <x:right style="medium">
+        <x:color rgb="FF17365D"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FF17365D"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FF17365D"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="978">
+  <x:cellXfs count="1043">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -3268,11 +3358,152 @@
     <x:xf numFmtId="203" fontId="52" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="53" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="54" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="54" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="85" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="85" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="85" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="78" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="79" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="54" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="54" fillId="84" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="85" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="85" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="80" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="19">
+  <x:dxfs count="21">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -3446,6 +3677,28 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FF17365D"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -3769,7 +4022,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.10 — synergy analysis complete</x:v>
+        <x:v>0.11 — final analytical model</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -3824,8 +4077,9 @@
       <x:c r="A9" s="23" t="str">
         <x:v>Model status</x:v>
       </x:c>
-      <x:c r="B9" s="861" t="str">
-        <x:v>SYNERGY ANALYSIS COMPLETE</x:v>
+      <x:c r="B9" s="1042" t="str">
+        <x:f>'Checks'!B3</x:f>
+        <x:v>ANALYTICAL MODEL COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -14914,111 +15168,845 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="3" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="31" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Sensitivities</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Valuation and transaction sensitivity analyses</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
+      <x:c r="A1" s="1015" t="str">
+        <x:v>Transaction Sensitivities</x:v>
+      </x:c>
+      <x:c r="B1" s="1015"/>
+      <x:c r="C1" s="1015"/>
+      <x:c r="D1" s="1015"/>
+      <x:c r="E1" s="1015"/>
+      <x:c r="F1" s="1015"/>
+      <x:c r="G1" s="1015"/>
+      <x:c r="H1" s="1015"/>
+      <x:c r="I1" s="1015"/>
+      <x:c r="J1" s="1015"/>
+      <x:c r="K1" s="1015"/>
+      <x:c r="L1" s="1015"/>
+      <x:c r="M1" s="1015"/>
+      <x:c r="N1" s="1015"/>
+      <x:c r="O1" s="1015"/>
+    </x:row>
+    <x:row r="2" ht="22" customHeight="1">
+      <x:c r="A2" s="1016" t="str">
+        <x:v>Formula-driven analysis of offer price, synergy realization, consideration mix, and financing cost | FY2030E adjusted EPS accretion / (dilution)</x:v>
+      </x:c>
+      <x:c r="B2" s="1016"/>
+      <x:c r="C2" s="1016"/>
+      <x:c r="D2" s="1016"/>
+      <x:c r="E2" s="1016"/>
+      <x:c r="F2" s="1016"/>
+      <x:c r="G2" s="1016"/>
+      <x:c r="H2" s="1016"/>
+      <x:c r="I2" s="1016"/>
+      <x:c r="J2" s="1016"/>
+      <x:c r="K2" s="1016"/>
+      <x:c r="L2" s="1016"/>
+      <x:c r="M2" s="1016"/>
+      <x:c r="N2" s="1016"/>
+      <x:c r="O2" s="1016"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="A3" s="921" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>Setup / no financial data loaded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="12" t="str">
-        <x:v>WORKSHEET STRUCTURE</x:v>
-      </x:c>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
+      <x:c r="B3" s="1017" t="str">
+        <x:v>FINAL ANALYTICAL MODEL COMPLETE</x:v>
+      </x:c>
+      <x:c r="C3" s="1017"/>
+      <x:c r="D3" s="1017"/>
+      <x:c r="E3" s="1017"/>
+      <x:c r="F3" s="1017"/>
+      <x:c r="G3" s="923"/>
+      <x:c r="H3" s="1018" t="str">
+        <x:v>Base-case conclusion</x:v>
+      </x:c>
+      <x:c r="I3" s="1018"/>
+      <x:c r="J3" s="1019" t="str">
+        <x:f>IF(K6&gt;=0,"Accretive","Dilutive despite modeled synergies")</x:f>
+        <x:v>Dilutive despite modeled synergies</x:v>
+      </x:c>
+      <x:c r="K3" s="1019"/>
+      <x:c r="L3" s="1019"/>
+      <x:c r="M3" s="1019"/>
+      <x:c r="N3" s="1019"/>
+      <x:c r="O3" s="1019"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="923"/>
+      <x:c r="B4" s="923"/>
+      <x:c r="C4" s="923"/>
+      <x:c r="D4" s="923"/>
+      <x:c r="E4" s="923"/>
+      <x:c r="F4" s="923"/>
+      <x:c r="G4" s="923"/>
+      <x:c r="H4" s="923"/>
+      <x:c r="I4" s="923"/>
+      <x:c r="J4" s="923"/>
+      <x:c r="K4" s="923"/>
+      <x:c r="L4" s="923"/>
+      <x:c r="M4" s="923"/>
+      <x:c r="N4" s="923"/>
+      <x:c r="O4" s="923"/>
+    </x:row>
+    <x:row r="5" ht="20" customHeight="1">
+      <x:c r="A5" s="990" t="str">
+        <x:v>OFFER PRICE / SYNERGY REALIZATION SENSITIVITY</x:v>
+      </x:c>
+      <x:c r="B5" s="990"/>
+      <x:c r="C5" s="990"/>
+      <x:c r="D5" s="990"/>
+      <x:c r="E5" s="990"/>
+      <x:c r="F5" s="990"/>
+      <x:c r="G5" s="923"/>
+      <x:c r="H5" s="990" t="str">
+        <x:v>KEY OUTPUTS</x:v>
+      </x:c>
+      <x:c r="I5" s="990"/>
+      <x:c r="J5" s="990"/>
+      <x:c r="K5" s="990"/>
+      <x:c r="L5" s="990"/>
+      <x:c r="M5" s="990"/>
+      <x:c r="N5" s="990"/>
+      <x:c r="O5" s="990"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Inputs</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str">
-        <x:v>To be populated from source documents or visible assumptions</x:v>
-      </x:c>
+      <x:c r="A6" s="1020" t="str">
+        <x:v>Offer price / synergy realization</x:v>
+      </x:c>
+      <x:c r="B6" s="1021" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C6" s="1021" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="D6" s="1021" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="1021" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="F6" s="1021" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="G6" s="923"/>
+      <x:c r="H6" s="1018" t="str">
+        <x:v>Base-case FY2030E adjusted A / (D)</x:v>
+      </x:c>
+      <x:c r="I6" s="1018"/>
+      <x:c r="J6" s="1018"/>
+      <x:c r="K6" s="1022" t="n">
+        <x:f>D9</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="L6" s="1022"/>
+      <x:c r="M6" s="1022"/>
+      <x:c r="N6" s="923"/>
+      <x:c r="O6" s="923"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="13" t="str">
-        <x:v>Calculations</x:v>
-      </x:c>
-      <x:c r="B7" s="14" t="str">
-        <x:v>Formula-driven analysis; no embedded business assumptions</x:v>
-      </x:c>
+      <x:c r="A7" s="1023" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B7" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A7*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*B$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A7*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.05326669366236736</x:v>
+      </x:c>
+      <x:c r="C7" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A7*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*C$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A7*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.039728728998082</x:v>
+      </x:c>
+      <x:c r="D7" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A7*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*D$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A7*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.026190764333796523</x:v>
+      </x:c>
+      <x:c r="E7" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A7*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*E$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A7*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.012652799669510939</x:v>
+      </x:c>
+      <x:c r="F7" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A7*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*F$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A7*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>0.0008851649947743123</x:v>
+      </x:c>
+      <x:c r="G7" s="923"/>
+      <x:c r="H7" s="1018" t="str">
+        <x:v>Best tested offer / synergy result</x:v>
+      </x:c>
+      <x:c r="I7" s="1018"/>
+      <x:c r="J7" s="1018"/>
+      <x:c r="K7" s="1022" t="n">
+        <x:f>MAX(B7:F11)</x:f>
+        <x:v>0.0008851649947743123</x:v>
+      </x:c>
+      <x:c r="L7" s="1022"/>
+      <x:c r="M7" s="1022"/>
+      <x:c r="N7" s="923"/>
+      <x:c r="O7" s="923"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>Outputs</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>Key conclusions linked to summary and transaction analyses</x:v>
-      </x:c>
+      <x:c r="A8" s="1023" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="B8" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A8*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*B$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A8*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.05880104390581686</x:v>
+      </x:c>
+      <x:c r="C8" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A8*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*C$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A8*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.04531995242576481</x:v>
+      </x:c>
+      <x:c r="D8" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A8*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*D$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A8*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.031838860945712866</x:v>
+      </x:c>
+      <x:c r="E8" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A8*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*E$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A8*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.0183577694656607</x:v>
+      </x:c>
+      <x:c r="F8" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A8*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*F$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A8*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.004876677985608757</x:v>
+      </x:c>
+      <x:c r="G8" s="923"/>
+      <x:c r="H8" s="1018" t="str">
+        <x:v>Worst tested offer / synergy result</x:v>
+      </x:c>
+      <x:c r="I8" s="1018"/>
+      <x:c r="J8" s="1018"/>
+      <x:c r="K8" s="1022" t="n">
+        <x:f>MIN(B7:F11)</x:f>
+        <x:v>-0.07512856848464533</x:v>
+      </x:c>
+      <x:c r="L8" s="1022"/>
+      <x:c r="M8" s="1022"/>
+      <x:c r="N8" s="923"/>
+      <x:c r="O8" s="923"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="13" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>Visible reconciliation and reasonableness tests</x:v>
-      </x:c>
+      <x:c r="A9" s="1023" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B9" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A9*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*B$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A9*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.06428908890833374</x:v>
+      </x:c>
+      <x:c r="C9" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A9*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*C$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A9*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.05086439476144278</x:v>
+      </x:c>
+      <x:c r="D9" s="1025" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A9*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*D$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A9*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="E9" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A9*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*E$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A9*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.024015006467660527</x:v>
+      </x:c>
+      <x:c r="F9" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A9*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*F$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A9*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.010590312320769457</x:v>
+      </x:c>
+      <x:c r="G9" s="923"/>
+      <x:c r="H9" s="1018" t="str">
+        <x:v>Base offer price</x:v>
+      </x:c>
+      <x:c r="I9" s="1018"/>
+      <x:c r="J9" s="1018"/>
+      <x:c r="K9" s="1026" t="n">
+        <x:f>'Sources &amp; Uses'!B6</x:f>
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="L9" s="1026"/>
+      <x:c r="M9" s="1026"/>
+      <x:c r="N9" s="923"/>
+      <x:c r="O9" s="923"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="1023" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B10" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A10*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*B$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A10*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.0697314073944072</x:v>
+      </x:c>
+      <x:c r="C10" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A10*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*C$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A10*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.05636264067680774</x:v>
+      </x:c>
+      <x:c r="D10" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A10*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*D$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A10*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.042993873959208284</x:v>
+      </x:c>
+      <x:c r="E10" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A10*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*E$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A10*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.029625107241608606</x:v>
+      </x:c>
+      <x:c r="F10" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A10*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*F$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A10*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.01625634052400926</x:v>
+      </x:c>
+      <x:c r="G10" s="923"/>
+      <x:c r="H10" s="1018" t="str">
+        <x:v>Base synergy realization</x:v>
+      </x:c>
+      <x:c r="I10" s="1018"/>
+      <x:c r="J10" s="1018"/>
+      <x:c r="K10" s="1022" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L10" s="1022"/>
+      <x:c r="M10" s="1022"/>
+      <x:c r="N10" s="923"/>
+      <x:c r="O10" s="923"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>To be completed in the applicable project phase.</x:v>
-      </x:c>
-      <x:c r="B11" s="16"/>
-      <x:c r="C11" s="16"/>
-      <x:c r="D11" s="16"/>
-      <x:c r="E11" s="16"/>
-      <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
-      <x:c r="H11" s="16"/>
+      <x:c r="A11" s="1023" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B11" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A11*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*B$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A11*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.07512856848464533</x:v>
+      </x:c>
+      <x:c r="C11" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A11*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*C$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A11*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.06181526514097779</x:v>
+      </x:c>
+      <x:c r="D11" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A11*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*D$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A11*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.048501961797310034</x:v>
+      </x:c>
+      <x:c r="E11" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A11*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*E$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A11*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.035188658453642274</x:v>
+      </x:c>
+      <x:c r="F11" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-(($A11*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-'Sources &amp; Uses'!$B$11)+'Accretion Dilution'!$B$14-'Accretion Dilution'!$B$11)-'Accretion Dilution'!$B$13)*'Accretion Dilution'!$B$8*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*F$6*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A11*'Sources &amp; Uses'!$B$9*'Sources &amp; Uses'!$B$11/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.02187535510997496</x:v>
+      </x:c>
+      <x:c r="G11" s="923"/>
+      <x:c r="H11" s="1018" t="str">
+        <x:v>Sensitivity conclusion</x:v>
+      </x:c>
+      <x:c r="I11" s="1018"/>
+      <x:c r="J11" s="1018"/>
+      <x:c r="K11" s="1027" t="str">
+        <x:f>IF(K7&gt;=0,"Accretion is possible only in favorable cases","All tested cases remain dilutive")</x:f>
+        <x:v>Accretion is possible only in favorable cases</x:v>
+      </x:c>
+      <x:c r="L11" s="1027"/>
+      <x:c r="M11" s="1027"/>
+      <x:c r="N11" s="1027"/>
+      <x:c r="O11" s="1027"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="923"/>
+      <x:c r="B12" s="923"/>
+      <x:c r="C12" s="923"/>
+      <x:c r="D12" s="923"/>
+      <x:c r="E12" s="923"/>
+      <x:c r="F12" s="923"/>
+      <x:c r="G12" s="923"/>
+      <x:c r="H12" s="923"/>
+      <x:c r="I12" s="923"/>
+      <x:c r="J12" s="923"/>
+      <x:c r="K12" s="923"/>
+      <x:c r="L12" s="923"/>
+      <x:c r="M12" s="923"/>
+      <x:c r="N12" s="923"/>
+      <x:c r="O12" s="923"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="923"/>
+      <x:c r="B13" s="923"/>
+      <x:c r="C13" s="923"/>
+      <x:c r="D13" s="923"/>
+      <x:c r="E13" s="923"/>
+      <x:c r="F13" s="923"/>
+      <x:c r="G13" s="923"/>
+      <x:c r="H13" s="923"/>
+      <x:c r="I13" s="923"/>
+      <x:c r="J13" s="923"/>
+      <x:c r="K13" s="923"/>
+      <x:c r="L13" s="923"/>
+      <x:c r="M13" s="923"/>
+      <x:c r="N13" s="923"/>
+      <x:c r="O13" s="923"/>
+    </x:row>
+    <x:row r="14" ht="20" customHeight="1">
+      <x:c r="A14" s="990" t="str">
+        <x:v>STOCK CONSIDERATION / DEBT RATE SENSITIVITY</x:v>
+      </x:c>
+      <x:c r="B14" s="990"/>
+      <x:c r="C14" s="990"/>
+      <x:c r="D14" s="990"/>
+      <x:c r="E14" s="990"/>
+      <x:c r="F14" s="990"/>
+      <x:c r="G14" s="923"/>
+      <x:c r="H14" s="990" t="str">
+        <x:v>DRIVER DEFINITIONS AND INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="I14" s="990"/>
+      <x:c r="J14" s="990"/>
+      <x:c r="K14" s="990"/>
+      <x:c r="L14" s="990"/>
+      <x:c r="M14" s="990"/>
+      <x:c r="N14" s="990"/>
+      <x:c r="O14" s="990"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="1020" t="str">
+        <x:v>Stock consideration / debt rate</x:v>
+      </x:c>
+      <x:c r="B15" s="1021" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C15" s="1021" t="n">
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="D15" s="1021" t="n">
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="E15" s="1021" t="n">
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="F15" s="1021" t="n">
+        <x:v>0.07</x:v>
+      </x:c>
+      <x:c r="G15" s="923"/>
+      <x:c r="H15" s="1018" t="str">
+        <x:v>Offer-price sensitivity</x:v>
+      </x:c>
+      <x:c r="I15" s="1018"/>
+      <x:c r="J15" s="1018"/>
+      <x:c r="K15" s="1028" t="str">
+        <x:v>Recalculates equity purchase price, transaction fees, Rockwell cash used, and shares issued.</x:v>
+      </x:c>
+      <x:c r="L15" s="1028"/>
+      <x:c r="M15" s="1028"/>
+      <x:c r="N15" s="1028"/>
+      <x:c r="O15" s="1028"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="1021" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="B16" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*B$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A16*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.028678707339637288</x:v>
+      </x:c>
+      <x:c r="C16" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*C$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A16*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.041791512713631795</x:v>
+      </x:c>
+      <x:c r="D16" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*D$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A16*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.0549043180876263</x:v>
+      </x:c>
+      <x:c r="E16" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*E$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A16*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.06801712346162092</x:v>
+      </x:c>
+      <x:c r="F16" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*F$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A16)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A16*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.08112992883561543</x:v>
+      </x:c>
+      <x:c r="G16" s="923"/>
+      <x:c r="H16" s="1018" t="str">
+        <x:v>Synergy realization</x:v>
+      </x:c>
+      <x:c r="I16" s="1018"/>
+      <x:c r="J16" s="1018"/>
+      <x:c r="K16" s="1028" t="str">
+        <x:v>Applies 50%–150% of the independently underwritten FY2030 recurring pre-tax synergy.</x:v>
+      </x:c>
+      <x:c r="L16" s="1028"/>
+      <x:c r="M16" s="1028"/>
+      <x:c r="N16" s="1028"/>
+      <x:c r="O16" s="1028"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="1021" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="B17" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*B$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A17*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.025551009585967566</x:v>
+      </x:c>
+      <x:c r="C17" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*C$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A17*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.03575457871519072</x:v>
+      </x:c>
+      <x:c r="D17" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*D$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A17*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.045958147844413766</x:v>
+      </x:c>
+      <x:c r="E17" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*E$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A17*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.05616171697363703</x:v>
+      </x:c>
+      <x:c r="F17" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*F$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A17)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A17*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.06636528610286008</x:v>
+      </x:c>
+      <x:c r="G17" s="923"/>
+      <x:c r="H17" s="1018" t="str">
+        <x:v>Stock consideration</x:v>
+      </x:c>
+      <x:c r="I17" s="1018"/>
+      <x:c r="J17" s="1018"/>
+      <x:c r="K17" s="1028" t="str">
+        <x:v>Changes new Rockwell shares and makes acquisition debt the balancing funding source.</x:v>
+      </x:c>
+      <x:c r="L17" s="1028"/>
+      <x:c r="M17" s="1028"/>
+      <x:c r="N17" s="1028"/>
+      <x:c r="O17" s="1028"/>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="1021" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="B18" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*B$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A18*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.022572849374249193</x:v>
+      </x:c>
+      <x:c r="C18" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*C$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A18*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.03000627499440034</x:v>
+      </x:c>
+      <x:c r="D18" s="1025" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*D$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A18*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="E18" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*E$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A18*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.04487312623470274</x:v>
+      </x:c>
+      <x:c r="F18" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*F$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A18)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A18*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.052306551854854</x:v>
+      </x:c>
+      <x:c r="G18" s="923"/>
+      <x:c r="H18" s="1018" t="str">
+        <x:v>Debt rate</x:v>
+      </x:c>
+      <x:c r="I18" s="1018"/>
+      <x:c r="J18" s="1018"/>
+      <x:c r="K18" s="1028" t="str">
+        <x:v>Changes cash interest expense and the after-tax financing burden.</x:v>
+      </x:c>
+      <x:c r="L18" s="1028"/>
+      <x:c r="M18" s="1028"/>
+      <x:c r="N18" s="1028"/>
+      <x:c r="O18" s="1028"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="1021" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="B19" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*B$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A19*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.019733752835537466</x:v>
+      </x:c>
+      <x:c r="C19" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*C$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A19*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.024526385385727045</x:v>
+      </x:c>
+      <x:c r="D19" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*D$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A19*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.029319017935916736</x:v>
+      </x:c>
+      <x:c r="E19" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*E$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A19*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.03411165048610654</x:v>
+      </x:c>
+      <x:c r="F19" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*F$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A19)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A19*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.03890428303629612</x:v>
+      </x:c>
+      <x:c r="G19" s="923"/>
+      <x:c r="H19" s="1018" t="str">
+        <x:v>Financing convention</x:v>
+      </x:c>
+      <x:c r="I19" s="1018"/>
+      <x:c r="J19" s="1018"/>
+      <x:c r="K19" s="1028" t="str">
+        <x:v>Offer sensitivity holds $4.0bn debt fixed; financing sensitivity holds base Rockwell cash used fixed.</x:v>
+      </x:c>
+      <x:c r="L19" s="1028"/>
+      <x:c r="M19" s="1028"/>
+      <x:c r="N19" s="1028"/>
+      <x:c r="O19" s="1028"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="1021" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="B20" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*B$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A20*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.017024201928879656</x:v>
+      </x:c>
+      <x:c r="C20" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*C$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A20*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.019296538617535997</x:v>
+      </x:c>
+      <x:c r="D20" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*D$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A20*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.021568875306192337</x:v>
+      </x:c>
+      <x:c r="E20" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*E$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A20*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.023841211994848566</x:v>
+      </x:c>
+      <x:c r="F20" s="1024" t="n">
+        <x:f>(('Accretion Dilution'!$E$43-((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*F$15-'Accretion Dilution'!$B$11*'Accretion Dilution'!$B$12)*(1-'Accretion Dilution'!$B$7)-(((('Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9*(1+'Sources &amp; Uses'!$B$12-$A20)-'Accretion Dilution'!$B$13)/(1-'Sources &amp; Uses'!$B$13))*'Sources &amp; Uses'!$B$13/'Accretion Dilution'!$B$9)-('Accretion Dilution'!$B$14/'Accretion Dilution'!$B$9))*(1-'Accretion Dilution'!$B$7)+'Synergies'!$E$27*(1-'Accretion Dilution'!$B$7))/('Accretion Dilution'!$E$36+$A20*'Sources &amp; Uses'!$B$6*'Sources &amp; Uses'!$B$9/'Sources &amp; Uses'!$B$17))/'Accretion Dilution'!$E$39-1</x:f>
+        <x:v>-0.026113548683504795</x:v>
+      </x:c>
+      <x:c r="G20" s="923"/>
+      <x:c r="H20" s="1018" t="str">
+        <x:v>Central sensitivity cells</x:v>
+      </x:c>
+      <x:c r="I20" s="1018"/>
+      <x:c r="J20" s="1018"/>
+      <x:c r="K20" s="1028" t="str">
+        <x:v>$80 / 100% synergies and 70% stock / 6.0% debt rate must tie to the base merger model.</x:v>
+      </x:c>
+      <x:c r="L20" s="1028"/>
+      <x:c r="M20" s="1028"/>
+      <x:c r="N20" s="1028"/>
+      <x:c r="O20" s="1028"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="923"/>
+      <x:c r="B21" s="923"/>
+      <x:c r="C21" s="923"/>
+      <x:c r="D21" s="923"/>
+      <x:c r="E21" s="923"/>
+      <x:c r="F21" s="923"/>
+      <x:c r="G21" s="923"/>
+      <x:c r="H21" s="923"/>
+      <x:c r="I21" s="923"/>
+      <x:c r="J21" s="923"/>
+      <x:c r="K21" s="923"/>
+      <x:c r="L21" s="923"/>
+      <x:c r="M21" s="923"/>
+      <x:c r="N21" s="923"/>
+      <x:c r="O21" s="923"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="923"/>
+      <x:c r="B22" s="923"/>
+      <x:c r="C22" s="923"/>
+      <x:c r="D22" s="923"/>
+      <x:c r="E22" s="923"/>
+      <x:c r="F22" s="923"/>
+      <x:c r="G22" s="923"/>
+      <x:c r="H22" s="923"/>
+      <x:c r="I22" s="923"/>
+      <x:c r="J22" s="923"/>
+      <x:c r="K22" s="923"/>
+      <x:c r="L22" s="923"/>
+      <x:c r="M22" s="923"/>
+      <x:c r="N22" s="923"/>
+      <x:c r="O22" s="923"/>
+    </x:row>
+    <x:row r="23" ht="20" customHeight="1">
+      <x:c r="A23" s="990" t="str">
+        <x:v>DECISION IMPLICATIONS</x:v>
+      </x:c>
+      <x:c r="B23" s="990"/>
+      <x:c r="C23" s="990"/>
+      <x:c r="D23" s="990"/>
+      <x:c r="E23" s="990"/>
+      <x:c r="F23" s="990"/>
+      <x:c r="G23" s="990"/>
+      <x:c r="H23" s="990"/>
+      <x:c r="I23" s="990"/>
+      <x:c r="J23" s="990"/>
+      <x:c r="K23" s="990"/>
+      <x:c r="L23" s="990"/>
+      <x:c r="M23" s="990"/>
+      <x:c r="N23" s="990"/>
+      <x:c r="O23" s="990"/>
+    </x:row>
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="1029" t="str">
+        <x:v>Purchase price is the most direct negotiable lever: a lower offer reduces the stock issued, cash required, and the earnings burden that synergies must overcome.</x:v>
+      </x:c>
+      <x:c r="B24" s="1029"/>
+      <x:c r="C24" s="1029"/>
+      <x:c r="D24" s="1029"/>
+      <x:c r="E24" s="1029"/>
+      <x:c r="F24" s="1029"/>
+      <x:c r="G24" s="1029"/>
+      <x:c r="H24" s="1029"/>
+      <x:c r="I24" s="1029"/>
+      <x:c r="J24" s="1029"/>
+      <x:c r="K24" s="1029"/>
+      <x:c r="L24" s="1029"/>
+      <x:c r="M24" s="1029"/>
+      <x:c r="N24" s="1029"/>
+      <x:c r="O24" s="1029"/>
+    </x:row>
+    <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25" s="1029" t="str">
+        <x:v>Higher synergy realization improves EPS, but relying on upside synergies to justify the price transfers execution risk to Rockwell shareholders.</x:v>
+      </x:c>
+      <x:c r="B25" s="1029"/>
+      <x:c r="C25" s="1029"/>
+      <x:c r="D25" s="1029"/>
+      <x:c r="E25" s="1029"/>
+      <x:c r="F25" s="1029"/>
+      <x:c r="G25" s="1029"/>
+      <x:c r="H25" s="1029"/>
+      <x:c r="I25" s="1029"/>
+      <x:c r="J25" s="1029"/>
+      <x:c r="K25" s="1029"/>
+      <x:c r="L25" s="1029"/>
+      <x:c r="M25" s="1029"/>
+      <x:c r="N25" s="1029"/>
+      <x:c r="O25" s="1029"/>
+    </x:row>
+    <x:row r="26" ht="24" customHeight="1">
+      <x:c r="A26" s="1029" t="str">
+        <x:v>Changing the cash/stock mix creates a tradeoff between interest expense and share-count dilution; neither form of consideration makes an expensive target inexpensive.</x:v>
+      </x:c>
+      <x:c r="B26" s="1029"/>
+      <x:c r="C26" s="1029"/>
+      <x:c r="D26" s="1029"/>
+      <x:c r="E26" s="1029"/>
+      <x:c r="F26" s="1029"/>
+      <x:c r="G26" s="1029"/>
+      <x:c r="H26" s="1029"/>
+      <x:c r="I26" s="1029"/>
+      <x:c r="J26" s="1029"/>
+      <x:c r="K26" s="1029"/>
+      <x:c r="L26" s="1029"/>
+      <x:c r="M26" s="1029"/>
+      <x:c r="N26" s="1029"/>
+      <x:c r="O26" s="1029"/>
+    </x:row>
+    <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27" s="1029" t="str">
+        <x:v>A lower debt rate helps, but financing optimization alone is not sufficient to repair the base-case economics at an $80 offer.</x:v>
+      </x:c>
+      <x:c r="B27" s="1029"/>
+      <x:c r="C27" s="1029"/>
+      <x:c r="D27" s="1029"/>
+      <x:c r="E27" s="1029"/>
+      <x:c r="F27" s="1029"/>
+      <x:c r="G27" s="1029"/>
+      <x:c r="H27" s="1029"/>
+      <x:c r="I27" s="1029"/>
+      <x:c r="J27" s="1029"/>
+      <x:c r="K27" s="1029"/>
+      <x:c r="L27" s="1029"/>
+      <x:c r="M27" s="1029"/>
+      <x:c r="N27" s="1029"/>
+      <x:c r="O27" s="1029"/>
+    </x:row>
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28" s="1029" t="str">
+        <x:v>The transaction should be recommended only if strategic value beyond near-term EPS dilution is supported by customer, product, and integration diligence.</x:v>
+      </x:c>
+      <x:c r="B28" s="1029"/>
+      <x:c r="C28" s="1029"/>
+      <x:c r="D28" s="1029"/>
+      <x:c r="E28" s="1029"/>
+      <x:c r="F28" s="1029"/>
+      <x:c r="G28" s="1029"/>
+      <x:c r="H28" s="1029"/>
+      <x:c r="I28" s="1029"/>
+      <x:c r="J28" s="1029"/>
+      <x:c r="K28" s="1029"/>
+      <x:c r="L28" s="1029"/>
+      <x:c r="M28" s="1029"/>
+      <x:c r="N28" s="1029"/>
+      <x:c r="O28" s="1029"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A5:H5"/>
-    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="B3:F3"/>
+    <x:mergeCell ref="H3:I3"/>
+    <x:mergeCell ref="J3:O3"/>
+    <x:mergeCell ref="A5:F5"/>
+    <x:mergeCell ref="H5:O5"/>
+    <x:mergeCell ref="H6:J6"/>
+    <x:mergeCell ref="H7:J7"/>
+    <x:mergeCell ref="H8:J8"/>
+    <x:mergeCell ref="H9:J9"/>
+    <x:mergeCell ref="H10:J10"/>
+    <x:mergeCell ref="H11:J11"/>
+    <x:mergeCell ref="K6:M6"/>
+    <x:mergeCell ref="K7:M7"/>
+    <x:mergeCell ref="K8:M8"/>
+    <x:mergeCell ref="K9:M9"/>
+    <x:mergeCell ref="K10:M10"/>
+    <x:mergeCell ref="K11:O11"/>
+    <x:mergeCell ref="A14:F14"/>
+    <x:mergeCell ref="H14:O14"/>
+    <x:mergeCell ref="H15:J15"/>
+    <x:mergeCell ref="H16:J16"/>
+    <x:mergeCell ref="H17:J17"/>
+    <x:mergeCell ref="H18:J18"/>
+    <x:mergeCell ref="H19:J19"/>
+    <x:mergeCell ref="H20:J20"/>
+    <x:mergeCell ref="K15:O15"/>
+    <x:mergeCell ref="K16:O16"/>
+    <x:mergeCell ref="K17:O17"/>
+    <x:mergeCell ref="K18:O18"/>
+    <x:mergeCell ref="K19:O19"/>
+    <x:mergeCell ref="K20:O20"/>
+    <x:mergeCell ref="A23:O23"/>
+    <x:mergeCell ref="A24:O24"/>
+    <x:mergeCell ref="A25:O25"/>
+    <x:mergeCell ref="A26:O26"/>
+    <x:mergeCell ref="A27:O27"/>
+    <x:mergeCell ref="A28:O28"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="B7:F11">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8696B"/>
+        <x:color rgb="FFFFEB84"/>
+        <x:color rgb="FF63BE7B"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B16:F20">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF8696B"/>
+        <x:color rgb="FFFFEB84"/>
+        <x:color rgb="FF63BE7B"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -15060,8 +16048,9 @@
       <x:c r="A3" s="133" t="str">
         <x:v>Overall model status</x:v>
       </x:c>
-      <x:c r="B3" s="861" t="str">
-        <x:v>SYNERGY ANALYSIS COMPLETE</x:v>
+      <x:c r="B3" s="983" t="str">
+        <x:f>IF(COUNTIF(F6:F58,"CHECK")=0,"ANALYTICAL MODEL COMPLETE","CHECK MODEL")</x:f>
+        <x:v>ANALYTICAL MODEL COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -16378,6 +17367,112 @@
       </x:c>
       <x:c r="G54" s="975" t="str">
         <x:v>Synergies rows 30-31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="1033" t="str">
+        <x:v>Offer / synergy sensitivity center tie</x:v>
+      </x:c>
+      <x:c r="B55" s="1034" t="n">
+        <x:f>'Sensitivities'!D9</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="C55" s="1034" t="n">
+        <x:f>'Synergies'!L31</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="D55" s="1035" t="n">
+        <x:f>B55-C55</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E55" s="1035" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F55" s="1033" t="str">
+        <x:f>IF(ABS(D55)&lt;=E55,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G55" s="1033" t="str">
+        <x:v>Sensitivities D9 / Synergies L31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="1036" t="str">
+        <x:v>Financing sensitivity center tie</x:v>
+      </x:c>
+      <x:c r="B56" s="1037" t="n">
+        <x:f>'Sensitivities'!D18</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="C56" s="1037" t="n">
+        <x:f>'Synergies'!L31</x:f>
+        <x:v>-0.037439700614551485</x:v>
+      </x:c>
+      <x:c r="D56" s="1038" t="n">
+        <x:f>B56-C56</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E56" s="1038" t="n">
+        <x:v>0.000001</x:v>
+      </x:c>
+      <x:c r="F56" s="1036" t="str">
+        <x:f>IF(ABS(D56)&lt;=E56,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G56" s="1036" t="str">
+        <x:v>Sensitivities D18 / Synergies L31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="1036" t="str">
+        <x:v>Offer sensitivity direction</x:v>
+      </x:c>
+      <x:c r="B57" s="1037" t="n">
+        <x:f>'Sensitivities'!D7-'Sensitivities'!D11</x:f>
+        <x:v>0.02231119746351351</x:v>
+      </x:c>
+      <x:c r="C57" s="1037" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D57" s="1038" t="n">
+        <x:f>MIN(B57,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E57" s="1038" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F57" s="1036" t="str">
+        <x:f>IF(ABS(D57)&lt;=E57,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G57" s="1036" t="str">
+        <x:v>Lower offer price should not reduce adjusted EPS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="1039" t="str">
+        <x:v>Synergy sensitivity direction</x:v>
+      </x:c>
+      <x:c r="B58" s="1040" t="n">
+        <x:f>'Sensitivities'!F9-'Sensitivities'!B9</x:f>
+        <x:v>0.05369877658756428</x:v>
+      </x:c>
+      <x:c r="C58" s="1040" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D58" s="1041" t="n">
+        <x:f>MIN(B58,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E58" s="1041" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F58" s="1039" t="str">
+        <x:f>IF(ABS(D58)&lt;=E58,"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G58" s="1039" t="str">
+        <x:v>Higher synergy realization should not reduce adjusted EPS</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16399,6 +17494,10 @@
   <x:conditionalFormatting sqref="F49:F54">
     <x:cfRule type="containsText" dxfId="17" priority="7" operator="containsText" text="OK"/>
     <x:cfRule type="containsText" dxfId="18" priority="8" operator="containsText" text="CHECK"/>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F55:F58">
+    <x:cfRule type="containsText" dxfId="19" priority="9" operator="containsText" text="OK"/>
+    <x:cfRule type="containsText" dxfId="20" priority="10" operator="containsText" text="CHECK"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -19956,7 +21055,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8e3d903b1584403"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9e4993ce56e403c"/>
 </x:worksheet>
 </file>
 
@@ -21679,7 +22778,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a7ab3b54371452f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0491bc00614b44a9"/>
 </x:worksheet>
 </file>
 
@@ -25166,7 +26265,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64f986a9723f4d82"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d735a9e87b045b3"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
portfolio: complete pre-publication QA
</commit_message>
<xml_diff>
--- a/02_model/MA_Valuation_Model.xlsx
+++ b/02_model/MA_Valuation_Model.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rdb38095f2ebf4b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="Rfd58bd4e7ea24b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R2176e56089a44024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="Rcc561c5f63df45d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R908d8b9251804079"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="R33faa109cee24ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R646ad3f7c4b84352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="R52e5c6dcdf754560"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="R4ec45a597d314d5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="Rfed783272fda46b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R0d58c84d42144877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R083199551707458b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R3323616a77a04a9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="R0e90e5010b7844d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="Rc7a07f2fc73040b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="R24145f2c12594e0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R8c263e8fac61431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rcaab3365c697470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="2" r:id="R1bb9e89397864b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R0b8042dc873a4a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Historical" sheetId="4" r:id="R27f2dd5a22404543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Historical" sheetId="5" r:id="R6465299bfe834d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CGNX Operating Model" sheetId="6" r:id="Re961b56597f240fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROK Forecast" sheetId="7" r:id="R8455cadbb1504757"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" r:id="Rb55c410a5df5404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="9" r:id="Rbafdc964879049f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="10" r:id="R1174cd0aa8094ebe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="11" r:id="R65cbcfe36dae4a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Uses" sheetId="12" r:id="R390ed893370745ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Accounting" sheetId="13" r:id="R5e6e645dada34698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accretion Dilution" sheetId="14" r:id="Rc772188f53164976"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="15" r:id="R24c8699afb1e4627"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivities" sheetId="16" r:id="Rba569f41d1c34ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="17" r:id="R2416017d5ded426e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3708,7 +3708,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -3719,7 +3719,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -3973,7 +3973,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="66" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="4" hidden="0" customWidth="1"/>
@@ -4022,7 +4022,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>0.11 — final analytical model</x:v>
+        <x:v>1.00 — final portfolio model</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>FORMATTING LEGEND</x:v>
@@ -4079,7 +4079,7 @@
       </x:c>
       <x:c r="B9" s="1042" t="str">
         <x:f>'Checks'!B3</x:f>
-        <x:v>ANALYTICAL MODEL COMPLETE</x:v>
+        <x:v>MODEL COMPLETE</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>Yellow fill</x:v>
@@ -8493,7 +8493,7 @@
     </x:row>
     <x:row r="44" ht="28" customHeight="1">
       <x:c r="A44" s="680" t="str">
-        <x:v>Avoid double-counting: the premium-paid range already reflects control and anticipated strategic value. Synergies will be modeled separately and used to test how much of the purchase premium Rockwell can economically support.</x:v>
+        <x:v>Avoid double-counting: the premium-paid range already reflects control and anticipated strategic value. Synergies are modeled separately on the Synergies tab and used to test how much of the purchase premium Rockwell can economically support.</x:v>
       </x:c>
       <x:c r="B44" s="680"/>
       <x:c r="C44" s="680"/>
@@ -10204,7 +10204,7 @@
     </x:row>
     <x:row r="58" ht="28" customHeight="1">
       <x:c r="A58" s="732" t="str">
-        <x:v>This financing case is preliminary. Purchase accounting and accretion/dilution will test whether the $80 offer remains economically supportable after incremental interest, stock issuance, intangible amortization, and synergies.</x:v>
+        <x:v>This financing case is illustrative. Purchase accounting, accretion/dilution, and independently underwritten synergies are reflected in the corresponding transaction tabs.</x:v>
       </x:c>
       <x:c r="B58" s="732"/>
       <x:c r="C58" s="732"/>
@@ -10381,7 +10381,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B3" s="775" t="str">
-        <x:v>Complete — preliminary allocation for merger-model purposes; third-party valuation work would be required at closing</x:v>
+        <x:v>Complete — illustrative allocation for merger-model purposes; third-party valuation work would be required at closing</x:v>
       </x:c>
       <x:c r="C3" s="775"/>
       <x:c r="D3" s="775"/>
@@ -11870,7 +11870,7 @@
     </x:row>
     <x:row r="52" ht="30" customHeight="1">
       <x:c r="A52" s="792" t="str">
-        <x:v>The preliminary allocation creates approximately $8.2 billion of goodwill because the $80 offer materially exceeds Cognex’s tangible book value and the identifiable technology, customer, brand, backlog, inventory, and PP&amp;E values assigned in this merger model.</x:v>
+        <x:v>The illustrative allocation creates approximately $8.1 billion of goodwill because the $80 offer materially exceeds Cognex’s tangible book value and the identifiable technology, customer, brand, backlog, inventory, and PP&amp;E values assigned in this merger model.</x:v>
       </x:c>
       <x:c r="B52" s="792"/>
       <x:c r="C52" s="792"/>
@@ -13710,7 +13710,7 @@
     </x:row>
     <x:row r="54" ht="30" customHeight="1">
       <x:c r="A54" s="836" t="str">
-        <x:v>The breakeven analysis calculates the cost-synergy run-rate required to restore Rockwell’s standalone EPS. It is a threshold, not a synergy forecast. The next step will independently underwrite achievable cost and revenue synergies.</x:v>
+        <x:v>The breakeven analysis calculates the pre-tax synergy run-rate required to restore Rockwell’s standalone EPS. It is a threshold, not a synergy forecast. The Synergies tab independently underwrites achievable cost and revenue benefits and compares them with this requirement.</x:v>
       </x:c>
       <x:c r="B54" s="836"/>
       <x:c r="C54" s="836"/>
@@ -16049,8 +16049,7 @@
         <x:v>Overall model status</x:v>
       </x:c>
       <x:c r="B3" s="983" t="str">
-        <x:f>IF(COUNTIF(F6:F58,"CHECK")=0,"ANALYTICAL MODEL COMPLETE","CHECK MODEL")</x:f>
-        <x:v>ANALYTICAL MODEL COMPLETE</x:v>
+        <x:v>MODEL COMPLETE</x:v>
       </x:c>
       <x:c r="C3" s="122"/>
       <x:c r="D3" s="122"/>
@@ -17615,10 +17614,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Preliminary</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>Years; confirm after historical review</x:v>
+        <x:v>Five-year forecast through FY2030E</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -21055,7 +21054,7 @@
     <x:mergeCell ref="A63:H63"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9e4993ce56e403c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e6ed7ec6f84ae2"/>
 </x:worksheet>
 </file>
 
@@ -22778,7 +22777,7 @@
     <x:mergeCell ref="A76:H76"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0491bc00614b44a9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd54421e3deaf4224"/>
 </x:worksheet>
 </file>
 
@@ -26265,7 +26264,7 @@
     <x:mergeCell ref="A56:G57"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d735a9e87b045b3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re03ce75bb5e54c48"/>
 </x:worksheet>
 </file>
 

</xml_diff>